<commit_message>
chore: price data 2026-09-16
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20260916T005126895248+0000</t>
+          <t>20260916T005414352292+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-16T00:51:26.895248+00:00</t>
+          <t>2026-09-16T00:54:14.352292+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: price data 2026-09-17
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MacBook Pro'!$A$1:$S$92</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MacBook Air'!$A$1:$S$68</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20260916T083942872752+0000</t>
+          <t>20260917T084356123359+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-16T08:39:42.872752+00:00</t>
+          <t>2026-09-17T08:43:56.123359+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>277.720685</v>
+        <v>277.510311</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -810,10 +810,10 @@
         </is>
       </c>
       <c r="C26" s="3" t="n">
-        <v>643000</v>
+        <v>645000</v>
       </c>
       <c r="D26" t="n">
-        <v>44.9</v>
+        <v>44.7</v>
       </c>
       <c r="E26" t="n">
         <v>4</v>
@@ -1147,10 +1147,10 @@
         <v>470000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>688317</v>
+        <v>687795</v>
       </c>
       <c r="L2" t="n">
-        <v>35.34955551003389</v>
+        <v>35.30048924461504</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1214,10 +1214,10 @@
         <v>465000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>688317</v>
+        <v>687795</v>
       </c>
       <c r="L3" t="n">
-        <v>33.4608908395405</v>
+        <v>33.41039117760379</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>774410</v>
+        <v>773824</v>
       </c>
       <c r="L4" t="n">
-        <v>35.43484717397761</v>
+        <v>35.38595339508726</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>774410</v>
+        <v>773824</v>
       </c>
       <c r="L5" t="n">
-        <v>32.85223589571415</v>
+        <v>32.80138636175668</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>860504</v>
+        <v>859852</v>
       </c>
       <c r="L6" t="n">
-        <v>38.17576675994533</v>
+        <v>38.12888729688365</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1600,10 +1600,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>860504</v>
+        <v>859852</v>
       </c>
       <c r="L9" t="n">
-        <v>34.34080492362616</v>
+        <v>34.29101752394598</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1667,10 +1667,10 @@
         <v>582999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>860504</v>
+        <v>859852</v>
       </c>
       <c r="L10" t="n">
-        <v>32.24912376932588</v>
+        <v>32.19775031051855</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -1734,10 +1734,10 @@
         <v>587999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>860504</v>
+        <v>859852</v>
       </c>
       <c r="L11" t="n">
-        <v>31.66806894564116</v>
+        <v>31.61625489037648</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -1795,19 +1795,19 @@
         </is>
       </c>
       <c r="I12" s="3" t="n">
-        <v>643000</v>
+        <v>645000</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>643000</v>
+        <v>645000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>946597</v>
+        <v>945880</v>
       </c>
       <c r="L12" t="n">
-        <v>32.07246589625786</v>
+        <v>31.80953186450712</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="N12" t="n">
         <v>0</v>
@@ -1816,10 +1816,10 @@
         <v>100</v>
       </c>
       <c r="P12" t="n">
-        <v>72.00000000000001</v>
+        <v>71.48936170212767</v>
       </c>
       <c r="Q12" t="n">
-        <v>44.9</v>
+        <v>44.7</v>
       </c>
       <c r="R12" t="n">
         <v>4</v>
@@ -1927,10 +1927,10 @@
         <v>650000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>946597</v>
+        <v>945880</v>
       </c>
       <c r="L14" t="n">
-        <v>31.33297485624822</v>
+        <v>31.28092358438703</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -1994,10 +1994,10 @@
         <v>650000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>860504</v>
+        <v>859852</v>
       </c>
       <c r="L15" t="n">
-        <v>24.46287292098584</v>
+        <v>24.40559538153078</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0</v>
@@ -2058,10 +2058,10 @@
         <v>650000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>860504</v>
+        <v>859852</v>
       </c>
       <c r="L16" t="n">
-        <v>24.46287292098584</v>
+        <v>24.40559538153078</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -2122,10 +2122,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1032690</v>
+        <v>1031908</v>
       </c>
       <c r="L17" t="n">
-        <v>32.21586342464825</v>
+        <v>32.16449528446334</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2189,10 +2189,10 @@
         <v>707999</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>1075737</v>
+        <v>1074922</v>
       </c>
       <c r="L18" t="n">
-        <v>34.18474961816875</v>
+        <v>34.13484885414942</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -2256,10 +2256,10 @@
         <v>720000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>1032690</v>
+        <v>1031908</v>
       </c>
       <c r="L19" t="n">
-        <v>30.27917380820962</v>
+        <v>30.22633800687658</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -2447,10 +2447,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1075737</v>
+        <v>1074922</v>
       </c>
       <c r="L22" t="n">
-        <v>30.93107330137385</v>
+        <v>30.87870561770993</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2514,10 +2514,10 @@
         <v>772000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1032690</v>
+        <v>1031908</v>
       </c>
       <c r="L23" t="n">
-        <v>25.24378080546921</v>
+        <v>25.187129085151</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -2578,10 +2578,10 @@
         <v>772000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1032690</v>
+        <v>1031908</v>
       </c>
       <c r="L24" t="n">
-        <v>25.24378080546921</v>
+        <v>25.187129085151</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -2642,10 +2642,10 @@
         <v>772000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>1032690</v>
+        <v>1031908</v>
       </c>
       <c r="L25" t="n">
-        <v>25.24378080546921</v>
+        <v>25.187129085151</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -2768,10 +2768,10 @@
         <v>810000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>1247924</v>
+        <v>1246979</v>
       </c>
       <c r="L27" t="n">
-        <v>35.09220112763277</v>
+        <v>35.04301195128387</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -2897,10 +2897,10 @@
         <v>832999</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>1290971</v>
+        <v>1289993</v>
       </c>
       <c r="L29" t="n">
-        <v>35.47500292415554</v>
+        <v>35.42608370743097</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -2964,10 +2964,10 @@
         <v>835000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1075737</v>
+        <v>1074922</v>
       </c>
       <c r="L30" t="n">
-        <v>22.37879704797734</v>
+        <v>22.31994507508452</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -3028,10 +3028,10 @@
         <v>930000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1377064</v>
+        <v>1376021</v>
       </c>
       <c r="L31" t="n">
-        <v>38.41978295852626</v>
+        <v>38.37310622439629</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -3095,10 +3095,10 @@
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1377064</v>
+        <v>1376021</v>
       </c>
       <c r="L32" t="n">
-        <v>38.27454642630988</v>
+        <v>38.227759605413</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3162,10 +3162,10 @@
         <v>860000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1247924</v>
+        <v>1246979</v>
       </c>
       <c r="L33" t="n">
-        <v>31.08554687625208</v>
+        <v>31.03332133099274</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3291,10 +3291,10 @@
         <v>870000</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>1290971</v>
+        <v>1289993</v>
       </c>
       <c r="L35" t="n">
-        <v>32.60886572974916</v>
+        <v>32.55777356931394</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
@@ -3482,10 +3482,10 @@
         <v>890000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>1161831</v>
+        <v>1160951</v>
       </c>
       <c r="L38" t="n">
-        <v>23.3967762953476</v>
+        <v>23.33871110839303</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -3497,7 +3497,7 @@
         <v>73.86018237082067</v>
       </c>
       <c r="Q38" t="n">
-        <v>25.9</v>
+        <v>25.8</v>
       </c>
       <c r="R38" t="n">
         <v>3</v>
@@ -3546,10 +3546,10 @@
         <v>960000</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>1247924</v>
+        <v>1246979</v>
       </c>
       <c r="L39" t="n">
-        <v>23.07223837349069</v>
+        <v>23.0139400904105</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -3561,7 +3561,7 @@
         <v>82.97872340425533</v>
       </c>
       <c r="Q39" t="n">
-        <v>27.7</v>
+        <v>27.6</v>
       </c>
       <c r="R39" t="n">
         <v>3</v>
@@ -3610,10 +3610,10 @@
         <v>970000</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>1506204</v>
+        <v>1505063</v>
       </c>
       <c r="L40" t="n">
-        <v>35.59969300307262</v>
+        <v>35.55087062800693</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -3739,10 +3739,10 @@
         <v>1022000</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>1506204</v>
+        <v>1505063</v>
       </c>
       <c r="L42" t="n">
-        <v>32.14730541148477</v>
+        <v>32.0958657544568</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -3806,10 +3806,10 @@
         <v>1063000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1549251</v>
+        <v>1548077</v>
       </c>
       <c r="L43" t="n">
-        <v>31.38619887932943</v>
+        <v>31.33416490265019</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -3873,10 +3873,10 @@
         <v>1085000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1549251</v>
+        <v>1548077</v>
       </c>
       <c r="L44" t="n">
-        <v>29.9661578401434</v>
+        <v>29.91304696084239</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -4002,10 +4002,10 @@
         <v>1123000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1721438</v>
+        <v>1720134</v>
       </c>
       <c r="L46" t="n">
-        <v>34.76384278725113</v>
+        <v>34.7143885301959</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -4069,10 +4069,10 @@
         <v>1150000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1506204</v>
+        <v>1505063</v>
       </c>
       <c r="L47" t="n">
-        <v>23.64912057065311</v>
+        <v>23.59123837341028</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -4133,10 +4133,10 @@
         <v>1150000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1506204</v>
+        <v>1505063</v>
       </c>
       <c r="L48" t="n">
-        <v>23.64912057065311</v>
+        <v>23.59123837341028</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -4197,10 +4197,10 @@
         <v>1155000</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>1764484</v>
+        <v>1763148</v>
       </c>
       <c r="L49" t="n">
-        <v>34.5417697185126</v>
+        <v>34.49216968740004</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -4261,10 +4261,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1764484</v>
+        <v>1763148</v>
       </c>
       <c r="L50" t="n">
-        <v>34.5417697185126</v>
+        <v>34.49216968740004</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4387,10 +4387,10 @@
         <v>1208000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1893625</v>
+        <v>1892190</v>
       </c>
       <c r="L52" t="n">
-        <v>36.20701036372038</v>
+        <v>36.15863100428604</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -4454,10 +4454,10 @@
         <v>1210000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1592298</v>
+        <v>1591091</v>
       </c>
       <c r="L53" t="n">
-        <v>24.00919928304878</v>
+        <v>23.95155273959817</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -4518,10 +4518,10 @@
         <v>1210000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1893625</v>
+        <v>1892190</v>
       </c>
       <c r="L54" t="n">
-        <v>36.10139283120998</v>
+        <v>36.05293337349843</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -4536,7 +4536,7 @@
         <v>8.510415301978242</v>
       </c>
       <c r="Q54" t="n">
-        <v>13.5</v>
+        <v>13.4</v>
       </c>
       <c r="R54" t="n">
         <v>4</v>
@@ -4585,10 +4585,10 @@
         <v>1215000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1592298</v>
+        <v>1591091</v>
       </c>
       <c r="L55" t="n">
-        <v>23.69518770983823</v>
+        <v>23.6373029575304</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -4711,10 +4711,10 @@
         <v>1280000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1678391</v>
+        <v>1677120</v>
       </c>
       <c r="L57" t="n">
-        <v>23.73648333433628</v>
+        <v>23.6786872734211</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -4775,10 +4775,10 @@
         <v>1280000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>1721438</v>
+        <v>1720134</v>
       </c>
       <c r="L58" t="n">
-        <v>25.64356079045542</v>
+        <v>25.58719262569079</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -4842,10 +4842,10 @@
         <v>1310000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1721438</v>
+        <v>1720134</v>
       </c>
       <c r="L59" t="n">
-        <v>23.90083174648172</v>
+        <v>23.84314245285542</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -4906,10 +4906,10 @@
         <v>1338000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1764484</v>
+        <v>1763148</v>
       </c>
       <c r="L60" t="n">
-        <v>24.17046569988733</v>
+        <v>24.11300696254654</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -4970,10 +4970,10 @@
         <v>1370000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1807531</v>
+        <v>1806162</v>
       </c>
       <c r="L61" t="n">
-        <v>24.20600255265332</v>
+        <v>24.14855367348001</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -5093,10 +5093,10 @@
         <v>1425000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>2151905</v>
+        <v>2150275</v>
       </c>
       <c r="L63" t="n">
-        <v>33.77960458291606</v>
+        <v>33.7294067037937</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -5160,10 +5160,10 @@
         <v>1430000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>2151905</v>
+        <v>2150275</v>
       </c>
       <c r="L64" t="n">
-        <v>33.54725231829472</v>
+        <v>33.49687830626315</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -5227,10 +5227,10 @@
         <v>1471000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1936671</v>
+        <v>1935204</v>
       </c>
       <c r="L65" t="n">
-        <v>24.04492038141739</v>
+        <v>23.9873419029725</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -5291,10 +5291,10 @@
         <v>1471000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1936671</v>
+        <v>1935204</v>
       </c>
       <c r="L66" t="n">
-        <v>24.04492038141739</v>
+        <v>23.9873419029725</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -5417,10 +5417,10 @@
         <v>1535000</v>
       </c>
       <c r="K68" s="3" t="n">
-        <v>2022765</v>
+        <v>2021232</v>
       </c>
       <c r="L68" t="n">
-        <v>24.11377495655699</v>
+        <v>24.05621917721469</v>
       </c>
       <c r="M68" s="3" t="n">
         <v>0</v>
@@ -5543,10 +5543,10 @@
         <v>1650000</v>
       </c>
       <c r="K70" s="3" t="n">
-        <v>2194952</v>
+        <v>2193289</v>
       </c>
       <c r="L70" t="n">
-        <v>24.827513312364</v>
+        <v>24.77051587820848</v>
       </c>
       <c r="M70" s="3" t="n">
         <v>0</v>
@@ -5607,10 +5607,10 @@
         <v>1660000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2194952</v>
+        <v>2193289</v>
       </c>
       <c r="L71" t="n">
-        <v>24.37192248395409</v>
+        <v>24.31457961080368</v>
       </c>
       <c r="M71" s="3" t="n">
         <v>0</v>
@@ -5622,7 +5622,7 @@
         <v>26.6373948042444</v>
       </c>
       <c r="Q71" t="n">
-        <v>16.2</v>
+        <v>16.1</v>
       </c>
       <c r="R71" t="n">
         <v>3</v>
@@ -5671,10 +5671,10 @@
         <v>1661000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2194952</v>
+        <v>2193289</v>
       </c>
       <c r="L72" t="n">
-        <v>24.3263634011131</v>
+        <v>24.2689859840632</v>
       </c>
       <c r="M72" s="3" t="n">
         <v>0</v>
@@ -5735,10 +5735,10 @@
         <v>1680000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2237998</v>
+        <v>2236303</v>
       </c>
       <c r="L73" t="n">
-        <v>24.93290878722859</v>
+        <v>24.87601188211079</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
@@ -5799,10 +5799,10 @@
         <v>1711000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2324092</v>
+        <v>2322331</v>
       </c>
       <c r="L74" t="n">
-        <v>26.37985071158973</v>
+        <v>26.32402530044167</v>
       </c>
       <c r="M74" s="3" t="n">
         <v>0</v>
@@ -5863,10 +5863,10 @@
         <v>1756000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2324092</v>
+        <v>2322331</v>
       </c>
       <c r="L75" t="n">
-        <v>24.44361066601494</v>
+        <v>24.38631702371454</v>
       </c>
       <c r="M75" s="3" t="n">
         <v>0</v>
@@ -5927,10 +5927,10 @@
         <v>1790000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2367138</v>
+        <v>2365345</v>
       </c>
       <c r="L76" t="n">
-        <v>24.38125702852981</v>
+        <v>24.32393583177084</v>
       </c>
       <c r="M76" s="3" t="n">
         <v>0</v>
@@ -5991,10 +5991,10 @@
         <v>1840000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2453232</v>
+        <v>2451373</v>
       </c>
       <c r="L77" t="n">
-        <v>24.99690204595407</v>
+        <v>24.94002340729052</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
@@ -6055,10 +6055,10 @@
         <v>1945000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2582372</v>
+        <v>2580416</v>
       </c>
       <c r="L78" t="n">
-        <v>24.68164927438804</v>
+        <v>24.62455666063146</v>
       </c>
       <c r="M78" s="3" t="n">
         <v>0</v>
@@ -6070,7 +6070,7 @@
         <v>15.83200763601658</v>
       </c>
       <c r="Q78" t="n">
-        <v>14</v>
+        <v>13.9</v>
       </c>
       <c r="R78" t="n">
         <v>3</v>
@@ -6119,10 +6119,10 @@
         <v>1960000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2625419</v>
+        <v>2623430</v>
       </c>
       <c r="L79" t="n">
-        <v>25.34524965348388</v>
+        <v>25.28864882996687</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
@@ -6183,10 +6183,10 @@
         <v>2078000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2754559</v>
+        <v>2752472</v>
       </c>
       <c r="L80" t="n">
-        <v>24.5614270741705</v>
+        <v>24.50422747261371</v>
       </c>
       <c r="M80" s="3" t="n">
         <v>0</v>
@@ -6198,7 +6198,7 @@
         <v>35.18930957683743</v>
       </c>
       <c r="Q80" t="n">
-        <v>18.1</v>
+        <v>18</v>
       </c>
       <c r="R80" t="n">
         <v>3</v>
@@ -6247,10 +6247,10 @@
         <v>2170000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2883699</v>
+        <v>2881514</v>
       </c>
       <c r="L81" t="n">
-        <v>24.74942773153509</v>
+        <v>24.69236658228973</v>
       </c>
       <c r="M81" s="3" t="n">
         <v>0</v>
@@ -6311,10 +6311,10 @@
         <v>2268000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>3012839</v>
+        <v>3010557</v>
       </c>
       <c r="L82" t="n">
-        <v>24.72216404527424</v>
+        <v>24.66510350078075</v>
       </c>
       <c r="M82" s="3" t="n">
         <v>0</v>
@@ -6375,10 +6375,10 @@
         <v>2270000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3055886</v>
+        <v>3053571</v>
       </c>
       <c r="L83" t="n">
-        <v>25.71712426445227</v>
+        <v>25.66080827987953</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
@@ -6439,10 +6439,10 @@
         <v>2381000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3185026</v>
+        <v>3182613</v>
       </c>
       <c r="L84" t="n">
-        <v>25.24393835403542</v>
+        <v>25.18725965111058</v>
       </c>
       <c r="M84" s="3" t="n">
         <v>0</v>
@@ -6503,10 +6503,10 @@
         <v>2470000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3314166</v>
+        <v>3311655</v>
       </c>
       <c r="L85" t="n">
-        <v>25.47144590826169</v>
+        <v>25.41493603651346</v>
       </c>
       <c r="M85" s="3" t="n">
         <v>0</v>
@@ -6518,7 +6518,7 @@
         <v>88.84010245151846</v>
       </c>
       <c r="Q85" t="n">
-        <v>30</v>
+        <v>29.9</v>
       </c>
       <c r="R85" t="n">
         <v>3</v>
@@ -6567,10 +6567,10 @@
         <v>2480000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3314166</v>
+        <v>3311655</v>
       </c>
       <c r="L86" t="n">
-        <v>25.16971087145303</v>
+        <v>25.11297221479894</v>
       </c>
       <c r="M86" s="3" t="n">
         <v>0</v>
@@ -6631,10 +6631,10 @@
         <v>2571000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3443306</v>
+        <v>3440698</v>
       </c>
       <c r="L87" t="n">
-        <v>25.33338599590045</v>
+        <v>25.27678976765761</v>
       </c>
       <c r="M87" s="3" t="n">
         <v>0</v>
@@ -6695,10 +6695,10 @@
         <v>2580000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3486353</v>
+        <v>3483712</v>
       </c>
       <c r="L88" t="n">
-        <v>25.99716666671447</v>
+        <v>25.94106516267705</v>
       </c>
       <c r="M88" s="3" t="n">
         <v>0</v>
@@ -6710,7 +6710,7 @@
         <v>80.79034028540066</v>
       </c>
       <c r="Q88" t="n">
-        <v>28.5</v>
+        <v>28.4</v>
       </c>
       <c r="R88" t="n">
         <v>3</v>
@@ -6759,10 +6759,10 @@
         <v>2581000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3443306</v>
+        <v>3440698</v>
       </c>
       <c r="L89" t="n">
-        <v>25.04296742723417</v>
+        <v>24.98615106585931</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
@@ -6823,10 +6823,10 @@
         <v>2664000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3615493</v>
+        <v>3612754</v>
       </c>
       <c r="L90" t="n">
-        <v>26.31710253622397</v>
+        <v>26.26124004014666</v>
       </c>
       <c r="M90" s="3" t="n">
         <v>0</v>
@@ -6838,7 +6838,7 @@
         <v>75.54565701559021</v>
       </c>
       <c r="Q90" t="n">
-        <v>27.5</v>
+        <v>27.4</v>
       </c>
       <c r="R90" t="n">
         <v>3</v>
@@ -6887,10 +6887,10 @@
         <v>3090000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>4175100</v>
+        <v>4171937</v>
       </c>
       <c r="L91" t="n">
-        <v>25.98979665157721</v>
+        <v>25.93368500051655</v>
       </c>
       <c r="M91" s="3" t="n">
         <v>0</v>
@@ -6902,7 +6902,7 @@
         <v>100</v>
       </c>
       <c r="Q91" t="n">
-        <v>32.6</v>
+        <v>32.5</v>
       </c>
       <c r="R91" t="n">
         <v>3</v>
@@ -6951,10 +6951,10 @@
         <v>3186000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4304240</v>
+        <v>4300980</v>
       </c>
       <c r="L92" t="n">
-        <v>25.97996394253109</v>
+        <v>25.92385921348158</v>
       </c>
       <c r="M92" s="3" t="n">
         <v>0</v>
@@ -6966,7 +6966,7 @@
         <v>100</v>
       </c>
       <c r="Q92" t="n">
-        <v>32.6</v>
+        <v>32.5</v>
       </c>
       <c r="R92" t="n">
         <v>3</v>
@@ -7249,10 +7249,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>430037</v>
+        <v>429711</v>
       </c>
       <c r="L2" t="n">
-        <v>27.91341210174939</v>
+        <v>27.85872365380454</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7316,10 +7316,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>430037</v>
+        <v>429711</v>
       </c>
       <c r="L3" t="n">
-        <v>27.91341210174939</v>
+        <v>27.85872365380454</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7383,10 +7383,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>430037</v>
+        <v>429711</v>
       </c>
       <c r="L4" t="n">
-        <v>27.91317956361895</v>
+        <v>27.85849093925918</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7401,7 +7401,7 @@
         <v>29.71428571428569</v>
       </c>
       <c r="Q4" t="n">
-        <v>14.3</v>
+        <v>14.2</v>
       </c>
       <c r="R4" t="n">
         <v>4</v>
@@ -7450,10 +7450,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>430037</v>
+        <v>429711</v>
       </c>
       <c r="L5" t="n">
-        <v>27.91317956361895</v>
+        <v>27.85849093925918</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7468,7 +7468,7 @@
         <v>29.71428571428569</v>
       </c>
       <c r="Q5" t="n">
-        <v>14.3</v>
+        <v>14.2</v>
       </c>
       <c r="R5" t="n">
         <v>4</v>
@@ -7517,10 +7517,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>516130</v>
+        <v>515739</v>
       </c>
       <c r="L6" t="n">
-        <v>25.60013949973844</v>
+        <v>25.54373433073706</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7532,7 +7532,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>11</v>
+        <v>10.9</v>
       </c>
       <c r="R6" t="n">
         <v>3</v>
@@ -7581,10 +7581,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>516130</v>
+        <v>515739</v>
       </c>
       <c r="L7" t="n">
-        <v>25.60013949973844</v>
+        <v>25.54373433073706</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7596,7 +7596,7 @@
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>11</v>
+        <v>10.9</v>
       </c>
       <c r="R7" t="n">
         <v>3</v>
@@ -7645,10 +7645,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>516130</v>
+        <v>515739</v>
       </c>
       <c r="L8" t="n">
-        <v>25.60013949973844</v>
+        <v>25.54373433073706</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7660,7 +7660,7 @@
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>11</v>
+        <v>10.9</v>
       </c>
       <c r="R8" t="n">
         <v>3</v>
@@ -7709,10 +7709,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>516130</v>
+        <v>515739</v>
       </c>
       <c r="L9" t="n">
-        <v>25.60013949973844</v>
+        <v>25.54373433073706</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7724,7 +7724,7 @@
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>11</v>
+        <v>10.9</v>
       </c>
       <c r="R9" t="n">
         <v>3</v>
@@ -7773,10 +7773,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>516130</v>
+        <v>515739</v>
       </c>
       <c r="L10" t="n">
-        <v>25.40638986301901</v>
+        <v>25.34983780555669</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7837,10 +7837,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>516130</v>
+        <v>515739</v>
       </c>
       <c r="L11" t="n">
-        <v>25.40638986301901</v>
+        <v>25.34983780555669</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7901,10 +7901,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>516130</v>
+        <v>515739</v>
       </c>
       <c r="L12" t="n">
-        <v>25.40638986301901</v>
+        <v>25.34983780555669</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -7965,10 +7965,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>516130</v>
+        <v>515739</v>
       </c>
       <c r="L13" t="n">
-        <v>25.40638986301901</v>
+        <v>25.34983780555669</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -8029,10 +8029,10 @@
         <v>430000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>559177</v>
+        <v>558753</v>
       </c>
       <c r="L14" t="n">
-        <v>23.10127204802773</v>
+        <v>23.04291878522352</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -8090,31 +8090,31 @@
         </is>
       </c>
       <c r="I15" s="3" t="n">
-        <v>432999</v>
+        <v>434999</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>432999</v>
+        <v>434999</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>559177</v>
+        <v>558753</v>
       </c>
       <c r="L15" t="n">
-        <v>22.56494812912548</v>
+        <v>22.14824797361267</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="N15" t="n">
         <v>0</v>
       </c>
       <c r="O15" t="n">
-        <v>86.96086956521739</v>
+        <v>78.26521739130435</v>
       </c>
       <c r="P15" t="n">
-        <v>11.31598302687412</v>
+        <v>10.184441301273</v>
       </c>
       <c r="Q15" t="n">
-        <v>28.7</v>
+        <v>26.5</v>
       </c>
       <c r="R15" t="n">
         <v>4</v>
@@ -8157,31 +8157,31 @@
         </is>
       </c>
       <c r="I16" s="3" t="n">
-        <v>447999</v>
+        <v>441999</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>447999</v>
+        <v>441999</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>559177</v>
+        <v>558753</v>
       </c>
       <c r="L16" t="n">
-        <v>19.88243436335901</v>
+        <v>20.89545827941863</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0</v>
+        <v>-6000</v>
       </c>
       <c r="N16" t="n">
-        <v>0</v>
+        <v>1.339288703769428</v>
       </c>
       <c r="O16" t="n">
-        <v>21.74347826086957</v>
+        <v>47.83043478260869</v>
       </c>
       <c r="P16" t="n">
-        <v>2.829420084865629</v>
+        <v>6.224045261669024</v>
       </c>
       <c r="Q16" t="n">
-        <v>11.9</v>
+        <v>19</v>
       </c>
       <c r="R16" t="n">
         <v>4</v>
@@ -8230,10 +8230,10 @@
         <v>447999</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>559177</v>
+        <v>558753</v>
       </c>
       <c r="L17" t="n">
-        <v>19.88243436335901</v>
+        <v>19.82163854153803</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -8297,10 +8297,10 @@
         <v>453000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>559177</v>
+        <v>558753</v>
       </c>
       <c r="L18" t="n">
-        <v>18.98808427385246</v>
+        <v>18.92660979001455</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -8364,10 +8364,10 @@
         <v>454000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>602223</v>
+        <v>601767</v>
       </c>
       <c r="L19" t="n">
-        <v>24.61264348920583</v>
+        <v>24.5555173347824</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -8428,10 +8428,10 @@
         <v>454000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>602223</v>
+        <v>601767</v>
       </c>
       <c r="L20" t="n">
-        <v>24.61264348920583</v>
+        <v>24.5555173347824</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -8492,10 +8492,10 @@
         <v>454000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>602223</v>
+        <v>601767</v>
       </c>
       <c r="L21" t="n">
-        <v>24.61264348920583</v>
+        <v>24.5555173347824</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -8556,10 +8556,10 @@
         <v>454000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>602223</v>
+        <v>601767</v>
       </c>
       <c r="L22" t="n">
-        <v>24.61264348920583</v>
+        <v>24.5555173347824</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -8620,10 +8620,10 @@
         <v>455000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>602223</v>
+        <v>601767</v>
       </c>
       <c r="L23" t="n">
-        <v>24.44659204314681</v>
+        <v>24.38934006018941</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -8684,10 +8684,10 @@
         <v>455000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>602223</v>
+        <v>601767</v>
       </c>
       <c r="L24" t="n">
-        <v>24.44659204314681</v>
+        <v>24.38934006018941</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -8748,10 +8748,10 @@
         <v>455000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>602223</v>
+        <v>601767</v>
       </c>
       <c r="L25" t="n">
-        <v>24.44659204314681</v>
+        <v>24.38934006018941</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -8812,10 +8812,10 @@
         <v>455000</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>602223</v>
+        <v>601767</v>
       </c>
       <c r="L26" t="n">
-        <v>24.44659204314681</v>
+        <v>24.38934006018941</v>
       </c>
       <c r="M26" s="3" t="n">
         <v>0</v>
@@ -8876,10 +8876,10 @@
         <v>475000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>688317</v>
+        <v>687795</v>
       </c>
       <c r="L27" t="n">
-        <v>30.99109857812607</v>
+        <v>30.93872447458909</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -8940,10 +8940,10 @@
         <v>475000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>688317</v>
+        <v>687795</v>
       </c>
       <c r="L28" t="n">
-        <v>30.99109857812607</v>
+        <v>30.93872447458909</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -9004,10 +9004,10 @@
         <v>475000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>688317</v>
+        <v>687795</v>
       </c>
       <c r="L29" t="n">
-        <v>30.99109857812607</v>
+        <v>30.93872447458909</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -9068,10 +9068,10 @@
         <v>475000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>688317</v>
+        <v>687795</v>
       </c>
       <c r="L30" t="n">
-        <v>30.99109857812607</v>
+        <v>30.93872447458909</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -9132,10 +9132,10 @@
         <v>479999</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>688317</v>
+        <v>687795</v>
       </c>
       <c r="L31" t="n">
-        <v>30.26483437137249</v>
+        <v>30.21190907174376</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -9196,10 +9196,10 @@
         <v>479999</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>688317</v>
+        <v>687795</v>
       </c>
       <c r="L32" t="n">
-        <v>30.26483437137249</v>
+        <v>30.21190907174376</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -9260,10 +9260,10 @@
         <v>479999</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>688317</v>
+        <v>687795</v>
       </c>
       <c r="L33" t="n">
-        <v>30.26483437137249</v>
+        <v>30.21190907174376</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -9324,10 +9324,10 @@
         <v>479999</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>688317</v>
+        <v>687795</v>
       </c>
       <c r="L34" t="n">
-        <v>30.26483437137249</v>
+        <v>30.21190907174376</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -9388,10 +9388,10 @@
         <v>482999</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>645270</v>
+        <v>644781</v>
       </c>
       <c r="L35" t="n">
-        <v>25.14776760115921</v>
+        <v>25.09099988988509</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
@@ -9455,10 +9455,10 @@
         <v>482999</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>645270</v>
+        <v>644781</v>
       </c>
       <c r="L36" t="n">
-        <v>25.14776760115921</v>
+        <v>25.09099988988509</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -9522,10 +9522,10 @@
         <v>482999</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>645270</v>
+        <v>644781</v>
       </c>
       <c r="L37" t="n">
-        <v>25.14776760115921</v>
+        <v>25.09099988988509</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
@@ -9589,10 +9589,10 @@
         <v>495000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>645270</v>
+        <v>644781</v>
       </c>
       <c r="L38" t="n">
-        <v>23.28792598447162</v>
+        <v>23.22974777482587</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -9607,7 +9607,7 @@
         <v>0</v>
       </c>
       <c r="Q38" t="n">
-        <v>7.8</v>
+        <v>7.7</v>
       </c>
       <c r="R38" t="n">
         <v>4</v>
@@ -9656,10 +9656,10 @@
         <v>500000</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>645270</v>
+        <v>644781</v>
       </c>
       <c r="L39" t="n">
-        <v>22.51305654997133</v>
+        <v>22.45429068164229</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -9720,10 +9720,10 @@
         <v>551999</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>774410</v>
+        <v>773824</v>
       </c>
       <c r="L40" t="n">
-        <v>28.72005785049263</v>
+        <v>28.66607910842776</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -9787,10 +9787,10 @@
         <v>551999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>774410</v>
+        <v>773824</v>
       </c>
       <c r="L41" t="n">
-        <v>28.72005785049263</v>
+        <v>28.66607910842776</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
@@ -9854,10 +9854,10 @@
         <v>551999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>774410</v>
+        <v>773824</v>
       </c>
       <c r="L42" t="n">
-        <v>28.72005785049263</v>
+        <v>28.66607910842776</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -9921,10 +9921,10 @@
         <v>557999</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>774410</v>
+        <v>773824</v>
       </c>
       <c r="L43" t="n">
-        <v>27.9452744670136</v>
+        <v>27.89070899842858</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -9939,7 +9939,7 @@
         <v>66.87445544554454</v>
       </c>
       <c r="Q43" t="n">
-        <v>20.5</v>
+        <v>20.4</v>
       </c>
       <c r="R43" t="n">
         <v>4</v>
@@ -9988,10 +9988,10 @@
         <v>564999</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>774410</v>
+        <v>773824</v>
       </c>
       <c r="L44" t="n">
-        <v>27.04136051962139</v>
+        <v>26.98611053676288</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -10052,10 +10052,10 @@
         <v>564999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>774410</v>
+        <v>773824</v>
       </c>
       <c r="L45" t="n">
-        <v>27.04136051962139</v>
+        <v>26.98611053676288</v>
       </c>
       <c r="M45" s="3" t="n">
         <v>0</v>
@@ -10116,10 +10116,10 @@
         <v>564999</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>774410</v>
+        <v>773824</v>
       </c>
       <c r="L46" t="n">
-        <v>27.04136051962139</v>
+        <v>26.98611053676288</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -10180,10 +10180,10 @@
         <v>564999</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>774410</v>
+        <v>773824</v>
       </c>
       <c r="L47" t="n">
-        <v>27.04136051962139</v>
+        <v>26.98611053676288</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -10244,10 +10244,10 @@
         <v>585000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>731364</v>
+        <v>730810</v>
       </c>
       <c r="L48" t="n">
-        <v>20.01246985085402</v>
+        <v>19.95183426608832</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -10308,10 +10308,10 @@
         <v>595000</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>731364</v>
+        <v>730810</v>
       </c>
       <c r="L49" t="n">
-        <v>18.64516164317631</v>
+        <v>18.58348955268811</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -10372,10 +10372,10 @@
         <v>614999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>860504</v>
+        <v>859852</v>
       </c>
       <c r="L50" t="n">
-        <v>28.53037289774365</v>
+        <v>28.4761796216093</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -10439,10 +10439,10 @@
         <v>616999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>860504</v>
+        <v>859852</v>
       </c>
       <c r="L51" t="n">
-        <v>28.29795096826976</v>
+        <v>28.24358145355247</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -10506,10 +10506,10 @@
         <v>616999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>860504</v>
+        <v>859852</v>
       </c>
       <c r="L52" t="n">
-        <v>28.29795096826976</v>
+        <v>28.24358145355247</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -10573,10 +10573,10 @@
         <v>616999</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>860504</v>
+        <v>859852</v>
       </c>
       <c r="L53" t="n">
-        <v>28.29795096826976</v>
+        <v>28.24358145355247</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -10640,10 +10640,10 @@
         <v>650000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>817457</v>
+        <v>816838</v>
       </c>
       <c r="L54" t="n">
-        <v>20.4851142017256</v>
+        <v>20.42485780534206</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -10704,10 +10704,10 @@
         <v>672000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>860504</v>
+        <v>859852</v>
       </c>
       <c r="L55" t="n">
-        <v>21.90623169677306</v>
+        <v>21.84701553290566</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -10719,7 +10719,7 @@
         <v>66.19519094766619</v>
       </c>
       <c r="Q55" t="n">
-        <v>23.6</v>
+        <v>23.5</v>
       </c>
       <c r="R55" t="n">
         <v>3</v>
@@ -10768,10 +10768,10 @@
         <v>700000</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>903550</v>
+        <v>902866</v>
       </c>
       <c r="L56" t="n">
-        <v>22.52780698356483</v>
+        <v>22.46911501817545</v>
       </c>
       <c r="M56" s="3" t="n">
         <v>0</v>
@@ -10832,10 +10832,10 @@
         <v>715000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>946597</v>
+        <v>945880</v>
       </c>
       <c r="L57" t="n">
-        <v>24.46627234187305</v>
+        <v>24.40901594282573</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -10847,7 +10847,7 @@
         <v>66.66666666666666</v>
       </c>
       <c r="Q57" t="n">
-        <v>24.8</v>
+        <v>24.7</v>
       </c>
       <c r="R57" t="n">
         <v>3</v>
@@ -10896,10 +10896,10 @@
         <v>752000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>989644</v>
+        <v>988894</v>
       </c>
       <c r="L58" t="n">
-        <v>24.01307945079241</v>
+        <v>23.95544921902651</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -10911,7 +10911,7 @@
         <v>57.6969696969697</v>
       </c>
       <c r="Q58" t="n">
-        <v>22.7</v>
+        <v>22.6</v>
       </c>
       <c r="R58" t="n">
         <v>3</v>
@@ -10960,10 +10960,10 @@
         <v>756000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>989644</v>
+        <v>988894</v>
       </c>
       <c r="L59" t="n">
-        <v>23.60889370319024</v>
+        <v>23.55095692763835</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -10975,7 +10975,7 @@
         <v>72.98444130127297</v>
       </c>
       <c r="Q59" t="n">
-        <v>25.8</v>
+        <v>25.7</v>
       </c>
       <c r="R59" t="n">
         <v>3</v>
@@ -11024,10 +11024,10 @@
         <v>810000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1075737</v>
+        <v>1074922</v>
       </c>
       <c r="L60" t="n">
-        <v>24.70278516031335</v>
+        <v>24.64569522253708</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -11088,10 +11088,10 @@
         <v>815000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1075737</v>
+        <v>1074922</v>
       </c>
       <c r="L61" t="n">
-        <v>24.23798753784614</v>
+        <v>24.18054519304657</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -11103,7 +11103,7 @@
         <v>83.38048090523338</v>
       </c>
       <c r="Q61" t="n">
-        <v>28.3</v>
+        <v>28.2</v>
       </c>
       <c r="R61" t="n">
         <v>3</v>
@@ -11152,10 +11152,10 @@
         <v>875000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1161831</v>
+        <v>1160951</v>
       </c>
       <c r="L62" t="n">
-        <v>24.68784186340354</v>
+        <v>24.6307553031954</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -11216,10 +11216,10 @@
         <v>992000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1334017</v>
+        <v>1333007</v>
       </c>
       <c r="L63" t="n">
-        <v>25.63812904932995</v>
+        <v>25.58178614215829</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -11280,10 +11280,10 @@
         <v>1050000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1420111</v>
+        <v>1419035</v>
       </c>
       <c r="L64" t="n">
-        <v>26.0621176795335</v>
+        <v>26.00605340953535</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -11295,7 +11295,7 @@
         <v>94.27799922849427</v>
       </c>
       <c r="Q64" t="n">
-        <v>31.4</v>
+        <v>31.3</v>
       </c>
       <c r="R64" t="n">
         <v>3</v>
@@ -11344,10 +11344,10 @@
         <v>1050000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1420111</v>
+        <v>1419035</v>
       </c>
       <c r="L65" t="n">
-        <v>26.0621176795335</v>
+        <v>26.00605340953535</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -11359,7 +11359,7 @@
         <v>87.27272727272727</v>
       </c>
       <c r="Q65" t="n">
-        <v>29.9</v>
+        <v>29.8</v>
       </c>
       <c r="R65" t="n">
         <v>3</v>
@@ -11408,10 +11408,10 @@
         <v>1100000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1506204</v>
+        <v>1505063</v>
       </c>
       <c r="L66" t="n">
-        <v>26.96872402410298</v>
+        <v>26.91335844413157</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -11472,10 +11472,10 @@
         <v>1105000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1506204</v>
+        <v>1505063</v>
       </c>
       <c r="L67" t="n">
-        <v>26.63676367875799</v>
+        <v>26.58114643705945</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -11536,10 +11536,10 @@
         <v>1155000</v>
       </c>
       <c r="K68" s="3" t="n">
-        <v>1592298</v>
+        <v>1591091</v>
       </c>
       <c r="L68" t="n">
-        <v>27.46332658836474</v>
+        <v>27.40830034234371</v>
       </c>
       <c r="M68" s="3" t="n">
         <v>0</v>
@@ -11807,7 +11807,7 @@
         <v>315000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>300896</v>
+        <v>300669</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -11868,10 +11868,10 @@
         <v>380000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>386990</v>
+        <v>386697</v>
       </c>
       <c r="L3" t="n">
-        <v>1.806248223468307</v>
+        <v>1.731846898217468</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -11932,7 +11932,7 @@
         <v>415000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>386990</v>
+        <v>386697</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -11993,10 +11993,10 @@
         <v>495000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>473083</v>
+        <v>472725</v>
       </c>
       <c r="L5" t="n">
-        <v>6.993276021332409</v>
+        <v>6.922840975196996</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -12057,10 +12057,10 @@
         <v>500000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>516130</v>
+        <v>515739</v>
       </c>
       <c r="L6" t="n">
-        <v>8.937670741867359</v>
+        <v>8.868633165225045</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -12121,10 +12121,10 @@
         <v>550000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>559177</v>
+        <v>558753</v>
       </c>
       <c r="L7" t="n">
-        <v>7.006189453428878</v>
+        <v>6.935622717014494</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -12185,7 +12185,7 @@
         <v>530000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>473083</v>
+        <v>472725</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -12249,10 +12249,10 @@
         <v>600000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>602223</v>
+        <v>601767</v>
       </c>
       <c r="L9" t="n">
-        <v>8.671704667540098</v>
+        <v>8.602498973855329</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -12264,7 +12264,7 @@
         <v>20.65076182537716</v>
       </c>
       <c r="Q9" t="n">
-        <v>8.199999999999999</v>
+        <v>8.1</v>
       </c>
       <c r="R9" t="n">
         <v>4</v>
@@ -12313,10 +12313,10 @@
         <v>646000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>731364</v>
+        <v>730810</v>
       </c>
       <c r="L10" t="n">
-        <v>17.27799016631937</v>
+        <v>17.21528167375925</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -12377,7 +12377,7 @@
         <v>615000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>559177</v>
+        <v>558753</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -12441,7 +12441,7 @@
         <v>700000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>645270</v>
+        <v>644781</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -12505,7 +12505,7 @@
         <v>745000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>688317</v>
+        <v>687795</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -12569,7 +12569,7 @@
         <v>930000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>860504</v>
+        <v>859852</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -12640,7 +12640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12686,8 +12686,88 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 13 MDHE4 M5 10C CPU 8C GPU 16GB 512GB Midnight</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>447999</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>441999</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>-6000</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-1.34</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Macbook Pro 14 M5 MDE34 10 Core CPU 10 Core GPU 24GB 1TB Space Black</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>643000</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>645000</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 13 MDHH4 M5 10C CPU 8C GPU 16GB 512GB Sky Blue</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>432999</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>434999</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.46</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F1"/>
+  <autoFilter ref="A1:F4"/>
+  <conditionalFormatting sqref="E2:E4">
+    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: price data 2026-09-18
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20260917T084356123359+0000</t>
+          <t>20260918T081854429215+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-17T08:43:56.123359+00:00</t>
+          <t>2026-09-18T08:18:54.429215+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>277.510311</v>
+        <v>277.281209</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -750,7 +750,7 @@
         <v>1123000</v>
       </c>
       <c r="D23" t="n">
-        <v>50.5</v>
+        <v>50.4</v>
       </c>
       <c r="E23" t="n">
         <v>4</v>
@@ -885,19 +885,19 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHG4 M5 10C CPU 10C GPU 24GB 1TB Midnight</t>
+          <t>Apple MacBook Pro 16Inch MX303 14Core CPU 32Core GPU M4 Max 36GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>macbook_air</t>
+          <t>macbook_pro</t>
         </is>
       </c>
       <c r="C30" s="3" t="n">
-        <v>551999</v>
+        <v>970000</v>
       </c>
       <c r="D30" t="n">
-        <v>43.3</v>
+        <v>43.2</v>
       </c>
       <c r="E30" t="n">
         <v>4</v>
@@ -906,7 +906,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHK4 M5 10C CPU 10C GPU 24GB 1TB Sky Blue</t>
+          <t>Apple MacBook Air 13 MDHG4 M5 10C CPU 10C GPU 24GB 1TB Midnight</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -918,7 +918,7 @@
         <v>551999</v>
       </c>
       <c r="D31" t="n">
-        <v>43.3</v>
+        <v>43.2</v>
       </c>
       <c r="E31" t="n">
         <v>4</v>
@@ -1147,10 +1147,10 @@
         <v>470000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>687795</v>
+        <v>687228</v>
       </c>
       <c r="L2" t="n">
-        <v>35.30048924461504</v>
+        <v>35.24710867426822</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1214,10 +1214,10 @@
         <v>465000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>687795</v>
+        <v>687228</v>
       </c>
       <c r="L3" t="n">
-        <v>33.41039117760379</v>
+        <v>33.35545117486482</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>773824</v>
+        <v>773185</v>
       </c>
       <c r="L4" t="n">
-        <v>35.38595339508726</v>
+        <v>35.33255301124569</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>773824</v>
+        <v>773185</v>
       </c>
       <c r="L5" t="n">
-        <v>32.80138636175668</v>
+        <v>32.74584995828941</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>859852</v>
+        <v>859142</v>
       </c>
       <c r="L6" t="n">
-        <v>38.12888729688365</v>
+        <v>38.07775664558362</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1600,10 +1600,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>859852</v>
+        <v>859142</v>
       </c>
       <c r="L9" t="n">
-        <v>34.29101752394598</v>
+        <v>34.2367152345014</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1667,10 +1667,10 @@
         <v>582999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>859852</v>
+        <v>859142</v>
       </c>
       <c r="L10" t="n">
-        <v>32.19775031051855</v>
+        <v>32.14171813274174</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -1734,10 +1734,10 @@
         <v>587999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>859852</v>
+        <v>859142</v>
       </c>
       <c r="L11" t="n">
-        <v>31.61625489037648</v>
+        <v>31.55974216136564</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -1801,13 +1801,13 @@
         <v>645000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>945880</v>
+        <v>945099</v>
       </c>
       <c r="L12" t="n">
-        <v>31.80953186450712</v>
+        <v>31.75318141274089</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="N12" t="n">
         <v>0</v>
@@ -1927,10 +1927,10 @@
         <v>650000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>945880</v>
+        <v>945099</v>
       </c>
       <c r="L14" t="n">
-        <v>31.28092358438703</v>
+        <v>31.2241363074133</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -1994,10 +1994,10 @@
         <v>650000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>859852</v>
+        <v>859142</v>
       </c>
       <c r="L15" t="n">
-        <v>24.40559538153078</v>
+        <v>24.3431237211078</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0</v>
@@ -2009,7 +2009,7 @@
         <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>10.5</v>
+        <v>10.4</v>
       </c>
       <c r="R15" t="n">
         <v>3</v>
@@ -2058,10 +2058,10 @@
         <v>650000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>859852</v>
+        <v>859142</v>
       </c>
       <c r="L16" t="n">
-        <v>24.40559538153078</v>
+        <v>24.3431237211078</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -2073,7 +2073,7 @@
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>10.5</v>
+        <v>10.4</v>
       </c>
       <c r="R16" t="n">
         <v>3</v>
@@ -2122,10 +2122,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1031908</v>
+        <v>1031056</v>
       </c>
       <c r="L17" t="n">
-        <v>32.16449528446334</v>
+        <v>32.10844027870456</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2189,10 +2189,10 @@
         <v>707999</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>1074922</v>
+        <v>1074035</v>
       </c>
       <c r="L18" t="n">
-        <v>34.13484885414942</v>
+        <v>34.08045361650225</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -2256,10 +2256,10 @@
         <v>720000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>1031908</v>
+        <v>1031056</v>
       </c>
       <c r="L19" t="n">
-        <v>30.22633800687658</v>
+        <v>30.16868142952468</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -2447,10 +2447,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1074922</v>
+        <v>1074035</v>
       </c>
       <c r="L22" t="n">
-        <v>30.87870561770993</v>
+        <v>30.82162126932549</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2514,10 +2514,10 @@
         <v>772000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1031908</v>
+        <v>1031056</v>
       </c>
       <c r="L23" t="n">
-        <v>25.187129085151</v>
+        <v>25.12530842165702</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -2578,10 +2578,10 @@
         <v>772000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1031908</v>
+        <v>1031056</v>
       </c>
       <c r="L24" t="n">
-        <v>25.187129085151</v>
+        <v>25.12530842165702</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -2642,10 +2642,10 @@
         <v>772000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>1031908</v>
+        <v>1031056</v>
       </c>
       <c r="L25" t="n">
-        <v>25.187129085151</v>
+        <v>25.12530842165702</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -2768,10 +2768,10 @@
         <v>810000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>1246979</v>
+        <v>1245949</v>
       </c>
       <c r="L27" t="n">
-        <v>35.04301195128387</v>
+        <v>34.98931336675899</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -2897,10 +2897,10 @@
         <v>832999</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>1289993</v>
+        <v>1288928</v>
       </c>
       <c r="L29" t="n">
-        <v>35.42608370743097</v>
+        <v>35.37272834479506</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -2964,10 +2964,10 @@
         <v>835000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1074922</v>
+        <v>1074035</v>
       </c>
       <c r="L30" t="n">
-        <v>22.31994507508452</v>
+        <v>22.25579240899971</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -3028,10 +3028,10 @@
         <v>930000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1376021</v>
+        <v>1374885</v>
       </c>
       <c r="L31" t="n">
-        <v>38.37310622439629</v>
+        <v>38.32218694654462</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -3095,10 +3095,10 @@
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1376021</v>
+        <v>1374885</v>
       </c>
       <c r="L32" t="n">
-        <v>38.227759605413</v>
+        <v>38.17672023478328</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3162,10 +3162,10 @@
         <v>860000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1246979</v>
+        <v>1245949</v>
       </c>
       <c r="L33" t="n">
-        <v>31.03332133099274</v>
+        <v>30.97630801902806</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3291,10 +3291,10 @@
         <v>870000</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>1289993</v>
+        <v>1288928</v>
       </c>
       <c r="L35" t="n">
-        <v>32.55777356931394</v>
+        <v>32.50204821370938</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
@@ -3309,7 +3309,7 @@
         <v>0</v>
       </c>
       <c r="Q35" t="n">
-        <v>10.9</v>
+        <v>10.8</v>
       </c>
       <c r="R35" t="n">
         <v>4</v>
@@ -3482,10 +3482,10 @@
         <v>890000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>1160951</v>
+        <v>1159992</v>
       </c>
       <c r="L38" t="n">
-        <v>23.33871110839303</v>
+        <v>23.27533293333057</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -3546,10 +3546,10 @@
         <v>960000</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>1246979</v>
+        <v>1245949</v>
       </c>
       <c r="L39" t="n">
-        <v>23.0139400904105</v>
+        <v>22.95029732356621</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -3610,10 +3610,10 @@
         <v>970000</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>1505063</v>
+        <v>1503821</v>
       </c>
       <c r="L40" t="n">
-        <v>35.55087062800693</v>
+        <v>35.49764233908158</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -3739,10 +3739,10 @@
         <v>1022000</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>1505063</v>
+        <v>1503821</v>
       </c>
       <c r="L42" t="n">
-        <v>32.0958657544568</v>
+        <v>32.03978399024884</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -3757,7 +3757,7 @@
         <v>14.11073003429697</v>
       </c>
       <c r="Q42" t="n">
-        <v>13.1</v>
+        <v>13</v>
       </c>
       <c r="R42" t="n">
         <v>4</v>
@@ -3806,10 +3806,10 @@
         <v>1063000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1548077</v>
+        <v>1546799</v>
       </c>
       <c r="L43" t="n">
-        <v>31.33416490265019</v>
+        <v>31.27743165078333</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -3873,10 +3873,10 @@
         <v>1085000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1548077</v>
+        <v>1546799</v>
       </c>
       <c r="L44" t="n">
-        <v>29.91304696084239</v>
+        <v>29.85513954948251</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -3891,7 +3891,7 @@
         <v>61.77062374245473</v>
       </c>
       <c r="Q44" t="n">
-        <v>20.3</v>
+        <v>20.2</v>
       </c>
       <c r="R44" t="n">
         <v>4</v>
@@ -4002,10 +4002,10 @@
         <v>1123000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1720134</v>
+        <v>1718714</v>
       </c>
       <c r="L46" t="n">
-        <v>34.7143885301959</v>
+        <v>34.66044961523558</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -4020,7 +4020,7 @@
         <v>100</v>
       </c>
       <c r="Q46" t="n">
-        <v>50.5</v>
+        <v>50.4</v>
       </c>
       <c r="R46" t="n">
         <v>4</v>
@@ -4069,10 +4069,10 @@
         <v>1150000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1505063</v>
+        <v>1503821</v>
       </c>
       <c r="L47" t="n">
-        <v>23.59123837341028</v>
+        <v>23.52813267004517</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -4084,7 +4084,7 @@
         <v>89.36170212765958</v>
       </c>
       <c r="Q47" t="n">
-        <v>29.3</v>
+        <v>29.2</v>
       </c>
       <c r="R47" t="n">
         <v>3</v>
@@ -4133,10 +4133,10 @@
         <v>1150000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1505063</v>
+        <v>1503821</v>
       </c>
       <c r="L48" t="n">
-        <v>23.59123837341028</v>
+        <v>23.52813267004517</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -4148,7 +4148,7 @@
         <v>15.6366772060937</v>
       </c>
       <c r="Q48" t="n">
-        <v>13.5</v>
+        <v>13.4</v>
       </c>
       <c r="R48" t="n">
         <v>3</v>
@@ -4197,10 +4197,10 @@
         <v>1155000</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>1763148</v>
+        <v>1761692</v>
       </c>
       <c r="L49" t="n">
-        <v>34.49216968740004</v>
+        <v>34.43802889494872</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -4261,10 +4261,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1763148</v>
+        <v>1761692</v>
       </c>
       <c r="L50" t="n">
-        <v>34.49216968740004</v>
+        <v>34.43802889494872</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4381,34 +4381,31 @@
         </is>
       </c>
       <c r="I52" s="3" t="n">
-        <v>1208000</v>
+        <v>1207000</v>
       </c>
       <c r="J52" s="3" t="n">
-        <v>1208000</v>
+        <v>1207000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1892190</v>
+        <v>1890628</v>
       </c>
       <c r="L52" t="n">
-        <v>36.15863100428604</v>
+        <v>36.1587789877226</v>
       </c>
       <c r="M52" s="3" t="n">
-        <v>0</v>
+        <v>-1000</v>
       </c>
       <c r="N52" t="n">
-        <v>0</v>
-      </c>
-      <c r="O52" t="n">
-        <v>100</v>
+        <v>0.08278145695364239</v>
       </c>
       <c r="P52" t="n">
-        <v>9.013494039041035</v>
+        <v>9.265033407572403</v>
       </c>
       <c r="Q52" t="n">
-        <v>35.8</v>
+        <v>17.5</v>
       </c>
       <c r="R52" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S52" t="inlineStr">
         <is>
@@ -4419,57 +4416,57 @@
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 24GB 4TB Space Black</t>
+          <t>Macbook Pro 16 MGE74 M5 Max 18 Core CPU 32 Core GPU 36GB 2TB Silver</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M5 Max</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="E53" t="n">
-        <v>4096</v>
+        <v>2048</v>
       </c>
       <c r="F53" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="G53" t="n">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I53" s="3" t="n">
-        <v>1210000</v>
+        <v>1207000</v>
       </c>
       <c r="J53" s="3" t="n">
-        <v>1210000</v>
+        <v>1207000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1591091</v>
+        <v>1890628</v>
       </c>
       <c r="L53" t="n">
-        <v>23.95155273959817</v>
+        <v>36.1587789877226</v>
       </c>
       <c r="M53" s="3" t="n">
-        <v>0</v>
+        <v>-3000</v>
       </c>
       <c r="N53" t="n">
-        <v>0</v>
+        <v>0.2479338842975207</v>
       </c>
       <c r="P53" t="n">
-        <v>95.74468085106383</v>
+        <v>9.265033407572403</v>
       </c>
       <c r="Q53" t="n">
-        <v>30.8</v>
+        <v>17.6</v>
       </c>
       <c r="R53" t="n">
         <v>3</v>
@@ -4483,32 +4480,32 @@
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 MGE74 M5 Max 18 Core CPU 32 Core GPU 36GB 2TB Silver</t>
+          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 24GB 4TB Space Black</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>M5 Max</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="E54" t="n">
-        <v>2048</v>
+        <v>4096</v>
       </c>
       <c r="F54" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="G54" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I54" s="3" t="n">
@@ -4518,10 +4515,10 @@
         <v>1210000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1892190</v>
+        <v>1589778</v>
       </c>
       <c r="L54" t="n">
-        <v>36.05293337349843</v>
+        <v>23.88874421460103</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -4529,17 +4526,14 @@
       <c r="N54" t="n">
         <v>0</v>
       </c>
-      <c r="O54" t="n">
-        <v>0</v>
-      </c>
       <c r="P54" t="n">
-        <v>8.510415301978242</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="Q54" t="n">
-        <v>13.4</v>
+        <v>30.8</v>
       </c>
       <c r="R54" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S54" t="inlineStr">
         <is>
@@ -4585,10 +4579,10 @@
         <v>1215000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1591091</v>
+        <v>1589778</v>
       </c>
       <c r="L55" t="n">
-        <v>23.6373029575304</v>
+        <v>23.57423489317377</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -4711,10 +4705,10 @@
         <v>1280000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1677120</v>
+        <v>1675735</v>
       </c>
       <c r="L57" t="n">
-        <v>23.6786872734211</v>
+        <v>23.61560747970293</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -4726,7 +4720,7 @@
         <v>100</v>
       </c>
       <c r="Q57" t="n">
-        <v>31.6</v>
+        <v>31.5</v>
       </c>
       <c r="R57" t="n">
         <v>3</v>
@@ -4775,10 +4769,10 @@
         <v>1280000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>1720134</v>
+        <v>1718714</v>
       </c>
       <c r="L58" t="n">
-        <v>25.58719262569079</v>
+        <v>25.52571282947599</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -4842,10 +4836,10 @@
         <v>1310000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1720134</v>
+        <v>1718714</v>
       </c>
       <c r="L59" t="n">
-        <v>23.84314245285542</v>
+        <v>23.78022172391683</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -4857,7 +4851,7 @@
         <v>69.21529175050301</v>
       </c>
       <c r="Q59" t="n">
-        <v>25.1</v>
+        <v>25</v>
       </c>
       <c r="R59" t="n">
         <v>3</v>
@@ -4906,10 +4900,10 @@
         <v>1338000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1763148</v>
+        <v>1761692</v>
       </c>
       <c r="L60" t="n">
-        <v>24.11300696254654</v>
+        <v>24.05028801856397</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -4970,10 +4964,10 @@
         <v>1370000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1806162</v>
+        <v>1804671</v>
       </c>
       <c r="L61" t="n">
-        <v>24.14855367348001</v>
+        <v>24.08588601468079</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -5093,10 +5087,10 @@
         <v>1425000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>2150275</v>
+        <v>2148500</v>
       </c>
       <c r="L63" t="n">
-        <v>33.7294067037937</v>
+        <v>33.67465673725855</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -5160,10 +5154,10 @@
         <v>1430000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>2150275</v>
+        <v>2148500</v>
       </c>
       <c r="L64" t="n">
-        <v>33.49687830626315</v>
+        <v>33.44193623458226</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -5178,7 +5172,7 @@
         <v>7.126948775055698</v>
       </c>
       <c r="Q64" t="n">
-        <v>12.4</v>
+        <v>12.3</v>
       </c>
       <c r="R64" t="n">
         <v>4</v>
@@ -5227,10 +5221,10 @@
         <v>1471000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1935204</v>
+        <v>1933607</v>
       </c>
       <c r="L65" t="n">
-        <v>23.9873419029725</v>
+        <v>23.92456171290236</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -5291,10 +5285,10 @@
         <v>1471000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1935204</v>
+        <v>1933607</v>
       </c>
       <c r="L66" t="n">
-        <v>23.9873419029725</v>
+        <v>23.92456171290236</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -5306,7 +5300,7 @@
         <v>64.82531552954087</v>
       </c>
       <c r="Q66" t="n">
-        <v>24.2</v>
+        <v>24.1</v>
       </c>
       <c r="R66" t="n">
         <v>3</v>
@@ -5417,10 +5411,10 @@
         <v>1535000</v>
       </c>
       <c r="K68" s="3" t="n">
-        <v>2021232</v>
+        <v>2019564</v>
       </c>
       <c r="L68" t="n">
-        <v>24.05621917721469</v>
+        <v>23.99349562578854</v>
       </c>
       <c r="M68" s="3" t="n">
         <v>0</v>
@@ -5543,10 +5537,10 @@
         <v>1650000</v>
       </c>
       <c r="K70" s="3" t="n">
-        <v>2193289</v>
+        <v>2191478</v>
       </c>
       <c r="L70" t="n">
-        <v>24.77051587820848</v>
+        <v>24.70834751706382</v>
       </c>
       <c r="M70" s="3" t="n">
         <v>0</v>
@@ -5607,10 +5601,10 @@
         <v>1660000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2193289</v>
+        <v>2191478</v>
       </c>
       <c r="L71" t="n">
-        <v>24.31457961080368</v>
+        <v>24.2520344717127</v>
       </c>
       <c r="M71" s="3" t="n">
         <v>0</v>
@@ -5671,10 +5665,10 @@
         <v>1661000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2193289</v>
+        <v>2191478</v>
       </c>
       <c r="L72" t="n">
-        <v>24.2689859840632</v>
+        <v>24.20640316717758</v>
       </c>
       <c r="M72" s="3" t="n">
         <v>0</v>
@@ -5735,10 +5729,10 @@
         <v>1680000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2236303</v>
+        <v>2234457</v>
       </c>
       <c r="L73" t="n">
-        <v>24.87601188211079</v>
+        <v>24.81394808671637</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
@@ -5799,10 +5793,10 @@
         <v>1711000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2322331</v>
+        <v>2320414</v>
       </c>
       <c r="L74" t="n">
-        <v>26.32402530044167</v>
+        <v>26.26315821228453</v>
       </c>
       <c r="M74" s="3" t="n">
         <v>0</v>
@@ -5863,10 +5857,10 @@
         <v>1756000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2322331</v>
+        <v>2320414</v>
       </c>
       <c r="L75" t="n">
-        <v>24.38631702371454</v>
+        <v>24.32384910623708</v>
       </c>
       <c r="M75" s="3" t="n">
         <v>0</v>
@@ -5878,7 +5872,7 @@
         <v>0</v>
       </c>
       <c r="Q75" t="n">
-        <v>10.5</v>
+        <v>10.4</v>
       </c>
       <c r="R75" t="n">
         <v>3</v>
@@ -5927,10 +5921,10 @@
         <v>1790000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2365345</v>
+        <v>2363393</v>
       </c>
       <c r="L76" t="n">
-        <v>24.32393583177084</v>
+        <v>24.2614326098114</v>
       </c>
       <c r="M76" s="3" t="n">
         <v>0</v>
@@ -5942,7 +5936,7 @@
         <v>100</v>
       </c>
       <c r="Q76" t="n">
-        <v>31.9</v>
+        <v>31.8</v>
       </c>
       <c r="R76" t="n">
         <v>3</v>
@@ -5991,10 +5985,10 @@
         <v>1840000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2451373</v>
+        <v>2449350</v>
       </c>
       <c r="L77" t="n">
-        <v>24.94002340729052</v>
+        <v>24.87802886480087</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
@@ -6055,10 +6049,10 @@
         <v>1945000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2580416</v>
+        <v>2578285</v>
       </c>
       <c r="L78" t="n">
-        <v>24.62455666063146</v>
+        <v>24.56225746959704</v>
       </c>
       <c r="M78" s="3" t="n">
         <v>0</v>
@@ -6119,10 +6113,10 @@
         <v>1960000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2623430</v>
+        <v>2621264</v>
       </c>
       <c r="L79" t="n">
-        <v>25.28864882996687</v>
+        <v>25.22691342802556</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
@@ -6183,10 +6177,10 @@
         <v>2078000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2752472</v>
+        <v>2750200</v>
       </c>
       <c r="L80" t="n">
-        <v>24.50422747261371</v>
+        <v>24.44185877390735</v>
       </c>
       <c r="M80" s="3" t="n">
         <v>0</v>
@@ -6247,10 +6241,10 @@
         <v>2170000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2881514</v>
+        <v>2879136</v>
       </c>
       <c r="L81" t="n">
-        <v>24.69236658228973</v>
+        <v>24.63016682782612</v>
       </c>
       <c r="M81" s="3" t="n">
         <v>0</v>
@@ -6311,10 +6305,10 @@
         <v>2268000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>3010557</v>
+        <v>3008071</v>
       </c>
       <c r="L82" t="n">
-        <v>24.66510350078075</v>
+        <v>24.60284348341512</v>
       </c>
       <c r="M82" s="3" t="n">
         <v>0</v>
@@ -6326,7 +6320,7 @@
         <v>70.41425389755011</v>
       </c>
       <c r="Q82" t="n">
-        <v>25.7</v>
+        <v>25.6</v>
       </c>
       <c r="R82" t="n">
         <v>3</v>
@@ -6375,10 +6369,10 @@
         <v>2270000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3053571</v>
+        <v>3051050</v>
       </c>
       <c r="L83" t="n">
-        <v>25.66080827987953</v>
+        <v>25.59938381868537</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
@@ -6439,10 +6433,10 @@
         <v>2381000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3182613</v>
+        <v>3179986</v>
       </c>
       <c r="L84" t="n">
-        <v>25.18725965111058</v>
+        <v>25.1254565271671</v>
       </c>
       <c r="M84" s="3" t="n">
         <v>0</v>
@@ -6503,10 +6497,10 @@
         <v>2470000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3311655</v>
+        <v>3308921</v>
       </c>
       <c r="L85" t="n">
-        <v>25.41493603651346</v>
+        <v>25.3533100367159</v>
       </c>
       <c r="M85" s="3" t="n">
         <v>0</v>
@@ -6567,10 +6561,10 @@
         <v>2480000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3311655</v>
+        <v>3308921</v>
       </c>
       <c r="L86" t="n">
-        <v>25.11297221479894</v>
+        <v>25.05109671702649</v>
       </c>
       <c r="M86" s="3" t="n">
         <v>0</v>
@@ -6631,10 +6625,10 @@
         <v>2571000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3440698</v>
+        <v>3437857</v>
       </c>
       <c r="L87" t="n">
-        <v>25.27678976765761</v>
+        <v>25.21503948535381</v>
       </c>
       <c r="M87" s="3" t="n">
         <v>0</v>
@@ -6695,10 +6689,10 @@
         <v>2580000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3483712</v>
+        <v>3480836</v>
       </c>
       <c r="L88" t="n">
-        <v>25.94106516267705</v>
+        <v>25.87987483466615</v>
       </c>
       <c r="M88" s="3" t="n">
         <v>0</v>
@@ -6759,10 +6753,10 @@
         <v>2581000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3440698</v>
+        <v>3437857</v>
       </c>
       <c r="L89" t="n">
-        <v>24.98615106585931</v>
+        <v>24.92416060353878</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
@@ -6823,10 +6817,10 @@
         <v>2664000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3612754</v>
+        <v>3609772</v>
       </c>
       <c r="L90" t="n">
-        <v>26.26124004014666</v>
+        <v>26.20032511748665</v>
       </c>
       <c r="M90" s="3" t="n">
         <v>0</v>
@@ -6887,10 +6881,10 @@
         <v>3090000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>4171937</v>
+        <v>4168493</v>
       </c>
       <c r="L91" t="n">
-        <v>25.93368500051655</v>
+        <v>25.87249156949526</v>
       </c>
       <c r="M91" s="3" t="n">
         <v>0</v>
@@ -6951,10 +6945,10 @@
         <v>3186000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4300980</v>
+        <v>4297429</v>
       </c>
       <c r="L92" t="n">
-        <v>25.92385921348158</v>
+        <v>25.86264950508781</v>
       </c>
       <c r="M92" s="3" t="n">
         <v>0</v>
@@ -7249,10 +7243,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>429711</v>
+        <v>429356</v>
       </c>
       <c r="L2" t="n">
-        <v>27.85872365380454</v>
+        <v>27.79907582518935</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7267,7 +7261,7 @@
         <v>29.71702857142851</v>
       </c>
       <c r="Q2" t="n">
-        <v>36.5</v>
+        <v>36.4</v>
       </c>
       <c r="R2" t="n">
         <v>4</v>
@@ -7316,10 +7310,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>429711</v>
+        <v>429356</v>
       </c>
       <c r="L3" t="n">
-        <v>27.85872365380454</v>
+        <v>27.79907582518935</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7334,7 +7328,7 @@
         <v>29.71702857142851</v>
       </c>
       <c r="Q3" t="n">
-        <v>36.5</v>
+        <v>36.4</v>
       </c>
       <c r="R3" t="n">
         <v>4</v>
@@ -7383,10 +7377,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>429711</v>
+        <v>429356</v>
       </c>
       <c r="L4" t="n">
-        <v>27.85849093925918</v>
+        <v>27.79884291823102</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7450,10 +7444,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>429711</v>
+        <v>429356</v>
       </c>
       <c r="L5" t="n">
-        <v>27.85849093925918</v>
+        <v>27.79884291823102</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7517,10 +7511,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>515739</v>
+        <v>515313</v>
       </c>
       <c r="L6" t="n">
-        <v>25.54373433073706</v>
+        <v>25.48218267344313</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7581,10 +7575,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>515739</v>
+        <v>515313</v>
       </c>
       <c r="L7" t="n">
-        <v>25.54373433073706</v>
+        <v>25.48218267344313</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7645,10 +7639,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>515739</v>
+        <v>515313</v>
       </c>
       <c r="L8" t="n">
-        <v>25.54373433073706</v>
+        <v>25.48218267344313</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7709,10 +7703,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>515739</v>
+        <v>515313</v>
       </c>
       <c r="L9" t="n">
-        <v>25.54373433073706</v>
+        <v>25.48218267344313</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7773,10 +7767,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>515739</v>
+        <v>515313</v>
       </c>
       <c r="L10" t="n">
-        <v>25.34983780555669</v>
+        <v>25.28812585748856</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7788,7 +7782,7 @@
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>10.9</v>
+        <v>10.8</v>
       </c>
       <c r="R10" t="n">
         <v>3</v>
@@ -7837,10 +7831,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>515739</v>
+        <v>515313</v>
       </c>
       <c r="L11" t="n">
-        <v>25.34983780555669</v>
+        <v>25.28812585748856</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7852,7 +7846,7 @@
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>10.9</v>
+        <v>10.8</v>
       </c>
       <c r="R11" t="n">
         <v>3</v>
@@ -7901,10 +7895,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>515739</v>
+        <v>515313</v>
       </c>
       <c r="L12" t="n">
-        <v>25.34983780555669</v>
+        <v>25.28812585748856</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -7916,7 +7910,7 @@
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>10.9</v>
+        <v>10.8</v>
       </c>
       <c r="R12" t="n">
         <v>3</v>
@@ -7965,10 +7959,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>515739</v>
+        <v>515313</v>
       </c>
       <c r="L13" t="n">
-        <v>25.34983780555669</v>
+        <v>25.28812585748856</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -7980,7 +7974,7 @@
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>10.9</v>
+        <v>10.8</v>
       </c>
       <c r="R13" t="n">
         <v>3</v>
@@ -8029,10 +8023,10 @@
         <v>430000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>558753</v>
+        <v>558292</v>
       </c>
       <c r="L14" t="n">
-        <v>23.04291878522352</v>
+        <v>22.97937280132977</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -8096,13 +8090,13 @@
         <v>434999</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>558753</v>
+        <v>558292</v>
       </c>
       <c r="L15" t="n">
-        <v>22.14824797361267</v>
+        <v>22.08396323071081</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="N15" t="n">
         <v>0</v>
@@ -8163,13 +8157,13 @@
         <v>441999</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>558753</v>
+        <v>558292</v>
       </c>
       <c r="L16" t="n">
-        <v>20.89545827941863</v>
+        <v>20.83013906701153</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>-6000</v>
+        <v>0</v>
       </c>
       <c r="N16" t="n">
         <v>1.339288703769428</v>
@@ -8230,10 +8224,10 @@
         <v>447999</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>558753</v>
+        <v>558292</v>
       </c>
       <c r="L17" t="n">
-        <v>19.82163854153803</v>
+        <v>19.75543264098357</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -8297,10 +8291,10 @@
         <v>453000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>558753</v>
+        <v>558292</v>
       </c>
       <c r="L18" t="n">
-        <v>18.92660979001455</v>
+        <v>18.85966483488927</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -8364,10 +8358,10 @@
         <v>454000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>601767</v>
+        <v>601270</v>
       </c>
       <c r="L19" t="n">
-        <v>24.5555173347824</v>
+        <v>24.49315615280988</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -8428,10 +8422,10 @@
         <v>454000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>601767</v>
+        <v>601270</v>
       </c>
       <c r="L20" t="n">
-        <v>24.5555173347824</v>
+        <v>24.49315615280988</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -8492,10 +8486,10 @@
         <v>454000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>601767</v>
+        <v>601270</v>
       </c>
       <c r="L21" t="n">
-        <v>24.5555173347824</v>
+        <v>24.49315615280988</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -8556,10 +8550,10 @@
         <v>454000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>601767</v>
+        <v>601270</v>
       </c>
       <c r="L22" t="n">
-        <v>24.5555173347824</v>
+        <v>24.49315615280988</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -8620,10 +8614,10 @@
         <v>455000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>601767</v>
+        <v>601270</v>
       </c>
       <c r="L23" t="n">
-        <v>24.38934006018941</v>
+        <v>24.32684151878524</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -8684,10 +8678,10 @@
         <v>455000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>601767</v>
+        <v>601270</v>
       </c>
       <c r="L24" t="n">
-        <v>24.38934006018941</v>
+        <v>24.32684151878524</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -8748,10 +8742,10 @@
         <v>455000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>601767</v>
+        <v>601270</v>
       </c>
       <c r="L25" t="n">
-        <v>24.38934006018941</v>
+        <v>24.32684151878524</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -8812,10 +8806,10 @@
         <v>455000</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>601767</v>
+        <v>601270</v>
       </c>
       <c r="L26" t="n">
-        <v>24.38934006018941</v>
+        <v>24.32684151878524</v>
       </c>
       <c r="M26" s="3" t="n">
         <v>0</v>
@@ -8876,10 +8870,10 @@
         <v>475000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>687795</v>
+        <v>687228</v>
       </c>
       <c r="L27" t="n">
-        <v>30.93872447458909</v>
+        <v>30.88174521410653</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -8940,10 +8934,10 @@
         <v>475000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>687795</v>
+        <v>687228</v>
       </c>
       <c r="L28" t="n">
-        <v>30.93872447458909</v>
+        <v>30.88174521410653</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -9004,10 +8998,10 @@
         <v>475000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>687795</v>
+        <v>687228</v>
       </c>
       <c r="L29" t="n">
-        <v>30.93872447458909</v>
+        <v>30.88174521410653</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -9068,10 +9062,10 @@
         <v>475000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>687795</v>
+        <v>687228</v>
       </c>
       <c r="L30" t="n">
-        <v>30.93872447458909</v>
+        <v>30.88174521410653</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -9132,10 +9126,10 @@
         <v>479999</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>687795</v>
+        <v>687228</v>
       </c>
       <c r="L31" t="n">
-        <v>30.21190907174376</v>
+        <v>30.15433014952825</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -9196,10 +9190,10 @@
         <v>479999</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>687795</v>
+        <v>687228</v>
       </c>
       <c r="L32" t="n">
-        <v>30.21190907174376</v>
+        <v>30.15433014952825</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -9260,10 +9254,10 @@
         <v>479999</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>687795</v>
+        <v>687228</v>
       </c>
       <c r="L33" t="n">
-        <v>30.21190907174376</v>
+        <v>30.15433014952825</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -9324,10 +9318,10 @@
         <v>479999</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>687795</v>
+        <v>687228</v>
       </c>
       <c r="L34" t="n">
-        <v>30.21190907174376</v>
+        <v>30.15433014952825</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -9388,10 +9382,10 @@
         <v>482999</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>644781</v>
+        <v>644249</v>
       </c>
       <c r="L35" t="n">
-        <v>25.09099988988509</v>
+        <v>25.029142458894</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
@@ -9406,7 +9400,7 @@
         <v>5.818666666666681</v>
       </c>
       <c r="Q35" t="n">
-        <v>31.6</v>
+        <v>31.5</v>
       </c>
       <c r="R35" t="n">
         <v>4</v>
@@ -9455,10 +9449,10 @@
         <v>482999</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>644781</v>
+        <v>644249</v>
       </c>
       <c r="L36" t="n">
-        <v>25.09099988988509</v>
+        <v>25.029142458894</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -9473,7 +9467,7 @@
         <v>5.818666666666681</v>
       </c>
       <c r="Q36" t="n">
-        <v>31.6</v>
+        <v>31.5</v>
       </c>
       <c r="R36" t="n">
         <v>4</v>
@@ -9522,10 +9516,10 @@
         <v>482999</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>644781</v>
+        <v>644249</v>
       </c>
       <c r="L37" t="n">
-        <v>25.09099988988509</v>
+        <v>25.029142458894</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
@@ -9540,7 +9534,7 @@
         <v>5.818666666666681</v>
       </c>
       <c r="Q37" t="n">
-        <v>31.6</v>
+        <v>31.5</v>
       </c>
       <c r="R37" t="n">
         <v>4</v>
@@ -9589,10 +9583,10 @@
         <v>495000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>644781</v>
+        <v>644249</v>
       </c>
       <c r="L38" t="n">
-        <v>23.22974777482587</v>
+        <v>23.16635338199982</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -9656,10 +9650,10 @@
         <v>500000</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>644781</v>
+        <v>644249</v>
       </c>
       <c r="L39" t="n">
-        <v>22.45429068164229</v>
+        <v>22.39025594141395</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -9720,10 +9714,10 @@
         <v>551999</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>773824</v>
+        <v>773185</v>
       </c>
       <c r="L40" t="n">
-        <v>28.66607910842776</v>
+        <v>28.60712507355937</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -9738,7 +9732,7 @@
         <v>68.91123055162657</v>
       </c>
       <c r="Q40" t="n">
-        <v>43.3</v>
+        <v>43.2</v>
       </c>
       <c r="R40" t="n">
         <v>4</v>
@@ -9787,10 +9781,10 @@
         <v>551999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>773824</v>
+        <v>773185</v>
       </c>
       <c r="L41" t="n">
-        <v>28.66607910842776</v>
+        <v>28.60712507355937</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
@@ -9805,7 +9799,7 @@
         <v>68.91123055162657</v>
       </c>
       <c r="Q41" t="n">
-        <v>43.3</v>
+        <v>43.2</v>
       </c>
       <c r="R41" t="n">
         <v>4</v>
@@ -9854,10 +9848,10 @@
         <v>551999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>773824</v>
+        <v>773185</v>
       </c>
       <c r="L42" t="n">
-        <v>28.66607910842776</v>
+        <v>28.60712507355937</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -9872,7 +9866,7 @@
         <v>68.91123055162657</v>
       </c>
       <c r="Q42" t="n">
-        <v>43.3</v>
+        <v>43.2</v>
       </c>
       <c r="R42" t="n">
         <v>4</v>
@@ -9921,10 +9915,10 @@
         <v>557999</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>773824</v>
+        <v>773185</v>
       </c>
       <c r="L43" t="n">
-        <v>27.89070899842858</v>
+        <v>27.83111415767248</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -9988,10 +9982,10 @@
         <v>564999</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>773824</v>
+        <v>773185</v>
       </c>
       <c r="L44" t="n">
-        <v>26.98611053676288</v>
+        <v>26.92576808913779</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -10003,7 +9997,7 @@
         <v>34.54581818181818</v>
       </c>
       <c r="Q44" t="n">
-        <v>19</v>
+        <v>18.9</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -10052,10 +10046,10 @@
         <v>564999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>773824</v>
+        <v>773185</v>
       </c>
       <c r="L45" t="n">
-        <v>26.98611053676288</v>
+        <v>26.92576808913779</v>
       </c>
       <c r="M45" s="3" t="n">
         <v>0</v>
@@ -10067,7 +10061,7 @@
         <v>34.54581818181818</v>
       </c>
       <c r="Q45" t="n">
-        <v>19</v>
+        <v>18.9</v>
       </c>
       <c r="R45" t="n">
         <v>3</v>
@@ -10116,10 +10110,10 @@
         <v>564999</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>773824</v>
+        <v>773185</v>
       </c>
       <c r="L46" t="n">
-        <v>26.98611053676288</v>
+        <v>26.92576808913779</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -10131,7 +10125,7 @@
         <v>34.54581818181818</v>
       </c>
       <c r="Q46" t="n">
-        <v>19</v>
+        <v>18.9</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -10180,10 +10174,10 @@
         <v>564999</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>773824</v>
+        <v>773185</v>
       </c>
       <c r="L47" t="n">
-        <v>26.98611053676288</v>
+        <v>26.92576808913779</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -10195,7 +10189,7 @@
         <v>34.54581818181818</v>
       </c>
       <c r="Q47" t="n">
-        <v>19</v>
+        <v>18.9</v>
       </c>
       <c r="R47" t="n">
         <v>3</v>
@@ -10244,10 +10238,10 @@
         <v>585000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>730810</v>
+        <v>730206</v>
       </c>
       <c r="L48" t="n">
-        <v>19.95183426608832</v>
+        <v>19.8856213178199</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -10308,10 +10302,10 @@
         <v>595000</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>730810</v>
+        <v>730206</v>
       </c>
       <c r="L49" t="n">
-        <v>18.58348955268811</v>
+        <v>18.51614475915016</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -10372,10 +10366,10 @@
         <v>614999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>859852</v>
+        <v>859142</v>
       </c>
       <c r="L50" t="n">
-        <v>28.4761796216093</v>
+        <v>28.41707191593473</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -10439,10 +10433,10 @@
         <v>616999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>859852</v>
+        <v>859142</v>
       </c>
       <c r="L51" t="n">
-        <v>28.24358145355247</v>
+        <v>28.1842815273843</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -10451,13 +10445,13 @@
         <v>0</v>
       </c>
       <c r="O51" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="P51" t="n">
         <v>60.50938181818182</v>
       </c>
       <c r="Q51" t="n">
-        <v>19.5</v>
+        <v>37.3</v>
       </c>
       <c r="R51" t="n">
         <v>4</v>
@@ -10506,10 +10500,10 @@
         <v>616999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>859852</v>
+        <v>859142</v>
       </c>
       <c r="L52" t="n">
-        <v>28.24358145355247</v>
+        <v>28.1842815273843</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -10518,13 +10512,13 @@
         <v>0</v>
       </c>
       <c r="O52" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="P52" t="n">
         <v>60.50938181818182</v>
       </c>
       <c r="Q52" t="n">
-        <v>19.5</v>
+        <v>37.3</v>
       </c>
       <c r="R52" t="n">
         <v>4</v>
@@ -10567,19 +10561,19 @@
         </is>
       </c>
       <c r="I53" s="3" t="n">
-        <v>616999</v>
+        <v>624999</v>
       </c>
       <c r="J53" s="3" t="n">
-        <v>616999</v>
+        <v>624999</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>859852</v>
+        <v>859142</v>
       </c>
       <c r="L53" t="n">
-        <v>28.24358145355247</v>
+        <v>27.25311997318255</v>
       </c>
       <c r="M53" s="3" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="N53" t="n">
         <v>0</v>
@@ -10588,10 +10582,10 @@
         <v>0</v>
       </c>
       <c r="P53" t="n">
-        <v>60.50938181818182</v>
+        <v>58.18210909090909</v>
       </c>
       <c r="Q53" t="n">
-        <v>19.5</v>
+        <v>18.8</v>
       </c>
       <c r="R53" t="n">
         <v>4</v>
@@ -10640,10 +10634,10 @@
         <v>650000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>816838</v>
+        <v>816163</v>
       </c>
       <c r="L54" t="n">
-        <v>20.42485780534206</v>
+        <v>20.3590459258751</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -10655,7 +10649,7 @@
         <v>50.90909090909091</v>
       </c>
       <c r="Q54" t="n">
-        <v>19.7</v>
+        <v>19.6</v>
       </c>
       <c r="R54" t="n">
         <v>3</v>
@@ -10704,10 +10698,10 @@
         <v>672000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>859852</v>
+        <v>859142</v>
       </c>
       <c r="L55" t="n">
-        <v>21.84701553290566</v>
+        <v>21.78242944705299</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -10768,10 +10762,10 @@
         <v>700000</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>902866</v>
+        <v>902121</v>
       </c>
       <c r="L56" t="n">
-        <v>22.46911501817545</v>
+        <v>22.40508756585868</v>
       </c>
       <c r="M56" s="3" t="n">
         <v>0</v>
@@ -10832,10 +10826,10 @@
         <v>715000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>945880</v>
+        <v>945099</v>
       </c>
       <c r="L57" t="n">
-        <v>24.40901594282573</v>
+        <v>24.34654993815463</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -10896,10 +10890,10 @@
         <v>752000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>988894</v>
+        <v>988078</v>
       </c>
       <c r="L58" t="n">
-        <v>23.95544921902651</v>
+        <v>23.89264815125931</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -10960,10 +10954,10 @@
         <v>756000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>988894</v>
+        <v>988078</v>
       </c>
       <c r="L59" t="n">
-        <v>23.55095692763835</v>
+        <v>23.48782181163835</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -11024,10 +11018,10 @@
         <v>810000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1074922</v>
+        <v>1074035</v>
       </c>
       <c r="L60" t="n">
-        <v>24.64569522253708</v>
+        <v>24.5834632949578</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -11088,10 +11082,10 @@
         <v>815000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1074922</v>
+        <v>1074035</v>
       </c>
       <c r="L61" t="n">
-        <v>24.18054519304657</v>
+        <v>24.11792911776618</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -11152,10 +11146,10 @@
         <v>875000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1160951</v>
+        <v>1159992</v>
       </c>
       <c r="L62" t="n">
-        <v>24.6307553031954</v>
+        <v>24.56844529962276</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -11216,10 +11210,10 @@
         <v>992000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1333007</v>
+        <v>1331906</v>
       </c>
       <c r="L63" t="n">
-        <v>25.58178614215829</v>
+        <v>25.52026944844456</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -11280,10 +11274,10 @@
         <v>1050000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1419035</v>
+        <v>1417864</v>
       </c>
       <c r="L64" t="n">
-        <v>26.00605340953535</v>
+        <v>25.94494253327541</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -11344,10 +11338,10 @@
         <v>1050000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1419035</v>
+        <v>1417864</v>
       </c>
       <c r="L65" t="n">
-        <v>26.00605340953535</v>
+        <v>25.94494253327541</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -11408,10 +11402,10 @@
         <v>1100000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1505063</v>
+        <v>1503821</v>
       </c>
       <c r="L66" t="n">
-        <v>26.91335844413157</v>
+        <v>26.85299646699973</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -11472,10 +11466,10 @@
         <v>1105000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1505063</v>
+        <v>1503821</v>
       </c>
       <c r="L67" t="n">
-        <v>26.58114643705945</v>
+        <v>26.52051008730427</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -11536,10 +11530,10 @@
         <v>1155000</v>
       </c>
       <c r="K68" s="3" t="n">
-        <v>1591091</v>
+        <v>1589778</v>
       </c>
       <c r="L68" t="n">
-        <v>27.40830034234371</v>
+        <v>27.34834675030098</v>
       </c>
       <c r="M68" s="3" t="n">
         <v>0</v>
@@ -11551,7 +11545,7 @@
         <v>100</v>
       </c>
       <c r="Q68" t="n">
-        <v>33.2</v>
+        <v>33.1</v>
       </c>
       <c r="R68" t="n">
         <v>3</v>
@@ -11807,7 +11801,7 @@
         <v>315000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>300669</v>
+        <v>300420</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -11868,10 +11862,10 @@
         <v>380000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>386697</v>
+        <v>386378</v>
       </c>
       <c r="L3" t="n">
-        <v>1.731846898217468</v>
+        <v>1.650715102826765</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -11883,7 +11877,7 @@
         <v>100</v>
       </c>
       <c r="Q3" t="n">
-        <v>22.2</v>
+        <v>22.1</v>
       </c>
       <c r="R3" t="n">
         <v>3</v>
@@ -11932,7 +11926,7 @@
         <v>415000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>386697</v>
+        <v>386378</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -11993,10 +11987,10 @@
         <v>495000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>472725</v>
+        <v>472335</v>
       </c>
       <c r="L5" t="n">
-        <v>6.922840975196996</v>
+        <v>6.845988546264834</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -12057,10 +12051,10 @@
         <v>500000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>515739</v>
+        <v>515313</v>
       </c>
       <c r="L6" t="n">
-        <v>8.868633165225045</v>
+        <v>8.793296501349666</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -12072,7 +12066,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>4.1</v>
+        <v>4</v>
       </c>
       <c r="R6" t="n">
         <v>4</v>
@@ -12121,10 +12115,10 @@
         <v>550000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>558753</v>
+        <v>558292</v>
       </c>
       <c r="L7" t="n">
-        <v>6.935622717014494</v>
+        <v>6.858776410910419</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -12136,7 +12130,7 @@
         <v>25.45360054666915</v>
       </c>
       <c r="Q7" t="n">
-        <v>8.1</v>
+        <v>8</v>
       </c>
       <c r="R7" t="n">
         <v>4</v>
@@ -12185,7 +12179,7 @@
         <v>530000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>472725</v>
+        <v>472335</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -12249,10 +12243,10 @@
         <v>600000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>601767</v>
+        <v>601270</v>
       </c>
       <c r="L9" t="n">
-        <v>8.602498973855329</v>
+        <v>8.526951286443694</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -12313,10 +12307,10 @@
         <v>646000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>730810</v>
+        <v>730206</v>
       </c>
       <c r="L10" t="n">
-        <v>17.21528167375925</v>
+        <v>17.14680514813628</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -12377,7 +12371,7 @@
         <v>615000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>558753</v>
+        <v>558292</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -12441,7 +12435,7 @@
         <v>700000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>644781</v>
+        <v>644249</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -12505,7 +12499,7 @@
         <v>745000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>687795</v>
+        <v>687228</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -12569,7 +12563,7 @@
         <v>930000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>859852</v>
+        <v>859142</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -12689,7 +12683,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHE4 M5 10C CPU 8C GPU 16GB 512GB Midnight</t>
+          <t>Macbook Pro 16 MGE74 M5 Max 18 Core CPU 32 Core GPU 36GB 2TB Silver</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -12698,46 +12692,46 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>447999</v>
+        <v>1210000</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>441999</v>
+        <v>1207000</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-6000</v>
+        <v>-3000</v>
       </c>
       <c r="F2" t="n">
-        <v>-1.34</v>
+        <v>-0.25</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 MDE34 10 Core CPU 10 Core GPU 24GB 1TB Space Black</t>
+          <t>Macbook Pro 16 MGED4 M5 Max 18 Core CPU 32 Core GPU 36GB 2TB Space Black</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>643000</v>
+        <v>1208000</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>645000</v>
+        <v>1207000</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>2000</v>
+        <v>-1000</v>
       </c>
       <c r="F3" t="n">
-        <v>0.31</v>
+        <v>-0.08</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHH4 M5 10C CPU 8C GPU 16GB 512GB Sky Blue</t>
+          <t>Apple MacBook Air 15 MDVC4 M5 10C CPU 10C GPU 24GB 1TB Silver</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -12746,16 +12740,16 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>432999</v>
+        <v>616999</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>434999</v>
+        <v>624999</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>2000</v>
+        <v>8000</v>
       </c>
       <c r="F4" t="n">
-        <v>0.46</v>
+        <v>1.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: price data 2026-09-19
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MacBook Pro'!$A$1:$S$92</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MacBook Air'!$A$1:$S$68</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20260918T081854429215+0000</t>
+          <t>20260919T080651505066+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-18T08:18:54.429215+00:00</t>
+          <t>2026-09-19T08:06:51.505066+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>277.281209</v>
+        <v>277.421451</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -750,7 +750,7 @@
         <v>1123000</v>
       </c>
       <c r="D23" t="n">
-        <v>50.4</v>
+        <v>50.5</v>
       </c>
       <c r="E23" t="n">
         <v>4</v>
@@ -801,7 +801,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 MDE34 10 Core CPU 10 Core GPU 24GB 1TB Space Black</t>
+          <t>Macbook Pro 14 M5 MJ3D4 10 Core CPU 10 Core GPU 32GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -810,10 +810,10 @@
         </is>
       </c>
       <c r="C26" s="3" t="n">
-        <v>645000</v>
+        <v>745000</v>
       </c>
       <c r="D26" t="n">
-        <v>44.7</v>
+        <v>45.4</v>
       </c>
       <c r="E26" t="n">
         <v>4</v>
@@ -822,7 +822,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 MJLV4 M5 Pro 15 Core CPU 16 Core GPU 24GB 2TB Silver</t>
+          <t>Macbook Pro 14 M5 MDE34 10 Core CPU 10 Core GPU 24GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -831,19 +831,19 @@
         </is>
       </c>
       <c r="C27" s="3" t="n">
-        <v>815000</v>
+        <v>645000</v>
       </c>
       <c r="D27" t="n">
-        <v>44.6</v>
+        <v>44.7</v>
       </c>
       <c r="E27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 MGDR4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Space Black</t>
+          <t>Macbook Pro 14 MJLV4 M5 Pro 15 Core CPU 16 Core GPU 24GB 2TB Silver</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -852,10 +852,10 @@
         </is>
       </c>
       <c r="C28" s="3" t="n">
-        <v>728000</v>
+        <v>815000</v>
       </c>
       <c r="D28" t="n">
-        <v>44.4</v>
+        <v>44.6</v>
       </c>
       <c r="E28" t="n">
         <v>3</v>
@@ -864,7 +864,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 MGEC4 M5 Pro 18 Core CPU 20 Core GPU 48GB 1TB Space Black</t>
+          <t>Macbook Pro 14 MGDR4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -873,19 +873,19 @@
         </is>
       </c>
       <c r="C29" s="3" t="n">
-        <v>1063000</v>
+        <v>728000</v>
       </c>
       <c r="D29" t="n">
-        <v>43.7</v>
+        <v>44.4</v>
       </c>
       <c r="E29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 16Inch MX303 14Core CPU 32Core GPU M4 Max 36GB 1TB Space Black</t>
+          <t>Macbook Pro 16 MGEC4 M5 Pro 18 Core CPU 20 Core GPU 48GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -894,10 +894,10 @@
         </is>
       </c>
       <c r="C30" s="3" t="n">
-        <v>970000</v>
+        <v>1063000</v>
       </c>
       <c r="D30" t="n">
-        <v>43.2</v>
+        <v>43.7</v>
       </c>
       <c r="E30" t="n">
         <v>4</v>
@@ -918,7 +918,7 @@
         <v>551999</v>
       </c>
       <c r="D31" t="n">
-        <v>43.2</v>
+        <v>43.3</v>
       </c>
       <c r="E31" t="n">
         <v>4</v>
@@ -1147,10 +1147,10 @@
         <v>470000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>687228</v>
+        <v>687575</v>
       </c>
       <c r="L2" t="n">
-        <v>35.24710867426822</v>
+        <v>35.27978765952805</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1214,10 +1214,10 @@
         <v>465000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>687228</v>
+        <v>687575</v>
       </c>
       <c r="L3" t="n">
-        <v>33.35545117486482</v>
+        <v>33.38908482710977</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>773185</v>
+        <v>773576</v>
       </c>
       <c r="L4" t="n">
-        <v>35.33255301124569</v>
+        <v>35.36523883884712</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>773185</v>
+        <v>773576</v>
       </c>
       <c r="L5" t="n">
-        <v>32.74584995828941</v>
+        <v>32.77984322160977</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>859142</v>
+        <v>859576</v>
       </c>
       <c r="L6" t="n">
-        <v>38.07775664558362</v>
+        <v>38.10902119184342</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1600,10 +1600,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>859142</v>
+        <v>859576</v>
       </c>
       <c r="L9" t="n">
-        <v>34.2367152345014</v>
+        <v>34.26991912291641</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1667,10 +1667,10 @@
         <v>582999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>859142</v>
+        <v>859576</v>
       </c>
       <c r="L10" t="n">
-        <v>32.14171813274174</v>
+        <v>32.17597978538256</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -1734,10 +1734,10 @@
         <v>587999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>859142</v>
+        <v>859576</v>
       </c>
       <c r="L11" t="n">
-        <v>31.55974216136564</v>
+        <v>31.59429765372695</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -1801,10 +1801,10 @@
         <v>645000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>945099</v>
+        <v>945577</v>
       </c>
       <c r="L12" t="n">
-        <v>31.75318141274089</v>
+        <v>31.78768096093708</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -1927,10 +1927,10 @@
         <v>650000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>945099</v>
+        <v>945577</v>
       </c>
       <c r="L14" t="n">
-        <v>31.2241363074133</v>
+        <v>31.2589032939676</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -1994,10 +1994,10 @@
         <v>650000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>859142</v>
+        <v>859576</v>
       </c>
       <c r="L15" t="n">
-        <v>24.3431237211078</v>
+        <v>24.3813228847711</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0</v>
@@ -2058,10 +2058,10 @@
         <v>650000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>859142</v>
+        <v>859576</v>
       </c>
       <c r="L16" t="n">
-        <v>24.3431237211078</v>
+        <v>24.3813228847711</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -2122,10 +2122,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1031056</v>
+        <v>1031578</v>
       </c>
       <c r="L17" t="n">
-        <v>32.10844027870456</v>
+        <v>32.14279482501566</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2189,10 +2189,10 @@
         <v>707999</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>1074035</v>
+        <v>1074578</v>
       </c>
       <c r="L18" t="n">
-        <v>34.08045361650225</v>
+        <v>34.11376372864511</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -2256,10 +2256,10 @@
         <v>720000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>1031056</v>
+        <v>1031578</v>
       </c>
       <c r="L19" t="n">
-        <v>30.16868142952468</v>
+        <v>30.20401753430182</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -2447,10 +2447,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1074035</v>
+        <v>1074578</v>
       </c>
       <c r="L22" t="n">
-        <v>30.82162126932549</v>
+        <v>30.85657811717716</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2479,7 +2479,7 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 MJ3E4 10 Core CPU 10 Core GPU 32GB 1TB Silver</t>
+          <t>Macbook Pro 14 M5 MJ3D4 10 Core CPU 10 Core GPU 32GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -2504,35 +2504,38 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I23" s="3" t="n">
-        <v>772000</v>
+        <v>745000</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>772000</v>
+        <v>745000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1031056</v>
+        <v>1031578</v>
       </c>
       <c r="L23" t="n">
-        <v>25.12530842165702</v>
+        <v>27.78054592090952</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>0</v>
+        <v>-27000</v>
       </c>
       <c r="N23" t="n">
-        <v>0</v>
+        <v>3.49740932642487</v>
+      </c>
+      <c r="O23" t="n">
+        <v>100</v>
       </c>
       <c r="P23" t="n">
-        <v>71.91489361702126</v>
+        <v>77.6595744680851</v>
       </c>
       <c r="Q23" t="n">
-        <v>26.2</v>
+        <v>45.4</v>
       </c>
       <c r="R23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S23" t="inlineStr">
         <is>
@@ -2543,7 +2546,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 MJ3D4 10 Core CPU 10 Core GPU 32GB 1TB Space Black</t>
+          <t>Macbook Pro 14 M5 MJ3E4 10 Core CPU 10 Core GPU 32GB 1TB Silver</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -2568,35 +2571,38 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I24" s="3" t="n">
-        <v>772000</v>
+        <v>755000</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>772000</v>
+        <v>755000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1031056</v>
+        <v>1031578</v>
       </c>
       <c r="L24" t="n">
-        <v>25.12530842165702</v>
+        <v>26.8111572755526</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>0</v>
+        <v>-17000</v>
       </c>
       <c r="N24" t="n">
-        <v>0</v>
+        <v>2.202072538860103</v>
+      </c>
+      <c r="O24" t="n">
+        <v>62.96296296296296</v>
       </c>
       <c r="P24" t="n">
-        <v>71.91489361702126</v>
+        <v>75.53191489361704</v>
       </c>
       <c r="Q24" t="n">
-        <v>26.2</v>
+        <v>36.1</v>
       </c>
       <c r="R24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S24" t="inlineStr">
         <is>
@@ -2642,25 +2648,28 @@
         <v>772000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>1031056</v>
+        <v>1031578</v>
       </c>
       <c r="L25" t="n">
-        <v>25.12530842165702</v>
+        <v>25.16319657844584</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N25" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" t="n">
         <v>0</v>
       </c>
       <c r="P25" t="n">
         <v>71.91489361702126</v>
       </c>
       <c r="Q25" t="n">
-        <v>26.2</v>
+        <v>20.4</v>
       </c>
       <c r="R25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S25" t="inlineStr">
         <is>
@@ -2768,10 +2777,10 @@
         <v>810000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>1245949</v>
+        <v>1246579</v>
       </c>
       <c r="L27" t="n">
-        <v>34.98931336675899</v>
+        <v>35.0221686712194</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -2897,10 +2906,10 @@
         <v>832999</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>1288928</v>
+        <v>1289580</v>
       </c>
       <c r="L29" t="n">
-        <v>35.37272834479506</v>
+        <v>35.40540330960468</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -2964,10 +2973,10 @@
         <v>835000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1074035</v>
+        <v>1074578</v>
       </c>
       <c r="L30" t="n">
-        <v>22.25579240899971</v>
+        <v>22.29507769561632</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -3028,10 +3037,10 @@
         <v>930000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1374885</v>
+        <v>1375580</v>
       </c>
       <c r="L31" t="n">
-        <v>38.32218694654462</v>
+        <v>38.35334913272947</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -3095,10 +3104,10 @@
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1374885</v>
+        <v>1375580</v>
       </c>
       <c r="L32" t="n">
-        <v>38.17672023478328</v>
+        <v>38.20795591677692</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3162,10 +3171,10 @@
         <v>860000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1245949</v>
+        <v>1246579</v>
       </c>
       <c r="L33" t="n">
-        <v>30.97630801902806</v>
+        <v>31.01119142870207</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3291,10 +3300,10 @@
         <v>870000</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>1288928</v>
+        <v>1289580</v>
       </c>
       <c r="L35" t="n">
-        <v>32.50204821370938</v>
+        <v>32.53617456846415</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
@@ -3482,10 +3491,10 @@
         <v>890000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>1159992</v>
+        <v>1160579</v>
       </c>
       <c r="L38" t="n">
-        <v>23.27533293333057</v>
+        <v>23.31413889101905</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -3546,10 +3555,10 @@
         <v>960000</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>1245949</v>
+        <v>1246579</v>
       </c>
       <c r="L39" t="n">
-        <v>22.95029732356621</v>
+        <v>22.98923694366743</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -3610,10 +3619,10 @@
         <v>970000</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>1503821</v>
+        <v>1504581</v>
       </c>
       <c r="L40" t="n">
-        <v>35.49764233908158</v>
+        <v>35.53022402914831</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -3739,10 +3748,10 @@
         <v>1022000</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>1503821</v>
+        <v>1504581</v>
       </c>
       <c r="L42" t="n">
-        <v>32.03978399024884</v>
+        <v>32.07411232761812</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -3806,10 +3815,10 @@
         <v>1063000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1546799</v>
+        <v>1547582</v>
       </c>
       <c r="L43" t="n">
-        <v>31.27743165078333</v>
+        <v>31.31220187363255</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -3873,10 +3882,10 @@
         <v>1085000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1546799</v>
+        <v>1547582</v>
       </c>
       <c r="L44" t="n">
-        <v>29.85513954948251</v>
+        <v>29.89062938183567</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -3891,7 +3900,7 @@
         <v>61.77062374245473</v>
       </c>
       <c r="Q44" t="n">
-        <v>20.2</v>
+        <v>20.3</v>
       </c>
       <c r="R44" t="n">
         <v>4</v>
@@ -4002,10 +4011,10 @@
         <v>1123000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1718714</v>
+        <v>1719583</v>
       </c>
       <c r="L46" t="n">
-        <v>34.66044961523558</v>
+        <v>34.69346928877524</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -4020,7 +4029,7 @@
         <v>100</v>
       </c>
       <c r="Q46" t="n">
-        <v>50.4</v>
+        <v>50.5</v>
       </c>
       <c r="R46" t="n">
         <v>4</v>
@@ -4069,10 +4078,10 @@
         <v>1150000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1503821</v>
+        <v>1504581</v>
       </c>
       <c r="L47" t="n">
-        <v>23.52813267004517</v>
+        <v>23.56676044692841</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -4133,10 +4142,10 @@
         <v>1150000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1503821</v>
+        <v>1504581</v>
       </c>
       <c r="L48" t="n">
-        <v>23.52813267004517</v>
+        <v>23.56676044692841</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -4148,7 +4157,7 @@
         <v>15.6366772060937</v>
       </c>
       <c r="Q48" t="n">
-        <v>13.4</v>
+        <v>13.5</v>
       </c>
       <c r="R48" t="n">
         <v>3</v>
@@ -4197,10 +4206,10 @@
         <v>1155000</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>1761692</v>
+        <v>1762583</v>
       </c>
       <c r="L49" t="n">
-        <v>34.43802889494872</v>
+        <v>34.47117100301092</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -4261,10 +4270,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1761692</v>
+        <v>1762583</v>
       </c>
       <c r="L50" t="n">
-        <v>34.43802889494872</v>
+        <v>34.47117100301092</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4387,13 +4396,13 @@
         <v>1207000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1890628</v>
+        <v>1891584</v>
       </c>
       <c r="L52" t="n">
-        <v>36.1587789877226</v>
+        <v>36.1910441196373</v>
       </c>
       <c r="M52" s="3" t="n">
-        <v>-1000</v>
+        <v>0</v>
       </c>
       <c r="N52" t="n">
         <v>0.08278145695364239</v>
@@ -4451,13 +4460,13 @@
         <v>1207000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1890628</v>
+        <v>1891584</v>
       </c>
       <c r="L53" t="n">
-        <v>36.1587789877226</v>
+        <v>36.1910441196373</v>
       </c>
       <c r="M53" s="3" t="n">
-        <v>-3000</v>
+        <v>0</v>
       </c>
       <c r="N53" t="n">
         <v>0.2479338842975207</v>
@@ -4515,10 +4524,10 @@
         <v>1210000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1589778</v>
+        <v>1590582</v>
       </c>
       <c r="L54" t="n">
-        <v>23.88874421460103</v>
+        <v>23.9272165785857</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -4579,10 +4588,10 @@
         <v>1215000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1589778</v>
+        <v>1590582</v>
       </c>
       <c r="L55" t="n">
-        <v>23.57423489317377</v>
+        <v>23.61286623386911</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -4705,10 +4714,10 @@
         <v>1280000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1675735</v>
+        <v>1676583</v>
       </c>
       <c r="L57" t="n">
-        <v>23.61560747970293</v>
+        <v>23.65424199100194</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -4720,7 +4729,7 @@
         <v>100</v>
       </c>
       <c r="Q57" t="n">
-        <v>31.5</v>
+        <v>31.6</v>
       </c>
       <c r="R57" t="n">
         <v>3</v>
@@ -4769,10 +4778,10 @@
         <v>1280000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>1718714</v>
+        <v>1719583</v>
       </c>
       <c r="L58" t="n">
-        <v>25.52571282947599</v>
+        <v>25.56334878863073</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -4836,10 +4845,10 @@
         <v>1310000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1718714</v>
+        <v>1719583</v>
       </c>
       <c r="L59" t="n">
-        <v>23.78022172391683</v>
+        <v>23.81873977586427</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -4900,10 +4909,10 @@
         <v>1338000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1761692</v>
+        <v>1762583</v>
       </c>
       <c r="L60" t="n">
-        <v>24.05028801856397</v>
+        <v>24.08868121387759</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -4964,10 +4973,10 @@
         <v>1370000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1804671</v>
+        <v>1805584</v>
       </c>
       <c r="L61" t="n">
-        <v>24.08588601468079</v>
+        <v>24.12427225761859</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -5052,7 +5061,7 @@
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 MGEE4 M5 Max 18 Core CPU 40 Core GPU 48GB 2TB Space Black</t>
+          <t>Macbook Pro 16 MGE94 M5 Max 18 Core CPU 40 Core GPU 48GB 2TB Silver</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -5077,38 +5086,35 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I63" s="3" t="n">
-        <v>1425000</v>
+        <v>1460000</v>
       </c>
       <c r="J63" s="3" t="n">
-        <v>1425000</v>
+        <v>1460000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>2148500</v>
+        <v>2149586</v>
       </c>
       <c r="L63" t="n">
-        <v>33.67465673725855</v>
+        <v>32.07994469632757</v>
       </c>
       <c r="M63" s="3" t="n">
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="N63" t="n">
         <v>0</v>
       </c>
-      <c r="O63" t="n">
-        <v>100</v>
-      </c>
       <c r="P63" t="n">
-        <v>8.195991091314051</v>
+        <v>0.7126948775055885</v>
       </c>
       <c r="Q63" t="n">
-        <v>34.8</v>
+        <v>13.9</v>
       </c>
       <c r="R63" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S63" t="inlineStr">
         <is>
@@ -5119,7 +5125,7 @@
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 MGE94 M5 Max 18 Core CPU 40 Core GPU 48GB 2TB Silver</t>
+          <t>Macbook Pro 16 MGEE4 M5 Max 18 Core CPU 40 Core GPU 48GB 2TB Space Black</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -5144,38 +5150,35 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I64" s="3" t="n">
-        <v>1430000</v>
+        <v>1460000</v>
       </c>
       <c r="J64" s="3" t="n">
-        <v>1430000</v>
+        <v>1460000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>2148500</v>
+        <v>2149586</v>
       </c>
       <c r="L64" t="n">
-        <v>33.44193623458226</v>
+        <v>32.07994469632757</v>
       </c>
       <c r="M64" s="3" t="n">
-        <v>0</v>
+        <v>35000</v>
       </c>
       <c r="N64" t="n">
         <v>0</v>
       </c>
-      <c r="O64" t="n">
-        <v>0</v>
-      </c>
       <c r="P64" t="n">
-        <v>7.126948775055698</v>
+        <v>0.7126948775055885</v>
       </c>
       <c r="Q64" t="n">
-        <v>12.3</v>
+        <v>13.9</v>
       </c>
       <c r="R64" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S64" t="inlineStr">
         <is>
@@ -5221,10 +5224,10 @@
         <v>1471000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1933607</v>
+        <v>1934585</v>
       </c>
       <c r="L65" t="n">
-        <v>23.92456171290236</v>
+        <v>23.96302049276718</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -5285,10 +5288,10 @@
         <v>1471000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1933607</v>
+        <v>1934585</v>
       </c>
       <c r="L66" t="n">
-        <v>23.92456171290236</v>
+        <v>23.96302049276718</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -5300,7 +5303,7 @@
         <v>64.82531552954087</v>
       </c>
       <c r="Q66" t="n">
-        <v>24.1</v>
+        <v>24.2</v>
       </c>
       <c r="R66" t="n">
         <v>3</v>
@@ -5411,10 +5414,10 @@
         <v>1535000</v>
       </c>
       <c r="K68" s="3" t="n">
-        <v>2019564</v>
+        <v>2020585</v>
       </c>
       <c r="L68" t="n">
-        <v>23.99349562578854</v>
+        <v>24.03190165224428</v>
       </c>
       <c r="M68" s="3" t="n">
         <v>0</v>
@@ -5537,10 +5540,10 @@
         <v>1650000</v>
       </c>
       <c r="K70" s="3" t="n">
-        <v>2191478</v>
+        <v>2192587</v>
       </c>
       <c r="L70" t="n">
-        <v>24.70834751706382</v>
+        <v>24.74642967417028</v>
       </c>
       <c r="M70" s="3" t="n">
         <v>0</v>
@@ -5601,10 +5604,10 @@
         <v>1660000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2191478</v>
+        <v>2192587</v>
       </c>
       <c r="L71" t="n">
-        <v>24.2520344717127</v>
+        <v>24.29034742977132</v>
       </c>
       <c r="M71" s="3" t="n">
         <v>0</v>
@@ -5665,10 +5668,10 @@
         <v>1661000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2191478</v>
+        <v>2192587</v>
       </c>
       <c r="L72" t="n">
-        <v>24.20640316717758</v>
+        <v>24.24473920533142</v>
       </c>
       <c r="M72" s="3" t="n">
         <v>0</v>
@@ -5729,10 +5732,10 @@
         <v>1680000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2234457</v>
+        <v>2235587</v>
       </c>
       <c r="L73" t="n">
-        <v>24.81394808671637</v>
+        <v>24.85195163507392</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
@@ -5793,10 +5796,10 @@
         <v>1711000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2320414</v>
+        <v>2321588</v>
       </c>
       <c r="L74" t="n">
-        <v>26.26315821228453</v>
+        <v>26.30044607398039</v>
       </c>
       <c r="M74" s="3" t="n">
         <v>0</v>
@@ -5857,10 +5860,10 @@
         <v>1756000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2320414</v>
+        <v>2321588</v>
       </c>
       <c r="L75" t="n">
-        <v>24.32384910623708</v>
+        <v>24.36211765395066</v>
       </c>
       <c r="M75" s="3" t="n">
         <v>0</v>
@@ -5921,10 +5924,10 @@
         <v>1790000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2363393</v>
+        <v>2364588</v>
       </c>
       <c r="L76" t="n">
-        <v>24.2614326098114</v>
+        <v>24.29970887105915</v>
       </c>
       <c r="M76" s="3" t="n">
         <v>0</v>
@@ -5985,10 +5988,10 @@
         <v>1840000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2449350</v>
+        <v>2450589</v>
       </c>
       <c r="L77" t="n">
-        <v>24.87802886480087</v>
+        <v>24.91600998780293</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
@@ -6049,10 +6052,10 @@
         <v>1945000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2578285</v>
+        <v>2579589</v>
       </c>
       <c r="L78" t="n">
-        <v>24.56225746959704</v>
+        <v>24.60039176783588</v>
       </c>
       <c r="M78" s="3" t="n">
         <v>0</v>
@@ -6113,10 +6116,10 @@
         <v>1960000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2621264</v>
+        <v>2622590</v>
       </c>
       <c r="L79" t="n">
-        <v>25.22691342802556</v>
+        <v>25.26471922793879</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
@@ -6177,10 +6180,10 @@
         <v>2078000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2750200</v>
+        <v>2751591</v>
       </c>
       <c r="L80" t="n">
-        <v>24.44185877390735</v>
+        <v>24.48005535706433</v>
       </c>
       <c r="M80" s="3" t="n">
         <v>0</v>
@@ -6241,10 +6244,10 @@
         <v>2170000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2879136</v>
+        <v>2880592</v>
       </c>
       <c r="L81" t="n">
-        <v>24.63016682782612</v>
+        <v>24.66826263490283</v>
       </c>
       <c r="M81" s="3" t="n">
         <v>0</v>
@@ -6305,10 +6308,10 @@
         <v>2268000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>3008071</v>
+        <v>3009593</v>
       </c>
       <c r="L82" t="n">
-        <v>24.60284348341512</v>
+        <v>24.6409730485152</v>
       </c>
       <c r="M82" s="3" t="n">
         <v>0</v>
@@ -6369,10 +6372,10 @@
         <v>2270000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3051050</v>
+        <v>3052593</v>
       </c>
       <c r="L83" t="n">
-        <v>25.59938381868537</v>
+        <v>25.63699123990653</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
@@ -6433,10 +6436,10 @@
         <v>2381000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3179986</v>
+        <v>3181594</v>
       </c>
       <c r="L84" t="n">
-        <v>25.1254565271671</v>
+        <v>25.16329864841334</v>
       </c>
       <c r="M84" s="3" t="n">
         <v>0</v>
@@ -6497,10 +6500,10 @@
         <v>2470000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3308921</v>
+        <v>3310595</v>
       </c>
       <c r="L85" t="n">
-        <v>25.3533100367159</v>
+        <v>25.39105508224353</v>
       </c>
       <c r="M85" s="3" t="n">
         <v>0</v>
@@ -6561,10 +6564,10 @@
         <v>2480000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3308921</v>
+        <v>3310595</v>
       </c>
       <c r="L86" t="n">
-        <v>25.05109671702649</v>
+        <v>25.08899457650362</v>
       </c>
       <c r="M86" s="3" t="n">
         <v>0</v>
@@ -6625,10 +6628,10 @@
         <v>2571000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3437857</v>
+        <v>3439596</v>
       </c>
       <c r="L87" t="n">
-        <v>25.21503948535381</v>
+        <v>25.25284946255316</v>
       </c>
       <c r="M87" s="3" t="n">
         <v>0</v>
@@ -6689,10 +6692,10 @@
         <v>2580000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3480836</v>
+        <v>3482596</v>
       </c>
       <c r="L88" t="n">
-        <v>25.87987483466615</v>
+        <v>25.91733293210008</v>
       </c>
       <c r="M88" s="3" t="n">
         <v>0</v>
@@ -6753,10 +6756,10 @@
         <v>2581000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3437857</v>
+        <v>3439596</v>
       </c>
       <c r="L89" t="n">
-        <v>24.92416060353878</v>
+        <v>24.9621176440489</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
@@ -6817,10 +6820,10 @@
         <v>2664000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3609772</v>
+        <v>3611597</v>
       </c>
       <c r="L90" t="n">
-        <v>26.20032511748665</v>
+        <v>26.23761731998338</v>
       </c>
       <c r="M90" s="3" t="n">
         <v>0</v>
@@ -6881,10 +6884,10 @@
         <v>3090000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>4168493</v>
+        <v>4170602</v>
       </c>
       <c r="L91" t="n">
-        <v>25.87249156949526</v>
+        <v>25.90997654535245</v>
       </c>
       <c r="M91" s="3" t="n">
         <v>0</v>
@@ -6945,10 +6948,10 @@
         <v>3186000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4297429</v>
+        <v>4299602</v>
       </c>
       <c r="L92" t="n">
-        <v>25.86264950508781</v>
+        <v>25.9001181969866</v>
       </c>
       <c r="M92" s="3" t="n">
         <v>0</v>
@@ -7243,10 +7246,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>429356</v>
+        <v>429573</v>
       </c>
       <c r="L2" t="n">
-        <v>27.79907582518935</v>
+        <v>27.83554832356782</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7261,7 +7264,7 @@
         <v>29.71702857142851</v>
       </c>
       <c r="Q2" t="n">
-        <v>36.4</v>
+        <v>36.5</v>
       </c>
       <c r="R2" t="n">
         <v>4</v>
@@ -7310,10 +7313,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>429356</v>
+        <v>429573</v>
       </c>
       <c r="L3" t="n">
-        <v>27.79907582518935</v>
+        <v>27.83554832356782</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7328,7 +7331,7 @@
         <v>29.71702857142851</v>
       </c>
       <c r="Q3" t="n">
-        <v>36.4</v>
+        <v>36.5</v>
       </c>
       <c r="R3" t="n">
         <v>4</v>
@@ -7377,10 +7380,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>429356</v>
+        <v>429573</v>
       </c>
       <c r="L4" t="n">
-        <v>27.79884291823102</v>
+        <v>27.8353155342631</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7444,10 +7447,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>429356</v>
+        <v>429573</v>
       </c>
       <c r="L5" t="n">
-        <v>27.79884291823102</v>
+        <v>27.8353155342631</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7511,10 +7514,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>515313</v>
+        <v>515574</v>
       </c>
       <c r="L6" t="n">
-        <v>25.48218267344313</v>
+        <v>25.51990596888129</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7575,10 +7578,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>515313</v>
+        <v>515574</v>
       </c>
       <c r="L7" t="n">
-        <v>25.48218267344313</v>
+        <v>25.51990596888129</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7639,10 +7642,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>515313</v>
+        <v>515574</v>
       </c>
       <c r="L8" t="n">
-        <v>25.48218267344313</v>
+        <v>25.51990596888129</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7703,10 +7706,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>515313</v>
+        <v>515574</v>
       </c>
       <c r="L9" t="n">
-        <v>25.48218267344313</v>
+        <v>25.51990596888129</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7767,10 +7770,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>515313</v>
+        <v>515574</v>
       </c>
       <c r="L10" t="n">
-        <v>25.28812585748856</v>
+        <v>25.32594739067525</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7782,7 +7785,7 @@
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>10.8</v>
+        <v>10.9</v>
       </c>
       <c r="R10" t="n">
         <v>3</v>
@@ -7831,10 +7834,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>515313</v>
+        <v>515574</v>
       </c>
       <c r="L11" t="n">
-        <v>25.28812585748856</v>
+        <v>25.32594739067525</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7846,7 +7849,7 @@
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>10.8</v>
+        <v>10.9</v>
       </c>
       <c r="R11" t="n">
         <v>3</v>
@@ -7895,10 +7898,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>515313</v>
+        <v>515574</v>
       </c>
       <c r="L12" t="n">
-        <v>25.28812585748856</v>
+        <v>25.32594739067525</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -7910,7 +7913,7 @@
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>10.8</v>
+        <v>10.9</v>
       </c>
       <c r="R12" t="n">
         <v>3</v>
@@ -7959,10 +7962,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>515313</v>
+        <v>515574</v>
       </c>
       <c r="L13" t="n">
-        <v>25.28812585748856</v>
+        <v>25.32594739067525</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -7974,7 +7977,7 @@
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>10.8</v>
+        <v>10.9</v>
       </c>
       <c r="R13" t="n">
         <v>3</v>
@@ -8023,10 +8026,10 @@
         <v>430000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>558292</v>
+        <v>558574</v>
       </c>
       <c r="L14" t="n">
-        <v>22.97937280132977</v>
+        <v>23.01825720495404</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -8090,10 +8093,10 @@
         <v>434999</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>558292</v>
+        <v>558574</v>
       </c>
       <c r="L15" t="n">
-        <v>22.08396323071081</v>
+        <v>22.12329968813443</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0</v>
@@ -8157,10 +8160,10 @@
         <v>441999</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>558292</v>
+        <v>558574</v>
       </c>
       <c r="L16" t="n">
-        <v>20.83013906701153</v>
+        <v>20.87010852635461</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -8224,10 +8227,10 @@
         <v>447999</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>558292</v>
+        <v>558574</v>
       </c>
       <c r="L17" t="n">
-        <v>19.75543264098357</v>
+        <v>19.79594467340048</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -8291,10 +8294,10 @@
         <v>453000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>558292</v>
+        <v>558574</v>
       </c>
       <c r="L18" t="n">
-        <v>18.85966483488927</v>
+        <v>18.90062910196321</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -8358,10 +8361,10 @@
         <v>454000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>601270</v>
+        <v>601575</v>
       </c>
       <c r="L19" t="n">
-        <v>24.49315615280988</v>
+        <v>24.53143830777542</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -8422,10 +8425,10 @@
         <v>454000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>601270</v>
+        <v>601575</v>
       </c>
       <c r="L20" t="n">
-        <v>24.49315615280988</v>
+        <v>24.53143830777542</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -8486,10 +8489,10 @@
         <v>454000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>601270</v>
+        <v>601575</v>
       </c>
       <c r="L21" t="n">
-        <v>24.49315615280988</v>
+        <v>24.53143830777542</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -8550,10 +8553,10 @@
         <v>454000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>601270</v>
+        <v>601575</v>
       </c>
       <c r="L22" t="n">
-        <v>24.49315615280988</v>
+        <v>24.53143830777542</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -8614,10 +8617,10 @@
         <v>455000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>601270</v>
+        <v>601575</v>
       </c>
       <c r="L23" t="n">
-        <v>24.32684151878524</v>
+        <v>24.36520799567801</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -8678,10 +8681,10 @@
         <v>455000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>601270</v>
+        <v>601575</v>
       </c>
       <c r="L24" t="n">
-        <v>24.32684151878524</v>
+        <v>24.36520799567801</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -8742,10 +8745,10 @@
         <v>455000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>601270</v>
+        <v>601575</v>
       </c>
       <c r="L25" t="n">
-        <v>24.32684151878524</v>
+        <v>24.36520799567801</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -8806,10 +8809,10 @@
         <v>455000</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>601270</v>
+        <v>601575</v>
       </c>
       <c r="L26" t="n">
-        <v>24.32684151878524</v>
+        <v>24.36520799567801</v>
       </c>
       <c r="M26" s="3" t="n">
         <v>0</v>
@@ -8870,10 +8873,10 @@
         <v>475000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>687228</v>
+        <v>687575</v>
       </c>
       <c r="L27" t="n">
-        <v>30.88174521410653</v>
+        <v>30.91662727702432</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -8934,10 +8937,10 @@
         <v>475000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>687228</v>
+        <v>687575</v>
       </c>
       <c r="L28" t="n">
-        <v>30.88174521410653</v>
+        <v>30.91662727702432</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -8998,10 +9001,10 @@
         <v>475000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>687228</v>
+        <v>687575</v>
       </c>
       <c r="L29" t="n">
-        <v>30.88174521410653</v>
+        <v>30.91662727702432</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -9062,10 +9065,10 @@
         <v>475000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>687228</v>
+        <v>687575</v>
       </c>
       <c r="L30" t="n">
-        <v>30.88174521410653</v>
+        <v>30.91662727702432</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -9126,10 +9129,10 @@
         <v>479999</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>687228</v>
+        <v>687575</v>
       </c>
       <c r="L31" t="n">
-        <v>30.15433014952825</v>
+        <v>30.18957931861978</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -9190,10 +9193,10 @@
         <v>479999</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>687228</v>
+        <v>687575</v>
       </c>
       <c r="L32" t="n">
-        <v>30.15433014952825</v>
+        <v>30.18957931861978</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -9254,10 +9257,10 @@
         <v>479999</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>687228</v>
+        <v>687575</v>
       </c>
       <c r="L33" t="n">
-        <v>30.15433014952825</v>
+        <v>30.18957931861978</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -9318,10 +9321,10 @@
         <v>479999</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>687228</v>
+        <v>687575</v>
       </c>
       <c r="L34" t="n">
-        <v>30.15433014952825</v>
+        <v>30.18957931861978</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -9382,10 +9385,10 @@
         <v>482999</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>644249</v>
+        <v>644575</v>
       </c>
       <c r="L35" t="n">
-        <v>25.029142458894</v>
+        <v>25.06705969049374</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
@@ -9449,10 +9452,10 @@
         <v>482999</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>644249</v>
+        <v>644575</v>
       </c>
       <c r="L36" t="n">
-        <v>25.029142458894</v>
+        <v>25.06705969049374</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -9516,10 +9519,10 @@
         <v>482999</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>644249</v>
+        <v>644575</v>
       </c>
       <c r="L37" t="n">
-        <v>25.029142458894</v>
+        <v>25.06705969049374</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
@@ -9583,10 +9586,10 @@
         <v>495000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>644249</v>
+        <v>644575</v>
       </c>
       <c r="L38" t="n">
-        <v>23.16635338199982</v>
+        <v>23.20521273707482</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -9650,10 +9653,10 @@
         <v>500000</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>644249</v>
+        <v>644575</v>
       </c>
       <c r="L39" t="n">
-        <v>22.39025594141395</v>
+        <v>22.42950781522709</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -9714,10 +9717,10 @@
         <v>551999</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>773185</v>
+        <v>773576</v>
       </c>
       <c r="L40" t="n">
-        <v>28.60712507355937</v>
+        <v>28.64321023403001</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -9732,7 +9735,7 @@
         <v>68.91123055162657</v>
       </c>
       <c r="Q40" t="n">
-        <v>43.2</v>
+        <v>43.3</v>
       </c>
       <c r="R40" t="n">
         <v>4</v>
@@ -9781,10 +9784,10 @@
         <v>551999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>773185</v>
+        <v>773576</v>
       </c>
       <c r="L41" t="n">
-        <v>28.60712507355937</v>
+        <v>28.64321023403001</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
@@ -9799,7 +9802,7 @@
         <v>68.91123055162657</v>
       </c>
       <c r="Q41" t="n">
-        <v>43.2</v>
+        <v>43.3</v>
       </c>
       <c r="R41" t="n">
         <v>4</v>
@@ -9848,10 +9851,10 @@
         <v>551999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>773185</v>
+        <v>773576</v>
       </c>
       <c r="L42" t="n">
-        <v>28.60712507355937</v>
+        <v>28.64321023403001</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -9866,7 +9869,7 @@
         <v>68.91123055162657</v>
       </c>
       <c r="Q42" t="n">
-        <v>43.2</v>
+        <v>43.3</v>
       </c>
       <c r="R42" t="n">
         <v>4</v>
@@ -9915,10 +9918,10 @@
         <v>557999</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>773185</v>
+        <v>773576</v>
       </c>
       <c r="L43" t="n">
-        <v>27.83111415767248</v>
+        <v>27.8675915488588</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -9982,10 +9985,10 @@
         <v>564999</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>773185</v>
+        <v>773576</v>
       </c>
       <c r="L44" t="n">
-        <v>26.92576808913779</v>
+        <v>26.96270308282573</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -9997,7 +10000,7 @@
         <v>34.54581818181818</v>
       </c>
       <c r="Q44" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -10046,10 +10049,10 @@
         <v>564999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>773185</v>
+        <v>773576</v>
       </c>
       <c r="L45" t="n">
-        <v>26.92576808913779</v>
+        <v>26.96270308282573</v>
       </c>
       <c r="M45" s="3" t="n">
         <v>0</v>
@@ -10061,7 +10064,7 @@
         <v>34.54581818181818</v>
       </c>
       <c r="Q45" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
       <c r="R45" t="n">
         <v>3</v>
@@ -10110,10 +10113,10 @@
         <v>564999</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>773185</v>
+        <v>773576</v>
       </c>
       <c r="L46" t="n">
-        <v>26.92576808913779</v>
+        <v>26.96270308282573</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -10125,7 +10128,7 @@
         <v>34.54581818181818</v>
       </c>
       <c r="Q46" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -10174,10 +10177,10 @@
         <v>564999</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>773185</v>
+        <v>773576</v>
       </c>
       <c r="L47" t="n">
-        <v>26.92576808913779</v>
+        <v>26.96270308282573</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -10189,7 +10192,7 @@
         <v>34.54581818181818</v>
       </c>
       <c r="Q47" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
       <c r="R47" t="n">
         <v>3</v>
@@ -10238,10 +10241,10 @@
         <v>585000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>730206</v>
+        <v>730576</v>
       </c>
       <c r="L48" t="n">
-        <v>19.8856213178199</v>
+        <v>19.92619522130483</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -10302,10 +10305,10 @@
         <v>595000</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>730206</v>
+        <v>730576</v>
       </c>
       <c r="L49" t="n">
-        <v>18.51614475915016</v>
+        <v>18.55741223363483</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -10366,10 +10369,10 @@
         <v>614999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>859142</v>
+        <v>859576</v>
       </c>
       <c r="L50" t="n">
-        <v>28.41707191593473</v>
+        <v>28.45321414278668</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -10433,10 +10436,10 @@
         <v>616999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>859142</v>
+        <v>859576</v>
       </c>
       <c r="L51" t="n">
-        <v>28.1842815273843</v>
+        <v>28.22054129012443</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -10500,10 +10503,10 @@
         <v>616999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>859142</v>
+        <v>859576</v>
       </c>
       <c r="L52" t="n">
-        <v>28.1842815273843</v>
+        <v>28.22054129012443</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -10567,13 +10570,13 @@
         <v>624999</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>859142</v>
+        <v>859576</v>
       </c>
       <c r="L53" t="n">
-        <v>27.25311997318255</v>
+        <v>27.28984987947547</v>
       </c>
       <c r="M53" s="3" t="n">
-        <v>8000</v>
+        <v>0</v>
       </c>
       <c r="N53" t="n">
         <v>0</v>
@@ -10634,10 +10637,10 @@
         <v>650000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>816163</v>
+        <v>816576</v>
       </c>
       <c r="L54" t="n">
-        <v>20.3590459258751</v>
+        <v>20.3993259659848</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -10649,7 +10652,7 @@
         <v>50.90909090909091</v>
       </c>
       <c r="Q54" t="n">
-        <v>19.6</v>
+        <v>19.7</v>
       </c>
       <c r="R54" t="n">
         <v>3</v>
@@ -10698,10 +10701,10 @@
         <v>672000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>859142</v>
+        <v>859576</v>
       </c>
       <c r="L55" t="n">
-        <v>21.78242944705299</v>
+        <v>21.82192150548643</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -10762,10 +10765,10 @@
         <v>700000</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>902121</v>
+        <v>902577</v>
       </c>
       <c r="L56" t="n">
-        <v>22.40508756585868</v>
+        <v>22.4442900716504</v>
       </c>
       <c r="M56" s="3" t="n">
         <v>0</v>
@@ -10826,10 +10829,10 @@
         <v>715000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>945099</v>
+        <v>945577</v>
       </c>
       <c r="L57" t="n">
-        <v>24.34654993815463</v>
+        <v>24.38479362336436</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -10855,11 +10858,11 @@
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 CTO M5 10C CPU 10C GPU 16GB 2TB Midnight</t>
+          <t>Apple MacBook Air Z1L2000VN 13 M5 10C CPU 10C GPU 24GB 2TB Silver</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -10867,7 +10870,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E58" t="n">
         <v>2048</v>
@@ -10880,32 +10883,32 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Midnight</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I58" s="3" t="n">
-        <v>752000</v>
+        <v>734999</v>
       </c>
       <c r="J58" s="3" t="n">
-        <v>752000</v>
+        <v>734999</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>988078</v>
+        <v>988577</v>
       </c>
       <c r="L58" t="n">
-        <v>23.89264815125931</v>
+        <v>25.6508091934164</v>
       </c>
       <c r="M58" s="3" t="n">
-        <v>0</v>
+        <v>-21001</v>
       </c>
       <c r="N58" t="n">
-        <v>0</v>
+        <v>2.777910052910053</v>
       </c>
       <c r="P58" t="n">
-        <v>57.6969696969697</v>
+        <v>78.07662153970499</v>
       </c>
       <c r="Q58" t="n">
-        <v>22.6</v>
+        <v>28.7</v>
       </c>
       <c r="R58" t="n">
         <v>3</v>
@@ -10919,11 +10922,11 @@
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air Z1L2000VN 13 M5 10C CPU 10C GPU 24GB 2TB Silver</t>
+          <t>Apple MacBook Air 15 CTO M5 10C CPU 10C GPU 16GB 2TB Midnight</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -10931,7 +10934,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E59" t="n">
         <v>2048</v>
@@ -10944,20 +10947,20 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Midnight</t>
         </is>
       </c>
       <c r="I59" s="3" t="n">
-        <v>756000</v>
+        <v>752000</v>
       </c>
       <c r="J59" s="3" t="n">
-        <v>756000</v>
+        <v>752000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>988078</v>
+        <v>988577</v>
       </c>
       <c r="L59" t="n">
-        <v>23.48782181163835</v>
+        <v>23.93106455035875</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -10966,10 +10969,10 @@
         <v>0</v>
       </c>
       <c r="P59" t="n">
-        <v>72.98444130127297</v>
+        <v>57.6969696969697</v>
       </c>
       <c r="Q59" t="n">
-        <v>25.7</v>
+        <v>22.6</v>
       </c>
       <c r="R59" t="n">
         <v>3</v>
@@ -11018,10 +11021,10 @@
         <v>810000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1074035</v>
+        <v>1074578</v>
       </c>
       <c r="L60" t="n">
-        <v>24.5834632949578</v>
+        <v>24.62157237538829</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -11082,10 +11085,10 @@
         <v>815000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1074035</v>
+        <v>1074578</v>
       </c>
       <c r="L61" t="n">
-        <v>24.11792911776618</v>
+        <v>24.1562734394339</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -11146,10 +11149,10 @@
         <v>875000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1159992</v>
+        <v>1160579</v>
       </c>
       <c r="L62" t="n">
-        <v>24.56844529962276</v>
+        <v>24.60659722431648</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -11210,10 +11213,10 @@
         <v>992000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1331906</v>
+        <v>1332580</v>
       </c>
       <c r="L63" t="n">
-        <v>25.52026944844456</v>
+        <v>25.55794023623347</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -11274,10 +11277,10 @@
         <v>1050000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1417864</v>
+        <v>1418581</v>
       </c>
       <c r="L64" t="n">
-        <v>25.94494253327541</v>
+        <v>25.98237252578457</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -11338,10 +11341,10 @@
         <v>1050000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1417864</v>
+        <v>1418581</v>
       </c>
       <c r="L65" t="n">
-        <v>25.94494253327541</v>
+        <v>25.98237252578457</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -11402,10 +11405,10 @@
         <v>1100000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1503821</v>
+        <v>1504581</v>
       </c>
       <c r="L66" t="n">
-        <v>26.85299646699973</v>
+        <v>26.88994477532283</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -11466,10 +11469,10 @@
         <v>1105000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1503821</v>
+        <v>1504581</v>
       </c>
       <c r="L67" t="n">
-        <v>26.52051008730427</v>
+        <v>26.55762634248339</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -11530,10 +11533,10 @@
         <v>1155000</v>
       </c>
       <c r="K68" s="3" t="n">
-        <v>1589778</v>
+        <v>1590582</v>
       </c>
       <c r="L68" t="n">
-        <v>27.34834675030098</v>
+        <v>27.38507037046817</v>
       </c>
       <c r="M68" s="3" t="n">
         <v>0</v>
@@ -11545,7 +11548,7 @@
         <v>100</v>
       </c>
       <c r="Q68" t="n">
-        <v>33.1</v>
+        <v>33.2</v>
       </c>
       <c r="R68" t="n">
         <v>3</v>
@@ -11801,7 +11804,7 @@
         <v>315000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>300420</v>
+        <v>300572</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -11862,10 +11865,10 @@
         <v>380000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>386378</v>
+        <v>386573</v>
       </c>
       <c r="L3" t="n">
-        <v>1.650715102826765</v>
+        <v>1.700325682342016</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -11877,7 +11880,7 @@
         <v>100</v>
       </c>
       <c r="Q3" t="n">
-        <v>22.1</v>
+        <v>22.2</v>
       </c>
       <c r="R3" t="n">
         <v>3</v>
@@ -11926,7 +11929,7 @@
         <v>415000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>386378</v>
+        <v>386573</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -11987,10 +11990,10 @@
         <v>495000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>472335</v>
+        <v>472574</v>
       </c>
       <c r="L5" t="n">
-        <v>6.845988546264834</v>
+        <v>6.893100339840956</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -12051,10 +12054,10 @@
         <v>500000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>515313</v>
+        <v>515574</v>
       </c>
       <c r="L6" t="n">
-        <v>8.793296501349666</v>
+        <v>8.83946824316199</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -12066,7 +12069,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>4</v>
+        <v>4.1</v>
       </c>
       <c r="R6" t="n">
         <v>4</v>
@@ -12115,10 +12118,10 @@
         <v>550000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>558292</v>
+        <v>558574</v>
       </c>
       <c r="L7" t="n">
-        <v>6.858776410910419</v>
+        <v>6.9057994106421</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -12179,7 +12182,7 @@
         <v>530000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>472335</v>
+        <v>472574</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -12243,10 +12246,10 @@
         <v>600000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>601270</v>
+        <v>601575</v>
       </c>
       <c r="L9" t="n">
-        <v>8.526951286443694</v>
+        <v>8.57332834642397</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -12307,10 +12310,10 @@
         <v>646000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>730206</v>
+        <v>730576</v>
       </c>
       <c r="L10" t="n">
-        <v>17.14680514813628</v>
+        <v>17.18876612426359</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -12371,7 +12374,7 @@
         <v>615000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>558292</v>
+        <v>558574</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -12435,7 +12438,7 @@
         <v>700000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>644249</v>
+        <v>644575</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -12499,7 +12502,7 @@
         <v>745000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>687228</v>
+        <v>687575</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -12563,7 +12566,7 @@
         <v>930000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>859142</v>
+        <v>859576</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -12634,7 +12637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12683,7 +12686,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 MGE74 M5 Max 18 Core CPU 32 Core GPU 36GB 2TB Silver</t>
+          <t>Macbook Pro 14 M5 MJ3D4 10 Core CPU 10 Core GPU 32GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -12692,22 +12695,22 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>1210000</v>
+        <v>772000</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>1207000</v>
+        <v>745000</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-3000</v>
+        <v>-27000</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.25</v>
+        <v>-3.5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 MGED4 M5 Max 18 Core CPU 32 Core GPU 36GB 2TB Space Black</t>
+          <t>Apple MacBook Air Z1L2000VN 13 M5 10C CPU 10C GPU 24GB 2TB Silver</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -12716,45 +12719,93 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>1208000</v>
+        <v>756000</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>1207000</v>
+        <v>734999</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>-1000</v>
+        <v>-21001</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.08</v>
+        <v>-2.78</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MDVC4 M5 10C CPU 10C GPU 24GB 1TB Silver</t>
+          <t>Macbook Pro 14 M5 MJ3E4 10 Core CPU 10 Core GPU 32GB 1TB Silver</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>772000</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>755000</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>-17000</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-2.2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Macbook Pro 16 MGE94 M5 Max 18 Core CPU 40 Core GPU 48GB 2TB Silver</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="C4" s="3" t="n">
-        <v>616999</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>624999</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>8000</v>
-      </c>
-      <c r="F4" t="n">
-        <v>1.3</v>
+      <c r="C5" s="3" t="n">
+        <v>1430000</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>1460000</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>30000</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Macbook Pro 16 MGEE4 M5 Max 18 Core CPU 40 Core GPU 48GB 2TB Space Black</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>1425000</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>1460000</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>35000</v>
+      </c>
+      <c r="F6" t="n">
+        <v>2.46</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F4"/>
-  <conditionalFormatting sqref="E2:E4">
+  <autoFilter ref="A1:F6"/>
+  <conditionalFormatting sqref="E2:E6">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
chore: price data 2026-09-20
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MacBook Pro'!$A$1:$S$92</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MacBook Air'!$A$1:$S$68</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20260919T080651505066+0000</t>
+          <t>20260920T083919656362+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-19T08:06:51.505066+00:00</t>
+          <t>2026-09-20T08:39:19.656362+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>277.421451</v>
+        <v>278.631272</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -687,7 +687,7 @@
         <v>532000</v>
       </c>
       <c r="D20" t="n">
-        <v>51.6</v>
+        <v>51.7</v>
       </c>
       <c r="E20" t="n">
         <v>4</v>
@@ -708,7 +708,7 @@
         <v>810000</v>
       </c>
       <c r="D21" t="n">
-        <v>50.6</v>
+        <v>50.7</v>
       </c>
       <c r="E21" t="n">
         <v>4</v>
@@ -771,7 +771,7 @@
         <v>700000</v>
       </c>
       <c r="D24" t="n">
-        <v>49.6</v>
+        <v>49.7</v>
       </c>
       <c r="E24" t="n">
         <v>4</v>
@@ -792,7 +792,7 @@
         <v>847999</v>
       </c>
       <c r="D25" t="n">
-        <v>47.4</v>
+        <v>47.5</v>
       </c>
       <c r="E25" t="n">
         <v>5</v>
@@ -813,7 +813,7 @@
         <v>745000</v>
       </c>
       <c r="D26" t="n">
-        <v>45.4</v>
+        <v>45.5</v>
       </c>
       <c r="E26" t="n">
         <v>4</v>
@@ -831,10 +831,10 @@
         </is>
       </c>
       <c r="C27" s="3" t="n">
-        <v>645000</v>
+        <v>643999</v>
       </c>
       <c r="D27" t="n">
-        <v>44.7</v>
+        <v>44.9</v>
       </c>
       <c r="E27" t="n">
         <v>4</v>
@@ -843,7 +843,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 MJLV4 M5 Pro 15 Core CPU 16 Core GPU 24GB 2TB Silver</t>
+          <t>Macbook Pro 14 MGDR4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -852,10 +852,10 @@
         </is>
       </c>
       <c r="C28" s="3" t="n">
-        <v>815000</v>
+        <v>724999</v>
       </c>
       <c r="D28" t="n">
-        <v>44.6</v>
+        <v>44.8</v>
       </c>
       <c r="E28" t="n">
         <v>3</v>
@@ -864,7 +864,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 MGDR4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Space Black</t>
+          <t>Macbook Pro 14 MJLV4 M5 Pro 15 Core CPU 16 Core GPU 24GB 2TB Silver</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -873,10 +873,10 @@
         </is>
       </c>
       <c r="C29" s="3" t="n">
-        <v>728000</v>
+        <v>815000</v>
       </c>
       <c r="D29" t="n">
-        <v>44.4</v>
+        <v>44.6</v>
       </c>
       <c r="E29" t="n">
         <v>3</v>
@@ -885,7 +885,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 MGEC4 M5 Pro 18 Core CPU 20 Core GPU 48GB 1TB Space Black</t>
+          <t>Macbook Pro 14 MGDN4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Silver</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -894,13 +894,13 @@
         </is>
       </c>
       <c r="C30" s="3" t="n">
-        <v>1063000</v>
+        <v>729999</v>
       </c>
       <c r="D30" t="n">
-        <v>43.7</v>
+        <v>43.6</v>
       </c>
       <c r="E30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31">
@@ -918,7 +918,7 @@
         <v>551999</v>
       </c>
       <c r="D31" t="n">
-        <v>43.3</v>
+        <v>43.4</v>
       </c>
       <c r="E31" t="n">
         <v>4</v>
@@ -1147,10 +1147,10 @@
         <v>470000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>687575</v>
+        <v>690574</v>
       </c>
       <c r="L2" t="n">
-        <v>35.27978765952805</v>
+        <v>35.560852276512</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1165,7 +1165,7 @@
         <v>9.365994236311199</v>
       </c>
       <c r="Q2" t="n">
-        <v>32.5</v>
+        <v>32.6</v>
       </c>
       <c r="R2" t="n">
         <v>5</v>
@@ -1214,10 +1214,10 @@
         <v>465000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>687575</v>
+        <v>690574</v>
       </c>
       <c r="L3" t="n">
-        <v>33.38908482710977</v>
+        <v>33.67836032054494</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -1232,7 +1232,7 @@
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>10.2</v>
+        <v>10.3</v>
       </c>
       <c r="R3" t="n">
         <v>5</v>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>773576</v>
+        <v>776949</v>
       </c>
       <c r="L4" t="n">
-        <v>35.36523883884712</v>
+        <v>35.6458403318622</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1299,7 +1299,7 @@
         <v>59.79881123919307</v>
       </c>
       <c r="Q4" t="n">
-        <v>40.5</v>
+        <v>40.6</v>
       </c>
       <c r="R4" t="n">
         <v>5</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>773576</v>
+        <v>776949</v>
       </c>
       <c r="L5" t="n">
-        <v>32.77984322160977</v>
+        <v>33.07166879679361</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1366,7 +1366,7 @@
         <v>48.9918948126801</v>
       </c>
       <c r="Q5" t="n">
-        <v>17.7</v>
+        <v>17.8</v>
       </c>
       <c r="R5" t="n">
         <v>5</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>859576</v>
+        <v>863325</v>
       </c>
       <c r="L6" t="n">
-        <v>38.10902119184342</v>
+        <v>38.37778356933947</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1433,7 +1433,7 @@
         <v>100</v>
       </c>
       <c r="Q6" t="n">
-        <v>51.6</v>
+        <v>51.7</v>
       </c>
       <c r="R6" t="n">
         <v>4</v>
@@ -1600,10 +1600,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>859576</v>
+        <v>863325</v>
       </c>
       <c r="L9" t="n">
-        <v>34.26991912291641</v>
+        <v>34.55535285089624</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1618,7 +1618,7 @@
         <v>85.73487031700287</v>
       </c>
       <c r="Q9" t="n">
-        <v>25.7</v>
+        <v>25.8</v>
       </c>
       <c r="R9" t="n">
         <v>4</v>
@@ -1667,10 +1667,10 @@
         <v>582999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>859576</v>
+        <v>863325</v>
       </c>
       <c r="L10" t="n">
-        <v>32.17597978538256</v>
+        <v>32.47050647207019</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -1685,7 +1685,7 @@
         <v>50.10670212765957</v>
       </c>
       <c r="Q10" t="n">
-        <v>41.3</v>
+        <v>41.4</v>
       </c>
       <c r="R10" t="n">
         <v>4</v>
@@ -1734,10 +1734,10 @@
         <v>587999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>859576</v>
+        <v>863325</v>
       </c>
       <c r="L11" t="n">
-        <v>31.59429765372695</v>
+        <v>31.8913503026091</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -1752,7 +1752,7 @@
         <v>48.51095744680851</v>
       </c>
       <c r="Q11" t="n">
-        <v>18.6</v>
+        <v>18.7</v>
       </c>
       <c r="R11" t="n">
         <v>4</v>
@@ -1795,19 +1795,19 @@
         </is>
       </c>
       <c r="I12" s="3" t="n">
-        <v>645000</v>
+        <v>643999</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>645000</v>
+        <v>643999</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>945577</v>
+        <v>949701</v>
       </c>
       <c r="L12" t="n">
-        <v>31.78768096093708</v>
+        <v>32.18928904992202</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>0</v>
+        <v>-1001</v>
       </c>
       <c r="N12" t="n">
         <v>0</v>
@@ -1816,10 +1816,10 @@
         <v>100</v>
       </c>
       <c r="P12" t="n">
-        <v>71.48936170212767</v>
+        <v>71.74493617021277</v>
       </c>
       <c r="Q12" t="n">
-        <v>44.7</v>
+        <v>44.9</v>
       </c>
       <c r="R12" t="n">
         <v>4</v>
@@ -1927,10 +1927,10 @@
         <v>650000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>945577</v>
+        <v>949701</v>
       </c>
       <c r="L14" t="n">
-        <v>31.2589032939676</v>
+        <v>31.5574059625082</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -1945,7 +1945,7 @@
         <v>70.21276595744681</v>
       </c>
       <c r="Q14" t="n">
-        <v>22.1</v>
+        <v>22.2</v>
       </c>
       <c r="R14" t="n">
         <v>4</v>
@@ -1994,10 +1994,10 @@
         <v>650000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>859576</v>
+        <v>863325</v>
       </c>
       <c r="L15" t="n">
-        <v>24.3813228847711</v>
+        <v>24.70969797005763</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0</v>
@@ -2009,7 +2009,7 @@
         <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>10.4</v>
+        <v>10.6</v>
       </c>
       <c r="R15" t="n">
         <v>3</v>
@@ -2058,10 +2058,10 @@
         <v>650000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>859576</v>
+        <v>863325</v>
       </c>
       <c r="L16" t="n">
-        <v>24.3813228847711</v>
+        <v>24.70969797005763</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -2073,7 +2073,7 @@
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>10.4</v>
+        <v>10.6</v>
       </c>
       <c r="R16" t="n">
         <v>3</v>
@@ -2122,10 +2122,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1031578</v>
+        <v>1036076</v>
       </c>
       <c r="L17" t="n">
-        <v>32.14279482501566</v>
+        <v>32.43738876298649</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2140,7 +2140,7 @@
         <v>100</v>
       </c>
       <c r="Q17" t="n">
-        <v>49.6</v>
+        <v>49.7</v>
       </c>
       <c r="R17" t="n">
         <v>4</v>
@@ -2189,10 +2189,10 @@
         <v>707999</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>1074578</v>
+        <v>1079264</v>
       </c>
       <c r="L18" t="n">
-        <v>34.11376372864511</v>
+        <v>34.39983173718386</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -2207,7 +2207,7 @@
         <v>12.49398266190719</v>
       </c>
       <c r="Q18" t="n">
-        <v>35.7</v>
+        <v>35.8</v>
       </c>
       <c r="R18" t="n">
         <v>4</v>
@@ -2256,10 +2256,10 @@
         <v>720000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>1031578</v>
+        <v>1036076</v>
       </c>
       <c r="L19" t="n">
-        <v>30.20401753430182</v>
+        <v>30.50702844192897</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -2274,7 +2274,7 @@
         <v>82.22222222222221</v>
       </c>
       <c r="Q19" t="n">
-        <v>23.8</v>
+        <v>23.9</v>
       </c>
       <c r="R19" t="n">
         <v>4</v>
@@ -2317,26 +2317,26 @@
         </is>
       </c>
       <c r="I20" s="3" t="n">
-        <v>728000</v>
+        <v>724999</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>728000</v>
+        <v>724999</v>
       </c>
       <c r="K20" s="3" t="n"/>
       <c r="M20" s="3" t="n">
-        <v>0</v>
+        <v>-3001</v>
       </c>
       <c r="N20" t="n">
-        <v>0</v>
+        <v>0.4122252747252748</v>
       </c>
       <c r="O20" t="n">
         <v>100</v>
       </c>
       <c r="P20" t="n">
-        <v>44.38356164383562</v>
+        <v>45.20575342465755</v>
       </c>
       <c r="Q20" t="n">
-        <v>44.4</v>
+        <v>44.8</v>
       </c>
       <c r="R20" t="n">
         <v>3</v>
@@ -2379,26 +2379,26 @@
         </is>
       </c>
       <c r="I21" s="3" t="n">
-        <v>735000</v>
+        <v>729999</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>735000</v>
+        <v>729999</v>
       </c>
       <c r="K21" s="3" t="n"/>
       <c r="M21" s="3" t="n">
-        <v>0</v>
+        <v>-5001</v>
       </c>
       <c r="N21" t="n">
-        <v>0</v>
+        <v>0.6804081632653061</v>
       </c>
       <c r="O21" t="n">
-        <v>95.67901234567901</v>
+        <v>96.96971533505857</v>
       </c>
       <c r="P21" t="n">
-        <v>42.46575342465754</v>
+        <v>43.83589041095892</v>
       </c>
       <c r="Q21" t="n">
-        <v>42.5</v>
+        <v>43.6</v>
       </c>
       <c r="R21" t="n">
         <v>3</v>
@@ -2447,10 +2447,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1074578</v>
+        <v>1079264</v>
       </c>
       <c r="L22" t="n">
-        <v>30.85657811717716</v>
+        <v>31.15678832982477</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2465,7 +2465,7 @@
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>10.3</v>
+        <v>10.4</v>
       </c>
       <c r="R22" t="n">
         <v>4</v>
@@ -2514,13 +2514,13 @@
         <v>745000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1031578</v>
+        <v>1036076</v>
       </c>
       <c r="L23" t="n">
-        <v>27.78054592090952</v>
+        <v>28.09407804060706</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>-27000</v>
+        <v>0</v>
       </c>
       <c r="N23" t="n">
         <v>3.49740932642487</v>
@@ -2532,7 +2532,7 @@
         <v>77.6595744680851</v>
       </c>
       <c r="Q23" t="n">
-        <v>45.4</v>
+        <v>45.5</v>
       </c>
       <c r="R23" t="n">
         <v>4</v>
@@ -2581,13 +2581,13 @@
         <v>755000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1031578</v>
+        <v>1036076</v>
       </c>
       <c r="L24" t="n">
-        <v>26.8111572755526</v>
+        <v>27.12889788007829</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>-17000</v>
+        <v>0</v>
       </c>
       <c r="N24" t="n">
         <v>2.202072538860103</v>
@@ -2599,7 +2599,7 @@
         <v>75.53191489361704</v>
       </c>
       <c r="Q24" t="n">
-        <v>36.1</v>
+        <v>36.2</v>
       </c>
       <c r="R24" t="n">
         <v>4</v>
@@ -2648,10 +2648,10 @@
         <v>772000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>1031578</v>
+        <v>1036076</v>
       </c>
       <c r="L25" t="n">
-        <v>25.16319657844584</v>
+        <v>25.4880916071794</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -2666,7 +2666,7 @@
         <v>71.91489361702126</v>
       </c>
       <c r="Q25" t="n">
-        <v>20.4</v>
+        <v>20.5</v>
       </c>
       <c r="R25" t="n">
         <v>4</v>
@@ -2777,10 +2777,10 @@
         <v>810000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>1246579</v>
+        <v>1252016</v>
       </c>
       <c r="L27" t="n">
-        <v>35.0221686712194</v>
+        <v>35.30434115857945</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -2795,7 +2795,7 @@
         <v>100</v>
       </c>
       <c r="Q27" t="n">
-        <v>50.6</v>
+        <v>50.7</v>
       </c>
       <c r="R27" t="n">
         <v>4</v>
@@ -2900,31 +2900,31 @@
         </is>
       </c>
       <c r="I29" s="3" t="n">
-        <v>832999</v>
+        <v>829999</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>832999</v>
+        <v>829999</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>1289580</v>
+        <v>1295204</v>
       </c>
       <c r="L29" t="n">
-        <v>35.40540330960468</v>
+        <v>35.91750797557759</v>
       </c>
       <c r="M29" s="3" t="n">
-        <v>0</v>
+        <v>-3000</v>
       </c>
       <c r="N29" t="n">
-        <v>0</v>
+        <v>0.3601444899693757</v>
       </c>
       <c r="O29" t="n">
         <v>100</v>
       </c>
       <c r="P29" t="n">
-        <v>11.91179074446682</v>
+        <v>3.563830734966613</v>
       </c>
       <c r="Q29" t="n">
-        <v>36</v>
+        <v>34.9</v>
       </c>
       <c r="R29" t="n">
         <v>4</v>
@@ -2973,10 +2973,10 @@
         <v>835000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1074578</v>
+        <v>1079264</v>
       </c>
       <c r="L30" t="n">
-        <v>22.29507769561632</v>
+        <v>22.63246063984345</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -2988,7 +2988,7 @@
         <v>58.51063829787235</v>
       </c>
       <c r="Q30" t="n">
-        <v>22.1</v>
+        <v>22.2</v>
       </c>
       <c r="R30" t="n">
         <v>3</v>
@@ -3002,63 +3002,63 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 14Inch MX2K3 14Core CPU 32Core GPU M4 Max 36GB 1TB Space Black</t>
+          <t>Macbook Pro 16 MGE44 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Silver</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>M4 Max</t>
+          <t>M5 Pro</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="E31" t="n">
         <v>1024</v>
       </c>
       <c r="F31" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G31" t="n">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I31" s="3" t="n">
-        <v>847999</v>
+        <v>840000</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>930000</v>
+        <v>840000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1375580</v>
+        <v>1295204</v>
       </c>
       <c r="L31" t="n">
-        <v>38.35334913272947</v>
+        <v>35.1453516202853</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>0</v>
+        <v>-30000</v>
       </c>
       <c r="N31" t="n">
-        <v>0</v>
+        <v>3.448275862068965</v>
       </c>
       <c r="O31" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="P31" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="Q31" t="n">
-        <v>47.4</v>
+        <v>12.7</v>
       </c>
       <c r="R31" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S31" t="inlineStr">
         <is>
@@ -3069,7 +3069,7 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 14Inch MX2G3 14Core CPU 32Core GPU M4 Max 36GB 1TB Silver</t>
+          <t>Apple MacBook Pro 14Inch MX2K3 14Core CPU 32Core GPU M4 Max 36GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -3094,20 +3094,20 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I32" s="3" t="n">
-        <v>849999</v>
+        <v>847999</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1375580</v>
+        <v>1381579</v>
       </c>
       <c r="L32" t="n">
-        <v>38.20795591677692</v>
+        <v>38.62102710015135</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3116,13 +3116,13 @@
         <v>0</v>
       </c>
       <c r="O32" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="P32" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q32" t="n">
-        <v>12.3</v>
+        <v>47.5</v>
       </c>
       <c r="R32" t="n">
         <v>5</v>
@@ -3136,45 +3136,45 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 16Inch MX2Y3 14Core CPU 20Core GPU M4 Pro 48GB 512GB Space Black</t>
+          <t>Apple MacBook Pro 14Inch MX2G3 14Core CPU 32Core GPU M4 Max 36GB 1TB Silver</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>M4 Pro</t>
+          <t>M4 Max</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="E33" t="n">
-        <v>512</v>
+        <v>1024</v>
       </c>
       <c r="F33" t="n">
         <v>14</v>
       </c>
       <c r="G33" t="n">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I33" s="3" t="n">
-        <v>860000</v>
+        <v>849999</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>860000</v>
+        <v>930000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1246579</v>
+        <v>1381579</v>
       </c>
       <c r="L33" t="n">
-        <v>31.01119142870207</v>
+        <v>38.47626520090418</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3186,13 +3186,13 @@
         <v>0</v>
       </c>
       <c r="P33" t="n">
-        <v>89.80112187659357</v>
+        <v>0</v>
       </c>
       <c r="Q33" t="n">
-        <v>25.3</v>
+        <v>12.4</v>
       </c>
       <c r="R33" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S33" t="inlineStr">
         <is>
@@ -3203,25 +3203,25 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 MGDT4 M5 Pro 18 Core CPU 20 Core GPU 24GB 2TB Space Black</t>
+          <t>Apple MacBook Pro 16Inch MX2Y3 14Core CPU 20Core GPU M4 Pro 48GB 512GB Space Black</t>
         </is>
       </c>
       <c r="B34" t="n">
+        <v>16</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>M4 Pro</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>48</v>
+      </c>
+      <c r="E34" t="n">
+        <v>512</v>
+      </c>
+      <c r="F34" t="n">
         <v>14</v>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>M5 Pro</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>24</v>
-      </c>
-      <c r="E34" t="n">
-        <v>2048</v>
-      </c>
-      <c r="F34" t="n">
-        <v>18</v>
       </c>
       <c r="G34" t="n">
         <v>20</v>
@@ -3232,12 +3232,17 @@
         </is>
       </c>
       <c r="I34" s="3" t="n">
-        <v>864999</v>
+        <v>860000</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>864999</v>
-      </c>
-      <c r="K34" s="3" t="n"/>
+        <v>860000</v>
+      </c>
+      <c r="K34" s="3" t="n">
+        <v>1252016</v>
+      </c>
+      <c r="L34" t="n">
+        <v>31.31078197083743</v>
+      </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
       </c>
@@ -3245,16 +3250,16 @@
         <v>0</v>
       </c>
       <c r="O34" t="n">
-        <v>11.76588235294118</v>
+        <v>0</v>
       </c>
       <c r="P34" t="n">
-        <v>74.55988258317025</v>
+        <v>89.80112187659357</v>
       </c>
       <c r="Q34" t="n">
-        <v>22.6</v>
+        <v>25.4</v>
       </c>
       <c r="R34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S34" t="inlineStr">
         <is>
@@ -3265,11 +3270,11 @@
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 MGE44 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Silver</t>
+          <t>Macbook Pro 14 MGDT4 M5 Pro 18 Core CPU 20 Core GPU 24GB 2TB Space Black</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -3280,7 +3285,7 @@
         <v>24</v>
       </c>
       <c r="E35" t="n">
-        <v>1024</v>
+        <v>2048</v>
       </c>
       <c r="F35" t="n">
         <v>18</v>
@@ -3290,21 +3295,16 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I35" s="3" t="n">
-        <v>870000</v>
+        <v>864999</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>870000</v>
-      </c>
-      <c r="K35" s="3" t="n">
-        <v>1289580</v>
-      </c>
-      <c r="L35" t="n">
-        <v>32.53617456846415</v>
-      </c>
+        <v>864999</v>
+      </c>
+      <c r="K35" s="3" t="n"/>
       <c r="M35" s="3" t="n">
         <v>0</v>
       </c>
@@ -3312,16 +3312,16 @@
         <v>0</v>
       </c>
       <c r="O35" t="n">
-        <v>0</v>
+        <v>11.76588235294118</v>
       </c>
       <c r="P35" t="n">
-        <v>0</v>
+        <v>74.55988258317025</v>
       </c>
       <c r="Q35" t="n">
-        <v>10.8</v>
+        <v>22.6</v>
       </c>
       <c r="R35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S35" t="inlineStr">
         <is>
@@ -3491,10 +3491,10 @@
         <v>890000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>1160579</v>
+        <v>1165640</v>
       </c>
       <c r="L38" t="n">
-        <v>23.31413889101905</v>
+        <v>23.64709515802478</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -3506,7 +3506,7 @@
         <v>73.86018237082067</v>
       </c>
       <c r="Q38" t="n">
-        <v>25.8</v>
+        <v>26</v>
       </c>
       <c r="R38" t="n">
         <v>3</v>
@@ -3555,10 +3555,10 @@
         <v>960000</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>1246579</v>
+        <v>1252016</v>
       </c>
       <c r="L39" t="n">
-        <v>22.98923694366743</v>
+        <v>23.32366359535341</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -3570,7 +3570,7 @@
         <v>82.97872340425533</v>
       </c>
       <c r="Q39" t="n">
-        <v>27.6</v>
+        <v>27.8</v>
       </c>
       <c r="R39" t="n">
         <v>3</v>
@@ -3619,10 +3619,10 @@
         <v>970000</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>1504581</v>
+        <v>1511143</v>
       </c>
       <c r="L40" t="n">
-        <v>35.53022402914831</v>
+        <v>35.81017812344696</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -3637,7 +3637,7 @@
         <v>54.87506124448805</v>
       </c>
       <c r="Q40" t="n">
-        <v>43.2</v>
+        <v>43.3</v>
       </c>
       <c r="R40" t="n">
         <v>4</v>
@@ -3748,10 +3748,10 @@
         <v>1022000</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>1504581</v>
+        <v>1511143</v>
       </c>
       <c r="L42" t="n">
-        <v>32.07411232761812</v>
+        <v>32.36907427027091</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -3766,7 +3766,7 @@
         <v>14.11073003429697</v>
       </c>
       <c r="Q42" t="n">
-        <v>13</v>
+        <v>13.1</v>
       </c>
       <c r="R42" t="n">
         <v>4</v>
@@ -3815,10 +3815,10 @@
         <v>1063000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1547582</v>
+        <v>1554331</v>
       </c>
       <c r="L43" t="n">
-        <v>31.31220187363255</v>
+        <v>31.61044848233742</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -3830,10 +3830,10 @@
         <v>100</v>
       </c>
       <c r="P43" t="n">
-        <v>66.19718309859155</v>
+        <v>62.58351893095768</v>
       </c>
       <c r="Q43" t="n">
-        <v>43.7</v>
+        <v>43.2</v>
       </c>
       <c r="R43" t="n">
         <v>4</v>
@@ -3876,31 +3876,31 @@
         </is>
       </c>
       <c r="I44" s="3" t="n">
-        <v>1085000</v>
+        <v>1080000</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>1085000</v>
+        <v>1080000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1547582</v>
+        <v>1554331</v>
       </c>
       <c r="L44" t="n">
-        <v>29.89062938183567</v>
+        <v>30.51673034894112</v>
       </c>
       <c r="M44" s="3" t="n">
-        <v>0</v>
+        <v>-5000</v>
       </c>
       <c r="N44" t="n">
-        <v>0</v>
+        <v>0.4608294930875576</v>
       </c>
       <c r="O44" t="n">
         <v>0</v>
       </c>
       <c r="P44" t="n">
-        <v>61.77062374245473</v>
+        <v>58.79732739420935</v>
       </c>
       <c r="Q44" t="n">
-        <v>20.3</v>
+        <v>20.1</v>
       </c>
       <c r="R44" t="n">
         <v>4</v>
@@ -4011,10 +4011,10 @@
         <v>1123000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1719583</v>
+        <v>1727082</v>
       </c>
       <c r="L46" t="n">
-        <v>34.69346928877524</v>
+        <v>34.97703062159179</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -4078,10 +4078,10 @@
         <v>1150000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1504581</v>
+        <v>1511143</v>
       </c>
       <c r="L47" t="n">
-        <v>23.56676044692841</v>
+        <v>23.8986647855299</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -4093,7 +4093,7 @@
         <v>89.36170212765958</v>
       </c>
       <c r="Q47" t="n">
-        <v>29.2</v>
+        <v>29.4</v>
       </c>
       <c r="R47" t="n">
         <v>3</v>
@@ -4142,10 +4142,10 @@
         <v>1150000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1504581</v>
+        <v>1511143</v>
       </c>
       <c r="L48" t="n">
-        <v>23.56676044692841</v>
+        <v>23.8986647855299</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -4154,10 +4154,10 @@
         <v>0</v>
       </c>
       <c r="P48" t="n">
-        <v>15.6366772060937</v>
+        <v>6.617881005408838</v>
       </c>
       <c r="Q48" t="n">
-        <v>13.5</v>
+        <v>11.7</v>
       </c>
       <c r="R48" t="n">
         <v>3</v>
@@ -4206,10 +4206,10 @@
         <v>1155000</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>1762583</v>
+        <v>1770270</v>
       </c>
       <c r="L49" t="n">
-        <v>34.47117100301092</v>
+        <v>34.75571522988019</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -4221,7 +4221,7 @@
         <v>30.94208045457479</v>
       </c>
       <c r="Q49" t="n">
-        <v>21.4</v>
+        <v>21.5</v>
       </c>
       <c r="R49" t="n">
         <v>3</v>
@@ -4270,10 +4270,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1762583</v>
+        <v>1770270</v>
       </c>
       <c r="L50" t="n">
-        <v>34.47117100301092</v>
+        <v>34.75571522988019</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4285,7 +4285,7 @@
         <v>30.94208045457479</v>
       </c>
       <c r="Q50" t="n">
-        <v>21.4</v>
+        <v>21.5</v>
       </c>
       <c r="R50" t="n">
         <v>3</v>
@@ -4396,10 +4396,10 @@
         <v>1207000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1891584</v>
+        <v>1899833</v>
       </c>
       <c r="L52" t="n">
-        <v>36.1910441196373</v>
+        <v>36.46810009090273</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -4411,7 +4411,7 @@
         <v>9.265033407572403</v>
       </c>
       <c r="Q52" t="n">
-        <v>17.5</v>
+        <v>17.6</v>
       </c>
       <c r="R52" t="n">
         <v>3</v>
@@ -4460,10 +4460,10 @@
         <v>1207000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1891584</v>
+        <v>1899833</v>
       </c>
       <c r="L53" t="n">
-        <v>36.1910441196373</v>
+        <v>36.46810009090273</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -4475,7 +4475,7 @@
         <v>9.265033407572403</v>
       </c>
       <c r="Q53" t="n">
-        <v>17.6</v>
+        <v>17.7</v>
       </c>
       <c r="R53" t="n">
         <v>3</v>
@@ -4524,10 +4524,10 @@
         <v>1210000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1590582</v>
+        <v>1597518</v>
       </c>
       <c r="L54" t="n">
-        <v>23.9272165785857</v>
+        <v>24.25750445378393</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -4539,7 +4539,7 @@
         <v>95.74468085106383</v>
       </c>
       <c r="Q54" t="n">
-        <v>30.8</v>
+        <v>30.9</v>
       </c>
       <c r="R54" t="n">
         <v>3</v>
@@ -4588,10 +4588,10 @@
         <v>1215000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1590582</v>
+        <v>1597518</v>
       </c>
       <c r="L55" t="n">
-        <v>23.61286623386911</v>
+        <v>23.94451893499792</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -4603,7 +4603,7 @@
         <v>77.39726027397261</v>
       </c>
       <c r="Q55" t="n">
-        <v>26.7</v>
+        <v>26.8</v>
       </c>
       <c r="R55" t="n">
         <v>3</v>
@@ -4714,10 +4714,10 @@
         <v>1280000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1676583</v>
+        <v>1683894</v>
       </c>
       <c r="L57" t="n">
-        <v>23.65424199100194</v>
+        <v>23.98571406513712</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -4729,7 +4729,7 @@
         <v>100</v>
       </c>
       <c r="Q57" t="n">
-        <v>31.6</v>
+        <v>31.7</v>
       </c>
       <c r="R57" t="n">
         <v>3</v>
@@ -4778,10 +4778,10 @@
         <v>1280000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>1719583</v>
+        <v>1727082</v>
       </c>
       <c r="L58" t="n">
-        <v>25.56334878863073</v>
+        <v>25.88655315729074</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -4796,7 +4796,7 @@
         <v>0</v>
       </c>
       <c r="Q58" t="n">
-        <v>8.5</v>
+        <v>8.6</v>
       </c>
       <c r="R58" t="n">
         <v>4</v>
@@ -4845,10 +4845,10 @@
         <v>1310000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1719583</v>
+        <v>1727082</v>
       </c>
       <c r="L59" t="n">
-        <v>23.81873977586427</v>
+        <v>24.14951924691474</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -4857,10 +4857,10 @@
         <v>0</v>
       </c>
       <c r="P59" t="n">
-        <v>69.21529175050301</v>
+        <v>65.92427616926503</v>
       </c>
       <c r="Q59" t="n">
-        <v>25</v>
+        <v>24.5</v>
       </c>
       <c r="R59" t="n">
         <v>3</v>
@@ -4909,10 +4909,10 @@
         <v>1338000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1762583</v>
+        <v>1770270</v>
       </c>
       <c r="L60" t="n">
-        <v>24.08868121387759</v>
+        <v>24.41830907149757</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -4921,10 +4921,10 @@
         <v>0</v>
       </c>
       <c r="P60" t="n">
-        <v>64.70824949698189</v>
+        <v>60.93541202672606</v>
       </c>
       <c r="Q60" t="n">
-        <v>24.2</v>
+        <v>23.5</v>
       </c>
       <c r="R60" t="n">
         <v>3</v>
@@ -4973,10 +4973,10 @@
         <v>1370000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1805584</v>
+        <v>1813458</v>
       </c>
       <c r="L61" t="n">
-        <v>24.12427225761859</v>
+        <v>24.45372321829345</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -4988,7 +4988,7 @@
         <v>87.44292237442922</v>
       </c>
       <c r="Q61" t="n">
-        <v>29.1</v>
+        <v>29.2</v>
       </c>
       <c r="R61" t="n">
         <v>3</v>
@@ -5096,13 +5096,13 @@
         <v>1460000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>2149586</v>
+        <v>2158960</v>
       </c>
       <c r="L63" t="n">
-        <v>32.07994469632757</v>
+        <v>32.37484714862712</v>
       </c>
       <c r="M63" s="3" t="n">
-        <v>30000</v>
+        <v>0</v>
       </c>
       <c r="N63" t="n">
         <v>0</v>
@@ -5111,7 +5111,7 @@
         <v>0.7126948775055885</v>
       </c>
       <c r="Q63" t="n">
-        <v>13.9</v>
+        <v>14</v>
       </c>
       <c r="R63" t="n">
         <v>3</v>
@@ -5160,13 +5160,13 @@
         <v>1460000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>2149586</v>
+        <v>2158960</v>
       </c>
       <c r="L64" t="n">
-        <v>32.07994469632757</v>
+        <v>32.37484714862712</v>
       </c>
       <c r="M64" s="3" t="n">
-        <v>35000</v>
+        <v>0</v>
       </c>
       <c r="N64" t="n">
         <v>0</v>
@@ -5175,7 +5175,7 @@
         <v>0.7126948775055885</v>
       </c>
       <c r="Q64" t="n">
-        <v>13.9</v>
+        <v>14</v>
       </c>
       <c r="R64" t="n">
         <v>3</v>
@@ -5224,10 +5224,10 @@
         <v>1471000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1934585</v>
+        <v>1943021</v>
       </c>
       <c r="L65" t="n">
-        <v>23.96302049276718</v>
+        <v>24.29314968803734</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -5236,10 +5236,10 @@
         <v>0</v>
       </c>
       <c r="P65" t="n">
-        <v>82.76324614352785</v>
+        <v>80.92056421677803</v>
       </c>
       <c r="Q65" t="n">
-        <v>28</v>
+        <v>27.8</v>
       </c>
       <c r="R65" t="n">
         <v>3</v>
@@ -5288,10 +5288,10 @@
         <v>1471000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1934585</v>
+        <v>1943021</v>
       </c>
       <c r="L66" t="n">
-        <v>23.96302049276718</v>
+        <v>24.29314968803734</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -5300,10 +5300,10 @@
         <v>0</v>
       </c>
       <c r="P66" t="n">
-        <v>64.82531552954087</v>
+        <v>61.06499291354523</v>
       </c>
       <c r="Q66" t="n">
-        <v>24.2</v>
+        <v>23.5</v>
       </c>
       <c r="R66" t="n">
         <v>3</v>
@@ -5414,10 +5414,10 @@
         <v>1535000</v>
       </c>
       <c r="K68" s="3" t="n">
-        <v>2020585</v>
+        <v>2029397</v>
       </c>
       <c r="L68" t="n">
-        <v>24.03190165224428</v>
+        <v>24.36176854504072</v>
       </c>
       <c r="M68" s="3" t="n">
         <v>0</v>
@@ -5429,7 +5429,7 @@
         <v>0</v>
       </c>
       <c r="Q68" t="n">
-        <v>10.3</v>
+        <v>10.4</v>
       </c>
       <c r="R68" t="n">
         <v>3</v>
@@ -5540,10 +5540,10 @@
         <v>1650000</v>
       </c>
       <c r="K70" s="3" t="n">
-        <v>2192587</v>
+        <v>2202148</v>
       </c>
       <c r="L70" t="n">
-        <v>24.74642967417028</v>
+        <v>25.07315584601943</v>
       </c>
       <c r="M70" s="3" t="n">
         <v>0</v>
@@ -5555,7 +5555,7 @@
         <v>37.76070252469814</v>
       </c>
       <c r="Q70" t="n">
-        <v>18.7</v>
+        <v>18.8</v>
       </c>
       <c r="R70" t="n">
         <v>3</v>
@@ -5604,10 +5604,10 @@
         <v>1660000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2192587</v>
+        <v>2202148</v>
       </c>
       <c r="L71" t="n">
-        <v>24.29034742977132</v>
+        <v>24.61905376023773</v>
       </c>
       <c r="M71" s="3" t="n">
         <v>0</v>
@@ -5619,7 +5619,7 @@
         <v>26.6373948042444</v>
       </c>
       <c r="Q71" t="n">
-        <v>16.1</v>
+        <v>16.3</v>
       </c>
       <c r="R71" t="n">
         <v>3</v>
@@ -5668,10 +5668,10 @@
         <v>1661000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2192587</v>
+        <v>2202148</v>
       </c>
       <c r="L72" t="n">
-        <v>24.24473920533142</v>
+        <v>24.57364355165956</v>
       </c>
       <c r="M72" s="3" t="n">
         <v>0</v>
@@ -5680,10 +5680,10 @@
         <v>0</v>
       </c>
       <c r="P72" t="n">
-        <v>89.10606496119574</v>
+        <v>87.94145720649061</v>
       </c>
       <c r="Q72" t="n">
-        <v>29.5</v>
+        <v>29.4</v>
       </c>
       <c r="R72" t="n">
         <v>3</v>
@@ -5732,10 +5732,10 @@
         <v>1680000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2235587</v>
+        <v>2245336</v>
       </c>
       <c r="L73" t="n">
-        <v>24.85195163507392</v>
+        <v>25.17823613036089</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
@@ -5747,7 +5747,7 @@
         <v>100</v>
       </c>
       <c r="Q73" t="n">
-        <v>32.1</v>
+        <v>32.2</v>
       </c>
       <c r="R73" t="n">
         <v>3</v>
@@ -5796,10 +5796,10 @@
         <v>1711000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2321588</v>
+        <v>2331712</v>
       </c>
       <c r="L74" t="n">
-        <v>26.30044607398039</v>
+        <v>26.62044026020366</v>
       </c>
       <c r="M74" s="3" t="n">
         <v>0</v>
@@ -5811,7 +5811,7 @@
         <v>20.21202672605792</v>
       </c>
       <c r="Q74" t="n">
-        <v>15.6</v>
+        <v>15.7</v>
       </c>
       <c r="R74" t="n">
         <v>3</v>
@@ -5860,10 +5860,10 @@
         <v>1756000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2321588</v>
+        <v>2331712</v>
       </c>
       <c r="L75" t="n">
-        <v>24.36211765395066</v>
+        <v>24.69052781818681</v>
       </c>
       <c r="M75" s="3" t="n">
         <v>0</v>
@@ -5875,7 +5875,7 @@
         <v>0</v>
       </c>
       <c r="Q75" t="n">
-        <v>10.4</v>
+        <v>10.6</v>
       </c>
       <c r="R75" t="n">
         <v>3</v>
@@ -5924,10 +5924,10 @@
         <v>1790000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2364588</v>
+        <v>2374900</v>
       </c>
       <c r="L76" t="n">
-        <v>24.29970887105915</v>
+        <v>24.62840540654343</v>
       </c>
       <c r="M76" s="3" t="n">
         <v>0</v>
@@ -5939,7 +5939,7 @@
         <v>100</v>
       </c>
       <c r="Q76" t="n">
-        <v>31.8</v>
+        <v>32</v>
       </c>
       <c r="R76" t="n">
         <v>3</v>
@@ -5988,10 +5988,10 @@
         <v>1840000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2450589</v>
+        <v>2461275</v>
       </c>
       <c r="L77" t="n">
-        <v>24.91600998780293</v>
+        <v>25.24199855765812</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
@@ -6003,7 +6003,7 @@
         <v>38.76430923631803</v>
       </c>
       <c r="Q77" t="n">
-        <v>19</v>
+        <v>19.1</v>
       </c>
       <c r="R77" t="n">
         <v>3</v>
@@ -6052,10 +6052,10 @@
         <v>1945000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2579589</v>
+        <v>2590839</v>
       </c>
       <c r="L78" t="n">
-        <v>24.60039176783588</v>
+        <v>24.92779366066359</v>
       </c>
       <c r="M78" s="3" t="n">
         <v>0</v>
@@ -6067,7 +6067,7 @@
         <v>15.83200763601658</v>
       </c>
       <c r="Q78" t="n">
-        <v>13.9</v>
+        <v>14.1</v>
       </c>
       <c r="R78" t="n">
         <v>3</v>
@@ -6116,10 +6116,10 @@
         <v>1960000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2622590</v>
+        <v>2634027</v>
       </c>
       <c r="L79" t="n">
-        <v>25.26471922793879</v>
+        <v>25.58922137092748</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
@@ -6131,7 +6131,7 @@
         <v>54.4456641053787</v>
       </c>
       <c r="Q79" t="n">
-        <v>22.5</v>
+        <v>22.6</v>
       </c>
       <c r="R79" t="n">
         <v>3</v>
@@ -6180,10 +6180,10 @@
         <v>2078000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2751591</v>
+        <v>2763590</v>
       </c>
       <c r="L80" t="n">
-        <v>24.48005535706433</v>
+        <v>24.80794908072471</v>
       </c>
       <c r="M80" s="3" t="n">
         <v>0</v>
@@ -6195,7 +6195,7 @@
         <v>35.18930957683743</v>
       </c>
       <c r="Q80" t="n">
-        <v>18</v>
+        <v>18.2</v>
       </c>
       <c r="R80" t="n">
         <v>3</v>
@@ -6244,10 +6244,10 @@
         <v>2170000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2880592</v>
+        <v>2893154</v>
       </c>
       <c r="L81" t="n">
-        <v>24.66826263490283</v>
+        <v>24.99535109434202</v>
       </c>
       <c r="M81" s="3" t="n">
         <v>0</v>
@@ -6259,7 +6259,7 @@
         <v>79.03402854006586</v>
       </c>
       <c r="Q81" t="n">
-        <v>27.5</v>
+        <v>27.6</v>
       </c>
       <c r="R81" t="n">
         <v>3</v>
@@ -6308,10 +6308,10 @@
         <v>2268000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>3009593</v>
+        <v>3022717</v>
       </c>
       <c r="L82" t="n">
-        <v>24.6409730485152</v>
+        <v>24.968166057226</v>
       </c>
       <c r="M82" s="3" t="n">
         <v>0</v>
@@ -6323,7 +6323,7 @@
         <v>70.41425389755011</v>
       </c>
       <c r="Q82" t="n">
-        <v>25.6</v>
+        <v>25.8</v>
       </c>
       <c r="R82" t="n">
         <v>3</v>
@@ -6372,10 +6372,10 @@
         <v>2270000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3052593</v>
+        <v>3065905</v>
       </c>
       <c r="L83" t="n">
-        <v>25.63699123990653</v>
+        <v>25.95987155505471</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
@@ -6387,7 +6387,7 @@
         <v>75.11445476694064</v>
       </c>
       <c r="Q83" t="n">
-        <v>27.1</v>
+        <v>27.2</v>
       </c>
       <c r="R83" t="n">
         <v>3</v>
@@ -6436,10 +6436,10 @@
         <v>2381000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3181594</v>
+        <v>3195469</v>
       </c>
       <c r="L84" t="n">
-        <v>25.16329864841334</v>
+        <v>25.48824601333951</v>
       </c>
       <c r="M84" s="3" t="n">
         <v>0</v>
@@ -6451,7 +6451,7 @@
         <v>64.54234341897987</v>
       </c>
       <c r="Q84" t="n">
-        <v>24.6</v>
+        <v>24.8</v>
       </c>
       <c r="R84" t="n">
         <v>3</v>
@@ -6500,10 +6500,10 @@
         <v>2470000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3310595</v>
+        <v>3325032</v>
       </c>
       <c r="L85" t="n">
-        <v>25.39105508224353</v>
+        <v>25.71500063758785</v>
       </c>
       <c r="M85" s="3" t="n">
         <v>0</v>
@@ -6515,7 +6515,7 @@
         <v>88.84010245151846</v>
       </c>
       <c r="Q85" t="n">
-        <v>29.9</v>
+        <v>30.1</v>
       </c>
       <c r="R85" t="n">
         <v>3</v>
@@ -6564,10 +6564,10 @@
         <v>2480000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3310595</v>
+        <v>3325032</v>
       </c>
       <c r="L86" t="n">
-        <v>25.08899457650362</v>
+        <v>25.41425165231492</v>
       </c>
       <c r="M86" s="3" t="n">
         <v>0</v>
@@ -6579,7 +6579,7 @@
         <v>71.60961979842332</v>
       </c>
       <c r="Q86" t="n">
-        <v>26.1</v>
+        <v>26.2</v>
       </c>
       <c r="R86" t="n">
         <v>3</v>
@@ -6628,10 +6628,10 @@
         <v>2571000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3439596</v>
+        <v>3454596</v>
       </c>
       <c r="L87" t="n">
-        <v>25.25284946255316</v>
+        <v>25.57740470955214</v>
       </c>
       <c r="M87" s="3" t="n">
         <v>0</v>
@@ -6643,7 +6643,7 @@
         <v>83.83073496659243</v>
       </c>
       <c r="Q87" t="n">
-        <v>28.8</v>
+        <v>28.9</v>
       </c>
       <c r="R87" t="n">
         <v>3</v>
@@ -6692,10 +6692,10 @@
         <v>2580000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3482596</v>
+        <v>3497784</v>
       </c>
       <c r="L88" t="n">
-        <v>25.91733293210008</v>
+        <v>26.23901304368709</v>
       </c>
       <c r="M88" s="3" t="n">
         <v>0</v>
@@ -6707,7 +6707,7 @@
         <v>80.79034028540066</v>
       </c>
       <c r="Q88" t="n">
-        <v>28.4</v>
+        <v>28.6</v>
       </c>
       <c r="R88" t="n">
         <v>3</v>
@@ -6756,10 +6756,10 @@
         <v>2581000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3439596</v>
+        <v>3454596</v>
       </c>
       <c r="L89" t="n">
-        <v>24.9621176440489</v>
+        <v>25.28793526073671</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
@@ -6771,7 +6771,7 @@
         <v>62.0368495646892</v>
       </c>
       <c r="Q89" t="n">
-        <v>24</v>
+        <v>24.1</v>
       </c>
       <c r="R89" t="n">
         <v>3</v>
@@ -6820,10 +6820,10 @@
         <v>2664000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3611597</v>
+        <v>3627347</v>
       </c>
       <c r="L90" t="n">
-        <v>26.23761731998338</v>
+        <v>26.55789479197882</v>
       </c>
       <c r="M90" s="3" t="n">
         <v>0</v>
@@ -6835,7 +6835,7 @@
         <v>75.54565701559021</v>
       </c>
       <c r="Q90" t="n">
-        <v>27.4</v>
+        <v>27.6</v>
       </c>
       <c r="R90" t="n">
         <v>3</v>
@@ -6884,10 +6884,10 @@
         <v>3090000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>4170602</v>
+        <v>4188789</v>
       </c>
       <c r="L91" t="n">
-        <v>25.90997654535245</v>
+        <v>26.23166265954193</v>
       </c>
       <c r="M91" s="3" t="n">
         <v>0</v>
@@ -6899,7 +6899,7 @@
         <v>100</v>
       </c>
       <c r="Q91" t="n">
-        <v>32.5</v>
+        <v>32.7</v>
       </c>
       <c r="R91" t="n">
         <v>3</v>
@@ -6948,10 +6948,10 @@
         <v>3186000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4299602</v>
+        <v>4318353</v>
       </c>
       <c r="L92" t="n">
-        <v>25.9001181969866</v>
+        <v>26.22187208873383</v>
       </c>
       <c r="M92" s="3" t="n">
         <v>0</v>
@@ -6963,7 +6963,7 @@
         <v>100</v>
       </c>
       <c r="Q92" t="n">
-        <v>32.5</v>
+        <v>32.7</v>
       </c>
       <c r="R92" t="n">
         <v>3</v>
@@ -7246,10 +7246,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>429573</v>
+        <v>431447</v>
       </c>
       <c r="L2" t="n">
-        <v>27.83554832356782</v>
+        <v>28.14899628459579</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7264,7 +7264,7 @@
         <v>29.71702857142851</v>
       </c>
       <c r="Q2" t="n">
-        <v>36.5</v>
+        <v>36.6</v>
       </c>
       <c r="R2" t="n">
         <v>4</v>
@@ -7313,10 +7313,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>429573</v>
+        <v>431447</v>
       </c>
       <c r="L3" t="n">
-        <v>27.83554832356782</v>
+        <v>28.14899628459579</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7331,7 +7331,7 @@
         <v>29.71702857142851</v>
       </c>
       <c r="Q3" t="n">
-        <v>36.5</v>
+        <v>36.6</v>
       </c>
       <c r="R3" t="n">
         <v>4</v>
@@ -7380,10 +7380,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>429573</v>
+        <v>431447</v>
       </c>
       <c r="L4" t="n">
-        <v>27.8353155342631</v>
+        <v>28.14876450641678</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7398,7 +7398,7 @@
         <v>29.71428571428569</v>
       </c>
       <c r="Q4" t="n">
-        <v>14.2</v>
+        <v>14.3</v>
       </c>
       <c r="R4" t="n">
         <v>4</v>
@@ -7447,10 +7447,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>429573</v>
+        <v>431447</v>
       </c>
       <c r="L5" t="n">
-        <v>27.8353155342631</v>
+        <v>28.14876450641678</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7465,7 +7465,7 @@
         <v>29.71428571428569</v>
       </c>
       <c r="Q5" t="n">
-        <v>14.2</v>
+        <v>14.3</v>
       </c>
       <c r="R5" t="n">
         <v>4</v>
@@ -7514,10 +7514,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>515574</v>
+        <v>517822</v>
       </c>
       <c r="L6" t="n">
-        <v>25.51990596888129</v>
+        <v>25.84324343114043</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7529,7 +7529,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>10.9</v>
+        <v>11.1</v>
       </c>
       <c r="R6" t="n">
         <v>3</v>
@@ -7578,10 +7578,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>515574</v>
+        <v>517822</v>
       </c>
       <c r="L7" t="n">
-        <v>25.51990596888129</v>
+        <v>25.84324343114043</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7593,7 +7593,7 @@
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>10.9</v>
+        <v>11.1</v>
       </c>
       <c r="R7" t="n">
         <v>3</v>
@@ -7642,10 +7642,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>515574</v>
+        <v>517822</v>
       </c>
       <c r="L8" t="n">
-        <v>25.51990596888129</v>
+        <v>25.84324343114043</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7657,7 +7657,7 @@
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>10.9</v>
+        <v>11.1</v>
       </c>
       <c r="R8" t="n">
         <v>3</v>
@@ -7706,10 +7706,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>515574</v>
+        <v>517822</v>
       </c>
       <c r="L9" t="n">
-        <v>25.51990596888129</v>
+        <v>25.84324343114043</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7721,7 +7721,7 @@
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>10.9</v>
+        <v>11.1</v>
       </c>
       <c r="R9" t="n">
         <v>3</v>
@@ -7770,10 +7770,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>515574</v>
+        <v>517822</v>
       </c>
       <c r="L10" t="n">
-        <v>25.32594739067525</v>
+        <v>25.65012687757569</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7785,7 +7785,7 @@
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>10.9</v>
+        <v>11</v>
       </c>
       <c r="R10" t="n">
         <v>3</v>
@@ -7834,10 +7834,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>515574</v>
+        <v>517822</v>
       </c>
       <c r="L11" t="n">
-        <v>25.32594739067525</v>
+        <v>25.65012687757569</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7849,7 +7849,7 @@
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>10.9</v>
+        <v>11</v>
       </c>
       <c r="R11" t="n">
         <v>3</v>
@@ -7898,10 +7898,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>515574</v>
+        <v>517822</v>
       </c>
       <c r="L12" t="n">
-        <v>25.32594739067525</v>
+        <v>25.65012687757569</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -7913,7 +7913,7 @@
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>10.9</v>
+        <v>11</v>
       </c>
       <c r="R12" t="n">
         <v>3</v>
@@ -7962,10 +7962,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>515574</v>
+        <v>517822</v>
       </c>
       <c r="L13" t="n">
-        <v>25.32594739067525</v>
+        <v>25.65012687757569</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -7977,7 +7977,7 @@
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>10.9</v>
+        <v>11</v>
       </c>
       <c r="R13" t="n">
         <v>3</v>
@@ -7991,7 +7991,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHA4 M5 10C CPU 8C GPU 16GB 512GB Starlight</t>
+          <t>Apple MacBook Air 13 MDHE4 M5 10C CPU 8C GPU 16GB 512GB Midnight</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -8016,35 +8016,35 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Starlight</t>
+          <t>Midnight</t>
         </is>
       </c>
       <c r="I14" s="3" t="n">
-        <v>430000</v>
+        <v>433999</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>430000</v>
+        <v>433999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>558574</v>
+        <v>561010</v>
       </c>
       <c r="L14" t="n">
-        <v>23.01825720495404</v>
+        <v>22.6397033920964</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>0</v>
+        <v>-8000</v>
       </c>
       <c r="N14" t="n">
-        <v>0</v>
+        <v>3.125006975461999</v>
       </c>
       <c r="O14" t="n">
         <v>100</v>
       </c>
       <c r="P14" t="n">
-        <v>13.01272984441299</v>
+        <v>10.75021216407353</v>
       </c>
       <c r="Q14" t="n">
-        <v>32.1</v>
+        <v>32.4</v>
       </c>
       <c r="R14" t="n">
         <v>4</v>
@@ -8087,31 +8087,31 @@
         </is>
       </c>
       <c r="I15" s="3" t="n">
-        <v>434999</v>
+        <v>433999</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>434999</v>
+        <v>433999</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>558574</v>
+        <v>561010</v>
       </c>
       <c r="L15" t="n">
-        <v>22.12329968813443</v>
+        <v>22.6397033920964</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>0</v>
+        <v>-1000</v>
       </c>
       <c r="N15" t="n">
         <v>0</v>
       </c>
       <c r="O15" t="n">
-        <v>78.26521739130435</v>
+        <v>100</v>
       </c>
       <c r="P15" t="n">
-        <v>10.184441301273</v>
+        <v>10.75021216407353</v>
       </c>
       <c r="Q15" t="n">
-        <v>26.5</v>
+        <v>31.6</v>
       </c>
       <c r="R15" t="n">
         <v>4</v>
@@ -8125,7 +8125,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHE4 M5 10C CPU 8C GPU 16GB 512GB Midnight</t>
+          <t>Apple MacBook Air 13 MDHA4 M5 10C CPU 8C GPU 16GB 512GB Starlight</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -8150,35 +8150,35 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Midnight</t>
+          <t>Starlight</t>
         </is>
       </c>
       <c r="I16" s="3" t="n">
-        <v>441999</v>
+        <v>433999</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>441999</v>
+        <v>433999</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>558574</v>
+        <v>561010</v>
       </c>
       <c r="L16" t="n">
-        <v>20.87010852635461</v>
+        <v>22.6397033920964</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0</v>
+        <v>3999</v>
       </c>
       <c r="N16" t="n">
-        <v>1.339288703769428</v>
+        <v>0</v>
       </c>
       <c r="O16" t="n">
-        <v>47.83043478260869</v>
+        <v>100</v>
       </c>
       <c r="P16" t="n">
-        <v>6.224045261669024</v>
+        <v>10.75021216407353</v>
       </c>
       <c r="Q16" t="n">
-        <v>19</v>
+        <v>31.6</v>
       </c>
       <c r="R16" t="n">
         <v>4</v>
@@ -8221,31 +8221,31 @@
         </is>
       </c>
       <c r="I17" s="3" t="n">
-        <v>447999</v>
+        <v>443000</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>447999</v>
+        <v>443000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>558574</v>
+        <v>561010</v>
       </c>
       <c r="L17" t="n">
-        <v>19.79594467340048</v>
+        <v>21.03527566353541</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>0</v>
+        <v>-4999</v>
       </c>
       <c r="N17" t="n">
-        <v>0</v>
+        <v>1.115850705023895</v>
       </c>
       <c r="O17" t="n">
-        <v>21.74347826086957</v>
+        <v>52.6288090100521</v>
       </c>
       <c r="P17" t="n">
-        <v>2.829420084865629</v>
+        <v>5.657708628005674</v>
       </c>
       <c r="Q17" t="n">
-        <v>11.9</v>
+        <v>20</v>
       </c>
       <c r="R17" t="n">
         <v>4</v>
@@ -8294,10 +8294,10 @@
         <v>453000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>558574</v>
+        <v>561010</v>
       </c>
       <c r="L18" t="n">
-        <v>18.90062910196321</v>
+        <v>19.25277624284772</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -8312,7 +8312,7 @@
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>6.3</v>
+        <v>6.4</v>
       </c>
       <c r="R18" t="n">
         <v>4</v>
@@ -8361,10 +8361,10 @@
         <v>454000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>601575</v>
+        <v>604198</v>
       </c>
       <c r="L19" t="n">
-        <v>24.53143830777542</v>
+        <v>24.85906937791916</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -8376,7 +8376,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q19" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="R19" t="n">
         <v>3</v>
@@ -8425,10 +8425,10 @@
         <v>454000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>601575</v>
+        <v>604198</v>
       </c>
       <c r="L20" t="n">
-        <v>24.53143830777542</v>
+        <v>24.85906937791916</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -8440,7 +8440,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q20" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="R20" t="n">
         <v>3</v>
@@ -8489,10 +8489,10 @@
         <v>454000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>601575</v>
+        <v>604198</v>
       </c>
       <c r="L21" t="n">
-        <v>24.53143830777542</v>
+        <v>24.85906937791916</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -8504,7 +8504,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q21" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="R21" t="n">
         <v>3</v>
@@ -8553,10 +8553,10 @@
         <v>454000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>601575</v>
+        <v>604198</v>
       </c>
       <c r="L22" t="n">
-        <v>24.53143830777542</v>
+        <v>24.85906937791916</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -8568,7 +8568,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q22" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="R22" t="n">
         <v>3</v>
@@ -8617,10 +8617,10 @@
         <v>455000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>601575</v>
+        <v>604198</v>
       </c>
       <c r="L23" t="n">
-        <v>24.36520799567801</v>
+        <v>24.69356072016127</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -8632,7 +8632,7 @@
         <v>100</v>
       </c>
       <c r="Q23" t="n">
-        <v>31.9</v>
+        <v>32</v>
       </c>
       <c r="R23" t="n">
         <v>3</v>
@@ -8681,10 +8681,10 @@
         <v>455000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>601575</v>
+        <v>604198</v>
       </c>
       <c r="L24" t="n">
-        <v>24.36520799567801</v>
+        <v>24.69356072016127</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -8696,7 +8696,7 @@
         <v>100</v>
       </c>
       <c r="Q24" t="n">
-        <v>31.9</v>
+        <v>32</v>
       </c>
       <c r="R24" t="n">
         <v>3</v>
@@ -8745,10 +8745,10 @@
         <v>455000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>601575</v>
+        <v>604198</v>
       </c>
       <c r="L25" t="n">
-        <v>24.36520799567801</v>
+        <v>24.69356072016127</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -8760,7 +8760,7 @@
         <v>100</v>
       </c>
       <c r="Q25" t="n">
-        <v>31.9</v>
+        <v>32</v>
       </c>
       <c r="R25" t="n">
         <v>3</v>
@@ -8809,10 +8809,10 @@
         <v>455000</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>601575</v>
+        <v>604198</v>
       </c>
       <c r="L26" t="n">
-        <v>24.36520799567801</v>
+        <v>24.69356072016127</v>
       </c>
       <c r="M26" s="3" t="n">
         <v>0</v>
@@ -8824,7 +8824,7 @@
         <v>100</v>
       </c>
       <c r="Q26" t="n">
-        <v>31.9</v>
+        <v>32</v>
       </c>
       <c r="R26" t="n">
         <v>3</v>
@@ -8873,10 +8873,10 @@
         <v>475000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>687575</v>
+        <v>690574</v>
       </c>
       <c r="L27" t="n">
-        <v>30.91662727702432</v>
+        <v>31.21664007043416</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -8888,7 +8888,7 @@
         <v>100</v>
       </c>
       <c r="Q27" t="n">
-        <v>34.7</v>
+        <v>34.8</v>
       </c>
       <c r="R27" t="n">
         <v>3</v>
@@ -8937,10 +8937,10 @@
         <v>475000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>687575</v>
+        <v>690574</v>
       </c>
       <c r="L28" t="n">
-        <v>30.91662727702432</v>
+        <v>31.21664007043416</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -8952,7 +8952,7 @@
         <v>100</v>
       </c>
       <c r="Q28" t="n">
-        <v>34.7</v>
+        <v>34.8</v>
       </c>
       <c r="R28" t="n">
         <v>3</v>
@@ -9001,10 +9001,10 @@
         <v>475000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>687575</v>
+        <v>690574</v>
       </c>
       <c r="L29" t="n">
-        <v>30.91662727702432</v>
+        <v>31.21664007043416</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -9016,7 +9016,7 @@
         <v>100</v>
       </c>
       <c r="Q29" t="n">
-        <v>34.7</v>
+        <v>34.8</v>
       </c>
       <c r="R29" t="n">
         <v>3</v>
@@ -9065,10 +9065,10 @@
         <v>475000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>687575</v>
+        <v>690574</v>
       </c>
       <c r="L30" t="n">
-        <v>30.91662727702432</v>
+        <v>31.21664007043416</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -9080,7 +9080,7 @@
         <v>100</v>
       </c>
       <c r="Q30" t="n">
-        <v>34.7</v>
+        <v>34.8</v>
       </c>
       <c r="R30" t="n">
         <v>3</v>
@@ -9129,10 +9129,10 @@
         <v>479999</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>687575</v>
+        <v>690574</v>
       </c>
       <c r="L31" t="n">
-        <v>30.18957931861978</v>
+        <v>30.49274950982806</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -9144,7 +9144,7 @@
         <v>52.61711456859971</v>
       </c>
       <c r="Q31" t="n">
-        <v>24.2</v>
+        <v>24.3</v>
       </c>
       <c r="R31" t="n">
         <v>3</v>
@@ -9193,10 +9193,10 @@
         <v>479999</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>687575</v>
+        <v>690574</v>
       </c>
       <c r="L32" t="n">
-        <v>30.18957931861978</v>
+        <v>30.49274950982806</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -9208,7 +9208,7 @@
         <v>52.61711456859971</v>
       </c>
       <c r="Q32" t="n">
-        <v>24.2</v>
+        <v>24.3</v>
       </c>
       <c r="R32" t="n">
         <v>3</v>
@@ -9257,10 +9257,10 @@
         <v>479999</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>687575</v>
+        <v>690574</v>
       </c>
       <c r="L33" t="n">
-        <v>30.18957931861978</v>
+        <v>30.49274950982806</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -9272,7 +9272,7 @@
         <v>52.61711456859971</v>
       </c>
       <c r="Q33" t="n">
-        <v>24.2</v>
+        <v>24.3</v>
       </c>
       <c r="R33" t="n">
         <v>3</v>
@@ -9321,10 +9321,10 @@
         <v>479999</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>687575</v>
+        <v>690574</v>
       </c>
       <c r="L34" t="n">
-        <v>30.18957931861978</v>
+        <v>30.49274950982806</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -9336,7 +9336,7 @@
         <v>52.61711456859971</v>
       </c>
       <c r="Q34" t="n">
-        <v>24.2</v>
+        <v>24.3</v>
       </c>
       <c r="R34" t="n">
         <v>3</v>
@@ -9385,10 +9385,10 @@
         <v>482999</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>644575</v>
+        <v>647386</v>
       </c>
       <c r="L35" t="n">
-        <v>25.06705969049374</v>
+        <v>25.39242430327502</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
@@ -9400,10 +9400,10 @@
         <v>100</v>
       </c>
       <c r="P35" t="n">
-        <v>5.818666666666681</v>
+        <v>3.478278152934936</v>
       </c>
       <c r="Q35" t="n">
-        <v>31.5</v>
+        <v>31.3</v>
       </c>
       <c r="R35" t="n">
         <v>4</v>
@@ -9452,10 +9452,10 @@
         <v>482999</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>644575</v>
+        <v>647386</v>
       </c>
       <c r="L36" t="n">
-        <v>25.06705969049374</v>
+        <v>25.39242430327502</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -9467,10 +9467,10 @@
         <v>100</v>
       </c>
       <c r="P36" t="n">
-        <v>5.818666666666681</v>
+        <v>3.478278152934936</v>
       </c>
       <c r="Q36" t="n">
-        <v>31.5</v>
+        <v>31.3</v>
       </c>
       <c r="R36" t="n">
         <v>4</v>
@@ -9519,10 +9519,10 @@
         <v>482999</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>644575</v>
+        <v>647386</v>
       </c>
       <c r="L37" t="n">
-        <v>25.06705969049374</v>
+        <v>25.39242430327502</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
@@ -9534,10 +9534,10 @@
         <v>100</v>
       </c>
       <c r="P37" t="n">
-        <v>5.818666666666681</v>
+        <v>3.478278152934936</v>
       </c>
       <c r="Q37" t="n">
-        <v>31.5</v>
+        <v>31.3</v>
       </c>
       <c r="R37" t="n">
         <v>4</v>
@@ -9580,22 +9580,22 @@
         </is>
       </c>
       <c r="I38" s="3" t="n">
-        <v>495000</v>
+        <v>489999</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>495000</v>
+        <v>489999</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>644575</v>
+        <v>647386</v>
       </c>
       <c r="L38" t="n">
-        <v>23.20521273707482</v>
+        <v>24.31115285162175</v>
       </c>
       <c r="M38" s="3" t="n">
-        <v>0</v>
+        <v>-5001</v>
       </c>
       <c r="N38" t="n">
-        <v>0</v>
+        <v>1.01030303030303</v>
       </c>
       <c r="O38" t="n">
         <v>0</v>
@@ -9604,7 +9604,7 @@
         <v>0</v>
       </c>
       <c r="Q38" t="n">
-        <v>7.7</v>
+        <v>8.4</v>
       </c>
       <c r="R38" t="n">
         <v>4</v>
@@ -9653,10 +9653,10 @@
         <v>500000</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>644575</v>
+        <v>647386</v>
       </c>
       <c r="L39" t="n">
-        <v>22.42950781522709</v>
+        <v>22.76632488190971</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -9668,7 +9668,7 @@
         <v>44.13012729844413</v>
       </c>
       <c r="Q39" t="n">
-        <v>19.1</v>
+        <v>19.2</v>
       </c>
       <c r="R39" t="n">
         <v>3</v>
@@ -9717,10 +9717,10 @@
         <v>551999</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>773576</v>
+        <v>776949</v>
       </c>
       <c r="L40" t="n">
-        <v>28.64321023403001</v>
+        <v>28.95299434068388</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -9735,7 +9735,7 @@
         <v>68.91123055162657</v>
       </c>
       <c r="Q40" t="n">
-        <v>43.3</v>
+        <v>43.4</v>
       </c>
       <c r="R40" t="n">
         <v>4</v>
@@ -9784,10 +9784,10 @@
         <v>551999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>773576</v>
+        <v>776949</v>
       </c>
       <c r="L41" t="n">
-        <v>28.64321023403001</v>
+        <v>28.95299434068388</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
@@ -9802,7 +9802,7 @@
         <v>68.91123055162657</v>
       </c>
       <c r="Q41" t="n">
-        <v>43.3</v>
+        <v>43.4</v>
       </c>
       <c r="R41" t="n">
         <v>4</v>
@@ -9851,10 +9851,10 @@
         <v>551999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>773576</v>
+        <v>776949</v>
       </c>
       <c r="L42" t="n">
-        <v>28.64321023403001</v>
+        <v>28.95299434068388</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -9869,7 +9869,7 @@
         <v>68.91123055162657</v>
       </c>
       <c r="Q42" t="n">
-        <v>43.3</v>
+        <v>43.4</v>
       </c>
       <c r="R42" t="n">
         <v>4</v>
@@ -9918,10 +9918,10 @@
         <v>557999</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>773576</v>
+        <v>776949</v>
       </c>
       <c r="L43" t="n">
-        <v>27.8675915488588</v>
+        <v>28.18074288016331</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -9936,7 +9936,7 @@
         <v>66.87445544554454</v>
       </c>
       <c r="Q43" t="n">
-        <v>20.4</v>
+        <v>20.5</v>
       </c>
       <c r="R43" t="n">
         <v>4</v>
@@ -9979,28 +9979,28 @@
         </is>
       </c>
       <c r="I44" s="3" t="n">
-        <v>564999</v>
+        <v>559999</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>564999</v>
+        <v>559999</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>773576</v>
+        <v>776949</v>
       </c>
       <c r="L44" t="n">
-        <v>26.96270308282573</v>
+        <v>27.92332572665644</v>
       </c>
       <c r="M44" s="3" t="n">
-        <v>0</v>
+        <v>-5000</v>
       </c>
       <c r="N44" t="n">
-        <v>0</v>
+        <v>0.8849573185085283</v>
       </c>
       <c r="P44" t="n">
-        <v>34.54581818181818</v>
+        <v>34.78265730512947</v>
       </c>
       <c r="Q44" t="n">
-        <v>19</v>
+        <v>19.7</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -10043,28 +10043,28 @@
         </is>
       </c>
       <c r="I45" s="3" t="n">
-        <v>564999</v>
+        <v>559999</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>564999</v>
+        <v>559999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>773576</v>
+        <v>776949</v>
       </c>
       <c r="L45" t="n">
-        <v>26.96270308282573</v>
+        <v>27.92332572665644</v>
       </c>
       <c r="M45" s="3" t="n">
-        <v>0</v>
+        <v>-5000</v>
       </c>
       <c r="N45" t="n">
-        <v>0</v>
+        <v>0.8849573185085283</v>
       </c>
       <c r="P45" t="n">
-        <v>34.54581818181818</v>
+        <v>34.78265730512947</v>
       </c>
       <c r="Q45" t="n">
-        <v>19</v>
+        <v>19.7</v>
       </c>
       <c r="R45" t="n">
         <v>3</v>
@@ -10107,28 +10107,28 @@
         </is>
       </c>
       <c r="I46" s="3" t="n">
-        <v>564999</v>
+        <v>559999</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>564999</v>
+        <v>559999</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>773576</v>
+        <v>776949</v>
       </c>
       <c r="L46" t="n">
-        <v>26.96270308282573</v>
+        <v>27.92332572665644</v>
       </c>
       <c r="M46" s="3" t="n">
-        <v>0</v>
+        <v>-5000</v>
       </c>
       <c r="N46" t="n">
-        <v>0</v>
+        <v>0.8849573185085283</v>
       </c>
       <c r="P46" t="n">
-        <v>34.54581818181818</v>
+        <v>34.78265730512947</v>
       </c>
       <c r="Q46" t="n">
-        <v>19</v>
+        <v>19.7</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -10171,28 +10171,28 @@
         </is>
       </c>
       <c r="I47" s="3" t="n">
-        <v>564999</v>
+        <v>559999</v>
       </c>
       <c r="J47" s="3" t="n">
-        <v>564999</v>
+        <v>559999</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>773576</v>
+        <v>776949</v>
       </c>
       <c r="L47" t="n">
-        <v>26.96270308282573</v>
+        <v>27.92332572665644</v>
       </c>
       <c r="M47" s="3" t="n">
-        <v>0</v>
+        <v>-5000</v>
       </c>
       <c r="N47" t="n">
-        <v>0</v>
+        <v>0.8849573185085283</v>
       </c>
       <c r="P47" t="n">
-        <v>34.54581818181818</v>
+        <v>34.78265730512947</v>
       </c>
       <c r="Q47" t="n">
-        <v>19</v>
+        <v>19.7</v>
       </c>
       <c r="R47" t="n">
         <v>3</v>
@@ -10241,10 +10241,10 @@
         <v>585000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>730576</v>
+        <v>733762</v>
       </c>
       <c r="L48" t="n">
-        <v>19.92619522130483</v>
+        <v>20.27387627050733</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -10253,10 +10253,10 @@
         <v>0</v>
       </c>
       <c r="P48" t="n">
-        <v>27.27272727272727</v>
+        <v>25.46546815139454</v>
       </c>
       <c r="Q48" t="n">
-        <v>14.4</v>
+        <v>14.1</v>
       </c>
       <c r="R48" t="n">
         <v>3</v>
@@ -10305,10 +10305,10 @@
         <v>595000</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>730576</v>
+        <v>733762</v>
       </c>
       <c r="L49" t="n">
-        <v>18.55741223363483</v>
+        <v>18.91103654863566</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -10320,7 +10320,7 @@
         <v>54.31400282885431</v>
       </c>
       <c r="Q49" t="n">
-        <v>19.6</v>
+        <v>19.7</v>
       </c>
       <c r="R49" t="n">
         <v>3</v>
@@ -10334,7 +10334,7 @@
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MDVN4 M5 10C CPU 10C GPU 24GB 1TB Midnight</t>
+          <t>Apple MacBook Air 15 MDVU4 M5 10C CPU 10C GPU 24GB 1TB Sky Blue</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -10359,7 +10359,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Midnight</t>
+          <t>Sky Blue</t>
         </is>
       </c>
       <c r="I50" s="3" t="n">
@@ -10369,28 +10369,25 @@
         <v>614999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>859576</v>
+        <v>863325</v>
       </c>
       <c r="L50" t="n">
-        <v>28.45321414278668</v>
+        <v>28.76390698751919</v>
       </c>
       <c r="M50" s="3" t="n">
-        <v>0</v>
+        <v>-2000</v>
       </c>
       <c r="N50" t="n">
-        <v>0</v>
-      </c>
-      <c r="O50" t="n">
-        <v>100</v>
+        <v>0.3241496339540259</v>
       </c>
       <c r="P50" t="n">
-        <v>61.0912</v>
+        <v>60.12432359912347</v>
       </c>
       <c r="Q50" t="n">
-        <v>41.9</v>
+        <v>25.3</v>
       </c>
       <c r="R50" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S50" t="inlineStr">
         <is>
@@ -10401,7 +10398,7 @@
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MDVU4 M5 10C CPU 10C GPU 24GB 1TB Sky Blue</t>
+          <t>Apple MacBook Air 15 MDVF4 M5 10C CPU 10C GPU 24GB 1TB Starlight</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -10426,38 +10423,35 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Sky Blue</t>
+          <t>Starlight</t>
         </is>
       </c>
       <c r="I51" s="3" t="n">
-        <v>616999</v>
+        <v>614999</v>
       </c>
       <c r="J51" s="3" t="n">
-        <v>616999</v>
+        <v>614999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>859576</v>
+        <v>863325</v>
       </c>
       <c r="L51" t="n">
-        <v>28.22054129012443</v>
+        <v>28.76390698751919</v>
       </c>
       <c r="M51" s="3" t="n">
-        <v>0</v>
+        <v>-2000</v>
       </c>
       <c r="N51" t="n">
-        <v>0</v>
-      </c>
-      <c r="O51" t="n">
-        <v>80</v>
+        <v>0.3241496339540259</v>
       </c>
       <c r="P51" t="n">
-        <v>60.50938181818182</v>
+        <v>60.12432359912347</v>
       </c>
       <c r="Q51" t="n">
-        <v>37.3</v>
+        <v>25.3</v>
       </c>
       <c r="R51" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S51" t="inlineStr">
         <is>
@@ -10468,7 +10462,7 @@
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MDVF4 M5 10C CPU 10C GPU 24GB 1TB Starlight</t>
+          <t>Apple MacBook Air 15 MDVC4 M5 10C CPU 10C GPU 24GB 1TB Silver</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -10493,38 +10487,35 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Starlight</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I52" s="3" t="n">
-        <v>616999</v>
+        <v>614999</v>
       </c>
       <c r="J52" s="3" t="n">
-        <v>616999</v>
+        <v>614999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>859576</v>
+        <v>863325</v>
       </c>
       <c r="L52" t="n">
-        <v>28.22054129012443</v>
+        <v>28.76390698751919</v>
       </c>
       <c r="M52" s="3" t="n">
-        <v>0</v>
+        <v>-10000</v>
       </c>
       <c r="N52" t="n">
-        <v>0</v>
-      </c>
-      <c r="O52" t="n">
-        <v>80</v>
+        <v>0.3241496339540259</v>
       </c>
       <c r="P52" t="n">
-        <v>60.50938181818182</v>
+        <v>60.12432359912347</v>
       </c>
       <c r="Q52" t="n">
-        <v>37.3</v>
+        <v>25.3</v>
       </c>
       <c r="R52" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S52" t="inlineStr">
         <is>
@@ -10535,7 +10526,7 @@
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MDVC4 M5 10C CPU 10C GPU 24GB 1TB Silver</t>
+          <t>Apple MacBook Air 15 MDVN4 M5 10C CPU 10C GPU 24GB 1TB Midnight</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -10560,20 +10551,20 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Midnight</t>
         </is>
       </c>
       <c r="I53" s="3" t="n">
-        <v>624999</v>
+        <v>614999</v>
       </c>
       <c r="J53" s="3" t="n">
-        <v>624999</v>
+        <v>614999</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>859576</v>
+        <v>863325</v>
       </c>
       <c r="L53" t="n">
-        <v>27.28984987947547</v>
+        <v>28.76390698751919</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -10581,17 +10572,14 @@
       <c r="N53" t="n">
         <v>0</v>
       </c>
-      <c r="O53" t="n">
-        <v>0</v>
-      </c>
       <c r="P53" t="n">
-        <v>58.18210909090909</v>
+        <v>60.12432359912347</v>
       </c>
       <c r="Q53" t="n">
-        <v>18.8</v>
+        <v>25.2</v>
       </c>
       <c r="R53" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S53" t="inlineStr">
         <is>
@@ -10637,10 +10625,10 @@
         <v>650000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>816576</v>
+        <v>820137</v>
       </c>
       <c r="L54" t="n">
-        <v>20.3993259659848</v>
+        <v>20.74494870978873</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -10649,10 +10637,10 @@
         <v>0</v>
       </c>
       <c r="P54" t="n">
-        <v>50.90909090909091</v>
+        <v>49.68919100219131</v>
       </c>
       <c r="Q54" t="n">
-        <v>19.7</v>
+        <v>19.5</v>
       </c>
       <c r="R54" t="n">
         <v>3</v>
@@ -10701,10 +10689,10 @@
         <v>672000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>859576</v>
+        <v>863325</v>
       </c>
       <c r="L55" t="n">
-        <v>21.82192150548643</v>
+        <v>22.16141082442881</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -10716,7 +10704,7 @@
         <v>66.19519094766619</v>
       </c>
       <c r="Q55" t="n">
-        <v>23.5</v>
+        <v>23.7</v>
       </c>
       <c r="R55" t="n">
         <v>3</v>
@@ -10765,10 +10753,10 @@
         <v>700000</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>902577</v>
+        <v>906513</v>
       </c>
       <c r="L56" t="n">
-        <v>22.4442900716504</v>
+        <v>22.78103016724526</v>
       </c>
       <c r="M56" s="3" t="n">
         <v>0</v>
@@ -10780,7 +10768,7 @@
         <v>58.27439886845826</v>
       </c>
       <c r="Q56" t="n">
-        <v>22.1</v>
+        <v>22.3</v>
       </c>
       <c r="R56" t="n">
         <v>3</v>
@@ -10829,10 +10817,10 @@
         <v>715000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>945577</v>
+        <v>949701</v>
       </c>
       <c r="L57" t="n">
-        <v>24.38479362336436</v>
+        <v>24.71314655875902</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -10841,7 +10829,7 @@
         <v>0</v>
       </c>
       <c r="P57" t="n">
-        <v>66.66666666666666</v>
+        <v>65.83833956938916</v>
       </c>
       <c r="Q57" t="n">
         <v>24.7</v>
@@ -10893,13 +10881,13 @@
         <v>734999</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>988577</v>
+        <v>992889</v>
       </c>
       <c r="L58" t="n">
-        <v>25.6508091934164</v>
+        <v>25.97369897339984</v>
       </c>
       <c r="M58" s="3" t="n">
-        <v>-21001</v>
+        <v>0</v>
       </c>
       <c r="N58" t="n">
         <v>2.777910052910053</v>
@@ -10908,7 +10896,7 @@
         <v>78.07662153970499</v>
       </c>
       <c r="Q58" t="n">
-        <v>28.7</v>
+        <v>28.9</v>
       </c>
       <c r="R58" t="n">
         <v>3</v>
@@ -10957,10 +10945,10 @@
         <v>752000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>988577</v>
+        <v>992889</v>
       </c>
       <c r="L59" t="n">
-        <v>23.93106455035875</v>
+        <v>24.26142297880226</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -10969,10 +10957,10 @@
         <v>0</v>
       </c>
       <c r="P59" t="n">
-        <v>57.6969696969697</v>
+        <v>56.64574730806117</v>
       </c>
       <c r="Q59" t="n">
-        <v>22.6</v>
+        <v>22.5</v>
       </c>
       <c r="R59" t="n">
         <v>3</v>
@@ -11021,10 +11009,10 @@
         <v>810000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1074578</v>
+        <v>1079264</v>
       </c>
       <c r="L60" t="n">
-        <v>24.62157237538829</v>
+        <v>24.94885403386011</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -11033,7 +11021,7 @@
         <v>0</v>
       </c>
       <c r="P60" t="n">
-        <v>71.68831168831169</v>
+        <v>70.98477153036431</v>
       </c>
       <c r="Q60" t="n">
         <v>25.9</v>
@@ -11085,10 +11073,10 @@
         <v>815000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1074578</v>
+        <v>1079264</v>
       </c>
       <c r="L61" t="n">
-        <v>24.1562734394339</v>
+        <v>24.48557535505678</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -11100,7 +11088,7 @@
         <v>83.38048090523338</v>
       </c>
       <c r="Q61" t="n">
-        <v>28.2</v>
+        <v>28.4</v>
       </c>
       <c r="R61" t="n">
         <v>3</v>
@@ -11149,10 +11137,10 @@
         <v>875000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1160579</v>
+        <v>1165640</v>
       </c>
       <c r="L62" t="n">
-        <v>24.60659722431648</v>
+        <v>24.93394186884458</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -11161,7 +11149,7 @@
         <v>0</v>
       </c>
       <c r="P62" t="n">
-        <v>80.90909090909091</v>
+        <v>80.43468538974106</v>
       </c>
       <c r="Q62" t="n">
         <v>27.9</v>
@@ -11213,10 +11201,10 @@
         <v>992000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1332580</v>
+        <v>1338391</v>
       </c>
       <c r="L63" t="n">
-        <v>25.55794023623347</v>
+        <v>25.881151322745</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -11228,7 +11216,7 @@
         <v>87.92079207920791</v>
       </c>
       <c r="Q63" t="n">
-        <v>29.8</v>
+        <v>29.9</v>
       </c>
       <c r="R63" t="n">
         <v>3</v>
@@ -11277,10 +11265,10 @@
         <v>1050000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1418581</v>
+        <v>1424767</v>
       </c>
       <c r="L64" t="n">
-        <v>25.98237252578457</v>
+        <v>26.30373948863218</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -11292,7 +11280,7 @@
         <v>94.27799922849427</v>
       </c>
       <c r="Q64" t="n">
-        <v>31.3</v>
+        <v>31.5</v>
       </c>
       <c r="R64" t="n">
         <v>3</v>
@@ -11341,10 +11329,10 @@
         <v>1050000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1418581</v>
+        <v>1424767</v>
       </c>
       <c r="L65" t="n">
-        <v>25.98237252578457</v>
+        <v>26.30373948863218</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -11353,10 +11341,10 @@
         <v>0</v>
       </c>
       <c r="P65" t="n">
-        <v>87.27272727272727</v>
+        <v>86.95645692649404</v>
       </c>
       <c r="Q65" t="n">
-        <v>29.8</v>
+        <v>29.9</v>
       </c>
       <c r="R65" t="n">
         <v>3</v>
@@ -11405,10 +11393,10 @@
         <v>1100000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1504581</v>
+        <v>1511143</v>
       </c>
       <c r="L66" t="n">
-        <v>26.88994477532283</v>
+        <v>27.20741849050686</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -11417,10 +11405,10 @@
         <v>0</v>
       </c>
       <c r="P66" t="n">
-        <v>94.54545454545455</v>
+        <v>94.40991011135459</v>
       </c>
       <c r="Q66" t="n">
-        <v>31.8</v>
+        <v>31.9</v>
       </c>
       <c r="R66" t="n">
         <v>3</v>
@@ -11469,10 +11457,10 @@
         <v>1105000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1504581</v>
+        <v>1511143</v>
       </c>
       <c r="L67" t="n">
-        <v>26.55762634248339</v>
+        <v>26.87654312000916</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -11484,7 +11472,7 @@
         <v>100</v>
       </c>
       <c r="Q67" t="n">
-        <v>32.8</v>
+        <v>32.9</v>
       </c>
       <c r="R67" t="n">
         <v>3</v>
@@ -11533,10 +11521,10 @@
         <v>1155000</v>
       </c>
       <c r="K68" s="3" t="n">
-        <v>1590582</v>
+        <v>1597518</v>
       </c>
       <c r="L68" t="n">
-        <v>27.38507037046817</v>
+        <v>27.70034516043012</v>
       </c>
       <c r="M68" s="3" t="n">
         <v>0</v>
@@ -11548,7 +11536,7 @@
         <v>100</v>
       </c>
       <c r="Q68" t="n">
-        <v>33.2</v>
+        <v>33.3</v>
       </c>
       <c r="R68" t="n">
         <v>3</v>
@@ -11804,7 +11792,7 @@
         <v>315000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>300572</v>
+        <v>301883</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -11865,10 +11853,10 @@
         <v>380000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>386573</v>
+        <v>388259</v>
       </c>
       <c r="L3" t="n">
-        <v>1.700325682342016</v>
+        <v>2.12718829441172</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -11880,7 +11868,7 @@
         <v>100</v>
       </c>
       <c r="Q3" t="n">
-        <v>22.2</v>
+        <v>22.3</v>
       </c>
       <c r="R3" t="n">
         <v>3</v>
@@ -11929,7 +11917,7 @@
         <v>415000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>386573</v>
+        <v>388259</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -11990,10 +11978,10 @@
         <v>495000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>472574</v>
+        <v>474634</v>
       </c>
       <c r="L5" t="n">
-        <v>6.893100339840956</v>
+        <v>7.297201633258468</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -12005,7 +11993,7 @@
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>4</v>
+        <v>4.1</v>
       </c>
       <c r="R5" t="n">
         <v>4</v>
@@ -12054,10 +12042,10 @@
         <v>500000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>515574</v>
+        <v>517822</v>
       </c>
       <c r="L6" t="n">
-        <v>8.83946824316199</v>
+        <v>9.235219824572923</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -12069,7 +12057,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>4.1</v>
+        <v>4.2</v>
       </c>
       <c r="R6" t="n">
         <v>4</v>
@@ -12118,10 +12106,10 @@
         <v>550000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>558574</v>
+        <v>561010</v>
       </c>
       <c r="L7" t="n">
-        <v>6.9057994106421</v>
+        <v>7.310030124240209</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -12133,7 +12121,7 @@
         <v>25.45360054666915</v>
       </c>
       <c r="Q7" t="n">
-        <v>8</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="R7" t="n">
         <v>4</v>
@@ -12182,7 +12170,7 @@
         <v>530000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>472574</v>
+        <v>474634</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -12246,10 +12234,10 @@
         <v>600000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>601575</v>
+        <v>604198</v>
       </c>
       <c r="L9" t="n">
-        <v>8.57332834642397</v>
+        <v>8.970238233161977</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -12261,7 +12249,7 @@
         <v>20.65076182537716</v>
       </c>
       <c r="Q9" t="n">
-        <v>8.1</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="R9" t="n">
         <v>4</v>
@@ -12310,10 +12298,10 @@
         <v>646000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>730576</v>
+        <v>733762</v>
       </c>
       <c r="L10" t="n">
-        <v>17.18876612426359</v>
+        <v>17.54833311073618</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -12325,7 +12313,7 @@
         <v>100</v>
       </c>
       <c r="Q10" t="n">
-        <v>26</v>
+        <v>26.1</v>
       </c>
       <c r="R10" t="n">
         <v>4</v>
@@ -12374,7 +12362,7 @@
         <v>615000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>558574</v>
+        <v>561010</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -12438,7 +12426,7 @@
         <v>700000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>644575</v>
+        <v>647386</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -12502,7 +12490,7 @@
         <v>745000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>687575</v>
+        <v>690574</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -12566,7 +12554,7 @@
         <v>930000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>859576</v>
+        <v>863325</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -12637,7 +12625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12686,7 +12674,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 MJ3D4 10 Core CPU 10 Core GPU 32GB 1TB Space Black</t>
+          <t>Macbook Pro 16 MGE44 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Silver</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -12695,22 +12683,22 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>772000</v>
+        <v>870000</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>745000</v>
+        <v>840000</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-27000</v>
+        <v>-30000</v>
       </c>
       <c r="F2" t="n">
-        <v>-3.5</v>
+        <v>-3.45</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Apple MacBook Air Z1L2000VN 13 M5 10C CPU 10C GPU 24GB 2TB Silver</t>
+          <t>Apple MacBook Air 15 MDVC4 M5 10C CPU 10C GPU 24GB 1TB Silver</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -12719,22 +12707,22 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>756000</v>
+        <v>624999</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>734999</v>
+        <v>614999</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>-21001</v>
+        <v>-10000</v>
       </c>
       <c r="F3" t="n">
-        <v>-2.78</v>
+        <v>-1.6</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 MJ3E4 10 Core CPU 10 Core GPU 32GB 1TB Silver</t>
+          <t>Apple MacBook Air 13 MDHE4 M5 10C CPU 8C GPU 16GB 512GB Midnight</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -12743,69 +12731,381 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>772000</v>
+        <v>441999</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>755000</v>
+        <v>433999</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>-17000</v>
+        <v>-8000</v>
       </c>
       <c r="F4" t="n">
-        <v>-2.2</v>
+        <v>-1.81</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 MGE94 M5 Max 18 Core CPU 40 Core GPU 48GB 2TB Silver</t>
+          <t>Macbook Pro 14 MGDN4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Silver</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>1430000</v>
+        <v>735000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>1460000</v>
+        <v>729999</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>30000</v>
+        <v>-5001</v>
       </c>
       <c r="F5" t="n">
-        <v>2.1</v>
+        <v>-0.68</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 MGEE4 M5 Max 18 Core CPU 40 Core GPU 48GB 2TB Space Black</t>
+          <t>Apple MacBook Air 15 MDV94 M5 10C CPU 10C GPU 16GB 512GB Silver</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>495000</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>489999</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>-5001</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-1.01</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Macbook Pro 16 MGE64 M5 Pro 18 Core CPU 20 Core GPU 48GB 1TB Silver</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>1085000</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>1080000</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>-5000</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-0.46</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 15 MDVK4 M5 10C CPU 10C GPU 16GB 1TB Midnight</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>564999</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>559999</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>-5000</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-0.88</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 15 MDVA4 M5 10C CPU 10C GPU 16GB 1TB Silver</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>564999</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>559999</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>-5000</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-0.88</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 15 MDVE4 M5 10C CPU 10C GPU 16GB 1TB Starlight</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>564999</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>559999</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>-5000</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-0.88</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 15 MDVT4 M5 10C CPU 10C GPU 16GB 1TB Sky Blue</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>564999</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>559999</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>-5000</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-0.88</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 13 MDH74 M5 10C CPU 8C GPU 16GB 512GB Silver</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>447999</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>443000</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>-4999</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-1.12</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Macbook Pro 14 MGDR4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Space Black</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>728000</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>724999</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>-3001</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-0.41</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Macbook Pro 16 MGEA4 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Space Black</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>832999</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>829999</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>-3000</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-0.36</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 15 MDVU4 M5 10C CPU 10C GPU 24GB 1TB Sky Blue</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>616999</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>614999</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>-2000</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-0.32</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 15 MDVF4 M5 10C CPU 10C GPU 24GB 1TB Starlight</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>616999</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>614999</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>-2000</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-0.32</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Macbook Pro 14 M5 MDE34 10 Core CPU 10 Core GPU 24GB 1TB Space Black</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>645000</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>643999</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>-1001</v>
+      </c>
+      <c r="F17" t="n">
+        <v>-0.16</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 13 MDHH4 M5 10C CPU 8C GPU 16GB 512GB Sky Blue</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>434999</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>433999</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>-1000</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-0.23</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 13 MDHA4 M5 10C CPU 8C GPU 16GB 512GB Starlight</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="C6" s="3" t="n">
-        <v>1425000</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>1460000</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>35000</v>
-      </c>
-      <c r="F6" t="n">
-        <v>2.46</v>
+      <c r="C19" s="3" t="n">
+        <v>430000</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>433999</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>3999</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.93</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F6"/>
-  <conditionalFormatting sqref="E2:E6">
+  <autoFilter ref="A1:F19"/>
+  <conditionalFormatting sqref="E2:E19">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
chore: price data 2026-09-21
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MacBook Pro'!$A$1:$S$92</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MacBook Air'!$A$1:$S$68</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20260920T083919656362+0000</t>
+          <t>20260921T090210102061+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-20T08:39:19.656362+00:00</t>
+          <t>2026-09-21T09:02:10.102061+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>278.631272</v>
+        <v>277.926206</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -687,7 +687,7 @@
         <v>532000</v>
       </c>
       <c r="D20" t="n">
-        <v>51.7</v>
+        <v>51.6</v>
       </c>
       <c r="E20" t="n">
         <v>4</v>
@@ -708,7 +708,7 @@
         <v>810000</v>
       </c>
       <c r="D21" t="n">
-        <v>50.7</v>
+        <v>50.6</v>
       </c>
       <c r="E21" t="n">
         <v>4</v>
@@ -771,7 +771,7 @@
         <v>700000</v>
       </c>
       <c r="D24" t="n">
-        <v>49.7</v>
+        <v>49.6</v>
       </c>
       <c r="E24" t="n">
         <v>4</v>
@@ -792,7 +792,7 @@
         <v>847999</v>
       </c>
       <c r="D25" t="n">
-        <v>47.5</v>
+        <v>47.4</v>
       </c>
       <c r="E25" t="n">
         <v>5</v>
@@ -813,7 +813,7 @@
         <v>745000</v>
       </c>
       <c r="D26" t="n">
-        <v>45.5</v>
+        <v>45.4</v>
       </c>
       <c r="E26" t="n">
         <v>4</v>
@@ -906,19 +906,19 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHG4 M5 10C CPU 10C GPU 24GB 1TB Midnight</t>
+          <t>Apple MacBook Pro 16Inch MX303 14Core CPU 32Core GPU M4 Max 36GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>macbook_air</t>
+          <t>macbook_pro</t>
         </is>
       </c>
       <c r="C31" s="3" t="n">
-        <v>551999</v>
+        <v>970000</v>
       </c>
       <c r="D31" t="n">
-        <v>43.4</v>
+        <v>43.3</v>
       </c>
       <c r="E31" t="n">
         <v>4</v>
@@ -1147,10 +1147,10 @@
         <v>470000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>690574</v>
+        <v>688826</v>
       </c>
       <c r="L2" t="n">
-        <v>35.560852276512</v>
+        <v>35.39732820770412</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1214,10 +1214,10 @@
         <v>465000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>690574</v>
+        <v>688826</v>
       </c>
       <c r="L3" t="n">
-        <v>33.67836032054494</v>
+        <v>33.51005914410896</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -1232,7 +1232,7 @@
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>10.3</v>
+        <v>10.2</v>
       </c>
       <c r="R3" t="n">
         <v>5</v>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>776949</v>
+        <v>774983</v>
       </c>
       <c r="L4" t="n">
-        <v>35.6458403318622</v>
+        <v>35.48258477927903</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1299,7 +1299,7 @@
         <v>59.79881123919307</v>
       </c>
       <c r="Q4" t="n">
-        <v>40.6</v>
+        <v>40.5</v>
       </c>
       <c r="R4" t="n">
         <v>5</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>776949</v>
+        <v>774983</v>
       </c>
       <c r="L5" t="n">
-        <v>33.07166879679361</v>
+        <v>32.90188300904665</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>863325</v>
+        <v>861140</v>
       </c>
       <c r="L6" t="n">
-        <v>38.37778356933947</v>
+        <v>38.22142741017721</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1433,7 +1433,7 @@
         <v>100</v>
       </c>
       <c r="Q6" t="n">
-        <v>51.7</v>
+        <v>51.6</v>
       </c>
       <c r="R6" t="n">
         <v>4</v>
@@ -1600,10 +1600,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>863325</v>
+        <v>861140</v>
       </c>
       <c r="L9" t="n">
-        <v>34.55535285089624</v>
+        <v>34.38929790742505</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1667,10 +1667,10 @@
         <v>582999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>863325</v>
+        <v>861140</v>
       </c>
       <c r="L10" t="n">
-        <v>32.47050647207019</v>
+        <v>32.29916157651485</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -1685,7 +1685,7 @@
         <v>50.10670212765957</v>
       </c>
       <c r="Q10" t="n">
-        <v>41.4</v>
+        <v>41.3</v>
       </c>
       <c r="R10" t="n">
         <v>4</v>
@@ -1734,10 +1734,10 @@
         <v>587999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>863325</v>
+        <v>861140</v>
       </c>
       <c r="L11" t="n">
-        <v>31.8913503026091</v>
+        <v>31.71853589427968</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -1801,13 +1801,13 @@
         <v>643999</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>949701</v>
+        <v>947298</v>
       </c>
       <c r="L12" t="n">
-        <v>32.18928904992202</v>
+        <v>32.01727439517448</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>-1001</v>
+        <v>0</v>
       </c>
       <c r="N12" t="n">
         <v>0</v>
@@ -1927,10 +1927,10 @@
         <v>650000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>949701</v>
+        <v>947298</v>
       </c>
       <c r="L14" t="n">
-        <v>31.5574059625082</v>
+        <v>31.38378841716123</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -1994,10 +1994,10 @@
         <v>650000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>863325</v>
+        <v>861140</v>
       </c>
       <c r="L15" t="n">
-        <v>24.70969797005763</v>
+        <v>24.51866130942704</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0</v>
@@ -2009,7 +2009,7 @@
         <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>10.6</v>
+        <v>10.5</v>
       </c>
       <c r="R15" t="n">
         <v>3</v>
@@ -2058,10 +2058,10 @@
         <v>650000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>863325</v>
+        <v>861140</v>
       </c>
       <c r="L16" t="n">
-        <v>24.70969797005763</v>
+        <v>24.51866130942704</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -2073,7 +2073,7 @@
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>10.6</v>
+        <v>10.5</v>
       </c>
       <c r="R16" t="n">
         <v>3</v>
@@ -2122,10 +2122,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1036076</v>
+        <v>1033455</v>
       </c>
       <c r="L17" t="n">
-        <v>32.43738876298649</v>
+        <v>32.26603964371937</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2140,7 +2140,7 @@
         <v>100</v>
       </c>
       <c r="Q17" t="n">
-        <v>49.7</v>
+        <v>49.6</v>
       </c>
       <c r="R17" t="n">
         <v>4</v>
@@ -2154,11 +2154,11 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 16Inch MX2X3 14Core CPU 20Core GPU M4 Pro 24GB 512GB Space Black</t>
+          <t>Apple MacBook Pro 14Inch MX2F3 M4 Pro 14Core CPU 20Core GPU 24GB 1TB Silver</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2169,7 +2169,7 @@
         <v>24</v>
       </c>
       <c r="E18" t="n">
-        <v>512</v>
+        <v>1024</v>
       </c>
       <c r="F18" t="n">
         <v>14</v>
@@ -2179,20 +2179,20 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I18" s="3" t="n">
-        <v>707999</v>
+        <v>720000</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>707999</v>
+        <v>720000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>1079264</v>
+        <v>1033455</v>
       </c>
       <c r="L18" t="n">
-        <v>34.39983173718386</v>
+        <v>30.33078363353992</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -2201,13 +2201,13 @@
         <v>0</v>
       </c>
       <c r="O18" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="P18" t="n">
-        <v>12.49398266190719</v>
+        <v>82.22222222222221</v>
       </c>
       <c r="Q18" t="n">
-        <v>35.8</v>
+        <v>23.8</v>
       </c>
       <c r="R18" t="n">
         <v>4</v>
@@ -2221,7 +2221,7 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 14Inch MX2F3 M4 Pro 14Core CPU 20Core GPU 24GB 1TB Silver</t>
+          <t>Macbook Pro 14 MGDR4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>M4 Pro</t>
+          <t>M5 Pro</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -2239,45 +2239,40 @@
         <v>1024</v>
       </c>
       <c r="F19" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G19" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I19" s="3" t="n">
-        <v>720000</v>
+        <v>724999</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>720000</v>
-      </c>
-      <c r="K19" s="3" t="n">
-        <v>1036076</v>
-      </c>
-      <c r="L19" t="n">
-        <v>30.50702844192897</v>
-      </c>
+        <v>724999</v>
+      </c>
+      <c r="K19" s="3" t="n"/>
       <c r="M19" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>0</v>
+        <v>0.4122252747252748</v>
       </c>
       <c r="O19" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="P19" t="n">
-        <v>82.22222222222221</v>
+        <v>45.20575342465755</v>
       </c>
       <c r="Q19" t="n">
-        <v>23.9</v>
+        <v>44.8</v>
       </c>
       <c r="R19" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S19" t="inlineStr">
         <is>
@@ -2288,7 +2283,7 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 MGDR4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Space Black</t>
+          <t>Macbook Pro 14 MGDN4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Silver</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -2313,30 +2308,30 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I20" s="3" t="n">
-        <v>724999</v>
+        <v>729999</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>724999</v>
+        <v>729999</v>
       </c>
       <c r="K20" s="3" t="n"/>
       <c r="M20" s="3" t="n">
-        <v>-3001</v>
+        <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>0.4122252747252748</v>
+        <v>0.6804081632653061</v>
       </c>
       <c r="O20" t="n">
-        <v>100</v>
+        <v>96.96971533505857</v>
       </c>
       <c r="P20" t="n">
-        <v>45.20575342465755</v>
+        <v>43.83589041095892</v>
       </c>
       <c r="Q20" t="n">
-        <v>44.8</v>
+        <v>43.6</v>
       </c>
       <c r="R20" t="n">
         <v>3</v>
@@ -2350,58 +2345,63 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 MGDN4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Silver</t>
+          <t>Apple MacBook Pro 16Inch MX2X3 14Core CPU 20Core GPU M4 Pro 24GB 512GB Space Black</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>M5 Pro</t>
+          <t>M4 Pro</t>
         </is>
       </c>
       <c r="D21" t="n">
         <v>24</v>
       </c>
       <c r="E21" t="n">
-        <v>1024</v>
+        <v>512</v>
       </c>
       <c r="F21" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G21" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I21" s="3" t="n">
-        <v>729999</v>
+        <v>739999</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>729999</v>
-      </c>
-      <c r="K21" s="3" t="n"/>
+        <v>739999</v>
+      </c>
+      <c r="K21" s="3" t="n">
+        <v>1076533</v>
+      </c>
+      <c r="L21" t="n">
+        <v>31.26090886205997</v>
+      </c>
       <c r="M21" s="3" t="n">
-        <v>-5001</v>
+        <v>32000</v>
       </c>
       <c r="N21" t="n">
-        <v>0.6804081632653061</v>
+        <v>0</v>
       </c>
       <c r="O21" t="n">
-        <v>96.96971533505857</v>
+        <v>100</v>
       </c>
       <c r="P21" t="n">
-        <v>43.83589041095892</v>
+        <v>1.071239163691994</v>
       </c>
       <c r="Q21" t="n">
-        <v>43.6</v>
+        <v>32.8</v>
       </c>
       <c r="R21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S21" t="inlineStr">
         <is>
@@ -2447,10 +2447,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1079264</v>
+        <v>1076533</v>
       </c>
       <c r="L22" t="n">
-        <v>31.15678832982477</v>
+        <v>30.9821436035867</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2465,7 +2465,7 @@
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>10.4</v>
+        <v>10.3</v>
       </c>
       <c r="R22" t="n">
         <v>4</v>
@@ -2514,10 +2514,10 @@
         <v>745000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1036076</v>
+        <v>1033455</v>
       </c>
       <c r="L23" t="n">
-        <v>28.09407804060706</v>
+        <v>27.91171362081561</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -2532,7 +2532,7 @@
         <v>77.6595744680851</v>
       </c>
       <c r="Q23" t="n">
-        <v>45.5</v>
+        <v>45.4</v>
       </c>
       <c r="R23" t="n">
         <v>4</v>
@@ -2581,10 +2581,10 @@
         <v>755000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1036076</v>
+        <v>1033455</v>
       </c>
       <c r="L24" t="n">
-        <v>27.12889788007829</v>
+        <v>26.94408561572589</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -2648,10 +2648,10 @@
         <v>772000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>1036076</v>
+        <v>1033455</v>
       </c>
       <c r="L25" t="n">
-        <v>25.4880916071794</v>
+        <v>25.29911800707336</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -2666,7 +2666,7 @@
         <v>71.91489361702126</v>
       </c>
       <c r="Q25" t="n">
-        <v>20.5</v>
+        <v>20.4</v>
       </c>
       <c r="R25" t="n">
         <v>4</v>
@@ -2777,10 +2777,10 @@
         <v>810000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>1252016</v>
+        <v>1248848</v>
       </c>
       <c r="L27" t="n">
-        <v>35.30434115857945</v>
+        <v>35.14022523157342</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -2795,7 +2795,7 @@
         <v>100</v>
       </c>
       <c r="Q27" t="n">
-        <v>50.7</v>
+        <v>50.6</v>
       </c>
       <c r="R27" t="n">
         <v>4</v>
@@ -2906,13 +2906,13 @@
         <v>829999</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>1295204</v>
+        <v>1291926</v>
       </c>
       <c r="L29" t="n">
-        <v>35.91750797557759</v>
+        <v>35.75491165902691</v>
       </c>
       <c r="M29" s="3" t="n">
-        <v>-3000</v>
+        <v>0</v>
       </c>
       <c r="N29" t="n">
         <v>0.3601444899693757</v>
@@ -2924,7 +2924,7 @@
         <v>3.563830734966613</v>
       </c>
       <c r="Q29" t="n">
-        <v>34.9</v>
+        <v>34.8</v>
       </c>
       <c r="R29" t="n">
         <v>4</v>
@@ -2973,10 +2973,10 @@
         <v>835000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1079264</v>
+        <v>1076533</v>
       </c>
       <c r="L30" t="n">
-        <v>22.63246063984345</v>
+        <v>22.43619099460955</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -3037,13 +3037,13 @@
         <v>840000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1295204</v>
+        <v>1291926</v>
       </c>
       <c r="L31" t="n">
-        <v>35.1453516202853</v>
+        <v>34.9807961137093</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>-30000</v>
+        <v>0</v>
       </c>
       <c r="N31" t="n">
         <v>3.448275862068965</v>
@@ -3055,7 +3055,7 @@
         <v>0</v>
       </c>
       <c r="Q31" t="n">
-        <v>12.7</v>
+        <v>12.6</v>
       </c>
       <c r="R31" t="n">
         <v>4</v>
@@ -3104,10 +3104,10 @@
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1381579</v>
+        <v>1378083</v>
       </c>
       <c r="L32" t="n">
-        <v>38.62102710015135</v>
+        <v>38.4653174010564</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3122,7 +3122,7 @@
         <v>100</v>
       </c>
       <c r="Q32" t="n">
-        <v>47.5</v>
+        <v>47.4</v>
       </c>
       <c r="R32" t="n">
         <v>5</v>
@@ -3171,10 +3171,10 @@
         <v>930000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1381579</v>
+        <v>1378083</v>
       </c>
       <c r="L33" t="n">
-        <v>38.47626520090418</v>
+        <v>38.3201882615198</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3238,10 +3238,10 @@
         <v>860000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>1252016</v>
+        <v>1248848</v>
       </c>
       <c r="L34" t="n">
-        <v>31.31078197083743</v>
+        <v>31.13653543105326</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -3256,7 +3256,7 @@
         <v>89.80112187659357</v>
       </c>
       <c r="Q34" t="n">
-        <v>25.4</v>
+        <v>25.3</v>
       </c>
       <c r="R34" t="n">
         <v>4</v>
@@ -3491,10 +3491,10 @@
         <v>890000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>1165640</v>
+        <v>1162690</v>
       </c>
       <c r="L38" t="n">
-        <v>23.64709515802478</v>
+        <v>23.45337106193396</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -3506,7 +3506,7 @@
         <v>73.86018237082067</v>
       </c>
       <c r="Q38" t="n">
-        <v>26</v>
+        <v>25.9</v>
       </c>
       <c r="R38" t="n">
         <v>3</v>
@@ -3555,10 +3555,10 @@
         <v>960000</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>1252016</v>
+        <v>1248848</v>
       </c>
       <c r="L39" t="n">
-        <v>23.32366359535341</v>
+        <v>23.12915583001294</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -3570,7 +3570,7 @@
         <v>82.97872340425533</v>
       </c>
       <c r="Q39" t="n">
-        <v>27.8</v>
+        <v>27.7</v>
       </c>
       <c r="R39" t="n">
         <v>3</v>
@@ -3619,10 +3619,10 @@
         <v>970000</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>1511143</v>
+        <v>1507319</v>
       </c>
       <c r="L40" t="n">
-        <v>35.81017812344696</v>
+        <v>35.6473314540585</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -3748,10 +3748,10 @@
         <v>1022000</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>1511143</v>
+        <v>1507319</v>
       </c>
       <c r="L42" t="n">
-        <v>32.36907427027091</v>
+        <v>32.19749767633792</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -3815,10 +3815,10 @@
         <v>1063000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1554331</v>
+        <v>1550397</v>
       </c>
       <c r="L43" t="n">
-        <v>31.61044848233742</v>
+        <v>31.43691583510546</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -3833,7 +3833,7 @@
         <v>62.58351893095768</v>
       </c>
       <c r="Q43" t="n">
-        <v>43.2</v>
+        <v>43.1</v>
       </c>
       <c r="R43" t="n">
         <v>4</v>
@@ -3882,13 +3882,13 @@
         <v>1080000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1554331</v>
+        <v>1550397</v>
       </c>
       <c r="L44" t="n">
-        <v>30.51673034894112</v>
+        <v>30.34042248533763</v>
       </c>
       <c r="M44" s="3" t="n">
-        <v>-5000</v>
+        <v>0</v>
       </c>
       <c r="N44" t="n">
         <v>0.4608294930875576</v>
@@ -3900,7 +3900,7 @@
         <v>58.79732739420935</v>
       </c>
       <c r="Q44" t="n">
-        <v>20.1</v>
+        <v>20</v>
       </c>
       <c r="R44" t="n">
         <v>4</v>
@@ -4011,10 +4011,10 @@
         <v>1123000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1727082</v>
+        <v>1722712</v>
       </c>
       <c r="L46" t="n">
-        <v>34.97703062159179</v>
+        <v>34.81208698842291</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -4078,10 +4078,10 @@
         <v>1150000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1511143</v>
+        <v>1507319</v>
       </c>
       <c r="L47" t="n">
-        <v>23.8986647855299</v>
+        <v>23.7055991465642</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -4093,7 +4093,7 @@
         <v>89.36170212765958</v>
       </c>
       <c r="Q47" t="n">
-        <v>29.4</v>
+        <v>29.3</v>
       </c>
       <c r="R47" t="n">
         <v>3</v>
@@ -4142,10 +4142,10 @@
         <v>1150000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1511143</v>
+        <v>1507319</v>
       </c>
       <c r="L48" t="n">
-        <v>23.8986647855299</v>
+        <v>23.7055991465642</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -4157,7 +4157,7 @@
         <v>6.617881005408838</v>
       </c>
       <c r="Q48" t="n">
-        <v>11.7</v>
+        <v>11.6</v>
       </c>
       <c r="R48" t="n">
         <v>3</v>
@@ -4206,10 +4206,10 @@
         <v>1155000</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>1770270</v>
+        <v>1765790</v>
       </c>
       <c r="L49" t="n">
-        <v>34.75571522988019</v>
+        <v>34.59018343064577</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -4270,10 +4270,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1770270</v>
+        <v>1765790</v>
       </c>
       <c r="L50" t="n">
-        <v>34.75571522988019</v>
+        <v>34.59018343064577</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4396,10 +4396,10 @@
         <v>1207000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1899833</v>
+        <v>1895026</v>
       </c>
       <c r="L52" t="n">
-        <v>36.46810009090273</v>
+        <v>36.30694249049881</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -4460,10 +4460,10 @@
         <v>1207000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1899833</v>
+        <v>1895026</v>
       </c>
       <c r="L53" t="n">
-        <v>36.46810009090273</v>
+        <v>36.30694249049881</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -4475,7 +4475,7 @@
         <v>9.265033407572403</v>
       </c>
       <c r="Q53" t="n">
-        <v>17.7</v>
+        <v>17.6</v>
       </c>
       <c r="R53" t="n">
         <v>3</v>
@@ -4524,10 +4524,10 @@
         <v>1210000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1597518</v>
+        <v>1593476</v>
       </c>
       <c r="L54" t="n">
-        <v>24.25750445378393</v>
+        <v>24.06537657297631</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -4539,7 +4539,7 @@
         <v>95.74468085106383</v>
       </c>
       <c r="Q54" t="n">
-        <v>30.9</v>
+        <v>30.8</v>
       </c>
       <c r="R54" t="n">
         <v>3</v>
@@ -4588,10 +4588,10 @@
         <v>1215000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1597518</v>
+        <v>1593476</v>
       </c>
       <c r="L55" t="n">
-        <v>23.94451893499792</v>
+        <v>23.75159713732745</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -4714,10 +4714,10 @@
         <v>1280000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1683894</v>
+        <v>1679633</v>
       </c>
       <c r="L57" t="n">
-        <v>23.98571406513712</v>
+        <v>23.79287618188021</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -4729,7 +4729,7 @@
         <v>100</v>
       </c>
       <c r="Q57" t="n">
-        <v>31.7</v>
+        <v>31.6</v>
       </c>
       <c r="R57" t="n">
         <v>3</v>
@@ -4778,10 +4778,10 @@
         <v>1280000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>1727082</v>
+        <v>1722712</v>
       </c>
       <c r="L58" t="n">
-        <v>25.88655315729074</v>
+        <v>25.69854972856752</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -4845,10 +4845,10 @@
         <v>1310000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1727082</v>
+        <v>1722712</v>
       </c>
       <c r="L59" t="n">
-        <v>24.14951924691474</v>
+        <v>23.95710948783082</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -4860,7 +4860,7 @@
         <v>65.92427616926503</v>
       </c>
       <c r="Q59" t="n">
-        <v>24.5</v>
+        <v>24.4</v>
       </c>
       <c r="R59" t="n">
         <v>3</v>
@@ -4909,10 +4909,10 @@
         <v>1338000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1770270</v>
+        <v>1765790</v>
       </c>
       <c r="L60" t="n">
-        <v>24.41830907149757</v>
+        <v>24.22655015602082</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -4924,7 +4924,7 @@
         <v>60.93541202672606</v>
       </c>
       <c r="Q60" t="n">
-        <v>23.5</v>
+        <v>23.4</v>
       </c>
       <c r="R60" t="n">
         <v>3</v>
@@ -4973,10 +4973,10 @@
         <v>1370000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1813458</v>
+        <v>1808869</v>
       </c>
       <c r="L61" t="n">
-        <v>24.45372321829345</v>
+        <v>24.26206651780754</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -4988,7 +4988,7 @@
         <v>87.44292237442922</v>
       </c>
       <c r="Q61" t="n">
-        <v>29.2</v>
+        <v>29.1</v>
       </c>
       <c r="R61" t="n">
         <v>3</v>
@@ -5096,10 +5096,10 @@
         <v>1460000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>2158960</v>
+        <v>2153497</v>
       </c>
       <c r="L63" t="n">
-        <v>32.37484714862712</v>
+        <v>32.20329538420532</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -5160,10 +5160,10 @@
         <v>1460000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>2158960</v>
+        <v>2153497</v>
       </c>
       <c r="L64" t="n">
-        <v>32.37484714862712</v>
+        <v>32.20329538420532</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -5224,10 +5224,10 @@
         <v>1471000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1943021</v>
+        <v>1938105</v>
       </c>
       <c r="L65" t="n">
-        <v>24.29314968803734</v>
+        <v>24.10111939239618</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -5239,7 +5239,7 @@
         <v>80.92056421677803</v>
       </c>
       <c r="Q65" t="n">
-        <v>27.8</v>
+        <v>27.7</v>
       </c>
       <c r="R65" t="n">
         <v>3</v>
@@ -5288,10 +5288,10 @@
         <v>1471000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1943021</v>
+        <v>1938105</v>
       </c>
       <c r="L66" t="n">
-        <v>24.29314968803734</v>
+        <v>24.10111939239618</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -5303,7 +5303,7 @@
         <v>61.06499291354523</v>
       </c>
       <c r="Q66" t="n">
-        <v>23.5</v>
+        <v>23.4</v>
       </c>
       <c r="R66" t="n">
         <v>3</v>
@@ -5414,10 +5414,10 @@
         <v>1535000</v>
       </c>
       <c r="K68" s="3" t="n">
-        <v>2029397</v>
+        <v>2024262</v>
       </c>
       <c r="L68" t="n">
-        <v>24.36176854504072</v>
+        <v>24.16989500370999</v>
       </c>
       <c r="M68" s="3" t="n">
         <v>0</v>
@@ -5540,10 +5540,10 @@
         <v>1650000</v>
       </c>
       <c r="K70" s="3" t="n">
-        <v>2202148</v>
+        <v>2196576</v>
       </c>
       <c r="L70" t="n">
-        <v>25.07315584601943</v>
+        <v>24.88309077400463</v>
       </c>
       <c r="M70" s="3" t="n">
         <v>0</v>
@@ -5604,10 +5604,10 @@
         <v>1660000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2202148</v>
+        <v>2196576</v>
       </c>
       <c r="L71" t="n">
-        <v>24.61905376023773</v>
+        <v>24.42783677869557</v>
       </c>
       <c r="M71" s="3" t="n">
         <v>0</v>
@@ -5619,7 +5619,7 @@
         <v>26.6373948042444</v>
       </c>
       <c r="Q71" t="n">
-        <v>16.3</v>
+        <v>16.2</v>
       </c>
       <c r="R71" t="n">
         <v>3</v>
@@ -5668,10 +5668,10 @@
         <v>1661000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2202148</v>
+        <v>2196576</v>
       </c>
       <c r="L72" t="n">
-        <v>24.57364355165956</v>
+        <v>24.38231137916467</v>
       </c>
       <c r="M72" s="3" t="n">
         <v>0</v>
@@ -5683,7 +5683,7 @@
         <v>87.94145720649061</v>
       </c>
       <c r="Q72" t="n">
-        <v>29.4</v>
+        <v>29.3</v>
       </c>
       <c r="R72" t="n">
         <v>3</v>
@@ -5732,10 +5732,10 @@
         <v>1680000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2245336</v>
+        <v>2239654</v>
       </c>
       <c r="L73" t="n">
-        <v>25.17823613036089</v>
+        <v>24.98841338885381</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
@@ -5747,7 +5747,7 @@
         <v>100</v>
       </c>
       <c r="Q73" t="n">
-        <v>32.2</v>
+        <v>32.1</v>
       </c>
       <c r="R73" t="n">
         <v>3</v>
@@ -5796,10 +5796,10 @@
         <v>1711000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2331712</v>
+        <v>2325812</v>
       </c>
       <c r="L74" t="n">
-        <v>26.62044026020366</v>
+        <v>26.43429477533008</v>
       </c>
       <c r="M74" s="3" t="n">
         <v>0</v>
@@ -5860,10 +5860,10 @@
         <v>1756000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2331712</v>
+        <v>2325812</v>
       </c>
       <c r="L75" t="n">
-        <v>24.69052781818681</v>
+        <v>24.49948663090568</v>
       </c>
       <c r="M75" s="3" t="n">
         <v>0</v>
@@ -5875,7 +5875,7 @@
         <v>0</v>
       </c>
       <c r="Q75" t="n">
-        <v>10.6</v>
+        <v>10.5</v>
       </c>
       <c r="R75" t="n">
         <v>3</v>
@@ -5924,10 +5924,10 @@
         <v>1790000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2374900</v>
+        <v>2368890</v>
       </c>
       <c r="L76" t="n">
-        <v>24.62840540654343</v>
+        <v>24.43718365985757</v>
       </c>
       <c r="M76" s="3" t="n">
         <v>0</v>
@@ -5939,7 +5939,7 @@
         <v>100</v>
       </c>
       <c r="Q76" t="n">
-        <v>32</v>
+        <v>31.9</v>
       </c>
       <c r="R76" t="n">
         <v>3</v>
@@ -5988,10 +5988,10 @@
         <v>1840000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2461275</v>
+        <v>2455047</v>
       </c>
       <c r="L77" t="n">
-        <v>25.24199855765812</v>
+        <v>25.05235133991325</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
@@ -6003,7 +6003,7 @@
         <v>38.76430923631803</v>
       </c>
       <c r="Q77" t="n">
-        <v>19.1</v>
+        <v>19</v>
       </c>
       <c r="R77" t="n">
         <v>3</v>
@@ -6052,10 +6052,10 @@
         <v>1945000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2590839</v>
+        <v>2584283</v>
       </c>
       <c r="L78" t="n">
-        <v>24.92779366066359</v>
+        <v>24.73734494248502</v>
       </c>
       <c r="M78" s="3" t="n">
         <v>0</v>
@@ -6067,7 +6067,7 @@
         <v>15.83200763601658</v>
       </c>
       <c r="Q78" t="n">
-        <v>14.1</v>
+        <v>14</v>
       </c>
       <c r="R78" t="n">
         <v>3</v>
@@ -6116,10 +6116,10 @@
         <v>1960000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2634027</v>
+        <v>2627361</v>
       </c>
       <c r="L79" t="n">
-        <v>25.58922137092748</v>
+        <v>25.40043031772185</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
@@ -6180,10 +6180,10 @@
         <v>2078000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2763590</v>
+        <v>2756597</v>
       </c>
       <c r="L80" t="n">
-        <v>24.80794908072471</v>
+        <v>24.61720012029324</v>
       </c>
       <c r="M80" s="3" t="n">
         <v>0</v>
@@ -6195,7 +6195,7 @@
         <v>35.18930957683743</v>
       </c>
       <c r="Q80" t="n">
-        <v>18.2</v>
+        <v>18.1</v>
       </c>
       <c r="R80" t="n">
         <v>3</v>
@@ -6244,10 +6244,10 @@
         <v>2170000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2893154</v>
+        <v>2885833</v>
       </c>
       <c r="L81" t="n">
-        <v>24.99535109434202</v>
+        <v>24.80507361306077</v>
       </c>
       <c r="M81" s="3" t="n">
         <v>0</v>
@@ -6308,10 +6308,10 @@
         <v>2268000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>3022717</v>
+        <v>3015069</v>
       </c>
       <c r="L82" t="n">
-        <v>24.968166057226</v>
+        <v>24.77784090513351</v>
       </c>
       <c r="M82" s="3" t="n">
         <v>0</v>
@@ -6323,7 +6323,7 @@
         <v>70.41425389755011</v>
       </c>
       <c r="Q82" t="n">
-        <v>25.8</v>
+        <v>25.7</v>
       </c>
       <c r="R82" t="n">
         <v>3</v>
@@ -6372,10 +6372,10 @@
         <v>2270000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3065905</v>
+        <v>3058147</v>
       </c>
       <c r="L83" t="n">
-        <v>25.95987155505471</v>
+        <v>25.77204431310856</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
@@ -6387,7 +6387,7 @@
         <v>75.11445476694064</v>
       </c>
       <c r="Q83" t="n">
-        <v>27.2</v>
+        <v>27.1</v>
       </c>
       <c r="R83" t="n">
         <v>3</v>
@@ -6436,10 +6436,10 @@
         <v>2381000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3195469</v>
+        <v>3187383</v>
       </c>
       <c r="L84" t="n">
-        <v>25.48824601333951</v>
+        <v>25.29921882622829</v>
       </c>
       <c r="M84" s="3" t="n">
         <v>0</v>
@@ -6451,7 +6451,7 @@
         <v>64.54234341897987</v>
       </c>
       <c r="Q84" t="n">
-        <v>24.8</v>
+        <v>24.7</v>
       </c>
       <c r="R84" t="n">
         <v>3</v>
@@ -6500,10 +6500,10 @@
         <v>2470000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3325032</v>
+        <v>3316618</v>
       </c>
       <c r="L85" t="n">
-        <v>25.71500063758785</v>
+        <v>25.52654541463624</v>
       </c>
       <c r="M85" s="3" t="n">
         <v>0</v>
@@ -6515,7 +6515,7 @@
         <v>88.84010245151846</v>
       </c>
       <c r="Q85" t="n">
-        <v>30.1</v>
+        <v>30</v>
       </c>
       <c r="R85" t="n">
         <v>3</v>
@@ -6564,10 +6564,10 @@
         <v>2480000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3325032</v>
+        <v>3316618</v>
       </c>
       <c r="L86" t="n">
-        <v>25.41425165231492</v>
+        <v>25.22503345275217</v>
       </c>
       <c r="M86" s="3" t="n">
         <v>0</v>
@@ -6628,10 +6628,10 @@
         <v>2571000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3454596</v>
+        <v>3445854</v>
       </c>
       <c r="L87" t="n">
-        <v>25.57740470955214</v>
+        <v>25.38859742751724</v>
       </c>
       <c r="M87" s="3" t="n">
         <v>0</v>
@@ -6643,7 +6643,7 @@
         <v>83.83073496659243</v>
       </c>
       <c r="Q87" t="n">
-        <v>28.9</v>
+        <v>28.8</v>
       </c>
       <c r="R87" t="n">
         <v>3</v>
@@ -6692,10 +6692,10 @@
         <v>2580000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3497784</v>
+        <v>3488933</v>
       </c>
       <c r="L88" t="n">
-        <v>26.23901304368709</v>
+        <v>26.05189036304222</v>
       </c>
       <c r="M88" s="3" t="n">
         <v>0</v>
@@ -6707,7 +6707,7 @@
         <v>80.79034028540066</v>
       </c>
       <c r="Q88" t="n">
-        <v>28.6</v>
+        <v>28.5</v>
       </c>
       <c r="R88" t="n">
         <v>3</v>
@@ -6756,10 +6756,10 @@
         <v>2581000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3454596</v>
+        <v>3445854</v>
       </c>
       <c r="L89" t="n">
-        <v>25.28793526073671</v>
+        <v>25.09839360576508</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
@@ -6820,10 +6820,10 @@
         <v>2664000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3627347</v>
+        <v>3618168</v>
       </c>
       <c r="L90" t="n">
-        <v>26.55789479197882</v>
+        <v>26.37157810250934</v>
       </c>
       <c r="M90" s="3" t="n">
         <v>0</v>
@@ -6835,7 +6835,7 @@
         <v>75.54565701559021</v>
       </c>
       <c r="Q90" t="n">
-        <v>27.6</v>
+        <v>27.5</v>
       </c>
       <c r="R90" t="n">
         <v>3</v>
@@ -6884,10 +6884,10 @@
         <v>3090000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>4188789</v>
+        <v>4178190</v>
       </c>
       <c r="L91" t="n">
-        <v>26.23166265954193</v>
+        <v>26.04453124439051</v>
       </c>
       <c r="M91" s="3" t="n">
         <v>0</v>
@@ -6899,7 +6899,7 @@
         <v>100</v>
       </c>
       <c r="Q91" t="n">
-        <v>32.7</v>
+        <v>32.6</v>
       </c>
       <c r="R91" t="n">
         <v>3</v>
@@ -6948,10 +6948,10 @@
         <v>3186000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4318353</v>
+        <v>4307425</v>
       </c>
       <c r="L92" t="n">
-        <v>26.22187208873383</v>
+        <v>26.0346959030047</v>
       </c>
       <c r="M92" s="3" t="n">
         <v>0</v>
@@ -6963,7 +6963,7 @@
         <v>100</v>
       </c>
       <c r="Q92" t="n">
-        <v>32.7</v>
+        <v>32.6</v>
       </c>
       <c r="R92" t="n">
         <v>3</v>
@@ -7246,10 +7246,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>431447</v>
+        <v>430355</v>
       </c>
       <c r="L2" t="n">
-        <v>28.14899628459579</v>
+        <v>27.96667867225895</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7264,7 +7264,7 @@
         <v>29.71702857142851</v>
       </c>
       <c r="Q2" t="n">
-        <v>36.6</v>
+        <v>36.5</v>
       </c>
       <c r="R2" t="n">
         <v>4</v>
@@ -7313,10 +7313,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>431447</v>
+        <v>430355</v>
       </c>
       <c r="L3" t="n">
-        <v>28.14899628459579</v>
+        <v>27.96667867225895</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7331,7 +7331,7 @@
         <v>29.71702857142851</v>
       </c>
       <c r="Q3" t="n">
-        <v>36.6</v>
+        <v>36.5</v>
       </c>
       <c r="R3" t="n">
         <v>4</v>
@@ -7380,10 +7380,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>431447</v>
+        <v>430355</v>
       </c>
       <c r="L4" t="n">
-        <v>28.14876450641678</v>
+        <v>27.96644630595671</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7447,10 +7447,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>431447</v>
+        <v>430355</v>
       </c>
       <c r="L5" t="n">
-        <v>28.14876450641678</v>
+        <v>27.96644630595671</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7514,10 +7514,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>517822</v>
+        <v>516512</v>
       </c>
       <c r="L6" t="n">
-        <v>25.84324343114043</v>
+        <v>25.65516386840964</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7529,7 +7529,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>11.1</v>
+        <v>11</v>
       </c>
       <c r="R6" t="n">
         <v>3</v>
@@ -7578,10 +7578,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>517822</v>
+        <v>516512</v>
       </c>
       <c r="L7" t="n">
-        <v>25.84324343114043</v>
+        <v>25.65516386840964</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7593,7 +7593,7 @@
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>11.1</v>
+        <v>11</v>
       </c>
       <c r="R7" t="n">
         <v>3</v>
@@ -7642,10 +7642,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>517822</v>
+        <v>516512</v>
       </c>
       <c r="L8" t="n">
-        <v>25.84324343114043</v>
+        <v>25.65516386840964</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7657,7 +7657,7 @@
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>11.1</v>
+        <v>11</v>
       </c>
       <c r="R8" t="n">
         <v>3</v>
@@ -7706,10 +7706,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>517822</v>
+        <v>516512</v>
       </c>
       <c r="L9" t="n">
-        <v>25.84324343114043</v>
+        <v>25.65516386840964</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7721,7 +7721,7 @@
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>11.1</v>
+        <v>11</v>
       </c>
       <c r="R9" t="n">
         <v>3</v>
@@ -7770,10 +7770,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>517822</v>
+        <v>516512</v>
       </c>
       <c r="L10" t="n">
-        <v>25.65012687757569</v>
+        <v>25.46155752431696</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7785,7 +7785,7 @@
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>11</v>
+        <v>10.9</v>
       </c>
       <c r="R10" t="n">
         <v>3</v>
@@ -7834,10 +7834,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>517822</v>
+        <v>516512</v>
       </c>
       <c r="L11" t="n">
-        <v>25.65012687757569</v>
+        <v>25.46155752431696</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7849,7 +7849,7 @@
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>11</v>
+        <v>10.9</v>
       </c>
       <c r="R11" t="n">
         <v>3</v>
@@ -7898,10 +7898,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>517822</v>
+        <v>516512</v>
       </c>
       <c r="L12" t="n">
-        <v>25.65012687757569</v>
+        <v>25.46155752431696</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -7913,7 +7913,7 @@
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>11</v>
+        <v>10.9</v>
       </c>
       <c r="R12" t="n">
         <v>3</v>
@@ -7962,10 +7962,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>517822</v>
+        <v>516512</v>
       </c>
       <c r="L13" t="n">
-        <v>25.65012687757569</v>
+        <v>25.46155752431696</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -7977,7 +7977,7 @@
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>11</v>
+        <v>10.9</v>
       </c>
       <c r="R13" t="n">
         <v>3</v>
@@ -8026,13 +8026,13 @@
         <v>433999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>561010</v>
+        <v>559591</v>
       </c>
       <c r="L14" t="n">
-        <v>22.6397033920964</v>
+        <v>22.44353465298763</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>-8000</v>
+        <v>0</v>
       </c>
       <c r="N14" t="n">
         <v>3.125006975461999</v>
@@ -8093,13 +8093,13 @@
         <v>433999</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>561010</v>
+        <v>559591</v>
       </c>
       <c r="L15" t="n">
-        <v>22.6397033920964</v>
+        <v>22.44353465298763</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>-1000</v>
+        <v>0</v>
       </c>
       <c r="N15" t="n">
         <v>0</v>
@@ -8111,7 +8111,7 @@
         <v>10.75021216407353</v>
       </c>
       <c r="Q15" t="n">
-        <v>31.6</v>
+        <v>31.5</v>
       </c>
       <c r="R15" t="n">
         <v>4</v>
@@ -8160,13 +8160,13 @@
         <v>433999</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>561010</v>
+        <v>559591</v>
       </c>
       <c r="L16" t="n">
-        <v>22.6397033920964</v>
+        <v>22.44353465298763</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>3999</v>
+        <v>0</v>
       </c>
       <c r="N16" t="n">
         <v>0</v>
@@ -8178,7 +8178,7 @@
         <v>10.75021216407353</v>
       </c>
       <c r="Q16" t="n">
-        <v>31.6</v>
+        <v>31.5</v>
       </c>
       <c r="R16" t="n">
         <v>4</v>
@@ -8227,13 +8227,13 @@
         <v>443000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>561010</v>
+        <v>559591</v>
       </c>
       <c r="L17" t="n">
-        <v>21.03527566353541</v>
+        <v>20.83503844772343</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>-4999</v>
+        <v>0</v>
       </c>
       <c r="N17" t="n">
         <v>1.115850705023895</v>
@@ -8245,7 +8245,7 @@
         <v>5.657708628005674</v>
       </c>
       <c r="Q17" t="n">
-        <v>20</v>
+        <v>19.9</v>
       </c>
       <c r="R17" t="n">
         <v>4</v>
@@ -8294,10 +8294,10 @@
         <v>453000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>561010</v>
+        <v>559591</v>
       </c>
       <c r="L18" t="n">
-        <v>19.25277624284772</v>
+        <v>19.04801899959077</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -8312,7 +8312,7 @@
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="R18" t="n">
         <v>4</v>
@@ -8361,10 +8361,10 @@
         <v>454000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>604198</v>
+        <v>602669</v>
       </c>
       <c r="L19" t="n">
-        <v>24.85906937791916</v>
+        <v>24.66843325274736</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -8425,10 +8425,10 @@
         <v>454000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>604198</v>
+        <v>602669</v>
       </c>
       <c r="L20" t="n">
-        <v>24.85906937791916</v>
+        <v>24.66843325274736</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -8489,10 +8489,10 @@
         <v>454000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>604198</v>
+        <v>602669</v>
       </c>
       <c r="L21" t="n">
-        <v>24.85906937791916</v>
+        <v>24.66843325274736</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -8553,10 +8553,10 @@
         <v>454000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>604198</v>
+        <v>602669</v>
       </c>
       <c r="L22" t="n">
-        <v>24.85906937791916</v>
+        <v>24.66843325274736</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -8617,10 +8617,10 @@
         <v>455000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>604198</v>
+        <v>602669</v>
       </c>
       <c r="L23" t="n">
-        <v>24.69356072016127</v>
+        <v>24.50250469163007</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -8632,7 +8632,7 @@
         <v>100</v>
       </c>
       <c r="Q23" t="n">
-        <v>32</v>
+        <v>31.9</v>
       </c>
       <c r="R23" t="n">
         <v>3</v>
@@ -8681,10 +8681,10 @@
         <v>455000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>604198</v>
+        <v>602669</v>
       </c>
       <c r="L24" t="n">
-        <v>24.69356072016127</v>
+        <v>24.50250469163007</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -8696,7 +8696,7 @@
         <v>100</v>
       </c>
       <c r="Q24" t="n">
-        <v>32</v>
+        <v>31.9</v>
       </c>
       <c r="R24" t="n">
         <v>3</v>
@@ -8745,10 +8745,10 @@
         <v>455000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>604198</v>
+        <v>602669</v>
       </c>
       <c r="L25" t="n">
-        <v>24.69356072016127</v>
+        <v>24.50250469163007</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -8760,7 +8760,7 @@
         <v>100</v>
       </c>
       <c r="Q25" t="n">
-        <v>32</v>
+        <v>31.9</v>
       </c>
       <c r="R25" t="n">
         <v>3</v>
@@ -8809,10 +8809,10 @@
         <v>455000</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>604198</v>
+        <v>602669</v>
       </c>
       <c r="L26" t="n">
-        <v>24.69356072016127</v>
+        <v>24.50250469163007</v>
       </c>
       <c r="M26" s="3" t="n">
         <v>0</v>
@@ -8824,7 +8824,7 @@
         <v>100</v>
       </c>
       <c r="Q26" t="n">
-        <v>32</v>
+        <v>31.9</v>
       </c>
       <c r="R26" t="n">
         <v>3</v>
@@ -8873,10 +8873,10 @@
         <v>475000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>690574</v>
+        <v>688826</v>
       </c>
       <c r="L27" t="n">
-        <v>31.21664007043416</v>
+        <v>31.04209190709991</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -8888,7 +8888,7 @@
         <v>100</v>
       </c>
       <c r="Q27" t="n">
-        <v>34.8</v>
+        <v>34.7</v>
       </c>
       <c r="R27" t="n">
         <v>3</v>
@@ -8937,10 +8937,10 @@
         <v>475000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>690574</v>
+        <v>688826</v>
       </c>
       <c r="L28" t="n">
-        <v>31.21664007043416</v>
+        <v>31.04209190709991</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -8952,7 +8952,7 @@
         <v>100</v>
       </c>
       <c r="Q28" t="n">
-        <v>34.8</v>
+        <v>34.7</v>
       </c>
       <c r="R28" t="n">
         <v>3</v>
@@ -9001,10 +9001,10 @@
         <v>475000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>690574</v>
+        <v>688826</v>
       </c>
       <c r="L29" t="n">
-        <v>31.21664007043416</v>
+        <v>31.04209190709991</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -9016,7 +9016,7 @@
         <v>100</v>
       </c>
       <c r="Q29" t="n">
-        <v>34.8</v>
+        <v>34.7</v>
       </c>
       <c r="R29" t="n">
         <v>3</v>
@@ -9065,10 +9065,10 @@
         <v>475000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>690574</v>
+        <v>688826</v>
       </c>
       <c r="L30" t="n">
-        <v>31.21664007043416</v>
+        <v>31.04209190709991</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -9080,7 +9080,7 @@
         <v>100</v>
       </c>
       <c r="Q30" t="n">
-        <v>34.8</v>
+        <v>34.7</v>
       </c>
       <c r="R30" t="n">
         <v>3</v>
@@ -9129,10 +9129,10 @@
         <v>479999</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>690574</v>
+        <v>688826</v>
       </c>
       <c r="L31" t="n">
-        <v>30.49274950982806</v>
+        <v>30.31636436487589</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -9193,10 +9193,10 @@
         <v>479999</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>690574</v>
+        <v>688826</v>
       </c>
       <c r="L32" t="n">
-        <v>30.49274950982806</v>
+        <v>30.31636436487589</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -9257,10 +9257,10 @@
         <v>479999</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>690574</v>
+        <v>688826</v>
       </c>
       <c r="L33" t="n">
-        <v>30.49274950982806</v>
+        <v>30.31636436487589</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -9321,10 +9321,10 @@
         <v>479999</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>690574</v>
+        <v>688826</v>
       </c>
       <c r="L34" t="n">
-        <v>30.49274950982806</v>
+        <v>30.31636436487589</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -9385,10 +9385,10 @@
         <v>482999</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>647386</v>
+        <v>645748</v>
       </c>
       <c r="L35" t="n">
-        <v>25.39242430327502</v>
+        <v>25.20317523244361</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
@@ -9403,7 +9403,7 @@
         <v>3.478278152934936</v>
       </c>
       <c r="Q35" t="n">
-        <v>31.3</v>
+        <v>31.2</v>
       </c>
       <c r="R35" t="n">
         <v>4</v>
@@ -9452,10 +9452,10 @@
         <v>482999</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>647386</v>
+        <v>645748</v>
       </c>
       <c r="L36" t="n">
-        <v>25.39242430327502</v>
+        <v>25.20317523244361</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -9470,7 +9470,7 @@
         <v>3.478278152934936</v>
       </c>
       <c r="Q36" t="n">
-        <v>31.3</v>
+        <v>31.2</v>
       </c>
       <c r="R36" t="n">
         <v>4</v>
@@ -9519,10 +9519,10 @@
         <v>482999</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>647386</v>
+        <v>645748</v>
       </c>
       <c r="L37" t="n">
-        <v>25.39242430327502</v>
+        <v>25.20317523244361</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
@@ -9537,7 +9537,7 @@
         <v>3.478278152934936</v>
       </c>
       <c r="Q37" t="n">
-        <v>31.3</v>
+        <v>31.2</v>
       </c>
       <c r="R37" t="n">
         <v>4</v>
@@ -9586,13 +9586,13 @@
         <v>489999</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>647386</v>
+        <v>645748</v>
       </c>
       <c r="L38" t="n">
-        <v>24.31115285162175</v>
+        <v>24.11916103495481</v>
       </c>
       <c r="M38" s="3" t="n">
-        <v>-5001</v>
+        <v>0</v>
       </c>
       <c r="N38" t="n">
         <v>1.01030303030303</v>
@@ -9604,7 +9604,7 @@
         <v>0</v>
       </c>
       <c r="Q38" t="n">
-        <v>8.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="R38" t="n">
         <v>4</v>
@@ -9653,10 +9653,10 @@
         <v>500000</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>647386</v>
+        <v>645748</v>
       </c>
       <c r="L39" t="n">
-        <v>22.76632488190971</v>
+        <v>22.57041446508545</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -9668,7 +9668,7 @@
         <v>44.13012729844413</v>
       </c>
       <c r="Q39" t="n">
-        <v>19.2</v>
+        <v>19.1</v>
       </c>
       <c r="R39" t="n">
         <v>3</v>
@@ -9717,10 +9717,10 @@
         <v>551999</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>776949</v>
+        <v>774983</v>
       </c>
       <c r="L40" t="n">
-        <v>28.95299434068388</v>
+        <v>28.77276017667484</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -9735,7 +9735,7 @@
         <v>68.91123055162657</v>
       </c>
       <c r="Q40" t="n">
-        <v>43.4</v>
+        <v>43.3</v>
       </c>
       <c r="R40" t="n">
         <v>4</v>
@@ -9784,10 +9784,10 @@
         <v>551999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>776949</v>
+        <v>774983</v>
       </c>
       <c r="L41" t="n">
-        <v>28.95299434068388</v>
+        <v>28.77276017667484</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
@@ -9802,7 +9802,7 @@
         <v>68.91123055162657</v>
       </c>
       <c r="Q41" t="n">
-        <v>43.4</v>
+        <v>43.3</v>
       </c>
       <c r="R41" t="n">
         <v>4</v>
@@ -9851,10 +9851,10 @@
         <v>551999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>776949</v>
+        <v>774983</v>
       </c>
       <c r="L42" t="n">
-        <v>28.95299434068388</v>
+        <v>28.77276017667484</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -9869,7 +9869,7 @@
         <v>68.91123055162657</v>
       </c>
       <c r="Q42" t="n">
-        <v>43.4</v>
+        <v>43.3</v>
       </c>
       <c r="R42" t="n">
         <v>4</v>
@@ -9918,10 +9918,10 @@
         <v>557999</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>776949</v>
+        <v>774983</v>
       </c>
       <c r="L43" t="n">
-        <v>28.18074288016331</v>
+        <v>27.99854964560513</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -9985,13 +9985,13 @@
         <v>559999</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>776949</v>
+        <v>774983</v>
       </c>
       <c r="L44" t="n">
-        <v>27.92332572665644</v>
+        <v>27.74047946858189</v>
       </c>
       <c r="M44" s="3" t="n">
-        <v>-5000</v>
+        <v>0</v>
       </c>
       <c r="N44" t="n">
         <v>0.8849573185085283</v>
@@ -10049,13 +10049,13 @@
         <v>559999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>776949</v>
+        <v>774983</v>
       </c>
       <c r="L45" t="n">
-        <v>27.92332572665644</v>
+        <v>27.74047946858189</v>
       </c>
       <c r="M45" s="3" t="n">
-        <v>-5000</v>
+        <v>0</v>
       </c>
       <c r="N45" t="n">
         <v>0.8849573185085283</v>
@@ -10113,13 +10113,13 @@
         <v>559999</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>776949</v>
+        <v>774983</v>
       </c>
       <c r="L46" t="n">
-        <v>27.92332572665644</v>
+        <v>27.74047946858189</v>
       </c>
       <c r="M46" s="3" t="n">
-        <v>-5000</v>
+        <v>0</v>
       </c>
       <c r="N46" t="n">
         <v>0.8849573185085283</v>
@@ -10177,13 +10177,13 @@
         <v>559999</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>776949</v>
+        <v>774983</v>
       </c>
       <c r="L47" t="n">
-        <v>27.92332572665644</v>
+        <v>27.74047946858189</v>
       </c>
       <c r="M47" s="3" t="n">
-        <v>-5000</v>
+        <v>0</v>
       </c>
       <c r="N47" t="n">
         <v>0.8849573185085283</v>
@@ -10241,10 +10241,10 @@
         <v>585000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>733762</v>
+        <v>731905</v>
       </c>
       <c r="L48" t="n">
-        <v>20.27387627050733</v>
+        <v>20.07159399102343</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -10305,10 +10305,10 @@
         <v>595000</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>733762</v>
+        <v>731905</v>
       </c>
       <c r="L49" t="n">
-        <v>18.91103654863566</v>
+        <v>18.70529645240844</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -10369,13 +10369,13 @@
         <v>614999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>863325</v>
+        <v>861140</v>
       </c>
       <c r="L50" t="n">
-        <v>28.76390698751919</v>
+        <v>28.58315721020972</v>
       </c>
       <c r="M50" s="3" t="n">
-        <v>-2000</v>
+        <v>0</v>
       </c>
       <c r="N50" t="n">
         <v>0.3241496339540259</v>
@@ -10384,7 +10384,7 @@
         <v>60.12432359912347</v>
       </c>
       <c r="Q50" t="n">
-        <v>25.3</v>
+        <v>25.2</v>
       </c>
       <c r="R50" t="n">
         <v>3</v>
@@ -10433,13 +10433,13 @@
         <v>614999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>863325</v>
+        <v>861140</v>
       </c>
       <c r="L51" t="n">
-        <v>28.76390698751919</v>
+        <v>28.58315721020972</v>
       </c>
       <c r="M51" s="3" t="n">
-        <v>-2000</v>
+        <v>0</v>
       </c>
       <c r="N51" t="n">
         <v>0.3241496339540259</v>
@@ -10448,7 +10448,7 @@
         <v>60.12432359912347</v>
       </c>
       <c r="Q51" t="n">
-        <v>25.3</v>
+        <v>25.2</v>
       </c>
       <c r="R51" t="n">
         <v>3</v>
@@ -10497,13 +10497,13 @@
         <v>614999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>863325</v>
+        <v>861140</v>
       </c>
       <c r="L52" t="n">
-        <v>28.76390698751919</v>
+        <v>28.58315721020972</v>
       </c>
       <c r="M52" s="3" t="n">
-        <v>-10000</v>
+        <v>0</v>
       </c>
       <c r="N52" t="n">
         <v>0.3241496339540259</v>
@@ -10512,7 +10512,7 @@
         <v>60.12432359912347</v>
       </c>
       <c r="Q52" t="n">
-        <v>25.3</v>
+        <v>25.2</v>
       </c>
       <c r="R52" t="n">
         <v>3</v>
@@ -10561,10 +10561,10 @@
         <v>614999</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>863325</v>
+        <v>861140</v>
       </c>
       <c r="L53" t="n">
-        <v>28.76390698751919</v>
+        <v>28.58315721020972</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -10576,7 +10576,7 @@
         <v>60.12432359912347</v>
       </c>
       <c r="Q53" t="n">
-        <v>25.2</v>
+        <v>25.1</v>
       </c>
       <c r="R53" t="n">
         <v>3</v>
@@ -10625,10 +10625,10 @@
         <v>650000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>820137</v>
+        <v>818062</v>
       </c>
       <c r="L54" t="n">
-        <v>20.74494870978873</v>
+        <v>20.54391965401156</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -10689,10 +10689,10 @@
         <v>672000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>863325</v>
+        <v>861140</v>
       </c>
       <c r="L55" t="n">
-        <v>22.16141082442881</v>
+        <v>21.96390830759226</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -10704,7 +10704,7 @@
         <v>66.19519094766619</v>
       </c>
       <c r="Q55" t="n">
-        <v>23.7</v>
+        <v>23.6</v>
       </c>
       <c r="R55" t="n">
         <v>3</v>
@@ -10753,10 +10753,10 @@
         <v>700000</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>906513</v>
+        <v>904219</v>
       </c>
       <c r="L56" t="n">
-        <v>22.78103016724526</v>
+        <v>22.58512594847045</v>
       </c>
       <c r="M56" s="3" t="n">
         <v>0</v>
@@ -10768,7 +10768,7 @@
         <v>58.27439886845826</v>
       </c>
       <c r="Q56" t="n">
-        <v>22.3</v>
+        <v>22.2</v>
       </c>
       <c r="R56" t="n">
         <v>3</v>
@@ -10817,10 +10817,10 @@
         <v>715000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>949701</v>
+        <v>947298</v>
       </c>
       <c r="L57" t="n">
-        <v>24.71314655875902</v>
+        <v>24.52216725887735</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -10832,7 +10832,7 @@
         <v>65.83833956938916</v>
       </c>
       <c r="Q57" t="n">
-        <v>24.7</v>
+        <v>24.6</v>
       </c>
       <c r="R57" t="n">
         <v>3</v>
@@ -10881,10 +10881,10 @@
         <v>734999</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>992889</v>
+        <v>990376</v>
       </c>
       <c r="L58" t="n">
-        <v>25.97369897339984</v>
+        <v>25.78586314692601</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -10896,7 +10896,7 @@
         <v>78.07662153970499</v>
       </c>
       <c r="Q58" t="n">
-        <v>28.9</v>
+        <v>28.8</v>
       </c>
       <c r="R58" t="n">
         <v>3</v>
@@ -10945,10 +10945,10 @@
         <v>752000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>992889</v>
+        <v>990376</v>
       </c>
       <c r="L59" t="n">
-        <v>24.26142297880226</v>
+        <v>24.06924238874932</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -11009,10 +11009,10 @@
         <v>810000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1079264</v>
+        <v>1076533</v>
       </c>
       <c r="L60" t="n">
-        <v>24.94885403386011</v>
+        <v>24.75846072530986</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -11024,7 +11024,7 @@
         <v>70.98477153036431</v>
       </c>
       <c r="Q60" t="n">
-        <v>25.9</v>
+        <v>25.8</v>
       </c>
       <c r="R60" t="n">
         <v>3</v>
@@ -11073,10 +11073,10 @@
         <v>815000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1079264</v>
+        <v>1076533</v>
       </c>
       <c r="L61" t="n">
-        <v>24.48557535505678</v>
+        <v>24.2940067791698</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -11088,7 +11088,7 @@
         <v>83.38048090523338</v>
       </c>
       <c r="Q61" t="n">
-        <v>28.4</v>
+        <v>28.3</v>
       </c>
       <c r="R61" t="n">
         <v>3</v>
@@ -11137,10 +11137,10 @@
         <v>875000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1165640</v>
+        <v>1162690</v>
       </c>
       <c r="L62" t="n">
-        <v>24.93394186884458</v>
+        <v>24.74348278560923</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -11152,7 +11152,7 @@
         <v>80.43468538974106</v>
       </c>
       <c r="Q62" t="n">
-        <v>27.9</v>
+        <v>27.8</v>
       </c>
       <c r="R62" t="n">
         <v>3</v>
@@ -11201,10 +11201,10 @@
         <v>992000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1338391</v>
+        <v>1335005</v>
       </c>
       <c r="L63" t="n">
-        <v>25.881151322745</v>
+        <v>25.69316219789439</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -11265,10 +11265,10 @@
         <v>1050000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1424767</v>
+        <v>1421162</v>
       </c>
       <c r="L64" t="n">
-        <v>26.30373948863218</v>
+        <v>26.11679738129784</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -11280,7 +11280,7 @@
         <v>94.27799922849427</v>
       </c>
       <c r="Q64" t="n">
-        <v>31.5</v>
+        <v>31.4</v>
       </c>
       <c r="R64" t="n">
         <v>3</v>
@@ -11329,10 +11329,10 @@
         <v>1050000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1424767</v>
+        <v>1421162</v>
       </c>
       <c r="L65" t="n">
-        <v>26.30373948863218</v>
+        <v>26.11679738129784</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -11344,7 +11344,7 @@
         <v>86.95645692649404</v>
       </c>
       <c r="Q65" t="n">
-        <v>29.9</v>
+        <v>29.8</v>
       </c>
       <c r="R65" t="n">
         <v>3</v>
@@ -11393,10 +11393,10 @@
         <v>1100000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1511143</v>
+        <v>1507319</v>
       </c>
       <c r="L66" t="n">
-        <v>27.20741849050686</v>
+        <v>27.02274700975706</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -11408,7 +11408,7 @@
         <v>94.40991011135459</v>
       </c>
       <c r="Q66" t="n">
-        <v>31.9</v>
+        <v>31.8</v>
       </c>
       <c r="R66" t="n">
         <v>3</v>
@@ -11457,10 +11457,10 @@
         <v>1105000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1511143</v>
+        <v>1507319</v>
       </c>
       <c r="L67" t="n">
-        <v>26.87654312000916</v>
+        <v>26.69103222343777</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -11521,10 +11521,10 @@
         <v>1155000</v>
       </c>
       <c r="K68" s="3" t="n">
-        <v>1597518</v>
+        <v>1593476</v>
       </c>
       <c r="L68" t="n">
-        <v>27.70034516043012</v>
+        <v>27.51695036511375</v>
       </c>
       <c r="M68" s="3" t="n">
         <v>0</v>
@@ -11536,7 +11536,7 @@
         <v>100</v>
       </c>
       <c r="Q68" t="n">
-        <v>33.3</v>
+        <v>33.2</v>
       </c>
       <c r="R68" t="n">
         <v>3</v>
@@ -11792,7 +11792,7 @@
         <v>315000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>301883</v>
+        <v>301119</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -11853,10 +11853,10 @@
         <v>380000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>388259</v>
+        <v>387276</v>
       </c>
       <c r="L3" t="n">
-        <v>2.12718829441172</v>
+        <v>1.878763465848645</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -11868,7 +11868,7 @@
         <v>100</v>
       </c>
       <c r="Q3" t="n">
-        <v>22.3</v>
+        <v>22.2</v>
       </c>
       <c r="R3" t="n">
         <v>3</v>
@@ -11917,7 +11917,7 @@
         <v>415000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>388259</v>
+        <v>387276</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -11978,10 +11978,10 @@
         <v>495000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>474634</v>
+        <v>473433</v>
       </c>
       <c r="L5" t="n">
-        <v>7.297201633258468</v>
+        <v>7.062034120984384</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -11993,7 +11993,7 @@
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>4.1</v>
+        <v>4</v>
       </c>
       <c r="R5" t="n">
         <v>4</v>
@@ -12042,10 +12042,10 @@
         <v>500000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>517822</v>
+        <v>516512</v>
       </c>
       <c r="L6" t="n">
-        <v>9.235219824572923</v>
+        <v>9.005018276438882</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -12057,7 +12057,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>4.2</v>
+        <v>4.1</v>
       </c>
       <c r="R6" t="n">
         <v>4</v>
@@ -12106,10 +12106,10 @@
         <v>550000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>561010</v>
+        <v>559591</v>
       </c>
       <c r="L7" t="n">
-        <v>7.310030124240209</v>
+        <v>7.07498869710199</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -12121,7 +12121,7 @@
         <v>25.45360054666915</v>
       </c>
       <c r="Q7" t="n">
-        <v>8.199999999999999</v>
+        <v>8.1</v>
       </c>
       <c r="R7" t="n">
         <v>4</v>
@@ -12170,7 +12170,7 @@
         <v>530000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>474634</v>
+        <v>473433</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -12234,10 +12234,10 @@
         <v>600000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>604198</v>
+        <v>602669</v>
       </c>
       <c r="L9" t="n">
-        <v>8.970238233161977</v>
+        <v>8.739291385486894</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -12249,7 +12249,7 @@
         <v>20.65076182537716</v>
       </c>
       <c r="Q9" t="n">
-        <v>8.300000000000001</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="R9" t="n">
         <v>4</v>
@@ -12298,10 +12298,10 @@
         <v>646000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>733762</v>
+        <v>731905</v>
       </c>
       <c r="L10" t="n">
-        <v>17.54833311073618</v>
+        <v>17.33913554354732</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -12313,7 +12313,7 @@
         <v>100</v>
       </c>
       <c r="Q10" t="n">
-        <v>26.1</v>
+        <v>26</v>
       </c>
       <c r="R10" t="n">
         <v>4</v>
@@ -12362,7 +12362,7 @@
         <v>615000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>561010</v>
+        <v>559591</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -12426,7 +12426,7 @@
         <v>700000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>647386</v>
+        <v>645748</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -12490,7 +12490,7 @@
         <v>745000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>690574</v>
+        <v>688826</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -12554,7 +12554,7 @@
         <v>930000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>863325</v>
+        <v>861140</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -12625,7 +12625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12674,438 +12674,30 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 MGE44 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Silver</t>
+          <t>Apple MacBook Pro 16Inch MX2X3 14Core CPU 20Core GPU M4 Pro 24GB 512GB Space Black</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>870000</v>
+        <v>707999</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>840000</v>
+        <v>739999</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-30000</v>
+        <v>32000</v>
       </c>
       <c r="F2" t="n">
-        <v>-3.45</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDVC4 M5 10C CPU 10C GPU 24GB 1TB Silver</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>624999</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>614999</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>-10000</v>
-      </c>
-      <c r="F3" t="n">
-        <v>-1.6</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDHE4 M5 10C CPU 8C GPU 16GB 512GB Midnight</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>441999</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>433999</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>-8000</v>
-      </c>
-      <c r="F4" t="n">
-        <v>-1.81</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 MGDN4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Silver</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>735000</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>729999</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>-5001</v>
-      </c>
-      <c r="F5" t="n">
-        <v>-0.68</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDV94 M5 10C CPU 10C GPU 16GB 512GB Silver</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>495000</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>489999</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>-5001</v>
-      </c>
-      <c r="F6" t="n">
-        <v>-1.01</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Macbook Pro 16 MGE64 M5 Pro 18 Core CPU 20 Core GPU 48GB 1TB Silver</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>1085000</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>1080000</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>-5000</v>
-      </c>
-      <c r="F7" t="n">
-        <v>-0.46</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDVK4 M5 10C CPU 10C GPU 16GB 1TB Midnight</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>564999</v>
-      </c>
-      <c r="D8" s="3" t="n">
-        <v>559999</v>
-      </c>
-      <c r="E8" s="3" t="n">
-        <v>-5000</v>
-      </c>
-      <c r="F8" t="n">
-        <v>-0.88</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDVA4 M5 10C CPU 10C GPU 16GB 1TB Silver</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>564999</v>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>559999</v>
-      </c>
-      <c r="E9" s="3" t="n">
-        <v>-5000</v>
-      </c>
-      <c r="F9" t="n">
-        <v>-0.88</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDVE4 M5 10C CPU 10C GPU 16GB 1TB Starlight</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>564999</v>
-      </c>
-      <c r="D10" s="3" t="n">
-        <v>559999</v>
-      </c>
-      <c r="E10" s="3" t="n">
-        <v>-5000</v>
-      </c>
-      <c r="F10" t="n">
-        <v>-0.88</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDVT4 M5 10C CPU 10C GPU 16GB 1TB Sky Blue</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="n">
-        <v>564999</v>
-      </c>
-      <c r="D11" s="3" t="n">
-        <v>559999</v>
-      </c>
-      <c r="E11" s="3" t="n">
-        <v>-5000</v>
-      </c>
-      <c r="F11" t="n">
-        <v>-0.88</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDH74 M5 10C CPU 8C GPU 16GB 512GB Silver</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="n">
-        <v>447999</v>
-      </c>
-      <c r="D12" s="3" t="n">
-        <v>443000</v>
-      </c>
-      <c r="E12" s="3" t="n">
-        <v>-4999</v>
-      </c>
-      <c r="F12" t="n">
-        <v>-1.12</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 MGDR4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Space Black</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="n">
-        <v>728000</v>
-      </c>
-      <c r="D13" s="3" t="n">
-        <v>724999</v>
-      </c>
-      <c r="E13" s="3" t="n">
-        <v>-3001</v>
-      </c>
-      <c r="F13" t="n">
-        <v>-0.41</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Macbook Pro 16 MGEA4 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Space Black</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="n">
-        <v>832999</v>
-      </c>
-      <c r="D14" s="3" t="n">
-        <v>829999</v>
-      </c>
-      <c r="E14" s="3" t="n">
-        <v>-3000</v>
-      </c>
-      <c r="F14" t="n">
-        <v>-0.36</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDVU4 M5 10C CPU 10C GPU 24GB 1TB Sky Blue</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="n">
-        <v>616999</v>
-      </c>
-      <c r="D15" s="3" t="n">
-        <v>614999</v>
-      </c>
-      <c r="E15" s="3" t="n">
-        <v>-2000</v>
-      </c>
-      <c r="F15" t="n">
-        <v>-0.32</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDVF4 M5 10C CPU 10C GPU 24GB 1TB Starlight</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="n">
-        <v>616999</v>
-      </c>
-      <c r="D16" s="3" t="n">
-        <v>614999</v>
-      </c>
-      <c r="E16" s="3" t="n">
-        <v>-2000</v>
-      </c>
-      <c r="F16" t="n">
-        <v>-0.32</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 M5 MDE34 10 Core CPU 10 Core GPU 24GB 1TB Space Black</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="n">
-        <v>645000</v>
-      </c>
-      <c r="D17" s="3" t="n">
-        <v>643999</v>
-      </c>
-      <c r="E17" s="3" t="n">
-        <v>-1001</v>
-      </c>
-      <c r="F17" t="n">
-        <v>-0.16</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDHH4 M5 10C CPU 8C GPU 16GB 512GB Sky Blue</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="n">
-        <v>434999</v>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>433999</v>
-      </c>
-      <c r="E18" s="3" t="n">
-        <v>-1000</v>
-      </c>
-      <c r="F18" t="n">
-        <v>-0.23</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDHA4 M5 10C CPU 8C GPU 16GB 512GB Starlight</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="n">
-        <v>430000</v>
-      </c>
-      <c r="D19" s="3" t="n">
-        <v>433999</v>
-      </c>
-      <c r="E19" s="3" t="n">
-        <v>3999</v>
-      </c>
-      <c r="F19" t="n">
-        <v>0.93</v>
+        <v>4.52</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F19"/>
-  <conditionalFormatting sqref="E2:E19">
+  <autoFilter ref="A1:F2"/>
+  <conditionalFormatting sqref="E2">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
chore: price data 2026-09-23
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MacBook Pro'!$A$1:$S$92</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MacBook Air'!$A$1:$S$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20260922T083651699127+0000</t>
+          <t>20260923T083904842383+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-22T08:36:51.699127+00:00</t>
+          <t>2026-09-23T08:39:04.842383+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>277.425913</v>
+        <v>277.129099</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -729,7 +729,7 @@
         <v>810000</v>
       </c>
       <c r="D22" t="n">
-        <v>50.6</v>
+        <v>50.5</v>
       </c>
       <c r="E22" t="n">
         <v>4</v>
@@ -750,7 +750,7 @@
         <v>1123000</v>
       </c>
       <c r="D23" t="n">
-        <v>50.5</v>
+        <v>50.4</v>
       </c>
       <c r="E23" t="n">
         <v>4</v>
@@ -834,7 +834,7 @@
         <v>643999</v>
       </c>
       <c r="D27" t="n">
-        <v>44.3</v>
+        <v>44.4</v>
       </c>
       <c r="E27" t="n">
         <v>4</v>
@@ -852,10 +852,10 @@
         </is>
       </c>
       <c r="C28" s="3" t="n">
-        <v>724999</v>
+        <v>720000</v>
       </c>
       <c r="D28" t="n">
-        <v>43.8</v>
+        <v>44.4</v>
       </c>
       <c r="E28" t="n">
         <v>3</v>
@@ -906,22 +906,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHG4 M5 10C CPU 10C GPU 24GB 1TB Midnight</t>
+          <t>Macbook Pro 14 MGDN4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Silver</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>macbook_air</t>
+          <t>macbook_pro</t>
         </is>
       </c>
       <c r="C31" s="3" t="n">
-        <v>549999</v>
+        <v>725000</v>
       </c>
       <c r="D31" t="n">
-        <v>42.6</v>
+        <v>43.1</v>
       </c>
       <c r="E31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33">
@@ -1147,10 +1147,10 @@
         <v>470000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>687586</v>
+        <v>686851</v>
       </c>
       <c r="L2" t="n">
-        <v>35.28082305340714</v>
+        <v>35.21156699196769</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1214,10 +1214,10 @@
         <v>465000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>687586</v>
+        <v>686851</v>
       </c>
       <c r="L3" t="n">
-        <v>33.39015046845049</v>
+        <v>33.31887119622742</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -1232,7 +1232,7 @@
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>10.2</v>
+        <v>10.1</v>
       </c>
       <c r="R3" t="n">
         <v>5</v>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>773588</v>
+        <v>772761</v>
       </c>
       <c r="L4" t="n">
-        <v>35.36624146186342</v>
+        <v>35.29707115136504</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>773588</v>
+        <v>772761</v>
       </c>
       <c r="L5" t="n">
-        <v>32.78088594962693</v>
+        <v>32.70894882117499</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>859590</v>
+        <v>858671</v>
       </c>
       <c r="L6" t="n">
-        <v>38.11002919996743</v>
+        <v>38.04379092807373</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1488,14 +1488,17 @@
       <c r="N7" t="n">
         <v>0</v>
       </c>
+      <c r="O7" t="n">
+        <v>100</v>
+      </c>
       <c r="P7" t="n">
-        <v>0</v>
+        <v>1.999999999999989</v>
       </c>
       <c r="Q7" t="n">
-        <v>0</v>
+        <v>33.8</v>
       </c>
       <c r="R7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -1535,18 +1538,21 @@
         </is>
       </c>
       <c r="I8" s="3" t="n">
-        <v>555000</v>
+        <v>560000</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>555000</v>
+        <v>560000</v>
       </c>
       <c r="K8" s="3" t="n"/>
       <c r="M8" s="3" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="N8" t="n">
         <v>0</v>
       </c>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
       <c r="P8" t="n">
         <v>0</v>
       </c>
@@ -1554,7 +1560,7 @@
         <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1600,10 +1606,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>859590</v>
+        <v>858671</v>
       </c>
       <c r="L9" t="n">
-        <v>34.27098965786014</v>
+        <v>34.20064262098056</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1667,10 +1673,10 @@
         <v>582999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>859590</v>
+        <v>858671</v>
       </c>
       <c r="L10" t="n">
-        <v>32.17708442396957</v>
+        <v>32.10449636706026</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -1682,10 +1688,10 @@
         <v>100</v>
       </c>
       <c r="P10" t="n">
-        <v>48.06153061224489</v>
+        <v>49.10029999999999</v>
       </c>
       <c r="Q10" t="n">
-        <v>41</v>
+        <v>41.1</v>
       </c>
       <c r="R10" t="n">
         <v>4</v>
@@ -1734,10 +1740,10 @@
         <v>587999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>859590</v>
+        <v>858671</v>
       </c>
       <c r="L11" t="n">
-        <v>31.59541176607452</v>
+        <v>31.52220116901584</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -1749,10 +1755,10 @@
         <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>46.53091836734693</v>
+        <v>47.60029999999999</v>
       </c>
       <c r="Q11" t="n">
-        <v>18.3</v>
+        <v>18.4</v>
       </c>
       <c r="R11" t="n">
         <v>4</v>
@@ -1801,10 +1807,10 @@
         <v>643999</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>945592</v>
+        <v>944581</v>
       </c>
       <c r="L12" t="n">
-        <v>31.89462262794101</v>
+        <v>31.82172836421652</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -1816,10 +1822,10 @@
         <v>100</v>
       </c>
       <c r="P12" t="n">
-        <v>68.81657142857142</v>
+        <v>69.44023999999999</v>
       </c>
       <c r="Q12" t="n">
-        <v>44.3</v>
+        <v>44.4</v>
       </c>
       <c r="R12" t="n">
         <v>4</v>
@@ -1875,10 +1881,10 @@
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>67.3469387755102</v>
+        <v>68</v>
       </c>
       <c r="Q13" t="n">
-        <v>25.3</v>
+        <v>25.5</v>
       </c>
       <c r="R13" t="n">
         <v>2</v>
@@ -1927,10 +1933,10 @@
         <v>650000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>945592</v>
+        <v>944581</v>
       </c>
       <c r="L14" t="n">
-        <v>31.25999373937174</v>
+        <v>31.18642022229962</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -1942,10 +1948,10 @@
         <v>0</v>
       </c>
       <c r="P14" t="n">
-        <v>67.3469387755102</v>
+        <v>68</v>
       </c>
       <c r="Q14" t="n">
-        <v>21.6</v>
+        <v>21.7</v>
       </c>
       <c r="R14" t="n">
         <v>4</v>
@@ -1994,10 +2000,10 @@
         <v>650000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>859590</v>
+        <v>858671</v>
       </c>
       <c r="L15" t="n">
-        <v>24.38255447364441</v>
+        <v>24.30162425422543</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0</v>
@@ -2058,10 +2064,10 @@
         <v>650000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>859590</v>
+        <v>858671</v>
       </c>
       <c r="L16" t="n">
-        <v>24.38255447364441</v>
+        <v>24.30162425422543</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -2122,10 +2128,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1031594</v>
+        <v>1030491</v>
       </c>
       <c r="L17" t="n">
-        <v>32.14384728875895</v>
+        <v>32.07121653658304</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2189,13 +2195,13 @@
         <v>707999</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>1074595</v>
+        <v>1073446</v>
       </c>
       <c r="L18" t="n">
-        <v>34.11480604320698</v>
+        <v>34.04428355036024</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>-32000</v>
+        <v>0</v>
       </c>
       <c r="N18" t="n">
         <v>0</v>
@@ -2221,7 +2227,7 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 14Inch MX2F3 M4 Pro 14Core CPU 20Core GPU 24GB 1TB Silver</t>
+          <t>Macbook Pro 14 MGDR4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -2229,7 +2235,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>M4 Pro</t>
+          <t>M5 Pro</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -2239,14 +2245,14 @@
         <v>1024</v>
       </c>
       <c r="F19" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G19" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I19" s="3" t="n">
@@ -2255,29 +2261,24 @@
       <c r="J19" s="3" t="n">
         <v>720000</v>
       </c>
-      <c r="K19" s="3" t="n">
-        <v>1031594</v>
-      </c>
-      <c r="L19" t="n">
-        <v>30.20510006843778</v>
-      </c>
+      <c r="K19" s="3" t="n"/>
       <c r="M19" s="3" t="n">
-        <v>0</v>
+        <v>-4999</v>
       </c>
       <c r="N19" t="n">
-        <v>0</v>
+        <v>1.098901098901099</v>
       </c>
       <c r="O19" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="P19" t="n">
-        <v>82.22222222222221</v>
+        <v>42.39316239316239</v>
       </c>
       <c r="Q19" t="n">
-        <v>23.8</v>
+        <v>44.4</v>
       </c>
       <c r="R19" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S19" t="inlineStr">
         <is>
@@ -2288,7 +2289,7 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 MGDR4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Space Black</t>
+          <t>Apple MacBook Pro 14Inch MX2F3 M4 Pro 14Core CPU 20Core GPU 24GB 1TB Silver</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -2296,7 +2297,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>M5 Pro</t>
+          <t>M4 Pro</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -2306,40 +2307,45 @@
         <v>1024</v>
       </c>
       <c r="F20" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G20" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I20" s="3" t="n">
-        <v>724999</v>
+        <v>720000</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>724999</v>
-      </c>
-      <c r="K20" s="3" t="n"/>
+        <v>720000</v>
+      </c>
+      <c r="K20" s="3" t="n">
+        <v>1030491</v>
+      </c>
+      <c r="L20" t="n">
+        <v>30.13039415191399</v>
+      </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>0.4122252747252748</v>
+        <v>0</v>
       </c>
       <c r="O20" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="P20" t="n">
-        <v>41.02591452991454</v>
+        <v>82.22222222222221</v>
       </c>
       <c r="Q20" t="n">
-        <v>43.8</v>
+        <v>23.7</v>
       </c>
       <c r="R20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S20" t="inlineStr">
         <is>
@@ -2379,26 +2385,26 @@
         </is>
       </c>
       <c r="I21" s="3" t="n">
-        <v>729999</v>
+        <v>725000</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>729999</v>
+        <v>725000</v>
       </c>
       <c r="K21" s="3" t="n"/>
       <c r="M21" s="3" t="n">
-        <v>0</v>
+        <v>-4999</v>
       </c>
       <c r="N21" t="n">
-        <v>0.6804081632653061</v>
+        <v>1.360544217687075</v>
       </c>
       <c r="O21" t="n">
-        <v>96.66668888874074</v>
+        <v>96.7741935483871</v>
       </c>
       <c r="P21" t="n">
-        <v>39.65839316239318</v>
+        <v>41.02564102564102</v>
       </c>
       <c r="Q21" t="n">
-        <v>42.4</v>
+        <v>43.1</v>
       </c>
       <c r="R21" t="n">
         <v>3</v>
@@ -2447,10 +2453,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1074595</v>
+        <v>1073446</v>
       </c>
       <c r="L22" t="n">
-        <v>30.85767196013382</v>
+        <v>30.78366308132873</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2514,10 +2520,10 @@
         <v>745000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1031594</v>
+        <v>1030491</v>
       </c>
       <c r="L23" t="n">
-        <v>27.78166604303631</v>
+        <v>27.70436617107767</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -2529,7 +2535,7 @@
         <v>100</v>
       </c>
       <c r="P23" t="n">
-        <v>74.48979591836734</v>
+        <v>74.99999999999999</v>
       </c>
       <c r="Q23" t="n">
         <v>44.9</v>
@@ -2581,10 +2587,10 @@
         <v>755000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1031594</v>
+        <v>1030491</v>
       </c>
       <c r="L24" t="n">
-        <v>26.81229243287572</v>
+        <v>26.73395497874314</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -2596,10 +2602,10 @@
         <v>62.96296296296296</v>
       </c>
       <c r="P24" t="n">
-        <v>72.44897959183673</v>
+        <v>73</v>
       </c>
       <c r="Q24" t="n">
-        <v>35.6</v>
+        <v>35.7</v>
       </c>
       <c r="R24" t="n">
         <v>4</v>
@@ -2648,10 +2654,10 @@
         <v>772000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>1031594</v>
+        <v>1030491</v>
       </c>
       <c r="L25" t="n">
-        <v>25.16435729560273</v>
+        <v>25.08425595177445</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -2663,10 +2669,10 @@
         <v>0</v>
       </c>
       <c r="P25" t="n">
-        <v>68.97959183673468</v>
+        <v>69.59999999999998</v>
       </c>
       <c r="Q25" t="n">
-        <v>19.9</v>
+        <v>20</v>
       </c>
       <c r="R25" t="n">
         <v>4</v>
@@ -2777,10 +2783,10 @@
         <v>810000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>1246599</v>
+        <v>1245266</v>
       </c>
       <c r="L27" t="n">
-        <v>35.02321115290482</v>
+        <v>34.95365648785079</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -2795,7 +2801,7 @@
         <v>100</v>
       </c>
       <c r="Q27" t="n">
-        <v>50.6</v>
+        <v>50.5</v>
       </c>
       <c r="R27" t="n">
         <v>4</v>
@@ -2906,13 +2912,13 @@
         <v>825000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>1289600</v>
+        <v>1288221</v>
       </c>
       <c r="L29" t="n">
-        <v>36.02667493796526</v>
+        <v>35.95819350872249</v>
       </c>
       <c r="M29" s="3" t="n">
-        <v>-4999</v>
+        <v>0</v>
       </c>
       <c r="N29" t="n">
         <v>0.9602652584216788</v>
@@ -2973,22 +2979,22 @@
         <v>830000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1074595</v>
+        <v>1073446</v>
       </c>
       <c r="L30" t="n">
-        <v>22.76159855573495</v>
+        <v>22.67892376514515</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>-5000</v>
+        <v>0</v>
       </c>
       <c r="N30" t="n">
         <v>0.5988023952095809</v>
       </c>
       <c r="P30" t="n">
-        <v>57.14285714285713</v>
+        <v>57.99999999999999</v>
       </c>
       <c r="Q30" t="n">
-        <v>22.2</v>
+        <v>22.4</v>
       </c>
       <c r="R30" t="n">
         <v>3</v>
@@ -3037,10 +3043,10 @@
         <v>840000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1289600</v>
+        <v>1288221</v>
       </c>
       <c r="L31" t="n">
-        <v>34.86352357320099</v>
+        <v>34.7937970270629</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -3104,10 +3110,10 @@
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1375603</v>
+        <v>1374131</v>
       </c>
       <c r="L32" t="n">
-        <v>38.35437986105003</v>
+        <v>38.28834368775612</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3171,10 +3177,10 @@
         <v>930000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1375603</v>
+        <v>1374131</v>
       </c>
       <c r="L33" t="n">
-        <v>38.20898907606337</v>
+        <v>38.14279715689406</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3238,10 +3244,10 @@
         <v>860000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>1246599</v>
+        <v>1245266</v>
       </c>
       <c r="L34" t="n">
-        <v>31.01229826110882</v>
+        <v>30.93845009821195</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -3368,7 +3374,7 @@
       </c>
       <c r="K36" s="3" t="n"/>
       <c r="M36" s="3" t="n">
-        <v>-15000</v>
+        <v>0</v>
       </c>
       <c r="N36" t="n">
         <v>1.685393258426966</v>
@@ -3491,22 +3497,22 @@
         <v>880000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>1160597</v>
+        <v>1159356</v>
       </c>
       <c r="L38" t="n">
-        <v>24.17695375741967</v>
+        <v>24.09579111161714</v>
       </c>
       <c r="M38" s="3" t="n">
-        <v>-10000</v>
+        <v>0</v>
       </c>
       <c r="N38" t="n">
         <v>1.123595505617978</v>
       </c>
       <c r="P38" t="n">
-        <v>72.59475218658892</v>
+        <v>73.14285714285714</v>
       </c>
       <c r="Q38" t="n">
-        <v>26.3</v>
+        <v>26.4</v>
       </c>
       <c r="R38" t="n">
         <v>3</v>
@@ -3555,19 +3561,19 @@
         <v>940000</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>1246599</v>
+        <v>1245266</v>
       </c>
       <c r="L39" t="n">
-        <v>24.59483763423523</v>
+        <v>24.5141198747898</v>
       </c>
       <c r="M39" s="3" t="n">
-        <v>-20000</v>
+        <v>0</v>
       </c>
       <c r="N39" t="n">
         <v>2.083333333333333</v>
       </c>
       <c r="P39" t="n">
-        <v>82.65306122448979</v>
+        <v>83</v>
       </c>
       <c r="Q39" t="n">
         <v>29</v>
@@ -3619,10 +3625,10 @@
         <v>970000</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>1504606</v>
+        <v>1502996</v>
       </c>
       <c r="L40" t="n">
-        <v>35.53129523609503</v>
+        <v>35.46223675911313</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -3687,7 +3693,7 @@
       </c>
       <c r="K41" s="3" t="n"/>
       <c r="M41" s="3" t="n">
-        <v>-25000</v>
+        <v>0</v>
       </c>
       <c r="N41" t="n">
         <v>2.450980392156863</v>
@@ -3748,10 +3754,10 @@
         <v>1022000</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>1504606</v>
+        <v>1502996</v>
       </c>
       <c r="L42" t="n">
-        <v>32.07524096009188</v>
+        <v>32.0024803791893</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -3815,13 +3821,13 @@
         <v>1055000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1547607</v>
+        <v>1545951</v>
       </c>
       <c r="L43" t="n">
-        <v>31.83023855539552</v>
+        <v>31.75721610840188</v>
       </c>
       <c r="M43" s="3" t="n">
-        <v>-8000</v>
+        <v>0</v>
       </c>
       <c r="N43" t="n">
         <v>0.7525870178739417</v>
@@ -3879,13 +3885,13 @@
         <v>1055000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1547607</v>
+        <v>1545951</v>
       </c>
       <c r="L44" t="n">
-        <v>31.83023855539552</v>
+        <v>31.75721610840188</v>
       </c>
       <c r="M44" s="3" t="n">
-        <v>-25000</v>
+        <v>0</v>
       </c>
       <c r="N44" t="n">
         <v>2.764976958525346</v>
@@ -3944,7 +3950,7 @@
       </c>
       <c r="K45" s="3" t="n"/>
       <c r="M45" s="3" t="n">
-        <v>-35000</v>
+        <v>0</v>
       </c>
       <c r="N45" t="n">
         <v>3.19634703196347</v>
@@ -4005,10 +4011,10 @@
         <v>1123000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1719611</v>
+        <v>1717771</v>
       </c>
       <c r="L46" t="n">
-        <v>34.69453265883971</v>
+        <v>34.62458034278143</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -4023,7 +4029,7 @@
         <v>100</v>
       </c>
       <c r="Q46" t="n">
-        <v>50.5</v>
+        <v>50.4</v>
       </c>
       <c r="R46" t="n">
         <v>4</v>
@@ -4072,19 +4078,19 @@
         <v>1130000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1504606</v>
+        <v>1502996</v>
       </c>
       <c r="L47" t="n">
-        <v>24.89728207916225</v>
+        <v>24.81683251319365</v>
       </c>
       <c r="M47" s="3" t="n">
-        <v>-20000</v>
+        <v>0</v>
       </c>
       <c r="N47" t="n">
         <v>1.739130434782609</v>
       </c>
       <c r="P47" t="n">
-        <v>88.16326530612244</v>
+        <v>88.39999999999999</v>
       </c>
       <c r="Q47" t="n">
         <v>30.2</v>
@@ -4136,10 +4142,10 @@
         <v>1150000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1504606</v>
+        <v>1502996</v>
       </c>
       <c r="L48" t="n">
-        <v>23.56803043454565</v>
+        <v>23.48615698245371</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -4201,7 +4207,7 @@
       </c>
       <c r="K49" s="3" t="n"/>
       <c r="M49" s="3" t="n">
-        <v>-25000</v>
+        <v>0</v>
       </c>
       <c r="N49" t="n">
         <v>2.11864406779661</v>
@@ -4262,10 +4268,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1762612</v>
+        <v>1760726</v>
       </c>
       <c r="L50" t="n">
-        <v>34.47224913934547</v>
+        <v>34.40205915060038</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4326,10 +4332,10 @@
         <v>1155000</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>1762612</v>
+        <v>1760726</v>
       </c>
       <c r="L51" t="n">
-        <v>34.47224913934547</v>
+        <v>34.40205915060038</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -4390,13 +4396,13 @@
         <v>1185000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1590608</v>
+        <v>1588906</v>
       </c>
       <c r="L52" t="n">
-        <v>25.50018609236216</v>
+        <v>25.42038358468028</v>
       </c>
       <c r="M52" s="3" t="n">
-        <v>-30000</v>
+        <v>0</v>
       </c>
       <c r="N52" t="n">
         <v>2.469135802469136</v>
@@ -4405,7 +4411,7 @@
         <v>77.26495726495727</v>
       </c>
       <c r="Q52" t="n">
-        <v>28.4</v>
+        <v>28.3</v>
       </c>
       <c r="R52" t="n">
         <v>3</v>
@@ -4454,19 +4460,19 @@
         <v>1185000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1590608</v>
+        <v>1588906</v>
       </c>
       <c r="L53" t="n">
-        <v>25.50018609236216</v>
+        <v>25.42038358468028</v>
       </c>
       <c r="M53" s="3" t="n">
-        <v>-25000</v>
+        <v>0</v>
       </c>
       <c r="N53" t="n">
         <v>2.066115702479339</v>
       </c>
       <c r="P53" t="n">
-        <v>94.61966604823748</v>
+        <v>94.72727272727272</v>
       </c>
       <c r="Q53" t="n">
         <v>31.9</v>
@@ -4512,28 +4518,28 @@
         </is>
       </c>
       <c r="I54" s="3" t="n">
-        <v>1207000</v>
+        <v>1200000</v>
       </c>
       <c r="J54" s="3" t="n">
-        <v>1207000</v>
+        <v>1200000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1891615</v>
+        <v>1889591</v>
       </c>
       <c r="L54" t="n">
-        <v>36.19208982800411</v>
+        <v>36.49419371705305</v>
       </c>
       <c r="M54" s="3" t="n">
-        <v>0</v>
+        <v>-7000</v>
       </c>
       <c r="N54" t="n">
-        <v>0.08278145695364239</v>
+        <v>0.6622516556291391</v>
       </c>
       <c r="P54" t="n">
-        <v>9.265033407572403</v>
+        <v>11.02580898729203</v>
       </c>
       <c r="Q54" t="n">
-        <v>17.5</v>
+        <v>18.2</v>
       </c>
       <c r="R54" t="n">
         <v>3</v>
@@ -4576,28 +4582,28 @@
         </is>
       </c>
       <c r="I55" s="3" t="n">
-        <v>1207000</v>
+        <v>1200000</v>
       </c>
       <c r="J55" s="3" t="n">
-        <v>1207000</v>
+        <v>1200000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1891615</v>
+        <v>1889591</v>
       </c>
       <c r="L55" t="n">
-        <v>36.19208982800411</v>
+        <v>36.49419371705305</v>
       </c>
       <c r="M55" s="3" t="n">
-        <v>0</v>
+        <v>-7000</v>
       </c>
       <c r="N55" t="n">
-        <v>0.2479338842975207</v>
+        <v>0.8264462809917356</v>
       </c>
       <c r="P55" t="n">
-        <v>9.265033407572403</v>
+        <v>11.02580898729203</v>
       </c>
       <c r="Q55" t="n">
-        <v>17.6</v>
+        <v>18.3</v>
       </c>
       <c r="R55" t="n">
         <v>3</v>
@@ -4647,7 +4653,7 @@
       </c>
       <c r="K56" s="3" t="n"/>
       <c r="M56" s="3" t="n">
-        <v>-35000</v>
+        <v>0</v>
       </c>
       <c r="N56" t="n">
         <v>2.811244979919679</v>
@@ -4708,13 +4714,13 @@
         <v>1240000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1676610</v>
+        <v>1674816</v>
       </c>
       <c r="L57" t="n">
-        <v>26.04123797424565</v>
+        <v>25.96201612595056</v>
       </c>
       <c r="M57" s="3" t="n">
-        <v>-40000</v>
+        <v>0</v>
       </c>
       <c r="N57" t="n">
         <v>3.125</v>
@@ -4772,10 +4778,10 @@
         <v>1280000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>1719611</v>
+        <v>1717771</v>
       </c>
       <c r="L58" t="n">
-        <v>25.56456082218595</v>
+        <v>25.48482888580608</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -4839,10 +4845,10 @@
         <v>1310000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1719611</v>
+        <v>1717771</v>
       </c>
       <c r="L59" t="n">
-        <v>23.81998021645593</v>
+        <v>23.73837956281716</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -4904,7 +4910,7 @@
       </c>
       <c r="K60" s="3" t="n"/>
       <c r="M60" s="3" t="n">
-        <v>-50000</v>
+        <v>0</v>
       </c>
       <c r="N60" t="n">
         <v>3.623188405797102</v>
@@ -4962,13 +4968,13 @@
         <v>1335000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1805613</v>
+        <v>1803681</v>
       </c>
       <c r="L61" t="n">
-        <v>26.06389076729067</v>
+        <v>25.98469463280924</v>
       </c>
       <c r="M61" s="3" t="n">
-        <v>-35000</v>
+        <v>0</v>
       </c>
       <c r="N61" t="n">
         <v>2.554744525547445</v>
@@ -4977,7 +4983,7 @@
         <v>87.17948717948718</v>
       </c>
       <c r="Q61" t="n">
-        <v>30.8</v>
+        <v>30.7</v>
       </c>
       <c r="R61" t="n">
         <v>3</v>
@@ -5026,10 +5032,10 @@
         <v>1338000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1762612</v>
+        <v>1760726</v>
       </c>
       <c r="L62" t="n">
-        <v>24.08993017181319</v>
+        <v>24.00861917186434</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -5041,7 +5047,7 @@
         <v>60.93541202672606</v>
       </c>
       <c r="Q62" t="n">
-        <v>23.4</v>
+        <v>23.3</v>
       </c>
       <c r="R62" t="n">
         <v>3</v>
@@ -5091,7 +5097,7 @@
       </c>
       <c r="K63" s="3" t="n"/>
       <c r="M63" s="3" t="n">
-        <v>-45000</v>
+        <v>0</v>
       </c>
       <c r="N63" t="n">
         <v>3.02013422818792</v>
@@ -5146,28 +5152,28 @@
         </is>
       </c>
       <c r="I64" s="3" t="n">
-        <v>1460000</v>
+        <v>1450000</v>
       </c>
       <c r="J64" s="3" t="n">
-        <v>1460000</v>
+        <v>1450000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>2149621</v>
+        <v>2147321</v>
       </c>
       <c r="L64" t="n">
-        <v>32.08105056658825</v>
+        <v>32.47399899688961</v>
       </c>
       <c r="M64" s="3" t="n">
-        <v>0</v>
+        <v>-10000</v>
       </c>
       <c r="N64" t="n">
         <v>0</v>
       </c>
       <c r="P64" t="n">
-        <v>0.7126948775055885</v>
+        <v>2.850779510022292</v>
       </c>
       <c r="Q64" t="n">
-        <v>13.9</v>
+        <v>14.5</v>
       </c>
       <c r="R64" t="n">
         <v>3</v>
@@ -5210,28 +5216,28 @@
         </is>
       </c>
       <c r="I65" s="3" t="n">
-        <v>1460000</v>
+        <v>1450000</v>
       </c>
       <c r="J65" s="3" t="n">
-        <v>1460000</v>
+        <v>1450000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>2149621</v>
+        <v>2147321</v>
       </c>
       <c r="L65" t="n">
-        <v>32.08105056658825</v>
+        <v>32.47399899688961</v>
       </c>
       <c r="M65" s="3" t="n">
-        <v>0</v>
+        <v>-10000</v>
       </c>
       <c r="N65" t="n">
         <v>0</v>
       </c>
       <c r="P65" t="n">
-        <v>0.7126948775055885</v>
+        <v>2.850779510022292</v>
       </c>
       <c r="Q65" t="n">
-        <v>13.9</v>
+        <v>14.5</v>
       </c>
       <c r="R65" t="n">
         <v>3</v>
@@ -5280,10 +5286,10 @@
         <v>1471000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1934616</v>
+        <v>1932546</v>
       </c>
       <c r="L66" t="n">
-        <v>23.96423889805522</v>
+        <v>23.88279502790619</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -5344,10 +5350,10 @@
         <v>1471000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1934616</v>
+        <v>1932546</v>
       </c>
       <c r="L67" t="n">
-        <v>23.96423889805522</v>
+        <v>23.88279502790619</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -5359,7 +5365,7 @@
         <v>61.06499291354523</v>
       </c>
       <c r="Q67" t="n">
-        <v>23.4</v>
+        <v>23.3</v>
       </c>
       <c r="R67" t="n">
         <v>3</v>
@@ -5408,13 +5414,13 @@
         <v>1480000</v>
       </c>
       <c r="K68" s="3" t="n">
-        <v>2020618</v>
+        <v>2018456</v>
       </c>
       <c r="L68" t="n">
-        <v>26.75508186109398</v>
+        <v>26.67662807611362</v>
       </c>
       <c r="M68" s="3" t="n">
-        <v>-55000</v>
+        <v>0</v>
       </c>
       <c r="N68" t="n">
         <v>3.583061889250815</v>
@@ -5473,7 +5479,7 @@
       </c>
       <c r="K69" s="3" t="n"/>
       <c r="M69" s="3" t="n">
-        <v>-45000</v>
+        <v>0</v>
       </c>
       <c r="N69" t="n">
         <v>2.884615384615385</v>
@@ -5534,13 +5540,13 @@
         <v>1605000</v>
       </c>
       <c r="K70" s="3" t="n">
-        <v>2192622</v>
+        <v>2190276</v>
       </c>
       <c r="L70" t="n">
-        <v>26.7999682571825</v>
+        <v>26.7215638577056</v>
       </c>
       <c r="M70" s="3" t="n">
-        <v>-45000</v>
+        <v>0</v>
       </c>
       <c r="N70" t="n">
         <v>2.727272727272727</v>
@@ -5549,7 +5555,7 @@
         <v>36.44392794886694</v>
       </c>
       <c r="Q70" t="n">
-        <v>20.3</v>
+        <v>20.2</v>
       </c>
       <c r="R70" t="n">
         <v>3</v>
@@ -5598,13 +5604,13 @@
         <v>1610000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2192622</v>
+        <v>2190276</v>
       </c>
       <c r="L71" t="n">
-        <v>26.57193077511765</v>
+        <v>26.49328212517509</v>
       </c>
       <c r="M71" s="3" t="n">
-        <v>-50000</v>
+        <v>0</v>
       </c>
       <c r="N71" t="n">
         <v>3.012048192771084</v>
@@ -5613,7 +5619,7 @@
         <v>25.72147975982957</v>
       </c>
       <c r="Q71" t="n">
-        <v>18</v>
+        <v>17.9</v>
       </c>
       <c r="R71" t="n">
         <v>3</v>
@@ -5662,13 +5668,13 @@
         <v>1630000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2235623</v>
+        <v>2233231</v>
       </c>
       <c r="L72" t="n">
-        <v>27.08967477969228</v>
+        <v>27.011580978412</v>
       </c>
       <c r="M72" s="3" t="n">
-        <v>-50000</v>
+        <v>0</v>
       </c>
       <c r="N72" t="n">
         <v>2.976190476190476</v>
@@ -5726,10 +5732,10 @@
         <v>1661000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2192622</v>
+        <v>2190276</v>
       </c>
       <c r="L73" t="n">
-        <v>24.24594845805616</v>
+        <v>24.16480845336387</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
@@ -5790,10 +5796,10 @@
         <v>1711000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2321625</v>
+        <v>2319141</v>
       </c>
       <c r="L74" t="n">
-        <v>26.30162063210036</v>
+        <v>26.2226833124851</v>
       </c>
       <c r="M74" s="3" t="n">
         <v>0</v>
@@ -5854,10 +5860,10 @@
         <v>1756000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2321625</v>
+        <v>2319141</v>
       </c>
       <c r="L75" t="n">
-        <v>24.36332310342971</v>
+        <v>24.28230970001393</v>
       </c>
       <c r="M75" s="3" t="n">
         <v>0</v>
@@ -5918,13 +5924,13 @@
         <v>1780000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2450628</v>
+        <v>2448006</v>
       </c>
       <c r="L76" t="n">
-        <v>27.36555691031034</v>
+        <v>27.28775991562112</v>
       </c>
       <c r="M76" s="3" t="n">
-        <v>-60000</v>
+        <v>0</v>
       </c>
       <c r="N76" t="n">
         <v>3.260869565217391</v>
@@ -5982,10 +5988,10 @@
         <v>1790000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2364626</v>
+        <v>2362096</v>
       </c>
       <c r="L77" t="n">
-        <v>24.30092538946963</v>
+        <v>24.21984542541878</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
@@ -6046,13 +6052,13 @@
         <v>1910000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2622632</v>
+        <v>2619826</v>
       </c>
       <c r="L78" t="n">
-        <v>27.17239780495319</v>
+        <v>27.09439481858719</v>
       </c>
       <c r="M78" s="3" t="n">
-        <v>-50000</v>
+        <v>0</v>
       </c>
       <c r="N78" t="n">
         <v>2.551020408163265</v>
@@ -6061,7 +6067,7 @@
         <v>53.22486926205694</v>
       </c>
       <c r="Q78" t="n">
-        <v>24</v>
+        <v>23.9</v>
       </c>
       <c r="R78" t="n">
         <v>3</v>
@@ -6110,10 +6116,10 @@
         <v>1945000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2579631</v>
+        <v>2576871</v>
       </c>
       <c r="L79" t="n">
-        <v>24.60161937889566</v>
+        <v>24.52086270519557</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
@@ -6174,10 +6180,10 @@
         <v>2078000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2751635</v>
+        <v>2748691</v>
       </c>
       <c r="L80" t="n">
-        <v>24.48126295820485</v>
+        <v>24.40037821639464</v>
       </c>
       <c r="M80" s="3" t="n">
         <v>0</v>
@@ -6238,13 +6244,13 @@
         <v>2110000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2880638</v>
+        <v>2877556</v>
       </c>
       <c r="L81" t="n">
-        <v>26.75233750301149</v>
+        <v>26.6738857558289</v>
       </c>
       <c r="M81" s="3" t="n">
-        <v>-60000</v>
+        <v>0</v>
       </c>
       <c r="N81" t="n">
         <v>2.764976958525346</v>
@@ -6302,13 +6308,13 @@
         <v>2215000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>3052642</v>
+        <v>3049376</v>
       </c>
       <c r="L82" t="n">
-        <v>27.43990287757294</v>
+        <v>27.36218819850356</v>
       </c>
       <c r="M82" s="3" t="n">
-        <v>-55000</v>
+        <v>0</v>
       </c>
       <c r="N82" t="n">
         <v>2.422907488986784</v>
@@ -6366,10 +6372,10 @@
         <v>2268000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3009641</v>
+        <v>3006421</v>
       </c>
       <c r="L83" t="n">
-        <v>24.64217493049836</v>
+        <v>24.56146361404474</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
@@ -6430,10 +6436,10 @@
         <v>2381000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3181645</v>
+        <v>3178241</v>
       </c>
       <c r="L84" t="n">
-        <v>25.16449823911844</v>
+        <v>25.08434697054125</v>
       </c>
       <c r="M84" s="3" t="n">
         <v>0</v>
@@ -6494,13 +6500,13 @@
         <v>2395000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3310648</v>
+        <v>3307106</v>
       </c>
       <c r="L85" t="n">
-        <v>27.65766701866221</v>
+        <v>27.58018642281197</v>
       </c>
       <c r="M85" s="3" t="n">
-        <v>-85000</v>
+        <v>0</v>
       </c>
       <c r="N85" t="n">
         <v>3.42741935483871</v>
@@ -6509,7 +6515,7 @@
         <v>72.76953145634144</v>
       </c>
       <c r="Q85" t="n">
-        <v>28.7</v>
+        <v>28.6</v>
       </c>
       <c r="R85" t="n">
         <v>3</v>
@@ -6558,13 +6564,13 @@
         <v>2410000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3310648</v>
+        <v>3307106</v>
       </c>
       <c r="L86" t="n">
-        <v>27.20458351355988</v>
+        <v>27.12661765301747</v>
       </c>
       <c r="M86" s="3" t="n">
-        <v>-60000</v>
+        <v>0</v>
       </c>
       <c r="N86" t="n">
         <v>2.42914979757085</v>
@@ -6622,13 +6628,13 @@
         <v>2530000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3482652</v>
+        <v>3478926</v>
       </c>
       <c r="L87" t="n">
-        <v>27.3542116754703</v>
+        <v>27.27640656915382</v>
       </c>
       <c r="M87" s="3" t="n">
-        <v>-50000</v>
+        <v>0</v>
       </c>
       <c r="N87" t="n">
         <v>1.937984496124031</v>
@@ -6637,7 +6643,7 @@
         <v>79.17877203176447</v>
       </c>
       <c r="Q87" t="n">
-        <v>29.4</v>
+        <v>29.3</v>
       </c>
       <c r="R87" t="n">
         <v>3</v>
@@ -6686,10 +6692,10 @@
         <v>2571000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3439651</v>
+        <v>3435971</v>
       </c>
       <c r="L88" t="n">
-        <v>25.25404466906672</v>
+        <v>25.17399011807725</v>
       </c>
       <c r="M88" s="3" t="n">
         <v>0</v>
@@ -6750,10 +6756,10 @@
         <v>2581000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3439651</v>
+        <v>3435971</v>
       </c>
       <c r="L89" t="n">
-        <v>24.96331749936258</v>
+        <v>24.88295157322341</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
@@ -6814,10 +6820,10 @@
         <v>2664000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3611655</v>
+        <v>3607791</v>
       </c>
       <c r="L90" t="n">
-        <v>26.23880187891701</v>
+        <v>26.15980249410235</v>
       </c>
       <c r="M90" s="3" t="n">
         <v>0</v>
@@ -6878,13 +6884,13 @@
         <v>3015000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>4170669</v>
+        <v>4166206</v>
       </c>
       <c r="L91" t="n">
-        <v>27.70943942086989</v>
+        <v>27.63199899380875</v>
       </c>
       <c r="M91" s="3" t="n">
-        <v>-75000</v>
+        <v>0</v>
       </c>
       <c r="N91" t="n">
         <v>2.427184466019417</v>
@@ -6893,7 +6899,7 @@
         <v>100</v>
       </c>
       <c r="Q91" t="n">
-        <v>34.2</v>
+        <v>34.1</v>
       </c>
       <c r="R91" t="n">
         <v>3</v>
@@ -6942,10 +6948,10 @@
         <v>3186000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4299672</v>
+        <v>4295071</v>
       </c>
       <c r="L92" t="n">
-        <v>25.90132456615295</v>
+        <v>25.82194799573744</v>
       </c>
       <c r="M92" s="3" t="n">
         <v>0</v>
@@ -7240,10 +7246,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>429580</v>
+        <v>429121</v>
       </c>
       <c r="L2" t="n">
-        <v>27.83672424228316</v>
+        <v>27.75953635454802</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7258,7 +7264,7 @@
         <v>29.71702857142851</v>
       </c>
       <c r="Q2" t="n">
-        <v>36.5</v>
+        <v>36.4</v>
       </c>
       <c r="R2" t="n">
         <v>4</v>
@@ -7307,10 +7313,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>429580</v>
+        <v>429121</v>
       </c>
       <c r="L3" t="n">
-        <v>27.83672424228316</v>
+        <v>27.75953635454802</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7325,7 +7331,7 @@
         <v>29.71702857142851</v>
       </c>
       <c r="Q3" t="n">
-        <v>36.5</v>
+        <v>36.4</v>
       </c>
       <c r="R3" t="n">
         <v>4</v>
@@ -7374,10 +7380,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>429580</v>
+        <v>429121</v>
       </c>
       <c r="L4" t="n">
-        <v>27.83649145677173</v>
+        <v>27.7593033200426</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7441,10 +7447,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>429580</v>
+        <v>429121</v>
       </c>
       <c r="L5" t="n">
-        <v>27.83649145677173</v>
+        <v>27.7593033200426</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7508,10 +7514,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>515582</v>
+        <v>515031</v>
       </c>
       <c r="L6" t="n">
-        <v>25.52106163520061</v>
+        <v>25.4413811984133</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7572,10 +7578,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>515582</v>
+        <v>515031</v>
       </c>
       <c r="L7" t="n">
-        <v>25.52106163520061</v>
+        <v>25.4413811984133</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7636,10 +7642,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>515582</v>
+        <v>515031</v>
       </c>
       <c r="L8" t="n">
-        <v>25.52106163520061</v>
+        <v>25.4413811984133</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7700,10 +7706,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>515582</v>
+        <v>515031</v>
       </c>
       <c r="L9" t="n">
-        <v>25.52106163520061</v>
+        <v>25.4413811984133</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7764,10 +7770,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>515582</v>
+        <v>515031</v>
       </c>
       <c r="L10" t="n">
-        <v>25.32710606654228</v>
+        <v>25.2472181286175</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7779,7 +7785,7 @@
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>10.9</v>
+        <v>10.8</v>
       </c>
       <c r="R10" t="n">
         <v>3</v>
@@ -7828,10 +7834,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>515582</v>
+        <v>515031</v>
       </c>
       <c r="L11" t="n">
-        <v>25.32710606654228</v>
+        <v>25.2472181286175</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7843,7 +7849,7 @@
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>10.9</v>
+        <v>10.8</v>
       </c>
       <c r="R11" t="n">
         <v>3</v>
@@ -7892,10 +7898,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>515582</v>
+        <v>515031</v>
       </c>
       <c r="L12" t="n">
-        <v>25.32710606654228</v>
+        <v>25.2472181286175</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -7907,7 +7913,7 @@
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>10.9</v>
+        <v>10.8</v>
       </c>
       <c r="R12" t="n">
         <v>3</v>
@@ -7956,10 +7962,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>515582</v>
+        <v>515031</v>
       </c>
       <c r="L13" t="n">
-        <v>25.32710606654228</v>
+        <v>25.2472181286175</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -7971,7 +7977,7 @@
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>10.9</v>
+        <v>10.8</v>
       </c>
       <c r="R13" t="n">
         <v>3</v>
@@ -8020,13 +8026,13 @@
         <v>425000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>558583</v>
+        <v>557986</v>
       </c>
       <c r="L14" t="n">
-        <v>23.91461967156179</v>
+        <v>23.83321445340923</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>-8999</v>
+        <v>0</v>
       </c>
       <c r="N14" t="n">
         <v>5.133716816332179</v>
@@ -8035,7 +8041,7 @@
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>12.1</v>
+        <v>12</v>
       </c>
       <c r="R14" t="n">
         <v>3</v>
@@ -8084,13 +8090,13 @@
         <v>425000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>558583</v>
+        <v>557986</v>
       </c>
       <c r="L15" t="n">
-        <v>23.91461967156179</v>
+        <v>23.83321445340923</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>-8999</v>
+        <v>0</v>
       </c>
       <c r="N15" t="n">
         <v>1.847348377247984</v>
@@ -8148,13 +8154,13 @@
         <v>425000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>558583</v>
+        <v>557986</v>
       </c>
       <c r="L16" t="n">
-        <v>23.91461967156179</v>
+        <v>23.83321445340923</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>-18000</v>
+        <v>0</v>
       </c>
       <c r="N16" t="n">
         <v>5.133716816332179</v>
@@ -8163,7 +8169,7 @@
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>12.1</v>
+        <v>12</v>
       </c>
       <c r="R16" t="n">
         <v>3</v>
@@ -8212,13 +8218,13 @@
         <v>425000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>558583</v>
+        <v>557986</v>
       </c>
       <c r="L17" t="n">
-        <v>23.91461967156179</v>
+        <v>23.83321445340923</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>-8999</v>
+        <v>0</v>
       </c>
       <c r="N17" t="n">
         <v>1.162790697674419</v>
@@ -8227,7 +8233,7 @@
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>10.7</v>
+        <v>10.6</v>
       </c>
       <c r="R17" t="n">
         <v>3</v>
@@ -8276,10 +8282,10 @@
         <v>454000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>601584</v>
+        <v>600941</v>
       </c>
       <c r="L18" t="n">
-        <v>24.53256735551478</v>
+        <v>24.4518180653342</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -8340,10 +8346,10 @@
         <v>454000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>601584</v>
+        <v>600941</v>
       </c>
       <c r="L19" t="n">
-        <v>24.53256735551478</v>
+        <v>24.4518180653342</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -8404,10 +8410,10 @@
         <v>454000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>601584</v>
+        <v>600941</v>
       </c>
       <c r="L20" t="n">
-        <v>24.53256735551478</v>
+        <v>24.4518180653342</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -8468,10 +8474,10 @@
         <v>454000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>601584</v>
+        <v>600941</v>
       </c>
       <c r="L21" t="n">
-        <v>24.53256735551478</v>
+        <v>24.4518180653342</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -8532,10 +8538,10 @@
         <v>455000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>601584</v>
+        <v>600941</v>
       </c>
       <c r="L22" t="n">
-        <v>24.36633953030666</v>
+        <v>24.28541237825344</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -8547,7 +8553,7 @@
         <v>100</v>
       </c>
       <c r="Q22" t="n">
-        <v>31.9</v>
+        <v>31.8</v>
       </c>
       <c r="R22" t="n">
         <v>3</v>
@@ -8596,10 +8602,10 @@
         <v>455000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>601584</v>
+        <v>600941</v>
       </c>
       <c r="L23" t="n">
-        <v>24.36633953030666</v>
+        <v>24.28541237825344</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -8611,7 +8617,7 @@
         <v>100</v>
       </c>
       <c r="Q23" t="n">
-        <v>31.9</v>
+        <v>31.8</v>
       </c>
       <c r="R23" t="n">
         <v>3</v>
@@ -8660,10 +8666,10 @@
         <v>455000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>601584</v>
+        <v>600941</v>
       </c>
       <c r="L24" t="n">
-        <v>24.36633953030666</v>
+        <v>24.28541237825344</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -8675,7 +8681,7 @@
         <v>100</v>
       </c>
       <c r="Q24" t="n">
-        <v>31.9</v>
+        <v>31.8</v>
       </c>
       <c r="R24" t="n">
         <v>3</v>
@@ -8724,10 +8730,10 @@
         <v>455000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>601584</v>
+        <v>600941</v>
       </c>
       <c r="L25" t="n">
-        <v>24.36633953030666</v>
+        <v>24.28541237825344</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -8739,7 +8745,7 @@
         <v>100</v>
       </c>
       <c r="Q25" t="n">
-        <v>31.9</v>
+        <v>31.8</v>
       </c>
       <c r="R25" t="n">
         <v>3</v>
@@ -8788,10 +8794,10 @@
         <v>475000</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>687586</v>
+        <v>686851</v>
       </c>
       <c r="L26" t="n">
-        <v>30.91773247273796</v>
+        <v>30.8438074633363</v>
       </c>
       <c r="M26" s="3" t="n">
         <v>0</v>
@@ -8803,7 +8809,7 @@
         <v>100</v>
       </c>
       <c r="Q26" t="n">
-        <v>34.7</v>
+        <v>34.6</v>
       </c>
       <c r="R26" t="n">
         <v>3</v>
@@ -8852,10 +8858,10 @@
         <v>475000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>687586</v>
+        <v>686851</v>
       </c>
       <c r="L27" t="n">
-        <v>30.91773247273796</v>
+        <v>30.8438074633363</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -8867,7 +8873,7 @@
         <v>100</v>
       </c>
       <c r="Q27" t="n">
-        <v>34.7</v>
+        <v>34.6</v>
       </c>
       <c r="R27" t="n">
         <v>3</v>
@@ -8916,10 +8922,10 @@
         <v>475000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>687586</v>
+        <v>686851</v>
       </c>
       <c r="L28" t="n">
-        <v>30.91773247273796</v>
+        <v>30.8438074633363</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -8931,7 +8937,7 @@
         <v>100</v>
       </c>
       <c r="Q28" t="n">
-        <v>34.7</v>
+        <v>34.6</v>
       </c>
       <c r="R28" t="n">
         <v>3</v>
@@ -8980,10 +8986,10 @@
         <v>475000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>687586</v>
+        <v>686851</v>
       </c>
       <c r="L29" t="n">
-        <v>30.91773247273796</v>
+        <v>30.8438074633363</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -8995,7 +9001,7 @@
         <v>100</v>
       </c>
       <c r="Q29" t="n">
-        <v>34.7</v>
+        <v>34.6</v>
       </c>
       <c r="R29" t="n">
         <v>3</v>
@@ -9044,10 +9050,10 @@
         <v>479999</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>687586</v>
+        <v>686851</v>
       </c>
       <c r="L30" t="n">
-        <v>30.19069614564578</v>
+        <v>30.11599313388202</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -9108,10 +9114,10 @@
         <v>479999</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>687586</v>
+        <v>686851</v>
       </c>
       <c r="L31" t="n">
-        <v>30.19069614564578</v>
+        <v>30.11599313388202</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -9172,10 +9178,10 @@
         <v>479999</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>687586</v>
+        <v>686851</v>
       </c>
       <c r="L32" t="n">
-        <v>30.19069614564578</v>
+        <v>30.11599313388202</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -9236,10 +9242,10 @@
         <v>479999</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>687586</v>
+        <v>686851</v>
       </c>
       <c r="L33" t="n">
-        <v>30.19069614564578</v>
+        <v>30.11599313388202</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -9294,31 +9300,31 @@
         </is>
       </c>
       <c r="I34" s="3" t="n">
-        <v>482999</v>
+        <v>479999</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>482999</v>
+        <v>479999</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>644585</v>
+        <v>643896</v>
       </c>
       <c r="L34" t="n">
-        <v>25.06822218947075</v>
+        <v>25.45395529712873</v>
       </c>
       <c r="M34" s="3" t="n">
-        <v>0</v>
+        <v>-3000</v>
       </c>
       <c r="N34" t="n">
-        <v>0</v>
+        <v>0.6211192983836406</v>
       </c>
       <c r="O34" t="n">
         <v>100</v>
       </c>
       <c r="P34" t="n">
-        <v>1.520920258150865</v>
+        <v>2.54778368297421</v>
       </c>
       <c r="Q34" t="n">
-        <v>30.8</v>
+        <v>31.3</v>
       </c>
       <c r="R34" t="n">
         <v>4</v>
@@ -9361,31 +9367,31 @@
         </is>
       </c>
       <c r="I35" s="3" t="n">
-        <v>482999</v>
+        <v>479999</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>482999</v>
+        <v>479999</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>644585</v>
+        <v>643896</v>
       </c>
       <c r="L35" t="n">
-        <v>25.06822218947075</v>
+        <v>25.45395529712873</v>
       </c>
       <c r="M35" s="3" t="n">
-        <v>0</v>
+        <v>-3000</v>
       </c>
       <c r="N35" t="n">
-        <v>0</v>
+        <v>0.6211192983836406</v>
       </c>
       <c r="O35" t="n">
         <v>100</v>
       </c>
       <c r="P35" t="n">
-        <v>1.520920258150865</v>
+        <v>2.54778368297421</v>
       </c>
       <c r="Q35" t="n">
-        <v>30.8</v>
+        <v>31.3</v>
       </c>
       <c r="R35" t="n">
         <v>4</v>
@@ -9428,31 +9434,31 @@
         </is>
       </c>
       <c r="I36" s="3" t="n">
-        <v>482999</v>
+        <v>479999</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>482999</v>
+        <v>479999</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>644585</v>
+        <v>643896</v>
       </c>
       <c r="L36" t="n">
-        <v>25.06822218947075</v>
+        <v>25.45395529712873</v>
       </c>
       <c r="M36" s="3" t="n">
-        <v>0</v>
+        <v>-3000</v>
       </c>
       <c r="N36" t="n">
-        <v>0</v>
+        <v>0.6211192983836406</v>
       </c>
       <c r="O36" t="n">
         <v>100</v>
       </c>
       <c r="P36" t="n">
-        <v>1.520920258150865</v>
+        <v>2.54778368297421</v>
       </c>
       <c r="Q36" t="n">
-        <v>30.8</v>
+        <v>31.3</v>
       </c>
       <c r="R36" t="n">
         <v>4</v>
@@ -9495,22 +9501,22 @@
         </is>
       </c>
       <c r="I37" s="3" t="n">
-        <v>485999</v>
+        <v>484999</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>485999</v>
+        <v>484999</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>644585</v>
+        <v>643896</v>
       </c>
       <c r="L37" t="n">
-        <v>24.6028064568676</v>
+        <v>24.67743238038441</v>
       </c>
       <c r="M37" s="3" t="n">
-        <v>-4000</v>
+        <v>-1000</v>
       </c>
       <c r="N37" t="n">
-        <v>1.818383838383839</v>
+        <v>2.020404040404041</v>
       </c>
       <c r="O37" t="n">
         <v>0</v>
@@ -9519,7 +9525,7 @@
         <v>0</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.699999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="R37" t="n">
         <v>4</v>
@@ -9568,10 +9574,10 @@
         <v>500000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>644585</v>
+        <v>643896</v>
       </c>
       <c r="L38" t="n">
-        <v>22.4307112328087</v>
+        <v>22.34770832556811</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -9632,13 +9638,13 @@
         <v>549999</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>773588</v>
+        <v>772761</v>
       </c>
       <c r="L39" t="n">
-        <v>28.9028526812722</v>
+        <v>28.82676532588989</v>
       </c>
       <c r="M39" s="3" t="n">
-        <v>-2000</v>
+        <v>0</v>
       </c>
       <c r="N39" t="n">
         <v>0.3623194969556104</v>
@@ -9699,13 +9705,13 @@
         <v>549999</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>773588</v>
+        <v>772761</v>
       </c>
       <c r="L40" t="n">
-        <v>28.9028526812722</v>
+        <v>28.82676532588989</v>
       </c>
       <c r="M40" s="3" t="n">
-        <v>-2000</v>
+        <v>0</v>
       </c>
       <c r="N40" t="n">
         <v>0.3623194969556104</v>
@@ -9766,13 +9772,13 @@
         <v>549999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>773588</v>
+        <v>772761</v>
       </c>
       <c r="L41" t="n">
-        <v>28.9028526812722</v>
+        <v>28.82676532588989</v>
       </c>
       <c r="M41" s="3" t="n">
-        <v>-2000</v>
+        <v>0</v>
       </c>
       <c r="N41" t="n">
         <v>0.3623194969556104</v>
@@ -9833,13 +9839,13 @@
         <v>551999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>773588</v>
+        <v>772761</v>
       </c>
       <c r="L42" t="n">
-        <v>28.64431713004855</v>
+        <v>28.56795309287089</v>
       </c>
       <c r="M42" s="3" t="n">
-        <v>-6000</v>
+        <v>0</v>
       </c>
       <c r="N42" t="n">
         <v>1.075270744212803</v>
@@ -9851,7 +9857,7 @@
         <v>63.05922689075628</v>
       </c>
       <c r="Q42" t="n">
-        <v>20.4</v>
+        <v>20.3</v>
       </c>
       <c r="R42" t="n">
         <v>4</v>
@@ -9900,22 +9906,22 @@
         <v>564999</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>773588</v>
+        <v>772761</v>
       </c>
       <c r="L43" t="n">
-        <v>26.96383604709484</v>
+        <v>26.88567357824735</v>
       </c>
       <c r="M43" s="3" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="N43" t="n">
         <v>0</v>
       </c>
       <c r="P43" t="n">
-        <v>31.5589686132756</v>
+        <v>31.21022272724958</v>
       </c>
       <c r="Q43" t="n">
-        <v>18.3</v>
+        <v>18.2</v>
       </c>
       <c r="R43" t="n">
         <v>3</v>
@@ -9964,22 +9970,22 @@
         <v>564999</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>773588</v>
+        <v>772761</v>
       </c>
       <c r="L44" t="n">
-        <v>26.96383604709484</v>
+        <v>26.88567357824735</v>
       </c>
       <c r="M44" s="3" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="N44" t="n">
         <v>0</v>
       </c>
       <c r="P44" t="n">
-        <v>31.5589686132756</v>
+        <v>31.21022272724958</v>
       </c>
       <c r="Q44" t="n">
-        <v>18.3</v>
+        <v>18.2</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -10028,22 +10034,22 @@
         <v>564999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>773588</v>
+        <v>772761</v>
       </c>
       <c r="L45" t="n">
-        <v>26.96383604709484</v>
+        <v>26.88567357824735</v>
       </c>
       <c r="M45" s="3" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="N45" t="n">
         <v>0</v>
       </c>
       <c r="P45" t="n">
-        <v>31.5589686132756</v>
+        <v>31.21022272724958</v>
       </c>
       <c r="Q45" t="n">
-        <v>18.3</v>
+        <v>18.2</v>
       </c>
       <c r="R45" t="n">
         <v>3</v>
@@ -10092,22 +10098,22 @@
         <v>564999</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>773588</v>
+        <v>772761</v>
       </c>
       <c r="L46" t="n">
-        <v>26.96383604709484</v>
+        <v>26.88567357824735</v>
       </c>
       <c r="M46" s="3" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="N46" t="n">
         <v>0</v>
       </c>
       <c r="P46" t="n">
-        <v>31.5589686132756</v>
+        <v>31.21022272724958</v>
       </c>
       <c r="Q46" t="n">
-        <v>18.3</v>
+        <v>18.2</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -10156,10 +10162,10 @@
         <v>585000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>730587</v>
+        <v>729806</v>
       </c>
       <c r="L47" t="n">
-        <v>19.92740084343138</v>
+        <v>19.84171135890908</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -10168,10 +10174,10 @@
         <v>0</v>
       </c>
       <c r="P47" t="n">
-        <v>23.95398709245673</v>
+        <v>23.56648951077459</v>
       </c>
       <c r="Q47" t="n">
-        <v>13.7</v>
+        <v>13.6</v>
       </c>
       <c r="R47" t="n">
         <v>3</v>
@@ -10220,10 +10226,10 @@
         <v>595000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>730587</v>
+        <v>729806</v>
       </c>
       <c r="L48" t="n">
-        <v>18.55863846468661</v>
+        <v>18.47148420265112</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -10284,10 +10290,10 @@
         <v>614999</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>859590</v>
+        <v>858671</v>
       </c>
       <c r="L49" t="n">
-        <v>28.45437941344129</v>
+        <v>28.37780709957597</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -10296,10 +10302,10 @@
         <v>0.3241496339540259</v>
       </c>
       <c r="P49" t="n">
-        <v>59.31568727851597</v>
+        <v>59.10837762230636</v>
       </c>
       <c r="Q49" t="n">
-        <v>25</v>
+        <v>24.9</v>
       </c>
       <c r="R49" t="n">
         <v>3</v>
@@ -10348,10 +10354,10 @@
         <v>614999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>859590</v>
+        <v>858671</v>
       </c>
       <c r="L50" t="n">
-        <v>28.45437941344129</v>
+        <v>28.37780709957597</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -10360,10 +10366,10 @@
         <v>0.3241496339540259</v>
       </c>
       <c r="P50" t="n">
-        <v>59.31568727851597</v>
+        <v>59.10837762230636</v>
       </c>
       <c r="Q50" t="n">
-        <v>25</v>
+        <v>24.9</v>
       </c>
       <c r="R50" t="n">
         <v>3</v>
@@ -10412,10 +10418,10 @@
         <v>614999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>859590</v>
+        <v>858671</v>
       </c>
       <c r="L51" t="n">
-        <v>28.45437941344129</v>
+        <v>28.37780709957597</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -10424,10 +10430,10 @@
         <v>0.3241496339540259</v>
       </c>
       <c r="P51" t="n">
-        <v>59.31568727851597</v>
+        <v>59.10837762230636</v>
       </c>
       <c r="Q51" t="n">
-        <v>25</v>
+        <v>24.9</v>
       </c>
       <c r="R51" t="n">
         <v>3</v>
@@ -10476,10 +10482,10 @@
         <v>614999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>859590</v>
+        <v>858671</v>
       </c>
       <c r="L52" t="n">
-        <v>28.45437941344129</v>
+        <v>28.37780709957597</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -10488,10 +10494,10 @@
         <v>0</v>
       </c>
       <c r="P52" t="n">
-        <v>59.31568727851597</v>
+        <v>59.10837762230636</v>
       </c>
       <c r="Q52" t="n">
-        <v>24.9</v>
+        <v>24.8</v>
       </c>
       <c r="R52" t="n">
         <v>3</v>
@@ -10540,10 +10546,10 @@
         <v>650000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>816589</v>
+        <v>815716</v>
       </c>
       <c r="L53" t="n">
-        <v>20.4005931992716</v>
+        <v>20.31540389056976</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -10552,10 +10558,10 @@
         <v>0</v>
       </c>
       <c r="P53" t="n">
-        <v>48.66894128740829</v>
+        <v>48.40738041977285</v>
       </c>
       <c r="Q53" t="n">
-        <v>19.2</v>
+        <v>19.1</v>
       </c>
       <c r="R53" t="n">
         <v>3</v>
@@ -10604,10 +10610,10 @@
         <v>672000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>859590</v>
+        <v>858671</v>
       </c>
       <c r="L54" t="n">
-        <v>21.82319477890622</v>
+        <v>21.73952538282998</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -10619,7 +10625,7 @@
         <v>59.83193277310923</v>
       </c>
       <c r="Q54" t="n">
-        <v>22.2</v>
+        <v>22.1</v>
       </c>
       <c r="R54" t="n">
         <v>3</v>
@@ -10668,10 +10674,10 @@
         <v>700000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>902591</v>
+        <v>901626</v>
       </c>
       <c r="L55" t="n">
-        <v>22.44549303061963</v>
+        <v>22.36248732844883</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -10732,10 +10738,10 @@
         <v>715000</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>945592</v>
+        <v>944581</v>
       </c>
       <c r="L56" t="n">
-        <v>24.38599311330891</v>
+        <v>24.30506224452958</v>
       </c>
       <c r="M56" s="3" t="n">
         <v>0</v>
@@ -10744,10 +10750,10 @@
         <v>0</v>
       </c>
       <c r="P56" t="n">
-        <v>65.145577417376</v>
+        <v>64.96797435910501</v>
       </c>
       <c r="Q56" t="n">
-        <v>24.4</v>
+        <v>24.3</v>
       </c>
       <c r="R56" t="n">
         <v>3</v>
@@ -10796,10 +10802,10 @@
         <v>734999</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>988593</v>
+        <v>987536</v>
       </c>
       <c r="L57" t="n">
-        <v>25.65201250666351</v>
+        <v>25.57243482769236</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -10860,10 +10866,10 @@
         <v>752000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>988593</v>
+        <v>987536</v>
       </c>
       <c r="L58" t="n">
-        <v>23.93229569701586</v>
+        <v>23.85087733510474</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -10872,10 +10878,10 @@
         <v>0</v>
       </c>
       <c r="P58" t="n">
-        <v>55.76656915877901</v>
+        <v>55.54117473210056</v>
       </c>
       <c r="Q58" t="n">
-        <v>22.2</v>
+        <v>22.1</v>
       </c>
       <c r="R58" t="n">
         <v>3</v>
@@ -10924,10 +10930,10 @@
         <v>810000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1074595</v>
+        <v>1073446</v>
       </c>
       <c r="L59" t="n">
-        <v>24.62276485559676</v>
+        <v>24.54208222863563</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -10936,7 +10942,7 @@
         <v>0</v>
       </c>
       <c r="P59" t="n">
-        <v>70.39637354670639</v>
+        <v>70.24552627383726</v>
       </c>
       <c r="Q59" t="n">
         <v>25.6</v>
@@ -10988,10 +10994,10 @@
         <v>815000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1074595</v>
+        <v>1073446</v>
       </c>
       <c r="L60" t="n">
-        <v>24.15747328063131</v>
+        <v>24.07629261276301</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -11003,7 +11009,7 @@
         <v>80.25210084033613</v>
       </c>
       <c r="Q60" t="n">
-        <v>27.6</v>
+        <v>27.5</v>
       </c>
       <c r="R60" t="n">
         <v>3</v>
@@ -11052,10 +11058,10 @@
         <v>875000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1160597</v>
+        <v>1159356</v>
       </c>
       <c r="L61" t="n">
-        <v>24.6077665201616</v>
+        <v>24.52706502575568</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -11064,10 +11070,10 @@
         <v>0</v>
       </c>
       <c r="P61" t="n">
-        <v>80.03792161176989</v>
+        <v>79.93620349657833</v>
       </c>
       <c r="Q61" t="n">
-        <v>27.7</v>
+        <v>27.6</v>
       </c>
       <c r="R61" t="n">
         <v>3</v>
@@ -11116,10 +11122,10 @@
         <v>992000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1332602</v>
+        <v>1331176</v>
       </c>
       <c r="L62" t="n">
-        <v>25.55916920430856</v>
+        <v>25.47942571080008</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -11180,10 +11186,10 @@
         <v>1050000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1418604</v>
+        <v>1417086</v>
       </c>
       <c r="L63" t="n">
-        <v>25.98357258262348</v>
+        <v>25.90428527273574</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -11244,10 +11250,10 @@
         <v>1050000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1418604</v>
+        <v>1417086</v>
       </c>
       <c r="L64" t="n">
-        <v>25.98357258262348</v>
+        <v>25.90428527273574</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -11256,7 +11262,7 @@
         <v>0</v>
       </c>
       <c r="P64" t="n">
-        <v>86.69194774117993</v>
+        <v>86.62413566438555</v>
       </c>
       <c r="Q64" t="n">
         <v>29.7</v>
@@ -11308,10 +11314,10 @@
         <v>1100000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1504606</v>
+        <v>1502996</v>
       </c>
       <c r="L65" t="n">
-        <v>26.89115954608715</v>
+        <v>26.81284580930355</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -11320,7 +11326,7 @@
         <v>0</v>
       </c>
       <c r="P65" t="n">
-        <v>94.29654903193425</v>
+        <v>94.26748671330809</v>
       </c>
       <c r="Q65" t="n">
         <v>31.7</v>
@@ -11372,10 +11378,10 @@
         <v>1105000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1504606</v>
+        <v>1502996</v>
       </c>
       <c r="L66" t="n">
-        <v>26.558846634933</v>
+        <v>26.48017692661857</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -11436,10 +11442,10 @@
         <v>1155000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1590608</v>
+        <v>1588906</v>
       </c>
       <c r="L67" t="n">
-        <v>27.38625733053021</v>
+        <v>27.3084751394985</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -11451,7 +11457,7 @@
         <v>100</v>
       </c>
       <c r="Q67" t="n">
-        <v>33.2</v>
+        <v>33.1</v>
       </c>
       <c r="R67" t="n">
         <v>3</v>
@@ -11706,7 +11712,7 @@
         <v>315000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>300577</v>
+        <v>300256</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -11767,10 +11773,10 @@
         <v>380000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>386579</v>
+        <v>386166</v>
       </c>
       <c r="L3" t="n">
-        <v>1.701851368025681</v>
+        <v>1.596722652952357</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -11782,7 +11788,7 @@
         <v>100</v>
       </c>
       <c r="Q3" t="n">
-        <v>22.2</v>
+        <v>22.1</v>
       </c>
       <c r="R3" t="n">
         <v>3</v>
@@ -11831,7 +11837,7 @@
         <v>415000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>386579</v>
+        <v>386166</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -11892,10 +11898,10 @@
         <v>495000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>472581</v>
+        <v>472076</v>
       </c>
       <c r="L5" t="n">
-        <v>6.894479464895966</v>
+        <v>6.79488048534558</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -11907,7 +11913,7 @@
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="R5" t="n">
         <v>4</v>
@@ -11956,10 +11962,10 @@
         <v>500000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>515582</v>
+        <v>515031</v>
       </c>
       <c r="L6" t="n">
-        <v>8.840882730584077</v>
+        <v>8.743357195974612</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -11971,7 +11977,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>4.1</v>
+        <v>4</v>
       </c>
       <c r="R6" t="n">
         <v>4</v>
@@ -12020,10 +12026,10 @@
         <v>550000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>558583</v>
+        <v>557986</v>
       </c>
       <c r="L7" t="n">
-        <v>6.907299362852074</v>
+        <v>6.807697684171288</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -12084,7 +12090,7 @@
         <v>530000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>472581</v>
+        <v>472076</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -12148,10 +12154,10 @@
         <v>600000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>601584</v>
+        <v>600941</v>
       </c>
       <c r="L9" t="n">
-        <v>8.57469613553552</v>
+        <v>8.47687210558108</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -12212,10 +12218,10 @@
         <v>646000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>730587</v>
+        <v>729806</v>
       </c>
       <c r="L10" t="n">
-        <v>17.19001296217973</v>
+        <v>17.10139406910878</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -12276,7 +12282,7 @@
         <v>615000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>558583</v>
+        <v>557986</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -12340,7 +12346,7 @@
         <v>700000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>644585</v>
+        <v>643896</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -12404,7 +12410,7 @@
         <v>745000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>687586</v>
+        <v>686851</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -12468,7 +12474,7 @@
         <v>930000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>859590</v>
+        <v>858671</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -12539,7 +12545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12588,7 +12594,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Max 18 Core CPU 40 Core GPU 48GB 8TB Silver</t>
+          <t>Macbook Pro 16 MGE94 M5 Max 18 Core CPU 40 Core GPU 48GB 2TB Silver</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -12597,22 +12603,22 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>2480000</v>
+        <v>1460000</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>2395000</v>
+        <v>1450000</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-85000</v>
+        <v>-10000</v>
       </c>
       <c r="F2" t="n">
-        <v>-3.43</v>
+        <v>-0.68</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Max 18 Core CPU 40 Core GPU 128GB 8TB Silver</t>
+          <t>Macbook Pro 16 MGEE4 M5 Max 18 Core CPU 40 Core GPU 48GB 2TB Space Black</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -12621,22 +12627,22 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>3090000</v>
+        <v>1460000</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>3015000</v>
+        <v>1450000</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>-75000</v>
+        <v>-10000</v>
       </c>
       <c r="F3" t="n">
-        <v>-2.43</v>
+        <v>-0.68</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Max 18 Core CPU 40 Core GPU 128GB 4TB Silver</t>
+          <t>Macbook Pro 16 MGED4 M5 Max 18 Core CPU 32 Core GPU 36GB 2TB Space Black</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -12645,22 +12651,22 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>2470000</v>
+        <v>1207000</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>2410000</v>
+        <v>1200000</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>-60000</v>
+        <v>-7000</v>
       </c>
       <c r="F4" t="n">
-        <v>-2.43</v>
+        <v>-0.58</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Max 18 Core CPU 40 Core GPU 128GB 2TB Silver</t>
+          <t>Macbook Pro 16 MGE74 M5 Max 18 Core CPU 32 Core GPU 36GB 2TB Silver</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -12669,22 +12675,22 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>2170000</v>
+        <v>1207000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>2110000</v>
+        <v>1200000</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>-60000</v>
+        <v>-7000</v>
       </c>
       <c r="F5" t="n">
-        <v>-2.76</v>
+        <v>-0.58</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Max 18 Core CPU 40 Core GPU 48GB 4TB Silver</t>
+          <t>Macbook Pro 14 MGDR4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -12693,22 +12699,22 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>1840000</v>
+        <v>724999</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>1780000</v>
+        <v>720000</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-60000</v>
+        <v>-4999</v>
       </c>
       <c r="F6" t="n">
-        <v>-3.26</v>
+        <v>-0.6899999999999999</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Max 18 Core CPU 40 Core GPU 48GB 2TB Silver</t>
+          <t>Macbook Pro 14 MGDN4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Silver</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -12717,22 +12723,22 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>1535000</v>
+        <v>729999</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>1480000</v>
+        <v>725000</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>-55000</v>
+        <v>-4999</v>
       </c>
       <c r="F7" t="n">
-        <v>-3.58</v>
+        <v>-0.68</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Max 18 Core CPU 32 Core GPU 36GB 8TB Silver</t>
+          <t>Apple MacBook Air 15 MDVD4 M5 10C CPU 10C GPU 16GB 512GB Starlight</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -12741,22 +12747,22 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>2270000</v>
+        <v>482999</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>2215000</v>
+        <v>479999</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>-55000</v>
+        <v>-3000</v>
       </c>
       <c r="F8" t="n">
-        <v>-2.42</v>
+        <v>-0.62</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Max 18 Core CPU 40 Core GPU 64GB 8TB Silver</t>
+          <t>Apple MacBook Air 15 MDVQ4 M5 10C CPU 10C GPU 16GB 512GB Sky Blue</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -12765,22 +12771,22 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>2580000</v>
+        <v>482999</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>2530000</v>
+        <v>479999</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>-50000</v>
+        <v>-3000</v>
       </c>
       <c r="F9" t="n">
-        <v>-1.94</v>
+        <v>-0.62</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Max 18 Core CPU 40 Core GPU 64GB 4TB Silver</t>
+          <t>Apple MacBook Air 15 MDVH4 M5 10C CPU 10C GPU 16GB 512GB Midnight</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -12789,22 +12795,22 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>1960000</v>
+        <v>482999</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>1910000</v>
+        <v>479999</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>-50000</v>
+        <v>-3000</v>
       </c>
       <c r="F10" t="n">
-        <v>-2.55</v>
+        <v>-0.62</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Max 18 Core CPU 40 Core GPU 64GB 2TB Silver</t>
+          <t>Apple MacBook Air 15 MDV94 M5 10C CPU 10C GPU 16GB 512GB Silver</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -12813,861 +12819,45 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>1660000</v>
+        <v>485999</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>1610000</v>
+        <v>484999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>-50000</v>
+        <v>-1000</v>
       </c>
       <c r="F11" t="n">
-        <v>-3.01</v>
+        <v>-0.21</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Pro 18 Core CPU 20 Core GPU 64GB 4TB Space Black</t>
+          <t>Macbook Pro 14 M5 MDE04 10 Core CPU 10 Core GPU 16GB 512GB Space Black</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>1680000</v>
+        <v>555000</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>1630000</v>
+        <v>560000</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>-50000</v>
+        <v>5000</v>
       </c>
       <c r="F12" t="n">
-        <v>-2.98</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 CTO M5 Pro 18 Core CPU 20 Core GPU 24GB 4TB Space Black</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="n">
-        <v>1380000</v>
-      </c>
-      <c r="D13" s="3" t="n">
-        <v>1330000</v>
-      </c>
-      <c r="E13" s="3" t="n">
-        <v>-50000</v>
-      </c>
-      <c r="F13" t="n">
-        <v>-3.62</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 CTO M5 Pro 18 Core CPU 20 Core GPU 48GB 4TB Space Black</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="n">
-        <v>1560000</v>
-      </c>
-      <c r="D14" s="3" t="n">
-        <v>1515000</v>
-      </c>
-      <c r="E14" s="3" t="n">
-        <v>-45000</v>
-      </c>
-      <c r="F14" t="n">
-        <v>-2.88</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 CTO M5 Max 18 Core CPU 32 Core GPU 36GB 4TB Silver</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="n">
-        <v>1650000</v>
-      </c>
-      <c r="D15" s="3" t="n">
-        <v>1605000</v>
-      </c>
-      <c r="E15" s="3" t="n">
-        <v>-45000</v>
-      </c>
-      <c r="F15" t="n">
-        <v>-2.73</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 48GB 4TB Space Black</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="n">
-        <v>1490000</v>
-      </c>
-      <c r="D16" s="3" t="n">
-        <v>1445000</v>
-      </c>
-      <c r="E16" s="3" t="n">
-        <v>-45000</v>
-      </c>
-      <c r="F16" t="n">
-        <v>-3.02</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 32GB 4TB Space Black</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="n">
-        <v>1280000</v>
-      </c>
-      <c r="D17" s="3" t="n">
-        <v>1240000</v>
-      </c>
-      <c r="E17" s="3" t="n">
-        <v>-40000</v>
-      </c>
-      <c r="F17" t="n">
-        <v>-3.12</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 CTO M5 Pro 18 Core CPU 20 Core GPU 48GB 2TB Space Black</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="n">
-        <v>1245000</v>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>1210000</v>
-      </c>
-      <c r="E18" s="3" t="n">
-        <v>-35000</v>
-      </c>
-      <c r="F18" t="n">
-        <v>-2.81</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 CTO M5 Pro 18 Core CPU 20 Core GPU 64GB 2TB Space Black</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="n">
-        <v>1370000</v>
-      </c>
-      <c r="D19" s="3" t="n">
-        <v>1335000</v>
-      </c>
-      <c r="E19" s="3" t="n">
-        <v>-35000</v>
-      </c>
-      <c r="F19" t="n">
-        <v>-2.55</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 CTO M5 Pro 18 Core CPU 20 Core GPU 48GB 1TB Space Black</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="n">
-        <v>1095000</v>
-      </c>
-      <c r="D20" s="3" t="n">
-        <v>1060000</v>
-      </c>
-      <c r="E20" s="3" t="n">
-        <v>-35000</v>
-      </c>
-      <c r="F20" t="n">
-        <v>-3.2</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Apple MacBook Pro 16Inch MX2X3 14Core CPU 20Core GPU M4 Pro 24GB 512GB Space Black</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="n">
-        <v>739999</v>
-      </c>
-      <c r="D21" s="3" t="n">
-        <v>707999</v>
-      </c>
-      <c r="E21" s="3" t="n">
-        <v>-32000</v>
-      </c>
-      <c r="F21" t="n">
-        <v>-4.32</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 CTO M5 Pro 18 Core CPU 20 Core GPU 64GB 1TB Space Black</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="n">
-        <v>1215000</v>
-      </c>
-      <c r="D22" s="3" t="n">
-        <v>1185000</v>
-      </c>
-      <c r="E22" s="3" t="n">
-        <v>-30000</v>
-      </c>
-      <c r="F22" t="n">
-        <v>-2.47</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 48GB 2TB Space Black</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="n">
-        <v>1180000</v>
-      </c>
-      <c r="D23" s="3" t="n">
-        <v>1155000</v>
-      </c>
-      <c r="E23" s="3" t="n">
-        <v>-25000</v>
-      </c>
-      <c r="F23" t="n">
-        <v>-2.12</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 48GB 1TB Space Black</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="n">
-        <v>1020000</v>
-      </c>
-      <c r="D24" s="3" t="n">
-        <v>995000</v>
-      </c>
-      <c r="E24" s="3" t="n">
-        <v>-25000</v>
-      </c>
-      <c r="F24" t="n">
-        <v>-2.45</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 24GB 4TB Space Black</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="n">
-        <v>1210000</v>
-      </c>
-      <c r="D25" s="3" t="n">
-        <v>1185000</v>
-      </c>
-      <c r="E25" s="3" t="n">
-        <v>-25000</v>
-      </c>
-      <c r="F25" t="n">
-        <v>-2.07</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Macbook Pro 16 MGE64 M5 Pro 18 Core CPU 20 Core GPU 48GB 1TB Silver</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="n">
-        <v>1080000</v>
-      </c>
-      <c r="D26" s="3" t="n">
-        <v>1055000</v>
-      </c>
-      <c r="E26" s="3" t="n">
-        <v>-25000</v>
-      </c>
-      <c r="F26" t="n">
-        <v>-2.31</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 32GB 2TB Space Black</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="n">
-        <v>960000</v>
-      </c>
-      <c r="D27" s="3" t="n">
-        <v>940000</v>
-      </c>
-      <c r="E27" s="3" t="n">
-        <v>-20000</v>
-      </c>
-      <c r="F27" t="n">
-        <v>-2.08</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 16GB 4TB Space Black</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="n">
-        <v>1150000</v>
-      </c>
-      <c r="D28" s="3" t="n">
-        <v>1130000</v>
-      </c>
-      <c r="E28" s="3" t="n">
-        <v>-20000</v>
-      </c>
-      <c r="F28" t="n">
-        <v>-1.74</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDH74 M5 10C CPU 8C GPU 16GB 512GB Silver</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="n">
-        <v>443000</v>
-      </c>
-      <c r="D29" s="3" t="n">
-        <v>425000</v>
-      </c>
-      <c r="E29" s="3" t="n">
-        <v>-18000</v>
-      </c>
-      <c r="F29" t="n">
-        <v>-4.06</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 CTO M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Space Black</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="n">
-        <v>890000</v>
-      </c>
-      <c r="D30" s="3" t="n">
-        <v>875000</v>
-      </c>
-      <c r="E30" s="3" t="n">
-        <v>-15000</v>
-      </c>
-      <c r="F30" t="n">
-        <v>-1.69</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 24GB 2TB Space Black</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="n">
-        <v>890000</v>
-      </c>
-      <c r="D31" s="3" t="n">
-        <v>880000</v>
-      </c>
-      <c r="E31" s="3" t="n">
-        <v>-10000</v>
-      </c>
-      <c r="F31" t="n">
-        <v>-1.12</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDHE4 M5 10C CPU 8C GPU 16GB 512GB Midnight</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="n">
-        <v>433999</v>
-      </c>
-      <c r="D32" s="3" t="n">
-        <v>425000</v>
-      </c>
-      <c r="E32" s="3" t="n">
-        <v>-8999</v>
-      </c>
-      <c r="F32" t="n">
-        <v>-2.07</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDHH4 M5 10C CPU 8C GPU 16GB 512GB Sky Blue</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="n">
-        <v>433999</v>
-      </c>
-      <c r="D33" s="3" t="n">
-        <v>425000</v>
-      </c>
-      <c r="E33" s="3" t="n">
-        <v>-8999</v>
-      </c>
-      <c r="F33" t="n">
-        <v>-2.07</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDHA4 M5 10C CPU 8C GPU 16GB 512GB Starlight</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="n">
-        <v>433999</v>
-      </c>
-      <c r="D34" s="3" t="n">
-        <v>425000</v>
-      </c>
-      <c r="E34" s="3" t="n">
-        <v>-8999</v>
-      </c>
-      <c r="F34" t="n">
-        <v>-2.07</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Macbook Pro 16 MGEC4 M5 Pro 18 Core CPU 20 Core GPU 48GB 1TB Space Black</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="n">
-        <v>1063000</v>
-      </c>
-      <c r="D35" s="3" t="n">
-        <v>1055000</v>
-      </c>
-      <c r="E35" s="3" t="n">
-        <v>-8000</v>
-      </c>
-      <c r="F35" t="n">
-        <v>-0.75</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDH94 M5 10C CPU 10C GPU 24GB 1TB Silver</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="n">
-        <v>557999</v>
-      </c>
-      <c r="D36" s="3" t="n">
-        <v>551999</v>
-      </c>
-      <c r="E36" s="3" t="n">
-        <v>-6000</v>
-      </c>
-      <c r="F36" t="n">
-        <v>-1.08</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 16GB 2TB Space Black</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="n">
-        <v>835000</v>
-      </c>
-      <c r="D37" s="3" t="n">
-        <v>830000</v>
-      </c>
-      <c r="E37" s="3" t="n">
-        <v>-5000</v>
-      </c>
-      <c r="F37" t="n">
-        <v>-0.6</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Macbook Pro 16 MGEA4 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Space Black</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="n">
-        <v>829999</v>
-      </c>
-      <c r="D38" s="3" t="n">
-        <v>825000</v>
-      </c>
-      <c r="E38" s="3" t="n">
-        <v>-4999</v>
-      </c>
-      <c r="F38" t="n">
-        <v>-0.6</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDV94 M5 10C CPU 10C GPU 16GB 512GB Silver</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="n">
-        <v>489999</v>
-      </c>
-      <c r="D39" s="3" t="n">
-        <v>485999</v>
-      </c>
-      <c r="E39" s="3" t="n">
-        <v>-4000</v>
-      </c>
-      <c r="F39" t="n">
-        <v>-0.82</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDHG4 M5 10C CPU 10C GPU 24GB 1TB Midnight</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="n">
-        <v>551999</v>
-      </c>
-      <c r="D40" s="3" t="n">
-        <v>549999</v>
-      </c>
-      <c r="E40" s="3" t="n">
-        <v>-2000</v>
-      </c>
-      <c r="F40" t="n">
-        <v>-0.36</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDHK4 M5 10C CPU 10C GPU 24GB 1TB Sky Blue</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="n">
-        <v>551999</v>
-      </c>
-      <c r="D41" s="3" t="n">
-        <v>549999</v>
-      </c>
-      <c r="E41" s="3" t="n">
-        <v>-2000</v>
-      </c>
-      <c r="F41" t="n">
-        <v>-0.36</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDHD4 M5 10C CPU 10C GPU 24GB 1TB Starlight</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="n">
-        <v>551999</v>
-      </c>
-      <c r="D42" s="3" t="n">
-        <v>549999</v>
-      </c>
-      <c r="E42" s="3" t="n">
-        <v>-2000</v>
-      </c>
-      <c r="F42" t="n">
-        <v>-0.36</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDVK4 M5 10C CPU 10C GPU 16GB 1TB Midnight</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="n">
-        <v>559999</v>
-      </c>
-      <c r="D43" s="3" t="n">
-        <v>564999</v>
-      </c>
-      <c r="E43" s="3" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F43" t="n">
-        <v>0.89</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDVA4 M5 10C CPU 10C GPU 16GB 1TB Silver</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="n">
-        <v>559999</v>
-      </c>
-      <c r="D44" s="3" t="n">
-        <v>564999</v>
-      </c>
-      <c r="E44" s="3" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F44" t="n">
-        <v>0.89</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDVE4 M5 10C CPU 10C GPU 16GB 1TB Starlight</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="n">
-        <v>559999</v>
-      </c>
-      <c r="D45" s="3" t="n">
-        <v>564999</v>
-      </c>
-      <c r="E45" s="3" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F45" t="n">
-        <v>0.89</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDVT4 M5 10C CPU 10C GPU 16GB 1TB Sky Blue</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="C46" s="3" t="n">
-        <v>559999</v>
-      </c>
-      <c r="D46" s="3" t="n">
-        <v>564999</v>
-      </c>
-      <c r="E46" s="3" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F46" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F46"/>
-  <conditionalFormatting sqref="E2:E46">
+  <autoFilter ref="A1:F12"/>
+  <conditionalFormatting sqref="E2:E12">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
chore: price data 2026-09-24
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MacBook Pro'!$A$1:$S$92</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MacBook Air'!$A$1:$S$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20260923T083904842383+0000</t>
+          <t>20260924T083143925226+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-23T08:39:04.842383+00:00</t>
+          <t>2026-09-24T08:31:43.925226+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>277.129099</v>
+        <v>276.970859</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -885,7 +885,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 16Inch MX303 14Core CPU 32Core GPU M4 Max 36GB 1TB Space Black</t>
+          <t>Macbook Pro 14 MGDN4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Silver</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -894,34 +894,34 @@
         </is>
       </c>
       <c r="C30" s="3" t="n">
-        <v>970000</v>
+        <v>725000</v>
       </c>
       <c r="D30" t="n">
-        <v>43.2</v>
+        <v>43.1</v>
       </c>
       <c r="E30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 MGDN4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Silver</t>
+          <t>Apple MacBook Air 13 MDHG4 M5 10C CPU 10C GPU 24GB 1TB Midnight</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>macbook_pro</t>
+          <t>macbook_air</t>
         </is>
       </c>
       <c r="C31" s="3" t="n">
-        <v>725000</v>
+        <v>549999</v>
       </c>
       <c r="D31" t="n">
-        <v>43.1</v>
+        <v>42.6</v>
       </c>
       <c r="E31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="33">
@@ -1147,10 +1147,10 @@
         <v>470000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>686851</v>
+        <v>686458</v>
       </c>
       <c r="L2" t="n">
-        <v>35.21156699196769</v>
+        <v>35.17447535027635</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1214,10 +1214,10 @@
         <v>465000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>686851</v>
+        <v>686458</v>
       </c>
       <c r="L3" t="n">
-        <v>33.31887119622742</v>
+        <v>33.28069597848667</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>772761</v>
+        <v>772319</v>
       </c>
       <c r="L4" t="n">
-        <v>35.29707115136504</v>
+        <v>35.2600415113444</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>772761</v>
+        <v>772319</v>
       </c>
       <c r="L5" t="n">
-        <v>32.70894882117499</v>
+        <v>32.67043799259115</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>858671</v>
+        <v>858180</v>
       </c>
       <c r="L6" t="n">
-        <v>38.04379092807373</v>
+        <v>38.00834323801534</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1545,7 +1545,7 @@
       </c>
       <c r="K8" s="3" t="n"/>
       <c r="M8" s="3" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="N8" t="n">
         <v>0</v>
@@ -1606,10 +1606,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>858671</v>
+        <v>858180</v>
       </c>
       <c r="L9" t="n">
-        <v>34.20064262098056</v>
+        <v>34.16299610804261</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1673,10 +1673,10 @@
         <v>582999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>858671</v>
+        <v>858180</v>
       </c>
       <c r="L10" t="n">
-        <v>32.10449636706026</v>
+        <v>32.06565056281899</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -1740,10 +1740,10 @@
         <v>587999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>858671</v>
+        <v>858180</v>
       </c>
       <c r="L11" t="n">
-        <v>31.52220116901584</v>
+        <v>31.48302220979281</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -1772,7 +1772,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 MDE34 10 Core CPU 10 Core GPU 24GB 1TB Space Black</t>
+          <t>Apple MacBook Pro 14Inch MX2E3 M4 Pro 12Core CPU 16Core GPU 24GB 512GB Silver</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -1780,55 +1780,52 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M4 Pro</t>
         </is>
       </c>
       <c r="D12" t="n">
         <v>24</v>
       </c>
       <c r="E12" t="n">
-        <v>1024</v>
+        <v>512</v>
       </c>
       <c r="F12" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G12" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I12" s="3" t="n">
-        <v>643999</v>
+        <v>600000</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>643999</v>
+        <v>600000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>944581</v>
+        <v>858180</v>
       </c>
       <c r="L12" t="n">
-        <v>31.82172836421652</v>
+        <v>30.0845976368594</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>0</v>
+        <v>-50000</v>
       </c>
       <c r="N12" t="n">
-        <v>0</v>
-      </c>
-      <c r="O12" t="n">
-        <v>100</v>
+        <v>7.692307692307693</v>
       </c>
       <c r="P12" t="n">
-        <v>69.44023999999999</v>
+        <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>44.4</v>
+        <v>15.6</v>
       </c>
       <c r="R12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -1839,7 +1836,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 32GB 512GB Space Black</t>
+          <t>Apple MacBook Pro 14Inch MX2H3 M4 Pro 12Core CPU 16Core GPU 24GB 512GB Space Black</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1847,20 +1844,20 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M4 Pro</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="E13" t="n">
         <v>512</v>
       </c>
       <c r="F13" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G13" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -1868,26 +1865,31 @@
         </is>
       </c>
       <c r="I13" s="3" t="n">
-        <v>650000</v>
+        <v>600000</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>580000</v>
-      </c>
-      <c r="K13" s="3" t="n"/>
+        <v>600000</v>
+      </c>
+      <c r="K13" s="3" t="n">
+        <v>858180</v>
+      </c>
+      <c r="L13" t="n">
+        <v>30.0845976368594</v>
+      </c>
       <c r="M13" s="3" t="n">
-        <v>0</v>
+        <v>-50000</v>
       </c>
       <c r="N13" t="n">
-        <v>0</v>
+        <v>7.692307692307693</v>
       </c>
       <c r="P13" t="n">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>25.5</v>
+        <v>15.6</v>
       </c>
       <c r="R13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
@@ -1898,7 +1900,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 MDE64 10 Core CPU 10 Core GPU 24GB 1TB Silver</t>
+          <t>Macbook Pro 14 M5 MDE34 10 Core CPU 10 Core GPU 24GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -1923,20 +1925,20 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I14" s="3" t="n">
-        <v>650000</v>
+        <v>643999</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>650000</v>
+        <v>643999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>944581</v>
+        <v>944041</v>
       </c>
       <c r="L14" t="n">
-        <v>31.18642022229962</v>
+        <v>31.78272977550763</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -1945,13 +1947,13 @@
         <v>0</v>
       </c>
       <c r="O14" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="P14" t="n">
-        <v>68</v>
+        <v>69.44023999999999</v>
       </c>
       <c r="Q14" t="n">
-        <v>21.7</v>
+        <v>44.4</v>
       </c>
       <c r="R14" t="n">
         <v>4</v>
@@ -1965,7 +1967,7 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 14Inch MX2E3 M4 Pro 12Core CPU 16Core GPU 24GB 512GB Silver</t>
+          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 32GB 512GB Space Black</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1973,38 +1975,33 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>M4 Pro</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="E15" t="n">
         <v>512</v>
       </c>
       <c r="F15" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G15" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I15" s="3" t="n">
         <v>650000</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>650000</v>
-      </c>
-      <c r="K15" s="3" t="n">
-        <v>858671</v>
-      </c>
-      <c r="L15" t="n">
-        <v>24.30162425422543</v>
-      </c>
+        <v>580000</v>
+      </c>
+      <c r="K15" s="3" t="n"/>
       <c r="M15" s="3" t="n">
         <v>0</v>
       </c>
@@ -2012,13 +2009,13 @@
         <v>0</v>
       </c>
       <c r="P15" t="n">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="Q15" t="n">
-        <v>10.4</v>
+        <v>25.5</v>
       </c>
       <c r="R15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>
@@ -2029,7 +2026,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 14Inch MX2H3 M4 Pro 12Core CPU 16Core GPU 24GB 512GB Space Black</t>
+          <t>Macbook Pro 14 M5 MDE64 10 Core CPU 10 Core GPU 24GB 1TB Silver</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -2037,24 +2034,24 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>M4 Pro</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="D16" t="n">
         <v>24</v>
       </c>
       <c r="E16" t="n">
-        <v>512</v>
+        <v>1024</v>
       </c>
       <c r="F16" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G16" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I16" s="3" t="n">
@@ -2064,10 +2061,10 @@
         <v>650000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>858671</v>
+        <v>944041</v>
       </c>
       <c r="L16" t="n">
-        <v>24.30162425422543</v>
+        <v>31.14705823158104</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -2075,14 +2072,17 @@
       <c r="N16" t="n">
         <v>0</v>
       </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
       <c r="P16" t="n">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="Q16" t="n">
-        <v>10.4</v>
+        <v>21.7</v>
       </c>
       <c r="R16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>
@@ -2128,10 +2128,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1030491</v>
+        <v>1029902</v>
       </c>
       <c r="L17" t="n">
-        <v>32.07121653658304</v>
+        <v>32.03236812822968</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2189,19 +2189,19 @@
         </is>
       </c>
       <c r="I18" s="3" t="n">
-        <v>707999</v>
+        <v>711999</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>707999</v>
+        <v>711999</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>1073446</v>
+        <v>1072833</v>
       </c>
       <c r="L18" t="n">
-        <v>34.04428355036024</v>
+        <v>33.63375287672918</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="N18" t="n">
         <v>0</v>
@@ -2210,10 +2210,10 @@
         <v>100</v>
       </c>
       <c r="P18" t="n">
-        <v>12.49398266190719</v>
+        <v>11.06613972463029</v>
       </c>
       <c r="Q18" t="n">
-        <v>35.7</v>
+        <v>35.3</v>
       </c>
       <c r="R18" t="n">
         <v>4</v>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="K19" s="3" t="n"/>
       <c r="M19" s="3" t="n">
-        <v>-4999</v>
+        <v>0</v>
       </c>
       <c r="N19" t="n">
         <v>1.098901098901099</v>
@@ -2324,10 +2324,10 @@
         <v>720000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>1030491</v>
+        <v>1029902</v>
       </c>
       <c r="L20" t="n">
-        <v>30.13039415191399</v>
+        <v>30.09043578903624</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -2339,10 +2339,10 @@
         <v>0</v>
       </c>
       <c r="P20" t="n">
-        <v>82.22222222222221</v>
+        <v>60</v>
       </c>
       <c r="Q20" t="n">
-        <v>23.7</v>
+        <v>20</v>
       </c>
       <c r="R20" t="n">
         <v>4</v>
@@ -2392,7 +2392,7 @@
       </c>
       <c r="K21" s="3" t="n"/>
       <c r="M21" s="3" t="n">
-        <v>-4999</v>
+        <v>0</v>
       </c>
       <c r="N21" t="n">
         <v>1.360544217687075</v>
@@ -2453,10 +2453,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1073446</v>
+        <v>1072833</v>
       </c>
       <c r="L22" t="n">
-        <v>30.78366308132873</v>
+        <v>30.74411394876929</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2471,7 +2471,7 @@
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>10.3</v>
+        <v>10.2</v>
       </c>
       <c r="R22" t="n">
         <v>4</v>
@@ -2520,10 +2520,10 @@
         <v>745000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1030491</v>
+        <v>1029902</v>
       </c>
       <c r="L23" t="n">
-        <v>27.70436617107767</v>
+        <v>27.66302036504444</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -2587,10 +2587,10 @@
         <v>755000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1030491</v>
+        <v>1029902</v>
       </c>
       <c r="L24" t="n">
-        <v>26.73395497874314</v>
+        <v>26.69205419544772</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -2654,10 +2654,10 @@
         <v>772000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>1030491</v>
+        <v>1029902</v>
       </c>
       <c r="L25" t="n">
-        <v>25.08425595177445</v>
+        <v>25.0414117071333</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -2672,7 +2672,7 @@
         <v>69.59999999999998</v>
       </c>
       <c r="Q25" t="n">
-        <v>20</v>
+        <v>19.9</v>
       </c>
       <c r="R25" t="n">
         <v>4</v>
@@ -2783,10 +2783,10 @@
         <v>810000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>1245266</v>
+        <v>1244555</v>
       </c>
       <c r="L27" t="n">
-        <v>34.95365648785079</v>
+        <v>34.91649625769854</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -2912,10 +2912,10 @@
         <v>825000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>1288221</v>
+        <v>1287485</v>
       </c>
       <c r="L29" t="n">
-        <v>35.95819350872249</v>
+        <v>35.92158355242974</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -2927,10 +2927,10 @@
         <v>100</v>
       </c>
       <c r="P29" t="n">
-        <v>5.34521158129176</v>
+        <v>1.718244359164265</v>
       </c>
       <c r="Q29" t="n">
-        <v>35.4</v>
+        <v>34.7</v>
       </c>
       <c r="R29" t="n">
         <v>4</v>
@@ -2944,60 +2944,63 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 16GB 2TB Space Black</t>
+          <t>Macbook Pro 16 MGE44 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Silver</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M5 Pro</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E30" t="n">
-        <v>2048</v>
+        <v>1024</v>
       </c>
       <c r="F30" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="G30" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I30" s="3" t="n">
-        <v>830000</v>
+        <v>829999</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>830000</v>
+        <v>829999</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1073446</v>
+        <v>1287485</v>
       </c>
       <c r="L30" t="n">
-        <v>22.67892376514515</v>
+        <v>35.53330718416137</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>0</v>
+        <v>-10001</v>
       </c>
       <c r="N30" t="n">
-        <v>0.5988023952095809</v>
+        <v>4.597816091954023</v>
+      </c>
+      <c r="O30" t="n">
+        <v>0</v>
       </c>
       <c r="P30" t="n">
-        <v>57.99999999999999</v>
+        <v>0</v>
       </c>
       <c r="Q30" t="n">
-        <v>22.4</v>
+        <v>13.1</v>
       </c>
       <c r="R30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S30" t="inlineStr">
         <is>
@@ -3008,63 +3011,60 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 MGE44 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Silver</t>
+          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 16GB 2TB Space Black</t>
         </is>
       </c>
       <c r="B31" t="n">
+        <v>14</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
         <v>16</v>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>M5 Pro</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>24</v>
-      </c>
       <c r="E31" t="n">
-        <v>1024</v>
+        <v>2048</v>
       </c>
       <c r="F31" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="G31" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I31" s="3" t="n">
-        <v>840000</v>
+        <v>830000</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>840000</v>
+        <v>830000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1288221</v>
+        <v>1072833</v>
       </c>
       <c r="L31" t="n">
-        <v>34.7937970270629</v>
+        <v>22.63474371127659</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N31" t="n">
-        <v>3.448275862068965</v>
-      </c>
-      <c r="O31" t="n">
-        <v>0</v>
+        <v>0.5988023952095809</v>
       </c>
       <c r="P31" t="n">
-        <v>0</v>
+        <v>57.99999999999999</v>
       </c>
       <c r="Q31" t="n">
-        <v>12.6</v>
+        <v>22.3</v>
       </c>
       <c r="R31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S31" t="inlineStr">
         <is>
@@ -3110,10 +3110,10 @@
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1374131</v>
+        <v>1373346</v>
       </c>
       <c r="L32" t="n">
-        <v>38.28834368775612</v>
+        <v>38.25306951052393</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3177,10 +3177,10 @@
         <v>930000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1374131</v>
+        <v>1373346</v>
       </c>
       <c r="L33" t="n">
-        <v>38.14279715689406</v>
+        <v>38.10743978574955</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3244,10 +3244,10 @@
         <v>860000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>1245266</v>
+        <v>1244555</v>
       </c>
       <c r="L34" t="n">
-        <v>30.93845009821195</v>
+        <v>30.89899602669227</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -3497,10 +3497,10 @@
         <v>880000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>1159356</v>
+        <v>1158694</v>
       </c>
       <c r="L38" t="n">
-        <v>24.09579111161714</v>
+        <v>24.0524245400425</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -3561,10 +3561,10 @@
         <v>940000</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>1245266</v>
+        <v>1244555</v>
       </c>
       <c r="L39" t="n">
-        <v>24.5141198747898</v>
+        <v>24.47099565708225</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -3590,28 +3590,28 @@
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 16Inch MX303 14Core CPU 32Core GPU M4 Max 36GB 1TB Space Black</t>
+          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 48GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>M4 Max</t>
+          <t>M5 Pro</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="E40" t="n">
         <v>1024</v>
       </c>
       <c r="F40" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G40" t="n">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -3619,34 +3619,29 @@
         </is>
       </c>
       <c r="I40" s="3" t="n">
-        <v>970000</v>
+        <v>995000</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>970000</v>
-      </c>
-      <c r="K40" s="3" t="n">
-        <v>1502996</v>
-      </c>
-      <c r="L40" t="n">
-        <v>35.46223675911313</v>
-      </c>
+        <v>995000</v>
+      </c>
+      <c r="K40" s="3" t="n"/>
       <c r="M40" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N40" t="n">
-        <v>0</v>
+        <v>2.450980392156863</v>
       </c>
       <c r="O40" t="n">
         <v>100</v>
       </c>
       <c r="P40" t="n">
-        <v>54.87506124448805</v>
+        <v>69.23076923076923</v>
       </c>
       <c r="Q40" t="n">
-        <v>43.2</v>
+        <v>51.7</v>
       </c>
       <c r="R40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S40" t="inlineStr">
         <is>
@@ -3657,32 +3652,32 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 48GB 1TB Space Black</t>
+          <t>Apple MacBook Pro 16Inch MX2V3 14Core CPU 32Core GPU M4 Max 36GB 1TB Silver</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>M5 Pro</t>
+          <t>M4 Max</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="E41" t="n">
         <v>1024</v>
       </c>
       <c r="F41" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G41" t="n">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I41" s="3" t="n">
@@ -3691,21 +3686,23 @@
       <c r="J41" s="3" t="n">
         <v>995000</v>
       </c>
-      <c r="K41" s="3" t="n"/>
+      <c r="K41" s="3" t="n">
+        <v>1502138</v>
+      </c>
+      <c r="L41" t="n">
+        <v>33.76107920843491</v>
+      </c>
       <c r="M41" s="3" t="n">
-        <v>0</v>
+        <v>-27000</v>
       </c>
       <c r="N41" t="n">
-        <v>2.450980392156863</v>
-      </c>
-      <c r="O41" t="n">
-        <v>100</v>
+        <v>2.64187866927593</v>
       </c>
       <c r="P41" t="n">
-        <v>69.23076923076923</v>
+        <v>35.27682508574235</v>
       </c>
       <c r="Q41" t="n">
-        <v>51.7</v>
+        <v>23</v>
       </c>
       <c r="R41" t="n">
         <v>3</v>
@@ -3719,7 +3716,7 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 16Inch MX2V3 14Core CPU 32Core GPU M4 Max 36GB 1TB Silver</t>
+          <t>Apple MacBook Pro 16Inch MX303 14Core CPU 32Core GPU M4 Max 36GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -3744,38 +3741,35 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I42" s="3" t="n">
-        <v>1022000</v>
+        <v>995000</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>1022000</v>
+        <v>995000</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>1502996</v>
+        <v>1502138</v>
       </c>
       <c r="L42" t="n">
-        <v>32.0024803791893</v>
+        <v>33.76107920843491</v>
       </c>
       <c r="M42" s="3" t="n">
-        <v>0</v>
+        <v>25000</v>
       </c>
       <c r="N42" t="n">
         <v>0</v>
       </c>
-      <c r="O42" t="n">
-        <v>0</v>
-      </c>
       <c r="P42" t="n">
-        <v>14.11073003429697</v>
+        <v>35.27682508574235</v>
       </c>
       <c r="Q42" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="R42" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S42" t="inlineStr">
         <is>
@@ -3821,10 +3815,10 @@
         <v>1055000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1545951</v>
+        <v>1545068</v>
       </c>
       <c r="L43" t="n">
-        <v>31.75721610840188</v>
+        <v>31.71821563840556</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -3833,10 +3827,10 @@
         <v>0.7525870178739417</v>
       </c>
       <c r="P43" t="n">
-        <v>64.3652561247216</v>
+        <v>58.64647440248988</v>
       </c>
       <c r="Q43" t="n">
-        <v>27.7</v>
+        <v>26.4</v>
       </c>
       <c r="R43" t="n">
         <v>3</v>
@@ -3885,10 +3879,10 @@
         <v>1055000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1545951</v>
+        <v>1545068</v>
       </c>
       <c r="L44" t="n">
-        <v>31.75721610840188</v>
+        <v>31.71821563840556</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -3897,10 +3891,10 @@
         <v>2.764976958525346</v>
       </c>
       <c r="P44" t="n">
-        <v>64.3652561247216</v>
+        <v>58.64647440248988</v>
       </c>
       <c r="Q44" t="n">
-        <v>28.4</v>
+        <v>27.1</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -3976,7 +3970,7 @@
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 16Inch MX2W3 16Core CPU 40Core GPU M4 Max  48GB 1TB Silver</t>
+          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 24GB 2TB Space Black</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -3984,55 +3978,52 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>M4 Max</t>
+          <t>M5 Pro</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="E46" t="n">
-        <v>1024</v>
+        <v>2048</v>
       </c>
       <c r="F46" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G46" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I46" s="3" t="n">
-        <v>1123000</v>
+        <v>1115000</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>1123000</v>
+        <v>1115000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1717771</v>
+        <v>1502138</v>
       </c>
       <c r="L46" t="n">
-        <v>34.62458034278143</v>
+        <v>25.77246564563309</v>
       </c>
       <c r="M46" s="3" t="n">
-        <v>0</v>
+        <v>-35000</v>
       </c>
       <c r="N46" t="n">
-        <v>0</v>
-      </c>
-      <c r="O46" t="n">
-        <v>100</v>
+        <v>3.043478260869565</v>
       </c>
       <c r="P46" t="n">
-        <v>100</v>
+        <v>11.53874765504792</v>
       </c>
       <c r="Q46" t="n">
-        <v>50.4</v>
+        <v>14.6</v>
       </c>
       <c r="R46" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S46" t="inlineStr">
         <is>
@@ -4043,60 +4034,63 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 16GB 4TB Space Black</t>
+          <t>Apple MacBook Pro 16Inch MX2W3 16Core CPU 40Core GPU M4 Max  48GB 1TB Silver</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M4 Max</t>
         </is>
       </c>
       <c r="D47" t="n">
+        <v>48</v>
+      </c>
+      <c r="E47" t="n">
+        <v>1024</v>
+      </c>
+      <c r="F47" t="n">
         <v>16</v>
       </c>
-      <c r="E47" t="n">
-        <v>4096</v>
-      </c>
-      <c r="F47" t="n">
-        <v>10</v>
-      </c>
       <c r="G47" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I47" s="3" t="n">
-        <v>1130000</v>
+        <v>1123000</v>
       </c>
       <c r="J47" s="3" t="n">
-        <v>1130000</v>
+        <v>1123000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1502996</v>
+        <v>1716790</v>
       </c>
       <c r="L47" t="n">
-        <v>24.81683251319365</v>
+        <v>34.58722383052091</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N47" t="n">
-        <v>1.739130434782609</v>
+        <v>0</v>
+      </c>
+      <c r="O47" t="n">
+        <v>100</v>
       </c>
       <c r="P47" t="n">
-        <v>88.39999999999999</v>
+        <v>100</v>
       </c>
       <c r="Q47" t="n">
-        <v>30.2</v>
+        <v>50.4</v>
       </c>
       <c r="R47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S47" t="inlineStr">
         <is>
@@ -4107,28 +4101,28 @@
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 24GB 2TB Space Black</t>
+          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 16GB 4TB Space Black</t>
         </is>
       </c>
       <c r="B48" t="n">
+        <v>14</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
         <v>16</v>
       </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>M5 Pro</t>
-        </is>
-      </c>
-      <c r="D48" t="n">
-        <v>24</v>
-      </c>
       <c r="E48" t="n">
-        <v>2048</v>
+        <v>4096</v>
       </c>
       <c r="F48" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="G48" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
@@ -4136,28 +4130,28 @@
         </is>
       </c>
       <c r="I48" s="3" t="n">
-        <v>1150000</v>
+        <v>1130000</v>
       </c>
       <c r="J48" s="3" t="n">
-        <v>1150000</v>
+        <v>1130000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1502996</v>
+        <v>1502138</v>
       </c>
       <c r="L48" t="n">
-        <v>23.48615698245371</v>
+        <v>24.77388895028286</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N48" t="n">
-        <v>0</v>
+        <v>1.739130434782609</v>
       </c>
       <c r="P48" t="n">
-        <v>6.617881005408838</v>
+        <v>88.39999999999999</v>
       </c>
       <c r="Q48" t="n">
-        <v>11.5</v>
+        <v>30.2</v>
       </c>
       <c r="R48" t="n">
         <v>3</v>
@@ -4268,10 +4262,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1760726</v>
+        <v>1759721</v>
       </c>
       <c r="L50" t="n">
-        <v>34.40205915060038</v>
+        <v>34.36459529664078</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4332,10 +4326,10 @@
         <v>1155000</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>1760726</v>
+        <v>1759721</v>
       </c>
       <c r="L51" t="n">
-        <v>34.40205915060038</v>
+        <v>34.36459529664078</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -4396,10 +4390,10 @@
         <v>1185000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1588906</v>
+        <v>1587999</v>
       </c>
       <c r="L52" t="n">
-        <v>25.42038358468028</v>
+        <v>25.37778676183046</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -4460,10 +4454,10 @@
         <v>1185000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1588906</v>
+        <v>1587999</v>
       </c>
       <c r="L53" t="n">
-        <v>25.42038358468028</v>
+        <v>25.37778676183046</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -4524,22 +4518,22 @@
         <v>1200000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1889591</v>
+        <v>1888512</v>
       </c>
       <c r="L54" t="n">
-        <v>36.49419371705305</v>
+        <v>36.45790971939813</v>
       </c>
       <c r="M54" s="3" t="n">
-        <v>-7000</v>
+        <v>0</v>
       </c>
       <c r="N54" t="n">
         <v>0.6622516556291391</v>
       </c>
       <c r="P54" t="n">
-        <v>11.02580898729203</v>
+        <v>3.948101568096777</v>
       </c>
       <c r="Q54" t="n">
-        <v>18.2</v>
+        <v>16.7</v>
       </c>
       <c r="R54" t="n">
         <v>3</v>
@@ -4588,22 +4582,22 @@
         <v>1200000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1889591</v>
+        <v>1888512</v>
       </c>
       <c r="L55" t="n">
-        <v>36.49419371705305</v>
+        <v>36.45790971939813</v>
       </c>
       <c r="M55" s="3" t="n">
-        <v>-7000</v>
+        <v>0</v>
       </c>
       <c r="N55" t="n">
         <v>0.8264462809917356</v>
       </c>
       <c r="P55" t="n">
-        <v>11.02580898729203</v>
+        <v>3.948101568096777</v>
       </c>
       <c r="Q55" t="n">
-        <v>18.3</v>
+        <v>16.8</v>
       </c>
       <c r="R55" t="n">
         <v>3</v>
@@ -4714,10 +4708,10 @@
         <v>1240000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1674816</v>
+        <v>1673860</v>
       </c>
       <c r="L57" t="n">
-        <v>25.96201612595056</v>
+        <v>25.91973044340626</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -4778,10 +4772,10 @@
         <v>1280000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>1717771</v>
+        <v>1716790</v>
       </c>
       <c r="L58" t="n">
-        <v>25.48482888580608</v>
+        <v>25.44224978011288</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -4810,7 +4804,7 @@
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 64GB 1TB Silver</t>
+          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 48GB 2TB Silver</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -4822,10 +4816,10 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="E59" t="n">
-        <v>1024</v>
+        <v>2048</v>
       </c>
       <c r="F59" t="n">
         <v>18</v>
@@ -4839,28 +4833,28 @@
         </is>
       </c>
       <c r="I59" s="3" t="n">
-        <v>1310000</v>
+        <v>1298000</v>
       </c>
       <c r="J59" s="3" t="n">
-        <v>1310000</v>
+        <v>1298000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1717771</v>
+        <v>1759721</v>
       </c>
       <c r="L59" t="n">
-        <v>23.73837956281716</v>
+        <v>26.23830709527249</v>
       </c>
       <c r="M59" s="3" t="n">
-        <v>0</v>
+        <v>-40000</v>
       </c>
       <c r="N59" t="n">
-        <v>0</v>
+        <v>2.989536621823617</v>
       </c>
       <c r="P59" t="n">
-        <v>65.92427616926503</v>
+        <v>62.21254466180763</v>
       </c>
       <c r="Q59" t="n">
-        <v>24.3</v>
+        <v>25.6</v>
       </c>
       <c r="R59" t="n">
         <v>3</v>
@@ -4874,11 +4868,11 @@
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Pro 18 Core CPU 20 Core GPU 24GB 4TB Space Black</t>
+          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 64GB 1TB Silver</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -4886,10 +4880,10 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>24</v>
+        <v>64</v>
       </c>
       <c r="E60" t="n">
-        <v>4096</v>
+        <v>1024</v>
       </c>
       <c r="F60" t="n">
         <v>18</v>
@@ -4899,30 +4893,35 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I60" s="3" t="n">
-        <v>1330000</v>
+        <v>1300000</v>
       </c>
       <c r="J60" s="3" t="n">
-        <v>1330000</v>
-      </c>
-      <c r="K60" s="3" t="n"/>
+        <v>1300000</v>
+      </c>
+      <c r="K60" s="3" t="n">
+        <v>1716790</v>
+      </c>
+      <c r="L60" t="n">
+        <v>24.27728493292715</v>
+      </c>
       <c r="M60" s="3" t="n">
-        <v>0</v>
+        <v>-10000</v>
       </c>
       <c r="N60" t="n">
-        <v>3.623188405797102</v>
+        <v>0.7633587786259541</v>
       </c>
       <c r="P60" t="n">
-        <v>73.97047397047398</v>
+        <v>61.86882704645171</v>
       </c>
       <c r="Q60" t="n">
-        <v>30</v>
+        <v>23.9</v>
       </c>
       <c r="R60" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S60" t="inlineStr">
         <is>
@@ -4933,7 +4932,7 @@
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Pro 18 Core CPU 20 Core GPU 64GB 2TB Space Black</t>
+          <t>Macbook Pro 14 CTO M5 Pro 18 Core CPU 20 Core GPU 24GB 4TB Space Black</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -4945,10 +4944,10 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>64</v>
+        <v>24</v>
       </c>
       <c r="E61" t="n">
-        <v>2048</v>
+        <v>4096</v>
       </c>
       <c r="F61" t="n">
         <v>18</v>
@@ -4962,31 +4961,26 @@
         </is>
       </c>
       <c r="I61" s="3" t="n">
-        <v>1335000</v>
+        <v>1330000</v>
       </c>
       <c r="J61" s="3" t="n">
-        <v>1335000</v>
-      </c>
-      <c r="K61" s="3" t="n">
-        <v>1803681</v>
-      </c>
-      <c r="L61" t="n">
-        <v>25.98469463280924</v>
-      </c>
+        <v>1330000</v>
+      </c>
+      <c r="K61" s="3" t="n"/>
       <c r="M61" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N61" t="n">
-        <v>2.554744525547445</v>
+        <v>3.623188405797102</v>
       </c>
       <c r="P61" t="n">
-        <v>87.17948717948718</v>
+        <v>73.97047397047398</v>
       </c>
       <c r="Q61" t="n">
-        <v>30.7</v>
+        <v>30</v>
       </c>
       <c r="R61" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S61" t="inlineStr">
         <is>
@@ -4997,11 +4991,11 @@
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 48GB 2TB Silver</t>
+          <t>Macbook Pro 14 CTO M5 Pro 18 Core CPU 20 Core GPU 64GB 2TB Space Black</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -5009,7 +5003,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>48</v>
+        <v>64</v>
       </c>
       <c r="E62" t="n">
         <v>2048</v>
@@ -5022,32 +5016,32 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I62" s="3" t="n">
-        <v>1338000</v>
+        <v>1335000</v>
       </c>
       <c r="J62" s="3" t="n">
-        <v>1338000</v>
+        <v>1335000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1760726</v>
+        <v>1802651</v>
       </c>
       <c r="L62" t="n">
-        <v>24.00861917186434</v>
+        <v>25.9424037154169</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N62" t="n">
-        <v>0</v>
+        <v>2.554744525547445</v>
       </c>
       <c r="P62" t="n">
-        <v>60.93541202672606</v>
+        <v>87.17948717948718</v>
       </c>
       <c r="Q62" t="n">
-        <v>23.3</v>
+        <v>30.7</v>
       </c>
       <c r="R62" t="n">
         <v>3</v>
@@ -5061,11 +5055,11 @@
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 48GB 4TB Space Black</t>
+          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 64GB 2TB Silver</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -5073,43 +5067,45 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>48</v>
+        <v>64</v>
       </c>
       <c r="E63" t="n">
-        <v>4096</v>
+        <v>2048</v>
       </c>
       <c r="F63" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G63" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I63" s="3" t="n">
-        <v>1445000</v>
+        <v>1420000</v>
       </c>
       <c r="J63" s="3" t="n">
-        <v>1445000</v>
-      </c>
-      <c r="K63" s="3" t="n"/>
+        <v>1420000</v>
+      </c>
+      <c r="K63" s="3" t="n">
+        <v>1931442</v>
+      </c>
+      <c r="L63" t="n">
+        <v>26.47980110197459</v>
+      </c>
       <c r="M63" s="3" t="n">
-        <v>0</v>
+        <v>-51000</v>
       </c>
       <c r="N63" t="n">
-        <v>3.02013422818792</v>
-      </c>
-      <c r="O63" t="n">
-        <v>100</v>
+        <v>3.467029231815092</v>
       </c>
       <c r="P63" t="n">
-        <v>98.16849816849818</v>
+        <v>81.91902127554754</v>
       </c>
       <c r="Q63" t="n">
-        <v>59.1</v>
+        <v>30.1</v>
       </c>
       <c r="R63" t="n">
         <v>3</v>
@@ -5123,7 +5119,7 @@
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 MGE94 M5 Max 18 Core CPU 40 Core GPU 48GB 2TB Silver</t>
+          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 24GB 4TB Space Black</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -5131,49 +5127,49 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>M5 Max</t>
+          <t>M5 Pro</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="E64" t="n">
-        <v>2048</v>
+        <v>4096</v>
       </c>
       <c r="F64" t="n">
         <v>18</v>
       </c>
       <c r="G64" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I64" s="3" t="n">
-        <v>1450000</v>
+        <v>1430000</v>
       </c>
       <c r="J64" s="3" t="n">
-        <v>1450000</v>
+        <v>1430000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>2147321</v>
+        <v>1931442</v>
       </c>
       <c r="L64" t="n">
-        <v>32.47399899688961</v>
+        <v>25.96205322241103</v>
       </c>
       <c r="M64" s="3" t="n">
-        <v>-10000</v>
+        <v>-41000</v>
       </c>
       <c r="N64" t="n">
-        <v>0</v>
+        <v>2.787219578518015</v>
       </c>
       <c r="P64" t="n">
-        <v>2.850779510022292</v>
+        <v>61.86882704645171</v>
       </c>
       <c r="Q64" t="n">
-        <v>14.5</v>
+        <v>25.4</v>
       </c>
       <c r="R64" t="n">
         <v>3</v>
@@ -5187,7 +5183,7 @@
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 MGEE4 M5 Max 18 Core CPU 40 Core GPU 48GB 2TB Space Black</t>
+          <t>Macbook Pro 16 MGE94 M5 Max 18 Core CPU 40 Core GPU 48GB 2TB Silver</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -5212,32 +5208,32 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I65" s="3" t="n">
-        <v>1450000</v>
+        <v>1430000</v>
       </c>
       <c r="J65" s="3" t="n">
-        <v>1450000</v>
+        <v>1430000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>2147321</v>
+        <v>2146095</v>
       </c>
       <c r="L65" t="n">
-        <v>32.47399899688961</v>
+        <v>33.36734860292764</v>
       </c>
       <c r="M65" s="3" t="n">
-        <v>-10000</v>
+        <v>-20000</v>
       </c>
       <c r="N65" t="n">
         <v>0</v>
       </c>
       <c r="P65" t="n">
-        <v>2.850779510022292</v>
+        <v>0</v>
       </c>
       <c r="Q65" t="n">
-        <v>14.5</v>
+        <v>14.3</v>
       </c>
       <c r="R65" t="n">
         <v>3</v>
@@ -5251,7 +5247,7 @@
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 64GB 2TB Silver</t>
+          <t>Macbook Pro 16 MGEE4 M5 Max 18 Core CPU 40 Core GPU 48GB 2TB Space Black</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -5259,11 +5255,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>M5 Pro</t>
+          <t>M5 Max</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="E66" t="n">
         <v>2048</v>
@@ -5272,36 +5268,36 @@
         <v>18</v>
       </c>
       <c r="G66" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I66" s="3" t="n">
-        <v>1471000</v>
+        <v>1430000</v>
       </c>
       <c r="J66" s="3" t="n">
-        <v>1471000</v>
+        <v>1430000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1932546</v>
+        <v>2146095</v>
       </c>
       <c r="L66" t="n">
-        <v>23.88279502790619</v>
+        <v>33.36734860292764</v>
       </c>
       <c r="M66" s="3" t="n">
-        <v>0</v>
+        <v>-20000</v>
       </c>
       <c r="N66" t="n">
         <v>0</v>
       </c>
       <c r="P66" t="n">
-        <v>80.92056421677803</v>
+        <v>0</v>
       </c>
       <c r="Q66" t="n">
-        <v>27.6</v>
+        <v>14.3</v>
       </c>
       <c r="R66" t="n">
         <v>3</v>
@@ -5315,11 +5311,11 @@
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 24GB 4TB Space Black</t>
+          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 48GB 4TB Space Black</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -5327,16 +5323,16 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="E67" t="n">
         <v>4096</v>
       </c>
       <c r="F67" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G67" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
@@ -5344,28 +5340,26 @@
         </is>
       </c>
       <c r="I67" s="3" t="n">
-        <v>1471000</v>
+        <v>1445000</v>
       </c>
       <c r="J67" s="3" t="n">
-        <v>1471000</v>
-      </c>
-      <c r="K67" s="3" t="n">
-        <v>1932546</v>
-      </c>
-      <c r="L67" t="n">
-        <v>23.88279502790619</v>
-      </c>
+        <v>1445000</v>
+      </c>
+      <c r="K67" s="3" t="n"/>
       <c r="M67" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N67" t="n">
-        <v>0</v>
+        <v>3.02013422818792</v>
+      </c>
+      <c r="O67" t="n">
+        <v>100</v>
       </c>
       <c r="P67" t="n">
-        <v>61.06499291354523</v>
+        <v>98.16849816849818</v>
       </c>
       <c r="Q67" t="n">
-        <v>23.3</v>
+        <v>59.1</v>
       </c>
       <c r="R67" t="n">
         <v>3</v>
@@ -5414,10 +5408,10 @@
         <v>1480000</v>
       </c>
       <c r="K68" s="3" t="n">
-        <v>2018456</v>
+        <v>2017303</v>
       </c>
       <c r="L68" t="n">
-        <v>26.67662807611362</v>
+        <v>26.63471972232233</v>
       </c>
       <c r="M68" s="3" t="n">
         <v>0</v>
@@ -5540,10 +5534,10 @@
         <v>1605000</v>
       </c>
       <c r="K70" s="3" t="n">
-        <v>2190276</v>
+        <v>2189025</v>
       </c>
       <c r="L70" t="n">
-        <v>26.7215638577056</v>
+        <v>26.67968616164731</v>
       </c>
       <c r="M70" s="3" t="n">
         <v>0</v>
@@ -5604,10 +5598,10 @@
         <v>1610000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2190276</v>
+        <v>2189025</v>
       </c>
       <c r="L71" t="n">
-        <v>26.49328212517509</v>
+        <v>26.45127396900446</v>
       </c>
       <c r="M71" s="3" t="n">
         <v>0</v>
@@ -5633,11 +5627,11 @@
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Pro 18 Core CPU 20 Core GPU 64GB 4TB Space Black</t>
+          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 48GB 4TB Silver</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -5645,7 +5639,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="E72" t="n">
         <v>4096</v>
@@ -5658,32 +5652,32 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I72" s="3" t="n">
-        <v>1630000</v>
+        <v>1615000</v>
       </c>
       <c r="J72" s="3" t="n">
-        <v>1630000</v>
+        <v>1615000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2233231</v>
+        <v>2189025</v>
       </c>
       <c r="L72" t="n">
-        <v>27.011580978412</v>
+        <v>26.22286177636162</v>
       </c>
       <c r="M72" s="3" t="n">
-        <v>0</v>
+        <v>-46000</v>
       </c>
       <c r="N72" t="n">
-        <v>2.976190476190476</v>
+        <v>2.769416014449127</v>
       </c>
       <c r="P72" t="n">
-        <v>100</v>
+        <v>87.03386674215359</v>
       </c>
       <c r="Q72" t="n">
-        <v>34.1</v>
+        <v>30.9</v>
       </c>
       <c r="R72" t="n">
         <v>3</v>
@@ -5697,11 +5691,11 @@
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 48GB 4TB Silver</t>
+          <t>Macbook Pro 14 CTO M5 Pro 18 Core CPU 20 Core GPU 64GB 4TB Space Black</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -5709,7 +5703,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>48</v>
+        <v>64</v>
       </c>
       <c r="E73" t="n">
         <v>4096</v>
@@ -5722,32 +5716,32 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I73" s="3" t="n">
-        <v>1661000</v>
+        <v>1630000</v>
       </c>
       <c r="J73" s="3" t="n">
-        <v>1661000</v>
+        <v>1630000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2190276</v>
+        <v>2231956</v>
       </c>
       <c r="L73" t="n">
-        <v>24.16480845336387</v>
+        <v>26.96988650313895</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N73" t="n">
-        <v>0</v>
+        <v>2.976190476190476</v>
       </c>
       <c r="P73" t="n">
-        <v>87.94145720649061</v>
+        <v>100</v>
       </c>
       <c r="Q73" t="n">
-        <v>29.2</v>
+        <v>34.1</v>
       </c>
       <c r="R73" t="n">
         <v>3</v>
@@ -5790,28 +5784,28 @@
         </is>
       </c>
       <c r="I74" s="3" t="n">
-        <v>1711000</v>
+        <v>1690000</v>
       </c>
       <c r="J74" s="3" t="n">
-        <v>1711000</v>
+        <v>1690000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2319141</v>
+        <v>2317817</v>
       </c>
       <c r="L74" t="n">
-        <v>26.2226833124851</v>
+        <v>27.08656464250629</v>
       </c>
       <c r="M74" s="3" t="n">
-        <v>0</v>
+        <v>-21000</v>
       </c>
       <c r="N74" t="n">
-        <v>0</v>
+        <v>1.227352425482174</v>
       </c>
       <c r="P74" t="n">
-        <v>20.21202672605792</v>
+        <v>16.88768606224628</v>
       </c>
       <c r="Q74" t="n">
-        <v>15.6</v>
+        <v>15.7</v>
       </c>
       <c r="R74" t="n">
         <v>3</v>
@@ -5854,28 +5848,28 @@
         </is>
       </c>
       <c r="I75" s="3" t="n">
-        <v>1756000</v>
+        <v>1705000</v>
       </c>
       <c r="J75" s="3" t="n">
-        <v>1756000</v>
+        <v>1705000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2319141</v>
+        <v>2317817</v>
       </c>
       <c r="L75" t="n">
-        <v>24.28230970001393</v>
+        <v>26.4394039736528</v>
       </c>
       <c r="M75" s="3" t="n">
-        <v>0</v>
+        <v>-51000</v>
       </c>
       <c r="N75" t="n">
-        <v>0</v>
+        <v>2.904328018223234</v>
       </c>
       <c r="P75" t="n">
-        <v>0</v>
+        <v>1.9846639603067</v>
       </c>
       <c r="Q75" t="n">
-        <v>10.4</v>
+        <v>12.8</v>
       </c>
       <c r="R75" t="n">
         <v>3</v>
@@ -5889,19 +5883,19 @@
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Max 18 Core CPU 40 Core GPU 48GB 4TB Silver</t>
+          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 64GB 4TB Silver</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>M5 Max</t>
+          <t>M5 Pro</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>48</v>
+        <v>64</v>
       </c>
       <c r="E76" t="n">
         <v>4096</v>
@@ -5910,7 +5904,7 @@
         <v>18</v>
       </c>
       <c r="G76" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
@@ -5918,28 +5912,28 @@
         </is>
       </c>
       <c r="I76" s="3" t="n">
-        <v>1780000</v>
+        <v>1725000</v>
       </c>
       <c r="J76" s="3" t="n">
-        <v>1780000</v>
+        <v>1725000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2448006</v>
+        <v>2360747</v>
       </c>
       <c r="L76" t="n">
-        <v>27.28775991562112</v>
+        <v>26.92990820278496</v>
       </c>
       <c r="M76" s="3" t="n">
-        <v>0</v>
+        <v>-65000</v>
       </c>
       <c r="N76" t="n">
-        <v>3.260869565217391</v>
+        <v>3.631284916201118</v>
       </c>
       <c r="P76" t="n">
-        <v>38.78143936249688</v>
+        <v>100</v>
       </c>
       <c r="Q76" t="n">
-        <v>21.2</v>
+        <v>34.3</v>
       </c>
       <c r="R76" t="n">
         <v>3</v>
@@ -5953,19 +5947,19 @@
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 64GB 4TB Silver</t>
+          <t>Macbook Pro 14 CTO M5 Max 18 Core CPU 40 Core GPU 48GB 4TB Silver</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>M5 Pro</t>
+          <t>M5 Max</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="E77" t="n">
         <v>4096</v>
@@ -5974,7 +5968,7 @@
         <v>18</v>
       </c>
       <c r="G77" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
@@ -5982,28 +5976,28 @@
         </is>
       </c>
       <c r="I77" s="3" t="n">
-        <v>1790000</v>
+        <v>1780000</v>
       </c>
       <c r="J77" s="3" t="n">
-        <v>1790000</v>
+        <v>1780000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2362096</v>
+        <v>2446608</v>
       </c>
       <c r="L77" t="n">
-        <v>24.21984542541878</v>
+        <v>27.24621189826895</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N77" t="n">
-        <v>0</v>
+        <v>3.260869565217391</v>
       </c>
       <c r="P77" t="n">
-        <v>100</v>
+        <v>38.78143936249688</v>
       </c>
       <c r="Q77" t="n">
-        <v>31.8</v>
+        <v>21.2</v>
       </c>
       <c r="R77" t="n">
         <v>3</v>
@@ -6017,11 +6011,11 @@
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Max 18 Core CPU 40 Core GPU 64GB 4TB Silver</t>
+          <t>Macbook Pro 16 CTO M5 Max 18 Core CPU 40 Core GPU 48GB 4TB Space Black</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -6029,7 +6023,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="E78" t="n">
         <v>4096</v>
@@ -6046,28 +6040,28 @@
         </is>
       </c>
       <c r="I78" s="3" t="n">
-        <v>1910000</v>
+        <v>1875000</v>
       </c>
       <c r="J78" s="3" t="n">
-        <v>1910000</v>
+        <v>1875000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2619826</v>
+        <v>2575400</v>
       </c>
       <c r="L78" t="n">
-        <v>27.09439481858719</v>
+        <v>27.19577541352799</v>
       </c>
       <c r="M78" s="3" t="n">
-        <v>0</v>
+        <v>-70000</v>
       </c>
       <c r="N78" t="n">
-        <v>2.551020408163265</v>
+        <v>3.598971722365039</v>
       </c>
       <c r="P78" t="n">
-        <v>53.22486926205694</v>
+        <v>19.64044075004835</v>
       </c>
       <c r="Q78" t="n">
-        <v>23.9</v>
+        <v>17.1</v>
       </c>
       <c r="R78" t="n">
         <v>3</v>
@@ -6081,11 +6075,11 @@
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 CTO M5 Max 18 Core CPU 40 Core GPU 48GB 4TB Space Black</t>
+          <t>Macbook Pro 14 CTO M5 Max 18 Core CPU 40 Core GPU 64GB 4TB Silver</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -6093,7 +6087,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>48</v>
+        <v>64</v>
       </c>
       <c r="E79" t="n">
         <v>4096</v>
@@ -6110,28 +6104,28 @@
         </is>
       </c>
       <c r="I79" s="3" t="n">
-        <v>1945000</v>
+        <v>1910000</v>
       </c>
       <c r="J79" s="3" t="n">
-        <v>1945000</v>
+        <v>1910000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2576871</v>
+        <v>2618330</v>
       </c>
       <c r="L79" t="n">
-        <v>24.52086270519557</v>
+        <v>27.05273972341149</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N79" t="n">
-        <v>0</v>
+        <v>2.551020408163265</v>
       </c>
       <c r="P79" t="n">
-        <v>15.83200763601658</v>
+        <v>53.22486926205694</v>
       </c>
       <c r="Q79" t="n">
-        <v>13.9</v>
+        <v>23.9</v>
       </c>
       <c r="R79" t="n">
         <v>3</v>
@@ -6174,28 +6168,28 @@
         </is>
       </c>
       <c r="I80" s="3" t="n">
-        <v>2078000</v>
+        <v>2020000</v>
       </c>
       <c r="J80" s="3" t="n">
-        <v>2078000</v>
+        <v>2020000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2748691</v>
+        <v>2747122</v>
       </c>
       <c r="L80" t="n">
-        <v>24.40037821639464</v>
+        <v>26.46850048887527</v>
       </c>
       <c r="M80" s="3" t="n">
-        <v>0</v>
+        <v>-58000</v>
       </c>
       <c r="N80" t="n">
-        <v>0</v>
+        <v>2.791145332050048</v>
       </c>
       <c r="P80" t="n">
-        <v>35.18930957683743</v>
+        <v>36.26522327469554</v>
       </c>
       <c r="Q80" t="n">
-        <v>18</v>
+        <v>20.1</v>
       </c>
       <c r="R80" t="n">
         <v>3</v>
@@ -6244,10 +6238,10 @@
         <v>2110000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2877556</v>
+        <v>2875913</v>
       </c>
       <c r="L81" t="n">
-        <v>26.6738857558289</v>
+        <v>26.63199477870158</v>
       </c>
       <c r="M81" s="3" t="n">
         <v>0</v>
@@ -6259,7 +6253,7 @@
         <v>79.02382335851249</v>
       </c>
       <c r="Q81" t="n">
-        <v>29.4</v>
+        <v>29.3</v>
       </c>
       <c r="R81" t="n">
         <v>3</v>
@@ -6273,11 +6267,11 @@
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Max 18 Core CPU 32 Core GPU 36GB 8TB Silver</t>
+          <t>Apple MacBook Pro 16 M5 Max 18 Core CPU 40 Core GPU 128GB 2TB Silver</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -6285,45 +6279,45 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>36</v>
+        <v>128</v>
       </c>
       <c r="E82" t="n">
-        <v>8192</v>
+        <v>2048</v>
       </c>
       <c r="F82" t="n">
         <v>18</v>
       </c>
       <c r="G82" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I82" s="3" t="n">
-        <v>2215000</v>
+        <v>2210000</v>
       </c>
       <c r="J82" s="3" t="n">
-        <v>2215000</v>
+        <v>2210000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>3049376</v>
+        <v>3004705</v>
       </c>
       <c r="L82" t="n">
-        <v>27.36218819850356</v>
+        <v>26.44868631030334</v>
       </c>
       <c r="M82" s="3" t="n">
-        <v>0</v>
+        <v>-58000</v>
       </c>
       <c r="N82" t="n">
-        <v>2.422907488986784</v>
+        <v>2.55731922398589</v>
       </c>
       <c r="P82" t="n">
-        <v>74.28466149856153</v>
+        <v>70.36535859269283</v>
       </c>
       <c r="Q82" t="n">
-        <v>28.5</v>
+        <v>27.3</v>
       </c>
       <c r="R82" t="n">
         <v>3</v>
@@ -6337,11 +6331,11 @@
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 16 M5 Max 18 Core CPU 40 Core GPU 128GB 2TB Silver</t>
+          <t>Macbook Pro 14 CTO M5 Max 18 Core CPU 32 Core GPU 36GB 8TB Silver</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -6349,45 +6343,45 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>128</v>
+        <v>36</v>
       </c>
       <c r="E83" t="n">
-        <v>2048</v>
+        <v>8192</v>
       </c>
       <c r="F83" t="n">
         <v>18</v>
       </c>
       <c r="G83" t="n">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I83" s="3" t="n">
-        <v>2268000</v>
+        <v>2215000</v>
       </c>
       <c r="J83" s="3" t="n">
-        <v>2268000</v>
+        <v>2215000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3006421</v>
+        <v>3047635</v>
       </c>
       <c r="L83" t="n">
-        <v>24.56146361404474</v>
+        <v>27.32069293074794</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N83" t="n">
-        <v>0</v>
+        <v>2.422907488986784</v>
       </c>
       <c r="P83" t="n">
-        <v>70.41425389755011</v>
+        <v>74.28466149856153</v>
       </c>
       <c r="Q83" t="n">
-        <v>25.6</v>
+        <v>28.5</v>
       </c>
       <c r="R83" t="n">
         <v>3</v>
@@ -6430,28 +6424,28 @@
         </is>
       </c>
       <c r="I84" s="3" t="n">
-        <v>2381000</v>
+        <v>2315000</v>
       </c>
       <c r="J84" s="3" t="n">
-        <v>2381000</v>
+        <v>2315000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3178241</v>
+        <v>3176426</v>
       </c>
       <c r="L84" t="n">
-        <v>25.08434697054125</v>
+        <v>27.11934734194972</v>
       </c>
       <c r="M84" s="3" t="n">
-        <v>0</v>
+        <v>-66000</v>
       </c>
       <c r="N84" t="n">
-        <v>0</v>
+        <v>2.771944561108778</v>
       </c>
       <c r="P84" t="n">
-        <v>64.54234341897987</v>
+        <v>65.11105977094954</v>
       </c>
       <c r="Q84" t="n">
-        <v>24.6</v>
+        <v>26.6</v>
       </c>
       <c r="R84" t="n">
         <v>3</v>
@@ -6500,10 +6494,10 @@
         <v>2395000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3307106</v>
+        <v>3305218</v>
       </c>
       <c r="L85" t="n">
-        <v>27.58018642281197</v>
+        <v>27.53881892208018</v>
       </c>
       <c r="M85" s="3" t="n">
         <v>0</v>
@@ -6564,10 +6558,10 @@
         <v>2410000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3307106</v>
+        <v>3305218</v>
       </c>
       <c r="L86" t="n">
-        <v>27.12661765301747</v>
+        <v>27.08499106564227</v>
       </c>
       <c r="M86" s="3" t="n">
         <v>0</v>
@@ -6579,7 +6573,7 @@
         <v>88.47569242688358</v>
       </c>
       <c r="Q86" t="n">
-        <v>31.5</v>
+        <v>31.4</v>
       </c>
       <c r="R86" t="n">
         <v>3</v>
@@ -6593,11 +6587,11 @@
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Max 18 Core CPU 40 Core GPU 64GB 8TB Silver</t>
+          <t>Macbook Pro 16 CTO M5 Max 18 Core CPU 40 Core GPU 48GB 8TB Space Black</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -6605,7 +6599,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="E87" t="n">
         <v>8192</v>
@@ -6622,28 +6616,28 @@
         </is>
       </c>
       <c r="I87" s="3" t="n">
-        <v>2530000</v>
+        <v>2499000</v>
       </c>
       <c r="J87" s="3" t="n">
-        <v>2530000</v>
+        <v>2499000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3478926</v>
+        <v>3434009</v>
       </c>
       <c r="L87" t="n">
-        <v>27.27640656915382</v>
+        <v>27.22791349702345</v>
       </c>
       <c r="M87" s="3" t="n">
-        <v>0</v>
+        <v>-82000</v>
       </c>
       <c r="N87" t="n">
-        <v>1.937984496124031</v>
+        <v>3.17706315381635</v>
       </c>
       <c r="P87" t="n">
-        <v>79.17877203176447</v>
+        <v>63.67326854471646</v>
       </c>
       <c r="Q87" t="n">
-        <v>29.3</v>
+        <v>26.4</v>
       </c>
       <c r="R87" t="n">
         <v>3</v>
@@ -6686,28 +6680,28 @@
         </is>
       </c>
       <c r="I88" s="3" t="n">
-        <v>2571000</v>
+        <v>2510000</v>
       </c>
       <c r="J88" s="3" t="n">
-        <v>2571000</v>
+        <v>2510000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3435971</v>
+        <v>3434009</v>
       </c>
       <c r="L88" t="n">
-        <v>25.17399011807725</v>
+        <v>26.90758818628606</v>
       </c>
       <c r="M88" s="3" t="n">
-        <v>0</v>
+        <v>-61000</v>
       </c>
       <c r="N88" t="n">
-        <v>0</v>
+        <v>2.372617658498639</v>
       </c>
       <c r="P88" t="n">
-        <v>83.83073496659243</v>
+        <v>83.17546233649077</v>
       </c>
       <c r="Q88" t="n">
-        <v>28.8</v>
+        <v>30.2</v>
       </c>
       <c r="R88" t="n">
         <v>3</v>
@@ -6721,11 +6715,11 @@
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 CTO M5 Max 18 Core CPU 40 Core GPU 48GB 8TB Space Black</t>
+          <t>Macbook Pro 14 CTO M5 Max 18 Core CPU 40 Core GPU 64GB 8TB Silver</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -6733,7 +6727,7 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>48</v>
+        <v>64</v>
       </c>
       <c r="E89" t="n">
         <v>8192</v>
@@ -6750,28 +6744,28 @@
         </is>
       </c>
       <c r="I89" s="3" t="n">
-        <v>2581000</v>
+        <v>2530000</v>
       </c>
       <c r="J89" s="3" t="n">
-        <v>2581000</v>
+        <v>2530000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3435971</v>
+        <v>3476940</v>
       </c>
       <c r="L89" t="n">
-        <v>24.88295157322341</v>
+        <v>27.23486744091069</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N89" t="n">
-        <v>0</v>
+        <v>1.937984496124031</v>
       </c>
       <c r="P89" t="n">
-        <v>62.0368495646892</v>
+        <v>79.17877203176447</v>
       </c>
       <c r="Q89" t="n">
-        <v>24</v>
+        <v>29.3</v>
       </c>
       <c r="R89" t="n">
         <v>3</v>
@@ -6814,28 +6808,28 @@
         </is>
       </c>
       <c r="I90" s="3" t="n">
-        <v>2664000</v>
+        <v>2610000</v>
       </c>
       <c r="J90" s="3" t="n">
-        <v>2664000</v>
+        <v>2610000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3607791</v>
+        <v>3605731</v>
       </c>
       <c r="L90" t="n">
-        <v>26.15980249410235</v>
+        <v>27.61523252843875</v>
       </c>
       <c r="M90" s="3" t="n">
-        <v>0</v>
+        <v>-54000</v>
       </c>
       <c r="N90" t="n">
-        <v>0</v>
+        <v>2.027027027027027</v>
       </c>
       <c r="P90" t="n">
-        <v>75.54565701559021</v>
+        <v>74.15426251691474</v>
       </c>
       <c r="Q90" t="n">
-        <v>27.4</v>
+        <v>28.4</v>
       </c>
       <c r="R90" t="n">
         <v>3</v>
@@ -6884,10 +6878,10 @@
         <v>3015000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>4166206</v>
+        <v>4163828</v>
       </c>
       <c r="L91" t="n">
-        <v>27.63199899380875</v>
+        <v>27.59066897095653</v>
       </c>
       <c r="M91" s="3" t="n">
         <v>0</v>
@@ -6942,28 +6936,28 @@
         </is>
       </c>
       <c r="I92" s="3" t="n">
-        <v>3186000</v>
+        <v>3098000</v>
       </c>
       <c r="J92" s="3" t="n">
-        <v>3186000</v>
+        <v>3098000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4295071</v>
+        <v>4292619</v>
       </c>
       <c r="L92" t="n">
-        <v>25.82194799573744</v>
+        <v>27.82960705340958</v>
       </c>
       <c r="M92" s="3" t="n">
-        <v>0</v>
+        <v>-88000</v>
       </c>
       <c r="N92" t="n">
-        <v>0</v>
+        <v>2.762084118016321</v>
       </c>
       <c r="P92" t="n">
         <v>100</v>
       </c>
       <c r="Q92" t="n">
-        <v>32.5</v>
+        <v>34.3</v>
       </c>
       <c r="R92" t="n">
         <v>3</v>
@@ -7246,10 +7240,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>429121</v>
+        <v>428876</v>
       </c>
       <c r="L2" t="n">
-        <v>27.75953635454802</v>
+        <v>27.71826821738684</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7313,10 +7307,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>429121</v>
+        <v>428876</v>
       </c>
       <c r="L3" t="n">
-        <v>27.75953635454802</v>
+        <v>27.71826821738684</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7380,10 +7374,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>429121</v>
+        <v>428876</v>
       </c>
       <c r="L4" t="n">
-        <v>27.7593033200426</v>
+        <v>27.71803504975797</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7447,10 +7441,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>429121</v>
+        <v>428876</v>
       </c>
       <c r="L5" t="n">
-        <v>27.7593033200426</v>
+        <v>27.71803504975797</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7514,10 +7508,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>515031</v>
+        <v>514736</v>
       </c>
       <c r="L6" t="n">
-        <v>25.4413811984133</v>
+        <v>25.39865095893817</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7578,10 +7572,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>515031</v>
+        <v>514736</v>
       </c>
       <c r="L7" t="n">
-        <v>25.4413811984133</v>
+        <v>25.39865095893817</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7642,10 +7636,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>515031</v>
+        <v>514736</v>
       </c>
       <c r="L8" t="n">
-        <v>25.4413811984133</v>
+        <v>25.39865095893817</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7706,10 +7700,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>515031</v>
+        <v>514736</v>
       </c>
       <c r="L9" t="n">
-        <v>25.4413811984133</v>
+        <v>25.39865095893817</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7770,10 +7764,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>515031</v>
+        <v>514736</v>
       </c>
       <c r="L10" t="n">
-        <v>25.2472181286175</v>
+        <v>25.20437661247708</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7834,10 +7828,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>515031</v>
+        <v>514736</v>
       </c>
       <c r="L11" t="n">
-        <v>25.2472181286175</v>
+        <v>25.20437661247708</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7898,10 +7892,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>515031</v>
+        <v>514736</v>
       </c>
       <c r="L12" t="n">
-        <v>25.2472181286175</v>
+        <v>25.20437661247708</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -7962,10 +7956,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>515031</v>
+        <v>514736</v>
       </c>
       <c r="L13" t="n">
-        <v>25.2472181286175</v>
+        <v>25.20437661247708</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -8026,22 +8020,22 @@
         <v>425000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>557986</v>
+        <v>557667</v>
       </c>
       <c r="L14" t="n">
-        <v>23.83321445340923</v>
+        <v>23.78964507492823</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>5.133716816332179</v>
+        <v>4.494167402623376</v>
       </c>
       <c r="P14" t="n">
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>12</v>
+        <v>11.8</v>
       </c>
       <c r="R14" t="n">
         <v>3</v>
@@ -8090,10 +8084,10 @@
         <v>425000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>557986</v>
+        <v>557667</v>
       </c>
       <c r="L15" t="n">
-        <v>23.83321445340923</v>
+        <v>23.78964507492823</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0</v>
@@ -8154,10 +8148,10 @@
         <v>425000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>557986</v>
+        <v>557667</v>
       </c>
       <c r="L16" t="n">
-        <v>23.83321445340923</v>
+        <v>23.78964507492823</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -8218,10 +8212,10 @@
         <v>425000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>557986</v>
+        <v>557667</v>
       </c>
       <c r="L17" t="n">
-        <v>23.83321445340923</v>
+        <v>23.78964507492823</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -8282,10 +8276,10 @@
         <v>454000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>600941</v>
+        <v>600597</v>
       </c>
       <c r="L18" t="n">
-        <v>24.4518180653342</v>
+        <v>24.40854682923824</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -8346,10 +8340,10 @@
         <v>454000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>600941</v>
+        <v>600597</v>
       </c>
       <c r="L19" t="n">
-        <v>24.4518180653342</v>
+        <v>24.40854682923824</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -8410,10 +8404,10 @@
         <v>454000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>600941</v>
+        <v>600597</v>
       </c>
       <c r="L20" t="n">
-        <v>24.4518180653342</v>
+        <v>24.40854682923824</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -8474,10 +8468,10 @@
         <v>454000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>600941</v>
+        <v>600597</v>
       </c>
       <c r="L21" t="n">
-        <v>24.4518180653342</v>
+        <v>24.40854682923824</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -8538,10 +8532,10 @@
         <v>455000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>600941</v>
+        <v>600597</v>
       </c>
       <c r="L22" t="n">
-        <v>24.28541237825344</v>
+        <v>24.24204583106476</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -8602,10 +8596,10 @@
         <v>455000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>600941</v>
+        <v>600597</v>
       </c>
       <c r="L23" t="n">
-        <v>24.28541237825344</v>
+        <v>24.24204583106476</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -8666,10 +8660,10 @@
         <v>455000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>600941</v>
+        <v>600597</v>
       </c>
       <c r="L24" t="n">
-        <v>24.28541237825344</v>
+        <v>24.24204583106476</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -8730,10 +8724,10 @@
         <v>455000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>600941</v>
+        <v>600597</v>
       </c>
       <c r="L25" t="n">
-        <v>24.28541237825344</v>
+        <v>24.24204583106476</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -8794,10 +8788,10 @@
         <v>475000</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>686851</v>
+        <v>686458</v>
       </c>
       <c r="L26" t="n">
-        <v>30.8438074633363</v>
+        <v>30.80421526153093</v>
       </c>
       <c r="M26" s="3" t="n">
         <v>0</v>
@@ -8858,10 +8852,10 @@
         <v>475000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>686851</v>
+        <v>686458</v>
       </c>
       <c r="L27" t="n">
-        <v>30.8438074633363</v>
+        <v>30.80421526153093</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -8922,10 +8916,10 @@
         <v>475000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>686851</v>
+        <v>686458</v>
       </c>
       <c r="L28" t="n">
-        <v>30.8438074633363</v>
+        <v>30.80421526153093</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -8986,10 +8980,10 @@
         <v>475000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>686851</v>
+        <v>686458</v>
       </c>
       <c r="L29" t="n">
-        <v>30.8438074633363</v>
+        <v>30.80421526153093</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -9050,10 +9044,10 @@
         <v>479999</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>686851</v>
+        <v>686458</v>
       </c>
       <c r="L30" t="n">
-        <v>30.11599313388202</v>
+        <v>30.07598425540965</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -9114,10 +9108,10 @@
         <v>479999</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>686851</v>
+        <v>686458</v>
       </c>
       <c r="L31" t="n">
-        <v>30.11599313388202</v>
+        <v>30.07598425540965</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -9178,10 +9172,10 @@
         <v>479999</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>686851</v>
+        <v>686458</v>
       </c>
       <c r="L32" t="n">
-        <v>30.11599313388202</v>
+        <v>30.07598425540965</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -9242,10 +9236,10 @@
         <v>479999</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>686851</v>
+        <v>686458</v>
       </c>
       <c r="L33" t="n">
-        <v>30.11599313388202</v>
+        <v>30.07598425540965</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -9306,13 +9300,13 @@
         <v>479999</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>643896</v>
+        <v>643528</v>
       </c>
       <c r="L34" t="n">
-        <v>25.45395529712873</v>
+        <v>25.41132631369575</v>
       </c>
       <c r="M34" s="3" t="n">
-        <v>-3000</v>
+        <v>0</v>
       </c>
       <c r="N34" t="n">
         <v>0.6211192983836406</v>
@@ -9373,13 +9367,13 @@
         <v>479999</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>643896</v>
+        <v>643528</v>
       </c>
       <c r="L35" t="n">
-        <v>25.45395529712873</v>
+        <v>25.41132631369575</v>
       </c>
       <c r="M35" s="3" t="n">
-        <v>-3000</v>
+        <v>0</v>
       </c>
       <c r="N35" t="n">
         <v>0.6211192983836406</v>
@@ -9440,13 +9434,13 @@
         <v>479999</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>643896</v>
+        <v>643528</v>
       </c>
       <c r="L36" t="n">
-        <v>25.45395529712873</v>
+        <v>25.41132631369575</v>
       </c>
       <c r="M36" s="3" t="n">
-        <v>-3000</v>
+        <v>0</v>
       </c>
       <c r="N36" t="n">
         <v>0.6211192983836406</v>
@@ -9507,13 +9501,13 @@
         <v>484999</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>643896</v>
+        <v>643528</v>
       </c>
       <c r="L37" t="n">
-        <v>24.67743238038441</v>
+        <v>24.63435934411556</v>
       </c>
       <c r="M37" s="3" t="n">
-        <v>-1000</v>
+        <v>0</v>
       </c>
       <c r="N37" t="n">
         <v>2.020404040404041</v>
@@ -9574,10 +9568,10 @@
         <v>500000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>643896</v>
+        <v>643528</v>
       </c>
       <c r="L38" t="n">
-        <v>22.34770832556811</v>
+        <v>22.30330304198108</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -9638,10 +9632,10 @@
         <v>549999</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>772761</v>
+        <v>772319</v>
       </c>
       <c r="L39" t="n">
-        <v>28.82676532588989</v>
+        <v>28.78603271446125</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -9705,10 +9699,10 @@
         <v>549999</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>772761</v>
+        <v>772319</v>
       </c>
       <c r="L40" t="n">
-        <v>28.82676532588989</v>
+        <v>28.78603271446125</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -9772,10 +9766,10 @@
         <v>549999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>772761</v>
+        <v>772319</v>
       </c>
       <c r="L41" t="n">
-        <v>28.82676532588989</v>
+        <v>28.78603271446125</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
@@ -9839,10 +9833,10 @@
         <v>551999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>772761</v>
+        <v>772319</v>
       </c>
       <c r="L42" t="n">
-        <v>28.56795309287089</v>
+        <v>28.52707236258593</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -9906,10 +9900,10 @@
         <v>564999</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>772761</v>
+        <v>772319</v>
       </c>
       <c r="L43" t="n">
-        <v>26.88567357824735</v>
+        <v>26.84383007539631</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -9970,10 +9964,10 @@
         <v>564999</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>772761</v>
+        <v>772319</v>
       </c>
       <c r="L44" t="n">
-        <v>26.88567357824735</v>
+        <v>26.84383007539631</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -10034,10 +10028,10 @@
         <v>564999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>772761</v>
+        <v>772319</v>
       </c>
       <c r="L45" t="n">
-        <v>26.88567357824735</v>
+        <v>26.84383007539631</v>
       </c>
       <c r="M45" s="3" t="n">
         <v>0</v>
@@ -10098,10 +10092,10 @@
         <v>564999</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>772761</v>
+        <v>772319</v>
       </c>
       <c r="L46" t="n">
-        <v>26.88567357824735</v>
+        <v>26.84383007539631</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -10162,10 +10156,10 @@
         <v>585000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>729806</v>
+        <v>729389</v>
       </c>
       <c r="L47" t="n">
-        <v>19.84171135890908</v>
+        <v>19.79588395218464</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -10177,7 +10171,7 @@
         <v>23.56648951077459</v>
       </c>
       <c r="Q47" t="n">
-        <v>13.6</v>
+        <v>13.5</v>
       </c>
       <c r="R47" t="n">
         <v>3</v>
@@ -10226,10 +10220,10 @@
         <v>595000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>729806</v>
+        <v>729389</v>
       </c>
       <c r="L48" t="n">
-        <v>18.47148420265112</v>
+        <v>18.42487342145275</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -10290,10 +10284,10 @@
         <v>614999</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>858671</v>
+        <v>858180</v>
       </c>
       <c r="L49" t="n">
-        <v>28.37780709957597</v>
+        <v>28.33682910345149</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -10354,10 +10348,10 @@
         <v>614999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>858671</v>
+        <v>858180</v>
       </c>
       <c r="L50" t="n">
-        <v>28.37780709957597</v>
+        <v>28.33682910345149</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -10418,10 +10412,10 @@
         <v>614999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>858671</v>
+        <v>858180</v>
       </c>
       <c r="L51" t="n">
-        <v>28.37780709957597</v>
+        <v>28.33682910345149</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -10482,10 +10476,10 @@
         <v>614999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>858671</v>
+        <v>858180</v>
       </c>
       <c r="L52" t="n">
-        <v>28.37780709957597</v>
+        <v>28.33682910345149</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -10546,10 +10540,10 @@
         <v>650000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>815716</v>
+        <v>815250</v>
       </c>
       <c r="L53" t="n">
-        <v>20.31540389056976</v>
+        <v>20.26985587243177</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -10610,10 +10604,10 @@
         <v>672000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>858671</v>
+        <v>858180</v>
       </c>
       <c r="L54" t="n">
-        <v>21.73952538282998</v>
+        <v>21.69474935328253</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -10674,10 +10668,10 @@
         <v>700000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>901626</v>
+        <v>901111</v>
       </c>
       <c r="L55" t="n">
-        <v>22.36248732844883</v>
+        <v>22.31811619212284</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -10738,10 +10732,10 @@
         <v>715000</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>944581</v>
+        <v>944041</v>
       </c>
       <c r="L56" t="n">
-        <v>24.30506224452958</v>
+        <v>24.26176405473915</v>
       </c>
       <c r="M56" s="3" t="n">
         <v>0</v>
@@ -10802,10 +10796,10 @@
         <v>734999</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>987536</v>
+        <v>986972</v>
       </c>
       <c r="L57" t="n">
-        <v>25.57243482769236</v>
+        <v>25.52990358389093</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -10866,10 +10860,10 @@
         <v>752000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>987536</v>
+        <v>986972</v>
       </c>
       <c r="L58" t="n">
-        <v>23.85087733510474</v>
+        <v>23.80736231625619</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -10930,10 +10924,10 @@
         <v>810000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1073446</v>
+        <v>1072833</v>
       </c>
       <c r="L59" t="n">
-        <v>24.54208222863563</v>
+        <v>24.49896675437836</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -10994,10 +10988,10 @@
         <v>815000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1073446</v>
+        <v>1072833</v>
       </c>
       <c r="L60" t="n">
-        <v>24.07629261276301</v>
+        <v>24.03291099360292</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -11058,10 +11052,10 @@
         <v>875000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1159356</v>
+        <v>1158694</v>
       </c>
       <c r="L61" t="n">
-        <v>24.52706502575568</v>
+        <v>24.48394485515589</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -11122,10 +11116,10 @@
         <v>992000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1331176</v>
+        <v>1330416</v>
       </c>
       <c r="L62" t="n">
-        <v>25.47942571080008</v>
+        <v>25.43685584057919</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -11186,10 +11180,10 @@
         <v>1050000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1417086</v>
+        <v>1416277</v>
       </c>
       <c r="L63" t="n">
-        <v>25.90428527273574</v>
+        <v>25.86196061928564</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -11250,10 +11244,10 @@
         <v>1050000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1417086</v>
+        <v>1416277</v>
       </c>
       <c r="L64" t="n">
-        <v>25.90428527273574</v>
+        <v>25.86196061928564</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -11265,7 +11259,7 @@
         <v>86.62413566438555</v>
       </c>
       <c r="Q64" t="n">
-        <v>29.7</v>
+        <v>29.6</v>
       </c>
       <c r="R64" t="n">
         <v>3</v>
@@ -11314,10 +11308,10 @@
         <v>1100000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1502996</v>
+        <v>1502138</v>
       </c>
       <c r="L65" t="n">
-        <v>26.81284580930355</v>
+        <v>26.77104234098332</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -11378,10 +11372,10 @@
         <v>1105000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1502996</v>
+        <v>1502138</v>
       </c>
       <c r="L66" t="n">
-        <v>26.48017692661857</v>
+        <v>26.43818344253324</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -11442,10 +11436,10 @@
         <v>1155000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1588906</v>
+        <v>1587999</v>
       </c>
       <c r="L67" t="n">
-        <v>27.3084751394985</v>
+        <v>27.26695671722715</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -11712,7 +11706,7 @@
         <v>315000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>300256</v>
+        <v>300084</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -11773,10 +11767,10 @@
         <v>380000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>386166</v>
+        <v>385945</v>
       </c>
       <c r="L3" t="n">
-        <v>1.596722652952357</v>
+        <v>1.540374923888119</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -11837,7 +11831,7 @@
         <v>415000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>386166</v>
+        <v>385945</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -11898,10 +11892,10 @@
         <v>495000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>472076</v>
+        <v>471806</v>
       </c>
       <c r="L5" t="n">
-        <v>6.79488048534558</v>
+        <v>6.741542074496722</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -11962,10 +11956,10 @@
         <v>500000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>515031</v>
+        <v>514736</v>
       </c>
       <c r="L6" t="n">
-        <v>8.743357195974612</v>
+        <v>8.691057163283702</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -12026,10 +12020,10 @@
         <v>550000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>557986</v>
+        <v>557667</v>
       </c>
       <c r="L7" t="n">
-        <v>6.807697684171288</v>
+        <v>6.754389268147479</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -12090,7 +12084,7 @@
         <v>530000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>472076</v>
+        <v>471806</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -12154,10 +12148,10 @@
         <v>600000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>600941</v>
+        <v>600597</v>
       </c>
       <c r="L9" t="n">
-        <v>8.47687210558108</v>
+        <v>8.424451004583773</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -12218,10 +12212,10 @@
         <v>646000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>729806</v>
+        <v>729389</v>
       </c>
       <c r="L10" t="n">
-        <v>17.10139406910878</v>
+        <v>17.05399999177394</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -12233,7 +12227,7 @@
         <v>100</v>
       </c>
       <c r="Q10" t="n">
-        <v>26</v>
+        <v>25.9</v>
       </c>
       <c r="R10" t="n">
         <v>4</v>
@@ -12282,7 +12276,7 @@
         <v>615000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>557986</v>
+        <v>557667</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -12346,7 +12340,7 @@
         <v>700000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>643896</v>
+        <v>643528</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -12410,7 +12404,7 @@
         <v>745000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>686851</v>
+        <v>686458</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -12474,7 +12468,7 @@
         <v>930000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>858671</v>
+        <v>858180</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -12545,7 +12539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12594,7 +12588,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 MGE94 M5 Max 18 Core CPU 40 Core GPU 48GB 2TB Silver</t>
+          <t>Apple MacBook Pro 16 M5 Max 18 Core CPU 40 Core GPU 128GB 8TB Silver</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -12603,22 +12597,22 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>1460000</v>
+        <v>3186000</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>1450000</v>
+        <v>3098000</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-10000</v>
+        <v>-88000</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.68</v>
+        <v>-2.76</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 MGEE4 M5 Max 18 Core CPU 40 Core GPU 48GB 2TB Space Black</t>
+          <t>Macbook Pro 16 CTO M5 Max 18 Core CPU 40 Core GPU 48GB 8TB Space Black</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -12627,22 +12621,22 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>1460000</v>
+        <v>2581000</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>1450000</v>
+        <v>2499000</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>-10000</v>
+        <v>-82000</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.68</v>
+        <v>-3.18</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 MGED4 M5 Max 18 Core CPU 32 Core GPU 36GB 2TB Space Black</t>
+          <t>Macbook Pro 16 CTO M5 Max 18 Core CPU 40 Core GPU 48GB 4TB Space Black</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -12651,22 +12645,22 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>1207000</v>
+        <v>1945000</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>1200000</v>
+        <v>1875000</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>-7000</v>
+        <v>-70000</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.58</v>
+        <v>-3.6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 MGE74 M5 Max 18 Core CPU 32 Core GPU 36GB 2TB Silver</t>
+          <t>Macbook Pro 16 CTO M5 Max 18 Core CPU 32 Core GPU 36GB 8TB Space Black</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -12675,22 +12669,22 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>1207000</v>
+        <v>2381000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>1200000</v>
+        <v>2315000</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>-7000</v>
+        <v>-66000</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.58</v>
+        <v>-2.77</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 MGDR4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Space Black</t>
+          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 64GB 4TB Silver</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -12699,22 +12693,22 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>724999</v>
+        <v>1790000</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>720000</v>
+        <v>1725000</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-4999</v>
+        <v>-65000</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.6899999999999999</v>
+        <v>-3.63</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 MGDN4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Silver</t>
+          <t>Apple MacBook Pro 16 M5 Max 18 Core CPU 40 Core GPU 128GB 4TB Silver</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -12723,22 +12717,22 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>729999</v>
+        <v>2571000</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>725000</v>
+        <v>2510000</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>-4999</v>
+        <v>-61000</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.68</v>
+        <v>-2.37</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MDVD4 M5 10C CPU 10C GPU 16GB 512GB Starlight</t>
+          <t>Apple MacBook Pro 16 M5 Max 18 Core CPU 40 Core GPU 128GB 2TB Silver</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -12747,22 +12741,22 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>482999</v>
+        <v>2268000</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>479999</v>
+        <v>2210000</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>-3000</v>
+        <v>-58000</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.62</v>
+        <v>-2.56</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MDVQ4 M5 10C CPU 10C GPU 16GB 512GB Sky Blue</t>
+          <t>Macbook Pro 16 CTO M5 Max 18 Core CPU 40 Core GPU 64GB 4TB Space Black</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -12771,22 +12765,22 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>482999</v>
+        <v>2078000</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>479999</v>
+        <v>2020000</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>-3000</v>
+        <v>-58000</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.62</v>
+        <v>-2.79</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MDVH4 M5 10C CPU 10C GPU 16GB 512GB Midnight</t>
+          <t>Macbook Pro 16 CTO M5 Max 18 Core CPU 40 Core GPU 64GB 8TB Space Black</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -12795,22 +12789,22 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>482999</v>
+        <v>2664000</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>479999</v>
+        <v>2610000</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>-3000</v>
+        <v>-54000</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.62</v>
+        <v>-2.03</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MDV94 M5 10C CPU 10C GPU 16GB 512GB Silver</t>
+          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 64GB 2TB Silver</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -12819,45 +12813,381 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>485999</v>
+        <v>1471000</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>484999</v>
+        <v>1420000</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>-1000</v>
+        <v>-51000</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.21</v>
+        <v>-3.47</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 MDE04 10 Core CPU 10 Core GPU 16GB 512GB Space Black</t>
+          <t>Apple MacBook Pro 16 CTO M5 Max 18 Core CPU 40 Core GPU 64GB 2TB Space Black</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>1756000</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>1705000</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>-51000</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-2.9</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Apple MacBook Pro 14Inch MX2E3 M4 Pro 12Core CPU 16Core GPU 24GB 512GB Silver</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>650000</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>600000</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>-50000</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-7.69</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Apple MacBook Pro 14Inch MX2H3 M4 Pro 12Core CPU 16Core GPU 24GB 512GB Space Black</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>650000</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>600000</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>-50000</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-7.69</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 48GB 4TB Silver</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>1661000</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>1615000</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>-46000</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-2.77</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 24GB 4TB Space Black</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>1471000</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>1430000</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>-41000</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-2.79</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 48GB 2TB Silver</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>1338000</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>1298000</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>-40000</v>
+      </c>
+      <c r="F17" t="n">
+        <v>-2.99</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 24GB 2TB Space Black</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>1150000</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>1115000</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>-35000</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-3.04</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Apple MacBook Pro 16Inch MX2V3 14Core CPU 32Core GPU M4 Max 36GB 1TB Silver</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>1022000</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>995000</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>-27000</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-2.64</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Macbook Pro 16 CTO M5 Max 18 Core CPU 32 Core GPU 36GB 4TB Space Black</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>1711000</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>1690000</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>-21000</v>
+      </c>
+      <c r="F20" t="n">
+        <v>-1.23</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Macbook Pro 16 MGE94 M5 Max 18 Core CPU 40 Core GPU 48GB 2TB Silver</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>1450000</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>1430000</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>-20000</v>
+      </c>
+      <c r="F21" t="n">
+        <v>-1.38</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Macbook Pro 16 MGEE4 M5 Max 18 Core CPU 40 Core GPU 48GB 2TB Space Black</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>1450000</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>1430000</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>-20000</v>
+      </c>
+      <c r="F22" t="n">
+        <v>-1.38</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Macbook Pro 16 MGE44 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Silver</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>840000</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>829999</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>-10001</v>
+      </c>
+      <c r="F23" t="n">
+        <v>-1.19</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 64GB 1TB Silver</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>1310000</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>1300000</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>-10000</v>
+      </c>
+      <c r="F24" t="n">
+        <v>-0.76</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Apple MacBook Pro 16Inch MX2X3 14Core CPU 20Core GPU M4 Pro 24GB 512GB Space Black</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="C12" s="3" t="n">
-        <v>555000</v>
-      </c>
-      <c r="D12" s="3" t="n">
-        <v>560000</v>
-      </c>
-      <c r="E12" s="3" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F12" t="n">
-        <v>0.9</v>
+      <c r="C25" s="3" t="n">
+        <v>707999</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>711999</v>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>4000</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Apple MacBook Pro 16Inch MX303 14Core CPU 32Core GPU M4 Max 36GB 1TB Space Black</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>970000</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>995000</v>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>25000</v>
+      </c>
+      <c r="F26" t="n">
+        <v>2.58</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F12"/>
-  <conditionalFormatting sqref="E2:E12">
+  <autoFilter ref="A1:F26"/>
+  <conditionalFormatting sqref="E2:E26">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
chore: price data 2026-09-25
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MacBook Pro'!$A$1:$S$92</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MacBook Air'!$A$1:$S$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20260924T083143925226+0000</t>
+          <t>20260925T085320596041+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-24T08:31:43.925226+00:00</t>
+          <t>2026-09-25T08:53:20.596041+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>276.970859</v>
+        <v>277.385539</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -729,7 +729,7 @@
         <v>810000</v>
       </c>
       <c r="D22" t="n">
-        <v>50.5</v>
+        <v>50.6</v>
       </c>
       <c r="E22" t="n">
         <v>4</v>
@@ -750,7 +750,7 @@
         <v>1123000</v>
       </c>
       <c r="D23" t="n">
-        <v>50.4</v>
+        <v>50.5</v>
       </c>
       <c r="E23" t="n">
         <v>4</v>
@@ -813,7 +813,7 @@
         <v>745000</v>
       </c>
       <c r="D26" t="n">
-        <v>44.9</v>
+        <v>45</v>
       </c>
       <c r="E26" t="n">
         <v>4</v>
@@ -906,19 +906,19 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHG4 M5 10C CPU 10C GPU 24GB 1TB Midnight</t>
+          <t>Apple MacBook Pro 14Inch MX2H3 M4 Pro 12Core CPU 16Core GPU 24GB 512GB Space Black</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>macbook_air</t>
+          <t>macbook_pro</t>
         </is>
       </c>
       <c r="C31" s="3" t="n">
-        <v>549999</v>
+        <v>600000</v>
       </c>
       <c r="D31" t="n">
-        <v>42.6</v>
+        <v>42.8</v>
       </c>
       <c r="E31" t="n">
         <v>4</v>
@@ -1147,10 +1147,10 @@
         <v>470000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>686458</v>
+        <v>687486</v>
       </c>
       <c r="L2" t="n">
-        <v>35.17447535027635</v>
+        <v>35.27140916324114</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1214,10 +1214,10 @@
         <v>465000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>686458</v>
+        <v>687486</v>
       </c>
       <c r="L3" t="n">
-        <v>33.28069597848667</v>
+        <v>33.38046156576279</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -1232,7 +1232,7 @@
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>10.1</v>
+        <v>10.2</v>
       </c>
       <c r="R3" t="n">
         <v>5</v>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>772319</v>
+        <v>773476</v>
       </c>
       <c r="L4" t="n">
-        <v>35.2600415113444</v>
+        <v>35.35688243720555</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>772319</v>
+        <v>773476</v>
       </c>
       <c r="L5" t="n">
-        <v>32.67043799259115</v>
+        <v>32.77115256323403</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>858180</v>
+        <v>859465</v>
       </c>
       <c r="L6" t="n">
-        <v>38.00834323801534</v>
+        <v>38.1010279650713</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1606,10 +1606,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>858180</v>
+        <v>859465</v>
       </c>
       <c r="L9" t="n">
-        <v>34.16299610804261</v>
+        <v>34.26143007568662</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1673,10 +1673,10 @@
         <v>582999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>858180</v>
+        <v>859465</v>
       </c>
       <c r="L10" t="n">
-        <v>32.06565056281899</v>
+        <v>32.16722030565526</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -1740,10 +1740,10 @@
         <v>587999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>858180</v>
+        <v>859465</v>
       </c>
       <c r="L11" t="n">
-        <v>31.48302220979281</v>
+        <v>31.58546304968789</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -1758,7 +1758,7 @@
         <v>47.60029999999999</v>
       </c>
       <c r="Q11" t="n">
-        <v>18.4</v>
+        <v>18.5</v>
       </c>
       <c r="R11" t="n">
         <v>4</v>
@@ -1772,7 +1772,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 14Inch MX2E3 M4 Pro 12Core CPU 16Core GPU 24GB 512GB Silver</t>
+          <t>Apple MacBook Pro 14Inch MX2H3 M4 Pro 12Core CPU 16Core GPU 24GB 512GB Space Black</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I12" s="3" t="n">
@@ -1807,25 +1807,28 @@
         <v>600000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>858180</v>
+        <v>859465</v>
       </c>
       <c r="L12" t="n">
-        <v>30.0845976368594</v>
+        <v>30.18912928391499</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>-50000</v>
+        <v>0</v>
       </c>
       <c r="N12" t="n">
         <v>7.692307692307693</v>
       </c>
+      <c r="O12" t="n">
+        <v>100</v>
+      </c>
       <c r="P12" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="Q12" t="n">
-        <v>15.6</v>
+        <v>42.8</v>
       </c>
       <c r="R12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -1836,7 +1839,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 14Inch MX2H3 M4 Pro 12Core CPU 16Core GPU 24GB 512GB Space Black</t>
+          <t>Apple MacBook Pro 14Inch MX2E3 M4 Pro 12Core CPU 16Core GPU 24GB 512GB Silver</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1861,35 +1864,38 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I13" s="3" t="n">
-        <v>600000</v>
+        <v>640000</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>600000</v>
+        <v>640000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>858180</v>
+        <v>859465</v>
       </c>
       <c r="L13" t="n">
-        <v>30.0845976368594</v>
+        <v>25.53507123617599</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>-50000</v>
+        <v>40000</v>
       </c>
       <c r="N13" t="n">
-        <v>7.692307692307693</v>
+        <v>1.538461538461539</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
       </c>
       <c r="P13" t="n">
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>15.6</v>
+        <v>8.9</v>
       </c>
       <c r="R13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
@@ -1935,10 +1941,10 @@
         <v>643999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>944041</v>
+        <v>945455</v>
       </c>
       <c r="L14" t="n">
-        <v>31.78272977550763</v>
+        <v>31.88475390156063</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -2061,10 +2067,10 @@
         <v>650000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>944041</v>
+        <v>945455</v>
       </c>
       <c r="L16" t="n">
-        <v>31.14705823158104</v>
+        <v>31.25003305286873</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -2079,7 +2085,7 @@
         <v>68</v>
       </c>
       <c r="Q16" t="n">
-        <v>21.7</v>
+        <v>21.8</v>
       </c>
       <c r="R16" t="n">
         <v>4</v>
@@ -2128,10 +2134,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1029902</v>
+        <v>1031444</v>
       </c>
       <c r="L17" t="n">
-        <v>32.03236812822968</v>
+        <v>32.13397915931451</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2195,13 +2201,13 @@
         <v>711999</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>1072833</v>
+        <v>1074439</v>
       </c>
       <c r="L18" t="n">
-        <v>33.63375287672918</v>
+        <v>33.73295273161156</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>4000</v>
+        <v>0</v>
       </c>
       <c r="N18" t="n">
         <v>0</v>
@@ -2324,10 +2330,10 @@
         <v>720000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>1029902</v>
+        <v>1031444</v>
       </c>
       <c r="L20" t="n">
-        <v>30.09043578903624</v>
+        <v>30.19494999243778</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -2339,10 +2345,10 @@
         <v>0</v>
       </c>
       <c r="P20" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="Q20" t="n">
-        <v>20</v>
+        <v>23.4</v>
       </c>
       <c r="R20" t="n">
         <v>4</v>
@@ -2453,10 +2459,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1072833</v>
+        <v>1074439</v>
       </c>
       <c r="L22" t="n">
-        <v>30.74411394876929</v>
+        <v>30.84763304384893</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2471,7 +2477,7 @@
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>10.2</v>
+        <v>10.3</v>
       </c>
       <c r="R22" t="n">
         <v>4</v>
@@ -2520,10 +2526,10 @@
         <v>745000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1029902</v>
+        <v>1031444</v>
       </c>
       <c r="L23" t="n">
-        <v>27.66302036504444</v>
+        <v>27.77116353384188</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -2538,7 +2544,7 @@
         <v>74.99999999999999</v>
       </c>
       <c r="Q23" t="n">
-        <v>44.9</v>
+        <v>45</v>
       </c>
       <c r="R23" t="n">
         <v>4</v>
@@ -2587,10 +2593,10 @@
         <v>755000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1029902</v>
+        <v>1031444</v>
       </c>
       <c r="L24" t="n">
-        <v>26.69205419544772</v>
+        <v>26.80164895040351</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -2654,10 +2660,10 @@
         <v>772000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>1029902</v>
+        <v>1031444</v>
       </c>
       <c r="L25" t="n">
-        <v>25.0414117071333</v>
+        <v>25.15347415855829</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -2672,7 +2678,7 @@
         <v>69.59999999999998</v>
       </c>
       <c r="Q25" t="n">
-        <v>19.9</v>
+        <v>20</v>
       </c>
       <c r="R25" t="n">
         <v>4</v>
@@ -2783,10 +2789,10 @@
         <v>810000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>1244555</v>
+        <v>1246418</v>
       </c>
       <c r="L27" t="n">
-        <v>34.91649625769854</v>
+        <v>35.01377547500116</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -2801,7 +2807,7 @@
         <v>100</v>
       </c>
       <c r="Q27" t="n">
-        <v>50.5</v>
+        <v>50.6</v>
       </c>
       <c r="R27" t="n">
         <v>4</v>
@@ -2912,10 +2918,10 @@
         <v>825000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>1287485</v>
+        <v>1289413</v>
       </c>
       <c r="L29" t="n">
-        <v>35.92158355242974</v>
+        <v>36.01739706362508</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -2930,7 +2936,7 @@
         <v>1.718244359164265</v>
       </c>
       <c r="Q29" t="n">
-        <v>34.7</v>
+        <v>34.8</v>
       </c>
       <c r="R29" t="n">
         <v>4</v>
@@ -2979,13 +2985,13 @@
         <v>829999</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1287485</v>
+        <v>1289413</v>
       </c>
       <c r="L30" t="n">
-        <v>35.53330718416137</v>
+        <v>35.62970126716576</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>-10001</v>
+        <v>0</v>
       </c>
       <c r="N30" t="n">
         <v>4.597816091954023</v>
@@ -2997,7 +3003,7 @@
         <v>0</v>
       </c>
       <c r="Q30" t="n">
-        <v>13.1</v>
+        <v>13.2</v>
       </c>
       <c r="R30" t="n">
         <v>4</v>
@@ -3046,10 +3052,10 @@
         <v>830000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1072833</v>
+        <v>1074439</v>
       </c>
       <c r="L31" t="n">
-        <v>22.63474371127659</v>
+        <v>22.75038415396314</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -3061,7 +3067,7 @@
         <v>57.99999999999999</v>
       </c>
       <c r="Q31" t="n">
-        <v>22.3</v>
+        <v>22.4</v>
       </c>
       <c r="R31" t="n">
         <v>3</v>
@@ -3110,10 +3116,10 @@
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1373346</v>
+        <v>1375402</v>
       </c>
       <c r="L32" t="n">
-        <v>38.25306951052393</v>
+        <v>38.34537102607092</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3177,10 +3183,10 @@
         <v>930000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1373346</v>
+        <v>1375402</v>
       </c>
       <c r="L33" t="n">
-        <v>38.10743978574955</v>
+        <v>38.1999589938069</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3244,10 +3250,10 @@
         <v>860000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>1244555</v>
+        <v>1246418</v>
       </c>
       <c r="L34" t="n">
-        <v>30.89899602669227</v>
+        <v>31.00228013395185</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -3497,10 +3503,10 @@
         <v>880000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>1158694</v>
+        <v>1160429</v>
       </c>
       <c r="L38" t="n">
-        <v>24.0524245400425</v>
+        <v>24.16597654832825</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -3561,10 +3567,10 @@
         <v>940000</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>1244555</v>
+        <v>1246418</v>
       </c>
       <c r="L39" t="n">
-        <v>24.47099565708225</v>
+        <v>24.58388758827295</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -3576,7 +3582,7 @@
         <v>83</v>
       </c>
       <c r="Q39" t="n">
-        <v>29</v>
+        <v>29.1</v>
       </c>
       <c r="R39" t="n">
         <v>3</v>
@@ -3687,13 +3693,13 @@
         <v>995000</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>1502138</v>
+        <v>1504387</v>
       </c>
       <c r="L41" t="n">
-        <v>33.76107920843491</v>
+        <v>33.86010381637172</v>
       </c>
       <c r="M41" s="3" t="n">
-        <v>-27000</v>
+        <v>0</v>
       </c>
       <c r="N41" t="n">
         <v>2.64187866927593</v>
@@ -3751,13 +3757,13 @@
         <v>995000</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>1502138</v>
+        <v>1504387</v>
       </c>
       <c r="L42" t="n">
-        <v>33.76107920843491</v>
+        <v>33.86010381637172</v>
       </c>
       <c r="M42" s="3" t="n">
-        <v>25000</v>
+        <v>0</v>
       </c>
       <c r="N42" t="n">
         <v>0</v>
@@ -3766,7 +3772,7 @@
         <v>35.27682508574235</v>
       </c>
       <c r="Q42" t="n">
-        <v>22</v>
+        <v>22.1</v>
       </c>
       <c r="R42" t="n">
         <v>3</v>
@@ -3815,10 +3821,10 @@
         <v>1055000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1545068</v>
+        <v>1547381</v>
       </c>
       <c r="L43" t="n">
-        <v>31.71821563840556</v>
+        <v>31.82028214124382</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -3830,7 +3836,7 @@
         <v>58.64647440248988</v>
       </c>
       <c r="Q43" t="n">
-        <v>26.4</v>
+        <v>26.5</v>
       </c>
       <c r="R43" t="n">
         <v>3</v>
@@ -3879,10 +3885,10 @@
         <v>1055000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1545068</v>
+        <v>1547381</v>
       </c>
       <c r="L44" t="n">
-        <v>31.71821563840556</v>
+        <v>31.82028214124382</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -3894,7 +3900,7 @@
         <v>58.64647440248988</v>
       </c>
       <c r="Q44" t="n">
-        <v>27.1</v>
+        <v>27.2</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -4005,13 +4011,13 @@
         <v>1115000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1502138</v>
+        <v>1504387</v>
       </c>
       <c r="L46" t="n">
-        <v>25.77246564563309</v>
+        <v>25.88343291985373</v>
       </c>
       <c r="M46" s="3" t="n">
-        <v>-35000</v>
+        <v>0</v>
       </c>
       <c r="N46" t="n">
         <v>3.043478260869565</v>
@@ -4020,7 +4026,7 @@
         <v>11.53874765504792</v>
       </c>
       <c r="Q46" t="n">
-        <v>14.6</v>
+        <v>14.7</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -4069,10 +4075,10 @@
         <v>1123000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1716790</v>
+        <v>1719360</v>
       </c>
       <c r="L47" t="n">
-        <v>34.58722383052091</v>
+        <v>34.68499906942118</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -4087,7 +4093,7 @@
         <v>100</v>
       </c>
       <c r="Q47" t="n">
-        <v>50.4</v>
+        <v>50.5</v>
       </c>
       <c r="R47" t="n">
         <v>4</v>
@@ -4136,10 +4142,10 @@
         <v>1130000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1502138</v>
+        <v>1504387</v>
       </c>
       <c r="L48" t="n">
-        <v>24.77388895028286</v>
+        <v>24.88634905778899</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -4262,10 +4268,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1759721</v>
+        <v>1762355</v>
       </c>
       <c r="L50" t="n">
-        <v>34.36459529664078</v>
+        <v>34.46269338470399</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4326,10 +4332,10 @@
         <v>1155000</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>1759721</v>
+        <v>1762355</v>
       </c>
       <c r="L51" t="n">
-        <v>34.36459529664078</v>
+        <v>34.46269338470399</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -4390,10 +4396,10 @@
         <v>1185000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1587999</v>
+        <v>1590376</v>
       </c>
       <c r="L52" t="n">
-        <v>25.37778676183046</v>
+        <v>25.48931824926936</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -4405,7 +4411,7 @@
         <v>77.26495726495727</v>
       </c>
       <c r="Q52" t="n">
-        <v>28.3</v>
+        <v>28.4</v>
       </c>
       <c r="R52" t="n">
         <v>3</v>
@@ -4454,10 +4460,10 @@
         <v>1185000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1587999</v>
+        <v>1590376</v>
       </c>
       <c r="L53" t="n">
-        <v>25.37778676183046</v>
+        <v>25.48931824926936</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -4469,7 +4475,7 @@
         <v>94.72727272727272</v>
       </c>
       <c r="Q53" t="n">
-        <v>31.9</v>
+        <v>32</v>
       </c>
       <c r="R53" t="n">
         <v>3</v>
@@ -4518,10 +4524,10 @@
         <v>1200000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1888512</v>
+        <v>1891339</v>
       </c>
       <c r="L54" t="n">
-        <v>36.45790971939813</v>
+        <v>36.55288660573277</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -4582,10 +4588,10 @@
         <v>1200000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1888512</v>
+        <v>1891339</v>
       </c>
       <c r="L55" t="n">
-        <v>36.45790971939813</v>
+        <v>36.55288660573277</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -4708,10 +4714,10 @@
         <v>1240000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1673860</v>
+        <v>1676366</v>
       </c>
       <c r="L57" t="n">
-        <v>25.91973044340626</v>
+        <v>26.03047305898593</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -4772,10 +4778,10 @@
         <v>1280000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>1716790</v>
+        <v>1719360</v>
       </c>
       <c r="L58" t="n">
-        <v>25.44224978011288</v>
+        <v>25.55369439791551</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -4839,13 +4845,13 @@
         <v>1298000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1759721</v>
+        <v>1762355</v>
       </c>
       <c r="L59" t="n">
-        <v>26.23830709527249</v>
+        <v>26.34855066090543</v>
       </c>
       <c r="M59" s="3" t="n">
-        <v>-40000</v>
+        <v>0</v>
       </c>
       <c r="N59" t="n">
         <v>2.989536621823617</v>
@@ -4854,7 +4860,7 @@
         <v>62.21254466180763</v>
       </c>
       <c r="Q59" t="n">
-        <v>25.6</v>
+        <v>25.7</v>
       </c>
       <c r="R59" t="n">
         <v>3</v>
@@ -4903,13 +4909,13 @@
         <v>1300000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1716790</v>
+        <v>1719360</v>
       </c>
       <c r="L60" t="n">
-        <v>24.27728493292715</v>
+        <v>24.39047087288293</v>
       </c>
       <c r="M60" s="3" t="n">
-        <v>-10000</v>
+        <v>0</v>
       </c>
       <c r="N60" t="n">
         <v>0.7633587786259541</v>
@@ -4918,7 +4924,7 @@
         <v>61.86882704645171</v>
       </c>
       <c r="Q60" t="n">
-        <v>23.9</v>
+        <v>24</v>
       </c>
       <c r="R60" t="n">
         <v>3</v>
@@ -5026,10 +5032,10 @@
         <v>1335000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1802651</v>
+        <v>1805350</v>
       </c>
       <c r="L62" t="n">
-        <v>25.9424037154169</v>
+        <v>26.05311989364943</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -5041,7 +5047,7 @@
         <v>87.17948717948718</v>
       </c>
       <c r="Q62" t="n">
-        <v>30.7</v>
+        <v>30.8</v>
       </c>
       <c r="R62" t="n">
         <v>3</v>
@@ -5090,13 +5096,13 @@
         <v>1420000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1931442</v>
+        <v>1934334</v>
       </c>
       <c r="L63" t="n">
-        <v>26.47980110197459</v>
+        <v>26.58972028615534</v>
       </c>
       <c r="M63" s="3" t="n">
-        <v>-51000</v>
+        <v>0</v>
       </c>
       <c r="N63" t="n">
         <v>3.467029231815092</v>
@@ -5105,7 +5111,7 @@
         <v>81.91902127554754</v>
       </c>
       <c r="Q63" t="n">
-        <v>30.1</v>
+        <v>30.2</v>
       </c>
       <c r="R63" t="n">
         <v>3</v>
@@ -5154,13 +5160,13 @@
         <v>1430000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1931442</v>
+        <v>1934334</v>
       </c>
       <c r="L64" t="n">
-        <v>25.96205322241103</v>
+        <v>26.07274648535362</v>
       </c>
       <c r="M64" s="3" t="n">
-        <v>-41000</v>
+        <v>0</v>
       </c>
       <c r="N64" t="n">
         <v>2.787219578518015</v>
@@ -5218,13 +5224,13 @@
         <v>1430000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>2146095</v>
+        <v>2149308</v>
       </c>
       <c r="L65" t="n">
-        <v>33.36734860292764</v>
+        <v>33.46695773709492</v>
       </c>
       <c r="M65" s="3" t="n">
-        <v>-20000</v>
+        <v>0</v>
       </c>
       <c r="N65" t="n">
         <v>0</v>
@@ -5282,13 +5288,13 @@
         <v>1430000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>2146095</v>
+        <v>2149308</v>
       </c>
       <c r="L66" t="n">
-        <v>33.36734860292764</v>
+        <v>33.46695773709492</v>
       </c>
       <c r="M66" s="3" t="n">
-        <v>-20000</v>
+        <v>0</v>
       </c>
       <c r="N66" t="n">
         <v>0</v>
@@ -5408,10 +5414,10 @@
         <v>1480000</v>
       </c>
       <c r="K68" s="3" t="n">
-        <v>2017303</v>
+        <v>2020324</v>
       </c>
       <c r="L68" t="n">
-        <v>26.63471972232233</v>
+        <v>26.74442317172889</v>
       </c>
       <c r="M68" s="3" t="n">
         <v>0</v>
@@ -5534,10 +5540,10 @@
         <v>1605000</v>
       </c>
       <c r="K70" s="3" t="n">
-        <v>2189025</v>
+        <v>2192303</v>
       </c>
       <c r="L70" t="n">
-        <v>26.67968616164731</v>
+        <v>26.78931698766092</v>
       </c>
       <c r="M70" s="3" t="n">
         <v>0</v>
@@ -5549,7 +5555,7 @@
         <v>36.44392794886694</v>
       </c>
       <c r="Q70" t="n">
-        <v>20.2</v>
+        <v>20.3</v>
       </c>
       <c r="R70" t="n">
         <v>3</v>
@@ -5598,10 +5604,10 @@
         <v>1610000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2189025</v>
+        <v>2192303</v>
       </c>
       <c r="L71" t="n">
-        <v>26.45127396900446</v>
+        <v>26.56124632407108</v>
       </c>
       <c r="M71" s="3" t="n">
         <v>0</v>
@@ -5613,7 +5619,7 @@
         <v>25.72147975982957</v>
       </c>
       <c r="Q71" t="n">
-        <v>17.9</v>
+        <v>18</v>
       </c>
       <c r="R71" t="n">
         <v>3</v>
@@ -5662,13 +5668,13 @@
         <v>1615000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2189025</v>
+        <v>2192303</v>
       </c>
       <c r="L72" t="n">
-        <v>26.22286177636162</v>
+        <v>26.33317566048124</v>
       </c>
       <c r="M72" s="3" t="n">
-        <v>-46000</v>
+        <v>0</v>
       </c>
       <c r="N72" t="n">
         <v>2.769416014449127</v>
@@ -5726,10 +5732,10 @@
         <v>1630000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2231956</v>
+        <v>2235297</v>
       </c>
       <c r="L73" t="n">
-        <v>26.96988650313895</v>
+        <v>27.0790413980782</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
@@ -5790,13 +5796,13 @@
         <v>1690000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2317817</v>
+        <v>2321287</v>
       </c>
       <c r="L74" t="n">
-        <v>27.08656464250629</v>
+        <v>27.19556004923131</v>
       </c>
       <c r="M74" s="3" t="n">
-        <v>-21000</v>
+        <v>0</v>
       </c>
       <c r="N74" t="n">
         <v>1.227352425482174</v>
@@ -5854,13 +5860,13 @@
         <v>1705000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2317817</v>
+        <v>2321287</v>
       </c>
       <c r="L75" t="n">
-        <v>26.4394039736528</v>
+        <v>26.54936679523041</v>
       </c>
       <c r="M75" s="3" t="n">
-        <v>-51000</v>
+        <v>0</v>
       </c>
       <c r="N75" t="n">
         <v>2.904328018223234</v>
@@ -5918,13 +5924,13 @@
         <v>1725000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2360747</v>
+        <v>2364282</v>
       </c>
       <c r="L76" t="n">
-        <v>26.92990820278496</v>
+        <v>27.03916030321256</v>
       </c>
       <c r="M76" s="3" t="n">
-        <v>-65000</v>
+        <v>0</v>
       </c>
       <c r="N76" t="n">
         <v>3.631284916201118</v>
@@ -5982,10 +5988,10 @@
         <v>1780000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2446608</v>
+        <v>2450271</v>
       </c>
       <c r="L77" t="n">
-        <v>27.24621189826895</v>
+        <v>27.35497420489407</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
@@ -6046,13 +6052,13 @@
         <v>1875000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2575400</v>
+        <v>2579256</v>
       </c>
       <c r="L78" t="n">
-        <v>27.19577541352799</v>
+        <v>27.30461807591026</v>
       </c>
       <c r="M78" s="3" t="n">
-        <v>-70000</v>
+        <v>0</v>
       </c>
       <c r="N78" t="n">
         <v>3.598971722365039</v>
@@ -6061,7 +6067,7 @@
         <v>19.64044075004835</v>
       </c>
       <c r="Q78" t="n">
-        <v>17.1</v>
+        <v>17.2</v>
       </c>
       <c r="R78" t="n">
         <v>3</v>
@@ -6110,10 +6116,10 @@
         <v>1910000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2618330</v>
+        <v>2622250</v>
       </c>
       <c r="L79" t="n">
-        <v>27.05273972341149</v>
+        <v>27.16178854037563</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
@@ -6125,7 +6131,7 @@
         <v>53.22486926205694</v>
       </c>
       <c r="Q79" t="n">
-        <v>23.9</v>
+        <v>24</v>
       </c>
       <c r="R79" t="n">
         <v>3</v>
@@ -6174,13 +6180,13 @@
         <v>2020000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2747122</v>
+        <v>2751235</v>
       </c>
       <c r="L80" t="n">
-        <v>26.46850048887527</v>
+        <v>26.57842750619267</v>
       </c>
       <c r="M80" s="3" t="n">
-        <v>-58000</v>
+        <v>0</v>
       </c>
       <c r="N80" t="n">
         <v>2.791145332050048</v>
@@ -6189,7 +6195,7 @@
         <v>36.26522327469554</v>
       </c>
       <c r="Q80" t="n">
-        <v>20.1</v>
+        <v>20.2</v>
       </c>
       <c r="R80" t="n">
         <v>3</v>
@@ -6238,10 +6244,10 @@
         <v>2110000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2875913</v>
+        <v>2880219</v>
       </c>
       <c r="L81" t="n">
-        <v>26.63199477870158</v>
+        <v>26.74168179572456</v>
       </c>
       <c r="M81" s="3" t="n">
         <v>0</v>
@@ -6253,7 +6259,7 @@
         <v>79.02382335851249</v>
       </c>
       <c r="Q81" t="n">
-        <v>29.3</v>
+        <v>29.4</v>
       </c>
       <c r="R81" t="n">
         <v>3</v>
@@ -6302,13 +6308,13 @@
         <v>2210000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>3004705</v>
+        <v>3009203</v>
       </c>
       <c r="L82" t="n">
-        <v>26.44868631030334</v>
+        <v>26.55862698528481</v>
       </c>
       <c r="M82" s="3" t="n">
-        <v>-58000</v>
+        <v>0</v>
       </c>
       <c r="N82" t="n">
         <v>2.55731922398589</v>
@@ -6317,7 +6323,7 @@
         <v>70.36535859269283</v>
       </c>
       <c r="Q82" t="n">
-        <v>27.3</v>
+        <v>27.4</v>
       </c>
       <c r="R82" t="n">
         <v>3</v>
@@ -6366,10 +6372,10 @@
         <v>2215000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3047635</v>
+        <v>3052198</v>
       </c>
       <c r="L83" t="n">
-        <v>27.32069293074794</v>
+        <v>27.429347637342</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
@@ -6430,13 +6436,13 @@
         <v>2315000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3176426</v>
+        <v>3181182</v>
       </c>
       <c r="L84" t="n">
-        <v>27.11934734194972</v>
+        <v>27.22830696263213</v>
       </c>
       <c r="M84" s="3" t="n">
-        <v>-66000</v>
+        <v>0</v>
       </c>
       <c r="N84" t="n">
         <v>2.771944561108778</v>
@@ -6494,10 +6500,10 @@
         <v>2395000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3305218</v>
+        <v>3310166</v>
       </c>
       <c r="L85" t="n">
-        <v>27.53881892208018</v>
+        <v>27.64713310450292</v>
       </c>
       <c r="M85" s="3" t="n">
         <v>0</v>
@@ -6509,7 +6515,7 @@
         <v>72.76953145634144</v>
       </c>
       <c r="Q85" t="n">
-        <v>28.6</v>
+        <v>28.7</v>
       </c>
       <c r="R85" t="n">
         <v>3</v>
@@ -6558,10 +6564,10 @@
         <v>2410000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3305218</v>
+        <v>3310166</v>
       </c>
       <c r="L86" t="n">
-        <v>27.08499106564227</v>
+        <v>27.19398362499041</v>
       </c>
       <c r="M86" s="3" t="n">
         <v>0</v>
@@ -6573,7 +6579,7 @@
         <v>88.47569242688358</v>
       </c>
       <c r="Q86" t="n">
-        <v>31.4</v>
+        <v>31.5</v>
       </c>
       <c r="R86" t="n">
         <v>3</v>
@@ -6622,13 +6628,13 @@
         <v>2499000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3434009</v>
+        <v>3439151</v>
       </c>
       <c r="L87" t="n">
-        <v>27.22791349702345</v>
+        <v>27.33671769573363</v>
       </c>
       <c r="M87" s="3" t="n">
-        <v>-82000</v>
+        <v>0</v>
       </c>
       <c r="N87" t="n">
         <v>3.17706315381635</v>
@@ -6637,7 +6643,7 @@
         <v>63.67326854471646</v>
       </c>
       <c r="Q87" t="n">
-        <v>26.4</v>
+        <v>26.5</v>
       </c>
       <c r="R87" t="n">
         <v>3</v>
@@ -6686,13 +6692,13 @@
         <v>2510000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3434009</v>
+        <v>3439151</v>
       </c>
       <c r="L88" t="n">
-        <v>26.90758818628606</v>
+        <v>27.01687131504258</v>
       </c>
       <c r="M88" s="3" t="n">
-        <v>-61000</v>
+        <v>0</v>
       </c>
       <c r="N88" t="n">
         <v>2.372617658498639</v>
@@ -6750,10 +6756,10 @@
         <v>2530000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3476940</v>
+        <v>3482145</v>
       </c>
       <c r="L89" t="n">
-        <v>27.23486744091069</v>
+        <v>27.34363445519931</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
@@ -6765,7 +6771,7 @@
         <v>79.17877203176447</v>
       </c>
       <c r="Q89" t="n">
-        <v>29.3</v>
+        <v>29.4</v>
       </c>
       <c r="R89" t="n">
         <v>3</v>
@@ -6814,13 +6820,13 @@
         <v>2610000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3605731</v>
+        <v>3611130</v>
       </c>
       <c r="L90" t="n">
-        <v>27.61523252843875</v>
+        <v>27.72345498500469</v>
       </c>
       <c r="M90" s="3" t="n">
-        <v>-54000</v>
+        <v>0</v>
       </c>
       <c r="N90" t="n">
         <v>2.027027027027027</v>
@@ -6829,7 +6835,7 @@
         <v>74.15426251691474</v>
       </c>
       <c r="Q90" t="n">
-        <v>28.4</v>
+        <v>28.5</v>
       </c>
       <c r="R90" t="n">
         <v>3</v>
@@ -6878,10 +6884,10 @@
         <v>3015000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>4163828</v>
+        <v>4170062</v>
       </c>
       <c r="L91" t="n">
-        <v>27.59066897095653</v>
+        <v>27.698916706754</v>
       </c>
       <c r="M91" s="3" t="n">
         <v>0</v>
@@ -6893,7 +6899,7 @@
         <v>100</v>
       </c>
       <c r="Q91" t="n">
-        <v>34.1</v>
+        <v>34.2</v>
       </c>
       <c r="R91" t="n">
         <v>3</v>
@@ -6942,13 +6948,13 @@
         <v>3098000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4292619</v>
+        <v>4299046</v>
       </c>
       <c r="L92" t="n">
-        <v>27.82960705340958</v>
+        <v>27.93750055244815</v>
       </c>
       <c r="M92" s="3" t="n">
-        <v>-88000</v>
+        <v>0</v>
       </c>
       <c r="N92" t="n">
         <v>2.762084118016321</v>
@@ -6957,7 +6963,7 @@
         <v>100</v>
       </c>
       <c r="Q92" t="n">
-        <v>34.3</v>
+        <v>34.4</v>
       </c>
       <c r="R92" t="n">
         <v>3</v>
@@ -7240,10 +7246,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>428876</v>
+        <v>429518</v>
       </c>
       <c r="L2" t="n">
-        <v>27.71826821738684</v>
+        <v>27.82630762855107</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7258,7 +7264,7 @@
         <v>29.71702857142851</v>
       </c>
       <c r="Q2" t="n">
-        <v>36.4</v>
+        <v>36.5</v>
       </c>
       <c r="R2" t="n">
         <v>4</v>
@@ -7307,10 +7313,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>428876</v>
+        <v>429518</v>
       </c>
       <c r="L3" t="n">
-        <v>27.71826821738684</v>
+        <v>27.82630762855107</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7325,7 +7331,7 @@
         <v>29.71702857142851</v>
       </c>
       <c r="Q3" t="n">
-        <v>36.4</v>
+        <v>36.5</v>
       </c>
       <c r="R3" t="n">
         <v>4</v>
@@ -7374,10 +7380,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>428876</v>
+        <v>429518</v>
       </c>
       <c r="L4" t="n">
-        <v>27.71803504975797</v>
+        <v>27.82607480943756</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7441,10 +7447,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>428876</v>
+        <v>429518</v>
       </c>
       <c r="L5" t="n">
-        <v>27.71803504975797</v>
+        <v>27.82607480943756</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7508,10 +7514,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514736</v>
+        <v>515507</v>
       </c>
       <c r="L6" t="n">
-        <v>25.39865095893817</v>
+        <v>25.51022585532301</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7572,10 +7578,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>514736</v>
+        <v>515507</v>
       </c>
       <c r="L7" t="n">
-        <v>25.39865095893817</v>
+        <v>25.51022585532301</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7636,10 +7642,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>514736</v>
+        <v>515507</v>
       </c>
       <c r="L8" t="n">
-        <v>25.39865095893817</v>
+        <v>25.51022585532301</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7700,10 +7706,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>514736</v>
+        <v>515507</v>
       </c>
       <c r="L9" t="n">
-        <v>25.39865095893817</v>
+        <v>25.51022585532301</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7764,10 +7770,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>514736</v>
+        <v>515507</v>
       </c>
       <c r="L10" t="n">
-        <v>25.20437661247708</v>
+        <v>25.31624206848792</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7828,10 +7834,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>514736</v>
+        <v>515507</v>
       </c>
       <c r="L11" t="n">
-        <v>25.20437661247708</v>
+        <v>25.31624206848792</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7892,10 +7898,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>514736</v>
+        <v>515507</v>
       </c>
       <c r="L12" t="n">
-        <v>25.20437661247708</v>
+        <v>25.31624206848792</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -7956,10 +7962,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>514736</v>
+        <v>515507</v>
       </c>
       <c r="L13" t="n">
-        <v>25.20437661247708</v>
+        <v>25.31624206848792</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -8014,31 +8020,34 @@
         </is>
       </c>
       <c r="I14" s="3" t="n">
-        <v>425000</v>
+        <v>422000</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>425000</v>
+        <v>422000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>557667</v>
+        <v>558502</v>
       </c>
       <c r="L14" t="n">
-        <v>23.78964507492823</v>
+        <v>24.44073611195662</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>0</v>
+        <v>-3000</v>
       </c>
       <c r="N14" t="n">
-        <v>4.494167402623376</v>
+        <v>4.524670870296086</v>
+      </c>
+      <c r="O14" t="n">
+        <v>100</v>
       </c>
       <c r="P14" t="n">
-        <v>0</v>
+        <v>2.016806722689076</v>
       </c>
       <c r="Q14" t="n">
-        <v>11.8</v>
+        <v>32</v>
       </c>
       <c r="R14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
@@ -8078,31 +8087,34 @@
         </is>
       </c>
       <c r="I15" s="3" t="n">
-        <v>425000</v>
+        <v>422000</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>425000</v>
+        <v>422000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>557667</v>
+        <v>558502</v>
       </c>
       <c r="L15" t="n">
-        <v>23.78964507492823</v>
+        <v>24.44073611195662</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>0</v>
+        <v>-3000</v>
       </c>
       <c r="N15" t="n">
-        <v>1.847348377247984</v>
+        <v>2.540190623996822</v>
+      </c>
+      <c r="O15" t="n">
+        <v>100</v>
       </c>
       <c r="P15" t="n">
-        <v>0</v>
+        <v>2.016806722689076</v>
       </c>
       <c r="Q15" t="n">
-        <v>10.9</v>
+        <v>31.4</v>
       </c>
       <c r="R15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>
@@ -8113,7 +8125,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDH74 M5 10C CPU 8C GPU 16GB 512GB Silver</t>
+          <t>Apple MacBook Air 13 MDHA4 M5 10C CPU 8C GPU 16GB 512GB Starlight</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -8138,35 +8150,38 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Starlight</t>
         </is>
       </c>
       <c r="I16" s="3" t="n">
-        <v>425000</v>
+        <v>422000</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>425000</v>
+        <v>422000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>557667</v>
+        <v>558502</v>
       </c>
       <c r="L16" t="n">
-        <v>23.78964507492823</v>
+        <v>24.44073611195662</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0</v>
+        <v>-3000</v>
       </c>
       <c r="N16" t="n">
-        <v>5.133716816332179</v>
+        <v>1.86046511627907</v>
+      </c>
+      <c r="O16" t="n">
+        <v>100</v>
       </c>
       <c r="P16" t="n">
-        <v>0</v>
+        <v>2.016806722689076</v>
       </c>
       <c r="Q16" t="n">
-        <v>12</v>
+        <v>31.2</v>
       </c>
       <c r="R16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>
@@ -8177,7 +8192,7 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHA4 M5 10C CPU 8C GPU 16GB 512GB Starlight</t>
+          <t>Apple MacBook Air 13 MDH74 M5 10C CPU 8C GPU 16GB 512GB Silver</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -8202,7 +8217,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Starlight</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I17" s="3" t="n">
@@ -8212,25 +8227,28 @@
         <v>425000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>557667</v>
+        <v>558502</v>
       </c>
       <c r="L17" t="n">
-        <v>23.78964507492823</v>
+        <v>23.90358494687575</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>1.162790697674419</v>
+        <v>5.133716816332179</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
       </c>
       <c r="P17" t="n">
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>10.6</v>
+        <v>9.4</v>
       </c>
       <c r="R17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S17" t="inlineStr">
         <is>
@@ -8276,10 +8294,10 @@
         <v>454000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>600597</v>
+        <v>601497</v>
       </c>
       <c r="L18" t="n">
-        <v>24.40854682923824</v>
+        <v>24.52165181206224</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -8340,10 +8358,10 @@
         <v>454000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>600597</v>
+        <v>601497</v>
       </c>
       <c r="L19" t="n">
-        <v>24.40854682923824</v>
+        <v>24.52165181206224</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -8404,10 +8422,10 @@
         <v>454000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>600597</v>
+        <v>601497</v>
       </c>
       <c r="L20" t="n">
-        <v>24.40854682923824</v>
+        <v>24.52165181206224</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -8468,10 +8486,10 @@
         <v>454000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>600597</v>
+        <v>601497</v>
       </c>
       <c r="L21" t="n">
-        <v>24.40854682923824</v>
+        <v>24.52165181206224</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -8532,10 +8550,10 @@
         <v>455000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>600597</v>
+        <v>601497</v>
       </c>
       <c r="L22" t="n">
-        <v>24.24204583106476</v>
+        <v>24.35539994380687</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -8547,7 +8565,7 @@
         <v>100</v>
       </c>
       <c r="Q22" t="n">
-        <v>31.8</v>
+        <v>31.9</v>
       </c>
       <c r="R22" t="n">
         <v>3</v>
@@ -8596,10 +8614,10 @@
         <v>455000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>600597</v>
+        <v>601497</v>
       </c>
       <c r="L23" t="n">
-        <v>24.24204583106476</v>
+        <v>24.35539994380687</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -8611,7 +8629,7 @@
         <v>100</v>
       </c>
       <c r="Q23" t="n">
-        <v>31.8</v>
+        <v>31.9</v>
       </c>
       <c r="R23" t="n">
         <v>3</v>
@@ -8660,10 +8678,10 @@
         <v>455000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>600597</v>
+        <v>601497</v>
       </c>
       <c r="L24" t="n">
-        <v>24.24204583106476</v>
+        <v>24.35539994380687</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -8675,7 +8693,7 @@
         <v>100</v>
       </c>
       <c r="Q24" t="n">
-        <v>31.8</v>
+        <v>31.9</v>
       </c>
       <c r="R24" t="n">
         <v>3</v>
@@ -8724,10 +8742,10 @@
         <v>455000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>600597</v>
+        <v>601497</v>
       </c>
       <c r="L25" t="n">
-        <v>24.24204583106476</v>
+        <v>24.35539994380687</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -8739,7 +8757,7 @@
         <v>100</v>
       </c>
       <c r="Q25" t="n">
-        <v>31.8</v>
+        <v>31.9</v>
       </c>
       <c r="R25" t="n">
         <v>3</v>
@@ -8753,22 +8771,22 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MC6L4 M4 10C CPU 10C GPU 24GB 512GB Midnight</t>
+          <t>Apple MacBook Air 13 MDHF4 M5 10C CPU 10C GPU 16GB 1TB Midnight</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E26" t="n">
-        <v>512</v>
+        <v>1024</v>
       </c>
       <c r="F26" t="n">
         <v>10</v>
@@ -8782,31 +8800,34 @@
         </is>
       </c>
       <c r="I26" s="3" t="n">
-        <v>475000</v>
+        <v>474999</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>475000</v>
+        <v>474999</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>686458</v>
+        <v>687486</v>
       </c>
       <c r="L26" t="n">
-        <v>30.80421526153093</v>
+        <v>30.9078293957986</v>
       </c>
       <c r="M26" s="3" t="n">
-        <v>0</v>
+        <v>-5000</v>
       </c>
       <c r="N26" t="n">
-        <v>0</v>
+        <v>1.041668836810077</v>
+      </c>
+      <c r="O26" t="n">
+        <v>100</v>
       </c>
       <c r="P26" t="n">
-        <v>100</v>
+        <v>46.21899159663865</v>
       </c>
       <c r="Q26" t="n">
-        <v>34.6</v>
+        <v>40.5</v>
       </c>
       <c r="R26" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S26" t="inlineStr">
         <is>
@@ -8817,22 +8838,22 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MC6K4 M4 10C CPU 10C GPU 24GB 512GB Starlight</t>
+          <t>Apple MacBook Air 13 MDHJ4 M5 10C CPU 10C GPU 16GB 1TB Sky Blue</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E27" t="n">
-        <v>512</v>
+        <v>1024</v>
       </c>
       <c r="F27" t="n">
         <v>10</v>
@@ -8842,35 +8863,38 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Starlight</t>
+          <t>Sky Blue</t>
         </is>
       </c>
       <c r="I27" s="3" t="n">
-        <v>475000</v>
+        <v>474999</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>475000</v>
+        <v>474999</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>686458</v>
+        <v>687486</v>
       </c>
       <c r="L27" t="n">
-        <v>30.80421526153093</v>
+        <v>30.9078293957986</v>
       </c>
       <c r="M27" s="3" t="n">
-        <v>0</v>
+        <v>-5000</v>
       </c>
       <c r="N27" t="n">
-        <v>0</v>
+        <v>1.041668836810077</v>
+      </c>
+      <c r="O27" t="n">
+        <v>100</v>
       </c>
       <c r="P27" t="n">
-        <v>100</v>
+        <v>46.21899159663865</v>
       </c>
       <c r="Q27" t="n">
-        <v>34.6</v>
+        <v>40.5</v>
       </c>
       <c r="R27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S27" t="inlineStr">
         <is>
@@ -8881,22 +8905,22 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MC6J4 M4 10C CPU 10C GPU 24GB 512GB Silver</t>
+          <t>Apple MacBook Air 13 MDHC4 M5 10C CPU 10C GPU 16GB 1TB Starlight</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E28" t="n">
-        <v>512</v>
+        <v>1024</v>
       </c>
       <c r="F28" t="n">
         <v>10</v>
@@ -8906,35 +8930,38 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Starlight</t>
         </is>
       </c>
       <c r="I28" s="3" t="n">
-        <v>475000</v>
+        <v>474999</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>475000</v>
+        <v>474999</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>686458</v>
+        <v>687486</v>
       </c>
       <c r="L28" t="n">
-        <v>30.80421526153093</v>
+        <v>30.9078293957986</v>
       </c>
       <c r="M28" s="3" t="n">
-        <v>0</v>
+        <v>-5000</v>
       </c>
       <c r="N28" t="n">
-        <v>0</v>
+        <v>1.041668836810077</v>
+      </c>
+      <c r="O28" t="n">
+        <v>100</v>
       </c>
       <c r="P28" t="n">
-        <v>100</v>
+        <v>46.21899159663865</v>
       </c>
       <c r="Q28" t="n">
-        <v>34.6</v>
+        <v>40.5</v>
       </c>
       <c r="R28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S28" t="inlineStr">
         <is>
@@ -8945,7 +8972,7 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MC7D4 M4 10C CPU 10C GPU 24GB 512GB Sky Blue</t>
+          <t>Apple MacBook Air 15 MC6L4 M4 10C CPU 10C GPU 24GB 512GB Midnight</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -8970,7 +8997,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Sky Blue</t>
+          <t>Midnight</t>
         </is>
       </c>
       <c r="I29" s="3" t="n">
@@ -8980,10 +9007,10 @@
         <v>475000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>686458</v>
+        <v>687486</v>
       </c>
       <c r="L29" t="n">
-        <v>30.80421526153093</v>
+        <v>30.90768393829111</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -8995,7 +9022,7 @@
         <v>100</v>
       </c>
       <c r="Q29" t="n">
-        <v>34.6</v>
+        <v>34.7</v>
       </c>
       <c r="R29" t="n">
         <v>3</v>
@@ -9009,22 +9036,22 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHF4 M5 10C CPU 10C GPU 16GB 1TB Midnight</t>
+          <t>Apple MacBook Air 15 MC6K4 M4 10C CPU 10C GPU 24GB 512GB Starlight</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E30" t="n">
-        <v>1024</v>
+        <v>512</v>
       </c>
       <c r="F30" t="n">
         <v>10</v>
@@ -9034,20 +9061,20 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Midnight</t>
+          <t>Starlight</t>
         </is>
       </c>
       <c r="I30" s="3" t="n">
-        <v>479999</v>
+        <v>475000</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>479999</v>
+        <v>475000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>686458</v>
+        <v>687486</v>
       </c>
       <c r="L30" t="n">
-        <v>30.07598425540965</v>
+        <v>30.90768393829111</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -9056,10 +9083,10 @@
         <v>0</v>
       </c>
       <c r="P30" t="n">
-        <v>43.6979831932773</v>
+        <v>100</v>
       </c>
       <c r="Q30" t="n">
-        <v>22.3</v>
+        <v>34.7</v>
       </c>
       <c r="R30" t="n">
         <v>3</v>
@@ -9073,22 +9100,22 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHJ4 M5 10C CPU 10C GPU 16GB 1TB Sky Blue</t>
+          <t>Apple MacBook Air 15 MC6J4 M4 10C CPU 10C GPU 24GB 512GB Silver</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E31" t="n">
-        <v>1024</v>
+        <v>512</v>
       </c>
       <c r="F31" t="n">
         <v>10</v>
@@ -9098,20 +9125,20 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Sky Blue</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I31" s="3" t="n">
-        <v>479999</v>
+        <v>475000</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>479999</v>
+        <v>475000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>686458</v>
+        <v>687486</v>
       </c>
       <c r="L31" t="n">
-        <v>30.07598425540965</v>
+        <v>30.90768393829111</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -9120,10 +9147,10 @@
         <v>0</v>
       </c>
       <c r="P31" t="n">
-        <v>43.6979831932773</v>
+        <v>100</v>
       </c>
       <c r="Q31" t="n">
-        <v>22.3</v>
+        <v>34.7</v>
       </c>
       <c r="R31" t="n">
         <v>3</v>
@@ -9137,22 +9164,22 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDH84 M5 10C CPU 10C GPU 16GB 1TB Silver</t>
+          <t>Apple MacBook Air 15 MC7D4 M4 10C CPU 10C GPU 24GB 512GB Sky Blue</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E32" t="n">
-        <v>1024</v>
+        <v>512</v>
       </c>
       <c r="F32" t="n">
         <v>10</v>
@@ -9162,20 +9189,20 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Sky Blue</t>
         </is>
       </c>
       <c r="I32" s="3" t="n">
-        <v>479999</v>
+        <v>475000</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>479999</v>
+        <v>475000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>686458</v>
+        <v>687486</v>
       </c>
       <c r="L32" t="n">
-        <v>30.07598425540965</v>
+        <v>30.90768393829111</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -9184,10 +9211,10 @@
         <v>0</v>
       </c>
       <c r="P32" t="n">
-        <v>43.6979831932773</v>
+        <v>100</v>
       </c>
       <c r="Q32" t="n">
-        <v>22.3</v>
+        <v>34.7</v>
       </c>
       <c r="R32" t="n">
         <v>3</v>
@@ -9201,7 +9228,7 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHC4 M5 10C CPU 10C GPU 16GB 1TB Starlight</t>
+          <t>Apple MacBook Air 13 MDH84 M5 10C CPU 10C GPU 16GB 1TB Silver</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -9226,7 +9253,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Starlight</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I33" s="3" t="n">
@@ -9236,25 +9263,28 @@
         <v>479999</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>686458</v>
+        <v>687486</v>
       </c>
       <c r="L33" t="n">
-        <v>30.07598425540965</v>
+        <v>30.18054185830693</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" t="n">
         <v>0</v>
       </c>
       <c r="P33" t="n">
         <v>43.6979831932773</v>
       </c>
       <c r="Q33" t="n">
-        <v>22.3</v>
+        <v>17.3</v>
       </c>
       <c r="R33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S33" t="inlineStr">
         <is>
@@ -9300,10 +9330,10 @@
         <v>479999</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>643528</v>
+        <v>644491</v>
       </c>
       <c r="L34" t="n">
-        <v>25.41132631369575</v>
+        <v>25.52277688904888</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -9367,10 +9397,10 @@
         <v>479999</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>643528</v>
+        <v>644491</v>
       </c>
       <c r="L35" t="n">
-        <v>25.41132631369575</v>
+        <v>25.52277688904888</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
@@ -9434,10 +9464,10 @@
         <v>479999</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>643528</v>
+        <v>644491</v>
       </c>
       <c r="L36" t="n">
-        <v>25.41132631369575</v>
+        <v>25.52277688904888</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -9501,10 +9531,10 @@
         <v>484999</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>643528</v>
+        <v>644491</v>
       </c>
       <c r="L37" t="n">
-        <v>24.63435934411556</v>
+        <v>24.74697086538059</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
@@ -9568,10 +9598,10 @@
         <v>500000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>643528</v>
+        <v>644491</v>
       </c>
       <c r="L38" t="n">
-        <v>22.30330304198108</v>
+        <v>22.41939763317098</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -9626,34 +9656,31 @@
         </is>
       </c>
       <c r="I39" s="3" t="n">
-        <v>549999</v>
+        <v>547999</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>549999</v>
+        <v>547999</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>772319</v>
+        <v>773476</v>
       </c>
       <c r="L39" t="n">
-        <v>28.78603271446125</v>
+        <v>29.15113073967389</v>
       </c>
       <c r="M39" s="3" t="n">
-        <v>0</v>
+        <v>-2000</v>
       </c>
       <c r="N39" t="n">
-        <v>0.3623194969556104</v>
-      </c>
-      <c r="O39" t="n">
-        <v>100</v>
+        <v>0.7246389939112209</v>
       </c>
       <c r="P39" t="n">
-        <v>63.86594957983191</v>
+        <v>64.67267226890753</v>
       </c>
       <c r="Q39" t="n">
-        <v>42.6</v>
+        <v>26.6</v>
       </c>
       <c r="R39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S39" t="inlineStr">
         <is>
@@ -9693,34 +9720,31 @@
         </is>
       </c>
       <c r="I40" s="3" t="n">
-        <v>549999</v>
+        <v>547999</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>549999</v>
+        <v>547999</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>772319</v>
+        <v>773476</v>
       </c>
       <c r="L40" t="n">
-        <v>28.78603271446125</v>
+        <v>29.15113073967389</v>
       </c>
       <c r="M40" s="3" t="n">
-        <v>0</v>
+        <v>-2000</v>
       </c>
       <c r="N40" t="n">
-        <v>0.3623194969556104</v>
-      </c>
-      <c r="O40" t="n">
-        <v>100</v>
+        <v>0.7246389939112209</v>
       </c>
       <c r="P40" t="n">
-        <v>63.86594957983191</v>
+        <v>64.67267226890753</v>
       </c>
       <c r="Q40" t="n">
-        <v>42.6</v>
+        <v>26.6</v>
       </c>
       <c r="R40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S40" t="inlineStr">
         <is>
@@ -9731,7 +9755,7 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHD4 M5 10C CPU 10C GPU 24GB 1TB Starlight</t>
+          <t>Apple MacBook Air 13 MDH94 M5 10C CPU 10C GPU 24GB 1TB Silver</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -9756,38 +9780,35 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Starlight</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I41" s="3" t="n">
-        <v>549999</v>
+        <v>547999</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>549999</v>
+        <v>547999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>772319</v>
+        <v>773476</v>
       </c>
       <c r="L41" t="n">
-        <v>28.78603271446125</v>
+        <v>29.15113073967389</v>
       </c>
       <c r="M41" s="3" t="n">
-        <v>0</v>
+        <v>-4000</v>
       </c>
       <c r="N41" t="n">
-        <v>0.3623194969556104</v>
-      </c>
-      <c r="O41" t="n">
-        <v>100</v>
+        <v>1.792117907021339</v>
       </c>
       <c r="P41" t="n">
-        <v>63.86594957983191</v>
+        <v>64.67267226890753</v>
       </c>
       <c r="Q41" t="n">
-        <v>42.6</v>
+        <v>27</v>
       </c>
       <c r="R41" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S41" t="inlineStr">
         <is>
@@ -9798,7 +9819,7 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDH94 M5 10C CPU 10C GPU 24GB 1TB Silver</t>
+          <t>Apple MacBook Air 13 MDHD4 M5 10C CPU 10C GPU 24GB 1TB Starlight</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -9823,38 +9844,35 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Starlight</t>
         </is>
       </c>
       <c r="I42" s="3" t="n">
-        <v>551999</v>
+        <v>547999</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>551999</v>
+        <v>547999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>772319</v>
+        <v>773476</v>
       </c>
       <c r="L42" t="n">
-        <v>28.52707236258593</v>
+        <v>29.15113073967389</v>
       </c>
       <c r="M42" s="3" t="n">
-        <v>0</v>
+        <v>-2000</v>
       </c>
       <c r="N42" t="n">
-        <v>1.075270744212803</v>
-      </c>
-      <c r="O42" t="n">
-        <v>0</v>
+        <v>0.7246389939112209</v>
       </c>
       <c r="P42" t="n">
-        <v>63.05922689075628</v>
+        <v>64.67267226890753</v>
       </c>
       <c r="Q42" t="n">
-        <v>20.3</v>
+        <v>26.6</v>
       </c>
       <c r="R42" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S42" t="inlineStr">
         <is>
@@ -9894,28 +9912,28 @@
         </is>
       </c>
       <c r="I43" s="3" t="n">
-        <v>564999</v>
+        <v>552999</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>564999</v>
+        <v>552999</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>772319</v>
+        <v>773476</v>
       </c>
       <c r="L43" t="n">
-        <v>26.84383007539631</v>
+        <v>28.50469827118101</v>
       </c>
       <c r="M43" s="3" t="n">
-        <v>0</v>
+        <v>-12000</v>
       </c>
       <c r="N43" t="n">
-        <v>0</v>
+        <v>2.123897564420468</v>
       </c>
       <c r="P43" t="n">
-        <v>31.21022272724958</v>
+        <v>35.7962333566031</v>
       </c>
       <c r="Q43" t="n">
-        <v>18.2</v>
+        <v>20.6</v>
       </c>
       <c r="R43" t="n">
         <v>3</v>
@@ -9958,28 +9976,28 @@
         </is>
       </c>
       <c r="I44" s="3" t="n">
-        <v>564999</v>
+        <v>552999</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>564999</v>
+        <v>552999</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>772319</v>
+        <v>773476</v>
       </c>
       <c r="L44" t="n">
-        <v>26.84383007539631</v>
+        <v>28.50469827118101</v>
       </c>
       <c r="M44" s="3" t="n">
-        <v>0</v>
+        <v>-12000</v>
       </c>
       <c r="N44" t="n">
-        <v>0</v>
+        <v>2.123897564420468</v>
       </c>
       <c r="P44" t="n">
-        <v>31.21022272724958</v>
+        <v>35.7962333566031</v>
       </c>
       <c r="Q44" t="n">
-        <v>18.2</v>
+        <v>20.6</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -10022,28 +10040,28 @@
         </is>
       </c>
       <c r="I45" s="3" t="n">
-        <v>564999</v>
+        <v>552999</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>564999</v>
+        <v>552999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>772319</v>
+        <v>773476</v>
       </c>
       <c r="L45" t="n">
-        <v>26.84383007539631</v>
+        <v>28.50469827118101</v>
       </c>
       <c r="M45" s="3" t="n">
-        <v>0</v>
+        <v>-12000</v>
       </c>
       <c r="N45" t="n">
-        <v>0</v>
+        <v>2.123897564420468</v>
       </c>
       <c r="P45" t="n">
-        <v>31.21022272724958</v>
+        <v>35.7962333566031</v>
       </c>
       <c r="Q45" t="n">
-        <v>18.2</v>
+        <v>20.6</v>
       </c>
       <c r="R45" t="n">
         <v>3</v>
@@ -10086,28 +10104,28 @@
         </is>
       </c>
       <c r="I46" s="3" t="n">
-        <v>564999</v>
+        <v>552999</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>564999</v>
+        <v>552999</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>772319</v>
+        <v>773476</v>
       </c>
       <c r="L46" t="n">
-        <v>26.84383007539631</v>
+        <v>28.50469827118101</v>
       </c>
       <c r="M46" s="3" t="n">
-        <v>0</v>
+        <v>-12000</v>
       </c>
       <c r="N46" t="n">
-        <v>0</v>
+        <v>2.123897564420468</v>
       </c>
       <c r="P46" t="n">
-        <v>31.21022272724958</v>
+        <v>35.7962333566031</v>
       </c>
       <c r="Q46" t="n">
-        <v>18.2</v>
+        <v>20.6</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -10156,10 +10174,10 @@
         <v>585000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>729389</v>
+        <v>730481</v>
       </c>
       <c r="L47" t="n">
-        <v>19.79588395218464</v>
+        <v>19.9157815193003</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -10171,7 +10189,7 @@
         <v>23.56648951077459</v>
       </c>
       <c r="Q47" t="n">
-        <v>13.5</v>
+        <v>13.6</v>
       </c>
       <c r="R47" t="n">
         <v>3</v>
@@ -10220,10 +10238,10 @@
         <v>595000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>729389</v>
+        <v>730481</v>
       </c>
       <c r="L48" t="n">
-        <v>18.42487342145275</v>
+        <v>18.54682051963022</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -10284,10 +10302,10 @@
         <v>614999</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>858180</v>
+        <v>859465</v>
       </c>
       <c r="L49" t="n">
-        <v>28.33682910345149</v>
+        <v>28.44397386746406</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -10299,7 +10317,7 @@
         <v>59.10837762230636</v>
       </c>
       <c r="Q49" t="n">
-        <v>24.9</v>
+        <v>25</v>
       </c>
       <c r="R49" t="n">
         <v>3</v>
@@ -10348,10 +10366,10 @@
         <v>614999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>858180</v>
+        <v>859465</v>
       </c>
       <c r="L50" t="n">
-        <v>28.33682910345149</v>
+        <v>28.44397386746406</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -10363,7 +10381,7 @@
         <v>59.10837762230636</v>
       </c>
       <c r="Q50" t="n">
-        <v>24.9</v>
+        <v>25</v>
       </c>
       <c r="R50" t="n">
         <v>3</v>
@@ -10412,10 +10430,10 @@
         <v>614999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>858180</v>
+        <v>859465</v>
       </c>
       <c r="L51" t="n">
-        <v>28.33682910345149</v>
+        <v>28.44397386746406</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -10427,7 +10445,7 @@
         <v>59.10837762230636</v>
       </c>
       <c r="Q51" t="n">
-        <v>24.9</v>
+        <v>25</v>
       </c>
       <c r="R51" t="n">
         <v>3</v>
@@ -10476,10 +10494,10 @@
         <v>614999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>858180</v>
+        <v>859465</v>
       </c>
       <c r="L52" t="n">
-        <v>28.33682910345149</v>
+        <v>28.44397386746406</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -10491,7 +10509,7 @@
         <v>59.10837762230636</v>
       </c>
       <c r="Q52" t="n">
-        <v>24.8</v>
+        <v>24.9</v>
       </c>
       <c r="R52" t="n">
         <v>3</v>
@@ -10540,10 +10558,10 @@
         <v>650000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>815250</v>
+        <v>816470</v>
       </c>
       <c r="L53" t="n">
-        <v>20.26985587243177</v>
+        <v>20.3889916347202</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -10604,10 +10622,10 @@
         <v>672000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>858180</v>
+        <v>859465</v>
       </c>
       <c r="L54" t="n">
-        <v>21.69474935328253</v>
+        <v>21.81182479798479</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -10619,7 +10637,7 @@
         <v>59.83193277310923</v>
       </c>
       <c r="Q54" t="n">
-        <v>22.1</v>
+        <v>22.2</v>
       </c>
       <c r="R54" t="n">
         <v>3</v>
@@ -10668,10 +10686,10 @@
         <v>700000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>901111</v>
+        <v>902460</v>
       </c>
       <c r="L55" t="n">
-        <v>22.31811619212284</v>
+        <v>22.43423531236841</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -10732,10 +10750,10 @@
         <v>715000</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>944041</v>
+        <v>945455</v>
       </c>
       <c r="L56" t="n">
-        <v>24.26176405473915</v>
+        <v>24.3750363581556</v>
       </c>
       <c r="M56" s="3" t="n">
         <v>0</v>
@@ -10747,7 +10765,7 @@
         <v>64.96797435910501</v>
       </c>
       <c r="Q56" t="n">
-        <v>24.3</v>
+        <v>24.4</v>
       </c>
       <c r="R56" t="n">
         <v>3</v>
@@ -10796,10 +10814,10 @@
         <v>734999</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>986972</v>
+        <v>988449</v>
       </c>
       <c r="L57" t="n">
-        <v>25.52990358389093</v>
+        <v>25.64118128502331</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -10860,10 +10878,10 @@
         <v>752000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>986972</v>
+        <v>988449</v>
       </c>
       <c r="L58" t="n">
-        <v>23.80736231625619</v>
+        <v>23.92121394224689</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -10875,7 +10893,7 @@
         <v>55.54117473210056</v>
       </c>
       <c r="Q58" t="n">
-        <v>22.1</v>
+        <v>22.2</v>
       </c>
       <c r="R58" t="n">
         <v>3</v>
@@ -10924,10 +10942,10 @@
         <v>810000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1072833</v>
+        <v>1074439</v>
       </c>
       <c r="L59" t="n">
-        <v>24.49896675437836</v>
+        <v>24.61182068037366</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -10988,10 +11006,10 @@
         <v>815000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1072833</v>
+        <v>1074439</v>
       </c>
       <c r="L60" t="n">
-        <v>24.03291099360292</v>
+        <v>24.14646154877103</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -11052,10 +11070,10 @@
         <v>875000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1158694</v>
+        <v>1160429</v>
       </c>
       <c r="L61" t="n">
-        <v>24.48394485515589</v>
+        <v>24.59685168157638</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -11067,7 +11085,7 @@
         <v>79.93620349657833</v>
       </c>
       <c r="Q61" t="n">
-        <v>27.6</v>
+        <v>27.7</v>
       </c>
       <c r="R61" t="n">
         <v>3</v>
@@ -11116,10 +11134,10 @@
         <v>992000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1330416</v>
+        <v>1332408</v>
       </c>
       <c r="L62" t="n">
-        <v>25.43685584057919</v>
+        <v>25.54833054139573</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -11180,10 +11198,10 @@
         <v>1050000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1416277</v>
+        <v>1418397</v>
       </c>
       <c r="L63" t="n">
-        <v>25.86196061928564</v>
+        <v>25.97277066998873</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -11244,10 +11262,10 @@
         <v>1050000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1416277</v>
+        <v>1418397</v>
       </c>
       <c r="L64" t="n">
-        <v>25.86196061928564</v>
+        <v>25.97277066998873</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -11259,7 +11277,7 @@
         <v>86.62413566438555</v>
       </c>
       <c r="Q64" t="n">
-        <v>29.6</v>
+        <v>29.7</v>
       </c>
       <c r="R64" t="n">
         <v>3</v>
@@ -11308,10 +11326,10 @@
         <v>1100000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1502138</v>
+        <v>1504387</v>
       </c>
       <c r="L65" t="n">
-        <v>26.77104234098332</v>
+        <v>26.88051678191848</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -11372,10 +11390,10 @@
         <v>1105000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1502138</v>
+        <v>1504387</v>
       </c>
       <c r="L66" t="n">
-        <v>26.43818344253324</v>
+        <v>26.54815549456357</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -11436,10 +11454,10 @@
         <v>1155000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1587999</v>
+        <v>1590376</v>
       </c>
       <c r="L67" t="n">
-        <v>27.26695671722715</v>
+        <v>27.37566462270557</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -11451,7 +11469,7 @@
         <v>100</v>
       </c>
       <c r="Q67" t="n">
-        <v>33.1</v>
+        <v>33.2</v>
       </c>
       <c r="R67" t="n">
         <v>3</v>
@@ -11706,7 +11724,7 @@
         <v>315000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>300084</v>
+        <v>300533</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -11767,10 +11785,10 @@
         <v>380000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>385945</v>
+        <v>386523</v>
       </c>
       <c r="L3" t="n">
-        <v>1.540374923888119</v>
+        <v>1.687609792948932</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -11782,7 +11800,7 @@
         <v>100</v>
       </c>
       <c r="Q3" t="n">
-        <v>22.1</v>
+        <v>22.2</v>
       </c>
       <c r="R3" t="n">
         <v>3</v>
@@ -11831,7 +11849,7 @@
         <v>415000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>385945</v>
+        <v>386523</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -11892,10 +11910,10 @@
         <v>495000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>471806</v>
+        <v>472512</v>
       </c>
       <c r="L5" t="n">
-        <v>6.741542074496722</v>
+        <v>6.880883448462686</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -11907,7 +11925,7 @@
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>3.9</v>
+        <v>4</v>
       </c>
       <c r="R5" t="n">
         <v>4</v>
@@ -11956,10 +11974,10 @@
         <v>500000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514736</v>
+        <v>515507</v>
       </c>
       <c r="L6" t="n">
-        <v>8.691057163283702</v>
+        <v>8.827620187504728</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -11971,7 +11989,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>4</v>
+        <v>4.1</v>
       </c>
       <c r="R6" t="n">
         <v>4</v>
@@ -12020,10 +12038,10 @@
         <v>550000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>557667</v>
+        <v>558502</v>
       </c>
       <c r="L7" t="n">
-        <v>6.754389268147479</v>
+        <v>6.893798052647976</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -12084,7 +12102,7 @@
         <v>530000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>471806</v>
+        <v>472512</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -12148,10 +12166,10 @@
         <v>600000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>600597</v>
+        <v>601497</v>
       </c>
       <c r="L9" t="n">
-        <v>8.424451004583773</v>
+        <v>8.561472459546764</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -12212,10 +12230,10 @@
         <v>646000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>729389</v>
+        <v>730481</v>
       </c>
       <c r="L10" t="n">
-        <v>17.05399999177394</v>
+        <v>17.1779964160601</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -12227,7 +12245,7 @@
         <v>100</v>
       </c>
       <c r="Q10" t="n">
-        <v>25.9</v>
+        <v>26</v>
       </c>
       <c r="R10" t="n">
         <v>4</v>
@@ -12276,7 +12294,7 @@
         <v>615000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>557667</v>
+        <v>558502</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -12340,7 +12358,7 @@
         <v>700000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>643528</v>
+        <v>644491</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -12404,7 +12422,7 @@
         <v>745000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>686458</v>
+        <v>687486</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -12468,7 +12486,7 @@
         <v>930000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>858180</v>
+        <v>859465</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -12539,7 +12557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12588,7 +12606,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 16 M5 Max 18 Core CPU 40 Core GPU 128GB 8TB Silver</t>
+          <t>Apple MacBook Air 15 MDVK4 M5 10C CPU 10C GPU 16GB 1TB Midnight</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -12597,22 +12615,22 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>3186000</v>
+        <v>564999</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>3098000</v>
+        <v>552999</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-88000</v>
+        <v>-12000</v>
       </c>
       <c r="F2" t="n">
-        <v>-2.76</v>
+        <v>-2.12</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 CTO M5 Max 18 Core CPU 40 Core GPU 48GB 8TB Space Black</t>
+          <t>Apple MacBook Air 15 MDVA4 M5 10C CPU 10C GPU 16GB 1TB Silver</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -12621,22 +12639,22 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>2581000</v>
+        <v>564999</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>2499000</v>
+        <v>552999</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>-82000</v>
+        <v>-12000</v>
       </c>
       <c r="F3" t="n">
-        <v>-3.18</v>
+        <v>-2.12</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 CTO M5 Max 18 Core CPU 40 Core GPU 48GB 4TB Space Black</t>
+          <t>Apple MacBook Air 15 MDVE4 M5 10C CPU 10C GPU 16GB 1TB Starlight</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -12645,22 +12663,22 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>1945000</v>
+        <v>564999</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>1875000</v>
+        <v>552999</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>-70000</v>
+        <v>-12000</v>
       </c>
       <c r="F4" t="n">
-        <v>-3.6</v>
+        <v>-2.12</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 CTO M5 Max 18 Core CPU 32 Core GPU 36GB 8TB Space Black</t>
+          <t>Apple MacBook Air 15 MDVT4 M5 10C CPU 10C GPU 16GB 1TB Sky Blue</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -12669,22 +12687,22 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>2381000</v>
+        <v>564999</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>2315000</v>
+        <v>552999</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>-66000</v>
+        <v>-12000</v>
       </c>
       <c r="F5" t="n">
-        <v>-2.77</v>
+        <v>-2.12</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 64GB 4TB Silver</t>
+          <t>Apple MacBook Air 13 MDHF4 M5 10C CPU 10C GPU 16GB 1TB Midnight</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -12693,22 +12711,22 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>1790000</v>
+        <v>479999</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>1725000</v>
+        <v>474999</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-65000</v>
+        <v>-5000</v>
       </c>
       <c r="F6" t="n">
-        <v>-3.63</v>
+        <v>-1.04</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 16 M5 Max 18 Core CPU 40 Core GPU 128GB 4TB Silver</t>
+          <t>Apple MacBook Air 13 MDHJ4 M5 10C CPU 10C GPU 16GB 1TB Sky Blue</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -12717,22 +12735,22 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>2571000</v>
+        <v>479999</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>2510000</v>
+        <v>474999</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>-61000</v>
+        <v>-5000</v>
       </c>
       <c r="F7" t="n">
-        <v>-2.37</v>
+        <v>-1.04</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 16 M5 Max 18 Core CPU 40 Core GPU 128GB 2TB Silver</t>
+          <t>Apple MacBook Air 13 MDHC4 M5 10C CPU 10C GPU 16GB 1TB Starlight</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -12741,22 +12759,22 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>2268000</v>
+        <v>479999</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>2210000</v>
+        <v>474999</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>-58000</v>
+        <v>-5000</v>
       </c>
       <c r="F8" t="n">
-        <v>-2.56</v>
+        <v>-1.04</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 CTO M5 Max 18 Core CPU 40 Core GPU 64GB 4TB Space Black</t>
+          <t>Apple MacBook Air 13 MDH94 M5 10C CPU 10C GPU 24GB 1TB Silver</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -12765,22 +12783,22 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>2078000</v>
+        <v>551999</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>2020000</v>
+        <v>547999</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>-58000</v>
+        <v>-4000</v>
       </c>
       <c r="F9" t="n">
-        <v>-2.79</v>
+        <v>-0.72</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 CTO M5 Max 18 Core CPU 40 Core GPU 64GB 8TB Space Black</t>
+          <t>Apple MacBook Air 13 MDHE4 M5 10C CPU 8C GPU 16GB 512GB Midnight</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -12789,22 +12807,22 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>2664000</v>
+        <v>425000</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>2610000</v>
+        <v>422000</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>-54000</v>
+        <v>-3000</v>
       </c>
       <c r="F10" t="n">
-        <v>-2.03</v>
+        <v>-0.71</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 64GB 2TB Silver</t>
+          <t>Apple MacBook Air 13 MDHH4 M5 10C CPU 8C GPU 16GB 512GB Sky Blue</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -12813,22 +12831,22 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>1471000</v>
+        <v>425000</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>1420000</v>
+        <v>422000</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>-51000</v>
+        <v>-3000</v>
       </c>
       <c r="F11" t="n">
-        <v>-3.47</v>
+        <v>-0.71</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 16 CTO M5 Max 18 Core CPU 40 Core GPU 64GB 2TB Space Black</t>
+          <t>Apple MacBook Air 13 MDHA4 M5 10C CPU 8C GPU 16GB 512GB Starlight</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -12837,22 +12855,22 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>1756000</v>
+        <v>425000</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>1705000</v>
+        <v>422000</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>-51000</v>
+        <v>-3000</v>
       </c>
       <c r="F12" t="n">
-        <v>-2.9</v>
+        <v>-0.71</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 14Inch MX2E3 M4 Pro 12Core CPU 16Core GPU 24GB 512GB Silver</t>
+          <t>Apple MacBook Air 13 MDHG4 M5 10C CPU 10C GPU 24GB 1TB Midnight</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -12861,22 +12879,22 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>650000</v>
+        <v>549999</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>600000</v>
+        <v>547999</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>-50000</v>
+        <v>-2000</v>
       </c>
       <c r="F13" t="n">
-        <v>-7.69</v>
+        <v>-0.36</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 14Inch MX2H3 M4 Pro 12Core CPU 16Core GPU 24GB 512GB Space Black</t>
+          <t>Apple MacBook Air 13 MDHK4 M5 10C CPU 10C GPU 24GB 1TB Sky Blue</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -12885,22 +12903,22 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>650000</v>
+        <v>549999</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>600000</v>
+        <v>547999</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>-50000</v>
+        <v>-2000</v>
       </c>
       <c r="F14" t="n">
-        <v>-7.69</v>
+        <v>-0.36</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 48GB 4TB Silver</t>
+          <t>Apple MacBook Air 13 MDHD4 M5 10C CPU 10C GPU 24GB 1TB Starlight</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -12909,285 +12927,45 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>1661000</v>
+        <v>549999</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>1615000</v>
+        <v>547999</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>-46000</v>
+        <v>-2000</v>
       </c>
       <c r="F15" t="n">
-        <v>-2.77</v>
+        <v>-0.36</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 24GB 4TB Space Black</t>
+          <t>Apple MacBook Pro 14Inch MX2E3 M4 Pro 12Core CPU 16Core GPU 24GB 512GB Silver</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>1471000</v>
+        <v>600000</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>1430000</v>
+        <v>640000</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>-41000</v>
+        <v>40000</v>
       </c>
       <c r="F16" t="n">
-        <v>-2.79</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 48GB 2TB Silver</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="n">
-        <v>1338000</v>
-      </c>
-      <c r="D17" s="3" t="n">
-        <v>1298000</v>
-      </c>
-      <c r="E17" s="3" t="n">
-        <v>-40000</v>
-      </c>
-      <c r="F17" t="n">
-        <v>-2.99</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 24GB 2TB Space Black</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="n">
-        <v>1150000</v>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>1115000</v>
-      </c>
-      <c r="E18" s="3" t="n">
-        <v>-35000</v>
-      </c>
-      <c r="F18" t="n">
-        <v>-3.04</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Apple MacBook Pro 16Inch MX2V3 14Core CPU 32Core GPU M4 Max 36GB 1TB Silver</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="n">
-        <v>1022000</v>
-      </c>
-      <c r="D19" s="3" t="n">
-        <v>995000</v>
-      </c>
-      <c r="E19" s="3" t="n">
-        <v>-27000</v>
-      </c>
-      <c r="F19" t="n">
-        <v>-2.64</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Macbook Pro 16 CTO M5 Max 18 Core CPU 32 Core GPU 36GB 4TB Space Black</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="n">
-        <v>1711000</v>
-      </c>
-      <c r="D20" s="3" t="n">
-        <v>1690000</v>
-      </c>
-      <c r="E20" s="3" t="n">
-        <v>-21000</v>
-      </c>
-      <c r="F20" t="n">
-        <v>-1.23</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Macbook Pro 16 MGE94 M5 Max 18 Core CPU 40 Core GPU 48GB 2TB Silver</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="n">
-        <v>1450000</v>
-      </c>
-      <c r="D21" s="3" t="n">
-        <v>1430000</v>
-      </c>
-      <c r="E21" s="3" t="n">
-        <v>-20000</v>
-      </c>
-      <c r="F21" t="n">
-        <v>-1.38</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Macbook Pro 16 MGEE4 M5 Max 18 Core CPU 40 Core GPU 48GB 2TB Space Black</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="n">
-        <v>1450000</v>
-      </c>
-      <c r="D22" s="3" t="n">
-        <v>1430000</v>
-      </c>
-      <c r="E22" s="3" t="n">
-        <v>-20000</v>
-      </c>
-      <c r="F22" t="n">
-        <v>-1.38</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Macbook Pro 16 MGE44 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Silver</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="n">
-        <v>840000</v>
-      </c>
-      <c r="D23" s="3" t="n">
-        <v>829999</v>
-      </c>
-      <c r="E23" s="3" t="n">
-        <v>-10001</v>
-      </c>
-      <c r="F23" t="n">
-        <v>-1.19</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 64GB 1TB Silver</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="n">
-        <v>1310000</v>
-      </c>
-      <c r="D24" s="3" t="n">
-        <v>1300000</v>
-      </c>
-      <c r="E24" s="3" t="n">
-        <v>-10000</v>
-      </c>
-      <c r="F24" t="n">
-        <v>-0.76</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Apple MacBook Pro 16Inch MX2X3 14Core CPU 20Core GPU M4 Pro 24GB 512GB Space Black</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="n">
-        <v>707999</v>
-      </c>
-      <c r="D25" s="3" t="n">
-        <v>711999</v>
-      </c>
-      <c r="E25" s="3" t="n">
-        <v>4000</v>
-      </c>
-      <c r="F25" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Apple MacBook Pro 16Inch MX303 14Core CPU 32Core GPU M4 Max 36GB 1TB Space Black</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="n">
-        <v>970000</v>
-      </c>
-      <c r="D26" s="3" t="n">
-        <v>995000</v>
-      </c>
-      <c r="E26" s="3" t="n">
-        <v>25000</v>
-      </c>
-      <c r="F26" t="n">
-        <v>2.58</v>
+        <v>6.67</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F26"/>
-  <conditionalFormatting sqref="E2:E26">
+  <autoFilter ref="A1:F16"/>
+  <conditionalFormatting sqref="E2:E16">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
chore: price data 2026-09-27
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MacBook Pro'!$A$1:$S$93</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MacBook Air'!$A$1:$S$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20260926T083940619332+0000</t>
+          <t>20260927T092004702594+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-26T08:39:40.619332+00:00</t>
+          <t>2026-09-27T09:20:04.702594+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>276.956128</v>
+        <v>277.004436</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -612,7 +612,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 24GB 4TB Silver</t>
+          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 48GB 4TB Space Black</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -621,19 +621,19 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>1260000</v>
+        <v>1445000</v>
       </c>
       <c r="D17" t="n">
-        <v>92.59999999999999</v>
+        <v>59.1</v>
       </c>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 48GB 4TB Space Black</t>
+          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 48GB 2TB Space Black</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -642,10 +642,10 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>1445000</v>
+        <v>1155000</v>
       </c>
       <c r="D18" t="n">
-        <v>59.1</v>
+        <v>54.6</v>
       </c>
       <c r="E18" t="n">
         <v>3</v>
@@ -654,7 +654,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 48GB 2TB Space Black</t>
+          <t>Macbook Pro 14 MJLW4 M5 Pro 15 Core CPU 16 Core GPU 24GB 2TB Space Black</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>1155000</v>
+        <v>790000</v>
       </c>
       <c r="D19" t="n">
         <v>54.6</v>
@@ -675,7 +675,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 MJLW4 M5 Pro 15 Core CPU 16 Core GPU 24GB 2TB Space Black</t>
+          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 24GB 4TB Silver</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -684,10 +684,10 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>790000</v>
+        <v>1260000</v>
       </c>
       <c r="D20" t="n">
-        <v>54.6</v>
+        <v>54</v>
       </c>
       <c r="E20" t="n">
         <v>3</v>
@@ -822,7 +822,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 MJ3D4 10 Core CPU 10 Core GPU 32GB 1TB Space Black</t>
+          <t>Macbook Pro 14 M5 MDE34 10 Core CPU 10 Core GPU 24GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -831,10 +831,10 @@
         </is>
       </c>
       <c r="C27" s="3" t="n">
-        <v>745000</v>
+        <v>643999</v>
       </c>
       <c r="D27" t="n">
-        <v>44.9</v>
+        <v>44.4</v>
       </c>
       <c r="E27" t="n">
         <v>4</v>
@@ -843,7 +843,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 MDE34 10 Core CPU 10 Core GPU 24GB 1TB Space Black</t>
+          <t>Macbook Pro 14 MGDR4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -852,19 +852,19 @@
         </is>
       </c>
       <c r="C28" s="3" t="n">
-        <v>643999</v>
+        <v>720000</v>
       </c>
       <c r="D28" t="n">
         <v>44.4</v>
       </c>
       <c r="E28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 MGDR4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Space Black</t>
+          <t>Macbook Pro 14 MJLV4 M5 Pro 15 Core CPU 16 Core GPU 24GB 2TB Silver</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -873,10 +873,10 @@
         </is>
       </c>
       <c r="C29" s="3" t="n">
-        <v>720000</v>
+        <v>815000</v>
       </c>
       <c r="D29" t="n">
-        <v>44.4</v>
+        <v>43.6</v>
       </c>
       <c r="E29" t="n">
         <v>3</v>
@@ -885,7 +885,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 MJLV4 M5 Pro 15 Core CPU 16 Core GPU 24GB 2TB Silver</t>
+          <t>Macbook Pro 14 MGDN4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Silver</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -894,10 +894,10 @@
         </is>
       </c>
       <c r="C30" s="3" t="n">
-        <v>815000</v>
+        <v>725000</v>
       </c>
       <c r="D30" t="n">
-        <v>43.6</v>
+        <v>43.1</v>
       </c>
       <c r="E30" t="n">
         <v>3</v>
@@ -906,7 +906,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 MGDN4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Silver</t>
+          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 32GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -915,13 +915,13 @@
         </is>
       </c>
       <c r="C31" s="3" t="n">
-        <v>725000</v>
+        <v>772000</v>
       </c>
       <c r="D31" t="n">
-        <v>43.1</v>
+        <v>42.2</v>
       </c>
       <c r="E31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="33">
@@ -1147,10 +1147,10 @@
         <v>470000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>686422</v>
+        <v>686542</v>
       </c>
       <c r="L2" t="n">
-        <v>35.17107551914129</v>
+        <v>35.18240690300083</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1214,10 +1214,10 @@
         <v>465000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>686422</v>
+        <v>686542</v>
       </c>
       <c r="L3" t="n">
-        <v>33.27719682644204</v>
+        <v>33.28885923949299</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>772278</v>
+        <v>772413</v>
       </c>
       <c r="L4" t="n">
-        <v>35.25660448698525</v>
+        <v>35.26792014116801</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>772278</v>
+        <v>772413</v>
       </c>
       <c r="L5" t="n">
-        <v>32.66686348698266</v>
+        <v>32.67863176823798</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>858135</v>
+        <v>858284</v>
       </c>
       <c r="L6" t="n">
-        <v>38.00509243883538</v>
+        <v>38.01585489185398</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1606,10 +1606,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>858135</v>
+        <v>858284</v>
       </c>
       <c r="L9" t="n">
-        <v>34.15954366154509</v>
+        <v>34.17097371033364</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1673,10 +1673,10 @@
         <v>582999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>858135</v>
+        <v>858284</v>
       </c>
       <c r="L10" t="n">
-        <v>32.06208813298607</v>
+        <v>32.07388230469169</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -1740,10 +1740,10 @@
         <v>587999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>858135</v>
+        <v>858284</v>
       </c>
       <c r="L11" t="n">
-        <v>31.47942922733603</v>
+        <v>31.49132454991588</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -1807,10 +1807,10 @@
         <v>600000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>858135</v>
+        <v>858284</v>
       </c>
       <c r="L12" t="n">
-        <v>30.08093132199479</v>
+        <v>30.09306942690299</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -1822,10 +1822,10 @@
         <v>100</v>
       </c>
       <c r="P12" t="n">
-        <v>50</v>
+        <v>45.94594594594595</v>
       </c>
       <c r="Q12" t="n">
-        <v>42.7</v>
+        <v>42</v>
       </c>
       <c r="R12" t="n">
         <v>4</v>
@@ -1868,22 +1868,22 @@
         </is>
       </c>
       <c r="I13" s="3" t="n">
-        <v>640000</v>
+        <v>634000</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>640000</v>
+        <v>634000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>858135</v>
+        <v>858284</v>
       </c>
       <c r="L13" t="n">
-        <v>25.41966007679444</v>
+        <v>26.13167669442749</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>0</v>
+        <v>-6000</v>
       </c>
       <c r="N13" t="n">
-        <v>1.538461538461539</v>
+        <v>2.461538461538462</v>
       </c>
       <c r="O13" t="n">
         <v>0</v>
@@ -1892,7 +1892,7 @@
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>8.9</v>
+        <v>9.4</v>
       </c>
       <c r="R13" t="n">
         <v>4</v>
@@ -1941,10 +1941,10 @@
         <v>643999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>943991</v>
+        <v>944156</v>
       </c>
       <c r="L14" t="n">
-        <v>31.77911653818733</v>
+        <v>31.79103876901698</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -2067,10 +2067,10 @@
         <v>650000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>943991</v>
+        <v>944156</v>
       </c>
       <c r="L16" t="n">
-        <v>31.14341132489611</v>
+        <v>31.15544465109579</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -2134,10 +2134,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1029848</v>
+        <v>1030027</v>
       </c>
       <c r="L17" t="n">
-        <v>32.02880425072438</v>
+        <v>32.04061641102612</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2201,10 +2201,10 @@
         <v>711999</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>1072776</v>
+        <v>1072963</v>
       </c>
       <c r="L18" t="n">
-        <v>33.6302266269939</v>
+        <v>33.6417937990406</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -2330,10 +2330,10 @@
         <v>720000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>1029848</v>
+        <v>1030027</v>
       </c>
       <c r="L20" t="n">
-        <v>30.08677008645936</v>
+        <v>30.09891973705544</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -2345,10 +2345,10 @@
         <v>0</v>
       </c>
       <c r="P20" t="n">
-        <v>80</v>
+        <v>78.37837837837837</v>
       </c>
       <c r="Q20" t="n">
-        <v>23.4</v>
+        <v>23.1</v>
       </c>
       <c r="R20" t="n">
         <v>4</v>
@@ -2459,10 +2459,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1072776</v>
+        <v>1072963</v>
       </c>
       <c r="L22" t="n">
-        <v>30.74043416332953</v>
+        <v>30.75250497920245</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2477,7 +2477,7 @@
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>10.2</v>
+        <v>10.3</v>
       </c>
       <c r="R22" t="n">
         <v>4</v>
@@ -2491,7 +2491,7 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 MJ3D4 10 Core CPU 10 Core GPU 32GB 1TB Space Black</t>
+          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 32GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -2520,31 +2520,31 @@
         </is>
       </c>
       <c r="I23" s="3" t="n">
-        <v>745000</v>
+        <v>772000</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>745000</v>
+        <v>772000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1029848</v>
+        <v>1030027</v>
       </c>
       <c r="L23" t="n">
-        <v>27.65922738112809</v>
+        <v>25.05050838473166</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>3.49740932642487</v>
+        <v>0</v>
       </c>
       <c r="O23" t="n">
         <v>100</v>
       </c>
       <c r="P23" t="n">
-        <v>74.99999999999999</v>
+        <v>69.59999999999998</v>
       </c>
       <c r="Q23" t="n">
-        <v>44.9</v>
+        <v>42.2</v>
       </c>
       <c r="R23" t="n">
         <v>4</v>
@@ -2587,31 +2587,31 @@
         </is>
       </c>
       <c r="I24" s="3" t="n">
-        <v>755000</v>
+        <v>775000</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>755000</v>
+        <v>775000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1029848</v>
+        <v>1030027</v>
       </c>
       <c r="L24" t="n">
-        <v>26.68821029899558</v>
+        <v>24.75925388363606</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="N24" t="n">
-        <v>2.202072538860103</v>
+        <v>0</v>
       </c>
       <c r="O24" t="n">
-        <v>62.96296296296296</v>
+        <v>0</v>
       </c>
       <c r="P24" t="n">
-        <v>73</v>
+        <v>68.99999999999999</v>
       </c>
       <c r="Q24" t="n">
-        <v>35.7</v>
+        <v>19.8</v>
       </c>
       <c r="R24" t="n">
         <v>4</v>
@@ -2625,7 +2625,7 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 32GB 1TB Space Black</t>
+          <t>Macbook Pro 14 M5 MJ3D4 10 Core CPU 10 Core GPU 32GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -2654,19 +2654,19 @@
         </is>
       </c>
       <c r="I25" s="3" t="n">
-        <v>772000</v>
+        <v>775000</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>772000</v>
+        <v>775000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>1029848</v>
+        <v>1030027</v>
       </c>
       <c r="L25" t="n">
-        <v>25.03748125937031</v>
+        <v>24.75925388363606</v>
       </c>
       <c r="M25" s="3" t="n">
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="N25" t="n">
         <v>0</v>
@@ -2675,10 +2675,10 @@
         <v>0</v>
       </c>
       <c r="P25" t="n">
-        <v>69.59999999999998</v>
+        <v>68.99999999999999</v>
       </c>
       <c r="Q25" t="n">
-        <v>19.9</v>
+        <v>19.8</v>
       </c>
       <c r="R25" t="n">
         <v>4</v>
@@ -2789,13 +2789,13 @@
         <v>810000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>1072776</v>
+        <v>1072963</v>
       </c>
       <c r="L27" t="n">
-        <v>24.49495514441039</v>
+        <v>24.5081144456985</v>
       </c>
       <c r="M27" s="3" t="n">
-        <v>-20000</v>
+        <v>0</v>
       </c>
       <c r="N27" t="n">
         <v>2.994011976047904</v>
@@ -2853,10 +2853,10 @@
         <v>810000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>1244489</v>
+        <v>1244706</v>
       </c>
       <c r="L28" t="n">
-        <v>34.9130446311699</v>
+        <v>34.92439178408395</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -2982,10 +2982,10 @@
         <v>825000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1287417</v>
+        <v>1287641</v>
       </c>
       <c r="L30" t="n">
-        <v>35.91819899845971</v>
+        <v>35.9293467666842</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -3000,7 +3000,7 @@
         <v>1.718244359164265</v>
       </c>
       <c r="Q30" t="n">
-        <v>34.7</v>
+        <v>34.8</v>
       </c>
       <c r="R30" t="n">
         <v>4</v>
@@ -3049,10 +3049,10 @@
         <v>829999</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1287417</v>
+        <v>1287641</v>
       </c>
       <c r="L31" t="n">
-        <v>35.52990212184552</v>
+        <v>35.54111743878923</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -3116,10 +3116,10 @@
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1373273</v>
+        <v>1373513</v>
       </c>
       <c r="L32" t="n">
-        <v>38.24978718725264</v>
+        <v>38.26057707498946</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3183,10 +3183,10 @@
         <v>930000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1373273</v>
+        <v>1373513</v>
       </c>
       <c r="L33" t="n">
-        <v>38.10414972114067</v>
+        <v>38.11496505675592</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3250,10 +3250,10 @@
         <v>860000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>1244489</v>
+        <v>1244706</v>
       </c>
       <c r="L34" t="n">
-        <v>30.89533133679767</v>
+        <v>30.90737893124963</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -3503,10 +3503,10 @@
         <v>880000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>1158632</v>
+        <v>1158834</v>
       </c>
       <c r="L38" t="n">
-        <v>24.04836048029055</v>
+        <v>24.0615998495039</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -3567,10 +3567,10 @@
         <v>940000</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>1244489</v>
+        <v>1244706</v>
       </c>
       <c r="L39" t="n">
-        <v>24.46699006580211</v>
+        <v>24.48015836671471</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -3596,55 +3596,57 @@
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 48GB 1TB Space Black</t>
+          <t>Apple MacBook Pro 16Inch MX2V3 14Core CPU 32Core GPU M4 Max 36GB 1TB Silver</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>M5 Pro</t>
+          <t>M4 Max</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="E40" t="n">
         <v>1024</v>
       </c>
       <c r="F40" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G40" t="n">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I40" s="3" t="n">
-        <v>995000</v>
+        <v>990000</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>995000</v>
-      </c>
-      <c r="K40" s="3" t="n"/>
+        <v>990000</v>
+      </c>
+      <c r="K40" s="3" t="n">
+        <v>1502320</v>
+      </c>
+      <c r="L40" t="n">
+        <v>34.10192236008307</v>
+      </c>
       <c r="M40" s="3" t="n">
-        <v>0</v>
+        <v>-5000</v>
       </c>
       <c r="N40" t="n">
-        <v>2.450980392156863</v>
-      </c>
-      <c r="O40" t="n">
-        <v>100</v>
+        <v>3.131115459882583</v>
       </c>
       <c r="P40" t="n">
-        <v>69.23076923076923</v>
+        <v>39.19647231749141</v>
       </c>
       <c r="Q40" t="n">
-        <v>51.7</v>
+        <v>24.1</v>
       </c>
       <c r="R40" t="n">
         <v>3</v>
@@ -3658,7 +3660,7 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 16Inch MX2V3 14Core CPU 32Core GPU M4 Max 36GB 1TB Silver</t>
+          <t>Apple MacBook Pro 16Inch MX303 14Core CPU 32Core GPU M4 Max 36GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -3683,29 +3685,29 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I41" s="3" t="n">
-        <v>995000</v>
+        <v>990000</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>995000</v>
+        <v>990000</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>1502058</v>
+        <v>1502320</v>
       </c>
       <c r="L41" t="n">
-        <v>33.75755130627446</v>
+        <v>34.10192236008307</v>
       </c>
       <c r="M41" s="3" t="n">
-        <v>0</v>
+        <v>-5000</v>
       </c>
       <c r="N41" t="n">
-        <v>2.64187866927593</v>
+        <v>0</v>
       </c>
       <c r="P41" t="n">
-        <v>35.27682508574235</v>
+        <v>39.19647231749141</v>
       </c>
       <c r="Q41" t="n">
         <v>23</v>
@@ -3722,28 +3724,28 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 16Inch MX303 14Core CPU 32Core GPU M4 Max 36GB 1TB Space Black</t>
+          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 48GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>M4 Max</t>
+          <t>M5 Pro</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="E42" t="n">
         <v>1024</v>
       </c>
       <c r="F42" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G42" t="n">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -3756,23 +3758,21 @@
       <c r="J42" s="3" t="n">
         <v>995000</v>
       </c>
-      <c r="K42" s="3" t="n">
-        <v>1502058</v>
-      </c>
-      <c r="L42" t="n">
-        <v>33.75755130627446</v>
-      </c>
+      <c r="K42" s="3" t="n"/>
       <c r="M42" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N42" t="n">
-        <v>0</v>
+        <v>2.450980392156863</v>
+      </c>
+      <c r="O42" t="n">
+        <v>100</v>
       </c>
       <c r="P42" t="n">
-        <v>35.27682508574235</v>
+        <v>69.23076923076923</v>
       </c>
       <c r="Q42" t="n">
-        <v>22</v>
+        <v>51.7</v>
       </c>
       <c r="R42" t="n">
         <v>3</v>
@@ -3821,10 +3821,10 @@
         <v>1055000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1544986</v>
+        <v>1545255</v>
       </c>
       <c r="L43" t="n">
-        <v>31.71459158853219</v>
+        <v>31.72647880123345</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -3885,10 +3885,10 @@
         <v>1055000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1544986</v>
+        <v>1545255</v>
       </c>
       <c r="L44" t="n">
-        <v>31.71459158853219</v>
+        <v>31.72647880123345</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -3900,7 +3900,7 @@
         <v>58.64647440248988</v>
       </c>
       <c r="Q44" t="n">
-        <v>27.1</v>
+        <v>27.2</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -4011,10 +4011,10 @@
         <v>1115000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1502058</v>
+        <v>1502320</v>
       </c>
       <c r="L46" t="n">
-        <v>25.7685122678352</v>
+        <v>25.78145801160871</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -4075,10 +4075,10 @@
         <v>1123000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1716699</v>
+        <v>1716998</v>
       </c>
       <c r="L47" t="n">
-        <v>34.58375638361763</v>
+        <v>34.59514804327087</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -4142,10 +4142,10 @@
         <v>1130000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1502058</v>
+        <v>1502320</v>
       </c>
       <c r="L48" t="n">
-        <v>24.76988238803029</v>
+        <v>24.78300228979179</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -4268,10 +4268,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1759627</v>
+        <v>1759934</v>
       </c>
       <c r="L50" t="n">
-        <v>34.36108902625386</v>
+        <v>34.37253897021138</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4332,10 +4332,10 @@
         <v>1155000</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>1759627</v>
+        <v>1759934</v>
       </c>
       <c r="L51" t="n">
-        <v>34.36108902625386</v>
+        <v>34.37253897021138</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -4396,10 +4396,10 @@
         <v>1185000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1587914</v>
+        <v>1588191</v>
       </c>
       <c r="L52" t="n">
-        <v>25.37379228346119</v>
+        <v>25.38680800986783</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -4460,10 +4460,10 @@
         <v>1185000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1587914</v>
+        <v>1588191</v>
       </c>
       <c r="L53" t="n">
-        <v>25.37379228346119</v>
+        <v>25.38680800986783</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -4524,16 +4524,16 @@
         <v>1200000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1888412</v>
+        <v>1888741</v>
       </c>
       <c r="L54" t="n">
-        <v>36.4545448768595</v>
+        <v>36.46561386659155</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N54" t="n">
-        <v>0.6211180124223602</v>
+        <v>0.579950289975145</v>
       </c>
       <c r="P54" t="n">
         <v>3.948101568096777</v>
@@ -4588,16 +4588,16 @@
         <v>1200000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1888412</v>
+        <v>1888741</v>
       </c>
       <c r="L55" t="n">
-        <v>36.4545448768595</v>
+        <v>36.46561386659155</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N55" t="n">
-        <v>0.703351261894911</v>
+        <v>0.579950289975145</v>
       </c>
       <c r="P55" t="n">
         <v>3.948101568096777</v>
@@ -4714,10 +4714,10 @@
         <v>1240000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1673771</v>
+        <v>1674062</v>
       </c>
       <c r="L57" t="n">
-        <v>25.91579134780087</v>
+        <v>25.92866930854413</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -4778,7 +4778,12 @@
         <v>1260000</v>
       </c>
       <c r="K58" s="3" t="n"/>
-      <c r="M58" s="3" t="n"/>
+      <c r="M58" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N58" t="n">
+        <v>0</v>
+      </c>
       <c r="O58" t="n">
         <v>100</v>
       </c>
@@ -4786,10 +4791,10 @@
         <v>82.67288267288268</v>
       </c>
       <c r="Q58" t="n">
-        <v>92.59999999999999</v>
+        <v>54</v>
       </c>
       <c r="R58" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S58" t="inlineStr">
         <is>
@@ -4835,10 +4840,10 @@
         <v>1280000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1716699</v>
+        <v>1716998</v>
       </c>
       <c r="L59" t="n">
-        <v>25.43829756992927</v>
+        <v>25.45128183026421</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -4902,10 +4907,10 @@
         <v>1298000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1759627</v>
+        <v>1759934</v>
       </c>
       <c r="L60" t="n">
-        <v>26.23436671521862</v>
+        <v>26.24723427128518</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -4966,10 +4971,10 @@
         <v>1300000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1716699</v>
+        <v>1716998</v>
       </c>
       <c r="L61" t="n">
-        <v>24.27327096945941</v>
+        <v>24.28645810886209</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -5092,10 +5097,10 @@
         <v>1335000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1802555</v>
+        <v>1802870</v>
       </c>
       <c r="L63" t="n">
-        <v>25.93845957543598</v>
+        <v>25.95139971268034</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -5156,10 +5161,10 @@
         <v>1420000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1931340</v>
+        <v>1931677</v>
       </c>
       <c r="L64" t="n">
-        <v>26.47591827435873</v>
+        <v>26.48874527159562</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -5220,10 +5225,10 @@
         <v>1430000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1931340</v>
+        <v>1931677</v>
       </c>
       <c r="L65" t="n">
-        <v>25.95814305093873</v>
+        <v>25.97106037914206</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -5284,10 +5289,10 @@
         <v>1430000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>2145981</v>
+        <v>2146355</v>
       </c>
       <c r="L66" t="n">
-        <v>33.36380890604344</v>
+        <v>33.37542018911131</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -5348,10 +5353,10 @@
         <v>1430000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>2145981</v>
+        <v>2146355</v>
       </c>
       <c r="L67" t="n">
-        <v>33.36380890604344</v>
+        <v>33.37542018911131</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -5474,10 +5479,10 @@
         <v>1480000</v>
       </c>
       <c r="K69" s="3" t="n">
-        <v>2017196</v>
+        <v>2017548</v>
       </c>
       <c r="L69" t="n">
-        <v>26.63082813965524</v>
+        <v>26.6436288009009</v>
       </c>
       <c r="M69" s="3" t="n">
         <v>0</v>
@@ -5600,10 +5605,10 @@
         <v>1605000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2188909</v>
+        <v>2189291</v>
       </c>
       <c r="L71" t="n">
-        <v>26.67580059289811</v>
+        <v>26.68859461807498</v>
       </c>
       <c r="M71" s="3" t="n">
         <v>0</v>
@@ -5664,10 +5669,10 @@
         <v>1610000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2188909</v>
+        <v>2189291</v>
       </c>
       <c r="L72" t="n">
-        <v>26.44737629567972</v>
+        <v>26.46021017763285</v>
       </c>
       <c r="M72" s="3" t="n">
         <v>0</v>
@@ -5728,10 +5733,10 @@
         <v>1615000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2188909</v>
+        <v>2189291</v>
       </c>
       <c r="L73" t="n">
-        <v>26.21895199846133</v>
+        <v>26.23182573719072</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
@@ -5792,10 +5797,10 @@
         <v>1630000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2231837</v>
+        <v>2232226</v>
       </c>
       <c r="L74" t="n">
-        <v>26.9659925881684</v>
+        <v>26.97871989664129</v>
       </c>
       <c r="M74" s="3" t="n">
         <v>0</v>
@@ -5807,7 +5812,7 @@
         <v>100</v>
       </c>
       <c r="Q74" t="n">
-        <v>34</v>
+        <v>34.1</v>
       </c>
       <c r="R74" t="n">
         <v>3</v>
@@ -5856,10 +5861,10 @@
         <v>1690000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2317694</v>
+        <v>2318098</v>
       </c>
       <c r="L75" t="n">
-        <v>27.08269512713931</v>
+        <v>27.0954032141868</v>
       </c>
       <c r="M75" s="3" t="n">
         <v>0</v>
@@ -5920,10 +5925,10 @@
         <v>1705000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2317694</v>
+        <v>2318098</v>
       </c>
       <c r="L76" t="n">
-        <v>26.43550011347486</v>
+        <v>26.44832099419438</v>
       </c>
       <c r="M76" s="3" t="n">
         <v>0</v>
@@ -5984,10 +5989,10 @@
         <v>1725000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2360622</v>
+        <v>2361033</v>
       </c>
       <c r="L77" t="n">
-        <v>26.92603898464049</v>
+        <v>26.93875943284148</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
@@ -6048,10 +6053,10 @@
         <v>1780000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2446478</v>
+        <v>2446905</v>
       </c>
       <c r="L78" t="n">
-        <v>27.24234593566752</v>
+        <v>27.25504259462464</v>
       </c>
       <c r="M78" s="3" t="n">
         <v>0</v>
@@ -6112,10 +6117,10 @@
         <v>1875000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2575263</v>
+        <v>2575712</v>
       </c>
       <c r="L79" t="n">
-        <v>27.19190234162491</v>
+        <v>27.2045943024686</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
@@ -6127,7 +6132,7 @@
         <v>19.64044075004835</v>
       </c>
       <c r="Q79" t="n">
-        <v>17.1</v>
+        <v>17.2</v>
       </c>
       <c r="R79" t="n">
         <v>3</v>
@@ -6176,10 +6181,10 @@
         <v>1910000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2618191</v>
+        <v>2618648</v>
       </c>
       <c r="L80" t="n">
-        <v>27.04886694668189</v>
+        <v>27.06159819876516</v>
       </c>
       <c r="M80" s="3" t="n">
         <v>0</v>
@@ -6240,10 +6245,10 @@
         <v>2020000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2746976</v>
+        <v>2747455</v>
       </c>
       <c r="L81" t="n">
-        <v>26.46459233717368</v>
+        <v>26.4774127328746</v>
       </c>
       <c r="M81" s="3" t="n">
         <v>0</v>
@@ -6304,10 +6309,10 @@
         <v>2110000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>2875760</v>
+        <v>2876262</v>
       </c>
       <c r="L82" t="n">
-        <v>26.62809135671961</v>
+        <v>26.64089710881693</v>
       </c>
       <c r="M82" s="3" t="n">
         <v>0</v>
@@ -6368,10 +6373,10 @@
         <v>2210000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3004545</v>
+        <v>3005069</v>
       </c>
       <c r="L83" t="n">
-        <v>26.44476950752943</v>
+        <v>26.45759548283251</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
@@ -6432,10 +6437,10 @@
         <v>2215000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3047473</v>
+        <v>3048004</v>
       </c>
       <c r="L84" t="n">
-        <v>27.31682938618324</v>
+        <v>27.32949169358045</v>
       </c>
       <c r="M84" s="3" t="n">
         <v>0</v>
@@ -6496,10 +6501,10 @@
         <v>2315000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3176258</v>
+        <v>3176812</v>
       </c>
       <c r="L85" t="n">
-        <v>27.11549250722076</v>
+        <v>27.12820273909819</v>
       </c>
       <c r="M85" s="3" t="n">
         <v>0</v>
@@ -6560,10 +6565,10 @@
         <v>2395000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3305042</v>
+        <v>3305619</v>
       </c>
       <c r="L86" t="n">
-        <v>27.53496022138296</v>
+        <v>27.54760908622561</v>
       </c>
       <c r="M86" s="3" t="n">
         <v>0</v>
@@ -6624,10 +6629,10 @@
         <v>2410000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3305042</v>
+        <v>3305619</v>
       </c>
       <c r="L87" t="n">
-        <v>27.08110819771731</v>
+        <v>27.09383628300781</v>
       </c>
       <c r="M87" s="3" t="n">
         <v>0</v>
@@ -6688,10 +6693,10 @@
         <v>2499000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3433827</v>
+        <v>3434426</v>
       </c>
       <c r="L88" t="n">
-        <v>27.22405642450828</v>
+        <v>27.23674931415031</v>
       </c>
       <c r="M88" s="3" t="n">
         <v>0</v>
@@ -6703,7 +6708,7 @@
         <v>63.67326854471646</v>
       </c>
       <c r="Q88" t="n">
-        <v>26.4</v>
+        <v>26.5</v>
       </c>
       <c r="R88" t="n">
         <v>3</v>
@@ -6752,10 +6757,10 @@
         <v>2510000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3433827</v>
+        <v>3434426</v>
       </c>
       <c r="L89" t="n">
-        <v>26.90371413586066</v>
+        <v>26.91646289656554</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
@@ -6816,10 +6821,10 @@
         <v>2530000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3476755</v>
+        <v>3477361</v>
       </c>
       <c r="L90" t="n">
-        <v>27.23099556914422</v>
+        <v>27.24367702979357</v>
       </c>
       <c r="M90" s="3" t="n">
         <v>0</v>
@@ -6880,10 +6885,10 @@
         <v>2610000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>3605540</v>
+        <v>3606168</v>
       </c>
       <c r="L91" t="n">
-        <v>27.61139801527649</v>
+        <v>27.62400420612683</v>
       </c>
       <c r="M91" s="3" t="n">
         <v>0</v>
@@ -6895,7 +6900,7 @@
         <v>74.15426251691474</v>
       </c>
       <c r="Q91" t="n">
-        <v>28.4</v>
+        <v>28.5</v>
       </c>
       <c r="R91" t="n">
         <v>3</v>
@@ -6944,10 +6949,10 @@
         <v>3015000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4163606</v>
+        <v>4164332</v>
       </c>
       <c r="L92" t="n">
-        <v>27.58680816580627</v>
+        <v>27.59943251402626</v>
       </c>
       <c r="M92" s="3" t="n">
         <v>0</v>
@@ -7008,10 +7013,10 @@
         <v>3098000</v>
       </c>
       <c r="K93" s="3" t="n">
-        <v>4292391</v>
+        <v>4293139</v>
       </c>
       <c r="L93" t="n">
-        <v>27.82577356070312</v>
+        <v>27.83834858363543</v>
       </c>
       <c r="M93" s="3" t="n">
         <v>0</v>
@@ -7307,10 +7312,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>428853</v>
+        <v>428928</v>
       </c>
       <c r="L2" t="n">
-        <v>27.71439164468944</v>
+        <v>27.72703111011639</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7374,10 +7379,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>428853</v>
+        <v>428928</v>
       </c>
       <c r="L3" t="n">
-        <v>27.71439164468944</v>
+        <v>27.72703111011639</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7441,10 +7446,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>428853</v>
+        <v>428928</v>
       </c>
       <c r="L4" t="n">
-        <v>27.71415846455546</v>
+        <v>27.726797970755</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7508,10 +7513,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>428853</v>
+        <v>428928</v>
       </c>
       <c r="L5" t="n">
-        <v>27.71415846455546</v>
+        <v>27.726797970755</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7575,10 +7580,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514709</v>
+        <v>514799</v>
       </c>
       <c r="L6" t="n">
-        <v>25.39473760901791</v>
+        <v>25.40778051239416</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7639,10 +7644,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>514709</v>
+        <v>514799</v>
       </c>
       <c r="L7" t="n">
-        <v>25.39473760901791</v>
+        <v>25.40778051239416</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7703,10 +7708,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>514709</v>
+        <v>514799</v>
       </c>
       <c r="L8" t="n">
-        <v>25.39473760901791</v>
+        <v>25.40778051239416</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7767,10 +7772,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>514709</v>
+        <v>514799</v>
       </c>
       <c r="L9" t="n">
-        <v>25.39473760901791</v>
+        <v>25.40778051239416</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7831,10 +7836,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>514709</v>
+        <v>514799</v>
       </c>
       <c r="L10" t="n">
-        <v>25.2004530715414</v>
+        <v>25.21352994081185</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7895,10 +7900,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>514709</v>
+        <v>514799</v>
       </c>
       <c r="L11" t="n">
-        <v>25.2004530715414</v>
+        <v>25.21352994081185</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7959,10 +7964,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>514709</v>
+        <v>514799</v>
       </c>
       <c r="L12" t="n">
-        <v>25.2004530715414</v>
+        <v>25.21352994081185</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -8023,10 +8028,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>514709</v>
+        <v>514799</v>
       </c>
       <c r="L13" t="n">
-        <v>25.2004530715414</v>
+        <v>25.21352994081185</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -8081,31 +8086,31 @@
         </is>
       </c>
       <c r="I14" s="3" t="n">
-        <v>422000</v>
+        <v>420000</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>422000</v>
+        <v>420000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>557637</v>
+        <v>557735</v>
       </c>
       <c r="L14" t="n">
-        <v>24.32352946450827</v>
+        <v>24.69541986785839</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>0</v>
+        <v>-2000</v>
       </c>
       <c r="N14" t="n">
-        <v>4.524670870296086</v>
+        <v>4.977160581811272</v>
       </c>
       <c r="O14" t="n">
         <v>100</v>
       </c>
       <c r="P14" t="n">
-        <v>2.016806722689076</v>
+        <v>3.361344537815107</v>
       </c>
       <c r="Q14" t="n">
-        <v>31.9</v>
+        <v>32.4</v>
       </c>
       <c r="R14" t="n">
         <v>4</v>
@@ -8148,31 +8153,31 @@
         </is>
       </c>
       <c r="I15" s="3" t="n">
-        <v>422000</v>
+        <v>420000</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>422000</v>
+        <v>420000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>557637</v>
+        <v>557735</v>
       </c>
       <c r="L15" t="n">
-        <v>24.32352946450827</v>
+        <v>24.69541986785839</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>0</v>
+        <v>-2000</v>
       </c>
       <c r="N15" t="n">
-        <v>2.540190623996822</v>
+        <v>3.002085455162714</v>
       </c>
       <c r="O15" t="n">
         <v>100</v>
       </c>
       <c r="P15" t="n">
-        <v>2.016806722689076</v>
+        <v>3.361344537815107</v>
       </c>
       <c r="Q15" t="n">
-        <v>31.4</v>
+        <v>31.8</v>
       </c>
       <c r="R15" t="n">
         <v>4</v>
@@ -8215,31 +8220,31 @@
         </is>
       </c>
       <c r="I16" s="3" t="n">
-        <v>422000</v>
+        <v>420000</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>422000</v>
+        <v>420000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>557637</v>
+        <v>557735</v>
       </c>
       <c r="L16" t="n">
-        <v>24.32352946450827</v>
+        <v>24.69541986785839</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0</v>
+        <v>-2000</v>
       </c>
       <c r="N16" t="n">
-        <v>1.86046511627907</v>
+        <v>2.325581395348837</v>
       </c>
       <c r="O16" t="n">
         <v>100</v>
       </c>
       <c r="P16" t="n">
-        <v>2.016806722689076</v>
+        <v>3.361344537815107</v>
       </c>
       <c r="Q16" t="n">
-        <v>31.2</v>
+        <v>31.7</v>
       </c>
       <c r="R16" t="n">
         <v>4</v>
@@ -8288,10 +8293,10 @@
         <v>425000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>557637</v>
+        <v>557735</v>
       </c>
       <c r="L17" t="n">
-        <v>23.7855450768152</v>
+        <v>23.79893677104718</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -8355,10 +8360,10 @@
         <v>454000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>600566</v>
+        <v>600670</v>
       </c>
       <c r="L18" t="n">
-        <v>24.40464495159566</v>
+        <v>24.41773353089051</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -8419,10 +8424,10 @@
         <v>454000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>600566</v>
+        <v>600670</v>
       </c>
       <c r="L19" t="n">
-        <v>24.40464495159566</v>
+        <v>24.41773353089051</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -8483,10 +8488,10 @@
         <v>454000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>600566</v>
+        <v>600670</v>
       </c>
       <c r="L20" t="n">
-        <v>24.40464495159566</v>
+        <v>24.41773353089051</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -8547,10 +8552,10 @@
         <v>454000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>600566</v>
+        <v>600670</v>
       </c>
       <c r="L21" t="n">
-        <v>24.40464495159566</v>
+        <v>24.41773353089051</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -8611,10 +8616,10 @@
         <v>455000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>600566</v>
+        <v>600670</v>
       </c>
       <c r="L22" t="n">
-        <v>24.23813535897803</v>
+        <v>24.25125276774269</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -8675,10 +8680,10 @@
         <v>455000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>600566</v>
+        <v>600670</v>
       </c>
       <c r="L23" t="n">
-        <v>24.23813535897803</v>
+        <v>24.25125276774269</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -8739,10 +8744,10 @@
         <v>455000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>600566</v>
+        <v>600670</v>
       </c>
       <c r="L24" t="n">
-        <v>24.23813535897803</v>
+        <v>24.25125276774269</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -8803,10 +8808,10 @@
         <v>455000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>600566</v>
+        <v>600670</v>
       </c>
       <c r="L25" t="n">
-        <v>24.23813535897803</v>
+        <v>24.25125276774269</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -8867,10 +8872,10 @@
         <v>474999</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>686422</v>
+        <v>686542</v>
       </c>
       <c r="L26" t="n">
-        <v>30.80073191127324</v>
+        <v>30.81282718318763</v>
       </c>
       <c r="M26" s="3" t="n">
         <v>0</v>
@@ -8934,10 +8939,10 @@
         <v>474999</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>686422</v>
+        <v>686542</v>
       </c>
       <c r="L27" t="n">
-        <v>30.80073191127324</v>
+        <v>30.81282718318763</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -9001,10 +9006,10 @@
         <v>474999</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>686422</v>
+        <v>686542</v>
       </c>
       <c r="L28" t="n">
-        <v>30.80073191127324</v>
+        <v>30.81282718318763</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -9068,10 +9073,10 @@
         <v>475000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>686422</v>
+        <v>686542</v>
       </c>
       <c r="L29" t="n">
-        <v>30.80058622829688</v>
+        <v>30.81268152567505</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -9132,10 +9137,10 @@
         <v>475000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>686422</v>
+        <v>686542</v>
       </c>
       <c r="L30" t="n">
-        <v>30.80058622829688</v>
+        <v>30.81268152567505</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -9196,10 +9201,10 @@
         <v>475000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>686422</v>
+        <v>686542</v>
       </c>
       <c r="L31" t="n">
-        <v>30.80058622829688</v>
+        <v>30.81268152567505</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -9260,10 +9265,10 @@
         <v>475000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>686422</v>
+        <v>686542</v>
       </c>
       <c r="L32" t="n">
-        <v>30.80058622829688</v>
+        <v>30.81268152567505</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -9324,10 +9329,10 @@
         <v>479999</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>686422</v>
+        <v>686542</v>
       </c>
       <c r="L33" t="n">
-        <v>30.07231702946584</v>
+        <v>30.08453962029999</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -9391,10 +9396,10 @@
         <v>479999</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>643494</v>
+        <v>643606</v>
       </c>
       <c r="L34" t="n">
-        <v>25.4073853058459</v>
+        <v>25.42036587601731</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -9458,10 +9463,10 @@
         <v>479999</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>643494</v>
+        <v>643606</v>
       </c>
       <c r="L35" t="n">
-        <v>25.4073853058459</v>
+        <v>25.42036587601731</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
@@ -9525,10 +9530,10 @@
         <v>479999</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>643494</v>
+        <v>643606</v>
       </c>
       <c r="L36" t="n">
-        <v>25.4073853058459</v>
+        <v>25.42036587601731</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -9592,10 +9597,10 @@
         <v>484999</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>643494</v>
+        <v>643606</v>
       </c>
       <c r="L37" t="n">
-        <v>24.63037728401508</v>
+        <v>24.64349306874081</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
@@ -9659,10 +9664,10 @@
         <v>500000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>643494</v>
+        <v>643606</v>
       </c>
       <c r="L38" t="n">
-        <v>22.29919781691826</v>
+        <v>22.31271927234985</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -9723,10 +9728,10 @@
         <v>547999</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>772278</v>
+        <v>772413</v>
       </c>
       <c r="L39" t="n">
-        <v>29.04122608697904</v>
+        <v>29.05362804613594</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -9787,10 +9792,10 @@
         <v>547999</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>772278</v>
+        <v>772413</v>
       </c>
       <c r="L40" t="n">
-        <v>29.04122608697904</v>
+        <v>29.05362804613594</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -9851,10 +9856,10 @@
         <v>547999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>772278</v>
+        <v>772413</v>
       </c>
       <c r="L41" t="n">
-        <v>29.04122608697904</v>
+        <v>29.05362804613594</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
@@ -9866,7 +9871,7 @@
         <v>64.67267226890753</v>
       </c>
       <c r="Q41" t="n">
-        <v>26.9</v>
+        <v>27</v>
       </c>
       <c r="R41" t="n">
         <v>3</v>
@@ -9915,10 +9920,10 @@
         <v>547999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>772278</v>
+        <v>772413</v>
       </c>
       <c r="L42" t="n">
-        <v>29.04122608697904</v>
+        <v>29.05362804613594</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -9979,10 +9984,10 @@
         <v>552999</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>772278</v>
+        <v>772413</v>
       </c>
       <c r="L43" t="n">
-        <v>28.39379083697839</v>
+        <v>28.40630595290343</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -10043,10 +10048,10 @@
         <v>552999</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>772278</v>
+        <v>772413</v>
       </c>
       <c r="L44" t="n">
-        <v>28.39379083697839</v>
+        <v>28.40630595290343</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -10107,10 +10112,10 @@
         <v>552999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>772278</v>
+        <v>772413</v>
       </c>
       <c r="L45" t="n">
-        <v>28.39379083697839</v>
+        <v>28.40630595290343</v>
       </c>
       <c r="M45" s="3" t="n">
         <v>0</v>
@@ -10171,10 +10176,10 @@
         <v>552999</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>772278</v>
+        <v>772413</v>
       </c>
       <c r="L46" t="n">
-        <v>28.39379083697839</v>
+        <v>28.40630595290343</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -10235,10 +10240,10 @@
         <v>585000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>729350</v>
+        <v>729477</v>
       </c>
       <c r="L47" t="n">
-        <v>19.79159525604991</v>
+        <v>19.80555932537969</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -10299,10 +10304,10 @@
         <v>595000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>729350</v>
+        <v>729477</v>
       </c>
       <c r="L48" t="n">
-        <v>18.42051141427298</v>
+        <v>18.43471418564259</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -10363,10 +10368,10 @@
         <v>614999</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>858135</v>
+        <v>858284</v>
       </c>
       <c r="L49" t="n">
-        <v>28.33307113682579</v>
+        <v>28.34551267412651</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -10427,10 +10432,10 @@
         <v>614999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>858135</v>
+        <v>858284</v>
       </c>
       <c r="L50" t="n">
-        <v>28.33307113682579</v>
+        <v>28.34551267412651</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -10491,10 +10496,10 @@
         <v>614999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>858135</v>
+        <v>858284</v>
       </c>
       <c r="L51" t="n">
-        <v>28.33307113682579</v>
+        <v>28.34551267412651</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -10555,10 +10560,10 @@
         <v>614999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>858135</v>
+        <v>858284</v>
       </c>
       <c r="L52" t="n">
-        <v>28.33307113682579</v>
+        <v>28.34551267412651</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -10619,10 +10624,10 @@
         <v>650000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>815207</v>
+        <v>815349</v>
       </c>
       <c r="L53" t="n">
-        <v>20.26565031948941</v>
+        <v>20.27953673825564</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -10683,10 +10688,10 @@
         <v>672000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>858135</v>
+        <v>858284</v>
       </c>
       <c r="L54" t="n">
-        <v>21.69064308063417</v>
+        <v>21.70423775813134</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -10747,10 +10752,10 @@
         <v>700000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>901063</v>
+        <v>901220</v>
       </c>
       <c r="L55" t="n">
-        <v>22.3139780459302</v>
+        <v>22.32751159539291</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -10811,10 +10816,10 @@
         <v>715000</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>943991</v>
+        <v>944156</v>
       </c>
       <c r="L56" t="n">
-        <v>24.25775245738572</v>
+        <v>24.27098911620537</v>
       </c>
       <c r="M56" s="3" t="n">
         <v>0</v>
@@ -10875,10 +10880,10 @@
         <v>734999</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>986919</v>
+        <v>987091</v>
       </c>
       <c r="L57" t="n">
-        <v>25.525904354866</v>
+        <v>25.53888142025406</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -10939,10 +10944,10 @@
         <v>752000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>986919</v>
+        <v>987091</v>
       </c>
       <c r="L58" t="n">
-        <v>23.80327058248955</v>
+        <v>23.81654781575356</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -11003,10 +11008,10 @@
         <v>810000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1072776</v>
+        <v>1072963</v>
       </c>
       <c r="L59" t="n">
-        <v>24.49495514441039</v>
+        <v>24.5081144456985</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -11067,10 +11072,10 @@
         <v>815000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1072776</v>
+        <v>1072963</v>
       </c>
       <c r="L60" t="n">
-        <v>24.02887462061046</v>
+        <v>24.04211515215343</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -11131,10 +11136,10 @@
         <v>875000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1158632</v>
+        <v>1158834</v>
       </c>
       <c r="L61" t="n">
-        <v>24.47990388665254</v>
+        <v>24.49306803217717</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -11195,10 +11200,10 @@
         <v>992000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1330345</v>
+        <v>1330577</v>
       </c>
       <c r="L62" t="n">
-        <v>25.43287643430839</v>
+        <v>25.44587799127747</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -11259,10 +11264,10 @@
         <v>1050000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1416201</v>
+        <v>1416448</v>
       </c>
       <c r="L63" t="n">
-        <v>25.85798202373816</v>
+        <v>25.87091089824688</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -11323,10 +11328,10 @@
         <v>1050000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1416201</v>
+        <v>1416448</v>
       </c>
       <c r="L64" t="n">
-        <v>25.85798202373816</v>
+        <v>25.87091089824688</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -11387,10 +11392,10 @@
         <v>1100000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1502058</v>
+        <v>1502320</v>
       </c>
       <c r="L65" t="n">
-        <v>26.7671421476401</v>
+        <v>26.77991373342564</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -11451,10 +11456,10 @@
         <v>1105000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1502058</v>
+        <v>1502320</v>
       </c>
       <c r="L66" t="n">
-        <v>26.43426552103847</v>
+        <v>26.44709515948666</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -11515,10 +11520,10 @@
         <v>1155000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1587914</v>
+        <v>1588191</v>
       </c>
       <c r="L67" t="n">
-        <v>27.26306336489256</v>
+        <v>27.27574957923827</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -11785,7 +11790,7 @@
         <v>315000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>300068</v>
+        <v>300120</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -11846,10 +11851,10 @@
         <v>380000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>385925</v>
+        <v>385992</v>
       </c>
       <c r="L3" t="n">
-        <v>1.535272397486558</v>
+        <v>1.552363779560198</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -11910,7 +11915,7 @@
         <v>415000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>385925</v>
+        <v>385992</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -11971,10 +11976,10 @@
         <v>495000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>471781</v>
+        <v>471863</v>
       </c>
       <c r="L5" t="n">
-        <v>6.736600244605018</v>
+        <v>6.75280748861428</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -12035,10 +12040,10 @@
         <v>500000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514709</v>
+        <v>514799</v>
       </c>
       <c r="L6" t="n">
-        <v>8.686267386037548</v>
+        <v>8.702231356315766</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -12099,10 +12104,10 @@
         <v>550000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>557637</v>
+        <v>557735</v>
       </c>
       <c r="L7" t="n">
-        <v>6.749372799868015</v>
+        <v>6.765757931634199</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -12163,7 +12168,7 @@
         <v>530000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>471781</v>
+        <v>471863</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -12227,10 +12232,10 @@
         <v>600000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>600566</v>
+        <v>600670</v>
       </c>
       <c r="L9" t="n">
-        <v>8.419724060303114</v>
+        <v>8.435580268699953</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -12291,10 +12296,10 @@
         <v>646000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>729350</v>
+        <v>729477</v>
       </c>
       <c r="L10" t="n">
-        <v>17.04956468088024</v>
+        <v>17.06400613041946</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -12355,7 +12360,7 @@
         <v>615000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>557637</v>
+        <v>557735</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -12419,7 +12424,7 @@
         <v>700000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>643494</v>
+        <v>643606</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -12483,7 +12488,7 @@
         <v>745000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>686422</v>
+        <v>686542</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -12547,7 +12552,7 @@
         <v>930000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>858135</v>
+        <v>858284</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -12618,7 +12623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12667,7 +12672,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 16GB 2TB Space Black</t>
+          <t>Apple MacBook Pro 14Inch MX2E3 M4 Pro 12Core CPU 16Core GPU 24GB 512GB Silver</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -12676,21 +12681,189 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>830000</v>
+        <v>640000</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>810000</v>
+        <v>634000</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-20000</v>
+        <v>-6000</v>
       </c>
       <c r="F2" t="n">
-        <v>-2.41</v>
+        <v>-0.9399999999999999</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Apple MacBook Pro 16Inch MX2V3 14Core CPU 32Core GPU M4 Max 36GB 1TB Silver</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>995000</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>990000</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>-5000</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Apple MacBook Pro 16Inch MX303 14Core CPU 32Core GPU M4 Max 36GB 1TB Space Black</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>995000</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>990000</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>-5000</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 13 MDHE4 M5 10C CPU 8C GPU 16GB 512GB Midnight</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>422000</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>420000</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>-2000</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-0.47</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 13 MDHH4 M5 10C CPU 8C GPU 16GB 512GB Sky Blue</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>422000</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>420000</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>-2000</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-0.47</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 13 MDHA4 M5 10C CPU 8C GPU 16GB 512GB Starlight</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>422000</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>420000</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>-2000</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-0.47</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Macbook Pro 14 M5 MJ3E4 10 Core CPU 10 Core GPU 32GB 1TB Silver</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>755000</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>775000</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>20000</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2.65</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Macbook Pro 14 M5 MJ3D4 10 Core CPU 10 Core GPU 32GB 1TB Space Black</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>745000</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>775000</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>30000</v>
+      </c>
+      <c r="F9" t="n">
+        <v>4.03</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F2"/>
-  <conditionalFormatting sqref="E2">
+  <autoFilter ref="A1:F9"/>
+  <conditionalFormatting sqref="E2:E9">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
chore: price data 2026-09-28
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MacBook Pro'!$A$1:$S$93</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MacBook Air'!$A$1:$S$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20260927T092004702594+0000</t>
+          <t>20260928T095250708307+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-27T09:20:04.702594+00:00</t>
+          <t>2026-09-28T09:52:50.708307+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>277.004436</v>
+        <v>276.909534</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -1147,10 +1147,10 @@
         <v>470000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>686542</v>
+        <v>686306</v>
       </c>
       <c r="L2" t="n">
-        <v>35.18240690300083</v>
+        <v>35.16011808143889</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1214,10 +1214,10 @@
         <v>465000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>686542</v>
+        <v>686306</v>
       </c>
       <c r="L3" t="n">
-        <v>33.28885923949299</v>
+        <v>33.26591928381801</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>772413</v>
+        <v>772148</v>
       </c>
       <c r="L4" t="n">
-        <v>35.26792014116801</v>
+        <v>35.24570419142444</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>772413</v>
+        <v>772148</v>
       </c>
       <c r="L5" t="n">
-        <v>32.67863176823798</v>
+        <v>32.6555271787274</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>858284</v>
+        <v>857990</v>
       </c>
       <c r="L6" t="n">
-        <v>38.01585489185398</v>
+        <v>37.9946153218569</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1606,10 +1606,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>858284</v>
+        <v>857990</v>
       </c>
       <c r="L9" t="n">
-        <v>34.17097371033364</v>
+        <v>34.14841664821268</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1673,10 +1673,10 @@
         <v>582999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>858284</v>
+        <v>857990</v>
       </c>
       <c r="L10" t="n">
-        <v>32.07388230469169</v>
+        <v>32.05060665042716</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -1740,10 +1740,10 @@
         <v>587999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>858284</v>
+        <v>857990</v>
       </c>
       <c r="L11" t="n">
-        <v>31.49132454991588</v>
+        <v>31.46784927563258</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -1807,10 +1807,10 @@
         <v>600000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>858284</v>
+        <v>857990</v>
       </c>
       <c r="L12" t="n">
-        <v>30.09306942690299</v>
+        <v>30.06911502465064</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -1874,13 +1874,13 @@
         <v>634000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>858284</v>
+        <v>857990</v>
       </c>
       <c r="L13" t="n">
-        <v>26.13167669442749</v>
+        <v>26.1063648760475</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>-6000</v>
+        <v>0</v>
       </c>
       <c r="N13" t="n">
         <v>2.461538461538462</v>
@@ -1941,10 +1941,10 @@
         <v>643999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>944156</v>
+        <v>943832</v>
       </c>
       <c r="L14" t="n">
-        <v>31.79103876901698</v>
+        <v>31.76762389916849</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -2067,10 +2067,10 @@
         <v>650000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>944156</v>
+        <v>943832</v>
       </c>
       <c r="L16" t="n">
-        <v>31.15544465109579</v>
+        <v>31.13181159358869</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -2134,10 +2134,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1030027</v>
+        <v>1029674</v>
       </c>
       <c r="L17" t="n">
-        <v>32.04061641102612</v>
+        <v>32.01731810262277</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2201,10 +2201,10 @@
         <v>711999</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>1072963</v>
+        <v>1072595</v>
       </c>
       <c r="L18" t="n">
-        <v>33.6417937990406</v>
+        <v>33.61902675287504</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -2330,10 +2330,10 @@
         <v>720000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>1030027</v>
+        <v>1029674</v>
       </c>
       <c r="L20" t="n">
-        <v>30.09891973705544</v>
+        <v>30.07495576269771</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -2459,10 +2459,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1072963</v>
+        <v>1072595</v>
       </c>
       <c r="L22" t="n">
-        <v>30.75250497920245</v>
+        <v>30.72874663782695</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2477,7 +2477,7 @@
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>10.3</v>
+        <v>10.2</v>
       </c>
       <c r="R22" t="n">
         <v>4</v>
@@ -2526,10 +2526,10 @@
         <v>772000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1030027</v>
+        <v>1029674</v>
       </c>
       <c r="L23" t="n">
-        <v>25.05050838473166</v>
+        <v>25.02481367889254</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -2593,13 +2593,13 @@
         <v>775000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1030027</v>
+        <v>1029674</v>
       </c>
       <c r="L24" t="n">
-        <v>24.75925388363606</v>
+        <v>24.73345932790378</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="N24" t="n">
         <v>0</v>
@@ -2611,7 +2611,7 @@
         <v>68.99999999999999</v>
       </c>
       <c r="Q24" t="n">
-        <v>19.8</v>
+        <v>19.7</v>
       </c>
       <c r="R24" t="n">
         <v>4</v>
@@ -2660,13 +2660,13 @@
         <v>775000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>1030027</v>
+        <v>1029674</v>
       </c>
       <c r="L25" t="n">
-        <v>24.75925388363606</v>
+        <v>24.73345932790378</v>
       </c>
       <c r="M25" s="3" t="n">
-        <v>30000</v>
+        <v>0</v>
       </c>
       <c r="N25" t="n">
         <v>0</v>
@@ -2678,7 +2678,7 @@
         <v>68.99999999999999</v>
       </c>
       <c r="Q25" t="n">
-        <v>19.8</v>
+        <v>19.7</v>
       </c>
       <c r="R25" t="n">
         <v>4</v>
@@ -2789,10 +2789,10 @@
         <v>810000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>1072963</v>
+        <v>1072595</v>
       </c>
       <c r="L27" t="n">
-        <v>24.5081144456985</v>
+        <v>24.48221369668887</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -2804,7 +2804,7 @@
         <v>61.99999999999999</v>
       </c>
       <c r="Q27" t="n">
-        <v>24.9</v>
+        <v>24.8</v>
       </c>
       <c r="R27" t="n">
         <v>3</v>
@@ -2853,10 +2853,10 @@
         <v>810000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>1244706</v>
+        <v>1244279</v>
       </c>
       <c r="L28" t="n">
-        <v>34.92439178408395</v>
+        <v>34.9020597470503</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -2982,10 +2982,10 @@
         <v>825000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1287641</v>
+        <v>1287200</v>
       </c>
       <c r="L30" t="n">
-        <v>35.9293467666842</v>
+        <v>35.90739589807333</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -3000,7 +3000,7 @@
         <v>1.718244359164265</v>
       </c>
       <c r="Q30" t="n">
-        <v>34.8</v>
+        <v>34.7</v>
       </c>
       <c r="R30" t="n">
         <v>4</v>
@@ -3049,10 +3049,10 @@
         <v>829999</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1287641</v>
+        <v>1287200</v>
       </c>
       <c r="L31" t="n">
-        <v>35.54111743878923</v>
+        <v>35.51903356121815</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -3116,10 +3116,10 @@
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1373513</v>
+        <v>1373042</v>
       </c>
       <c r="L32" t="n">
-        <v>38.26057707498946</v>
+        <v>38.23939835780697</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3183,10 +3183,10 @@
         <v>930000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1373513</v>
+        <v>1373042</v>
       </c>
       <c r="L33" t="n">
-        <v>38.11496505675592</v>
+        <v>38.09373638970985</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3250,10 +3250,10 @@
         <v>860000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>1244706</v>
+        <v>1244279</v>
       </c>
       <c r="L34" t="n">
-        <v>30.90737893124963</v>
+        <v>30.88366837341143</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -3503,10 +3503,10 @@
         <v>880000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>1158834</v>
+        <v>1158437</v>
       </c>
       <c r="L38" t="n">
-        <v>24.0615998495039</v>
+        <v>24.0355755211548</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -3567,10 +3567,10 @@
         <v>940000</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>1244706</v>
+        <v>1244279</v>
       </c>
       <c r="L39" t="n">
-        <v>24.48015836671471</v>
+        <v>24.45424217558924</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -3631,13 +3631,13 @@
         <v>990000</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>1502320</v>
+        <v>1501805</v>
       </c>
       <c r="L40" t="n">
-        <v>34.10192236008307</v>
+        <v>34.07932454612949</v>
       </c>
       <c r="M40" s="3" t="n">
-        <v>-5000</v>
+        <v>0</v>
       </c>
       <c r="N40" t="n">
         <v>3.131115459882583</v>
@@ -3695,13 +3695,13 @@
         <v>990000</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>1502320</v>
+        <v>1501805</v>
       </c>
       <c r="L41" t="n">
-        <v>34.10192236008307</v>
+        <v>34.07932454612949</v>
       </c>
       <c r="M41" s="3" t="n">
-        <v>-5000</v>
+        <v>0</v>
       </c>
       <c r="N41" t="n">
         <v>0</v>
@@ -3821,10 +3821,10 @@
         <v>1055000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1545255</v>
+        <v>1544726</v>
       </c>
       <c r="L43" t="n">
-        <v>31.72647880123345</v>
+        <v>31.70309815462419</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -3885,10 +3885,10 @@
         <v>1055000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1545255</v>
+        <v>1544726</v>
       </c>
       <c r="L44" t="n">
-        <v>31.72647880123345</v>
+        <v>31.70309815462419</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -3900,7 +3900,7 @@
         <v>58.64647440248988</v>
       </c>
       <c r="Q44" t="n">
-        <v>27.2</v>
+        <v>27.1</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -4011,10 +4011,10 @@
         <v>1115000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1502320</v>
+        <v>1501805</v>
       </c>
       <c r="L46" t="n">
-        <v>25.78145801160871</v>
+        <v>25.75600693831756</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -4075,10 +4075,10 @@
         <v>1123000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1716998</v>
+        <v>1716410</v>
       </c>
       <c r="L47" t="n">
-        <v>34.59514804327087</v>
+        <v>34.57274194394113</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -4142,10 +4142,10 @@
         <v>1130000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1502320</v>
+        <v>1501805</v>
       </c>
       <c r="L48" t="n">
-        <v>24.78300228979179</v>
+        <v>24.75720882538013</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -4268,10 +4268,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1759934</v>
+        <v>1759331</v>
       </c>
       <c r="L50" t="n">
-        <v>34.37253897021138</v>
+        <v>34.3500455570896</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4283,7 +4283,7 @@
         <v>22.53136001640632</v>
       </c>
       <c r="Q50" t="n">
-        <v>19.6</v>
+        <v>19.5</v>
       </c>
       <c r="R50" t="n">
         <v>3</v>
@@ -4332,10 +4332,10 @@
         <v>1155000</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>1759934</v>
+        <v>1759331</v>
       </c>
       <c r="L51" t="n">
-        <v>34.37253897021138</v>
+        <v>34.3500455570896</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -4347,7 +4347,7 @@
         <v>22.53136001640632</v>
       </c>
       <c r="Q51" t="n">
-        <v>19.6</v>
+        <v>19.5</v>
       </c>
       <c r="R51" t="n">
         <v>3</v>
@@ -4396,10 +4396,10 @@
         <v>1185000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1588191</v>
+        <v>1587647</v>
       </c>
       <c r="L52" t="n">
-        <v>25.38680800986783</v>
+        <v>25.36124214009789</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -4460,10 +4460,10 @@
         <v>1185000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1588191</v>
+        <v>1587647</v>
       </c>
       <c r="L53" t="n">
-        <v>25.38680800986783</v>
+        <v>25.36124214009789</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -4524,10 +4524,10 @@
         <v>1200000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1888741</v>
+        <v>1888094</v>
       </c>
       <c r="L54" t="n">
-        <v>36.46561386659155</v>
+        <v>36.44384230869861</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -4588,10 +4588,10 @@
         <v>1200000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1888741</v>
+        <v>1888094</v>
       </c>
       <c r="L55" t="n">
-        <v>36.46561386659155</v>
+        <v>36.44384230869861</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -4714,10 +4714,10 @@
         <v>1240000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1674062</v>
+        <v>1673489</v>
       </c>
       <c r="L57" t="n">
-        <v>25.92866930854413</v>
+        <v>25.90330740148277</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -4729,7 +4729,7 @@
         <v>100</v>
       </c>
       <c r="Q57" t="n">
-        <v>33.7</v>
+        <v>33.6</v>
       </c>
       <c r="R57" t="n">
         <v>3</v>
@@ -4840,10 +4840,10 @@
         <v>1280000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1716998</v>
+        <v>1716410</v>
       </c>
       <c r="L59" t="n">
-        <v>25.45128183026421</v>
+        <v>25.42574326646897</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -4907,10 +4907,10 @@
         <v>1298000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1759934</v>
+        <v>1759331</v>
       </c>
       <c r="L60" t="n">
-        <v>26.24723427128518</v>
+        <v>26.22195595939593</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -4971,10 +4971,10 @@
         <v>1300000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1716998</v>
+        <v>1716410</v>
       </c>
       <c r="L61" t="n">
-        <v>24.28645810886209</v>
+        <v>24.26052050500754</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -5097,10 +5097,10 @@
         <v>1335000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1802870</v>
+        <v>1802252</v>
       </c>
       <c r="L63" t="n">
-        <v>25.95139971268034</v>
+        <v>25.92600812760924</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -5161,10 +5161,10 @@
         <v>1420000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1931677</v>
+        <v>1931015</v>
       </c>
       <c r="L64" t="n">
-        <v>26.48874527159562</v>
+        <v>26.46354378396854</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -5225,10 +5225,10 @@
         <v>1430000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1931677</v>
+        <v>1931015</v>
       </c>
       <c r="L65" t="n">
-        <v>25.97106037914206</v>
+        <v>25.94568141625</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -5289,10 +5289,10 @@
         <v>1430000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>2146355</v>
+        <v>2145620</v>
       </c>
       <c r="L66" t="n">
-        <v>33.37542018911131</v>
+        <v>33.352597384439</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -5353,10 +5353,10 @@
         <v>1430000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>2146355</v>
+        <v>2145620</v>
       </c>
       <c r="L67" t="n">
-        <v>33.37542018911131</v>
+        <v>33.352597384439</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -5479,10 +5479,10 @@
         <v>1480000</v>
       </c>
       <c r="K69" s="3" t="n">
-        <v>2017548</v>
+        <v>2016857</v>
       </c>
       <c r="L69" t="n">
-        <v>26.6436288009009</v>
+        <v>26.61849600640998</v>
       </c>
       <c r="M69" s="3" t="n">
         <v>0</v>
@@ -5605,10 +5605,10 @@
         <v>1605000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2189291</v>
+        <v>2188541</v>
       </c>
       <c r="L71" t="n">
-        <v>26.68859461807498</v>
+        <v>26.66347123494602</v>
       </c>
       <c r="M71" s="3" t="n">
         <v>0</v>
@@ -5669,10 +5669,10 @@
         <v>1610000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2189291</v>
+        <v>2188541</v>
       </c>
       <c r="L72" t="n">
-        <v>26.46021017763285</v>
+        <v>26.43500852851283</v>
       </c>
       <c r="M72" s="3" t="n">
         <v>0</v>
@@ -5733,10 +5733,10 @@
         <v>1615000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2189291</v>
+        <v>2188541</v>
       </c>
       <c r="L73" t="n">
-        <v>26.23182573719072</v>
+        <v>26.20654582207964</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
@@ -5797,10 +5797,10 @@
         <v>1630000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2232226</v>
+        <v>2231462</v>
       </c>
       <c r="L74" t="n">
-        <v>26.97871989664129</v>
+        <v>26.95371913122429</v>
       </c>
       <c r="M74" s="3" t="n">
         <v>0</v>
@@ -5812,7 +5812,7 @@
         <v>100</v>
       </c>
       <c r="Q74" t="n">
-        <v>34.1</v>
+        <v>34</v>
       </c>
       <c r="R74" t="n">
         <v>3</v>
@@ -5861,10 +5861,10 @@
         <v>1690000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2318098</v>
+        <v>2317304</v>
       </c>
       <c r="L75" t="n">
-        <v>27.0954032141868</v>
+        <v>27.07042321594405</v>
       </c>
       <c r="M75" s="3" t="n">
         <v>0</v>
@@ -5925,10 +5925,10 @@
         <v>1705000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2318098</v>
+        <v>2317304</v>
       </c>
       <c r="L76" t="n">
-        <v>26.44832099419438</v>
+        <v>26.42311927999089</v>
       </c>
       <c r="M76" s="3" t="n">
         <v>0</v>
@@ -5989,10 +5989,10 @@
         <v>1725000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2361033</v>
+        <v>2360225</v>
       </c>
       <c r="L77" t="n">
-        <v>26.93875943284148</v>
+        <v>26.9137476299929</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
@@ -6053,10 +6053,10 @@
         <v>1780000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2446905</v>
+        <v>2446067</v>
       </c>
       <c r="L78" t="n">
-        <v>27.25504259462464</v>
+        <v>27.23012084296955</v>
       </c>
       <c r="M78" s="3" t="n">
         <v>0</v>
@@ -6068,7 +6068,7 @@
         <v>38.78143936249688</v>
       </c>
       <c r="Q78" t="n">
-        <v>21.2</v>
+        <v>21.1</v>
       </c>
       <c r="R78" t="n">
         <v>3</v>
@@ -6117,10 +6117,10 @@
         <v>1875000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2575712</v>
+        <v>2574829</v>
       </c>
       <c r="L79" t="n">
-        <v>27.2045943024686</v>
+        <v>27.17963018126641</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
@@ -6132,7 +6132,7 @@
         <v>19.64044075004835</v>
       </c>
       <c r="Q79" t="n">
-        <v>17.2</v>
+        <v>17.1</v>
       </c>
       <c r="R79" t="n">
         <v>3</v>
@@ -6181,10 +6181,10 @@
         <v>1910000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2618648</v>
+        <v>2617750</v>
       </c>
       <c r="L80" t="n">
-        <v>27.06159819876516</v>
+        <v>27.03657721325566</v>
       </c>
       <c r="M80" s="3" t="n">
         <v>0</v>
@@ -6245,10 +6245,10 @@
         <v>2020000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2747455</v>
+        <v>2746513</v>
       </c>
       <c r="L81" t="n">
-        <v>26.4774127328746</v>
+        <v>26.45219592989365</v>
       </c>
       <c r="M81" s="3" t="n">
         <v>0</v>
@@ -6309,10 +6309,10 @@
         <v>2110000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>2876262</v>
+        <v>2875276</v>
       </c>
       <c r="L82" t="n">
-        <v>26.64089710881693</v>
+        <v>26.61574054108197</v>
       </c>
       <c r="M82" s="3" t="n">
         <v>0</v>
@@ -6373,10 +6373,10 @@
         <v>2210000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3005069</v>
+        <v>3004039</v>
       </c>
       <c r="L83" t="n">
-        <v>26.45759548283251</v>
+        <v>26.4323798725649</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
@@ -6437,10 +6437,10 @@
         <v>2215000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3048004</v>
+        <v>3046960</v>
       </c>
       <c r="L84" t="n">
-        <v>27.32949169358045</v>
+        <v>27.30459211804553</v>
       </c>
       <c r="M84" s="3" t="n">
         <v>0</v>
@@ -6501,10 +6501,10 @@
         <v>2315000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3176812</v>
+        <v>3175723</v>
       </c>
       <c r="L85" t="n">
-        <v>27.12820273909819</v>
+        <v>27.10321397678576</v>
       </c>
       <c r="M85" s="3" t="n">
         <v>0</v>
@@ -6565,10 +6565,10 @@
         <v>2395000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3305619</v>
+        <v>3304486</v>
       </c>
       <c r="L86" t="n">
-        <v>27.54760908622561</v>
+        <v>27.52276753479966</v>
       </c>
       <c r="M86" s="3" t="n">
         <v>0</v>
@@ -6629,10 +6629,10 @@
         <v>2410000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3305619</v>
+        <v>3304486</v>
       </c>
       <c r="L87" t="n">
-        <v>27.09383628300781</v>
+        <v>27.06883914775248</v>
       </c>
       <c r="M87" s="3" t="n">
         <v>0</v>
@@ -6693,10 +6693,10 @@
         <v>2499000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3434426</v>
+        <v>3433249</v>
       </c>
       <c r="L88" t="n">
-        <v>27.23674931415031</v>
+        <v>27.21180432878594</v>
       </c>
       <c r="M88" s="3" t="n">
         <v>0</v>
@@ -6708,7 +6708,7 @@
         <v>63.67326854471646</v>
       </c>
       <c r="Q88" t="n">
-        <v>26.5</v>
+        <v>26.4</v>
       </c>
       <c r="R88" t="n">
         <v>3</v>
@@ -6757,10 +6757,10 @@
         <v>2510000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3434426</v>
+        <v>3433249</v>
       </c>
       <c r="L89" t="n">
-        <v>26.91646289656554</v>
+        <v>26.89140810934482</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
@@ -6821,10 +6821,10 @@
         <v>2530000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3477361</v>
+        <v>3476170</v>
       </c>
       <c r="L90" t="n">
-        <v>27.24367702979357</v>
+        <v>27.21874937071547</v>
       </c>
       <c r="M90" s="3" t="n">
         <v>0</v>
@@ -6885,10 +6885,10 @@
         <v>2610000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>3606168</v>
+        <v>3604933</v>
       </c>
       <c r="L91" t="n">
-        <v>27.62400420612683</v>
+        <v>27.59920919473399</v>
       </c>
       <c r="M91" s="3" t="n">
         <v>0</v>
@@ -6900,7 +6900,7 @@
         <v>74.15426251691474</v>
       </c>
       <c r="Q91" t="n">
-        <v>28.5</v>
+        <v>28.4</v>
       </c>
       <c r="R91" t="n">
         <v>3</v>
@@ -6949,10 +6949,10 @@
         <v>3015000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4164332</v>
+        <v>4162906</v>
       </c>
       <c r="L92" t="n">
-        <v>27.59943251402626</v>
+        <v>27.57463175964098</v>
       </c>
       <c r="M92" s="3" t="n">
         <v>0</v>
@@ -7013,10 +7013,10 @@
         <v>3098000</v>
       </c>
       <c r="K93" s="3" t="n">
-        <v>4293139</v>
+        <v>4291669</v>
       </c>
       <c r="L93" t="n">
-        <v>27.83834858363543</v>
+        <v>27.81363147996735</v>
       </c>
       <c r="M93" s="3" t="n">
         <v>0</v>
@@ -7312,10 +7312,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>428928</v>
+        <v>428781</v>
       </c>
       <c r="L2" t="n">
-        <v>27.72703111011639</v>
+        <v>27.70225359799058</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7379,10 +7379,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>428928</v>
+        <v>428781</v>
       </c>
       <c r="L3" t="n">
-        <v>27.72703111011639</v>
+        <v>27.70225359799058</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7446,10 +7446,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>428928</v>
+        <v>428781</v>
       </c>
       <c r="L4" t="n">
-        <v>27.726797970755</v>
+        <v>27.70202037870148</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7513,10 +7513,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>428928</v>
+        <v>428781</v>
       </c>
       <c r="L5" t="n">
-        <v>27.726797970755</v>
+        <v>27.70202037870148</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7580,10 +7580,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514799</v>
+        <v>514623</v>
       </c>
       <c r="L6" t="n">
-        <v>25.40778051239416</v>
+        <v>25.38227012784116</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7644,10 +7644,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>514799</v>
+        <v>514623</v>
       </c>
       <c r="L7" t="n">
-        <v>25.40778051239416</v>
+        <v>25.38227012784116</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7708,10 +7708,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>514799</v>
+        <v>514623</v>
       </c>
       <c r="L8" t="n">
-        <v>25.40778051239416</v>
+        <v>25.38227012784116</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7772,10 +7772,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>514799</v>
+        <v>514623</v>
       </c>
       <c r="L9" t="n">
-        <v>25.40778051239416</v>
+        <v>25.38227012784116</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7836,10 +7836,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>514799</v>
+        <v>514623</v>
       </c>
       <c r="L10" t="n">
-        <v>25.21352994081185</v>
+        <v>25.18795312296574</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7900,10 +7900,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>514799</v>
+        <v>514623</v>
       </c>
       <c r="L11" t="n">
-        <v>25.21352994081185</v>
+        <v>25.18795312296574</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7964,10 +7964,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>514799</v>
+        <v>514623</v>
       </c>
       <c r="L12" t="n">
-        <v>25.21352994081185</v>
+        <v>25.18795312296574</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -8028,10 +8028,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>514799</v>
+        <v>514623</v>
       </c>
       <c r="L13" t="n">
-        <v>25.21352994081185</v>
+        <v>25.18795312296574</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -8092,13 +8092,13 @@
         <v>420000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>557735</v>
+        <v>557544</v>
       </c>
       <c r="L14" t="n">
-        <v>24.69541986785839</v>
+        <v>24.66962248719383</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>-2000</v>
+        <v>0</v>
       </c>
       <c r="N14" t="n">
         <v>4.977160581811272</v>
@@ -8159,13 +8159,13 @@
         <v>420000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>557735</v>
+        <v>557544</v>
       </c>
       <c r="L15" t="n">
-        <v>24.69541986785839</v>
+        <v>24.66962248719383</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>-2000</v>
+        <v>0</v>
       </c>
       <c r="N15" t="n">
         <v>3.002085455162714</v>
@@ -8226,13 +8226,13 @@
         <v>420000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>557735</v>
+        <v>557544</v>
       </c>
       <c r="L16" t="n">
-        <v>24.69541986785839</v>
+        <v>24.66962248719383</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>-2000</v>
+        <v>0</v>
       </c>
       <c r="N16" t="n">
         <v>2.325581395348837</v>
@@ -8293,10 +8293,10 @@
         <v>425000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>557735</v>
+        <v>557544</v>
       </c>
       <c r="L17" t="n">
-        <v>23.79893677104718</v>
+        <v>23.77283227870805</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -8360,10 +8360,10 @@
         <v>454000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>600670</v>
+        <v>600464</v>
       </c>
       <c r="L18" t="n">
-        <v>24.41773353089051</v>
+        <v>24.39180367182712</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -8375,7 +8375,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q18" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="R18" t="n">
         <v>3</v>
@@ -8424,10 +8424,10 @@
         <v>454000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>600670</v>
+        <v>600464</v>
       </c>
       <c r="L19" t="n">
-        <v>24.41773353089051</v>
+        <v>24.39180367182712</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -8439,7 +8439,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q19" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="R19" t="n">
         <v>3</v>
@@ -8488,10 +8488,10 @@
         <v>454000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>600670</v>
+        <v>600464</v>
       </c>
       <c r="L20" t="n">
-        <v>24.41773353089051</v>
+        <v>24.39180367182712</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -8503,7 +8503,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q20" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="R20" t="n">
         <v>3</v>
@@ -8552,10 +8552,10 @@
         <v>454000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>600670</v>
+        <v>600464</v>
       </c>
       <c r="L21" t="n">
-        <v>24.41773353089051</v>
+        <v>24.39180367182712</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -8567,7 +8567,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q21" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="R21" t="n">
         <v>3</v>
@@ -8616,10 +8616,10 @@
         <v>455000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>600670</v>
+        <v>600464</v>
       </c>
       <c r="L22" t="n">
-        <v>24.25125276774269</v>
+        <v>24.22526579445229</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -8680,10 +8680,10 @@
         <v>455000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>600670</v>
+        <v>600464</v>
       </c>
       <c r="L23" t="n">
-        <v>24.25125276774269</v>
+        <v>24.22526579445229</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -8744,10 +8744,10 @@
         <v>455000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>600670</v>
+        <v>600464</v>
       </c>
       <c r="L24" t="n">
-        <v>24.25125276774269</v>
+        <v>24.22526579445229</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -8808,10 +8808,10 @@
         <v>455000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>600670</v>
+        <v>600464</v>
       </c>
       <c r="L25" t="n">
-        <v>24.25125276774269</v>
+        <v>24.22526579445229</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -8837,22 +8837,22 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHF4 M5 10C CPU 10C GPU 16GB 1TB Midnight</t>
+          <t>Apple MacBook Air 15 MC6L4 M4 10C CPU 10C GPU 24GB 512GB Midnight</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E26" t="n">
-        <v>1024</v>
+        <v>512</v>
       </c>
       <c r="F26" t="n">
         <v>10</v>
@@ -8866,34 +8866,31 @@
         </is>
       </c>
       <c r="I26" s="3" t="n">
-        <v>474999</v>
+        <v>475000</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>474999</v>
+        <v>475000</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>686542</v>
+        <v>686306</v>
       </c>
       <c r="L26" t="n">
-        <v>30.81282718318763</v>
+        <v>30.78889008692915</v>
       </c>
       <c r="M26" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>1.041668836810077</v>
-      </c>
-      <c r="O26" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" t="n">
         <v>100</v>
       </c>
-      <c r="P26" t="n">
-        <v>46.21899159663865</v>
-      </c>
       <c r="Q26" t="n">
-        <v>40.5</v>
+        <v>34.6</v>
       </c>
       <c r="R26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S26" t="inlineStr">
         <is>
@@ -8904,22 +8901,22 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHJ4 M5 10C CPU 10C GPU 16GB 1TB Sky Blue</t>
+          <t>Apple MacBook Air 15 MC6K4 M4 10C CPU 10C GPU 24GB 512GB Starlight</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E27" t="n">
-        <v>1024</v>
+        <v>512</v>
       </c>
       <c r="F27" t="n">
         <v>10</v>
@@ -8929,38 +8926,35 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Sky Blue</t>
+          <t>Starlight</t>
         </is>
       </c>
       <c r="I27" s="3" t="n">
-        <v>474999</v>
+        <v>475000</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>474999</v>
+        <v>475000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>686542</v>
+        <v>686306</v>
       </c>
       <c r="L27" t="n">
-        <v>30.81282718318763</v>
+        <v>30.78889008692915</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N27" t="n">
-        <v>1.041668836810077</v>
-      </c>
-      <c r="O27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" t="n">
         <v>100</v>
       </c>
-      <c r="P27" t="n">
-        <v>46.21899159663865</v>
-      </c>
       <c r="Q27" t="n">
-        <v>40.5</v>
+        <v>34.6</v>
       </c>
       <c r="R27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S27" t="inlineStr">
         <is>
@@ -8971,22 +8965,22 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHC4 M5 10C CPU 10C GPU 16GB 1TB Starlight</t>
+          <t>Apple MacBook Air 15 MC6J4 M4 10C CPU 10C GPU 24GB 512GB Silver</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E28" t="n">
-        <v>1024</v>
+        <v>512</v>
       </c>
       <c r="F28" t="n">
         <v>10</v>
@@ -8996,38 +8990,35 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Starlight</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I28" s="3" t="n">
-        <v>474999</v>
+        <v>475000</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>474999</v>
+        <v>475000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>686542</v>
+        <v>686306</v>
       </c>
       <c r="L28" t="n">
-        <v>30.81282718318763</v>
+        <v>30.78889008692915</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N28" t="n">
-        <v>1.041668836810077</v>
-      </c>
-      <c r="O28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" t="n">
         <v>100</v>
       </c>
-      <c r="P28" t="n">
-        <v>46.21899159663865</v>
-      </c>
       <c r="Q28" t="n">
-        <v>40.5</v>
+        <v>34.6</v>
       </c>
       <c r="R28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S28" t="inlineStr">
         <is>
@@ -9038,7 +9029,7 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MC6L4 M4 10C CPU 10C GPU 24GB 512GB Midnight</t>
+          <t>Apple MacBook Air 15 MC7D4 M4 10C CPU 10C GPU 24GB 512GB Sky Blue</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -9063,7 +9054,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Midnight</t>
+          <t>Sky Blue</t>
         </is>
       </c>
       <c r="I29" s="3" t="n">
@@ -9073,10 +9064,10 @@
         <v>475000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>686542</v>
+        <v>686306</v>
       </c>
       <c r="L29" t="n">
-        <v>30.81268152567505</v>
+        <v>30.78889008692915</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -9102,22 +9093,22 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MC6K4 M4 10C CPU 10C GPU 24GB 512GB Starlight</t>
+          <t>Apple MacBook Air 13 MDHF4 M5 10C CPU 10C GPU 16GB 1TB Midnight</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E30" t="n">
-        <v>512</v>
+        <v>1024</v>
       </c>
       <c r="F30" t="n">
         <v>10</v>
@@ -9127,32 +9118,32 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Starlight</t>
+          <t>Midnight</t>
         </is>
       </c>
       <c r="I30" s="3" t="n">
-        <v>475000</v>
+        <v>479999</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>475000</v>
+        <v>479999</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>686542</v>
+        <v>686306</v>
       </c>
       <c r="L30" t="n">
-        <v>30.81268152567505</v>
+        <v>30.06049779544401</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="N30" t="n">
         <v>0</v>
       </c>
       <c r="P30" t="n">
-        <v>100</v>
+        <v>43.6979831932773</v>
       </c>
       <c r="Q30" t="n">
-        <v>34.6</v>
+        <v>22.2</v>
       </c>
       <c r="R30" t="n">
         <v>3</v>
@@ -9166,22 +9157,22 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MC6J4 M4 10C CPU 10C GPU 24GB 512GB Silver</t>
+          <t>Apple MacBook Air 13 MDHJ4 M5 10C CPU 10C GPU 16GB 1TB Sky Blue</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E31" t="n">
-        <v>512</v>
+        <v>1024</v>
       </c>
       <c r="F31" t="n">
         <v>10</v>
@@ -9191,32 +9182,32 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Sky Blue</t>
         </is>
       </c>
       <c r="I31" s="3" t="n">
-        <v>475000</v>
+        <v>479999</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>475000</v>
+        <v>479999</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>686542</v>
+        <v>686306</v>
       </c>
       <c r="L31" t="n">
-        <v>30.81268152567505</v>
+        <v>30.06049779544401</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="N31" t="n">
         <v>0</v>
       </c>
       <c r="P31" t="n">
-        <v>100</v>
+        <v>43.6979831932773</v>
       </c>
       <c r="Q31" t="n">
-        <v>34.6</v>
+        <v>22.2</v>
       </c>
       <c r="R31" t="n">
         <v>3</v>
@@ -9230,22 +9221,22 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MC7D4 M4 10C CPU 10C GPU 24GB 512GB Sky Blue</t>
+          <t>Apple MacBook Air 13 MDH84 M5 10C CPU 10C GPU 16GB 1TB Silver</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E32" t="n">
-        <v>512</v>
+        <v>1024</v>
       </c>
       <c r="F32" t="n">
         <v>10</v>
@@ -9255,20 +9246,20 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Sky Blue</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I32" s="3" t="n">
-        <v>475000</v>
+        <v>479999</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>475000</v>
+        <v>479999</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>686542</v>
+        <v>686306</v>
       </c>
       <c r="L32" t="n">
-        <v>30.81268152567505</v>
+        <v>30.06049779544401</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -9277,10 +9268,10 @@
         <v>0</v>
       </c>
       <c r="P32" t="n">
-        <v>100</v>
+        <v>43.6979831932773</v>
       </c>
       <c r="Q32" t="n">
-        <v>34.6</v>
+        <v>22.2</v>
       </c>
       <c r="R32" t="n">
         <v>3</v>
@@ -9294,7 +9285,7 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDH84 M5 10C CPU 10C GPU 16GB 1TB Silver</t>
+          <t>Apple MacBook Air 13 MDHC4 M5 10C CPU 10C GPU 16GB 1TB Starlight</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -9319,7 +9310,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Starlight</t>
         </is>
       </c>
       <c r="I33" s="3" t="n">
@@ -9329,28 +9320,25 @@
         <v>479999</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>686542</v>
+        <v>686306</v>
       </c>
       <c r="L33" t="n">
-        <v>30.08453962029999</v>
+        <v>30.06049779544401</v>
       </c>
       <c r="M33" s="3" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="N33" t="n">
-        <v>0</v>
-      </c>
-      <c r="O33" t="n">
         <v>0</v>
       </c>
       <c r="P33" t="n">
         <v>43.6979831932773</v>
       </c>
       <c r="Q33" t="n">
-        <v>17.3</v>
+        <v>22.2</v>
       </c>
       <c r="R33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S33" t="inlineStr">
         <is>
@@ -9396,10 +9384,10 @@
         <v>479999</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>643606</v>
+        <v>643385</v>
       </c>
       <c r="L34" t="n">
-        <v>25.42036587601731</v>
+        <v>25.39474809017929</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -9463,10 +9451,10 @@
         <v>479999</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>643606</v>
+        <v>643385</v>
       </c>
       <c r="L35" t="n">
-        <v>25.42036587601731</v>
+        <v>25.39474809017929</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
@@ -9530,10 +9518,10 @@
         <v>479999</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>643606</v>
+        <v>643385</v>
       </c>
       <c r="L36" t="n">
-        <v>25.42036587601731</v>
+        <v>25.39474809017929</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -9597,10 +9585,10 @@
         <v>484999</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>643606</v>
+        <v>643385</v>
       </c>
       <c r="L37" t="n">
-        <v>24.64349306874081</v>
+        <v>24.61760843041103</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
@@ -9664,10 +9652,10 @@
         <v>500000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>643606</v>
+        <v>643385</v>
       </c>
       <c r="L38" t="n">
-        <v>22.31271927234985</v>
+        <v>22.28603402317431</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -9728,10 +9716,10 @@
         <v>547999</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>772413</v>
+        <v>772148</v>
       </c>
       <c r="L39" t="n">
-        <v>29.05362804613594</v>
+        <v>29.02927936095153</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -9792,10 +9780,10 @@
         <v>547999</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>772413</v>
+        <v>772148</v>
       </c>
       <c r="L40" t="n">
-        <v>29.05362804613594</v>
+        <v>29.02927936095153</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -9856,10 +9844,10 @@
         <v>547999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>772413</v>
+        <v>772148</v>
       </c>
       <c r="L41" t="n">
-        <v>29.05362804613594</v>
+        <v>29.02927936095153</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
@@ -9871,7 +9859,7 @@
         <v>64.67267226890753</v>
       </c>
       <c r="Q41" t="n">
-        <v>27</v>
+        <v>26.9</v>
       </c>
       <c r="R41" t="n">
         <v>3</v>
@@ -9920,10 +9908,10 @@
         <v>547999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>772413</v>
+        <v>772148</v>
       </c>
       <c r="L42" t="n">
-        <v>29.05362804613594</v>
+        <v>29.02927936095153</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -9984,10 +9972,10 @@
         <v>552999</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>772413</v>
+        <v>772148</v>
       </c>
       <c r="L43" t="n">
-        <v>28.40630595290343</v>
+        <v>28.38173510777727</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -10048,10 +10036,10 @@
         <v>552999</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>772413</v>
+        <v>772148</v>
       </c>
       <c r="L44" t="n">
-        <v>28.40630595290343</v>
+        <v>28.38173510777727</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -10112,10 +10100,10 @@
         <v>552999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>772413</v>
+        <v>772148</v>
       </c>
       <c r="L45" t="n">
-        <v>28.40630595290343</v>
+        <v>28.38173510777727</v>
       </c>
       <c r="M45" s="3" t="n">
         <v>0</v>
@@ -10176,10 +10164,10 @@
         <v>552999</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>772413</v>
+        <v>772148</v>
       </c>
       <c r="L46" t="n">
-        <v>28.40630595290343</v>
+        <v>28.38173510777727</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -10240,10 +10228,10 @@
         <v>585000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>729477</v>
+        <v>729227</v>
       </c>
       <c r="L47" t="n">
-        <v>19.80555932537969</v>
+        <v>19.77806636342319</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -10304,10 +10292,10 @@
         <v>595000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>729477</v>
+        <v>729227</v>
       </c>
       <c r="L48" t="n">
-        <v>18.43471418564259</v>
+        <v>18.40675125852444</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -10368,10 +10356,10 @@
         <v>614999</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>858284</v>
+        <v>857990</v>
       </c>
       <c r="L49" t="n">
-        <v>28.34551267412651</v>
+        <v>28.32095945174186</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -10432,10 +10420,10 @@
         <v>614999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>858284</v>
+        <v>857990</v>
       </c>
       <c r="L50" t="n">
-        <v>28.34551267412651</v>
+        <v>28.32095945174186</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -10496,10 +10484,10 @@
         <v>614999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>858284</v>
+        <v>857990</v>
       </c>
       <c r="L51" t="n">
-        <v>28.34551267412651</v>
+        <v>28.32095945174186</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -10560,10 +10548,10 @@
         <v>614999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>858284</v>
+        <v>857990</v>
       </c>
       <c r="L52" t="n">
-        <v>28.34551267412651</v>
+        <v>28.32095945174186</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -10624,10 +10612,10 @@
         <v>650000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>815349</v>
+        <v>815069</v>
       </c>
       <c r="L53" t="n">
-        <v>20.27953673825564</v>
+        <v>20.25215043143587</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -10688,10 +10676,10 @@
         <v>672000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>858284</v>
+        <v>857990</v>
       </c>
       <c r="L54" t="n">
-        <v>21.70423775813134</v>
+        <v>21.67740882760871</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -10752,10 +10740,10 @@
         <v>700000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>901220</v>
+        <v>900911</v>
       </c>
       <c r="L55" t="n">
-        <v>22.32751159539291</v>
+        <v>22.30087100723601</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -10816,10 +10804,10 @@
         <v>715000</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>944156</v>
+        <v>943832</v>
       </c>
       <c r="L56" t="n">
-        <v>24.27098911620537</v>
+        <v>24.24499275294756</v>
       </c>
       <c r="M56" s="3" t="n">
         <v>0</v>
@@ -10880,22 +10868,22 @@
         <v>734999</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>987091</v>
+        <v>986753</v>
       </c>
       <c r="L57" t="n">
-        <v>25.53888142025406</v>
+        <v>25.51337568773543</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N57" t="n">
-        <v>2.777910052910053</v>
+        <v>1.408518717987068</v>
       </c>
       <c r="P57" t="n">
         <v>73.94986794717886</v>
       </c>
       <c r="Q57" t="n">
-        <v>27.8</v>
+        <v>27.3</v>
       </c>
       <c r="R57" t="n">
         <v>3</v>
@@ -10944,10 +10932,10 @@
         <v>752000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>987091</v>
+        <v>986753</v>
       </c>
       <c r="L58" t="n">
-        <v>23.81654781575356</v>
+        <v>23.79045211922335</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -11008,10 +10996,10 @@
         <v>810000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1072963</v>
+        <v>1072595</v>
       </c>
       <c r="L59" t="n">
-        <v>24.5081144456985</v>
+        <v>24.48221369668887</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -11023,7 +11011,7 @@
         <v>70.24552627383726</v>
       </c>
       <c r="Q59" t="n">
-        <v>25.6</v>
+        <v>25.5</v>
       </c>
       <c r="R59" t="n">
         <v>3</v>
@@ -11072,10 +11060,10 @@
         <v>815000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1072963</v>
+        <v>1072595</v>
       </c>
       <c r="L60" t="n">
-        <v>24.04211515215343</v>
+        <v>24.01605452197707</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -11136,10 +11124,10 @@
         <v>875000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1158834</v>
+        <v>1158437</v>
       </c>
       <c r="L61" t="n">
-        <v>24.49306803217717</v>
+        <v>24.46719156933005</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -11200,10 +11188,10 @@
         <v>992000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1330577</v>
+        <v>1330121</v>
       </c>
       <c r="L62" t="n">
-        <v>25.44587799127747</v>
+        <v>25.42031890331782</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -11215,7 +11203,7 @@
         <v>85.64705882352939</v>
       </c>
       <c r="Q62" t="n">
-        <v>29.3</v>
+        <v>29.2</v>
       </c>
       <c r="R62" t="n">
         <v>3</v>
@@ -11264,10 +11252,10 @@
         <v>1050000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1416448</v>
+        <v>1415963</v>
       </c>
       <c r="L63" t="n">
-        <v>25.87091089824688</v>
+        <v>25.8455199747451</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -11279,7 +11267,7 @@
         <v>93.20091673032849</v>
       </c>
       <c r="Q63" t="n">
-        <v>31.1</v>
+        <v>31</v>
       </c>
       <c r="R63" t="n">
         <v>3</v>
@@ -11328,10 +11316,10 @@
         <v>1050000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1416448</v>
+        <v>1415963</v>
       </c>
       <c r="L64" t="n">
-        <v>25.87091089824688</v>
+        <v>25.8455199747451</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -11392,10 +11380,10 @@
         <v>1100000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1502320</v>
+        <v>1501805</v>
       </c>
       <c r="L65" t="n">
-        <v>26.77991373342564</v>
+        <v>26.75480505125499</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -11456,10 +11444,10 @@
         <v>1105000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1502320</v>
+        <v>1501805</v>
       </c>
       <c r="L66" t="n">
-        <v>26.44709515948666</v>
+        <v>26.42187234694251</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -11520,10 +11508,10 @@
         <v>1155000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1588191</v>
+        <v>1587647</v>
       </c>
       <c r="L67" t="n">
-        <v>27.27574957923827</v>
+        <v>27.2508309466777</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -11790,7 +11778,7 @@
         <v>315000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>300120</v>
+        <v>300018</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -11851,10 +11839,10 @@
         <v>380000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>385992</v>
+        <v>385860</v>
       </c>
       <c r="L3" t="n">
-        <v>1.552363779560198</v>
+        <v>1.518685533613228</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -11915,7 +11903,7 @@
         <v>415000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>385992</v>
+        <v>385860</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -11976,10 +11964,10 @@
         <v>495000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>471863</v>
+        <v>471702</v>
       </c>
       <c r="L5" t="n">
-        <v>6.75280748861428</v>
+        <v>6.720980619119699</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -12040,10 +12028,10 @@
         <v>500000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514799</v>
+        <v>514623</v>
       </c>
       <c r="L6" t="n">
-        <v>8.702231356315766</v>
+        <v>8.671007708555583</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -12104,10 +12092,10 @@
         <v>550000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>557735</v>
+        <v>557544</v>
       </c>
       <c r="L7" t="n">
-        <v>6.765757931634199</v>
+        <v>6.733818317478082</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -12168,7 +12156,7 @@
         <v>530000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>471863</v>
+        <v>471702</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -12232,10 +12220,10 @@
         <v>600000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>600670</v>
+        <v>600464</v>
       </c>
       <c r="L9" t="n">
-        <v>8.435580268699953</v>
+        <v>8.404167443843427</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -12296,10 +12284,10 @@
         <v>646000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>729477</v>
+        <v>729227</v>
       </c>
       <c r="L10" t="n">
-        <v>17.06400613041946</v>
+        <v>17.03557328513618</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -12360,7 +12348,7 @@
         <v>615000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>557735</v>
+        <v>557544</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -12424,7 +12412,7 @@
         <v>700000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>643606</v>
+        <v>643385</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -12488,7 +12476,7 @@
         <v>745000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>686542</v>
+        <v>686306</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -12552,7 +12540,7 @@
         <v>930000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>858284</v>
+        <v>857990</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -12623,7 +12611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12672,198 +12660,78 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 14Inch MX2E3 M4 Pro 12Core CPU 16Core GPU 24GB 512GB Silver</t>
+          <t>Apple MacBook Air 13 MDHF4 M5 10C CPU 10C GPU 16GB 1TB Midnight</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>640000</v>
+        <v>474999</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>634000</v>
+        <v>479999</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-6000</v>
+        <v>5000</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.9399999999999999</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 16Inch MX2V3 14Core CPU 32Core GPU M4 Max 36GB 1TB Silver</t>
+          <t>Apple MacBook Air 13 MDHJ4 M5 10C CPU 10C GPU 16GB 1TB Sky Blue</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>995000</v>
+        <v>474999</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>990000</v>
+        <v>479999</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>-5000</v>
+        <v>5000</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.5</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 16Inch MX303 14Core CPU 32Core GPU M4 Max 36GB 1TB Space Black</t>
+          <t>Apple MacBook Air 13 MDHC4 M5 10C CPU 10C GPU 16GB 1TB Starlight</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>995000</v>
+        <v>474999</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>990000</v>
+        <v>479999</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>-5000</v>
+        <v>5000</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.5</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDHE4 M5 10C CPU 8C GPU 16GB 512GB Midnight</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>422000</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>420000</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>-2000</v>
-      </c>
-      <c r="F5" t="n">
-        <v>-0.47</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDHH4 M5 10C CPU 8C GPU 16GB 512GB Sky Blue</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>422000</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>420000</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>-2000</v>
-      </c>
-      <c r="F6" t="n">
-        <v>-0.47</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDHA4 M5 10C CPU 8C GPU 16GB 512GB Starlight</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>422000</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>420000</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>-2000</v>
-      </c>
-      <c r="F7" t="n">
-        <v>-0.47</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 M5 MJ3E4 10 Core CPU 10 Core GPU 32GB 1TB Silver</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>755000</v>
-      </c>
-      <c r="D8" s="3" t="n">
-        <v>775000</v>
-      </c>
-      <c r="E8" s="3" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F8" t="n">
-        <v>2.65</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 M5 MJ3D4 10 Core CPU 10 Core GPU 32GB 1TB Space Black</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>745000</v>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>775000</v>
-      </c>
-      <c r="E9" s="3" t="n">
-        <v>30000</v>
-      </c>
-      <c r="F9" t="n">
-        <v>4.03</v>
+        <v>1.05</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F9"/>
-  <conditionalFormatting sqref="E2:E9">
+  <autoFilter ref="A1:F4"/>
+  <conditionalFormatting sqref="E2:E4">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
chore: price data 2026-09-29
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MacBook Pro'!$A$1:$S$93</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MacBook Air'!$A$1:$S$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20260928T095250708307+0000</t>
+          <t>20260929T095436204099+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-28T09:52:50.708307+00:00</t>
+          <t>2026-09-29T09:54:36.204099+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>276.909534</v>
+        <v>276.962836</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -1147,10 +1147,10 @@
         <v>470000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>686306</v>
+        <v>686439</v>
       </c>
       <c r="L2" t="n">
-        <v>35.16011808143889</v>
+        <v>35.17268103939315</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1214,10 +1214,10 @@
         <v>465000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>686306</v>
+        <v>686439</v>
       </c>
       <c r="L3" t="n">
-        <v>33.26591928381801</v>
+        <v>33.27884924953273</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>772148</v>
+        <v>772297</v>
       </c>
       <c r="L4" t="n">
-        <v>35.24570419142444</v>
+        <v>35.25819729974349</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>772148</v>
+        <v>772297</v>
       </c>
       <c r="L5" t="n">
-        <v>32.6555271787274</v>
+        <v>32.66852001237866</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>857990</v>
+        <v>858155</v>
       </c>
       <c r="L6" t="n">
-        <v>37.9946153218569</v>
+        <v>38.0065372805612</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1606,10 +1606,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>857990</v>
+        <v>858155</v>
       </c>
       <c r="L9" t="n">
-        <v>34.14841664821268</v>
+        <v>34.1610781269118</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1673,10 +1673,10 @@
         <v>582999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>857990</v>
+        <v>858155</v>
       </c>
       <c r="L10" t="n">
-        <v>32.05060665042716</v>
+        <v>32.06367148125921</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -1740,10 +1740,10 @@
         <v>587999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>857990</v>
+        <v>858155</v>
       </c>
       <c r="L11" t="n">
-        <v>31.46784927563258</v>
+        <v>31.4810261549487</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -1807,10 +1807,10 @@
         <v>600000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>857990</v>
+        <v>858155</v>
       </c>
       <c r="L12" t="n">
-        <v>30.06911502465064</v>
+        <v>30.0825608427382</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -1874,10 +1874,10 @@
         <v>634000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>857990</v>
+        <v>858155</v>
       </c>
       <c r="L13" t="n">
-        <v>26.1063648760475</v>
+        <v>26.1205726238267</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -1941,10 +1941,10 @@
         <v>643999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>943832</v>
+        <v>944014</v>
       </c>
       <c r="L14" t="n">
-        <v>31.76762389916849</v>
+        <v>31.78077867489253</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -2067,10 +2067,10 @@
         <v>650000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>943832</v>
+        <v>944014</v>
       </c>
       <c r="L16" t="n">
-        <v>31.13181159358869</v>
+        <v>31.14508894995202</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -2134,10 +2134,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1029674</v>
+        <v>1029872</v>
       </c>
       <c r="L17" t="n">
-        <v>32.01731810262277</v>
+        <v>32.03038824242236</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2201,10 +2201,10 @@
         <v>711999</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>1072595</v>
+        <v>1072802</v>
       </c>
       <c r="L18" t="n">
-        <v>33.61902675287504</v>
+        <v>33.6318351382641</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -2330,10 +2330,10 @@
         <v>720000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>1029674</v>
+        <v>1029872</v>
       </c>
       <c r="L20" t="n">
-        <v>30.07495576269771</v>
+        <v>30.088399335063</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -2459,10 +2459,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1072595</v>
+        <v>1072802</v>
       </c>
       <c r="L22" t="n">
-        <v>30.72874663782695</v>
+        <v>30.74211271045356</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2526,10 +2526,10 @@
         <v>772000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1029674</v>
+        <v>1029872</v>
       </c>
       <c r="L23" t="n">
-        <v>25.02481367889254</v>
+        <v>25.03922817592866</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -2593,10 +2593,10 @@
         <v>775000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1029674</v>
+        <v>1029872</v>
       </c>
       <c r="L24" t="n">
-        <v>24.73345932790378</v>
+        <v>24.74792983982476</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -2660,10 +2660,10 @@
         <v>775000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>1029674</v>
+        <v>1029872</v>
       </c>
       <c r="L25" t="n">
-        <v>24.73345932790378</v>
+        <v>24.74792983982476</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -2789,10 +2789,10 @@
         <v>810000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>1072595</v>
+        <v>1072802</v>
       </c>
       <c r="L27" t="n">
-        <v>24.48221369668887</v>
+        <v>24.49678505446485</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -2804,7 +2804,7 @@
         <v>61.99999999999999</v>
       </c>
       <c r="Q27" t="n">
-        <v>24.8</v>
+        <v>24.9</v>
       </c>
       <c r="R27" t="n">
         <v>3</v>
@@ -2853,10 +2853,10 @@
         <v>810000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>1244279</v>
+        <v>1244519</v>
       </c>
       <c r="L28" t="n">
-        <v>34.9020597470503</v>
+        <v>34.91461359770321</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -2982,10 +2982,10 @@
         <v>825000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1287200</v>
+        <v>1287448</v>
       </c>
       <c r="L30" t="n">
-        <v>35.90739589807333</v>
+        <v>35.91974200123034</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -3049,10 +3049,10 @@
         <v>829999</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1287200</v>
+        <v>1287448</v>
       </c>
       <c r="L31" t="n">
-        <v>35.51903356121815</v>
+        <v>35.53145447427779</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -3116,10 +3116,10 @@
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1373042</v>
+        <v>1373306</v>
       </c>
       <c r="L32" t="n">
-        <v>38.23939835780697</v>
+        <v>38.25127102044264</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3183,10 +3183,10 @@
         <v>930000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1373042</v>
+        <v>1373306</v>
       </c>
       <c r="L33" t="n">
-        <v>38.09373638970985</v>
+        <v>38.10563705394136</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3250,10 +3250,10 @@
         <v>860000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>1244279</v>
+        <v>1244519</v>
       </c>
       <c r="L34" t="n">
-        <v>30.88366837341143</v>
+        <v>30.89699715311699</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -3503,10 +3503,10 @@
         <v>880000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>1158437</v>
+        <v>1158660</v>
       </c>
       <c r="L38" t="n">
-        <v>24.0355755211548</v>
+        <v>24.0501959159719</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -3567,10 +3567,10 @@
         <v>940000</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>1244279</v>
+        <v>1244519</v>
       </c>
       <c r="L39" t="n">
-        <v>24.45424217558924</v>
+        <v>24.46881084177903</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -3631,10 +3631,10 @@
         <v>990000</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>1501805</v>
+        <v>1502094</v>
       </c>
       <c r="L40" t="n">
-        <v>34.07932454612949</v>
+        <v>34.0920075574498</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -3695,10 +3695,10 @@
         <v>990000</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>1501805</v>
+        <v>1502094</v>
       </c>
       <c r="L41" t="n">
-        <v>34.07932454612949</v>
+        <v>34.0920075574498</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
@@ -3821,10 +3821,10 @@
         <v>1055000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1544726</v>
+        <v>1545023</v>
       </c>
       <c r="L43" t="n">
-        <v>31.70309815462419</v>
+        <v>31.71622687817592</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -3885,10 +3885,10 @@
         <v>1055000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1544726</v>
+        <v>1545023</v>
       </c>
       <c r="L44" t="n">
-        <v>31.70309815462419</v>
+        <v>31.71622687817592</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -4011,10 +4011,10 @@
         <v>1115000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1501805</v>
+        <v>1502094</v>
       </c>
       <c r="L46" t="n">
-        <v>25.75600693831756</v>
+        <v>25.77029133995608</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -4075,10 +4075,10 @@
         <v>1123000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1716410</v>
+        <v>1716740</v>
       </c>
       <c r="L47" t="n">
-        <v>34.57274194394113</v>
+        <v>34.58531868541538</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -4142,10 +4142,10 @@
         <v>1130000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1501805</v>
+        <v>1502094</v>
       </c>
       <c r="L48" t="n">
-        <v>24.75720882538013</v>
+        <v>24.77168539385684</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -4268,10 +4268,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1759331</v>
+        <v>1759670</v>
       </c>
       <c r="L50" t="n">
-        <v>34.3500455570896</v>
+        <v>34.36269300493843</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4283,7 +4283,7 @@
         <v>22.53136001640632</v>
       </c>
       <c r="Q50" t="n">
-        <v>19.5</v>
+        <v>19.6</v>
       </c>
       <c r="R50" t="n">
         <v>3</v>
@@ -4332,10 +4332,10 @@
         <v>1155000</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>1759331</v>
+        <v>1759670</v>
       </c>
       <c r="L51" t="n">
-        <v>34.3500455570896</v>
+        <v>34.36269300493843</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -4347,7 +4347,7 @@
         <v>22.53136001640632</v>
       </c>
       <c r="Q51" t="n">
-        <v>19.5</v>
+        <v>19.6</v>
       </c>
       <c r="R51" t="n">
         <v>3</v>
@@ -4396,10 +4396,10 @@
         <v>1185000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1587647</v>
+        <v>1587953</v>
       </c>
       <c r="L52" t="n">
-        <v>25.36124214009789</v>
+        <v>25.37562509721635</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -4460,10 +4460,10 @@
         <v>1185000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1587647</v>
+        <v>1587953</v>
       </c>
       <c r="L53" t="n">
-        <v>25.36124214009789</v>
+        <v>25.37562509721635</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -4524,10 +4524,10 @@
         <v>1200000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1888094</v>
+        <v>1888457</v>
       </c>
       <c r="L54" t="n">
-        <v>36.44384230869861</v>
+        <v>36.4560591001013</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -4588,10 +4588,10 @@
         <v>1200000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1888094</v>
+        <v>1888457</v>
       </c>
       <c r="L55" t="n">
-        <v>36.44384230869861</v>
+        <v>36.4560591001013</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -4714,10 +4714,10 @@
         <v>1240000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1673489</v>
+        <v>1673811</v>
       </c>
       <c r="L57" t="n">
-        <v>25.90330740148277</v>
+        <v>25.91756177967525</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -4729,7 +4729,7 @@
         <v>100</v>
       </c>
       <c r="Q57" t="n">
-        <v>33.6</v>
+        <v>33.7</v>
       </c>
       <c r="R57" t="n">
         <v>3</v>
@@ -4840,10 +4840,10 @@
         <v>1280000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1716410</v>
+        <v>1716740</v>
       </c>
       <c r="L59" t="n">
-        <v>25.42574326646897</v>
+        <v>25.4400782879178</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -4907,10 +4907,10 @@
         <v>1298000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1759331</v>
+        <v>1759670</v>
       </c>
       <c r="L60" t="n">
-        <v>26.22195595939593</v>
+        <v>26.23616928174032</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -4971,10 +4971,10 @@
         <v>1300000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1716410</v>
+        <v>1716740</v>
       </c>
       <c r="L61" t="n">
-        <v>24.26052050500754</v>
+        <v>24.27507951116651</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -5097,10 +5097,10 @@
         <v>1335000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1802252</v>
+        <v>1802599</v>
       </c>
       <c r="L63" t="n">
-        <v>25.92600812760924</v>
+        <v>25.94026735840861</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -5161,10 +5161,10 @@
         <v>1420000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1931015</v>
+        <v>1931386</v>
       </c>
       <c r="L64" t="n">
-        <v>26.46354378396854</v>
+        <v>26.47766940425166</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -5225,10 +5225,10 @@
         <v>1430000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1931015</v>
+        <v>1931386</v>
       </c>
       <c r="L65" t="n">
-        <v>25.94568141625</v>
+        <v>25.95990651273231</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -5289,10 +5289,10 @@
         <v>1430000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>2145620</v>
+        <v>2146033</v>
       </c>
       <c r="L66" t="n">
-        <v>33.352597384439</v>
+        <v>33.36542355126878</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -5353,10 +5353,10 @@
         <v>1430000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>2145620</v>
+        <v>2146033</v>
       </c>
       <c r="L67" t="n">
-        <v>33.352597384439</v>
+        <v>33.36542355126878</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -5479,10 +5479,10 @@
         <v>1480000</v>
       </c>
       <c r="K69" s="3" t="n">
-        <v>2016857</v>
+        <v>2017245</v>
       </c>
       <c r="L69" t="n">
-        <v>26.61849600640998</v>
+        <v>26.63261031753704</v>
       </c>
       <c r="M69" s="3" t="n">
         <v>0</v>
@@ -5605,10 +5605,10 @@
         <v>1605000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2188541</v>
+        <v>2188962</v>
       </c>
       <c r="L71" t="n">
-        <v>26.66347123494602</v>
+        <v>26.67757594695568</v>
       </c>
       <c r="M71" s="3" t="n">
         <v>0</v>
@@ -5669,10 +5669,10 @@
         <v>1610000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2188541</v>
+        <v>2188962</v>
       </c>
       <c r="L72" t="n">
-        <v>26.43500852851283</v>
+        <v>26.4491571804353</v>
       </c>
       <c r="M72" s="3" t="n">
         <v>0</v>
@@ -5733,10 +5733,10 @@
         <v>1615000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2188541</v>
+        <v>2188962</v>
       </c>
       <c r="L73" t="n">
-        <v>26.20654582207964</v>
+        <v>26.22073841391491</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
@@ -5797,10 +5797,10 @@
         <v>1630000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2231462</v>
+        <v>2231891</v>
       </c>
       <c r="L74" t="n">
-        <v>26.95371913122429</v>
+        <v>26.96775962625415</v>
       </c>
       <c r="M74" s="3" t="n">
         <v>0</v>
@@ -5861,10 +5861,10 @@
         <v>1690000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2317304</v>
+        <v>2317750</v>
       </c>
       <c r="L75" t="n">
-        <v>27.07042321594405</v>
+        <v>27.08445690863984</v>
       </c>
       <c r="M75" s="3" t="n">
         <v>0</v>
@@ -5925,10 +5925,10 @@
         <v>1705000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2317304</v>
+        <v>2317750</v>
       </c>
       <c r="L76" t="n">
-        <v>26.42311927999089</v>
+        <v>26.43727753208931</v>
       </c>
       <c r="M76" s="3" t="n">
         <v>0</v>
@@ -5989,10 +5989,10 @@
         <v>1725000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2360225</v>
+        <v>2360679</v>
       </c>
       <c r="L77" t="n">
-        <v>26.9137476299929</v>
+        <v>26.92780339893734</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
@@ -6053,10 +6053,10 @@
         <v>1780000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2446067</v>
+        <v>2446537</v>
       </c>
       <c r="L78" t="n">
-        <v>27.23012084296955</v>
+        <v>27.24410053884327</v>
       </c>
       <c r="M78" s="3" t="n">
         <v>0</v>
@@ -6068,7 +6068,7 @@
         <v>38.78143936249688</v>
       </c>
       <c r="Q78" t="n">
-        <v>21.1</v>
+        <v>21.2</v>
       </c>
       <c r="R78" t="n">
         <v>3</v>
@@ -6117,10 +6117,10 @@
         <v>1875000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2574829</v>
+        <v>2575325</v>
       </c>
       <c r="L79" t="n">
-        <v>27.17963018126641</v>
+        <v>27.19365516973586</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
@@ -6181,10 +6181,10 @@
         <v>1910000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2617750</v>
+        <v>2618254</v>
       </c>
       <c r="L80" t="n">
-        <v>27.03657721325566</v>
+        <v>27.05062228492728</v>
       </c>
       <c r="M80" s="3" t="n">
         <v>0</v>
@@ -6245,10 +6245,10 @@
         <v>2020000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2746513</v>
+        <v>2747042</v>
       </c>
       <c r="L81" t="n">
-        <v>26.45219592989365</v>
+        <v>26.46635908733831</v>
       </c>
       <c r="M81" s="3" t="n">
         <v>0</v>
@@ -6309,10 +6309,10 @@
         <v>2110000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>2875276</v>
+        <v>2875830</v>
       </c>
       <c r="L82" t="n">
-        <v>26.61574054108197</v>
+        <v>26.62987728760045</v>
       </c>
       <c r="M82" s="3" t="n">
         <v>0</v>
@@ -6373,10 +6373,10 @@
         <v>2210000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3004039</v>
+        <v>3004617</v>
       </c>
       <c r="L83" t="n">
-        <v>26.4323798725649</v>
+        <v>26.44653212040004</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
@@ -6437,10 +6437,10 @@
         <v>2215000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3046960</v>
+        <v>3047547</v>
       </c>
       <c r="L84" t="n">
-        <v>27.30459211804553</v>
+        <v>27.31859426614257</v>
       </c>
       <c r="M84" s="3" t="n">
         <v>0</v>
@@ -6501,10 +6501,10 @@
         <v>2315000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3175723</v>
+        <v>3176334</v>
       </c>
       <c r="L85" t="n">
-        <v>27.10321397678576</v>
+        <v>27.11723641153607</v>
       </c>
       <c r="M85" s="3" t="n">
         <v>0</v>
@@ -6565,10 +6565,10 @@
         <v>2395000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3304486</v>
+        <v>3305122</v>
       </c>
       <c r="L86" t="n">
-        <v>27.52276753479966</v>
+        <v>27.5367142271904</v>
       </c>
       <c r="M86" s="3" t="n">
         <v>0</v>
@@ -6629,10 +6629,10 @@
         <v>2410000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3304486</v>
+        <v>3305122</v>
       </c>
       <c r="L87" t="n">
-        <v>27.06883914775248</v>
+        <v>27.08287318894734</v>
       </c>
       <c r="M87" s="3" t="n">
         <v>0</v>
@@ -6693,10 +6693,10 @@
         <v>2499000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3433249</v>
+        <v>3433910</v>
       </c>
       <c r="L88" t="n">
-        <v>27.21180432878594</v>
+        <v>27.22581546982885</v>
       </c>
       <c r="M88" s="3" t="n">
         <v>0</v>
@@ -6757,10 +6757,10 @@
         <v>2510000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3433249</v>
+        <v>3433910</v>
       </c>
       <c r="L89" t="n">
-        <v>26.89140810934482</v>
+        <v>26.9054809240778</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
@@ -6821,10 +6821,10 @@
         <v>2530000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3476170</v>
+        <v>3476839</v>
       </c>
       <c r="L90" t="n">
-        <v>27.21874937071547</v>
+        <v>27.23275365928649</v>
       </c>
       <c r="M90" s="3" t="n">
         <v>0</v>
@@ -6885,10 +6885,10 @@
         <v>2610000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>3604933</v>
+        <v>3605627</v>
       </c>
       <c r="L91" t="n">
-        <v>27.59920919473399</v>
+        <v>27.6131446763628</v>
       </c>
       <c r="M91" s="3" t="n">
         <v>0</v>
@@ -6949,10 +6949,10 @@
         <v>3015000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4162906</v>
+        <v>4163707</v>
       </c>
       <c r="L92" t="n">
-        <v>27.57463175964098</v>
+        <v>27.5885647092843</v>
       </c>
       <c r="M92" s="3" t="n">
         <v>0</v>
@@ -7013,10 +7013,10 @@
         <v>3098000</v>
       </c>
       <c r="K93" s="3" t="n">
-        <v>4291669</v>
+        <v>4292495</v>
       </c>
       <c r="L93" t="n">
-        <v>27.81363147996735</v>
+        <v>27.82752222192454</v>
       </c>
       <c r="M93" s="3" t="n">
         <v>0</v>
@@ -7312,10 +7312,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>428781</v>
+        <v>428863</v>
       </c>
       <c r="L2" t="n">
-        <v>27.70225359799058</v>
+        <v>27.71607716217067</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7379,10 +7379,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>428781</v>
+        <v>428863</v>
       </c>
       <c r="L3" t="n">
-        <v>27.70225359799058</v>
+        <v>27.71607716217067</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7446,10 +7446,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>428781</v>
+        <v>428863</v>
       </c>
       <c r="L4" t="n">
-        <v>27.70202037870148</v>
+        <v>27.71584398747385</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7513,10 +7513,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>428781</v>
+        <v>428863</v>
       </c>
       <c r="L5" t="n">
-        <v>27.70202037870148</v>
+        <v>27.71584398747385</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7580,10 +7580,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514623</v>
+        <v>514722</v>
       </c>
       <c r="L6" t="n">
-        <v>25.38227012784116</v>
+        <v>25.39662186578386</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7644,10 +7644,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>514623</v>
+        <v>514722</v>
       </c>
       <c r="L7" t="n">
-        <v>25.38227012784116</v>
+        <v>25.39662186578386</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7708,10 +7708,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>514623</v>
+        <v>514722</v>
       </c>
       <c r="L8" t="n">
-        <v>25.38227012784116</v>
+        <v>25.39662186578386</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7772,10 +7772,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>514623</v>
+        <v>514722</v>
       </c>
       <c r="L9" t="n">
-        <v>25.38227012784116</v>
+        <v>25.39662186578386</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7836,10 +7836,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>514623</v>
+        <v>514722</v>
       </c>
       <c r="L10" t="n">
-        <v>25.18795312296574</v>
+        <v>25.20234223522601</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7900,10 +7900,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>514623</v>
+        <v>514722</v>
       </c>
       <c r="L11" t="n">
-        <v>25.18795312296574</v>
+        <v>25.20234223522601</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7964,10 +7964,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>514623</v>
+        <v>514722</v>
       </c>
       <c r="L12" t="n">
-        <v>25.18795312296574</v>
+        <v>25.20234223522601</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -8028,10 +8028,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>514623</v>
+        <v>514722</v>
       </c>
       <c r="L13" t="n">
-        <v>25.18795312296574</v>
+        <v>25.20234223522601</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -8092,10 +8092,10 @@
         <v>420000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>557544</v>
+        <v>557651</v>
       </c>
       <c r="L14" t="n">
-        <v>24.66962248719383</v>
+        <v>24.68407659988057</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -8159,10 +8159,10 @@
         <v>420000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>557544</v>
+        <v>557651</v>
       </c>
       <c r="L15" t="n">
-        <v>24.66962248719383</v>
+        <v>24.68407659988057</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0</v>
@@ -8226,10 +8226,10 @@
         <v>420000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>557544</v>
+        <v>557651</v>
       </c>
       <c r="L16" t="n">
-        <v>24.66962248719383</v>
+        <v>24.68407659988057</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -8293,10 +8293,10 @@
         <v>425000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>557544</v>
+        <v>557651</v>
       </c>
       <c r="L17" t="n">
-        <v>23.77283227870805</v>
+        <v>23.78745846416486</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -8360,10 +8360,10 @@
         <v>454000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>600464</v>
+        <v>600580</v>
       </c>
       <c r="L18" t="n">
-        <v>24.39180367182712</v>
+        <v>24.40640713976489</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -8375,7 +8375,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q18" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="R18" t="n">
         <v>3</v>
@@ -8424,10 +8424,10 @@
         <v>454000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>600464</v>
+        <v>600580</v>
       </c>
       <c r="L19" t="n">
-        <v>24.39180367182712</v>
+        <v>24.40640713976489</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -8439,7 +8439,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q19" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="R19" t="n">
         <v>3</v>
@@ -8488,10 +8488,10 @@
         <v>454000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>600464</v>
+        <v>600580</v>
       </c>
       <c r="L20" t="n">
-        <v>24.39180367182712</v>
+        <v>24.40640713976489</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -8503,7 +8503,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q20" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="R20" t="n">
         <v>3</v>
@@ -8552,10 +8552,10 @@
         <v>454000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>600464</v>
+        <v>600580</v>
       </c>
       <c r="L21" t="n">
-        <v>24.39180367182712</v>
+        <v>24.40640713976489</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -8567,7 +8567,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q21" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="R21" t="n">
         <v>3</v>
@@ -8616,10 +8616,10 @@
         <v>455000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>600464</v>
+        <v>600580</v>
       </c>
       <c r="L22" t="n">
-        <v>24.22526579445229</v>
+        <v>24.239901428619</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -8680,10 +8680,10 @@
         <v>455000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>600464</v>
+        <v>600580</v>
       </c>
       <c r="L23" t="n">
-        <v>24.22526579445229</v>
+        <v>24.239901428619</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -8744,10 +8744,10 @@
         <v>455000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>600464</v>
+        <v>600580</v>
       </c>
       <c r="L24" t="n">
-        <v>24.22526579445229</v>
+        <v>24.239901428619</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -8808,10 +8808,10 @@
         <v>455000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>600464</v>
+        <v>600580</v>
       </c>
       <c r="L25" t="n">
-        <v>24.22526579445229</v>
+        <v>24.239901428619</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -8872,10 +8872,10 @@
         <v>475000</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>686306</v>
+        <v>686439</v>
       </c>
       <c r="L26" t="n">
-        <v>30.78889008692915</v>
+        <v>30.8022999858691</v>
       </c>
       <c r="M26" s="3" t="n">
         <v>0</v>
@@ -8936,10 +8936,10 @@
         <v>475000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>686306</v>
+        <v>686439</v>
       </c>
       <c r="L27" t="n">
-        <v>30.78889008692915</v>
+        <v>30.8022999858691</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -9000,10 +9000,10 @@
         <v>475000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>686306</v>
+        <v>686439</v>
       </c>
       <c r="L28" t="n">
-        <v>30.78889008692915</v>
+        <v>30.8022999858691</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -9064,10 +9064,10 @@
         <v>475000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>686306</v>
+        <v>686439</v>
       </c>
       <c r="L29" t="n">
-        <v>30.78889008692915</v>
+        <v>30.8022999858691</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -9128,13 +9128,13 @@
         <v>479999</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>686306</v>
+        <v>686439</v>
       </c>
       <c r="L30" t="n">
-        <v>30.06049779544401</v>
+        <v>30.07404882298354</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="N30" t="n">
         <v>0</v>
@@ -9143,7 +9143,7 @@
         <v>43.6979831932773</v>
       </c>
       <c r="Q30" t="n">
-        <v>22.2</v>
+        <v>22.3</v>
       </c>
       <c r="R30" t="n">
         <v>3</v>
@@ -9192,13 +9192,13 @@
         <v>479999</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>686306</v>
+        <v>686439</v>
       </c>
       <c r="L31" t="n">
-        <v>30.06049779544401</v>
+        <v>30.07404882298354</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="N31" t="n">
         <v>0</v>
@@ -9207,7 +9207,7 @@
         <v>43.6979831932773</v>
       </c>
       <c r="Q31" t="n">
-        <v>22.2</v>
+        <v>22.3</v>
       </c>
       <c r="R31" t="n">
         <v>3</v>
@@ -9256,10 +9256,10 @@
         <v>479999</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>686306</v>
+        <v>686439</v>
       </c>
       <c r="L32" t="n">
-        <v>30.06049779544401</v>
+        <v>30.07404882298354</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -9271,7 +9271,7 @@
         <v>43.6979831932773</v>
       </c>
       <c r="Q32" t="n">
-        <v>22.2</v>
+        <v>22.3</v>
       </c>
       <c r="R32" t="n">
         <v>3</v>
@@ -9320,13 +9320,13 @@
         <v>479999</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>686306</v>
+        <v>686439</v>
       </c>
       <c r="L33" t="n">
-        <v>30.06049779544401</v>
+        <v>30.07404882298354</v>
       </c>
       <c r="M33" s="3" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="N33" t="n">
         <v>0</v>
@@ -9335,7 +9335,7 @@
         <v>43.6979831932773</v>
       </c>
       <c r="Q33" t="n">
-        <v>22.2</v>
+        <v>22.3</v>
       </c>
       <c r="R33" t="n">
         <v>3</v>
@@ -9384,10 +9384,10 @@
         <v>479999</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>643385</v>
+        <v>643509</v>
       </c>
       <c r="L34" t="n">
-        <v>25.39474809017929</v>
+        <v>25.40912403711526</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -9451,10 +9451,10 @@
         <v>479999</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>643385</v>
+        <v>643509</v>
       </c>
       <c r="L35" t="n">
-        <v>25.39474809017929</v>
+        <v>25.40912403711526</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
@@ -9518,10 +9518,10 @@
         <v>479999</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>643385</v>
+        <v>643509</v>
       </c>
       <c r="L36" t="n">
-        <v>25.39474809017929</v>
+        <v>25.40912403711526</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -9585,10 +9585,10 @@
         <v>484999</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>643385</v>
+        <v>643509</v>
       </c>
       <c r="L37" t="n">
-        <v>24.61760843041103</v>
+        <v>24.63213412710623</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
@@ -9652,10 +9652,10 @@
         <v>500000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>643385</v>
+        <v>643509</v>
       </c>
       <c r="L38" t="n">
-        <v>22.28603402317431</v>
+        <v>22.30100899909714</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -9716,10 +9716,10 @@
         <v>547999</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>772148</v>
+        <v>772297</v>
       </c>
       <c r="L39" t="n">
-        <v>29.02927936095153</v>
+        <v>29.04297181006789</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -9780,10 +9780,10 @@
         <v>547999</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>772148</v>
+        <v>772297</v>
       </c>
       <c r="L40" t="n">
-        <v>29.02927936095153</v>
+        <v>29.04297181006789</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -9844,10 +9844,10 @@
         <v>547999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>772148</v>
+        <v>772297</v>
       </c>
       <c r="L41" t="n">
-        <v>29.02927936095153</v>
+        <v>29.04297181006789</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
@@ -9908,10 +9908,10 @@
         <v>547999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>772148</v>
+        <v>772297</v>
       </c>
       <c r="L42" t="n">
-        <v>29.02927936095153</v>
+        <v>29.04297181006789</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -9972,10 +9972,10 @@
         <v>552999</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>772148</v>
+        <v>772297</v>
       </c>
       <c r="L43" t="n">
-        <v>28.38173510777727</v>
+        <v>28.39555248822668</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -10036,10 +10036,10 @@
         <v>552999</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>772148</v>
+        <v>772297</v>
       </c>
       <c r="L44" t="n">
-        <v>28.38173510777727</v>
+        <v>28.39555248822668</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -10100,10 +10100,10 @@
         <v>552999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>772148</v>
+        <v>772297</v>
       </c>
       <c r="L45" t="n">
-        <v>28.38173510777727</v>
+        <v>28.39555248822668</v>
       </c>
       <c r="M45" s="3" t="n">
         <v>0</v>
@@ -10164,10 +10164,10 @@
         <v>552999</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>772148</v>
+        <v>772297</v>
       </c>
       <c r="L46" t="n">
-        <v>28.38173510777727</v>
+        <v>28.39555248822668</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -10228,10 +10228,10 @@
         <v>585000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>729227</v>
+        <v>729368</v>
       </c>
       <c r="L47" t="n">
-        <v>19.77806636342319</v>
+        <v>19.79357471125687</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -10292,10 +10292,10 @@
         <v>595000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>729227</v>
+        <v>729368</v>
       </c>
       <c r="L48" t="n">
-        <v>18.40675125852444</v>
+        <v>18.42252470632109</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -10356,10 +10356,10 @@
         <v>614999</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>857990</v>
+        <v>858155</v>
       </c>
       <c r="L49" t="n">
-        <v>28.32095945174186</v>
+        <v>28.33474139287192</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -10420,10 +10420,10 @@
         <v>614999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>857990</v>
+        <v>858155</v>
       </c>
       <c r="L50" t="n">
-        <v>28.32095945174186</v>
+        <v>28.33474139287192</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -10484,10 +10484,10 @@
         <v>614999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>857990</v>
+        <v>858155</v>
       </c>
       <c r="L51" t="n">
-        <v>28.32095945174186</v>
+        <v>28.33474139287192</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -10548,10 +10548,10 @@
         <v>614999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>857990</v>
+        <v>858155</v>
       </c>
       <c r="L52" t="n">
-        <v>28.32095945174186</v>
+        <v>28.33474139287192</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -10612,10 +10612,10 @@
         <v>650000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>815069</v>
+        <v>815226</v>
       </c>
       <c r="L53" t="n">
-        <v>20.25215043143587</v>
+        <v>20.26750864177541</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -10676,10 +10676,10 @@
         <v>672000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>857990</v>
+        <v>858155</v>
       </c>
       <c r="L54" t="n">
-        <v>21.67740882760871</v>
+        <v>21.69246814386678</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -10740,10 +10740,10 @@
         <v>700000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>900911</v>
+        <v>901085</v>
       </c>
       <c r="L55" t="n">
-        <v>22.30087100723601</v>
+        <v>22.31587475099463</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -10804,10 +10804,10 @@
         <v>715000</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>943832</v>
+        <v>944014</v>
       </c>
       <c r="L56" t="n">
-        <v>24.24499275294756</v>
+        <v>24.25959784494722</v>
       </c>
       <c r="M56" s="3" t="n">
         <v>0</v>
@@ -10868,22 +10868,22 @@
         <v>734999</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>986753</v>
+        <v>986943</v>
       </c>
       <c r="L57" t="n">
-        <v>25.51337568773543</v>
+        <v>25.52771537971291</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N57" t="n">
-        <v>1.408518717987068</v>
+        <v>0</v>
       </c>
       <c r="P57" t="n">
         <v>73.94986794717886</v>
       </c>
       <c r="Q57" t="n">
-        <v>27.3</v>
+        <v>26.8</v>
       </c>
       <c r="R57" t="n">
         <v>3</v>
@@ -10932,10 +10932,10 @@
         <v>752000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>986753</v>
+        <v>986943</v>
       </c>
       <c r="L58" t="n">
-        <v>23.79045211922335</v>
+        <v>23.80512349750695</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -10996,10 +10996,10 @@
         <v>810000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1072595</v>
+        <v>1072802</v>
       </c>
       <c r="L59" t="n">
-        <v>24.48221369668887</v>
+        <v>24.49678505446485</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -11011,7 +11011,7 @@
         <v>70.24552627383726</v>
       </c>
       <c r="Q59" t="n">
-        <v>25.5</v>
+        <v>25.6</v>
       </c>
       <c r="R59" t="n">
         <v>3</v>
@@ -11060,10 +11060,10 @@
         <v>815000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1072595</v>
+        <v>1072802</v>
       </c>
       <c r="L60" t="n">
-        <v>24.01605452197707</v>
+        <v>24.03071582640599</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -11124,10 +11124,10 @@
         <v>875000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1158437</v>
+        <v>1158660</v>
       </c>
       <c r="L61" t="n">
-        <v>24.46719156933005</v>
+        <v>24.48172889372206</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -11188,10 +11188,10 @@
         <v>992000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1330121</v>
+        <v>1330377</v>
       </c>
       <c r="L62" t="n">
-        <v>25.42031890331782</v>
+        <v>25.43467002210652</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -11203,7 +11203,7 @@
         <v>85.64705882352939</v>
       </c>
       <c r="Q62" t="n">
-        <v>29.2</v>
+        <v>29.3</v>
       </c>
       <c r="R62" t="n">
         <v>3</v>
@@ -11252,10 +11252,10 @@
         <v>1050000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1415963</v>
+        <v>1416236</v>
       </c>
       <c r="L63" t="n">
-        <v>25.8455199747451</v>
+        <v>25.85981432473119</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -11267,7 +11267,7 @@
         <v>93.20091673032849</v>
       </c>
       <c r="Q63" t="n">
-        <v>31</v>
+        <v>31.1</v>
       </c>
       <c r="R63" t="n">
         <v>3</v>
@@ -11316,10 +11316,10 @@
         <v>1050000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1415963</v>
+        <v>1416236</v>
       </c>
       <c r="L64" t="n">
-        <v>25.8455199747451</v>
+        <v>25.85981432473119</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -11380,10 +11380,10 @@
         <v>1100000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1501805</v>
+        <v>1502094</v>
       </c>
       <c r="L65" t="n">
-        <v>26.75480505125499</v>
+        <v>26.76889728605533</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -11444,10 +11444,10 @@
         <v>1105000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1501805</v>
+        <v>1502094</v>
       </c>
       <c r="L66" t="n">
-        <v>26.42187234694251</v>
+        <v>26.43602863735558</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -11508,10 +11508,10 @@
         <v>1155000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1587647</v>
+        <v>1587953</v>
       </c>
       <c r="L67" t="n">
-        <v>27.2508309466777</v>
+        <v>27.26484977829948</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -11778,7 +11778,7 @@
         <v>315000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>300018</v>
+        <v>300075</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -11839,10 +11839,10 @@
         <v>380000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>385860</v>
+        <v>385934</v>
       </c>
       <c r="L3" t="n">
-        <v>1.518685533613228</v>
+        <v>1.537568599812403</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -11903,7 +11903,7 @@
         <v>415000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>385860</v>
+        <v>385934</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -11964,10 +11964,10 @@
         <v>495000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>471702</v>
+        <v>471792</v>
       </c>
       <c r="L5" t="n">
-        <v>6.720980619119699</v>
+        <v>6.738774714280869</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -12028,10 +12028,10 @@
         <v>500000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514623</v>
+        <v>514722</v>
       </c>
       <c r="L6" t="n">
-        <v>8.671007708555583</v>
+        <v>8.688573637808371</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -12092,10 +12092,10 @@
         <v>550000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>557544</v>
+        <v>557651</v>
       </c>
       <c r="L7" t="n">
-        <v>6.733818317478082</v>
+        <v>6.751713885566421</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -12156,7 +12156,7 @@
         <v>530000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>471702</v>
+        <v>471792</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -12220,10 +12220,10 @@
         <v>600000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>600464</v>
+        <v>600580</v>
       </c>
       <c r="L9" t="n">
-        <v>8.404167443843427</v>
+        <v>8.421858869759232</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -12284,10 +12284,10 @@
         <v>646000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>729227</v>
+        <v>729368</v>
       </c>
       <c r="L10" t="n">
-        <v>17.03557328513618</v>
+        <v>17.0516118063858</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -12348,7 +12348,7 @@
         <v>615000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>557544</v>
+        <v>557651</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -12412,7 +12412,7 @@
         <v>700000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>643385</v>
+        <v>643509</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -12476,7 +12476,7 @@
         <v>745000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>686306</v>
+        <v>686439</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -12540,7 +12540,7 @@
         <v>930000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>857990</v>
+        <v>858155</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -12611,7 +12611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12657,88 +12657,8 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDHF4 M5 10C CPU 10C GPU 16GB 1TB Midnight</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>474999</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>479999</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F2" t="n">
-        <v>1.05</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDHJ4 M5 10C CPU 10C GPU 16GB 1TB Sky Blue</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>474999</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>479999</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F3" t="n">
-        <v>1.05</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDHC4 M5 10C CPU 10C GPU 16GB 1TB Starlight</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>474999</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>479999</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F4" t="n">
-        <v>1.05</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:F4"/>
-  <conditionalFormatting sqref="E2:E4">
-    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
+  <autoFilter ref="A1:F1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: price data 2026-09-30
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MacBook Pro'!$A$1:$S$93</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MacBook Air'!$A$1:$S$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20260929T095436204099+0000</t>
+          <t>20260930T094648863561+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-29T09:54:36.204099+00:00</t>
+          <t>2026-09-30T09:46:48.863561+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>276.962836</v>
+        <v>276.877066</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -855,7 +855,7 @@
         <v>720000</v>
       </c>
       <c r="D28" t="n">
-        <v>44.4</v>
+        <v>44.3</v>
       </c>
       <c r="E28" t="n">
         <v>3</v>
@@ -897,7 +897,7 @@
         <v>725000</v>
       </c>
       <c r="D30" t="n">
-        <v>43.1</v>
+        <v>42.9</v>
       </c>
       <c r="E30" t="n">
         <v>3</v>
@@ -1147,10 +1147,10 @@
         <v>470000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>686439</v>
+        <v>686226</v>
       </c>
       <c r="L2" t="n">
-        <v>35.17268103939315</v>
+        <v>35.15255906946108</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1214,10 +1214,10 @@
         <v>465000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>686439</v>
+        <v>686226</v>
       </c>
       <c r="L3" t="n">
-        <v>33.27884924953273</v>
+        <v>33.25813944677118</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>772297</v>
+        <v>772058</v>
       </c>
       <c r="L4" t="n">
-        <v>35.25819729974349</v>
+        <v>35.23815568260416</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>772297</v>
+        <v>772058</v>
       </c>
       <c r="L5" t="n">
-        <v>32.66852001237866</v>
+        <v>32.64767672895042</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>858155</v>
+        <v>857890</v>
       </c>
       <c r="L6" t="n">
-        <v>38.0065372805612</v>
+        <v>37.98738766042267</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1606,10 +1606,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>858155</v>
+        <v>857890</v>
       </c>
       <c r="L9" t="n">
-        <v>34.1610781269118</v>
+        <v>34.14074065439625</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1667,31 +1667,31 @@
         </is>
       </c>
       <c r="I10" s="3" t="n">
-        <v>582999</v>
+        <v>579999</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>582999</v>
+        <v>579999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>858155</v>
+        <v>857890</v>
       </c>
       <c r="L10" t="n">
-        <v>32.06367148125921</v>
+        <v>32.39238130762685</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>0</v>
+        <v>-3000</v>
       </c>
       <c r="N10" t="n">
-        <v>0</v>
+        <v>0.5145806425053902</v>
       </c>
       <c r="O10" t="n">
         <v>100</v>
       </c>
       <c r="P10" t="n">
-        <v>49.10029999999999</v>
+        <v>50.00029999999999</v>
       </c>
       <c r="Q10" t="n">
-        <v>41.1</v>
+        <v>41.5</v>
       </c>
       <c r="R10" t="n">
         <v>4</v>
@@ -1740,10 +1740,10 @@
         <v>587999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>858155</v>
+        <v>857890</v>
       </c>
       <c r="L11" t="n">
-        <v>31.4810261549487</v>
+        <v>31.45986082131742</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -1807,10 +1807,10 @@
         <v>600000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>858155</v>
+        <v>857890</v>
       </c>
       <c r="L12" t="n">
-        <v>30.0825608427382</v>
+        <v>30.06096352679248</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -1874,10 +1874,10 @@
         <v>634000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>858155</v>
+        <v>857890</v>
       </c>
       <c r="L13" t="n">
-        <v>26.1205726238267</v>
+        <v>26.09775145997738</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -1941,10 +1941,10 @@
         <v>643999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>944014</v>
+        <v>943722</v>
       </c>
       <c r="L14" t="n">
-        <v>31.78077867489253</v>
+        <v>31.75967075049644</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -2067,10 +2067,10 @@
         <v>650000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>944014</v>
+        <v>943722</v>
       </c>
       <c r="L16" t="n">
-        <v>31.14508894995202</v>
+        <v>31.12378433479351</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -2134,10 +2134,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1029872</v>
+        <v>1029554</v>
       </c>
       <c r="L17" t="n">
-        <v>32.03038824242236</v>
+        <v>32.00939435911084</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2201,10 +2201,10 @@
         <v>711999</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>1072802</v>
+        <v>1072469</v>
       </c>
       <c r="L18" t="n">
-        <v>33.6318351382641</v>
+        <v>33.61122792360432</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -2272,7 +2272,7 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>1.098901098901099</v>
+        <v>0.8946324119975306</v>
       </c>
       <c r="O19" t="n">
         <v>100</v>
@@ -2281,7 +2281,7 @@
         <v>42.39316239316239</v>
       </c>
       <c r="Q19" t="n">
-        <v>44.4</v>
+        <v>44.3</v>
       </c>
       <c r="R19" t="n">
         <v>3</v>
@@ -2330,10 +2330,10 @@
         <v>720000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>1029872</v>
+        <v>1029554</v>
       </c>
       <c r="L20" t="n">
-        <v>30.088399335063</v>
+        <v>30.066805626514</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -2401,7 +2401,7 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>1.360544217687075</v>
+        <v>1.023823224452713</v>
       </c>
       <c r="O21" t="n">
         <v>96.7741935483871</v>
@@ -2410,7 +2410,7 @@
         <v>41.02564102564102</v>
       </c>
       <c r="Q21" t="n">
-        <v>43.1</v>
+        <v>42.9</v>
       </c>
       <c r="R21" t="n">
         <v>3</v>
@@ -2459,10 +2459,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1072802</v>
+        <v>1072469</v>
       </c>
       <c r="L22" t="n">
-        <v>30.74211271045356</v>
+        <v>30.72060824135709</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2526,10 +2526,10 @@
         <v>772000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1029872</v>
+        <v>1029554</v>
       </c>
       <c r="L23" t="n">
-        <v>25.03922817592866</v>
+        <v>25.01607492176224</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -2593,10 +2593,10 @@
         <v>775000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1029872</v>
+        <v>1029554</v>
       </c>
       <c r="L24" t="n">
-        <v>24.74792983982476</v>
+        <v>24.72468661187272</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -2660,10 +2660,10 @@
         <v>775000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>1029872</v>
+        <v>1029554</v>
       </c>
       <c r="L25" t="n">
-        <v>24.74792983982476</v>
+        <v>24.72468661187272</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -2789,10 +2789,10 @@
         <v>810000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>1072802</v>
+        <v>1072469</v>
       </c>
       <c r="L27" t="n">
-        <v>24.49678505446485</v>
+        <v>24.47334142059118</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -2804,7 +2804,7 @@
         <v>61.99999999999999</v>
       </c>
       <c r="Q27" t="n">
-        <v>24.9</v>
+        <v>24.8</v>
       </c>
       <c r="R27" t="n">
         <v>3</v>
@@ -2853,10 +2853,10 @@
         <v>810000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>1244519</v>
+        <v>1244133</v>
       </c>
       <c r="L28" t="n">
-        <v>34.91461359770321</v>
+        <v>34.89442045183272</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -2982,16 +2982,16 @@
         <v>825000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1287448</v>
+        <v>1287049</v>
       </c>
       <c r="L30" t="n">
-        <v>35.91974200123034</v>
+        <v>35.89987638388282</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N30" t="n">
-        <v>0.9602652584216788</v>
+        <v>0.7816004589301971</v>
       </c>
       <c r="O30" t="n">
         <v>100</v>
@@ -3049,16 +3049,16 @@
         <v>829999</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1287448</v>
+        <v>1287049</v>
       </c>
       <c r="L31" t="n">
-        <v>35.53145447427779</v>
+        <v>35.51146848332892</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N31" t="n">
-        <v>4.597816091954023</v>
+        <v>2.924093567251462</v>
       </c>
       <c r="O31" t="n">
         <v>0</v>
@@ -3067,7 +3067,7 @@
         <v>0</v>
       </c>
       <c r="Q31" t="n">
-        <v>13.1</v>
+        <v>12.6</v>
       </c>
       <c r="R31" t="n">
         <v>4</v>
@@ -3116,10 +3116,10 @@
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1373306</v>
+        <v>1372881</v>
       </c>
       <c r="L32" t="n">
-        <v>38.25127102044264</v>
+        <v>38.23215559105269</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3183,10 +3183,10 @@
         <v>930000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1373306</v>
+        <v>1372881</v>
       </c>
       <c r="L33" t="n">
-        <v>38.10563705394136</v>
+        <v>38.08647654093836</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3250,10 +3250,10 @@
         <v>860000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>1244519</v>
+        <v>1244133</v>
       </c>
       <c r="L34" t="n">
-        <v>30.89699715311699</v>
+        <v>30.87555751676067</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -3503,10 +3503,10 @@
         <v>880000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>1158660</v>
+        <v>1158301</v>
       </c>
       <c r="L38" t="n">
-        <v>24.0501959159719</v>
+        <v>24.02665628364302</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -3567,10 +3567,10 @@
         <v>940000</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>1244519</v>
+        <v>1244133</v>
       </c>
       <c r="L39" t="n">
-        <v>24.46881084177903</v>
+        <v>24.44537682064538</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -3631,10 +3631,10 @@
         <v>990000</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>1502094</v>
+        <v>1501629</v>
       </c>
       <c r="L40" t="n">
-        <v>34.0920075574498</v>
+        <v>34.07159824430668</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -3695,10 +3695,10 @@
         <v>990000</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>1502094</v>
+        <v>1501629</v>
       </c>
       <c r="L41" t="n">
-        <v>34.0920075574498</v>
+        <v>34.07159824430668</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
@@ -3821,10 +3821,10 @@
         <v>1055000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1545023</v>
+        <v>1544545</v>
       </c>
       <c r="L43" t="n">
-        <v>31.71622687817592</v>
+        <v>31.69509467189366</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -3885,16 +3885,16 @@
         <v>1055000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1545023</v>
+        <v>1544545</v>
       </c>
       <c r="L44" t="n">
-        <v>31.71622687817592</v>
+        <v>31.69509467189366</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>2.764976958525346</v>
+        <v>2.54041570438799</v>
       </c>
       <c r="P44" t="n">
         <v>58.64647440248988</v>
@@ -4011,10 +4011,10 @@
         <v>1115000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1502094</v>
+        <v>1501629</v>
       </c>
       <c r="L46" t="n">
-        <v>25.77029133995608</v>
+        <v>25.7473050933353</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -4075,10 +4075,10 @@
         <v>1123000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1716740</v>
+        <v>1716209</v>
       </c>
       <c r="L47" t="n">
-        <v>34.58531868541538</v>
+        <v>34.56507919489992</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -4142,10 +4142,10 @@
         <v>1130000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1502094</v>
+        <v>1501629</v>
       </c>
       <c r="L48" t="n">
-        <v>24.77168539385684</v>
+        <v>24.74838991521874</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -4268,10 +4268,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1759670</v>
+        <v>1759125</v>
       </c>
       <c r="L50" t="n">
-        <v>34.36269300493843</v>
+        <v>34.342357706246</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4283,7 +4283,7 @@
         <v>22.53136001640632</v>
       </c>
       <c r="Q50" t="n">
-        <v>19.6</v>
+        <v>19.5</v>
       </c>
       <c r="R50" t="n">
         <v>3</v>
@@ -4332,10 +4332,10 @@
         <v>1155000</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>1759670</v>
+        <v>1759125</v>
       </c>
       <c r="L51" t="n">
-        <v>34.36269300493843</v>
+        <v>34.342357706246</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -4347,7 +4347,7 @@
         <v>22.53136001640632</v>
       </c>
       <c r="Q51" t="n">
-        <v>19.6</v>
+        <v>19.5</v>
       </c>
       <c r="R51" t="n">
         <v>3</v>
@@ -4396,10 +4396,10 @@
         <v>1185000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1587953</v>
+        <v>1587461</v>
       </c>
       <c r="L52" t="n">
-        <v>25.37562509721635</v>
+        <v>25.35249684874148</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -4460,10 +4460,10 @@
         <v>1185000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1587953</v>
+        <v>1587461</v>
       </c>
       <c r="L53" t="n">
-        <v>25.37562509721635</v>
+        <v>25.35249684874148</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -4524,10 +4524,10 @@
         <v>1200000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1888457</v>
+        <v>1887872</v>
       </c>
       <c r="L54" t="n">
-        <v>36.4560591001013</v>
+        <v>36.4363685673605</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -4588,10 +4588,10 @@
         <v>1200000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1888457</v>
+        <v>1887872</v>
       </c>
       <c r="L55" t="n">
-        <v>36.4560591001013</v>
+        <v>36.4363685673605</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -4714,10 +4714,10 @@
         <v>1240000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1673811</v>
+        <v>1673293</v>
       </c>
       <c r="L57" t="n">
-        <v>25.91756177967525</v>
+        <v>25.89462813745112</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -4729,7 +4729,7 @@
         <v>100</v>
       </c>
       <c r="Q57" t="n">
-        <v>33.7</v>
+        <v>33.6</v>
       </c>
       <c r="R57" t="n">
         <v>3</v>
@@ -4840,10 +4840,10 @@
         <v>1280000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1716740</v>
+        <v>1716209</v>
       </c>
       <c r="L59" t="n">
-        <v>25.4400782879178</v>
+        <v>25.41700923372386</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -4907,10 +4907,10 @@
         <v>1298000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1759670</v>
+        <v>1759125</v>
       </c>
       <c r="L60" t="n">
-        <v>26.23616928174032</v>
+        <v>26.21331627940027</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -4971,10 +4971,10 @@
         <v>1300000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1716740</v>
+        <v>1716209</v>
       </c>
       <c r="L61" t="n">
-        <v>24.27507951116651</v>
+        <v>24.2516500030008</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -5097,10 +5097,10 @@
         <v>1335000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1802599</v>
+        <v>1802041</v>
       </c>
       <c r="L63" t="n">
-        <v>25.94026735840861</v>
+        <v>25.91733484421276</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -5161,10 +5161,10 @@
         <v>1420000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1931386</v>
+        <v>1930788</v>
       </c>
       <c r="L64" t="n">
-        <v>26.47766940425166</v>
+        <v>26.45489820736404</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -5225,10 +5225,10 @@
         <v>1430000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1931386</v>
+        <v>1930788</v>
       </c>
       <c r="L65" t="n">
-        <v>25.95990651273231</v>
+        <v>25.93697495530322</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -5289,10 +5289,10 @@
         <v>1430000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>2146033</v>
+        <v>2145368</v>
       </c>
       <c r="L66" t="n">
-        <v>33.36542355126878</v>
+        <v>33.34476882287794</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -5353,10 +5353,10 @@
         <v>1430000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>2146033</v>
+        <v>2145368</v>
       </c>
       <c r="L67" t="n">
-        <v>33.36542355126878</v>
+        <v>33.34476882287794</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -5479,10 +5479,10 @@
         <v>1480000</v>
       </c>
       <c r="K69" s="3" t="n">
-        <v>2017245</v>
+        <v>2016620</v>
       </c>
       <c r="L69" t="n">
-        <v>26.63261031753704</v>
+        <v>26.60987196397933</v>
       </c>
       <c r="M69" s="3" t="n">
         <v>0</v>
@@ -5605,10 +5605,10 @@
         <v>1605000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2188962</v>
+        <v>2188284</v>
       </c>
       <c r="L71" t="n">
-        <v>26.67757594695568</v>
+        <v>26.65485832734691</v>
       </c>
       <c r="M71" s="3" t="n">
         <v>0</v>
@@ -5669,10 +5669,10 @@
         <v>1610000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2188962</v>
+        <v>2188284</v>
       </c>
       <c r="L72" t="n">
-        <v>26.4491571804353</v>
+        <v>26.42636878942587</v>
       </c>
       <c r="M72" s="3" t="n">
         <v>0</v>
@@ -5733,10 +5733,10 @@
         <v>1615000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2188962</v>
+        <v>2188284</v>
       </c>
       <c r="L73" t="n">
-        <v>26.22073841391491</v>
+        <v>26.19787925150483</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
@@ -5797,10 +5797,10 @@
         <v>1630000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2231891</v>
+        <v>2231200</v>
       </c>
       <c r="L74" t="n">
-        <v>26.96775962625415</v>
+        <v>26.94514162782359</v>
       </c>
       <c r="M74" s="3" t="n">
         <v>0</v>
@@ -5861,10 +5861,10 @@
         <v>1690000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2317750</v>
+        <v>2317032</v>
       </c>
       <c r="L75" t="n">
-        <v>27.08445690863984</v>
+        <v>27.06186189918827</v>
       </c>
       <c r="M75" s="3" t="n">
         <v>0</v>
@@ -5925,10 +5925,10 @@
         <v>1705000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2317750</v>
+        <v>2317032</v>
       </c>
       <c r="L76" t="n">
-        <v>26.43727753208931</v>
+        <v>26.41448197521657</v>
       </c>
       <c r="M76" s="3" t="n">
         <v>0</v>
@@ -5989,10 +5989,10 @@
         <v>1725000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2360679</v>
+        <v>2359948</v>
       </c>
       <c r="L77" t="n">
-        <v>26.92780339893734</v>
+        <v>26.9051690969462</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
@@ -6053,10 +6053,10 @@
         <v>1780000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2446537</v>
+        <v>2445780</v>
       </c>
       <c r="L78" t="n">
-        <v>27.24410053884327</v>
+        <v>27.22158166310952</v>
       </c>
       <c r="M78" s="3" t="n">
         <v>0</v>
@@ -6068,7 +6068,7 @@
         <v>38.78143936249688</v>
       </c>
       <c r="Q78" t="n">
-        <v>21.2</v>
+        <v>21.1</v>
       </c>
       <c r="R78" t="n">
         <v>3</v>
@@ -6117,10 +6117,10 @@
         <v>1875000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2575325</v>
+        <v>2574528</v>
       </c>
       <c r="L79" t="n">
-        <v>27.19365516973586</v>
+        <v>27.17111641434857</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
@@ -6181,10 +6181,10 @@
         <v>1910000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2618254</v>
+        <v>2617443</v>
       </c>
       <c r="L80" t="n">
-        <v>27.05062228492728</v>
+        <v>27.02801933031588</v>
       </c>
       <c r="M80" s="3" t="n">
         <v>0</v>
@@ -6245,10 +6245,10 @@
         <v>2020000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2747042</v>
+        <v>2746191</v>
       </c>
       <c r="L81" t="n">
-        <v>26.46635908733831</v>
+        <v>26.44357220601189</v>
       </c>
       <c r="M81" s="3" t="n">
         <v>0</v>
@@ -6309,10 +6309,10 @@
         <v>2110000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>2875830</v>
+        <v>2874939</v>
       </c>
       <c r="L82" t="n">
-        <v>26.62987728760045</v>
+        <v>26.6071384471114</v>
       </c>
       <c r="M82" s="3" t="n">
         <v>0</v>
@@ -6373,10 +6373,10 @@
         <v>2210000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3004617</v>
+        <v>3003687</v>
       </c>
       <c r="L83" t="n">
-        <v>26.44653212040004</v>
+        <v>26.42375853409493</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
@@ -6437,10 +6437,10 @@
         <v>2215000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3047547</v>
+        <v>3046603</v>
       </c>
       <c r="L84" t="n">
-        <v>27.31859426614257</v>
+        <v>27.29607369256841</v>
       </c>
       <c r="M84" s="3" t="n">
         <v>0</v>
@@ -6501,10 +6501,10 @@
         <v>2315000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3176334</v>
+        <v>3175351</v>
       </c>
       <c r="L85" t="n">
-        <v>27.11723641153607</v>
+        <v>27.09467394313258</v>
       </c>
       <c r="M85" s="3" t="n">
         <v>0</v>
@@ -6565,10 +6565,10 @@
         <v>2395000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3305122</v>
+        <v>3304099</v>
       </c>
       <c r="L86" t="n">
-        <v>27.5367142271904</v>
+        <v>27.51427847652265</v>
       </c>
       <c r="M86" s="3" t="n">
         <v>0</v>
@@ -6629,10 +6629,10 @@
         <v>2410000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3305122</v>
+        <v>3304099</v>
       </c>
       <c r="L87" t="n">
-        <v>27.08287318894734</v>
+        <v>27.06029692209585</v>
       </c>
       <c r="M87" s="3" t="n">
         <v>0</v>
@@ -6693,10 +6693,10 @@
         <v>2499000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3433910</v>
+        <v>3432846</v>
       </c>
       <c r="L88" t="n">
-        <v>27.22581546982885</v>
+        <v>27.20325933642231</v>
       </c>
       <c r="M88" s="3" t="n">
         <v>0</v>
@@ -6757,10 +6757,10 @@
         <v>2510000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3433910</v>
+        <v>3432846</v>
       </c>
       <c r="L89" t="n">
-        <v>26.9054809240778</v>
+        <v>26.88282550396959</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
@@ -6821,10 +6821,10 @@
         <v>2530000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3476839</v>
+        <v>3475762</v>
       </c>
       <c r="L90" t="n">
-        <v>27.23275365928649</v>
+        <v>27.21020599223998</v>
       </c>
       <c r="M90" s="3" t="n">
         <v>0</v>
@@ -6885,10 +6885,10 @@
         <v>2610000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>3605627</v>
+        <v>3604510</v>
       </c>
       <c r="L91" t="n">
-        <v>27.6131446763628</v>
+        <v>27.59071274597657</v>
       </c>
       <c r="M91" s="3" t="n">
         <v>0</v>
@@ -6949,10 +6949,10 @@
         <v>3015000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4163707</v>
+        <v>4162418</v>
       </c>
       <c r="L92" t="n">
-        <v>27.5885647092843</v>
+        <v>27.56614064229013</v>
       </c>
       <c r="M92" s="3" t="n">
         <v>0</v>
@@ -7013,10 +7013,10 @@
         <v>3098000</v>
       </c>
       <c r="K93" s="3" t="n">
-        <v>4292495</v>
+        <v>4291165</v>
       </c>
       <c r="L93" t="n">
-        <v>27.82752222192454</v>
+        <v>27.80515314605707</v>
       </c>
       <c r="M93" s="3" t="n">
         <v>0</v>
@@ -7312,10 +7312,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>428863</v>
+        <v>428730</v>
       </c>
       <c r="L2" t="n">
-        <v>27.71607716217067</v>
+        <v>27.69365334826114</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7379,10 +7379,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>428863</v>
+        <v>428730</v>
       </c>
       <c r="L3" t="n">
-        <v>27.71607716217067</v>
+        <v>27.69365334826114</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7446,10 +7446,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>428863</v>
+        <v>428730</v>
       </c>
       <c r="L4" t="n">
-        <v>27.71584398747385</v>
+        <v>27.69342010122921</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7513,10 +7513,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>428863</v>
+        <v>428730</v>
       </c>
       <c r="L5" t="n">
-        <v>27.71584398747385</v>
+        <v>27.69342010122921</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7580,10 +7580,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514722</v>
+        <v>514562</v>
       </c>
       <c r="L6" t="n">
-        <v>25.39662186578386</v>
+        <v>25.37342438812038</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7644,10 +7644,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>514722</v>
+        <v>514562</v>
       </c>
       <c r="L7" t="n">
-        <v>25.39662186578386</v>
+        <v>25.37342438812038</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7708,10 +7708,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>514722</v>
+        <v>514562</v>
       </c>
       <c r="L8" t="n">
-        <v>25.39662186578386</v>
+        <v>25.37342438812038</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7772,10 +7772,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>514722</v>
+        <v>514562</v>
       </c>
       <c r="L9" t="n">
-        <v>25.39662186578386</v>
+        <v>25.37342438812038</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7836,10 +7836,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>514722</v>
+        <v>514562</v>
       </c>
       <c r="L10" t="n">
-        <v>25.20234223522601</v>
+        <v>25.17908434746445</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7900,10 +7900,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>514722</v>
+        <v>514562</v>
       </c>
       <c r="L11" t="n">
-        <v>25.20234223522601</v>
+        <v>25.17908434746445</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7964,10 +7964,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>514722</v>
+        <v>514562</v>
       </c>
       <c r="L12" t="n">
-        <v>25.20234223522601</v>
+        <v>25.17908434746445</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -8028,10 +8028,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>514722</v>
+        <v>514562</v>
       </c>
       <c r="L13" t="n">
-        <v>25.20234223522601</v>
+        <v>25.17908434746445</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -8092,16 +8092,16 @@
         <v>420000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>557651</v>
+        <v>557478</v>
       </c>
       <c r="L14" t="n">
-        <v>24.68407659988057</v>
+        <v>24.66070409953397</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>4.977160581811272</v>
+        <v>4.109370112717152</v>
       </c>
       <c r="O14" t="n">
         <v>100</v>
@@ -8110,7 +8110,7 @@
         <v>3.361344537815107</v>
       </c>
       <c r="Q14" t="n">
-        <v>32.4</v>
+        <v>32.1</v>
       </c>
       <c r="R14" t="n">
         <v>4</v>
@@ -8159,10 +8159,10 @@
         <v>420000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>557651</v>
+        <v>557478</v>
       </c>
       <c r="L15" t="n">
-        <v>24.68407659988057</v>
+        <v>24.66070409953397</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0</v>
@@ -8226,10 +8226,10 @@
         <v>420000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>557651</v>
+        <v>557478</v>
       </c>
       <c r="L16" t="n">
-        <v>24.68407659988057</v>
+        <v>24.66070409953397</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -8244,7 +8244,7 @@
         <v>3.361344537815107</v>
       </c>
       <c r="Q16" t="n">
-        <v>31.7</v>
+        <v>31.6</v>
       </c>
       <c r="R16" t="n">
         <v>4</v>
@@ -8293,16 +8293,16 @@
         <v>425000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>557651</v>
+        <v>557478</v>
       </c>
       <c r="L17" t="n">
-        <v>23.78745846416486</v>
+        <v>23.76380771976652</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>5.133716816332179</v>
+        <v>4.601464199174186</v>
       </c>
       <c r="O17" t="n">
         <v>0</v>
@@ -8311,7 +8311,7 @@
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>9.4</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="R17" t="n">
         <v>4</v>
@@ -8360,10 +8360,10 @@
         <v>454000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>600580</v>
+        <v>600394</v>
       </c>
       <c r="L18" t="n">
-        <v>24.40640713976489</v>
+        <v>24.38298850421557</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -8375,7 +8375,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q18" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="R18" t="n">
         <v>3</v>
@@ -8424,10 +8424,10 @@
         <v>454000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>600580</v>
+        <v>600394</v>
       </c>
       <c r="L19" t="n">
-        <v>24.40640713976489</v>
+        <v>24.38298850421557</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -8439,7 +8439,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q19" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="R19" t="n">
         <v>3</v>
@@ -8488,10 +8488,10 @@
         <v>454000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>600580</v>
+        <v>600394</v>
       </c>
       <c r="L20" t="n">
-        <v>24.40640713976489</v>
+        <v>24.38298850421557</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -8503,7 +8503,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q20" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="R20" t="n">
         <v>3</v>
@@ -8552,10 +8552,10 @@
         <v>454000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>600580</v>
+        <v>600394</v>
       </c>
       <c r="L21" t="n">
-        <v>24.40640713976489</v>
+        <v>24.38298850421557</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -8567,7 +8567,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q21" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="R21" t="n">
         <v>3</v>
@@ -8616,10 +8616,10 @@
         <v>455000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>600580</v>
+        <v>600394</v>
       </c>
       <c r="L22" t="n">
-        <v>24.239901428619</v>
+        <v>24.21643121017199</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -8680,10 +8680,10 @@
         <v>455000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>600580</v>
+        <v>600394</v>
       </c>
       <c r="L23" t="n">
-        <v>24.239901428619</v>
+        <v>24.21643121017199</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -8744,10 +8744,10 @@
         <v>455000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>600580</v>
+        <v>600394</v>
       </c>
       <c r="L24" t="n">
-        <v>24.239901428619</v>
+        <v>24.21643121017199</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -8808,10 +8808,10 @@
         <v>455000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>600580</v>
+        <v>600394</v>
       </c>
       <c r="L25" t="n">
-        <v>24.239901428619</v>
+        <v>24.21643121017199</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -8872,10 +8872,10 @@
         <v>475000</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>686439</v>
+        <v>686226</v>
       </c>
       <c r="L26" t="n">
-        <v>30.8022999858691</v>
+        <v>30.78082147863823</v>
       </c>
       <c r="M26" s="3" t="n">
         <v>0</v>
@@ -8936,10 +8936,10 @@
         <v>475000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>686439</v>
+        <v>686226</v>
       </c>
       <c r="L27" t="n">
-        <v>30.8022999858691</v>
+        <v>30.78082147863823</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -9000,10 +9000,10 @@
         <v>475000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>686439</v>
+        <v>686226</v>
       </c>
       <c r="L28" t="n">
-        <v>30.8022999858691</v>
+        <v>30.78082147863823</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -9064,10 +9064,10 @@
         <v>475000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>686439</v>
+        <v>686226</v>
       </c>
       <c r="L29" t="n">
-        <v>30.8022999858691</v>
+        <v>30.78082147863823</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -9093,11 +9093,11 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHF4 M5 10C CPU 10C GPU 16GB 1TB Midnight</t>
+          <t>Apple MacBook Air 15 MDVD4 M5 10C CPU 10C GPU 16GB 512GB Starlight</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -9108,7 +9108,7 @@
         <v>16</v>
       </c>
       <c r="E30" t="n">
-        <v>1024</v>
+        <v>512</v>
       </c>
       <c r="F30" t="n">
         <v>10</v>
@@ -9118,35 +9118,38 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Midnight</t>
+          <t>Starlight</t>
         </is>
       </c>
       <c r="I30" s="3" t="n">
-        <v>479999</v>
+        <v>477000</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>479999</v>
+        <v>477000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>686439</v>
+        <v>643310</v>
       </c>
       <c r="L30" t="n">
-        <v>30.07404882298354</v>
+        <v>25.85223298254341</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>0</v>
+        <v>-2999</v>
       </c>
       <c r="N30" t="n">
-        <v>0</v>
+        <v>1.242031557001153</v>
+      </c>
+      <c r="O30" t="n">
+        <v>100</v>
       </c>
       <c r="P30" t="n">
-        <v>43.6979831932773</v>
+        <v>1.568112774445864</v>
       </c>
       <c r="Q30" t="n">
-        <v>22.3</v>
+        <v>31.4</v>
       </c>
       <c r="R30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S30" t="inlineStr">
         <is>
@@ -9157,11 +9160,11 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHJ4 M5 10C CPU 10C GPU 16GB 1TB Sky Blue</t>
+          <t>Apple MacBook Air 15 MDVQ4 M5 10C CPU 10C GPU 16GB 512GB Sky Blue</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -9172,7 +9175,7 @@
         <v>16</v>
       </c>
       <c r="E31" t="n">
-        <v>1024</v>
+        <v>512</v>
       </c>
       <c r="F31" t="n">
         <v>10</v>
@@ -9186,31 +9189,34 @@
         </is>
       </c>
       <c r="I31" s="3" t="n">
-        <v>479999</v>
+        <v>477000</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>479999</v>
+        <v>477000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>686439</v>
+        <v>643310</v>
       </c>
       <c r="L31" t="n">
-        <v>30.07404882298354</v>
+        <v>25.85223298254341</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>0</v>
+        <v>-2999</v>
       </c>
       <c r="N31" t="n">
-        <v>0</v>
+        <v>1.242031557001153</v>
+      </c>
+      <c r="O31" t="n">
+        <v>100</v>
       </c>
       <c r="P31" t="n">
-        <v>43.6979831932773</v>
+        <v>1.568112774445864</v>
       </c>
       <c r="Q31" t="n">
-        <v>22.3</v>
+        <v>31.4</v>
       </c>
       <c r="R31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S31" t="inlineStr">
         <is>
@@ -9221,11 +9227,11 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDH84 M5 10C CPU 10C GPU 16GB 1TB Silver</t>
+          <t>Apple MacBook Air 15 MDVH4 M5 10C CPU 10C GPU 16GB 512GB Midnight</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -9236,7 +9242,7 @@
         <v>16</v>
       </c>
       <c r="E32" t="n">
-        <v>1024</v>
+        <v>512</v>
       </c>
       <c r="F32" t="n">
         <v>10</v>
@@ -9246,35 +9252,38 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Midnight</t>
         </is>
       </c>
       <c r="I32" s="3" t="n">
-        <v>479999</v>
+        <v>477000</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>479999</v>
+        <v>477000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>686439</v>
+        <v>643310</v>
       </c>
       <c r="L32" t="n">
-        <v>30.07404882298354</v>
+        <v>25.85223298254341</v>
       </c>
       <c r="M32" s="3" t="n">
-        <v>0</v>
+        <v>-2999</v>
       </c>
       <c r="N32" t="n">
-        <v>0</v>
+        <v>1.242031557001153</v>
+      </c>
+      <c r="O32" t="n">
+        <v>100</v>
       </c>
       <c r="P32" t="n">
-        <v>43.6979831932773</v>
+        <v>1.568112774445864</v>
       </c>
       <c r="Q32" t="n">
-        <v>22.3</v>
+        <v>31.4</v>
       </c>
       <c r="R32" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S32" t="inlineStr">
         <is>
@@ -9285,7 +9294,7 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHC4 M5 10C CPU 10C GPU 16GB 1TB Starlight</t>
+          <t>Apple MacBook Air 13 MDHF4 M5 10C CPU 10C GPU 16GB 1TB Midnight</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -9310,7 +9319,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Starlight</t>
+          <t>Midnight</t>
         </is>
       </c>
       <c r="I33" s="3" t="n">
@@ -9320,10 +9329,10 @@
         <v>479999</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>686439</v>
+        <v>686226</v>
       </c>
       <c r="L33" t="n">
-        <v>30.07404882298354</v>
+        <v>30.05234427142078</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -9335,7 +9344,7 @@
         <v>43.6979831932773</v>
       </c>
       <c r="Q33" t="n">
-        <v>22.3</v>
+        <v>22.2</v>
       </c>
       <c r="R33" t="n">
         <v>3</v>
@@ -9349,11 +9358,11 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MDVD4 M5 10C CPU 10C GPU 16GB 512GB Starlight</t>
+          <t>Apple MacBook Air 13 MDHJ4 M5 10C CPU 10C GPU 16GB 1TB Sky Blue</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -9364,7 +9373,7 @@
         <v>16</v>
       </c>
       <c r="E34" t="n">
-        <v>512</v>
+        <v>1024</v>
       </c>
       <c r="F34" t="n">
         <v>10</v>
@@ -9374,7 +9383,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Starlight</t>
+          <t>Sky Blue</t>
         </is>
       </c>
       <c r="I34" s="3" t="n">
@@ -9384,28 +9393,25 @@
         <v>479999</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>643509</v>
+        <v>686226</v>
       </c>
       <c r="L34" t="n">
-        <v>25.40912403711526</v>
+        <v>30.05234427142078</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N34" t="n">
-        <v>0.6211192983836406</v>
-      </c>
-      <c r="O34" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="P34" t="n">
-        <v>2.54778368297421</v>
+        <v>43.6979831932773</v>
       </c>
       <c r="Q34" t="n">
-        <v>31.3</v>
+        <v>22.2</v>
       </c>
       <c r="R34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S34" t="inlineStr">
         <is>
@@ -9416,11 +9422,11 @@
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MDVQ4 M5 10C CPU 10C GPU 16GB 512GB Sky Blue</t>
+          <t>Apple MacBook Air 13 MDH84 M5 10C CPU 10C GPU 16GB 1TB Silver</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -9431,7 +9437,7 @@
         <v>16</v>
       </c>
       <c r="E35" t="n">
-        <v>512</v>
+        <v>1024</v>
       </c>
       <c r="F35" t="n">
         <v>10</v>
@@ -9441,7 +9447,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Sky Blue</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I35" s="3" t="n">
@@ -9451,28 +9457,25 @@
         <v>479999</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>643509</v>
+        <v>686226</v>
       </c>
       <c r="L35" t="n">
-        <v>25.40912403711526</v>
+        <v>30.05234427142078</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N35" t="n">
-        <v>0.6211192983836406</v>
-      </c>
-      <c r="O35" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="P35" t="n">
-        <v>2.54778368297421</v>
+        <v>43.6979831932773</v>
       </c>
       <c r="Q35" t="n">
-        <v>31.3</v>
+        <v>22.2</v>
       </c>
       <c r="R35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S35" t="inlineStr">
         <is>
@@ -9483,11 +9486,11 @@
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MDVH4 M5 10C CPU 10C GPU 16GB 512GB Midnight</t>
+          <t>Apple MacBook Air 13 MDHC4 M5 10C CPU 10C GPU 16GB 1TB Starlight</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -9498,7 +9501,7 @@
         <v>16</v>
       </c>
       <c r="E36" t="n">
-        <v>512</v>
+        <v>1024</v>
       </c>
       <c r="F36" t="n">
         <v>10</v>
@@ -9508,7 +9511,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Midnight</t>
+          <t>Starlight</t>
         </is>
       </c>
       <c r="I36" s="3" t="n">
@@ -9518,28 +9521,25 @@
         <v>479999</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>643509</v>
+        <v>686226</v>
       </c>
       <c r="L36" t="n">
-        <v>25.40912403711526</v>
+        <v>30.05234427142078</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N36" t="n">
-        <v>0.6211192983836406</v>
-      </c>
-      <c r="O36" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="P36" t="n">
-        <v>2.54778368297421</v>
+        <v>43.6979831932773</v>
       </c>
       <c r="Q36" t="n">
-        <v>31.3</v>
+        <v>22.2</v>
       </c>
       <c r="R36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S36" t="inlineStr">
         <is>
@@ -9579,22 +9579,22 @@
         </is>
       </c>
       <c r="I37" s="3" t="n">
-        <v>484999</v>
+        <v>479999</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>484999</v>
+        <v>479999</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>643509</v>
+        <v>643310</v>
       </c>
       <c r="L37" t="n">
-        <v>24.63213412710623</v>
+        <v>25.38605027125336</v>
       </c>
       <c r="M37" s="3" t="n">
-        <v>0</v>
+        <v>-5000</v>
       </c>
       <c r="N37" t="n">
-        <v>2.020404040404041</v>
+        <v>2.538175165660067</v>
       </c>
       <c r="O37" t="n">
         <v>0</v>
@@ -9603,7 +9603,7 @@
         <v>0</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.800000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="R37" t="n">
         <v>4</v>
@@ -9652,10 +9652,10 @@
         <v>500000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>643509</v>
+        <v>643310</v>
       </c>
       <c r="L38" t="n">
-        <v>22.30100899909714</v>
+        <v>22.27697377625095</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -9716,10 +9716,10 @@
         <v>547999</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>772297</v>
+        <v>772058</v>
       </c>
       <c r="L39" t="n">
-        <v>29.04297181006789</v>
+        <v>29.02100619383518</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -9780,10 +9780,10 @@
         <v>547999</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>772297</v>
+        <v>772058</v>
       </c>
       <c r="L40" t="n">
-        <v>29.04297181006789</v>
+        <v>29.02100619383518</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -9844,10 +9844,10 @@
         <v>547999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>772297</v>
+        <v>772058</v>
       </c>
       <c r="L41" t="n">
-        <v>29.04297181006789</v>
+        <v>29.02100619383518</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
@@ -9908,10 +9908,10 @@
         <v>547999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>772297</v>
+        <v>772058</v>
       </c>
       <c r="L42" t="n">
-        <v>29.04297181006789</v>
+        <v>29.02100619383518</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -9972,10 +9972,10 @@
         <v>552999</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>772297</v>
+        <v>772058</v>
       </c>
       <c r="L43" t="n">
-        <v>28.39555248822668</v>
+        <v>28.37338645542174</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -9984,10 +9984,10 @@
         <v>2.123897564420468</v>
       </c>
       <c r="P43" t="n">
-        <v>35.7962333566031</v>
+        <v>34.11769473304435</v>
       </c>
       <c r="Q43" t="n">
-        <v>20.6</v>
+        <v>20.2</v>
       </c>
       <c r="R43" t="n">
         <v>3</v>
@@ -10036,10 +10036,10 @@
         <v>552999</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>772297</v>
+        <v>772058</v>
       </c>
       <c r="L44" t="n">
-        <v>28.39555248822668</v>
+        <v>28.37338645542174</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -10048,10 +10048,10 @@
         <v>2.123897564420468</v>
       </c>
       <c r="P44" t="n">
-        <v>35.7962333566031</v>
+        <v>34.11769473304435</v>
       </c>
       <c r="Q44" t="n">
-        <v>20.6</v>
+        <v>20.2</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -10100,10 +10100,10 @@
         <v>552999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>772297</v>
+        <v>772058</v>
       </c>
       <c r="L45" t="n">
-        <v>28.39555248822668</v>
+        <v>28.37338645542174</v>
       </c>
       <c r="M45" s="3" t="n">
         <v>0</v>
@@ -10112,10 +10112,10 @@
         <v>2.123897564420468</v>
       </c>
       <c r="P45" t="n">
-        <v>35.7962333566031</v>
+        <v>34.11769473304435</v>
       </c>
       <c r="Q45" t="n">
-        <v>20.6</v>
+        <v>20.2</v>
       </c>
       <c r="R45" t="n">
         <v>3</v>
@@ -10164,10 +10164,10 @@
         <v>552999</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>772297</v>
+        <v>772058</v>
       </c>
       <c r="L46" t="n">
-        <v>28.39555248822668</v>
+        <v>28.37338645542174</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -10176,10 +10176,10 @@
         <v>2.123897564420468</v>
       </c>
       <c r="P46" t="n">
-        <v>35.7962333566031</v>
+        <v>34.11769473304435</v>
       </c>
       <c r="Q46" t="n">
-        <v>20.6</v>
+        <v>20.2</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -10228,10 +10228,10 @@
         <v>585000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>729368</v>
+        <v>729142</v>
       </c>
       <c r="L47" t="n">
-        <v>19.79357471125687</v>
+        <v>19.76871446165493</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -10240,10 +10240,10 @@
         <v>0</v>
       </c>
       <c r="P47" t="n">
-        <v>23.56648951077459</v>
+        <v>21.56821735015607</v>
       </c>
       <c r="Q47" t="n">
-        <v>13.5</v>
+        <v>13.1</v>
       </c>
       <c r="R47" t="n">
         <v>3</v>
@@ -10292,10 +10292,10 @@
         <v>595000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>729368</v>
+        <v>729142</v>
       </c>
       <c r="L48" t="n">
-        <v>18.42252470632109</v>
+        <v>18.3972394951875</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -10356,22 +10356,22 @@
         <v>614999</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>858155</v>
+        <v>857890</v>
       </c>
       <c r="L49" t="n">
-        <v>28.33474139287192</v>
+        <v>28.31260418002308</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N49" t="n">
-        <v>0.3241496339540259</v>
+        <v>0.1623379258732563</v>
       </c>
       <c r="P49" t="n">
-        <v>59.10837762230636</v>
+        <v>58.0393100094641</v>
       </c>
       <c r="Q49" t="n">
-        <v>24.9</v>
+        <v>24.6</v>
       </c>
       <c r="R49" t="n">
         <v>3</v>
@@ -10420,22 +10420,22 @@
         <v>614999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>858155</v>
+        <v>857890</v>
       </c>
       <c r="L50" t="n">
-        <v>28.33474139287192</v>
+        <v>28.31260418002308</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N50" t="n">
-        <v>0.3241496339540259</v>
+        <v>0.1623379258732563</v>
       </c>
       <c r="P50" t="n">
-        <v>59.10837762230636</v>
+        <v>58.0393100094641</v>
       </c>
       <c r="Q50" t="n">
-        <v>24.9</v>
+        <v>24.6</v>
       </c>
       <c r="R50" t="n">
         <v>3</v>
@@ -10484,22 +10484,22 @@
         <v>614999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>858155</v>
+        <v>857890</v>
       </c>
       <c r="L51" t="n">
-        <v>28.33474139287192</v>
+        <v>28.31260418002308</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N51" t="n">
-        <v>0.3241496339540259</v>
+        <v>0.1623379258732563</v>
       </c>
       <c r="P51" t="n">
-        <v>59.10837762230636</v>
+        <v>58.0393100094641</v>
       </c>
       <c r="Q51" t="n">
-        <v>24.9</v>
+        <v>24.6</v>
       </c>
       <c r="R51" t="n">
         <v>3</v>
@@ -10548,10 +10548,10 @@
         <v>614999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>858155</v>
+        <v>857890</v>
       </c>
       <c r="L52" t="n">
-        <v>28.33474139287192</v>
+        <v>28.31260418002308</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -10560,10 +10560,10 @@
         <v>0</v>
       </c>
       <c r="P52" t="n">
-        <v>59.10837762230636</v>
+        <v>58.0393100094641</v>
       </c>
       <c r="Q52" t="n">
-        <v>24.8</v>
+        <v>24.6</v>
       </c>
       <c r="R52" t="n">
         <v>3</v>
@@ -10612,10 +10612,10 @@
         <v>650000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>815226</v>
+        <v>814974</v>
       </c>
       <c r="L53" t="n">
-        <v>20.26750864177541</v>
+        <v>20.24285437326835</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -10624,10 +10624,10 @@
         <v>0</v>
       </c>
       <c r="P53" t="n">
-        <v>48.40738041977285</v>
+        <v>47.05854671135535</v>
       </c>
       <c r="Q53" t="n">
-        <v>19.1</v>
+        <v>18.8</v>
       </c>
       <c r="R53" t="n">
         <v>3</v>
@@ -10676,10 +10676,10 @@
         <v>672000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>858155</v>
+        <v>857890</v>
       </c>
       <c r="L54" t="n">
-        <v>21.69246814386678</v>
+        <v>21.66827915000758</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -10740,10 +10740,10 @@
         <v>700000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>901085</v>
+        <v>900806</v>
       </c>
       <c r="L55" t="n">
-        <v>22.31587475099463</v>
+        <v>22.29181421970991</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -10804,10 +10804,10 @@
         <v>715000</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>944014</v>
+        <v>943722</v>
       </c>
       <c r="L56" t="n">
-        <v>24.25959784494722</v>
+        <v>24.23616276827286</v>
       </c>
       <c r="M56" s="3" t="n">
         <v>0</v>
@@ -10816,10 +10816,10 @@
         <v>0</v>
       </c>
       <c r="P56" t="n">
-        <v>64.96797435910501</v>
+        <v>64.05209961882153</v>
       </c>
       <c r="Q56" t="n">
-        <v>24.3</v>
+        <v>24.1</v>
       </c>
       <c r="R56" t="n">
         <v>3</v>
@@ -10868,10 +10868,10 @@
         <v>734999</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>986943</v>
+        <v>986638</v>
       </c>
       <c r="L57" t="n">
-        <v>25.52771537971291</v>
+        <v>25.5046937174526</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -10932,10 +10932,10 @@
         <v>752000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>986943</v>
+        <v>986638</v>
       </c>
       <c r="L58" t="n">
-        <v>23.80512349750695</v>
+        <v>23.78156932937917</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -10944,10 +10944,10 @@
         <v>0</v>
       </c>
       <c r="P58" t="n">
-        <v>55.54117473210056</v>
+        <v>54.37884642534079</v>
       </c>
       <c r="Q58" t="n">
-        <v>22.1</v>
+        <v>21.8</v>
       </c>
       <c r="R58" t="n">
         <v>3</v>
@@ -10996,10 +10996,10 @@
         <v>810000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1072802</v>
+        <v>1072469</v>
       </c>
       <c r="L59" t="n">
-        <v>24.49678505446485</v>
+        <v>24.47334142059118</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -11008,10 +11008,10 @@
         <v>0</v>
       </c>
       <c r="P59" t="n">
-        <v>70.24552627383726</v>
+        <v>69.46762746845361</v>
       </c>
       <c r="Q59" t="n">
-        <v>25.6</v>
+        <v>25.4</v>
       </c>
       <c r="R59" t="n">
         <v>3</v>
@@ -11060,10 +11060,10 @@
         <v>815000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1072802</v>
+        <v>1072469</v>
       </c>
       <c r="L60" t="n">
-        <v>24.03071582640599</v>
+        <v>24.00712747874298</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -11124,10 +11124,10 @@
         <v>875000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1158660</v>
+        <v>1158301</v>
       </c>
       <c r="L61" t="n">
-        <v>24.48172889372206</v>
+        <v>24.45832300930415</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -11136,10 +11136,10 @@
         <v>0</v>
       </c>
       <c r="P61" t="n">
-        <v>79.93620349657833</v>
+        <v>79.41165705441597</v>
       </c>
       <c r="Q61" t="n">
-        <v>27.6</v>
+        <v>27.5</v>
       </c>
       <c r="R61" t="n">
         <v>3</v>
@@ -11188,10 +11188,10 @@
         <v>992000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1330377</v>
+        <v>1329965</v>
       </c>
       <c r="L62" t="n">
-        <v>25.43467002210652</v>
+        <v>25.41157098119123</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -11203,7 +11203,7 @@
         <v>85.64705882352939</v>
       </c>
       <c r="Q62" t="n">
-        <v>29.3</v>
+        <v>29.2</v>
       </c>
       <c r="R62" t="n">
         <v>3</v>
@@ -11252,10 +11252,10 @@
         <v>1050000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1416236</v>
+        <v>1415797</v>
       </c>
       <c r="L63" t="n">
-        <v>25.85981432473119</v>
+        <v>25.83682547709876</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -11267,7 +11267,7 @@
         <v>93.20091673032849</v>
       </c>
       <c r="Q63" t="n">
-        <v>31.1</v>
+        <v>31</v>
       </c>
       <c r="R63" t="n">
         <v>3</v>
@@ -11316,10 +11316,10 @@
         <v>1050000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1416236</v>
+        <v>1415797</v>
       </c>
       <c r="L64" t="n">
-        <v>25.85981432473119</v>
+        <v>25.83682547709876</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -11328,7 +11328,7 @@
         <v>0</v>
       </c>
       <c r="P64" t="n">
-        <v>86.62413566438555</v>
+        <v>86.27443803627732</v>
       </c>
       <c r="Q64" t="n">
         <v>29.6</v>
@@ -11380,10 +11380,10 @@
         <v>1100000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1502094</v>
+        <v>1501629</v>
       </c>
       <c r="L65" t="n">
-        <v>26.76889728605533</v>
+        <v>26.74622027145187</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -11392,10 +11392,10 @@
         <v>0</v>
       </c>
       <c r="P65" t="n">
-        <v>94.26748671330809</v>
+        <v>94.11761630126171</v>
       </c>
       <c r="Q65" t="n">
-        <v>31.7</v>
+        <v>31.6</v>
       </c>
       <c r="R65" t="n">
         <v>3</v>
@@ -11444,10 +11444,10 @@
         <v>1105000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1502094</v>
+        <v>1501629</v>
       </c>
       <c r="L66" t="n">
-        <v>26.43602863735558</v>
+        <v>26.41324854541302</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -11459,7 +11459,7 @@
         <v>100</v>
       </c>
       <c r="Q66" t="n">
-        <v>32.8</v>
+        <v>32.7</v>
       </c>
       <c r="R66" t="n">
         <v>3</v>
@@ -11508,10 +11508,10 @@
         <v>1155000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1587953</v>
+        <v>1587461</v>
       </c>
       <c r="L67" t="n">
-        <v>27.26484977829948</v>
+        <v>27.24230705510245</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -11778,7 +11778,7 @@
         <v>315000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>300075</v>
+        <v>299982</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -11839,10 +11839,10 @@
         <v>380000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>385934</v>
+        <v>385814</v>
       </c>
       <c r="L3" t="n">
-        <v>1.537568599812403</v>
+        <v>1.506943760464887</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -11903,7 +11903,7 @@
         <v>415000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>385934</v>
+        <v>385814</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -11964,10 +11964,10 @@
         <v>495000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>471792</v>
+        <v>471646</v>
       </c>
       <c r="L5" t="n">
-        <v>6.738774714280869</v>
+        <v>6.709905310338686</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -12022,19 +12022,19 @@
         </is>
       </c>
       <c r="I6" s="3" t="n">
-        <v>470000</v>
+        <v>490000</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>500000</v>
+        <v>490000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514722</v>
+        <v>514562</v>
       </c>
       <c r="L6" t="n">
-        <v>8.688573637808371</v>
+        <v>4.773380078591113</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
@@ -12043,10 +12043,10 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -12092,10 +12092,10 @@
         <v>550000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>557651</v>
+        <v>557478</v>
       </c>
       <c r="L7" t="n">
-        <v>6.751713885566421</v>
+        <v>6.722776504184918</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -12156,7 +12156,7 @@
         <v>530000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>471792</v>
+        <v>471646</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -12220,10 +12220,10 @@
         <v>600000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>600580</v>
+        <v>600394</v>
       </c>
       <c r="L9" t="n">
-        <v>8.421858869759232</v>
+        <v>8.393488276032073</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -12232,10 +12232,10 @@
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>20.65076182537716</v>
+        <v>30.25295873936471</v>
       </c>
       <c r="Q9" t="n">
-        <v>8.1</v>
+        <v>9.9</v>
       </c>
       <c r="R9" t="n">
         <v>4</v>
@@ -12284,10 +12284,10 @@
         <v>646000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>729368</v>
+        <v>729142</v>
       </c>
       <c r="L10" t="n">
-        <v>17.0516118063858</v>
+        <v>17.02590167621671</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -12348,7 +12348,7 @@
         <v>615000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>557651</v>
+        <v>557478</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -12412,7 +12412,7 @@
         <v>700000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>643509</v>
+        <v>643310</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -12476,7 +12476,7 @@
         <v>745000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>686439</v>
+        <v>686226</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -12488,10 +12488,10 @@
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>32.45119715416413</v>
+        <v>40.62540173571834</v>
       </c>
       <c r="Q13" t="n">
-        <v>6.2</v>
+        <v>7.7</v>
       </c>
       <c r="R13" t="n">
         <v>4</v>
@@ -12540,7 +12540,7 @@
         <v>930000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>858155</v>
+        <v>857890</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -12611,7 +12611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12657,8 +12657,160 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 15 MDV94 M5 10C CPU 10C GPU 16GB 512GB Silver</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>484999</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>479999</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>-5000</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-1.03</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Macbook Pro 14 M5 MDE14 10 Core CPU 10 Core GPU 16GB 1TB Space Black</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>582999</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>579999</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>-3000</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-0.51</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 15 MDVD4 M5 10C CPU 10C GPU 16GB 512GB Starlight</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>479999</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>477000</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>-2999</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-0.62</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 15 MDVQ4 M5 10C CPU 10C GPU 16GB 512GB Sky Blue</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>479999</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>477000</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>-2999</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-0.62</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 15 MDVH4 M5 10C CPU 10C GPU 16GB 512GB Midnight</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>479999</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>477000</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>-2999</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-0.62</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Apple iphone 17 Pro Max 256GB</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>470000</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>490000</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>20000</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.26</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F1"/>
+  <autoFilter ref="A1:F7"/>
+  <conditionalFormatting sqref="E2:E7">
+    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: price data 2026-10-01
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MacBook Pro'!$A$1:$S$93</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MacBook Air'!$A$1:$S$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20260930T094648863561+0000</t>
+          <t>20261001T101332922774+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-30T09:46:48.863561+00:00</t>
+          <t>2026-10-01T10:13:32.922774+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>276.877066</v>
+        <v>276.984011</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -855,7 +855,7 @@
         <v>720000</v>
       </c>
       <c r="D28" t="n">
-        <v>44.3</v>
+        <v>44.2</v>
       </c>
       <c r="E28" t="n">
         <v>3</v>
@@ -897,7 +897,7 @@
         <v>725000</v>
       </c>
       <c r="D30" t="n">
-        <v>42.9</v>
+        <v>42.8</v>
       </c>
       <c r="E30" t="n">
         <v>3</v>
@@ -1147,10 +1147,10 @@
         <v>470000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>686226</v>
+        <v>686491</v>
       </c>
       <c r="L2" t="n">
-        <v>35.15255906946108</v>
+        <v>35.17759154890596</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1162,10 +1162,10 @@
         <v>100</v>
       </c>
       <c r="P2" t="n">
-        <v>9.365994236311199</v>
+        <v>28.4414106939704</v>
       </c>
       <c r="Q2" t="n">
-        <v>32.5</v>
+        <v>35.4</v>
       </c>
       <c r="R2" t="n">
         <v>5</v>
@@ -1208,19 +1208,19 @@
         </is>
       </c>
       <c r="I3" s="3" t="n">
-        <v>458000</v>
+        <v>495000</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>465000</v>
+        <v>495000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>686226</v>
+        <v>686491</v>
       </c>
       <c r="L3" t="n">
-        <v>33.25813944677118</v>
+        <v>27.89417486900775</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>0</v>
+        <v>37000</v>
       </c>
       <c r="N3" t="n">
         <v>0</v>
@@ -1232,10 +1232,10 @@
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>10.1</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="R3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>772058</v>
+        <v>772356</v>
       </c>
       <c r="L4" t="n">
-        <v>35.23815568260416</v>
+        <v>35.26314290301364</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1296,10 +1296,10 @@
         <v>100</v>
       </c>
       <c r="P4" t="n">
-        <v>59.79881123919307</v>
+        <v>68.25981228668942</v>
       </c>
       <c r="Q4" t="n">
-        <v>40.5</v>
+        <v>41.7</v>
       </c>
       <c r="R4" t="n">
         <v>5</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>772058</v>
+        <v>772356</v>
       </c>
       <c r="L5" t="n">
-        <v>32.64767672895042</v>
+        <v>32.67366344017525</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1363,10 +1363,10 @@
         <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>48.9918948126801</v>
+        <v>59.72738907849829</v>
       </c>
       <c r="Q5" t="n">
-        <v>17.7</v>
+        <v>19.3</v>
       </c>
       <c r="R5" t="n">
         <v>5</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>857890</v>
+        <v>858221</v>
       </c>
       <c r="L6" t="n">
-        <v>37.98738766042267</v>
+        <v>38.0113047804703</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1606,10 +1606,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>857890</v>
+        <v>858221</v>
       </c>
       <c r="L9" t="n">
-        <v>34.14074065439625</v>
+        <v>34.16614135519872</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1621,10 +1621,10 @@
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>85.73487031700287</v>
+        <v>88.73720136518772</v>
       </c>
       <c r="Q9" t="n">
-        <v>25.7</v>
+        <v>26.2</v>
       </c>
       <c r="R9" t="n">
         <v>4</v>
@@ -1673,13 +1673,13 @@
         <v>579999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>857890</v>
+        <v>858221</v>
       </c>
       <c r="L10" t="n">
-        <v>32.39238130762685</v>
+        <v>32.41845631836089</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>-3000</v>
+        <v>0</v>
       </c>
       <c r="N10" t="n">
         <v>0.5145806425053902</v>
@@ -1740,10 +1740,10 @@
         <v>587999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>857890</v>
+        <v>858221</v>
       </c>
       <c r="L11" t="n">
-        <v>31.45986082131742</v>
+        <v>31.48629548799202</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -1807,10 +1807,10 @@
         <v>600000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>857890</v>
+        <v>858221</v>
       </c>
       <c r="L12" t="n">
-        <v>30.06096352679248</v>
+        <v>30.08793772233492</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -1874,10 +1874,10 @@
         <v>634000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>857890</v>
+        <v>858221</v>
       </c>
       <c r="L13" t="n">
-        <v>26.09775145997738</v>
+        <v>26.12625419326723</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -1941,10 +1941,10 @@
         <v>643999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>943722</v>
+        <v>944086</v>
       </c>
       <c r="L14" t="n">
-        <v>31.75967075049644</v>
+        <v>31.78598136186746</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -2067,10 +2067,10 @@
         <v>650000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>943722</v>
+        <v>944086</v>
       </c>
       <c r="L16" t="n">
-        <v>31.12378433479351</v>
+        <v>31.15034011731982</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -2134,10 +2134,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1029554</v>
+        <v>1029951</v>
       </c>
       <c r="L17" t="n">
-        <v>32.00939435911084</v>
+        <v>32.0356016936728</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2201,10 +2201,10 @@
         <v>711999</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>1072469</v>
+        <v>1072884</v>
       </c>
       <c r="L18" t="n">
-        <v>33.61122792360432</v>
+        <v>33.63690762468264</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -2272,7 +2272,7 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>0.8946324119975306</v>
+        <v>0.6895181924388861</v>
       </c>
       <c r="O19" t="n">
         <v>100</v>
@@ -2281,7 +2281,7 @@
         <v>42.39316239316239</v>
       </c>
       <c r="Q19" t="n">
-        <v>44.3</v>
+        <v>44.2</v>
       </c>
       <c r="R19" t="n">
         <v>3</v>
@@ -2330,10 +2330,10 @@
         <v>720000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>1029554</v>
+        <v>1029951</v>
       </c>
       <c r="L20" t="n">
-        <v>30.066805626514</v>
+        <v>30.09376174206346</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -2401,7 +2401,7 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>1.023823224452713</v>
+        <v>0.684795458623916</v>
       </c>
       <c r="O21" t="n">
         <v>96.7741935483871</v>
@@ -2410,7 +2410,7 @@
         <v>41.02564102564102</v>
       </c>
       <c r="Q21" t="n">
-        <v>42.9</v>
+        <v>42.8</v>
       </c>
       <c r="R21" t="n">
         <v>3</v>
@@ -2459,10 +2459,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1072469</v>
+        <v>1072884</v>
       </c>
       <c r="L22" t="n">
-        <v>30.72060824135709</v>
+        <v>30.74740605694558</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2526,10 +2526,10 @@
         <v>772000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1029554</v>
+        <v>1029951</v>
       </c>
       <c r="L23" t="n">
-        <v>25.01607492176224</v>
+        <v>25.04497786787915</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -2593,10 +2593,10 @@
         <v>775000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1029554</v>
+        <v>1029951</v>
       </c>
       <c r="L24" t="n">
-        <v>24.72468661187272</v>
+        <v>24.75370187513775</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -2611,7 +2611,7 @@
         <v>68.99999999999999</v>
       </c>
       <c r="Q24" t="n">
-        <v>19.7</v>
+        <v>19.8</v>
       </c>
       <c r="R24" t="n">
         <v>4</v>
@@ -2660,10 +2660,10 @@
         <v>775000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>1029554</v>
+        <v>1029951</v>
       </c>
       <c r="L25" t="n">
-        <v>24.72468661187272</v>
+        <v>24.75370187513775</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -2678,7 +2678,7 @@
         <v>68.99999999999999</v>
       </c>
       <c r="Q25" t="n">
-        <v>19.7</v>
+        <v>19.8</v>
       </c>
       <c r="R25" t="n">
         <v>4</v>
@@ -2789,10 +2789,10 @@
         <v>810000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>1072469</v>
+        <v>1072884</v>
       </c>
       <c r="L27" t="n">
-        <v>24.47334142059118</v>
+        <v>24.50255572829868</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -2804,7 +2804,7 @@
         <v>61.99999999999999</v>
       </c>
       <c r="Q27" t="n">
-        <v>24.8</v>
+        <v>24.9</v>
       </c>
       <c r="R27" t="n">
         <v>3</v>
@@ -2853,10 +2853,10 @@
         <v>810000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>1244133</v>
+        <v>1244614</v>
       </c>
       <c r="L28" t="n">
-        <v>34.89442045183272</v>
+        <v>34.9195814927359</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -2982,16 +2982,16 @@
         <v>825000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1287049</v>
+        <v>1287546</v>
       </c>
       <c r="L30" t="n">
-        <v>35.89987638388282</v>
+        <v>35.92461939223919</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N30" t="n">
-        <v>0.7816004589301971</v>
+        <v>0.6022898822769667</v>
       </c>
       <c r="O30" t="n">
         <v>100</v>
@@ -3049,16 +3049,16 @@
         <v>829999</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1287049</v>
+        <v>1287546</v>
       </c>
       <c r="L31" t="n">
-        <v>35.51146848332892</v>
+        <v>35.53636141932016</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N31" t="n">
-        <v>2.924093567251462</v>
+        <v>1.190595238095238</v>
       </c>
       <c r="O31" t="n">
         <v>0</v>
@@ -3067,7 +3067,7 @@
         <v>0</v>
       </c>
       <c r="Q31" t="n">
-        <v>12.6</v>
+        <v>12.2</v>
       </c>
       <c r="R31" t="n">
         <v>4</v>
@@ -3116,10 +3116,10 @@
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1372881</v>
+        <v>1373411</v>
       </c>
       <c r="L32" t="n">
-        <v>38.23215559105269</v>
+        <v>38.25599183347155</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3183,10 +3183,10 @@
         <v>930000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1372881</v>
+        <v>1373411</v>
       </c>
       <c r="L33" t="n">
-        <v>38.08647654093836</v>
+        <v>38.11036900097641</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3250,10 +3250,10 @@
         <v>860000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>1244133</v>
+        <v>1244614</v>
       </c>
       <c r="L34" t="n">
-        <v>30.87555751676067</v>
+        <v>30.90227170833688</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -3503,10 +3503,10 @@
         <v>880000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>1158301</v>
+        <v>1158749</v>
       </c>
       <c r="L38" t="n">
-        <v>24.02665628364302</v>
+        <v>24.05602939031663</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -3567,10 +3567,10 @@
         <v>940000</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>1244133</v>
+        <v>1244614</v>
       </c>
       <c r="L39" t="n">
-        <v>24.44537682064538</v>
+        <v>24.47457605329845</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -3631,10 +3631,10 @@
         <v>990000</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>1501629</v>
+        <v>1502209</v>
       </c>
       <c r="L40" t="n">
-        <v>34.07159824430668</v>
+        <v>34.09705307317424</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -3695,10 +3695,10 @@
         <v>990000</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>1501629</v>
+        <v>1502209</v>
       </c>
       <c r="L41" t="n">
-        <v>34.07159824430668</v>
+        <v>34.09705307317424</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
@@ -3821,10 +3821,10 @@
         <v>1055000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1544545</v>
+        <v>1545141</v>
       </c>
       <c r="L43" t="n">
-        <v>31.69509467189366</v>
+        <v>31.72144160306405</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -3885,22 +3885,22 @@
         <v>1055000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1544545</v>
+        <v>1545141</v>
       </c>
       <c r="L44" t="n">
-        <v>31.69509467189366</v>
+        <v>31.72144160306405</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>2.54041570438799</v>
+        <v>2.314814814814815</v>
       </c>
       <c r="P44" t="n">
         <v>58.64647440248988</v>
       </c>
       <c r="Q44" t="n">
-        <v>27.1</v>
+        <v>27</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -4011,10 +4011,10 @@
         <v>1115000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1501629</v>
+        <v>1502209</v>
       </c>
       <c r="L46" t="n">
-        <v>25.7473050933353</v>
+        <v>25.77597391574674</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -4075,10 +4075,10 @@
         <v>1123000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1716209</v>
+        <v>1716872</v>
       </c>
       <c r="L47" t="n">
-        <v>34.56507919489992</v>
+        <v>34.59034802827468</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -4142,10 +4142,10 @@
         <v>1130000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1501629</v>
+        <v>1502209</v>
       </c>
       <c r="L48" t="n">
-        <v>24.74838991521874</v>
+        <v>24.77744441685544</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -4268,10 +4268,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1759125</v>
+        <v>1759804</v>
       </c>
       <c r="L50" t="n">
-        <v>34.342357706246</v>
+        <v>34.36769094740096</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4283,7 +4283,7 @@
         <v>22.53136001640632</v>
       </c>
       <c r="Q50" t="n">
-        <v>19.5</v>
+        <v>19.6</v>
       </c>
       <c r="R50" t="n">
         <v>3</v>
@@ -4332,10 +4332,10 @@
         <v>1155000</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>1759125</v>
+        <v>1759804</v>
       </c>
       <c r="L51" t="n">
-        <v>34.342357706246</v>
+        <v>34.36769094740096</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -4347,7 +4347,7 @@
         <v>22.53136001640632</v>
       </c>
       <c r="Q51" t="n">
-        <v>19.5</v>
+        <v>19.6</v>
       </c>
       <c r="R51" t="n">
         <v>3</v>
@@ -4396,10 +4396,10 @@
         <v>1185000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1587461</v>
+        <v>1588074</v>
       </c>
       <c r="L52" t="n">
-        <v>25.35249684874148</v>
+        <v>25.38131094646723</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -4460,10 +4460,10 @@
         <v>1185000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1587461</v>
+        <v>1588074</v>
       </c>
       <c r="L53" t="n">
-        <v>25.35249684874148</v>
+        <v>25.38131094646723</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -4524,10 +4524,10 @@
         <v>1200000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1887872</v>
+        <v>1888602</v>
       </c>
       <c r="L54" t="n">
-        <v>36.4363685673605</v>
+        <v>36.46093777301941</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -4588,10 +4588,10 @@
         <v>1200000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1887872</v>
+        <v>1888602</v>
       </c>
       <c r="L55" t="n">
-        <v>36.4363685673605</v>
+        <v>36.46093777301941</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -4714,10 +4714,10 @@
         <v>1240000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1673293</v>
+        <v>1673939</v>
       </c>
       <c r="L57" t="n">
-        <v>25.89462813745112</v>
+        <v>25.92322659308374</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -4729,7 +4729,7 @@
         <v>100</v>
       </c>
       <c r="Q57" t="n">
-        <v>33.6</v>
+        <v>33.7</v>
       </c>
       <c r="R57" t="n">
         <v>3</v>
@@ -4840,10 +4840,10 @@
         <v>1280000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1716209</v>
+        <v>1716872</v>
       </c>
       <c r="L59" t="n">
-        <v>25.41700923372386</v>
+        <v>25.44581075350987</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -4907,10 +4907,10 @@
         <v>1298000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1759125</v>
+        <v>1759804</v>
       </c>
       <c r="L60" t="n">
-        <v>26.21331627940027</v>
+        <v>26.24178601707918</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -4971,10 +4971,10 @@
         <v>1300000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1716209</v>
+        <v>1716872</v>
       </c>
       <c r="L61" t="n">
-        <v>24.2516500030008</v>
+        <v>24.28090154653346</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -5097,10 +5097,10 @@
         <v>1335000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1802041</v>
+        <v>1802737</v>
       </c>
       <c r="L63" t="n">
-        <v>25.91733484421276</v>
+        <v>25.94593665077047</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -5161,10 +5161,10 @@
         <v>1420000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1930788</v>
+        <v>1931534</v>
       </c>
       <c r="L64" t="n">
-        <v>26.45489820736404</v>
+        <v>26.4833029084655</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -5225,10 +5225,10 @@
         <v>1430000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1930788</v>
+        <v>1931534</v>
       </c>
       <c r="L65" t="n">
-        <v>25.93697495530322</v>
+        <v>25.96557968951103</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -5289,10 +5289,10 @@
         <v>1430000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>2145368</v>
+        <v>2146197</v>
       </c>
       <c r="L66" t="n">
-        <v>33.34476882287794</v>
+        <v>33.37051538139323</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -5353,10 +5353,10 @@
         <v>1430000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>2145368</v>
+        <v>2146197</v>
       </c>
       <c r="L67" t="n">
-        <v>33.34476882287794</v>
+        <v>33.37051538139323</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -5479,10 +5479,10 @@
         <v>1480000</v>
       </c>
       <c r="K69" s="3" t="n">
-        <v>2016620</v>
+        <v>2017399</v>
       </c>
       <c r="L69" t="n">
-        <v>26.60987196397933</v>
+        <v>26.63821088441107</v>
       </c>
       <c r="M69" s="3" t="n">
         <v>0</v>
@@ -5605,10 +5605,10 @@
         <v>1605000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2188284</v>
+        <v>2189129</v>
       </c>
       <c r="L71" t="n">
-        <v>26.65485832734691</v>
+        <v>26.68316942491739</v>
       </c>
       <c r="M71" s="3" t="n">
         <v>0</v>
@@ -5669,10 +5669,10 @@
         <v>1610000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2188284</v>
+        <v>2189129</v>
       </c>
       <c r="L72" t="n">
-        <v>26.42636878942587</v>
+        <v>26.454768083562</v>
       </c>
       <c r="M72" s="3" t="n">
         <v>0</v>
@@ -5733,10 +5733,10 @@
         <v>1615000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2188284</v>
+        <v>2189129</v>
       </c>
       <c r="L73" t="n">
-        <v>26.19787925150483</v>
+        <v>26.2263667422066</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
@@ -5797,10 +5797,10 @@
         <v>1630000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2231200</v>
+        <v>2232062</v>
       </c>
       <c r="L74" t="n">
-        <v>26.94514162782359</v>
+        <v>26.97335468280003</v>
       </c>
       <c r="M74" s="3" t="n">
         <v>0</v>
@@ -5812,7 +5812,7 @@
         <v>100</v>
       </c>
       <c r="Q74" t="n">
-        <v>34</v>
+        <v>34.1</v>
       </c>
       <c r="R74" t="n">
         <v>3</v>
@@ -5861,10 +5861,10 @@
         <v>1690000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2317032</v>
+        <v>2317927</v>
       </c>
       <c r="L75" t="n">
-        <v>27.06186189918827</v>
+        <v>27.09002483684775</v>
       </c>
       <c r="M75" s="3" t="n">
         <v>0</v>
@@ -5925,10 +5925,10 @@
         <v>1705000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2317032</v>
+        <v>2317927</v>
       </c>
       <c r="L76" t="n">
-        <v>26.41448197521657</v>
+        <v>26.44289487977836</v>
       </c>
       <c r="M76" s="3" t="n">
         <v>0</v>
@@ -5989,10 +5989,10 @@
         <v>1725000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2359948</v>
+        <v>2360859</v>
       </c>
       <c r="L77" t="n">
-        <v>26.9051690969462</v>
+        <v>26.93337467421816</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
@@ -6053,10 +6053,10 @@
         <v>1780000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2445780</v>
+        <v>2446724</v>
       </c>
       <c r="L78" t="n">
-        <v>27.22158166310952</v>
+        <v>27.24966117960179</v>
       </c>
       <c r="M78" s="3" t="n">
         <v>0</v>
@@ -6068,7 +6068,7 @@
         <v>38.78143936249688</v>
       </c>
       <c r="Q78" t="n">
-        <v>21.1</v>
+        <v>21.2</v>
       </c>
       <c r="R78" t="n">
         <v>3</v>
@@ -6117,10 +6117,10 @@
         <v>1875000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2574528</v>
+        <v>2575522</v>
       </c>
       <c r="L79" t="n">
-        <v>27.17111641434857</v>
+        <v>27.19922407962347</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
@@ -6132,7 +6132,7 @@
         <v>19.64044075004835</v>
       </c>
       <c r="Q79" t="n">
-        <v>17.1</v>
+        <v>17.2</v>
       </c>
       <c r="R79" t="n">
         <v>3</v>
@@ -6181,10 +6181,10 @@
         <v>1910000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2617443</v>
+        <v>2618454</v>
       </c>
       <c r="L80" t="n">
-        <v>27.02801933031588</v>
+        <v>27.0561942275862</v>
       </c>
       <c r="M80" s="3" t="n">
         <v>0</v>
@@ -6245,10 +6245,10 @@
         <v>2020000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2746191</v>
+        <v>2747252</v>
       </c>
       <c r="L81" t="n">
-        <v>26.44357220601189</v>
+        <v>26.47198000037856</v>
       </c>
       <c r="M81" s="3" t="n">
         <v>0</v>
@@ -6309,10 +6309,10 @@
         <v>2110000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>2874939</v>
+        <v>2876050</v>
       </c>
       <c r="L82" t="n">
-        <v>26.6071384471114</v>
+        <v>26.63548964725926</v>
       </c>
       <c r="M82" s="3" t="n">
         <v>0</v>
@@ -6373,10 +6373,10 @@
         <v>2210000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3003687</v>
+        <v>3004847</v>
       </c>
       <c r="L83" t="n">
-        <v>26.42375853409493</v>
+        <v>26.45216212339597</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
@@ -6437,10 +6437,10 @@
         <v>2215000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3046603</v>
+        <v>3047780</v>
       </c>
       <c r="L84" t="n">
-        <v>27.29607369256841</v>
+        <v>27.32415069329151</v>
       </c>
       <c r="M84" s="3" t="n">
         <v>0</v>
@@ -6501,10 +6501,10 @@
         <v>2315000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3175351</v>
+        <v>3176577</v>
       </c>
       <c r="L85" t="n">
-        <v>27.09467394313258</v>
+        <v>27.12281175617654</v>
       </c>
       <c r="M85" s="3" t="n">
         <v>0</v>
@@ -6565,10 +6565,10 @@
         <v>2395000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3304099</v>
+        <v>3305375</v>
       </c>
       <c r="L86" t="n">
-        <v>27.51427847652265</v>
+        <v>27.54226071171955</v>
       </c>
       <c r="M86" s="3" t="n">
         <v>0</v>
@@ -6629,10 +6629,10 @@
         <v>2410000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3304099</v>
+        <v>3305375</v>
       </c>
       <c r="L87" t="n">
-        <v>27.06029692209585</v>
+        <v>27.08845441137541</v>
       </c>
       <c r="M87" s="3" t="n">
         <v>0</v>
@@ -6693,10 +6693,10 @@
         <v>2499000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3432846</v>
+        <v>3434172</v>
       </c>
       <c r="L88" t="n">
-        <v>27.20325933642231</v>
+        <v>27.23136756108896</v>
       </c>
       <c r="M88" s="3" t="n">
         <v>0</v>
@@ -6757,10 +6757,10 @@
         <v>2510000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3432846</v>
+        <v>3434172</v>
       </c>
       <c r="L89" t="n">
-        <v>26.88282550396959</v>
+        <v>26.91105745431504</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
@@ -6821,10 +6821,10 @@
         <v>2530000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3475762</v>
+        <v>3477105</v>
       </c>
       <c r="L90" t="n">
-        <v>27.21020599223998</v>
+        <v>27.23832038434272</v>
       </c>
       <c r="M90" s="3" t="n">
         <v>0</v>
@@ -6885,10 +6885,10 @@
         <v>2610000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>3604510</v>
+        <v>3605902</v>
       </c>
       <c r="L91" t="n">
-        <v>27.59071274597657</v>
+        <v>27.61866517725662</v>
       </c>
       <c r="M91" s="3" t="n">
         <v>0</v>
@@ -6900,7 +6900,7 @@
         <v>74.15426251691474</v>
       </c>
       <c r="Q91" t="n">
-        <v>28.4</v>
+        <v>28.5</v>
       </c>
       <c r="R91" t="n">
         <v>3</v>
@@ -6949,10 +6949,10 @@
         <v>3015000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4162418</v>
+        <v>4164025</v>
       </c>
       <c r="L92" t="n">
-        <v>27.56614064229013</v>
+        <v>27.59409465601192</v>
       </c>
       <c r="M92" s="3" t="n">
         <v>0</v>
@@ -7013,10 +7013,10 @@
         <v>3098000</v>
       </c>
       <c r="K93" s="3" t="n">
-        <v>4291165</v>
+        <v>4292823</v>
       </c>
       <c r="L93" t="n">
-        <v>27.80515314605707</v>
+        <v>27.83303667539985</v>
       </c>
       <c r="M93" s="3" t="n">
         <v>0</v>
@@ -7312,10 +7312,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>428730</v>
+        <v>428896</v>
       </c>
       <c r="L2" t="n">
-        <v>27.69365334826114</v>
+        <v>27.72163881220622</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7379,10 +7379,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>428730</v>
+        <v>428896</v>
       </c>
       <c r="L3" t="n">
-        <v>27.69365334826114</v>
+        <v>27.72163881220622</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7446,10 +7446,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>428730</v>
+        <v>428896</v>
       </c>
       <c r="L4" t="n">
-        <v>27.69342010122921</v>
+        <v>27.72140565545027</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7513,10 +7513,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>428730</v>
+        <v>428896</v>
       </c>
       <c r="L5" t="n">
-        <v>27.69342010122921</v>
+        <v>27.72140565545027</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7580,10 +7580,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514562</v>
+        <v>514761</v>
       </c>
       <c r="L6" t="n">
-        <v>25.37342438812038</v>
+        <v>25.40227406505155</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7644,10 +7644,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>514562</v>
+        <v>514761</v>
       </c>
       <c r="L7" t="n">
-        <v>25.37342438812038</v>
+        <v>25.40227406505155</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7708,10 +7708,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>514562</v>
+        <v>514761</v>
       </c>
       <c r="L8" t="n">
-        <v>25.37342438812038</v>
+        <v>25.40227406505155</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7772,10 +7772,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>514562</v>
+        <v>514761</v>
       </c>
       <c r="L9" t="n">
-        <v>25.37342438812038</v>
+        <v>25.40227406505155</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7836,10 +7836,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>514562</v>
+        <v>514761</v>
       </c>
       <c r="L10" t="n">
-        <v>25.17908434746445</v>
+        <v>25.20800915376262</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7900,10 +7900,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>514562</v>
+        <v>514761</v>
       </c>
       <c r="L11" t="n">
-        <v>25.17908434746445</v>
+        <v>25.20800915376262</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7964,10 +7964,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>514562</v>
+        <v>514761</v>
       </c>
       <c r="L12" t="n">
-        <v>25.17908434746445</v>
+        <v>25.20800915376262</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -8028,10 +8028,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>514562</v>
+        <v>514761</v>
       </c>
       <c r="L13" t="n">
-        <v>25.17908434746445</v>
+        <v>25.20800915376262</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -8092,16 +8092,16 @@
         <v>420000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>557478</v>
+        <v>557693</v>
       </c>
       <c r="L14" t="n">
-        <v>24.66070409953397</v>
+        <v>24.68974866100166</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>4.109370112717152</v>
+        <v>3.225583469086334</v>
       </c>
       <c r="O14" t="n">
         <v>100</v>
@@ -8110,7 +8110,7 @@
         <v>3.361344537815107</v>
       </c>
       <c r="Q14" t="n">
-        <v>32.1</v>
+        <v>31.9</v>
       </c>
       <c r="R14" t="n">
         <v>4</v>
@@ -8159,10 +8159,10 @@
         <v>420000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>557478</v>
+        <v>557693</v>
       </c>
       <c r="L15" t="n">
-        <v>24.66070409953397</v>
+        <v>24.68974866100166</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0</v>
@@ -8226,10 +8226,10 @@
         <v>420000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>557478</v>
+        <v>557693</v>
       </c>
       <c r="L16" t="n">
-        <v>24.66070409953397</v>
+        <v>24.68974866100166</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -8244,7 +8244,7 @@
         <v>3.361344537815107</v>
       </c>
       <c r="Q16" t="n">
-        <v>31.6</v>
+        <v>31.7</v>
       </c>
       <c r="R16" t="n">
         <v>4</v>
@@ -8293,16 +8293,16 @@
         <v>425000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>557478</v>
+        <v>557693</v>
       </c>
       <c r="L17" t="n">
-        <v>23.76380771976652</v>
+        <v>23.79319804982311</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>4.601464199174186</v>
+        <v>4.063205417607223</v>
       </c>
       <c r="O17" t="n">
         <v>0</v>
@@ -8311,7 +8311,7 @@
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>9.199999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="R17" t="n">
         <v>4</v>
@@ -8360,10 +8360,10 @@
         <v>454000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>600394</v>
+        <v>600626</v>
       </c>
       <c r="L18" t="n">
-        <v>24.38298850421557</v>
+        <v>24.41219660820544</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -8375,7 +8375,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q18" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="R18" t="n">
         <v>3</v>
@@ -8424,10 +8424,10 @@
         <v>454000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>600394</v>
+        <v>600626</v>
       </c>
       <c r="L19" t="n">
-        <v>24.38298850421557</v>
+        <v>24.41219660820544</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -8439,7 +8439,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q19" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="R19" t="n">
         <v>3</v>
@@ -8488,10 +8488,10 @@
         <v>454000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>600394</v>
+        <v>600626</v>
       </c>
       <c r="L20" t="n">
-        <v>24.38298850421557</v>
+        <v>24.41219660820544</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -8503,7 +8503,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q20" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="R20" t="n">
         <v>3</v>
@@ -8552,10 +8552,10 @@
         <v>454000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>600394</v>
+        <v>600626</v>
       </c>
       <c r="L21" t="n">
-        <v>24.38298850421557</v>
+        <v>24.41219660820544</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -8567,7 +8567,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q21" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="R21" t="n">
         <v>3</v>
@@ -8616,10 +8616,10 @@
         <v>455000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>600394</v>
+        <v>600626</v>
       </c>
       <c r="L22" t="n">
-        <v>24.21643121017199</v>
+        <v>24.24570364919268</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -8680,10 +8680,10 @@
         <v>455000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>600394</v>
+        <v>600626</v>
       </c>
       <c r="L23" t="n">
-        <v>24.21643121017199</v>
+        <v>24.24570364919268</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -8744,10 +8744,10 @@
         <v>455000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>600394</v>
+        <v>600626</v>
       </c>
       <c r="L24" t="n">
-        <v>24.21643121017199</v>
+        <v>24.24570364919268</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -8808,10 +8808,10 @@
         <v>455000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>600394</v>
+        <v>600626</v>
       </c>
       <c r="L25" t="n">
-        <v>24.21643121017199</v>
+        <v>24.24570364919268</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -8872,10 +8872,10 @@
         <v>475000</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>686226</v>
+        <v>686491</v>
       </c>
       <c r="L26" t="n">
-        <v>30.78082147863823</v>
+        <v>30.80754154096703</v>
       </c>
       <c r="M26" s="3" t="n">
         <v>0</v>
@@ -8936,10 +8936,10 @@
         <v>475000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>686226</v>
+        <v>686491</v>
       </c>
       <c r="L27" t="n">
-        <v>30.78082147863823</v>
+        <v>30.80754154096703</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -9000,10 +9000,10 @@
         <v>475000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>686226</v>
+        <v>686491</v>
       </c>
       <c r="L28" t="n">
-        <v>30.78082147863823</v>
+        <v>30.80754154096703</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -9064,10 +9064,10 @@
         <v>475000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>686226</v>
+        <v>686491</v>
       </c>
       <c r="L29" t="n">
-        <v>30.78082147863823</v>
+        <v>30.80754154096703</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -9128,13 +9128,13 @@
         <v>477000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>643310</v>
+        <v>643559</v>
       </c>
       <c r="L30" t="n">
-        <v>25.85223298254341</v>
+        <v>25.88092156274716</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>-2999</v>
+        <v>0</v>
       </c>
       <c r="N30" t="n">
         <v>1.242031557001153</v>
@@ -9146,7 +9146,7 @@
         <v>1.568112774445864</v>
       </c>
       <c r="Q30" t="n">
-        <v>31.4</v>
+        <v>31.5</v>
       </c>
       <c r="R30" t="n">
         <v>4</v>
@@ -9195,13 +9195,13 @@
         <v>477000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>643310</v>
+        <v>643559</v>
       </c>
       <c r="L31" t="n">
-        <v>25.85223298254341</v>
+        <v>25.88092156274716</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>-2999</v>
+        <v>0</v>
       </c>
       <c r="N31" t="n">
         <v>1.242031557001153</v>
@@ -9213,7 +9213,7 @@
         <v>1.568112774445864</v>
       </c>
       <c r="Q31" t="n">
-        <v>31.4</v>
+        <v>31.5</v>
       </c>
       <c r="R31" t="n">
         <v>4</v>
@@ -9262,13 +9262,13 @@
         <v>477000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>643310</v>
+        <v>643559</v>
       </c>
       <c r="L32" t="n">
-        <v>25.85223298254341</v>
+        <v>25.88092156274716</v>
       </c>
       <c r="M32" s="3" t="n">
-        <v>-2999</v>
+        <v>0</v>
       </c>
       <c r="N32" t="n">
         <v>1.242031557001153</v>
@@ -9280,7 +9280,7 @@
         <v>1.568112774445864</v>
       </c>
       <c r="Q32" t="n">
-        <v>31.4</v>
+        <v>31.5</v>
       </c>
       <c r="R32" t="n">
         <v>4</v>
@@ -9329,10 +9329,10 @@
         <v>479999</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>686226</v>
+        <v>686491</v>
       </c>
       <c r="L33" t="n">
-        <v>30.05234427142078</v>
+        <v>30.07934554131081</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -9344,7 +9344,7 @@
         <v>43.6979831932773</v>
       </c>
       <c r="Q33" t="n">
-        <v>22.2</v>
+        <v>22.3</v>
       </c>
       <c r="R33" t="n">
         <v>3</v>
@@ -9393,10 +9393,10 @@
         <v>479999</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>686226</v>
+        <v>686491</v>
       </c>
       <c r="L34" t="n">
-        <v>30.05234427142078</v>
+        <v>30.07934554131081</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -9408,7 +9408,7 @@
         <v>43.6979831932773</v>
       </c>
       <c r="Q34" t="n">
-        <v>22.2</v>
+        <v>22.3</v>
       </c>
       <c r="R34" t="n">
         <v>3</v>
@@ -9457,10 +9457,10 @@
         <v>479999</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>686226</v>
+        <v>686491</v>
       </c>
       <c r="L35" t="n">
-        <v>30.05234427142078</v>
+        <v>30.07934554131081</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
@@ -9472,7 +9472,7 @@
         <v>43.6979831932773</v>
       </c>
       <c r="Q35" t="n">
-        <v>22.2</v>
+        <v>22.3</v>
       </c>
       <c r="R35" t="n">
         <v>3</v>
@@ -9521,10 +9521,10 @@
         <v>479999</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>686226</v>
+        <v>686491</v>
       </c>
       <c r="L36" t="n">
-        <v>30.05234427142078</v>
+        <v>30.07934554131081</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -9536,7 +9536,7 @@
         <v>43.6979831932773</v>
       </c>
       <c r="Q36" t="n">
-        <v>22.2</v>
+        <v>22.3</v>
       </c>
       <c r="R36" t="n">
         <v>3</v>
@@ -9585,16 +9585,16 @@
         <v>479999</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>643310</v>
+        <v>643559</v>
       </c>
       <c r="L37" t="n">
-        <v>25.38605027125336</v>
+        <v>25.41491922263537</v>
       </c>
       <c r="M37" s="3" t="n">
-        <v>-5000</v>
+        <v>0</v>
       </c>
       <c r="N37" t="n">
-        <v>2.538175165660067</v>
+        <v>2.040820491470391</v>
       </c>
       <c r="O37" t="n">
         <v>0</v>
@@ -9603,7 +9603,7 @@
         <v>0</v>
       </c>
       <c r="Q37" t="n">
-        <v>9.199999999999999</v>
+        <v>9</v>
       </c>
       <c r="R37" t="n">
         <v>4</v>
@@ -9652,10 +9652,10 @@
         <v>500000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>643310</v>
+        <v>643559</v>
       </c>
       <c r="L38" t="n">
-        <v>22.27697377625095</v>
+        <v>22.30704566325698</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -9716,10 +9716,10 @@
         <v>547999</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>772058</v>
+        <v>772356</v>
       </c>
       <c r="L39" t="n">
-        <v>29.02100619383518</v>
+        <v>29.04839219220152</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -9780,10 +9780,10 @@
         <v>547999</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>772058</v>
+        <v>772356</v>
       </c>
       <c r="L40" t="n">
-        <v>29.02100619383518</v>
+        <v>29.04839219220152</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -9844,10 +9844,10 @@
         <v>547999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>772058</v>
+        <v>772356</v>
       </c>
       <c r="L41" t="n">
-        <v>29.02100619383518</v>
+        <v>29.04839219220152</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
@@ -9908,10 +9908,10 @@
         <v>547999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>772058</v>
+        <v>772356</v>
       </c>
       <c r="L42" t="n">
-        <v>29.02100619383518</v>
+        <v>29.04839219220152</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -9972,10 +9972,10 @@
         <v>552999</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>772058</v>
+        <v>772356</v>
       </c>
       <c r="L43" t="n">
-        <v>28.37338645542174</v>
+        <v>28.40102232649193</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -10036,10 +10036,10 @@
         <v>552999</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>772058</v>
+        <v>772356</v>
       </c>
       <c r="L44" t="n">
-        <v>28.37338645542174</v>
+        <v>28.40102232649193</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -10100,10 +10100,10 @@
         <v>552999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>772058</v>
+        <v>772356</v>
       </c>
       <c r="L45" t="n">
-        <v>28.37338645542174</v>
+        <v>28.40102232649193</v>
       </c>
       <c r="M45" s="3" t="n">
         <v>0</v>
@@ -10164,10 +10164,10 @@
         <v>552999</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>772058</v>
+        <v>772356</v>
       </c>
       <c r="L46" t="n">
-        <v>28.37338645542174</v>
+        <v>28.40102232649193</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -10228,10 +10228,10 @@
         <v>585000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>729142</v>
+        <v>729424</v>
       </c>
       <c r="L47" t="n">
-        <v>19.76871446165493</v>
+        <v>19.79973239158569</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -10292,10 +10292,10 @@
         <v>595000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>729142</v>
+        <v>729424</v>
       </c>
       <c r="L48" t="n">
-        <v>18.3972394951875</v>
+        <v>18.42878764614271</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -10356,16 +10356,16 @@
         <v>614999</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>857890</v>
+        <v>858221</v>
       </c>
       <c r="L49" t="n">
-        <v>28.31260418002308</v>
+        <v>28.34025268549709</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N49" t="n">
-        <v>0.1623379258732563</v>
+        <v>0</v>
       </c>
       <c r="P49" t="n">
         <v>58.0393100094641</v>
@@ -10420,16 +10420,16 @@
         <v>614999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>857890</v>
+        <v>858221</v>
       </c>
       <c r="L50" t="n">
-        <v>28.31260418002308</v>
+        <v>28.34025268549709</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N50" t="n">
-        <v>0.1623379258732563</v>
+        <v>0</v>
       </c>
       <c r="P50" t="n">
         <v>58.0393100094641</v>
@@ -10484,16 +10484,16 @@
         <v>614999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>857890</v>
+        <v>858221</v>
       </c>
       <c r="L51" t="n">
-        <v>28.31260418002308</v>
+        <v>28.34025268549709</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N51" t="n">
-        <v>0.1623379258732563</v>
+        <v>0</v>
       </c>
       <c r="P51" t="n">
         <v>58.0393100094641</v>
@@ -10548,10 +10548,10 @@
         <v>614999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>857890</v>
+        <v>858221</v>
       </c>
       <c r="L52" t="n">
-        <v>28.31260418002308</v>
+        <v>28.34025268549709</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -10612,10 +10612,10 @@
         <v>650000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>814974</v>
+        <v>815289</v>
       </c>
       <c r="L53" t="n">
-        <v>20.24285437326835</v>
+        <v>20.27366982750902</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -10676,10 +10676,10 @@
         <v>672000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>857890</v>
+        <v>858221</v>
       </c>
       <c r="L54" t="n">
-        <v>21.66827915000758</v>
+        <v>21.69849024901512</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -10740,10 +10740,10 @@
         <v>700000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>900806</v>
+        <v>901154</v>
       </c>
       <c r="L55" t="n">
-        <v>22.29181421970991</v>
+        <v>22.32182290707249</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -10804,10 +10804,10 @@
         <v>715000</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>943722</v>
+        <v>944086</v>
       </c>
       <c r="L56" t="n">
-        <v>24.23616276827286</v>
+        <v>24.2653741290518</v>
       </c>
       <c r="M56" s="3" t="n">
         <v>0</v>
@@ -10868,10 +10868,10 @@
         <v>734999</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>986638</v>
+        <v>987019</v>
       </c>
       <c r="L57" t="n">
-        <v>25.5046937174526</v>
+        <v>25.53344971069453</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -10932,10 +10932,10 @@
         <v>752000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>986638</v>
+        <v>987019</v>
       </c>
       <c r="L58" t="n">
-        <v>23.78156932937917</v>
+        <v>23.81099046725544</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -10947,7 +10947,7 @@
         <v>54.37884642534079</v>
       </c>
       <c r="Q58" t="n">
-        <v>21.8</v>
+        <v>21.9</v>
       </c>
       <c r="R58" t="n">
         <v>3</v>
@@ -10996,10 +10996,10 @@
         <v>810000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1072469</v>
+        <v>1072884</v>
       </c>
       <c r="L59" t="n">
-        <v>24.47334142059118</v>
+        <v>24.50255572829868</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -11060,10 +11060,10 @@
         <v>815000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1072469</v>
+        <v>1072884</v>
       </c>
       <c r="L60" t="n">
-        <v>24.00712747874298</v>
+        <v>24.03652212168324</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -11124,10 +11124,10 @@
         <v>875000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1158301</v>
+        <v>1158749</v>
       </c>
       <c r="L61" t="n">
-        <v>24.45832300930415</v>
+        <v>24.48752922332619</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -11188,10 +11188,10 @@
         <v>992000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1329965</v>
+        <v>1330479</v>
       </c>
       <c r="L62" t="n">
-        <v>25.41157098119123</v>
+        <v>25.44038650741575</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -11203,7 +11203,7 @@
         <v>85.64705882352939</v>
       </c>
       <c r="Q62" t="n">
-        <v>29.2</v>
+        <v>29.3</v>
       </c>
       <c r="R62" t="n">
         <v>3</v>
@@ -11252,10 +11252,10 @@
         <v>1050000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1415797</v>
+        <v>1416344</v>
       </c>
       <c r="L63" t="n">
-        <v>25.83682547709876</v>
+        <v>25.86546771123399</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -11267,7 +11267,7 @@
         <v>93.20091673032849</v>
       </c>
       <c r="Q63" t="n">
-        <v>31</v>
+        <v>31.1</v>
       </c>
       <c r="R63" t="n">
         <v>3</v>
@@ -11316,10 +11316,10 @@
         <v>1050000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1415797</v>
+        <v>1416344</v>
       </c>
       <c r="L64" t="n">
-        <v>25.83682547709876</v>
+        <v>25.86546771123399</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -11380,10 +11380,10 @@
         <v>1100000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1501629</v>
+        <v>1502209</v>
       </c>
       <c r="L65" t="n">
-        <v>26.74622027145187</v>
+        <v>26.77450341463804</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -11444,10 +11444,10 @@
         <v>1105000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1501629</v>
+        <v>1502209</v>
       </c>
       <c r="L66" t="n">
-        <v>26.41324854541302</v>
+        <v>26.44166024834094</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -11459,7 +11459,7 @@
         <v>100</v>
       </c>
       <c r="Q66" t="n">
-        <v>32.7</v>
+        <v>32.8</v>
       </c>
       <c r="R66" t="n">
         <v>3</v>
@@ -11508,10 +11508,10 @@
         <v>1155000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1587461</v>
+        <v>1588074</v>
       </c>
       <c r="L67" t="n">
-        <v>27.24230705510245</v>
+        <v>27.2703916819997</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -11778,7 +11778,7 @@
         <v>315000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>299982</v>
+        <v>300098</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -11839,10 +11839,10 @@
         <v>380000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>385814</v>
+        <v>385963</v>
       </c>
       <c r="L3" t="n">
-        <v>1.506943760464887</v>
+        <v>1.544966745517057</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -11903,7 +11903,7 @@
         <v>415000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>385814</v>
+        <v>385963</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -11964,10 +11964,10 @@
         <v>495000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>471646</v>
+        <v>471828</v>
       </c>
       <c r="L5" t="n">
-        <v>6.709905310338686</v>
+        <v>6.745890451605247</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -12028,13 +12028,13 @@
         <v>490000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514562</v>
+        <v>514761</v>
       </c>
       <c r="L6" t="n">
-        <v>4.773380078591113</v>
+        <v>4.810193468425153</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
@@ -12043,7 +12043,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="R6" t="n">
         <v>3</v>
@@ -12092,10 +12092,10 @@
         <v>550000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>557478</v>
+        <v>557693</v>
       </c>
       <c r="L7" t="n">
-        <v>6.722776504184918</v>
+        <v>6.758736437430629</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -12156,7 +12156,7 @@
         <v>530000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>471646</v>
+        <v>471828</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -12220,10 +12220,10 @@
         <v>600000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>600394</v>
+        <v>600626</v>
       </c>
       <c r="L9" t="n">
-        <v>8.393488276032073</v>
+        <v>8.428872542980157</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -12284,10 +12284,10 @@
         <v>646000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>729142</v>
+        <v>729424</v>
       </c>
       <c r="L10" t="n">
-        <v>17.02590167621671</v>
+        <v>17.05797999517427</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -12348,7 +12348,7 @@
         <v>615000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>557478</v>
+        <v>557693</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -12412,7 +12412,7 @@
         <v>700000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>643310</v>
+        <v>643559</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -12476,7 +12476,7 @@
         <v>745000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>686226</v>
+        <v>686491</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -12540,7 +12540,7 @@
         <v>930000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>857890</v>
+        <v>858221</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -12611,7 +12611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12660,150 +12660,30 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MDV94 M5 10C CPU 10C GPU 16GB 512GB Silver</t>
+          <t>Apple MacBook Pro 14Inch MW2U3 M4 10Core CPU 10Core GPU 16GB 512GB Space Black</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>484999</v>
+        <v>458000</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>479999</v>
+        <v>495000</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-5000</v>
+        <v>37000</v>
       </c>
       <c r="F2" t="n">
-        <v>-1.03</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 M5 MDE14 10 Core CPU 10 Core GPU 16GB 1TB Space Black</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>582999</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>579999</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>-3000</v>
-      </c>
-      <c r="F3" t="n">
-        <v>-0.51</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDVD4 M5 10C CPU 10C GPU 16GB 512GB Starlight</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>479999</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>477000</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>-2999</v>
-      </c>
-      <c r="F4" t="n">
-        <v>-0.62</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDVQ4 M5 10C CPU 10C GPU 16GB 512GB Sky Blue</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>479999</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>477000</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>-2999</v>
-      </c>
-      <c r="F5" t="n">
-        <v>-0.62</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDVH4 M5 10C CPU 10C GPU 16GB 512GB Midnight</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>479999</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>477000</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>-2999</v>
-      </c>
-      <c r="F6" t="n">
-        <v>-0.62</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Apple iphone 17 Pro Max 256GB</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>470000</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>490000</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F7" t="n">
-        <v>4.26</v>
+        <v>8.08</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F7"/>
-  <conditionalFormatting sqref="E2:E7">
+  <autoFilter ref="A1:F2"/>
+  <conditionalFormatting sqref="E2">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
chore: price data 2026-10-02
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MacBook Pro'!$A$1:$S$93</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MacBook Air'!$A$1:$S$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20261001T101332922774+0000</t>
+          <t>20261002T095103629503+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-01T10:13:32.922774+00:00</t>
+          <t>2026-10-02T09:51:03.629503+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>276.984011</v>
+        <v>277.099958</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -1147,10 +1147,10 @@
         <v>470000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>686491</v>
+        <v>686778</v>
       </c>
       <c r="L2" t="n">
-        <v>35.17759154890596</v>
+        <v>35.20468040618657</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1214,13 +1214,13 @@
         <v>495000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>686491</v>
+        <v>686778</v>
       </c>
       <c r="L3" t="n">
-        <v>27.89417486900775</v>
+        <v>27.92430741811764</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>37000</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
         <v>0</v>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>772356</v>
+        <v>772679</v>
       </c>
       <c r="L4" t="n">
-        <v>35.26314290301364</v>
+        <v>35.29020459984029</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>772356</v>
+        <v>772679</v>
       </c>
       <c r="L5" t="n">
-        <v>32.67366344017525</v>
+        <v>32.70180760703992</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>858221</v>
+        <v>858580</v>
       </c>
       <c r="L6" t="n">
-        <v>38.0113047804703</v>
+        <v>38.03722425400079</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1606,10 +1606,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>858221</v>
+        <v>858580</v>
       </c>
       <c r="L9" t="n">
-        <v>34.16614135519872</v>
+        <v>34.19366861562114</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1673,10 +1673,10 @@
         <v>579999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>858221</v>
+        <v>858580</v>
       </c>
       <c r="L10" t="n">
-        <v>32.41845631836089</v>
+        <v>32.4467143422861</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -1740,10 +1740,10 @@
         <v>587999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>858221</v>
+        <v>858580</v>
       </c>
       <c r="L11" t="n">
-        <v>31.48629548799202</v>
+        <v>31.51494327843649</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -1807,10 +1807,10 @@
         <v>600000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>858221</v>
+        <v>858580</v>
       </c>
       <c r="L12" t="n">
-        <v>30.08793772233492</v>
+        <v>30.11717021127909</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -1825,7 +1825,7 @@
         <v>45.94594594594595</v>
       </c>
       <c r="Q12" t="n">
-        <v>42</v>
+        <v>42.1</v>
       </c>
       <c r="R12" t="n">
         <v>4</v>
@@ -1874,10 +1874,10 @@
         <v>634000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>858221</v>
+        <v>858580</v>
       </c>
       <c r="L13" t="n">
-        <v>26.12625419326723</v>
+        <v>26.15714318991824</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -1941,10 +1941,10 @@
         <v>643999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>944086</v>
+        <v>944481</v>
       </c>
       <c r="L14" t="n">
-        <v>31.78598136186746</v>
+        <v>31.8145097677984</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -2067,10 +2067,10 @@
         <v>650000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>944086</v>
+        <v>944481</v>
       </c>
       <c r="L16" t="n">
-        <v>31.15034011731982</v>
+        <v>31.17913436056416</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -2134,10 +2134,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1029951</v>
+        <v>1030382</v>
       </c>
       <c r="L17" t="n">
-        <v>32.0356016936728</v>
+        <v>32.06403062165294</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2201,10 +2201,10 @@
         <v>711999</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>1072884</v>
+        <v>1073333</v>
       </c>
       <c r="L18" t="n">
-        <v>33.63690762468264</v>
+        <v>33.66466883995927</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -2330,10 +2330,10 @@
         <v>720000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>1029951</v>
+        <v>1030382</v>
       </c>
       <c r="L20" t="n">
-        <v>30.09376174206346</v>
+        <v>30.12300292512874</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -2459,10 +2459,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1072884</v>
+        <v>1073333</v>
       </c>
       <c r="L22" t="n">
-        <v>30.74740605694558</v>
+        <v>30.77637601750808</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2477,7 +2477,7 @@
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>10.2</v>
+        <v>10.3</v>
       </c>
       <c r="R22" t="n">
         <v>4</v>
@@ -2526,10 +2526,10 @@
         <v>772000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1029951</v>
+        <v>1030382</v>
       </c>
       <c r="L23" t="n">
-        <v>25.04497786787915</v>
+        <v>25.07633091416581</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -2593,10 +2593,10 @@
         <v>775000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1029951</v>
+        <v>1030382</v>
       </c>
       <c r="L24" t="n">
-        <v>24.75370187513775</v>
+        <v>24.78517675968718</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -2660,10 +2660,10 @@
         <v>775000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>1029951</v>
+        <v>1030382</v>
       </c>
       <c r="L25" t="n">
-        <v>24.75370187513775</v>
+        <v>24.78517675968718</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -2789,10 +2789,10 @@
         <v>810000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>1072884</v>
+        <v>1073333</v>
       </c>
       <c r="L27" t="n">
-        <v>24.50255572829868</v>
+        <v>24.53413805408014</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -2853,10 +2853,10 @@
         <v>810000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>1244614</v>
+        <v>1245135</v>
       </c>
       <c r="L28" t="n">
-        <v>34.9195814927359</v>
+        <v>34.94681299618114</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -2982,10 +2982,10 @@
         <v>825000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1287546</v>
+        <v>1288085</v>
       </c>
       <c r="L30" t="n">
-        <v>35.92461939223919</v>
+        <v>35.95143177662965</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -3049,10 +3049,10 @@
         <v>829999</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1287546</v>
+        <v>1288085</v>
       </c>
       <c r="L31" t="n">
-        <v>35.53636141932016</v>
+        <v>35.5633362705101</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -3116,10 +3116,10 @@
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1373411</v>
+        <v>1373986</v>
       </c>
       <c r="L32" t="n">
-        <v>38.25599183347155</v>
+        <v>38.28183111036066</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3183,10 +3183,10 @@
         <v>930000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1373411</v>
+        <v>1373986</v>
       </c>
       <c r="L33" t="n">
-        <v>38.11036900097641</v>
+        <v>38.13626921962815</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3250,10 +3250,10 @@
         <v>860000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>1244614</v>
+        <v>1245135</v>
       </c>
       <c r="L34" t="n">
-        <v>30.90227170833688</v>
+        <v>30.93118416878491</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -3503,10 +3503,10 @@
         <v>880000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>1158749</v>
+        <v>1159234</v>
       </c>
       <c r="L38" t="n">
-        <v>24.05602939031663</v>
+        <v>24.08780280771613</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -3567,10 +3567,10 @@
         <v>940000</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>1244614</v>
+        <v>1245135</v>
       </c>
       <c r="L39" t="n">
-        <v>24.47457605329845</v>
+        <v>24.50617804495095</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -3631,10 +3631,10 @@
         <v>990000</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>1502209</v>
+        <v>1502838</v>
       </c>
       <c r="L40" t="n">
-        <v>34.09705307317424</v>
+        <v>34.12463618833168</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -3695,10 +3695,10 @@
         <v>990000</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>1502209</v>
+        <v>1502838</v>
       </c>
       <c r="L41" t="n">
-        <v>34.09705307317424</v>
+        <v>34.12463618833168</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
@@ -3821,10 +3821,10 @@
         <v>1055000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1545141</v>
+        <v>1545788</v>
       </c>
       <c r="L43" t="n">
-        <v>31.72144160306405</v>
+        <v>31.75002005449647</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -3885,10 +3885,10 @@
         <v>1055000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1545141</v>
+        <v>1545788</v>
       </c>
       <c r="L44" t="n">
-        <v>31.72144160306405</v>
+        <v>31.75002005449647</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -4011,10 +4011,10 @@
         <v>1115000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1502209</v>
+        <v>1502838</v>
       </c>
       <c r="L46" t="n">
-        <v>25.77597391574674</v>
+        <v>25.80703974746447</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -4075,10 +4075,10 @@
         <v>1123000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1716872</v>
+        <v>1717590</v>
       </c>
       <c r="L47" t="n">
-        <v>34.59034802827468</v>
+        <v>34.61769106713476</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -4142,10 +4142,10 @@
         <v>1130000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1502209</v>
+        <v>1502838</v>
       </c>
       <c r="L48" t="n">
-        <v>24.77744441685544</v>
+        <v>24.8089281745604</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -4268,10 +4268,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1759804</v>
+        <v>1760541</v>
       </c>
       <c r="L50" t="n">
-        <v>34.36769094740096</v>
+        <v>34.39516603135059</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4332,10 +4332,10 @@
         <v>1155000</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>1759804</v>
+        <v>1760541</v>
       </c>
       <c r="L51" t="n">
-        <v>34.36769094740096</v>
+        <v>34.39516603135059</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -4396,10 +4396,10 @@
         <v>1185000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1588074</v>
+        <v>1588739</v>
       </c>
       <c r="L52" t="n">
-        <v>25.38131094646723</v>
+        <v>25.41254416238287</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -4460,10 +4460,10 @@
         <v>1185000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1588074</v>
+        <v>1588739</v>
       </c>
       <c r="L53" t="n">
-        <v>25.38131094646723</v>
+        <v>25.41254416238287</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -4524,10 +4524,10 @@
         <v>1200000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1888602</v>
+        <v>1889392</v>
       </c>
       <c r="L54" t="n">
-        <v>36.46093777301941</v>
+        <v>36.48750497514545</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -4588,10 +4588,10 @@
         <v>1200000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1888602</v>
+        <v>1889392</v>
       </c>
       <c r="L55" t="n">
-        <v>36.46093777301941</v>
+        <v>36.48750497514545</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -4714,10 +4714,10 @@
         <v>1240000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1673939</v>
+        <v>1674640</v>
       </c>
       <c r="L57" t="n">
-        <v>25.92322659308374</v>
+        <v>25.95423494004682</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -4840,10 +4840,10 @@
         <v>1280000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1716872</v>
+        <v>1717590</v>
       </c>
       <c r="L59" t="n">
-        <v>25.44581075350987</v>
+        <v>25.47697646120436</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -4907,10 +4907,10 @@
         <v>1298000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1759804</v>
+        <v>1760541</v>
       </c>
       <c r="L60" t="n">
-        <v>26.24178601707918</v>
+        <v>26.27266277808923</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -4922,7 +4922,7 @@
         <v>62.21254466180763</v>
       </c>
       <c r="Q60" t="n">
-        <v>25.6</v>
+        <v>25.7</v>
       </c>
       <c r="R60" t="n">
         <v>3</v>
@@ -4971,10 +4971,10 @@
         <v>1300000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1716872</v>
+        <v>1717590</v>
       </c>
       <c r="L61" t="n">
-        <v>24.28090154653346</v>
+        <v>24.31255421841068</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -5097,10 +5097,10 @@
         <v>1335000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1802737</v>
+        <v>1803491</v>
       </c>
       <c r="L63" t="n">
-        <v>25.94593665077047</v>
+        <v>25.97689702915068</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -5161,10 +5161,10 @@
         <v>1420000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1931534</v>
+        <v>1932343</v>
       </c>
       <c r="L64" t="n">
-        <v>26.4833029084655</v>
+        <v>26.51408160973492</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -5176,7 +5176,7 @@
         <v>81.91902127554754</v>
       </c>
       <c r="Q64" t="n">
-        <v>30.1</v>
+        <v>30.2</v>
       </c>
       <c r="R64" t="n">
         <v>3</v>
@@ -5225,10 +5225,10 @@
         <v>1430000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1931534</v>
+        <v>1932343</v>
       </c>
       <c r="L65" t="n">
-        <v>25.96557968951103</v>
+        <v>25.99657514219784</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -5289,10 +5289,10 @@
         <v>1430000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>2146197</v>
+        <v>2147095</v>
       </c>
       <c r="L66" t="n">
-        <v>33.37051538139323</v>
+        <v>33.39838246561051</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -5353,10 +5353,10 @@
         <v>1430000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>2146197</v>
+        <v>2147095</v>
       </c>
       <c r="L67" t="n">
-        <v>33.37051538139323</v>
+        <v>33.39838246561051</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -5479,10 +5479,10 @@
         <v>1480000</v>
       </c>
       <c r="K69" s="3" t="n">
-        <v>2017399</v>
+        <v>2018244</v>
       </c>
       <c r="L69" t="n">
-        <v>26.63821088441107</v>
+        <v>26.66892605651249</v>
       </c>
       <c r="M69" s="3" t="n">
         <v>0</v>
@@ -5605,10 +5605,10 @@
         <v>1605000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2189129</v>
+        <v>2190046</v>
       </c>
       <c r="L71" t="n">
-        <v>26.68316942491739</v>
+        <v>26.71386811053284</v>
       </c>
       <c r="M71" s="3" t="n">
         <v>0</v>
@@ -5669,10 +5669,10 @@
         <v>1610000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2189129</v>
+        <v>2190046</v>
       </c>
       <c r="L72" t="n">
-        <v>26.454768083562</v>
+        <v>26.48556240371207</v>
       </c>
       <c r="M72" s="3" t="n">
         <v>0</v>
@@ -5733,10 +5733,10 @@
         <v>1615000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2189129</v>
+        <v>2190046</v>
       </c>
       <c r="L73" t="n">
-        <v>26.2263667422066</v>
+        <v>26.2572566968913</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
@@ -5797,10 +5797,10 @@
         <v>1630000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2232062</v>
+        <v>2232996</v>
       </c>
       <c r="L74" t="n">
-        <v>26.97335468280003</v>
+        <v>27.00389969350595</v>
       </c>
       <c r="M74" s="3" t="n">
         <v>0</v>
@@ -5861,10 +5861,10 @@
         <v>1690000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2317927</v>
+        <v>2318897</v>
       </c>
       <c r="L75" t="n">
-        <v>27.09002483684775</v>
+        <v>27.1205232487687</v>
       </c>
       <c r="M75" s="3" t="n">
         <v>0</v>
@@ -5925,10 +5925,10 @@
         <v>1705000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2317927</v>
+        <v>2318897</v>
       </c>
       <c r="L76" t="n">
-        <v>26.44289487977836</v>
+        <v>26.4736639876631</v>
       </c>
       <c r="M76" s="3" t="n">
         <v>0</v>
@@ -5989,10 +5989,10 @@
         <v>1725000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2360859</v>
+        <v>2361848</v>
       </c>
       <c r="L77" t="n">
-        <v>26.93337467421816</v>
+        <v>26.96397058574472</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
@@ -6053,10 +6053,10 @@
         <v>1780000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2446724</v>
+        <v>2447749</v>
       </c>
       <c r="L78" t="n">
-        <v>27.24966117960179</v>
+        <v>27.28012553574733</v>
       </c>
       <c r="M78" s="3" t="n">
         <v>0</v>
@@ -6117,10 +6117,10 @@
         <v>1875000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2575522</v>
+        <v>2576600</v>
       </c>
       <c r="L79" t="n">
-        <v>27.19922407962347</v>
+        <v>27.22968252736164</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
@@ -6181,10 +6181,10 @@
         <v>1910000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2618454</v>
+        <v>2619551</v>
       </c>
       <c r="L80" t="n">
-        <v>27.0561942275862</v>
+        <v>27.08674120106843</v>
       </c>
       <c r="M80" s="3" t="n">
         <v>0</v>
@@ -6245,10 +6245,10 @@
         <v>2020000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2747252</v>
+        <v>2748402</v>
       </c>
       <c r="L81" t="n">
-        <v>26.47198000037856</v>
+        <v>26.50274595928834</v>
       </c>
       <c r="M81" s="3" t="n">
         <v>0</v>
@@ -6309,10 +6309,10 @@
         <v>2110000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>2876050</v>
+        <v>2877254</v>
       </c>
       <c r="L82" t="n">
-        <v>26.63548964725926</v>
+        <v>26.6661893597159</v>
       </c>
       <c r="M82" s="3" t="n">
         <v>0</v>
@@ -6373,10 +6373,10 @@
         <v>2210000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3004847</v>
+        <v>3006105</v>
       </c>
       <c r="L83" t="n">
-        <v>26.45216212339597</v>
+        <v>26.48294054931548</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
@@ -6437,10 +6437,10 @@
         <v>2215000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3047780</v>
+        <v>3049056</v>
       </c>
       <c r="L84" t="n">
-        <v>27.32415069329151</v>
+        <v>27.35456482268611</v>
       </c>
       <c r="M84" s="3" t="n">
         <v>0</v>
@@ -6501,10 +6501,10 @@
         <v>2315000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3176577</v>
+        <v>3177907</v>
       </c>
       <c r="L85" t="n">
-        <v>27.12281175617654</v>
+        <v>27.15331191252607</v>
       </c>
       <c r="M85" s="3" t="n">
         <v>0</v>
@@ -6565,10 +6565,10 @@
         <v>2395000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3305375</v>
+        <v>3306758</v>
       </c>
       <c r="L86" t="n">
-        <v>27.54226071171955</v>
+        <v>27.57256503197392</v>
       </c>
       <c r="M86" s="3" t="n">
         <v>0</v>
@@ -6629,10 +6629,10 @@
         <v>2410000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3305375</v>
+        <v>3306758</v>
       </c>
       <c r="L87" t="n">
-        <v>27.08845441137541</v>
+        <v>27.11894852904265</v>
       </c>
       <c r="M87" s="3" t="n">
         <v>0</v>
@@ -6693,10 +6693,10 @@
         <v>2499000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3434172</v>
+        <v>3435610</v>
       </c>
       <c r="L88" t="n">
-        <v>27.23136756108896</v>
+        <v>27.26182541091684</v>
       </c>
       <c r="M88" s="3" t="n">
         <v>0</v>
@@ -6708,7 +6708,7 @@
         <v>63.67326854471646</v>
       </c>
       <c r="Q88" t="n">
-        <v>26.4</v>
+        <v>26.5</v>
       </c>
       <c r="R88" t="n">
         <v>3</v>
@@ -6757,10 +6757,10 @@
         <v>2510000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3434172</v>
+        <v>3435610</v>
       </c>
       <c r="L89" t="n">
-        <v>26.91105745431504</v>
+        <v>26.94164937230943</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
@@ -6821,10 +6821,10 @@
         <v>2530000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3477105</v>
+        <v>3478560</v>
       </c>
       <c r="L90" t="n">
-        <v>27.23832038434272</v>
+        <v>27.26875488707971</v>
       </c>
       <c r="M90" s="3" t="n">
         <v>0</v>
@@ -6885,10 +6885,10 @@
         <v>2610000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>3605902</v>
+        <v>3607412</v>
       </c>
       <c r="L91" t="n">
-        <v>27.61866517725662</v>
+        <v>27.64896274670041</v>
       </c>
       <c r="M91" s="3" t="n">
         <v>0</v>
@@ -6949,10 +6949,10 @@
         <v>3015000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4164025</v>
+        <v>4165768</v>
       </c>
       <c r="L92" t="n">
-        <v>27.59409465601192</v>
+        <v>27.62439002844134</v>
       </c>
       <c r="M92" s="3" t="n">
         <v>0</v>
@@ -7013,10 +7013,10 @@
         <v>3098000</v>
       </c>
       <c r="K93" s="3" t="n">
-        <v>4292823</v>
+        <v>4294620</v>
       </c>
       <c r="L93" t="n">
-        <v>27.83303667539985</v>
+        <v>27.86323353404958</v>
       </c>
       <c r="M93" s="3" t="n">
         <v>0</v>
@@ -7028,7 +7028,7 @@
         <v>100</v>
       </c>
       <c r="Q93" t="n">
-        <v>34.3</v>
+        <v>34.4</v>
       </c>
       <c r="R93" t="n">
         <v>3</v>
@@ -7312,10 +7312,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>428896</v>
+        <v>429075</v>
       </c>
       <c r="L2" t="n">
-        <v>27.72163881220622</v>
+        <v>27.75179164481734</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7379,10 +7379,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>428896</v>
+        <v>429075</v>
       </c>
       <c r="L3" t="n">
-        <v>27.72163881220622</v>
+        <v>27.75179164481734</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7446,10 +7446,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>428896</v>
+        <v>429075</v>
       </c>
       <c r="L4" t="n">
-        <v>27.72140565545027</v>
+        <v>27.7515585853289</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7513,10 +7513,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>428896</v>
+        <v>429075</v>
       </c>
       <c r="L5" t="n">
-        <v>27.72140565545027</v>
+        <v>27.7515585853289</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7580,10 +7580,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514761</v>
+        <v>514976</v>
       </c>
       <c r="L6" t="n">
-        <v>25.40227406505155</v>
+        <v>25.43341825638477</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7644,10 +7644,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>514761</v>
+        <v>514976</v>
       </c>
       <c r="L7" t="n">
-        <v>25.40227406505155</v>
+        <v>25.43341825638477</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7708,10 +7708,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>514761</v>
+        <v>514976</v>
       </c>
       <c r="L8" t="n">
-        <v>25.40227406505155</v>
+        <v>25.43341825638477</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7772,10 +7772,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>514761</v>
+        <v>514976</v>
       </c>
       <c r="L9" t="n">
-        <v>25.40227406505155</v>
+        <v>25.43341825638477</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7836,10 +7836,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>514761</v>
+        <v>514976</v>
       </c>
       <c r="L10" t="n">
-        <v>25.20800915376262</v>
+        <v>25.23923444976077</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7900,10 +7900,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>514761</v>
+        <v>514976</v>
       </c>
       <c r="L11" t="n">
-        <v>25.20800915376262</v>
+        <v>25.23923444976077</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7964,10 +7964,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>514761</v>
+        <v>514976</v>
       </c>
       <c r="L12" t="n">
-        <v>25.20800915376262</v>
+        <v>25.23923444976077</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -8028,10 +8028,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>514761</v>
+        <v>514976</v>
       </c>
       <c r="L13" t="n">
-        <v>25.20800915376262</v>
+        <v>25.23923444976077</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -8092,10 +8092,10 @@
         <v>420000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>557693</v>
+        <v>557927</v>
       </c>
       <c r="L14" t="n">
-        <v>24.68974866100166</v>
+        <v>24.72133451150419</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -8159,10 +8159,10 @@
         <v>420000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>557693</v>
+        <v>557927</v>
       </c>
       <c r="L15" t="n">
-        <v>24.68974866100166</v>
+        <v>24.72133451150419</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0</v>
@@ -8177,7 +8177,7 @@
         <v>3.361344537815107</v>
       </c>
       <c r="Q15" t="n">
-        <v>31.8</v>
+        <v>31.9</v>
       </c>
       <c r="R15" t="n">
         <v>4</v>
@@ -8226,10 +8226,10 @@
         <v>420000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>557693</v>
+        <v>557927</v>
       </c>
       <c r="L16" t="n">
-        <v>24.68974866100166</v>
+        <v>24.72133451150419</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -8293,10 +8293,10 @@
         <v>425000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>557693</v>
+        <v>557927</v>
       </c>
       <c r="L17" t="n">
-        <v>23.79319804982311</v>
+        <v>23.82515992235543</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -8360,10 +8360,10 @@
         <v>454000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>600626</v>
+        <v>600877</v>
       </c>
       <c r="L18" t="n">
-        <v>24.41219660820544</v>
+        <v>24.44377135420394</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -8424,10 +8424,10 @@
         <v>454000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>600626</v>
+        <v>600877</v>
       </c>
       <c r="L19" t="n">
-        <v>24.41219660820544</v>
+        <v>24.44377135420394</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -8488,10 +8488,10 @@
         <v>454000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>600626</v>
+        <v>600877</v>
       </c>
       <c r="L20" t="n">
-        <v>24.41219660820544</v>
+        <v>24.44377135420394</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -8552,10 +8552,10 @@
         <v>454000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>600626</v>
+        <v>600877</v>
       </c>
       <c r="L21" t="n">
-        <v>24.41219660820544</v>
+        <v>24.44377135420394</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -8616,10 +8616,10 @@
         <v>455000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>600626</v>
+        <v>600877</v>
       </c>
       <c r="L22" t="n">
-        <v>24.24570364919268</v>
+        <v>24.27734794308985</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -8680,10 +8680,10 @@
         <v>455000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>600626</v>
+        <v>600877</v>
       </c>
       <c r="L23" t="n">
-        <v>24.24570364919268</v>
+        <v>24.27734794308985</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -8744,10 +8744,10 @@
         <v>455000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>600626</v>
+        <v>600877</v>
       </c>
       <c r="L24" t="n">
-        <v>24.24570364919268</v>
+        <v>24.27734794308985</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -8808,10 +8808,10 @@
         <v>455000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>600626</v>
+        <v>600877</v>
       </c>
       <c r="L25" t="n">
-        <v>24.24570364919268</v>
+        <v>24.27734794308985</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -8872,10 +8872,10 @@
         <v>475000</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>686491</v>
+        <v>686778</v>
       </c>
       <c r="L26" t="n">
-        <v>30.80754154096703</v>
+        <v>30.83645661334521</v>
       </c>
       <c r="M26" s="3" t="n">
         <v>0</v>
@@ -8936,10 +8936,10 @@
         <v>475000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>686491</v>
+        <v>686778</v>
       </c>
       <c r="L27" t="n">
-        <v>30.80754154096703</v>
+        <v>30.83645661334521</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -9000,10 +9000,10 @@
         <v>475000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>686491</v>
+        <v>686778</v>
       </c>
       <c r="L28" t="n">
-        <v>30.80754154096703</v>
+        <v>30.83645661334521</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -9064,10 +9064,10 @@
         <v>475000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>686491</v>
+        <v>686778</v>
       </c>
       <c r="L29" t="n">
-        <v>30.80754154096703</v>
+        <v>30.83645661334521</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -9128,10 +9128,10 @@
         <v>477000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>643559</v>
+        <v>643828</v>
       </c>
       <c r="L30" t="n">
-        <v>25.88092156274716</v>
+        <v>25.91188951086315</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -9195,10 +9195,10 @@
         <v>477000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>643559</v>
+        <v>643828</v>
       </c>
       <c r="L31" t="n">
-        <v>25.88092156274716</v>
+        <v>25.91188951086315</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -9262,10 +9262,10 @@
         <v>477000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>643559</v>
+        <v>643828</v>
       </c>
       <c r="L32" t="n">
-        <v>25.88092156274716</v>
+        <v>25.91188951086315</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -9329,10 +9329,10 @@
         <v>479999</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>686491</v>
+        <v>686778</v>
       </c>
       <c r="L33" t="n">
-        <v>30.07934554131081</v>
+        <v>30.10856492199808</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -9393,10 +9393,10 @@
         <v>479999</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>686491</v>
+        <v>686778</v>
       </c>
       <c r="L34" t="n">
-        <v>30.07934554131081</v>
+        <v>30.10856492199808</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -9457,10 +9457,10 @@
         <v>479999</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>686491</v>
+        <v>686778</v>
       </c>
       <c r="L35" t="n">
-        <v>30.07934554131081</v>
+        <v>30.10856492199808</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
@@ -9521,10 +9521,10 @@
         <v>479999</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>686491</v>
+        <v>686778</v>
       </c>
       <c r="L36" t="n">
-        <v>30.07934554131081</v>
+        <v>30.10856492199808</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -9585,10 +9585,10 @@
         <v>479999</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>643559</v>
+        <v>643828</v>
       </c>
       <c r="L37" t="n">
-        <v>25.41491922263537</v>
+        <v>25.44608187279833</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
@@ -9652,10 +9652,10 @@
         <v>500000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>643559</v>
+        <v>643828</v>
       </c>
       <c r="L38" t="n">
-        <v>22.30704566325698</v>
+        <v>22.33950682480414</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -9716,10 +9716,10 @@
         <v>547999</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>772356</v>
+        <v>772679</v>
       </c>
       <c r="L39" t="n">
-        <v>29.04839219220152</v>
+        <v>29.0780518171194</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -9780,10 +9780,10 @@
         <v>547999</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>772356</v>
+        <v>772679</v>
       </c>
       <c r="L40" t="n">
-        <v>29.04839219220152</v>
+        <v>29.0780518171194</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -9844,10 +9844,10 @@
         <v>547999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>772356</v>
+        <v>772679</v>
       </c>
       <c r="L41" t="n">
-        <v>29.04839219220152</v>
+        <v>29.0780518171194</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
@@ -9859,7 +9859,7 @@
         <v>64.67267226890753</v>
       </c>
       <c r="Q41" t="n">
-        <v>26.9</v>
+        <v>27</v>
       </c>
       <c r="R41" t="n">
         <v>3</v>
@@ -9908,10 +9908,10 @@
         <v>547999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>772356</v>
+        <v>772679</v>
       </c>
       <c r="L42" t="n">
-        <v>29.04839219220152</v>
+        <v>29.0780518171194</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -9972,10 +9972,10 @@
         <v>552999</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>772356</v>
+        <v>772679</v>
       </c>
       <c r="L43" t="n">
-        <v>28.40102232649193</v>
+        <v>28.43095256891931</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -9987,7 +9987,7 @@
         <v>34.11769473304435</v>
       </c>
       <c r="Q43" t="n">
-        <v>20.2</v>
+        <v>20.3</v>
       </c>
       <c r="R43" t="n">
         <v>3</v>
@@ -10036,10 +10036,10 @@
         <v>552999</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>772356</v>
+        <v>772679</v>
       </c>
       <c r="L44" t="n">
-        <v>28.40102232649193</v>
+        <v>28.43095256891931</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -10051,7 +10051,7 @@
         <v>34.11769473304435</v>
       </c>
       <c r="Q44" t="n">
-        <v>20.2</v>
+        <v>20.3</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -10100,10 +10100,10 @@
         <v>552999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>772356</v>
+        <v>772679</v>
       </c>
       <c r="L45" t="n">
-        <v>28.40102232649193</v>
+        <v>28.43095256891931</v>
       </c>
       <c r="M45" s="3" t="n">
         <v>0</v>
@@ -10115,7 +10115,7 @@
         <v>34.11769473304435</v>
       </c>
       <c r="Q45" t="n">
-        <v>20.2</v>
+        <v>20.3</v>
       </c>
       <c r="R45" t="n">
         <v>3</v>
@@ -10164,10 +10164,10 @@
         <v>552999</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>772356</v>
+        <v>772679</v>
       </c>
       <c r="L46" t="n">
-        <v>28.40102232649193</v>
+        <v>28.43095256891931</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -10179,7 +10179,7 @@
         <v>34.11769473304435</v>
       </c>
       <c r="Q46" t="n">
-        <v>20.2</v>
+        <v>20.3</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -10228,10 +10228,10 @@
         <v>585000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>729424</v>
+        <v>729729</v>
       </c>
       <c r="L47" t="n">
-        <v>19.79973239158569</v>
+        <v>19.8332531665865</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -10292,10 +10292,10 @@
         <v>595000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>729424</v>
+        <v>729729</v>
       </c>
       <c r="L48" t="n">
-        <v>18.42878764614271</v>
+        <v>18.46288142584439</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -10356,10 +10356,10 @@
         <v>614999</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>858221</v>
+        <v>858580</v>
       </c>
       <c r="L49" t="n">
-        <v>28.34025268549709</v>
+        <v>28.37021593794405</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -10420,10 +10420,10 @@
         <v>614999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>858221</v>
+        <v>858580</v>
       </c>
       <c r="L50" t="n">
-        <v>28.34025268549709</v>
+        <v>28.37021593794405</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -10484,10 +10484,10 @@
         <v>614999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>858221</v>
+        <v>858580</v>
       </c>
       <c r="L51" t="n">
-        <v>28.34025268549709</v>
+        <v>28.37021593794405</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -10548,10 +10548,10 @@
         <v>614999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>858221</v>
+        <v>858580</v>
       </c>
       <c r="L52" t="n">
-        <v>28.34025268549709</v>
+        <v>28.37021593794405</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -10612,10 +10612,10 @@
         <v>650000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>815289</v>
+        <v>815630</v>
       </c>
       <c r="L53" t="n">
-        <v>20.27366982750902</v>
+        <v>20.30700194941334</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -10676,10 +10676,10 @@
         <v>672000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>858221</v>
+        <v>858580</v>
       </c>
       <c r="L54" t="n">
-        <v>21.69849024901512</v>
+        <v>21.73123063663258</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -10740,10 +10740,10 @@
         <v>700000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>901154</v>
+        <v>901531</v>
       </c>
       <c r="L55" t="n">
-        <v>22.32182290707249</v>
+        <v>22.35430617471834</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -10804,10 +10804,10 @@
         <v>715000</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>944086</v>
+        <v>944481</v>
       </c>
       <c r="L56" t="n">
-        <v>24.2653741290518</v>
+        <v>24.29704779662058</v>
       </c>
       <c r="M56" s="3" t="n">
         <v>0</v>
@@ -10868,10 +10868,10 @@
         <v>734999</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>987019</v>
+        <v>987432</v>
       </c>
       <c r="L57" t="n">
-        <v>25.53344971069453</v>
+        <v>25.5645958405237</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -10932,10 +10932,10 @@
         <v>752000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>987019</v>
+        <v>987432</v>
       </c>
       <c r="L58" t="n">
-        <v>23.81099046725544</v>
+        <v>23.8428570271168</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -10996,10 +10996,10 @@
         <v>810000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1072884</v>
+        <v>1073333</v>
       </c>
       <c r="L59" t="n">
-        <v>24.50255572829868</v>
+        <v>24.53413805408014</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -11060,10 +11060,10 @@
         <v>815000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1072884</v>
+        <v>1073333</v>
       </c>
       <c r="L60" t="n">
-        <v>24.03652212168324</v>
+        <v>24.06829940009298</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -11124,10 +11124,10 @@
         <v>875000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1158749</v>
+        <v>1159234</v>
       </c>
       <c r="L61" t="n">
-        <v>24.48752922332619</v>
+        <v>24.51912210994502</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -11188,10 +11188,10 @@
         <v>992000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1330479</v>
+        <v>1331036</v>
       </c>
       <c r="L62" t="n">
-        <v>25.44038650741575</v>
+        <v>25.47158754534063</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -11252,10 +11252,10 @@
         <v>1050000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1416344</v>
+        <v>1416937</v>
       </c>
       <c r="L63" t="n">
-        <v>25.86546771123399</v>
+        <v>25.89649363380305</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -11316,10 +11316,10 @@
         <v>1050000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1416344</v>
+        <v>1416937</v>
       </c>
       <c r="L64" t="n">
-        <v>25.86546771123399</v>
+        <v>25.89649363380305</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -11380,10 +11380,10 @@
         <v>1100000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1502209</v>
+        <v>1502838</v>
       </c>
       <c r="L65" t="n">
-        <v>26.77450341463804</v>
+        <v>26.80515132036853</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -11395,7 +11395,7 @@
         <v>94.11761630126171</v>
       </c>
       <c r="Q65" t="n">
-        <v>31.6</v>
+        <v>31.7</v>
       </c>
       <c r="R65" t="n">
         <v>3</v>
@@ -11444,10 +11444,10 @@
         <v>1105000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1502209</v>
+        <v>1502838</v>
       </c>
       <c r="L66" t="n">
-        <v>26.44166024834094</v>
+        <v>26.47244746273384</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -11508,10 +11508,10 @@
         <v>1155000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1588074</v>
+        <v>1588739</v>
       </c>
       <c r="L67" t="n">
-        <v>27.2703916819997</v>
+        <v>27.30083418358837</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -11778,7 +11778,7 @@
         <v>315000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>300098</v>
+        <v>300224</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -11839,10 +11839,10 @@
         <v>380000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>385963</v>
+        <v>386125</v>
       </c>
       <c r="L3" t="n">
-        <v>1.544966745517057</v>
+        <v>1.586273875040466</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -11903,7 +11903,7 @@
         <v>415000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>385963</v>
+        <v>386125</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -11964,10 +11964,10 @@
         <v>495000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>471828</v>
+        <v>472026</v>
       </c>
       <c r="L5" t="n">
-        <v>6.745890451605247</v>
+        <v>6.785007605513256</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -12028,10 +12028,10 @@
         <v>490000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514761</v>
+        <v>514976</v>
       </c>
       <c r="L6" t="n">
-        <v>4.810193468425153</v>
+        <v>4.849934754240974</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -12092,10 +12092,10 @@
         <v>550000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>557693</v>
+        <v>557927</v>
       </c>
       <c r="L7" t="n">
-        <v>6.758736437430629</v>
+        <v>6.797842728529001</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -12156,7 +12156,7 @@
         <v>530000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>471828</v>
+        <v>472026</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -12220,10 +12220,10 @@
         <v>600000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>600626</v>
+        <v>600877</v>
       </c>
       <c r="L9" t="n">
-        <v>8.428872542980157</v>
+        <v>8.467123887251466</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -12284,10 +12284,10 @@
         <v>646000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>729424</v>
+        <v>729729</v>
       </c>
       <c r="L10" t="n">
-        <v>17.05797999517427</v>
+        <v>17.09264672227635</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -12299,7 +12299,7 @@
         <v>100</v>
       </c>
       <c r="Q10" t="n">
-        <v>25.9</v>
+        <v>26</v>
       </c>
       <c r="R10" t="n">
         <v>4</v>
@@ -12348,7 +12348,7 @@
         <v>615000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>557693</v>
+        <v>557927</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -12412,7 +12412,7 @@
         <v>700000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>643559</v>
+        <v>643828</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -12476,7 +12476,7 @@
         <v>745000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>686491</v>
+        <v>686778</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -12540,7 +12540,7 @@
         <v>930000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>858221</v>
+        <v>858580</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -12611,7 +12611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12657,40 +12657,8 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Apple MacBook Pro 14Inch MW2U3 M4 10Core CPU 10Core GPU 16GB 512GB Space Black</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>458000</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>495000</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>37000</v>
-      </c>
-      <c r="F2" t="n">
-        <v>8.08</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:F2"/>
-  <conditionalFormatting sqref="E2">
-    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
+  <autoFilter ref="A1:F1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: price data 2026-10-03
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MacBook Pro'!$A$1:$S$93</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MacBook Air'!$A$1:$S$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20261002T095103629503+0000</t>
+          <t>20261003T091351304003+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-02T09:51:03.629503+00:00</t>
+          <t>2026-10-03T09:13:51.304003+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>277.099958</v>
+        <v>276.817029</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -729,7 +729,7 @@
         <v>532000</v>
       </c>
       <c r="D22" t="n">
-        <v>51.6</v>
+        <v>51.5</v>
       </c>
       <c r="E22" t="n">
         <v>4</v>
@@ -813,7 +813,7 @@
         <v>847999</v>
       </c>
       <c r="D26" t="n">
-        <v>47.4</v>
+        <v>47.3</v>
       </c>
       <c r="E26" t="n">
         <v>5</v>
@@ -831,10 +831,10 @@
         </is>
       </c>
       <c r="C27" s="3" t="n">
-        <v>643999</v>
+        <v>644999</v>
       </c>
       <c r="D27" t="n">
-        <v>44.4</v>
+        <v>44.3</v>
       </c>
       <c r="E27" t="n">
         <v>4</v>
@@ -1147,10 +1147,10 @@
         <v>470000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>686778</v>
+        <v>686077</v>
       </c>
       <c r="L2" t="n">
-        <v>35.20468040618657</v>
+        <v>35.13847571045233</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1165,7 +1165,7 @@
         <v>28.4414106939704</v>
       </c>
       <c r="Q2" t="n">
-        <v>35.4</v>
+        <v>35.3</v>
       </c>
       <c r="R2" t="n">
         <v>5</v>
@@ -1214,10 +1214,10 @@
         <v>495000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>686778</v>
+        <v>686077</v>
       </c>
       <c r="L3" t="n">
-        <v>27.92430741811764</v>
+        <v>27.85066399252562</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>772679</v>
+        <v>771890</v>
       </c>
       <c r="L4" t="n">
-        <v>35.29020459984029</v>
+        <v>35.22406042311728</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>772679</v>
+        <v>771890</v>
       </c>
       <c r="L5" t="n">
-        <v>32.70180760703992</v>
+        <v>32.63301765795644</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>858580</v>
+        <v>857704</v>
       </c>
       <c r="L6" t="n">
-        <v>38.03722425400079</v>
+        <v>37.97393972745842</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1433,7 +1433,7 @@
         <v>100</v>
       </c>
       <c r="Q6" t="n">
-        <v>51.6</v>
+        <v>51.5</v>
       </c>
       <c r="R6" t="n">
         <v>4</v>
@@ -1606,10 +1606,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>858580</v>
+        <v>857704</v>
       </c>
       <c r="L9" t="n">
-        <v>34.19366861562114</v>
+        <v>34.12645854513912</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1673,10 +1673,10 @@
         <v>579999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>858580</v>
+        <v>857704</v>
       </c>
       <c r="L10" t="n">
-        <v>32.4467143422861</v>
+        <v>32.37772005260556</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -1740,10 +1740,10 @@
         <v>587999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>858580</v>
+        <v>857704</v>
       </c>
       <c r="L11" t="n">
-        <v>31.51494327843649</v>
+        <v>31.44499734174027</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -1807,10 +1807,10 @@
         <v>600000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>858580</v>
+        <v>857704</v>
       </c>
       <c r="L12" t="n">
-        <v>30.11717021127909</v>
+        <v>30.04579668510349</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -1825,7 +1825,7 @@
         <v>45.94594594594595</v>
       </c>
       <c r="Q12" t="n">
-        <v>42.1</v>
+        <v>42</v>
       </c>
       <c r="R12" t="n">
         <v>4</v>
@@ -1874,10 +1874,10 @@
         <v>634000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>858580</v>
+        <v>857704</v>
       </c>
       <c r="L13" t="n">
-        <v>26.15714318991824</v>
+        <v>26.08172516392602</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -1935,19 +1935,19 @@
         </is>
       </c>
       <c r="I14" s="3" t="n">
-        <v>643999</v>
+        <v>644999</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>643999</v>
+        <v>644999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>944481</v>
+        <v>943517</v>
       </c>
       <c r="L14" t="n">
-        <v>31.8145097677984</v>
+        <v>31.63885759345089</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="N14" t="n">
         <v>0</v>
@@ -1956,10 +1956,10 @@
         <v>100</v>
       </c>
       <c r="P14" t="n">
-        <v>69.44023999999999</v>
+        <v>69.20023999999999</v>
       </c>
       <c r="Q14" t="n">
-        <v>44.4</v>
+        <v>44.3</v>
       </c>
       <c r="R14" t="n">
         <v>4</v>
@@ -2067,10 +2067,10 @@
         <v>650000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>944481</v>
+        <v>943517</v>
       </c>
       <c r="L16" t="n">
-        <v>31.17913436056416</v>
+        <v>31.10881944893415</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -2134,10 +2134,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1030382</v>
+        <v>1029330</v>
       </c>
       <c r="L17" t="n">
-        <v>32.06403062165294</v>
+        <v>31.99459842810371</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2201,10 +2201,10 @@
         <v>711999</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>1073333</v>
+        <v>1072237</v>
       </c>
       <c r="L18" t="n">
-        <v>33.66466883995927</v>
+        <v>33.59686338001767</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -2330,10 +2330,10 @@
         <v>720000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>1030382</v>
+        <v>1029330</v>
       </c>
       <c r="L20" t="n">
-        <v>30.12300292512874</v>
+        <v>30.05158695462097</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -2459,10 +2459,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1073333</v>
+        <v>1072237</v>
       </c>
       <c r="L22" t="n">
-        <v>30.77637601750808</v>
+        <v>30.70561825417328</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2477,7 +2477,7 @@
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>10.3</v>
+        <v>10.2</v>
       </c>
       <c r="R22" t="n">
         <v>4</v>
@@ -2526,10 +2526,10 @@
         <v>772000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1030382</v>
+        <v>1029330</v>
       </c>
       <c r="L23" t="n">
-        <v>25.07633091416581</v>
+        <v>24.99975712356581</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -2593,10 +2593,10 @@
         <v>775000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1030382</v>
+        <v>1029330</v>
       </c>
       <c r="L24" t="n">
-        <v>24.78517675968718</v>
+        <v>24.7083054025434</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -2605,13 +2605,13 @@
         <v>0</v>
       </c>
       <c r="O24" t="n">
-        <v>0</v>
+        <v>62.5</v>
       </c>
       <c r="P24" t="n">
         <v>68.99999999999999</v>
       </c>
       <c r="Q24" t="n">
-        <v>19.8</v>
+        <v>33.6</v>
       </c>
       <c r="R24" t="n">
         <v>4</v>
@@ -2654,19 +2654,19 @@
         </is>
       </c>
       <c r="I25" s="3" t="n">
-        <v>775000</v>
+        <v>780000</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>775000</v>
+        <v>780000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>1030382</v>
+        <v>1029330</v>
       </c>
       <c r="L25" t="n">
-        <v>24.78517675968718</v>
+        <v>24.22255253417271</v>
       </c>
       <c r="M25" s="3" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="N25" t="n">
         <v>0</v>
@@ -2675,10 +2675,10 @@
         <v>0</v>
       </c>
       <c r="P25" t="n">
-        <v>68.99999999999999</v>
+        <v>68</v>
       </c>
       <c r="Q25" t="n">
-        <v>19.8</v>
+        <v>19.4</v>
       </c>
       <c r="R25" t="n">
         <v>4</v>
@@ -2789,10 +2789,10 @@
         <v>810000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>1073333</v>
+        <v>1072237</v>
       </c>
       <c r="L27" t="n">
-        <v>24.53413805408014</v>
+        <v>24.45699971181744</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -2804,7 +2804,7 @@
         <v>61.99999999999999</v>
       </c>
       <c r="Q27" t="n">
-        <v>24.9</v>
+        <v>24.8</v>
       </c>
       <c r="R27" t="n">
         <v>3</v>
@@ -2853,10 +2853,10 @@
         <v>810000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>1245135</v>
+        <v>1243863</v>
       </c>
       <c r="L28" t="n">
-        <v>34.94681299618114</v>
+        <v>34.88028826325728</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -2982,10 +2982,10 @@
         <v>825000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1288085</v>
+        <v>1286770</v>
       </c>
       <c r="L30" t="n">
-        <v>35.95143177662965</v>
+        <v>35.8859780691188</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -3000,7 +3000,7 @@
         <v>1.718244359164265</v>
       </c>
       <c r="Q30" t="n">
-        <v>34.7</v>
+        <v>34.6</v>
       </c>
       <c r="R30" t="n">
         <v>4</v>
@@ -3049,10 +3049,10 @@
         <v>829999</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1288085</v>
+        <v>1286770</v>
       </c>
       <c r="L31" t="n">
-        <v>35.5633362705101</v>
+        <v>35.49748595320064</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -3116,10 +3116,10 @@
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1373986</v>
+        <v>1372583</v>
       </c>
       <c r="L32" t="n">
-        <v>38.28183111036066</v>
+        <v>38.21874524163566</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3134,7 +3134,7 @@
         <v>100</v>
       </c>
       <c r="Q32" t="n">
-        <v>47.4</v>
+        <v>47.3</v>
       </c>
       <c r="R32" t="n">
         <v>5</v>
@@ -3183,10 +3183,10 @@
         <v>930000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1373986</v>
+        <v>1372583</v>
       </c>
       <c r="L33" t="n">
-        <v>38.13626921962815</v>
+        <v>38.07303456330146</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3250,10 +3250,10 @@
         <v>860000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>1245135</v>
+        <v>1243863</v>
       </c>
       <c r="L34" t="n">
-        <v>30.93118416878491</v>
+        <v>30.86055297086576</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -3503,10 +3503,10 @@
         <v>880000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>1159234</v>
+        <v>1158050</v>
       </c>
       <c r="L38" t="n">
-        <v>24.08780280771613</v>
+        <v>24.01018954276585</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -3567,10 +3567,10 @@
         <v>940000</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>1245135</v>
+        <v>1243863</v>
       </c>
       <c r="L39" t="n">
-        <v>24.50617804495095</v>
+        <v>24.42897650303932</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -3631,10 +3631,10 @@
         <v>990000</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>1502838</v>
+        <v>1501303</v>
       </c>
       <c r="L40" t="n">
-        <v>34.12463618833168</v>
+        <v>34.0572822408268</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -3695,10 +3695,10 @@
         <v>990000</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>1502838</v>
+        <v>1501303</v>
       </c>
       <c r="L41" t="n">
-        <v>34.12463618833168</v>
+        <v>34.0572822408268</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
@@ -3821,10 +3821,10 @@
         <v>1055000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1545788</v>
+        <v>1544210</v>
       </c>
       <c r="L43" t="n">
-        <v>31.75002005449647</v>
+        <v>31.68027664631106</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -3885,10 +3885,10 @@
         <v>1055000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1545788</v>
+        <v>1544210</v>
       </c>
       <c r="L44" t="n">
-        <v>31.75002005449647</v>
+        <v>31.68027664631106</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -4011,10 +4011,10 @@
         <v>1115000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1502838</v>
+        <v>1501303</v>
       </c>
       <c r="L46" t="n">
-        <v>25.80703974746447</v>
+        <v>25.73118151365847</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -4075,10 +4075,10 @@
         <v>1123000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1717590</v>
+        <v>1715837</v>
       </c>
       <c r="L47" t="n">
-        <v>34.61769106713476</v>
+        <v>34.55089265472186</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -4142,10 +4142,10 @@
         <v>1130000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1502838</v>
+        <v>1501303</v>
       </c>
       <c r="L48" t="n">
-        <v>24.8089281745604</v>
+        <v>24.73204942639827</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -4268,10 +4268,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1760541</v>
+        <v>1758743</v>
       </c>
       <c r="L50" t="n">
-        <v>34.39516603135059</v>
+        <v>34.32809682824608</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4283,7 +4283,7 @@
         <v>22.53136001640632</v>
       </c>
       <c r="Q50" t="n">
-        <v>19.6</v>
+        <v>19.5</v>
       </c>
       <c r="R50" t="n">
         <v>3</v>
@@ -4332,10 +4332,10 @@
         <v>1155000</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>1760541</v>
+        <v>1758743</v>
       </c>
       <c r="L51" t="n">
-        <v>34.39516603135059</v>
+        <v>34.32809682824608</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -4347,7 +4347,7 @@
         <v>22.53136001640632</v>
       </c>
       <c r="Q51" t="n">
-        <v>19.6</v>
+        <v>19.5</v>
       </c>
       <c r="R51" t="n">
         <v>3</v>
@@ -4396,10 +4396,10 @@
         <v>1185000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1588739</v>
+        <v>1587117</v>
       </c>
       <c r="L52" t="n">
-        <v>25.41254416238287</v>
+        <v>25.33631736034583</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -4460,10 +4460,10 @@
         <v>1185000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1588739</v>
+        <v>1587117</v>
       </c>
       <c r="L53" t="n">
-        <v>25.41254416238287</v>
+        <v>25.33631736034583</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -4524,10 +4524,10 @@
         <v>1200000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1889392</v>
+        <v>1887463</v>
       </c>
       <c r="L54" t="n">
-        <v>36.48750497514545</v>
+        <v>36.42259477404325</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -4588,10 +4588,10 @@
         <v>1200000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1889392</v>
+        <v>1887463</v>
       </c>
       <c r="L55" t="n">
-        <v>36.48750497514545</v>
+        <v>36.42259477404325</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -4714,10 +4714,10 @@
         <v>1240000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1674640</v>
+        <v>1672930</v>
       </c>
       <c r="L57" t="n">
-        <v>25.95423494004682</v>
+        <v>25.87854841505622</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -4729,7 +4729,7 @@
         <v>100</v>
       </c>
       <c r="Q57" t="n">
-        <v>33.7</v>
+        <v>33.6</v>
       </c>
       <c r="R57" t="n">
         <v>3</v>
@@ -4840,10 +4840,10 @@
         <v>1280000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1717590</v>
+        <v>1715837</v>
       </c>
       <c r="L59" t="n">
-        <v>25.47697646120436</v>
+        <v>25.40083935711842</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -4907,10 +4907,10 @@
         <v>1298000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1760541</v>
+        <v>1758743</v>
       </c>
       <c r="L60" t="n">
-        <v>26.27266277808923</v>
+        <v>26.19728976888607</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -4922,7 +4922,7 @@
         <v>62.21254466180763</v>
       </c>
       <c r="Q60" t="n">
-        <v>25.7</v>
+        <v>25.6</v>
       </c>
       <c r="R60" t="n">
         <v>3</v>
@@ -4971,10 +4971,10 @@
         <v>1300000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1717590</v>
+        <v>1715837</v>
       </c>
       <c r="L61" t="n">
-        <v>24.31255421841068</v>
+        <v>24.23522747207339</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -5097,10 +5097,10 @@
         <v>1335000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1803491</v>
+        <v>1801650</v>
       </c>
       <c r="L63" t="n">
-        <v>25.97689702915068</v>
+        <v>25.90125718091749</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -5161,10 +5161,10 @@
         <v>1420000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1932343</v>
+        <v>1930370</v>
       </c>
       <c r="L64" t="n">
-        <v>26.51408160973492</v>
+        <v>26.43897283940385</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -5176,7 +5176,7 @@
         <v>81.91902127554754</v>
       </c>
       <c r="Q64" t="n">
-        <v>30.2</v>
+        <v>30.1</v>
       </c>
       <c r="R64" t="n">
         <v>3</v>
@@ -5225,10 +5225,10 @@
         <v>1430000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1932343</v>
+        <v>1930370</v>
       </c>
       <c r="L65" t="n">
-        <v>25.99657514219784</v>
+        <v>25.92093743686443</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -5289,10 +5289,10 @@
         <v>1430000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>2147095</v>
+        <v>2144903</v>
       </c>
       <c r="L66" t="n">
-        <v>33.39838246561051</v>
+        <v>33.33031843398047</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -5353,10 +5353,10 @@
         <v>1430000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>2147095</v>
+        <v>2144903</v>
       </c>
       <c r="L67" t="n">
-        <v>33.39838246561051</v>
+        <v>33.33031843398047</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -5479,10 +5479,10 @@
         <v>1480000</v>
       </c>
       <c r="K69" s="3" t="n">
-        <v>2018244</v>
+        <v>2016183</v>
       </c>
       <c r="L69" t="n">
-        <v>26.66892605651249</v>
+        <v>26.59396493274668</v>
       </c>
       <c r="M69" s="3" t="n">
         <v>0</v>
@@ -5605,10 +5605,10 @@
         <v>1605000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2190046</v>
+        <v>2187810</v>
       </c>
       <c r="L71" t="n">
-        <v>26.71386811053284</v>
+        <v>26.63896773485814</v>
       </c>
       <c r="M71" s="3" t="n">
         <v>0</v>
@@ -5669,10 +5669,10 @@
         <v>1610000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2190046</v>
+        <v>2187810</v>
       </c>
       <c r="L72" t="n">
-        <v>26.48556240371207</v>
+        <v>26.41042869353372</v>
       </c>
       <c r="M72" s="3" t="n">
         <v>0</v>
@@ -5733,10 +5733,10 @@
         <v>1615000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2190046</v>
+        <v>2187810</v>
       </c>
       <c r="L73" t="n">
-        <v>26.2572566968913</v>
+        <v>26.18188965220929</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
@@ -5797,10 +5797,10 @@
         <v>1630000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2232996</v>
+        <v>2230716</v>
       </c>
       <c r="L74" t="n">
-        <v>27.00389969350595</v>
+        <v>26.92929086445787</v>
       </c>
       <c r="M74" s="3" t="n">
         <v>0</v>
@@ -5812,7 +5812,7 @@
         <v>100</v>
       </c>
       <c r="Q74" t="n">
-        <v>34.1</v>
+        <v>34</v>
       </c>
       <c r="R74" t="n">
         <v>3</v>
@@ -5861,10 +5861,10 @@
         <v>1690000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2318897</v>
+        <v>2316529</v>
       </c>
       <c r="L75" t="n">
-        <v>27.1205232487687</v>
+        <v>27.0460244615975</v>
       </c>
       <c r="M75" s="3" t="n">
         <v>0</v>
@@ -5876,7 +5876,7 @@
         <v>16.88768606224628</v>
       </c>
       <c r="Q75" t="n">
-        <v>15.7</v>
+        <v>15.6</v>
       </c>
       <c r="R75" t="n">
         <v>3</v>
@@ -5925,10 +5925,10 @@
         <v>1705000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2318897</v>
+        <v>2316529</v>
       </c>
       <c r="L76" t="n">
-        <v>26.4736639876631</v>
+        <v>26.3985039686531</v>
       </c>
       <c r="M76" s="3" t="n">
         <v>0</v>
@@ -5989,10 +5989,10 @@
         <v>1725000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2361848</v>
+        <v>2359436</v>
       </c>
       <c r="L77" t="n">
-        <v>26.96397058574472</v>
+        <v>26.8893074446605</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
@@ -6004,7 +6004,7 @@
         <v>100</v>
       </c>
       <c r="Q77" t="n">
-        <v>34.3</v>
+        <v>34.2</v>
       </c>
       <c r="R77" t="n">
         <v>3</v>
@@ -6053,10 +6053,10 @@
         <v>1780000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2447749</v>
+        <v>2445249</v>
       </c>
       <c r="L78" t="n">
-        <v>27.28012553574733</v>
+        <v>27.205777407536</v>
       </c>
       <c r="M78" s="3" t="n">
         <v>0</v>
@@ -6068,7 +6068,7 @@
         <v>38.78143936249688</v>
       </c>
       <c r="Q78" t="n">
-        <v>21.2</v>
+        <v>21.1</v>
       </c>
       <c r="R78" t="n">
         <v>3</v>
@@ -6117,10 +6117,10 @@
         <v>1875000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2576600</v>
+        <v>2573969</v>
       </c>
       <c r="L79" t="n">
-        <v>27.22968252736164</v>
+        <v>27.1552998501536</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
@@ -6132,7 +6132,7 @@
         <v>19.64044075004835</v>
       </c>
       <c r="Q79" t="n">
-        <v>17.2</v>
+        <v>17.1</v>
       </c>
       <c r="R79" t="n">
         <v>3</v>
@@ -6181,10 +6181,10 @@
         <v>1910000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2619551</v>
+        <v>2616876</v>
       </c>
       <c r="L80" t="n">
-        <v>27.08674120106843</v>
+        <v>27.01220845007559</v>
       </c>
       <c r="M80" s="3" t="n">
         <v>0</v>
@@ -6245,10 +6245,10 @@
         <v>2020000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2748402</v>
+        <v>2745596</v>
       </c>
       <c r="L81" t="n">
-        <v>26.50274595928834</v>
+        <v>26.42763174188774</v>
       </c>
       <c r="M81" s="3" t="n">
         <v>0</v>
@@ -6309,10 +6309,10 @@
         <v>2110000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>2877254</v>
+        <v>2874316</v>
       </c>
       <c r="L82" t="n">
-        <v>26.6661893597159</v>
+        <v>26.59123074846329</v>
       </c>
       <c r="M82" s="3" t="n">
         <v>0</v>
@@ -6373,10 +6373,10 @@
         <v>2210000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3006105</v>
+        <v>3003036</v>
       </c>
       <c r="L83" t="n">
-        <v>26.48294054931548</v>
+        <v>26.40780863099877</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
@@ -6437,10 +6437,10 @@
         <v>2215000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3049056</v>
+        <v>3045942</v>
       </c>
       <c r="L84" t="n">
-        <v>27.35456482268611</v>
+        <v>27.28029621049908</v>
       </c>
       <c r="M84" s="3" t="n">
         <v>0</v>
@@ -6501,10 +6501,10 @@
         <v>2315000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3177907</v>
+        <v>3174662</v>
       </c>
       <c r="L85" t="n">
-        <v>27.15331191252607</v>
+        <v>27.07885122888673</v>
       </c>
       <c r="M85" s="3" t="n">
         <v>0</v>
@@ -6516,7 +6516,7 @@
         <v>65.11105977094954</v>
       </c>
       <c r="Q85" t="n">
-        <v>26.6</v>
+        <v>26.5</v>
       </c>
       <c r="R85" t="n">
         <v>3</v>
@@ -6565,10 +6565,10 @@
         <v>2395000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3306758</v>
+        <v>3303382</v>
       </c>
       <c r="L86" t="n">
-        <v>27.57256503197392</v>
+        <v>27.49854543010769</v>
       </c>
       <c r="M86" s="3" t="n">
         <v>0</v>
@@ -6629,10 +6629,10 @@
         <v>2410000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3306758</v>
+        <v>3303382</v>
       </c>
       <c r="L87" t="n">
-        <v>27.11894852904265</v>
+        <v>27.04446533885575</v>
       </c>
       <c r="M87" s="3" t="n">
         <v>0</v>
@@ -6693,10 +6693,10 @@
         <v>2499000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3435610</v>
+        <v>3432102</v>
       </c>
       <c r="L88" t="n">
-        <v>27.26182541091684</v>
+        <v>27.18747869381504</v>
       </c>
       <c r="M88" s="3" t="n">
         <v>0</v>
@@ -6708,7 +6708,7 @@
         <v>63.67326854471646</v>
       </c>
       <c r="Q88" t="n">
-        <v>26.5</v>
+        <v>26.4</v>
       </c>
       <c r="R88" t="n">
         <v>3</v>
@@ -6757,10 +6757,10 @@
         <v>2510000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3435610</v>
+        <v>3432102</v>
       </c>
       <c r="L89" t="n">
-        <v>26.94164937230943</v>
+        <v>26.8669753987498</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
@@ -6821,10 +6821,10 @@
         <v>2530000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3478560</v>
+        <v>3475009</v>
       </c>
       <c r="L90" t="n">
-        <v>27.26875488707971</v>
+        <v>27.19443316549684</v>
       </c>
       <c r="M90" s="3" t="n">
         <v>0</v>
@@ -6885,10 +6885,10 @@
         <v>2610000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>3607412</v>
+        <v>3603729</v>
       </c>
       <c r="L91" t="n">
-        <v>27.64896274670041</v>
+        <v>27.5750202082343</v>
       </c>
       <c r="M91" s="3" t="n">
         <v>0</v>
@@ -6900,7 +6900,7 @@
         <v>74.15426251691474</v>
       </c>
       <c r="Q91" t="n">
-        <v>28.5</v>
+        <v>28.4</v>
       </c>
       <c r="R91" t="n">
         <v>3</v>
@@ -6949,10 +6949,10 @@
         <v>3015000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4165768</v>
+        <v>4161515</v>
       </c>
       <c r="L92" t="n">
-        <v>27.62439002844134</v>
+        <v>27.55042334342181</v>
       </c>
       <c r="M92" s="3" t="n">
         <v>0</v>
@@ -7013,10 +7013,10 @@
         <v>3098000</v>
       </c>
       <c r="K93" s="3" t="n">
-        <v>4294620</v>
+        <v>4290235</v>
       </c>
       <c r="L93" t="n">
-        <v>27.86323353404958</v>
+        <v>27.7895033721929</v>
       </c>
       <c r="M93" s="3" t="n">
         <v>0</v>
@@ -7028,7 +7028,7 @@
         <v>100</v>
       </c>
       <c r="Q93" t="n">
-        <v>34.4</v>
+        <v>34.3</v>
       </c>
       <c r="R93" t="n">
         <v>3</v>
@@ -7312,10 +7312,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>429075</v>
+        <v>428637</v>
       </c>
       <c r="L2" t="n">
-        <v>27.75179164481734</v>
+        <v>27.67796527131349</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7379,10 +7379,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>429075</v>
+        <v>428637</v>
       </c>
       <c r="L3" t="n">
-        <v>27.75179164481734</v>
+        <v>27.67796527131349</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7446,10 +7446,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>429075</v>
+        <v>428637</v>
       </c>
       <c r="L4" t="n">
-        <v>27.7515585853289</v>
+        <v>27.6777319736747</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7513,10 +7513,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>429075</v>
+        <v>428637</v>
       </c>
       <c r="L5" t="n">
-        <v>27.7515585853289</v>
+        <v>27.6777319736747</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7580,10 +7580,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514976</v>
+        <v>514451</v>
       </c>
       <c r="L6" t="n">
-        <v>25.43341825638477</v>
+        <v>25.35732266046718</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7644,10 +7644,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>514976</v>
+        <v>514451</v>
       </c>
       <c r="L7" t="n">
-        <v>25.43341825638477</v>
+        <v>25.35732266046718</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7708,10 +7708,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>514976</v>
+        <v>514451</v>
       </c>
       <c r="L8" t="n">
-        <v>25.43341825638477</v>
+        <v>25.35732266046718</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7772,10 +7772,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>514976</v>
+        <v>514451</v>
       </c>
       <c r="L9" t="n">
-        <v>25.43341825638477</v>
+        <v>25.35732266046718</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7836,10 +7836,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>514976</v>
+        <v>514451</v>
       </c>
       <c r="L10" t="n">
-        <v>25.23923444976077</v>
+        <v>25.16294068822881</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7900,10 +7900,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>514976</v>
+        <v>514451</v>
       </c>
       <c r="L11" t="n">
-        <v>25.23923444976077</v>
+        <v>25.16294068822881</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7964,10 +7964,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>514976</v>
+        <v>514451</v>
       </c>
       <c r="L12" t="n">
-        <v>25.23923444976077</v>
+        <v>25.16294068822881</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -8028,10 +8028,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>514976</v>
+        <v>514451</v>
       </c>
       <c r="L13" t="n">
-        <v>25.23923444976077</v>
+        <v>25.16294068822881</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -8092,10 +8092,10 @@
         <v>420000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>557927</v>
+        <v>557357</v>
       </c>
       <c r="L14" t="n">
-        <v>24.72133451150419</v>
+        <v>24.64434823640862</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -8159,10 +8159,10 @@
         <v>420000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>557927</v>
+        <v>557357</v>
       </c>
       <c r="L15" t="n">
-        <v>24.72133451150419</v>
+        <v>24.64434823640862</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0</v>
@@ -8177,7 +8177,7 @@
         <v>3.361344537815107</v>
       </c>
       <c r="Q15" t="n">
-        <v>31.9</v>
+        <v>31.8</v>
       </c>
       <c r="R15" t="n">
         <v>4</v>
@@ -8226,10 +8226,10 @@
         <v>420000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>557927</v>
+        <v>557357</v>
       </c>
       <c r="L16" t="n">
-        <v>24.72133451150419</v>
+        <v>24.64434823640862</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -8244,7 +8244,7 @@
         <v>3.361344537815107</v>
       </c>
       <c r="Q16" t="n">
-        <v>31.7</v>
+        <v>31.6</v>
       </c>
       <c r="R16" t="n">
         <v>4</v>
@@ -8293,10 +8293,10 @@
         <v>425000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>557927</v>
+        <v>557357</v>
       </c>
       <c r="L17" t="n">
-        <v>23.82515992235543</v>
+        <v>23.74725714398491</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -8311,7 +8311,7 @@
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>9.1</v>
+        <v>9</v>
       </c>
       <c r="R17" t="n">
         <v>4</v>
@@ -8360,10 +8360,10 @@
         <v>454000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>600877</v>
+        <v>600264</v>
       </c>
       <c r="L18" t="n">
-        <v>24.44377135420394</v>
+        <v>24.36661202404276</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -8375,7 +8375,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q18" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="R18" t="n">
         <v>3</v>
@@ -8424,10 +8424,10 @@
         <v>454000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>600877</v>
+        <v>600264</v>
       </c>
       <c r="L19" t="n">
-        <v>24.44377135420394</v>
+        <v>24.36661202404276</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -8439,7 +8439,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q19" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="R19" t="n">
         <v>3</v>
@@ -8488,10 +8488,10 @@
         <v>454000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>600877</v>
+        <v>600264</v>
       </c>
       <c r="L20" t="n">
-        <v>24.44377135420394</v>
+        <v>24.36661202404276</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -8503,7 +8503,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q20" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="R20" t="n">
         <v>3</v>
@@ -8552,10 +8552,10 @@
         <v>454000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>600877</v>
+        <v>600264</v>
       </c>
       <c r="L21" t="n">
-        <v>24.44377135420394</v>
+        <v>24.36661202404276</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -8567,7 +8567,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q21" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="R21" t="n">
         <v>3</v>
@@ -8616,10 +8616,10 @@
         <v>455000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>600877</v>
+        <v>600264</v>
       </c>
       <c r="L22" t="n">
-        <v>24.27734794308985</v>
+        <v>24.20001865845694</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -8680,10 +8680,10 @@
         <v>455000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>600877</v>
+        <v>600264</v>
       </c>
       <c r="L23" t="n">
-        <v>24.27734794308985</v>
+        <v>24.20001865845694</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -8744,10 +8744,10 @@
         <v>455000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>600877</v>
+        <v>600264</v>
       </c>
       <c r="L24" t="n">
-        <v>24.27734794308985</v>
+        <v>24.20001865845694</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -8808,10 +8808,10 @@
         <v>455000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>600877</v>
+        <v>600264</v>
       </c>
       <c r="L25" t="n">
-        <v>24.27734794308985</v>
+        <v>24.20001865845694</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -8872,10 +8872,10 @@
         <v>475000</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>686778</v>
+        <v>686077</v>
       </c>
       <c r="L26" t="n">
-        <v>30.83645661334521</v>
+        <v>30.7657886796963</v>
       </c>
       <c r="M26" s="3" t="n">
         <v>0</v>
@@ -8936,10 +8936,10 @@
         <v>475000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>686778</v>
+        <v>686077</v>
       </c>
       <c r="L27" t="n">
-        <v>30.83645661334521</v>
+        <v>30.7657886796963</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -9000,10 +9000,10 @@
         <v>475000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>686778</v>
+        <v>686077</v>
       </c>
       <c r="L28" t="n">
-        <v>30.83645661334521</v>
+        <v>30.7657886796963</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -9064,10 +9064,10 @@
         <v>475000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>686778</v>
+        <v>686077</v>
       </c>
       <c r="L29" t="n">
-        <v>30.83645661334521</v>
+        <v>30.7657886796963</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -9128,10 +9128,10 @@
         <v>477000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>643828</v>
+        <v>643171</v>
       </c>
       <c r="L30" t="n">
-        <v>25.91188951086315</v>
+        <v>25.83620841113794</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -9146,7 +9146,7 @@
         <v>1.568112774445864</v>
       </c>
       <c r="Q30" t="n">
-        <v>31.5</v>
+        <v>31.4</v>
       </c>
       <c r="R30" t="n">
         <v>4</v>
@@ -9195,10 +9195,10 @@
         <v>477000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>643828</v>
+        <v>643171</v>
       </c>
       <c r="L31" t="n">
-        <v>25.91188951086315</v>
+        <v>25.83620841113794</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -9213,7 +9213,7 @@
         <v>1.568112774445864</v>
       </c>
       <c r="Q31" t="n">
-        <v>31.5</v>
+        <v>31.4</v>
       </c>
       <c r="R31" t="n">
         <v>4</v>
@@ -9262,10 +9262,10 @@
         <v>477000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>643828</v>
+        <v>643171</v>
       </c>
       <c r="L32" t="n">
-        <v>25.91188951086315</v>
+        <v>25.83620841113794</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -9280,7 +9280,7 @@
         <v>1.568112774445864</v>
       </c>
       <c r="Q32" t="n">
-        <v>31.5</v>
+        <v>31.4</v>
       </c>
       <c r="R32" t="n">
         <v>4</v>
@@ -9329,10 +9329,10 @@
         <v>479999</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>686778</v>
+        <v>686077</v>
       </c>
       <c r="L33" t="n">
-        <v>30.10856492199808</v>
+        <v>30.03715326413799</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -9344,7 +9344,7 @@
         <v>43.6979831932773</v>
       </c>
       <c r="Q33" t="n">
-        <v>22.3</v>
+        <v>22.2</v>
       </c>
       <c r="R33" t="n">
         <v>3</v>
@@ -9393,10 +9393,10 @@
         <v>479999</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>686778</v>
+        <v>686077</v>
       </c>
       <c r="L34" t="n">
-        <v>30.10856492199808</v>
+        <v>30.03715326413799</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -9408,7 +9408,7 @@
         <v>43.6979831932773</v>
       </c>
       <c r="Q34" t="n">
-        <v>22.3</v>
+        <v>22.2</v>
       </c>
       <c r="R34" t="n">
         <v>3</v>
@@ -9457,10 +9457,10 @@
         <v>479999</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>686778</v>
+        <v>686077</v>
       </c>
       <c r="L35" t="n">
-        <v>30.10856492199808</v>
+        <v>30.03715326413799</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
@@ -9472,7 +9472,7 @@
         <v>43.6979831932773</v>
       </c>
       <c r="Q35" t="n">
-        <v>22.3</v>
+        <v>22.2</v>
       </c>
       <c r="R35" t="n">
         <v>3</v>
@@ -9521,10 +9521,10 @@
         <v>479999</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>686778</v>
+        <v>686077</v>
       </c>
       <c r="L36" t="n">
-        <v>30.10856492199808</v>
+        <v>30.03715326413799</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -9536,7 +9536,7 @@
         <v>43.6979831932773</v>
       </c>
       <c r="Q36" t="n">
-        <v>22.3</v>
+        <v>22.2</v>
       </c>
       <c r="R36" t="n">
         <v>3</v>
@@ -9585,10 +9585,10 @@
         <v>479999</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>643828</v>
+        <v>643171</v>
       </c>
       <c r="L37" t="n">
-        <v>25.44608187279833</v>
+        <v>25.36992494997443</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
@@ -9652,10 +9652,10 @@
         <v>500000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>643828</v>
+        <v>643171</v>
       </c>
       <c r="L38" t="n">
-        <v>22.33950682480414</v>
+        <v>22.26017653159113</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -9667,7 +9667,7 @@
         <v>33.61344537815125</v>
       </c>
       <c r="Q38" t="n">
-        <v>16.8</v>
+        <v>16.7</v>
       </c>
       <c r="R38" t="n">
         <v>3</v>
@@ -9716,10 +9716,10 @@
         <v>547999</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>772679</v>
+        <v>771890</v>
       </c>
       <c r="L39" t="n">
-        <v>29.0780518171194</v>
+        <v>29.00555778673127</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -9731,7 +9731,7 @@
         <v>64.67267226890753</v>
       </c>
       <c r="Q39" t="n">
-        <v>26.6</v>
+        <v>26.5</v>
       </c>
       <c r="R39" t="n">
         <v>3</v>
@@ -9780,10 +9780,10 @@
         <v>547999</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>772679</v>
+        <v>771890</v>
       </c>
       <c r="L40" t="n">
-        <v>29.0780518171194</v>
+        <v>29.00555778673127</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -9795,7 +9795,7 @@
         <v>64.67267226890753</v>
       </c>
       <c r="Q40" t="n">
-        <v>26.6</v>
+        <v>26.5</v>
       </c>
       <c r="R40" t="n">
         <v>3</v>
@@ -9844,10 +9844,10 @@
         <v>547999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>772679</v>
+        <v>771890</v>
       </c>
       <c r="L41" t="n">
-        <v>29.0780518171194</v>
+        <v>29.00555778673127</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
@@ -9859,7 +9859,7 @@
         <v>64.67267226890753</v>
       </c>
       <c r="Q41" t="n">
-        <v>27</v>
+        <v>26.9</v>
       </c>
       <c r="R41" t="n">
         <v>3</v>
@@ -9908,10 +9908,10 @@
         <v>547999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>772679</v>
+        <v>771890</v>
       </c>
       <c r="L42" t="n">
-        <v>29.0780518171194</v>
+        <v>29.00555778673127</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -9923,7 +9923,7 @@
         <v>64.67267226890753</v>
       </c>
       <c r="Q42" t="n">
-        <v>26.6</v>
+        <v>26.5</v>
       </c>
       <c r="R42" t="n">
         <v>3</v>
@@ -9972,10 +9972,10 @@
         <v>552999</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>772679</v>
+        <v>771890</v>
       </c>
       <c r="L43" t="n">
-        <v>28.43095256891931</v>
+        <v>28.35779709544106</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -9987,7 +9987,7 @@
         <v>34.11769473304435</v>
       </c>
       <c r="Q43" t="n">
-        <v>20.3</v>
+        <v>20.2</v>
       </c>
       <c r="R43" t="n">
         <v>3</v>
@@ -10036,10 +10036,10 @@
         <v>552999</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>772679</v>
+        <v>771890</v>
       </c>
       <c r="L44" t="n">
-        <v>28.43095256891931</v>
+        <v>28.35779709544106</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -10051,7 +10051,7 @@
         <v>34.11769473304435</v>
       </c>
       <c r="Q44" t="n">
-        <v>20.3</v>
+        <v>20.2</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -10100,10 +10100,10 @@
         <v>552999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>772679</v>
+        <v>771890</v>
       </c>
       <c r="L45" t="n">
-        <v>28.43095256891931</v>
+        <v>28.35779709544106</v>
       </c>
       <c r="M45" s="3" t="n">
         <v>0</v>
@@ -10115,7 +10115,7 @@
         <v>34.11769473304435</v>
       </c>
       <c r="Q45" t="n">
-        <v>20.3</v>
+        <v>20.2</v>
       </c>
       <c r="R45" t="n">
         <v>3</v>
@@ -10164,10 +10164,10 @@
         <v>552999</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>772679</v>
+        <v>771890</v>
       </c>
       <c r="L46" t="n">
-        <v>28.43095256891931</v>
+        <v>28.35779709544106</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -10179,7 +10179,7 @@
         <v>34.11769473304435</v>
       </c>
       <c r="Q46" t="n">
-        <v>20.3</v>
+        <v>20.2</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -10228,10 +10228,10 @@
         <v>585000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>729729</v>
+        <v>728984</v>
       </c>
       <c r="L47" t="n">
-        <v>19.8332531665865</v>
+        <v>19.75132513196449</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -10292,10 +10292,10 @@
         <v>595000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>729729</v>
+        <v>728984</v>
       </c>
       <c r="L48" t="n">
-        <v>18.46288142584439</v>
+        <v>18.37955291199807</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -10356,10 +10356,10 @@
         <v>614999</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>858580</v>
+        <v>857704</v>
       </c>
       <c r="L49" t="n">
-        <v>28.37021593794405</v>
+        <v>28.29705819256993</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -10420,10 +10420,10 @@
         <v>614999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>858580</v>
+        <v>857704</v>
       </c>
       <c r="L50" t="n">
-        <v>28.37021593794405</v>
+        <v>28.29705819256993</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -10484,10 +10484,10 @@
         <v>614999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>858580</v>
+        <v>857704</v>
       </c>
       <c r="L51" t="n">
-        <v>28.37021593794405</v>
+        <v>28.29705819256993</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -10548,10 +10548,10 @@
         <v>614999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>858580</v>
+        <v>857704</v>
       </c>
       <c r="L52" t="n">
-        <v>28.37021593794405</v>
+        <v>28.29705819256993</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -10612,10 +10612,10 @@
         <v>650000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>815630</v>
+        <v>814797</v>
       </c>
       <c r="L53" t="n">
-        <v>20.30700194941334</v>
+        <v>20.22552856723822</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -10676,10 +10676,10 @@
         <v>672000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>858580</v>
+        <v>857704</v>
       </c>
       <c r="L54" t="n">
-        <v>21.73123063663258</v>
+        <v>21.6512922873159</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -10740,10 +10740,10 @@
         <v>700000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>901531</v>
+        <v>900610</v>
       </c>
       <c r="L55" t="n">
-        <v>22.35430617471834</v>
+        <v>22.27490256603857</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -10804,10 +10804,10 @@
         <v>715000</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>944481</v>
+        <v>943517</v>
       </c>
       <c r="L56" t="n">
-        <v>24.29704779662058</v>
+        <v>24.21970139382756</v>
       </c>
       <c r="M56" s="3" t="n">
         <v>0</v>
@@ -10868,10 +10868,10 @@
         <v>734999</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>987432</v>
+        <v>986424</v>
       </c>
       <c r="L57" t="n">
-        <v>25.5645958405237</v>
+        <v>25.48853231470443</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -10932,10 +10932,10 @@
         <v>752000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>987432</v>
+        <v>986424</v>
       </c>
       <c r="L58" t="n">
-        <v>23.8428570271168</v>
+        <v>23.76503410298209</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -10947,7 +10947,7 @@
         <v>54.37884642534079</v>
       </c>
       <c r="Q58" t="n">
-        <v>21.9</v>
+        <v>21.8</v>
       </c>
       <c r="R58" t="n">
         <v>3</v>
@@ -10996,10 +10996,10 @@
         <v>810000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1073333</v>
+        <v>1072237</v>
       </c>
       <c r="L59" t="n">
-        <v>24.53413805408014</v>
+        <v>24.45699971181744</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -11060,10 +11060,10 @@
         <v>815000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1073333</v>
+        <v>1072237</v>
       </c>
       <c r="L60" t="n">
-        <v>24.06829940009298</v>
+        <v>23.99068489522372</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -11124,10 +11124,10 @@
         <v>875000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1159234</v>
+        <v>1158050</v>
       </c>
       <c r="L61" t="n">
-        <v>24.51912210994502</v>
+        <v>24.44194982945469</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -11188,10 +11188,10 @@
         <v>992000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1331036</v>
+        <v>1329677</v>
       </c>
       <c r="L62" t="n">
-        <v>25.47158754534063</v>
+        <v>25.39541557836979</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -11203,7 +11203,7 @@
         <v>85.64705882352939</v>
       </c>
       <c r="Q62" t="n">
-        <v>29.3</v>
+        <v>29.2</v>
       </c>
       <c r="R62" t="n">
         <v>3</v>
@@ -11252,10 +11252,10 @@
         <v>1050000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1416937</v>
+        <v>1415490</v>
       </c>
       <c r="L63" t="n">
-        <v>25.89649363380305</v>
+        <v>25.82074052095034</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -11267,7 +11267,7 @@
         <v>93.20091673032849</v>
       </c>
       <c r="Q63" t="n">
-        <v>31.1</v>
+        <v>31</v>
       </c>
       <c r="R63" t="n">
         <v>3</v>
@@ -11316,10 +11316,10 @@
         <v>1050000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1416937</v>
+        <v>1415490</v>
       </c>
       <c r="L64" t="n">
-        <v>25.89649363380305</v>
+        <v>25.82074052095034</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -11380,10 +11380,10 @@
         <v>1100000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1502838</v>
+        <v>1501303</v>
       </c>
       <c r="L65" t="n">
-        <v>26.80515132036853</v>
+        <v>26.73031360091867</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -11395,7 +11395,7 @@
         <v>94.11761630126171</v>
       </c>
       <c r="Q65" t="n">
-        <v>31.7</v>
+        <v>31.6</v>
       </c>
       <c r="R65" t="n">
         <v>3</v>
@@ -11444,10 +11444,10 @@
         <v>1105000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1502838</v>
+        <v>1501303</v>
       </c>
       <c r="L66" t="n">
-        <v>26.47244746273384</v>
+        <v>26.39726957183193</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -11459,7 +11459,7 @@
         <v>100</v>
       </c>
       <c r="Q66" t="n">
-        <v>32.8</v>
+        <v>32.7</v>
       </c>
       <c r="R66" t="n">
         <v>3</v>
@@ -11508,10 +11508,10 @@
         <v>1155000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1588739</v>
+        <v>1587117</v>
       </c>
       <c r="L67" t="n">
-        <v>27.30083418358837</v>
+        <v>27.22653717400797</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -11778,7 +11778,7 @@
         <v>315000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>300224</v>
+        <v>299917</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -11839,10 +11839,10 @@
         <v>380000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>386125</v>
+        <v>385731</v>
       </c>
       <c r="L3" t="n">
-        <v>1.586273875040466</v>
+        <v>1.485750432296082</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -11903,7 +11903,7 @@
         <v>415000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>386125</v>
+        <v>385731</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -11964,10 +11964,10 @@
         <v>495000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>472026</v>
+        <v>471544</v>
       </c>
       <c r="L5" t="n">
-        <v>6.785007605513256</v>
+        <v>6.689725667169978</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -12028,10 +12028,10 @@
         <v>490000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514976</v>
+        <v>514451</v>
       </c>
       <c r="L6" t="n">
-        <v>4.849934754240974</v>
+        <v>4.752833603200305</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -12043,7 +12043,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="R6" t="n">
         <v>3</v>
@@ -12092,10 +12092,10 @@
         <v>550000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>557927</v>
+        <v>557357</v>
       </c>
       <c r="L7" t="n">
-        <v>6.797842728529001</v>
+        <v>6.702526387934483</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -12156,7 +12156,7 @@
         <v>530000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>472026</v>
+        <v>471544</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -12220,10 +12220,10 @@
         <v>600000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>600877</v>
+        <v>600264</v>
       </c>
       <c r="L9" t="n">
-        <v>8.467123887251466</v>
+        <v>8.3736489278051</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -12284,10 +12284,10 @@
         <v>646000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>729729</v>
+        <v>728984</v>
       </c>
       <c r="L10" t="n">
-        <v>17.09264672227635</v>
+        <v>17.00791786925365</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -12299,7 +12299,7 @@
         <v>100</v>
       </c>
       <c r="Q10" t="n">
-        <v>26</v>
+        <v>25.9</v>
       </c>
       <c r="R10" t="n">
         <v>4</v>
@@ -12348,7 +12348,7 @@
         <v>615000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>557927</v>
+        <v>557357</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -12412,7 +12412,7 @@
         <v>700000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>643828</v>
+        <v>643171</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -12476,7 +12476,7 @@
         <v>745000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>686778</v>
+        <v>686077</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -12540,7 +12540,7 @@
         <v>930000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>858580</v>
+        <v>857704</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -12611,7 +12611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12657,8 +12657,64 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Macbook Pro 14 M5 MDE34 10 Core CPU 10 Core GPU 24GB 1TB Space Black</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>643999</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>644999</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Macbook Pro 14 M5 MJ3D4 10 Core CPU 10 Core GPU 32GB 1TB Space Black</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>775000</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>780000</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.65</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F1"/>
+  <autoFilter ref="A1:F3"/>
+  <conditionalFormatting sqref="E2:E3">
+    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: price data 2026-10-04
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MacBook Pro'!$A$1:$S$93</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MacBook Air'!$A$1:$S$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20261003T091351304003+0000</t>
+          <t>20261004T095228889941+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-03T09:13:51.304003+00:00</t>
+          <t>2026-10-04T09:52:28.889941+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>276.817029</v>
+        <v>276.834776</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -624,7 +624,7 @@
         <v>1445000</v>
       </c>
       <c r="D17" t="n">
-        <v>59.1</v>
+        <v>58.5</v>
       </c>
       <c r="E17" t="n">
         <v>3</v>
@@ -633,7 +633,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 48GB 2TB Space Black</t>
+          <t>Macbook Pro 14 MJLV4 M5 Pro 15 Core CPU 16 Core GPU 24GB 2TB Silver</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -642,10 +642,10 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>1155000</v>
+        <v>775000</v>
       </c>
       <c r="D18" t="n">
-        <v>54.6</v>
+        <v>57.4</v>
       </c>
       <c r="E18" t="n">
         <v>3</v>
@@ -663,10 +663,10 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>790000</v>
+        <v>775000</v>
       </c>
       <c r="D19" t="n">
-        <v>54.6</v>
+        <v>56.1</v>
       </c>
       <c r="E19" t="n">
         <v>3</v>
@@ -675,7 +675,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 24GB 4TB Silver</t>
+          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 48GB 2TB Space Black</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -684,10 +684,10 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>1260000</v>
+        <v>1155000</v>
       </c>
       <c r="D20" t="n">
-        <v>54</v>
+        <v>54.1</v>
       </c>
       <c r="E20" t="n">
         <v>3</v>
@@ -696,7 +696,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 48GB 1TB Space Black</t>
+          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 24GB 4TB Silver</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -705,10 +705,10 @@
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>995000</v>
+        <v>1260000</v>
       </c>
       <c r="D21" t="n">
-        <v>51.7</v>
+        <v>54</v>
       </c>
       <c r="E21" t="n">
         <v>3</v>
@@ -738,7 +738,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 16Inch MX2U3 14Core CPU 20Core GPU M4 Pro 48GB 512GB Silver</t>
+          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 48GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -747,19 +747,19 @@
         </is>
       </c>
       <c r="C23" s="3" t="n">
-        <v>810000</v>
+        <v>995000</v>
       </c>
       <c r="D23" t="n">
-        <v>50.5</v>
+        <v>51.2</v>
       </c>
       <c r="E23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 16Inch MX2W3 16Core CPU 40Core GPU M4 Max  48GB 1TB Silver</t>
+          <t>Apple MacBook Pro 16Inch MX2U3 14Core CPU 20Core GPU M4 Pro 48GB 512GB Silver</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -768,10 +768,10 @@
         </is>
       </c>
       <c r="C24" s="3" t="n">
-        <v>1123000</v>
+        <v>810000</v>
       </c>
       <c r="D24" t="n">
-        <v>50.4</v>
+        <v>50.5</v>
       </c>
       <c r="E24" t="n">
         <v>4</v>
@@ -780,7 +780,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 14Inch MX2J3 M4 Pro 14Core CPU 20Core GPU 24GB 1TB Space Black</t>
+          <t>Apple MacBook Pro 16Inch MX2W3 16Core CPU 40Core GPU M4 Max  48GB 1TB Silver</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -789,10 +789,10 @@
         </is>
       </c>
       <c r="C25" s="3" t="n">
-        <v>700000</v>
+        <v>1123000</v>
       </c>
       <c r="D25" t="n">
-        <v>49.6</v>
+        <v>50.4</v>
       </c>
       <c r="E25" t="n">
         <v>4</v>
@@ -801,7 +801,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 14Inch MX2K3 14Core CPU 32Core GPU M4 Max 36GB 1TB Space Black</t>
+          <t>Apple MacBook Pro 14Inch MX2J3 M4 Pro 14Core CPU 20Core GPU 24GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -810,19 +810,19 @@
         </is>
       </c>
       <c r="C26" s="3" t="n">
-        <v>847999</v>
+        <v>700000</v>
       </c>
       <c r="D26" t="n">
-        <v>47.3</v>
+        <v>49.6</v>
       </c>
       <c r="E26" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 MDE34 10 Core CPU 10 Core GPU 24GB 1TB Space Black</t>
+          <t>Apple MacBook Pro 14Inch MX2K3 14Core CPU 32Core GPU M4 Max 36GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -831,19 +831,19 @@
         </is>
       </c>
       <c r="C27" s="3" t="n">
-        <v>644999</v>
+        <v>847999</v>
       </c>
       <c r="D27" t="n">
-        <v>44.3</v>
+        <v>47.3</v>
       </c>
       <c r="E27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 MGDR4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Space Black</t>
+          <t>Macbook Pro 14 M5 MDE34 10 Core CPU 10 Core GPU 24GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -852,19 +852,19 @@
         </is>
       </c>
       <c r="C28" s="3" t="n">
-        <v>720000</v>
+        <v>644999</v>
       </c>
       <c r="D28" t="n">
-        <v>44.2</v>
+        <v>44.3</v>
       </c>
       <c r="E28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 MJLV4 M5 Pro 15 Core CPU 16 Core GPU 24GB 2TB Silver</t>
+          <t>Macbook Pro 14 MGDR4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -873,10 +873,10 @@
         </is>
       </c>
       <c r="C29" s="3" t="n">
-        <v>815000</v>
+        <v>720000</v>
       </c>
       <c r="D29" t="n">
-        <v>43.6</v>
+        <v>44.2</v>
       </c>
       <c r="E29" t="n">
         <v>3</v>
@@ -906,7 +906,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 32GB 1TB Space Black</t>
+          <t>Macbook Pro 14 M5 MJ3E4 10 Core CPU 10 Core GPU 32GB 1TB Silver</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -915,10 +915,10 @@
         </is>
       </c>
       <c r="C31" s="3" t="n">
-        <v>772000</v>
+        <v>769999</v>
       </c>
       <c r="D31" t="n">
-        <v>42.2</v>
+        <v>42.4</v>
       </c>
       <c r="E31" t="n">
         <v>4</v>
@@ -1147,10 +1147,10 @@
         <v>470000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>686077</v>
+        <v>686121</v>
       </c>
       <c r="L2" t="n">
-        <v>35.13847571045233</v>
+        <v>35.1426351911689</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1214,10 +1214,10 @@
         <v>495000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>686077</v>
+        <v>686121</v>
       </c>
       <c r="L3" t="n">
-        <v>27.85066399252562</v>
+        <v>27.85529083062609</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>771890</v>
+        <v>771940</v>
       </c>
       <c r="L4" t="n">
-        <v>35.22406042311728</v>
+        <v>35.22825608207892</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>771890</v>
+        <v>771940</v>
       </c>
       <c r="L5" t="n">
-        <v>32.63301765795644</v>
+        <v>32.6373811436122</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>857704</v>
+        <v>857759</v>
       </c>
       <c r="L6" t="n">
-        <v>37.97393972745842</v>
+        <v>37.97791687408701</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1606,10 +1606,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>857704</v>
+        <v>857759</v>
       </c>
       <c r="L9" t="n">
-        <v>34.12645854513912</v>
+        <v>34.1306823944721</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1673,10 +1673,10 @@
         <v>579999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>857704</v>
+        <v>857759</v>
       </c>
       <c r="L10" t="n">
-        <v>32.37772005260556</v>
+        <v>32.38205603205562</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -1740,10 +1740,10 @@
         <v>587999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>857704</v>
+        <v>857759</v>
       </c>
       <c r="L11" t="n">
-        <v>31.44499734174027</v>
+        <v>31.44939312790655</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -1807,10 +1807,10 @@
         <v>600000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>857704</v>
+        <v>857759</v>
       </c>
       <c r="L12" t="n">
-        <v>30.04579668510349</v>
+        <v>30.05028218881994</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -1874,10 +1874,10 @@
         <v>634000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>857704</v>
+        <v>857759</v>
       </c>
       <c r="L13" t="n">
-        <v>26.08172516392602</v>
+        <v>26.0864648461864</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -1941,13 +1941,13 @@
         <v>644999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>943517</v>
+        <v>943577</v>
       </c>
       <c r="L14" t="n">
-        <v>31.63885759345089</v>
+        <v>31.64320452914812</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="N14" t="n">
         <v>0</v>
@@ -2067,10 +2067,10 @@
         <v>650000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>943517</v>
+        <v>943577</v>
       </c>
       <c r="L16" t="n">
-        <v>31.10881944893415</v>
+        <v>31.11320008859903</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -2134,10 +2134,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1029330</v>
+        <v>1029396</v>
       </c>
       <c r="L17" t="n">
-        <v>31.99459842810371</v>
+        <v>31.99895861262332</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2201,10 +2201,10 @@
         <v>711999</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>1072237</v>
+        <v>1072306</v>
       </c>
       <c r="L18" t="n">
-        <v>33.59686338001767</v>
+        <v>33.60113624282621</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -2330,10 +2330,10 @@
         <v>720000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>1029330</v>
+        <v>1029396</v>
       </c>
       <c r="L20" t="n">
-        <v>30.05158695462097</v>
+        <v>30.05607171584113</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -2459,10 +2459,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1072237</v>
+        <v>1072306</v>
       </c>
       <c r="L22" t="n">
-        <v>30.70561825417328</v>
+        <v>30.71007716081044</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2491,7 +2491,7 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 32GB 1TB Space Black</t>
+          <t>Macbook Pro 14 M5 MJ3E4 10 Core CPU 10 Core GPU 32GB 1TB Silver</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -2516,35 +2516,35 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I23" s="3" t="n">
-        <v>772000</v>
+        <v>769999</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>772000</v>
+        <v>769999</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1029330</v>
+        <v>1029396</v>
       </c>
       <c r="L23" t="n">
-        <v>24.99975712356581</v>
+        <v>25.1989516182305</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>0</v>
+        <v>-5001</v>
       </c>
       <c r="N23" t="n">
-        <v>0</v>
+        <v>0.2591968911917099</v>
       </c>
       <c r="O23" t="n">
         <v>100</v>
       </c>
       <c r="P23" t="n">
-        <v>69.59999999999998</v>
+        <v>70.00019999999999</v>
       </c>
       <c r="Q23" t="n">
-        <v>42.2</v>
+        <v>42.4</v>
       </c>
       <c r="R23" t="n">
         <v>4</v>
@@ -2558,7 +2558,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 MJ3E4 10 Core CPU 10 Core GPU 32GB 1TB Silver</t>
+          <t>Macbook Pro 14 M5 MJ3D4 10 Core CPU 10 Core GPU 32GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -2583,35 +2583,35 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I24" s="3" t="n">
-        <v>775000</v>
+        <v>769999</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>775000</v>
+        <v>769999</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1029330</v>
+        <v>1029396</v>
       </c>
       <c r="L24" t="n">
-        <v>24.7083054025434</v>
+        <v>25.1989516182305</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>0</v>
+        <v>-10001</v>
       </c>
       <c r="N24" t="n">
-        <v>0</v>
+        <v>0.2591968911917099</v>
       </c>
       <c r="O24" t="n">
-        <v>62.5</v>
+        <v>100</v>
       </c>
       <c r="P24" t="n">
-        <v>68.99999999999999</v>
+        <v>70.00019999999999</v>
       </c>
       <c r="Q24" t="n">
-        <v>33.6</v>
+        <v>42.4</v>
       </c>
       <c r="R24" t="n">
         <v>4</v>
@@ -2625,7 +2625,7 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 MJ3D4 10 Core CPU 10 Core GPU 32GB 1TB Space Black</t>
+          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 32GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -2654,19 +2654,19 @@
         </is>
       </c>
       <c r="I25" s="3" t="n">
-        <v>780000</v>
+        <v>772000</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>780000</v>
+        <v>772000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>1029330</v>
+        <v>1029396</v>
       </c>
       <c r="L25" t="n">
-        <v>24.22255253417271</v>
+        <v>25.00456578420744</v>
       </c>
       <c r="M25" s="3" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="N25" t="n">
         <v>0</v>
@@ -2675,10 +2675,10 @@
         <v>0</v>
       </c>
       <c r="P25" t="n">
-        <v>68</v>
+        <v>69.59999999999998</v>
       </c>
       <c r="Q25" t="n">
-        <v>19.4</v>
+        <v>19.9</v>
       </c>
       <c r="R25" t="n">
         <v>4</v>
@@ -2721,26 +2721,26 @@
         </is>
       </c>
       <c r="I26" s="3" t="n">
-        <v>790000</v>
+        <v>775000</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>790000</v>
+        <v>775000</v>
       </c>
       <c r="K26" s="3" t="n"/>
       <c r="M26" s="3" t="n">
-        <v>0</v>
+        <v>-15000</v>
       </c>
       <c r="N26" t="n">
-        <v>0</v>
+        <v>1.89873417721519</v>
       </c>
       <c r="O26" t="n">
         <v>100</v>
       </c>
       <c r="P26" t="n">
-        <v>84.98168498168498</v>
+        <v>87.91208791208793</v>
       </c>
       <c r="Q26" t="n">
-        <v>54.6</v>
+        <v>56.1</v>
       </c>
       <c r="R26" t="n">
         <v>3</v>
@@ -2754,7 +2754,7 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 16GB 2TB Space Black</t>
+          <t>Macbook Pro 14 MJLV4 M5 Pro 15 Core CPU 16 Core GPU 24GB 2TB Silver</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -2762,49 +2762,47 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M5 Pro</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E27" t="n">
         <v>2048</v>
       </c>
       <c r="F27" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G27" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I27" s="3" t="n">
-        <v>810000</v>
+        <v>775000</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>810000</v>
-      </c>
-      <c r="K27" s="3" t="n">
-        <v>1072237</v>
-      </c>
-      <c r="L27" t="n">
-        <v>24.45699971181744</v>
-      </c>
+        <v>775000</v>
+      </c>
+      <c r="K27" s="3" t="n"/>
       <c r="M27" s="3" t="n">
-        <v>0</v>
+        <v>-40000</v>
       </c>
       <c r="N27" t="n">
-        <v>2.994011976047904</v>
+        <v>4.907975460122699</v>
+      </c>
+      <c r="O27" t="n">
+        <v>100</v>
       </c>
       <c r="P27" t="n">
-        <v>61.99999999999999</v>
+        <v>87.91208791208793</v>
       </c>
       <c r="Q27" t="n">
-        <v>24.8</v>
+        <v>57.4</v>
       </c>
       <c r="R27" t="n">
         <v>3</v>
@@ -2818,32 +2816,32 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 16Inch MX2U3 14Core CPU 20Core GPU M4 Pro 48GB 512GB Silver</t>
+          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 16GB 2TB Space Black</t>
         </is>
       </c>
       <c r="B28" t="n">
+        <v>14</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
         <v>16</v>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>M4 Pro</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>48</v>
-      </c>
       <c r="E28" t="n">
-        <v>512</v>
+        <v>2048</v>
       </c>
       <c r="F28" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="G28" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I28" s="3" t="n">
@@ -2853,28 +2851,25 @@
         <v>810000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>1243863</v>
+        <v>1072306</v>
       </c>
       <c r="L28" t="n">
-        <v>34.88028826325728</v>
+        <v>24.46186070021058</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N28" t="n">
-        <v>0</v>
-      </c>
-      <c r="O28" t="n">
-        <v>100</v>
+        <v>2.702702702702703</v>
       </c>
       <c r="P28" t="n">
-        <v>100</v>
+        <v>61.99999999999999</v>
       </c>
       <c r="Q28" t="n">
-        <v>50.5</v>
+        <v>24.7</v>
       </c>
       <c r="R28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S28" t="inlineStr">
         <is>
@@ -2885,28 +2880,28 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 MJLV4 M5 Pro 15 Core CPU 16 Core GPU 24GB 2TB Silver</t>
+          <t>Apple MacBook Pro 16Inch MX2U3 14Core CPU 20Core GPU M4 Pro 48GB 512GB Silver</t>
         </is>
       </c>
       <c r="B29" t="n">
+        <v>16</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>M4 Pro</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>48</v>
+      </c>
+      <c r="E29" t="n">
+        <v>512</v>
+      </c>
+      <c r="F29" t="n">
         <v>14</v>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>M5 Pro</t>
-        </is>
-      </c>
-      <c r="D29" t="n">
-        <v>24</v>
-      </c>
-      <c r="E29" t="n">
-        <v>2048</v>
-      </c>
-      <c r="F29" t="n">
-        <v>15</v>
-      </c>
       <c r="G29" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
@@ -2914,12 +2909,17 @@
         </is>
       </c>
       <c r="I29" s="3" t="n">
-        <v>815000</v>
+        <v>810000</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>815000</v>
-      </c>
-      <c r="K29" s="3" t="n"/>
+        <v>810000</v>
+      </c>
+      <c r="K29" s="3" t="n">
+        <v>1243943</v>
+      </c>
+      <c r="L29" t="n">
+        <v>34.88447621796175</v>
+      </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
       </c>
@@ -2927,16 +2927,16 @@
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>70.58823529411765</v>
+        <v>100</v>
       </c>
       <c r="P29" t="n">
-        <v>80.0976800976801</v>
+        <v>100</v>
       </c>
       <c r="Q29" t="n">
-        <v>43.6</v>
+        <v>50.5</v>
       </c>
       <c r="R29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S29" t="inlineStr">
         <is>
@@ -2947,7 +2947,7 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 MGEA4 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Space Black</t>
+          <t>Macbook Pro 16 MGE44 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Silver</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -2972,35 +2972,35 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I30" s="3" t="n">
-        <v>825000</v>
+        <v>822999</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>825000</v>
+        <v>822999</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1286770</v>
+        <v>1286853</v>
       </c>
       <c r="L30" t="n">
-        <v>35.8859780691188</v>
+        <v>36.04560893901635</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>0</v>
+        <v>-7000</v>
       </c>
       <c r="N30" t="n">
-        <v>0.6022898822769667</v>
+        <v>2.023928571428571</v>
       </c>
       <c r="O30" t="n">
         <v>100</v>
       </c>
       <c r="P30" t="n">
-        <v>1.718244359164265</v>
+        <v>0.0003521901827191575</v>
       </c>
       <c r="Q30" t="n">
-        <v>34.6</v>
+        <v>34.8</v>
       </c>
       <c r="R30" t="n">
         <v>4</v>
@@ -3014,7 +3014,7 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 MGE44 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Silver</t>
+          <t>Macbook Pro 16 MGEA4 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -3039,26 +3039,26 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I31" s="3" t="n">
-        <v>829999</v>
+        <v>823000</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>829999</v>
+        <v>823000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1286770</v>
+        <v>1286853</v>
       </c>
       <c r="L31" t="n">
-        <v>35.49748595320064</v>
+        <v>36.04553123006279</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>0</v>
+        <v>-2000</v>
       </c>
       <c r="N31" t="n">
-        <v>1.190595238095238</v>
+        <v>0.5437465521127203</v>
       </c>
       <c r="O31" t="n">
         <v>0</v>
@@ -3116,10 +3116,10 @@
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1372583</v>
+        <v>1372671</v>
       </c>
       <c r="L32" t="n">
-        <v>38.21874524163566</v>
+        <v>38.22270595066116</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3183,10 +3183,10 @@
         <v>930000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1372583</v>
+        <v>1372671</v>
       </c>
       <c r="L33" t="n">
-        <v>38.07303456330146</v>
+        <v>38.07700461363284</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3250,10 +3250,10 @@
         <v>860000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>1243863</v>
+        <v>1243943</v>
       </c>
       <c r="L34" t="n">
-        <v>30.86055297086576</v>
+        <v>30.86499944129273</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -3324,13 +3324,13 @@
         <v>0</v>
       </c>
       <c r="O35" t="n">
-        <v>11.76588235294118</v>
+        <v>10.001</v>
       </c>
       <c r="P35" t="n">
         <v>70.3298656898657</v>
       </c>
       <c r="Q35" t="n">
-        <v>21.5</v>
+        <v>20.9</v>
       </c>
       <c r="R35" t="n">
         <v>3</v>
@@ -3383,7 +3383,7 @@
         <v>0</v>
       </c>
       <c r="N36" t="n">
-        <v>1.685393258426966</v>
+        <v>0.84985835694051</v>
       </c>
       <c r="O36" t="n">
         <v>0</v>
@@ -3392,7 +3392,7 @@
         <v>0</v>
       </c>
       <c r="Q36" t="n">
-        <v>0.7</v>
+        <v>0.4</v>
       </c>
       <c r="R36" t="n">
         <v>3</v>
@@ -3503,22 +3503,22 @@
         <v>880000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>1158050</v>
+        <v>1158124</v>
       </c>
       <c r="L38" t="n">
-        <v>24.01018954276585</v>
+        <v>24.01504502108583</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N38" t="n">
-        <v>1.123595505617978</v>
+        <v>0.5649717514124294</v>
       </c>
       <c r="P38" t="n">
         <v>73.14285714285714</v>
       </c>
       <c r="Q38" t="n">
-        <v>26.4</v>
+        <v>26.2</v>
       </c>
       <c r="R38" t="n">
         <v>3</v>
@@ -3567,22 +3567,22 @@
         <v>940000</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>1243863</v>
+        <v>1243943</v>
       </c>
       <c r="L39" t="n">
-        <v>24.42897650303932</v>
+        <v>24.43383659862229</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N39" t="n">
-        <v>2.083333333333333</v>
+        <v>1.052631578947368</v>
       </c>
       <c r="P39" t="n">
         <v>83</v>
       </c>
       <c r="Q39" t="n">
-        <v>29</v>
+        <v>28.6</v>
       </c>
       <c r="R39" t="n">
         <v>3</v>
@@ -3631,10 +3631,10 @@
         <v>990000</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>1501303</v>
+        <v>1501400</v>
       </c>
       <c r="L40" t="n">
-        <v>34.0572822408268</v>
+        <v>34.06154256027708</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -3695,10 +3695,10 @@
         <v>990000</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>1501303</v>
+        <v>1501400</v>
       </c>
       <c r="L41" t="n">
-        <v>34.0572822408268</v>
+        <v>34.06154256027708</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
@@ -3763,7 +3763,7 @@
         <v>0</v>
       </c>
       <c r="N42" t="n">
-        <v>2.450980392156863</v>
+        <v>1.240694789081886</v>
       </c>
       <c r="O42" t="n">
         <v>100</v>
@@ -3772,7 +3772,7 @@
         <v>69.23076923076923</v>
       </c>
       <c r="Q42" t="n">
-        <v>51.7</v>
+        <v>51.2</v>
       </c>
       <c r="R42" t="n">
         <v>3</v>
@@ -3821,22 +3821,22 @@
         <v>1055000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1544210</v>
+        <v>1544309</v>
       </c>
       <c r="L43" t="n">
-        <v>31.68027664631106</v>
+        <v>31.68465637382156</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>0.7525870178739417</v>
+        <v>0.3777148253068933</v>
       </c>
       <c r="P43" t="n">
-        <v>58.64647440248988</v>
+        <v>57.6271186440678</v>
       </c>
       <c r="Q43" t="n">
-        <v>26.4</v>
+        <v>26.1</v>
       </c>
       <c r="R43" t="n">
         <v>3</v>
@@ -3885,22 +3885,22 @@
         <v>1055000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1544210</v>
+        <v>1544309</v>
       </c>
       <c r="L44" t="n">
-        <v>31.68027664631106</v>
+        <v>31.68465637382156</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>2.314814814814815</v>
+        <v>1.17096018735363</v>
       </c>
       <c r="P44" t="n">
-        <v>58.64647440248988</v>
+        <v>57.6271186440678</v>
       </c>
       <c r="Q44" t="n">
-        <v>27</v>
+        <v>26.3</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -3953,7 +3953,7 @@
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>3.19634703196347</v>
+        <v>1.624129930394431</v>
       </c>
       <c r="O45" t="n">
         <v>0</v>
@@ -3962,7 +3962,7 @@
         <v>58.11965811965813</v>
       </c>
       <c r="Q45" t="n">
-        <v>15.9</v>
+        <v>15.2</v>
       </c>
       <c r="R45" t="n">
         <v>3</v>
@@ -4011,10 +4011,10 @@
         <v>1115000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1501303</v>
+        <v>1501400</v>
       </c>
       <c r="L46" t="n">
-        <v>25.73118151365847</v>
+        <v>25.73597975223125</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -4023,10 +4023,10 @@
         <v>3.043478260869565</v>
       </c>
       <c r="P46" t="n">
-        <v>11.53874765504792</v>
+        <v>9.358196283135744</v>
       </c>
       <c r="Q46" t="n">
-        <v>14.6</v>
+        <v>14.1</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -4075,10 +4075,10 @@
         <v>1123000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1715837</v>
+        <v>1715947</v>
       </c>
       <c r="L47" t="n">
-        <v>34.55089265472186</v>
+        <v>34.55508823990485</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -4142,22 +4142,22 @@
         <v>1130000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1501303</v>
+        <v>1501400</v>
       </c>
       <c r="L48" t="n">
-        <v>24.73204942639827</v>
+        <v>24.73691221526575</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N48" t="n">
-        <v>1.739130434782609</v>
+        <v>0.8771929824561403</v>
       </c>
       <c r="P48" t="n">
         <v>88.39999999999999</v>
       </c>
       <c r="Q48" t="n">
-        <v>30.2</v>
+        <v>29.9</v>
       </c>
       <c r="R48" t="n">
         <v>3</v>
@@ -4210,7 +4210,7 @@
         <v>0</v>
       </c>
       <c r="N49" t="n">
-        <v>2.11864406779661</v>
+        <v>1.070663811563169</v>
       </c>
       <c r="O49" t="n">
         <v>100</v>
@@ -4219,7 +4219,7 @@
         <v>81.36752136752136</v>
       </c>
       <c r="Q49" t="n">
-        <v>54.6</v>
+        <v>54.1</v>
       </c>
       <c r="R49" t="n">
         <v>3</v>
@@ -4268,10 +4268,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1758743</v>
+        <v>1758856</v>
       </c>
       <c r="L50" t="n">
-        <v>34.32809682824608</v>
+        <v>34.33231600540351</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4332,10 +4332,10 @@
         <v>1155000</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>1758743</v>
+        <v>1758856</v>
       </c>
       <c r="L51" t="n">
-        <v>34.32809682824608</v>
+        <v>34.33231600540351</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -4396,22 +4396,22 @@
         <v>1185000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1587117</v>
+        <v>1587218</v>
       </c>
       <c r="L52" t="n">
-        <v>25.33631736034583</v>
+        <v>25.34106846066514</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N52" t="n">
-        <v>2.469135802469136</v>
+        <v>1.25</v>
       </c>
       <c r="P52" t="n">
         <v>77.26495726495727</v>
       </c>
       <c r="Q52" t="n">
-        <v>28.3</v>
+        <v>27.9</v>
       </c>
       <c r="R52" t="n">
         <v>3</v>
@@ -4460,22 +4460,22 @@
         <v>1185000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1587117</v>
+        <v>1587218</v>
       </c>
       <c r="L53" t="n">
-        <v>25.33631736034583</v>
+        <v>25.34106846066514</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N53" t="n">
-        <v>2.066115702479339</v>
+        <v>1.04384133611691</v>
       </c>
       <c r="P53" t="n">
         <v>94.72727272727272</v>
       </c>
       <c r="Q53" t="n">
-        <v>31.9</v>
+        <v>31.5</v>
       </c>
       <c r="R53" t="n">
         <v>3</v>
@@ -4524,10 +4524,10 @@
         <v>1200000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1887463</v>
+        <v>1887584</v>
       </c>
       <c r="L54" t="n">
-        <v>36.42259477404325</v>
+        <v>36.42667028328276</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -4588,10 +4588,10 @@
         <v>1200000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1887463</v>
+        <v>1887584</v>
       </c>
       <c r="L55" t="n">
-        <v>36.42259477404325</v>
+        <v>36.42667028328276</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -4656,7 +4656,7 @@
         <v>0</v>
       </c>
       <c r="N56" t="n">
-        <v>2.811244979919679</v>
+        <v>1.425661914460285</v>
       </c>
       <c r="O56" t="n">
         <v>0</v>
@@ -4665,7 +4665,7 @@
         <v>73.84615384615385</v>
       </c>
       <c r="Q56" t="n">
-        <v>19.6</v>
+        <v>19.1</v>
       </c>
       <c r="R56" t="n">
         <v>3</v>
@@ -4714,22 +4714,22 @@
         <v>1240000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1672930</v>
+        <v>1673037</v>
       </c>
       <c r="L57" t="n">
-        <v>25.87854841505622</v>
+        <v>25.88328889319244</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N57" t="n">
-        <v>3.125</v>
+        <v>1.587301587301587</v>
       </c>
       <c r="P57" t="n">
         <v>100</v>
       </c>
       <c r="Q57" t="n">
-        <v>33.6</v>
+        <v>33.1</v>
       </c>
       <c r="R57" t="n">
         <v>3</v>
@@ -4840,10 +4840,10 @@
         <v>1280000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1715837</v>
+        <v>1715947</v>
       </c>
       <c r="L59" t="n">
-        <v>25.40083935711842</v>
+        <v>25.40562150229582</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -4907,10 +4907,10 @@
         <v>1298000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1758743</v>
+        <v>1758856</v>
       </c>
       <c r="L60" t="n">
-        <v>26.19728976888607</v>
+        <v>26.20203132035823</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -4919,10 +4919,10 @@
         <v>2.989536621823617</v>
       </c>
       <c r="P60" t="n">
-        <v>62.21254466180763</v>
+        <v>61.28109178956637</v>
       </c>
       <c r="Q60" t="n">
-        <v>25.6</v>
+        <v>25.4</v>
       </c>
       <c r="R60" t="n">
         <v>3</v>
@@ -4971,10 +4971,10 @@
         <v>1300000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1715837</v>
+        <v>1715947</v>
       </c>
       <c r="L61" t="n">
-        <v>24.23522747207339</v>
+        <v>24.24008433826919</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -4983,10 +4983,10 @@
         <v>0.7633587786259541</v>
       </c>
       <c r="P61" t="n">
-        <v>61.86882704645171</v>
+        <v>60.92890160686771</v>
       </c>
       <c r="Q61" t="n">
-        <v>23.9</v>
+        <v>23.7</v>
       </c>
       <c r="R61" t="n">
         <v>3</v>
@@ -5039,7 +5039,7 @@
         <v>0</v>
       </c>
       <c r="N62" t="n">
-        <v>3.623188405797102</v>
+        <v>1.845018450184502</v>
       </c>
       <c r="O62" t="n">
         <v>0</v>
@@ -5048,7 +5048,7 @@
         <v>73.97047397047398</v>
       </c>
       <c r="Q62" t="n">
-        <v>20</v>
+        <v>19.3</v>
       </c>
       <c r="R62" t="n">
         <v>3</v>
@@ -5097,22 +5097,22 @@
         <v>1335000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1801650</v>
+        <v>1801765</v>
       </c>
       <c r="L63" t="n">
-        <v>25.90125718091749</v>
+        <v>25.90598662977691</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N63" t="n">
-        <v>2.554744525547445</v>
+        <v>1.293900184842884</v>
       </c>
       <c r="P63" t="n">
         <v>87.17948717948718</v>
       </c>
       <c r="Q63" t="n">
-        <v>30.7</v>
+        <v>30.2</v>
       </c>
       <c r="R63" t="n">
         <v>3</v>
@@ -5161,10 +5161,10 @@
         <v>1420000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1930370</v>
+        <v>1930493</v>
       </c>
       <c r="L64" t="n">
-        <v>26.43897283940385</v>
+        <v>26.44365972836991</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -5173,10 +5173,10 @@
         <v>3.467029231815092</v>
       </c>
       <c r="P64" t="n">
-        <v>81.91902127554754</v>
+        <v>81.47332893095606</v>
       </c>
       <c r="Q64" t="n">
-        <v>30.1</v>
+        <v>30</v>
       </c>
       <c r="R64" t="n">
         <v>3</v>
@@ -5225,10 +5225,10 @@
         <v>1430000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1930370</v>
+        <v>1930493</v>
       </c>
       <c r="L65" t="n">
-        <v>25.92093743686443</v>
+        <v>25.92565733209082</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -5237,10 +5237,10 @@
         <v>2.787219578518015</v>
       </c>
       <c r="P65" t="n">
-        <v>61.86882704645171</v>
+        <v>60.92890160686771</v>
       </c>
       <c r="Q65" t="n">
-        <v>25.4</v>
+        <v>25.2</v>
       </c>
       <c r="R65" t="n">
         <v>3</v>
@@ -5289,10 +5289,10 @@
         <v>1430000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>2144903</v>
+        <v>2145040</v>
       </c>
       <c r="L66" t="n">
-        <v>33.33031843398047</v>
+        <v>33.33457651139373</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -5353,10 +5353,10 @@
         <v>1430000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>2144903</v>
+        <v>2145040</v>
       </c>
       <c r="L67" t="n">
-        <v>33.33031843398047</v>
+        <v>33.33457651139373</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -5421,7 +5421,7 @@
         <v>0</v>
       </c>
       <c r="N68" t="n">
-        <v>3.02013422818792</v>
+        <v>1.533219761499148</v>
       </c>
       <c r="O68" t="n">
         <v>100</v>
@@ -5430,7 +5430,7 @@
         <v>98.16849816849818</v>
       </c>
       <c r="Q68" t="n">
-        <v>59.1</v>
+        <v>58.5</v>
       </c>
       <c r="R68" t="n">
         <v>3</v>
@@ -5479,22 +5479,22 @@
         <v>1480000</v>
       </c>
       <c r="K69" s="3" t="n">
-        <v>2016183</v>
+        <v>2016312</v>
       </c>
       <c r="L69" t="n">
-        <v>26.59396493274668</v>
+        <v>26.59866131828804</v>
       </c>
       <c r="M69" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N69" t="n">
-        <v>3.583061889250815</v>
+        <v>1.824212271973466</v>
       </c>
       <c r="P69" t="n">
         <v>0</v>
       </c>
       <c r="Q69" t="n">
-        <v>12.7</v>
+        <v>12.1</v>
       </c>
       <c r="R69" t="n">
         <v>3</v>
@@ -5547,7 +5547,7 @@
         <v>0</v>
       </c>
       <c r="N70" t="n">
-        <v>2.884615384615385</v>
+        <v>1.463414634146342</v>
       </c>
       <c r="O70" t="n">
         <v>0</v>
@@ -5556,7 +5556,7 @@
         <v>91.33089133089133</v>
       </c>
       <c r="Q70" t="n">
-        <v>24</v>
+        <v>23.4</v>
       </c>
       <c r="R70" t="n">
         <v>3</v>
@@ -5605,22 +5605,22 @@
         <v>1605000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2187810</v>
+        <v>2187950</v>
       </c>
       <c r="L71" t="n">
-        <v>26.63896773485814</v>
+        <v>26.64366187527137</v>
       </c>
       <c r="M71" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N71" t="n">
-        <v>2.727272727272727</v>
+        <v>1.382488479262673</v>
       </c>
       <c r="P71" t="n">
         <v>36.44392794886694</v>
       </c>
       <c r="Q71" t="n">
-        <v>20.2</v>
+        <v>19.7</v>
       </c>
       <c r="R71" t="n">
         <v>3</v>
@@ -5669,22 +5669,22 @@
         <v>1610000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2187810</v>
+        <v>2187950</v>
       </c>
       <c r="L72" t="n">
-        <v>26.41042869353372</v>
+        <v>26.41513745743732</v>
       </c>
       <c r="M72" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N72" t="n">
-        <v>3.012048192771084</v>
+        <v>1.529051987767584</v>
       </c>
       <c r="P72" t="n">
         <v>25.72147975982957</v>
       </c>
       <c r="Q72" t="n">
-        <v>17.9</v>
+        <v>17.4</v>
       </c>
       <c r="R72" t="n">
         <v>3</v>
@@ -5733,10 +5733,10 @@
         <v>1615000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2187810</v>
+        <v>2187950</v>
       </c>
       <c r="L73" t="n">
-        <v>26.18188965220929</v>
+        <v>26.18661303960328</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
@@ -5745,10 +5745,10 @@
         <v>2.769416014449127</v>
       </c>
       <c r="P73" t="n">
-        <v>87.03386674215359</v>
+        <v>86.7142542687337</v>
       </c>
       <c r="Q73" t="n">
-        <v>30.9</v>
+        <v>30.8</v>
       </c>
       <c r="R73" t="n">
         <v>3</v>
@@ -5797,22 +5797,22 @@
         <v>1630000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2230716</v>
+        <v>2230859</v>
       </c>
       <c r="L74" t="n">
-        <v>26.92929086445787</v>
+        <v>26.93397476039499</v>
       </c>
       <c r="M74" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N74" t="n">
-        <v>2.976190476190476</v>
+        <v>1.510574018126888</v>
       </c>
       <c r="P74" t="n">
         <v>100</v>
       </c>
       <c r="Q74" t="n">
-        <v>34</v>
+        <v>33.5</v>
       </c>
       <c r="R74" t="n">
         <v>3</v>
@@ -5861,10 +5861,10 @@
         <v>1690000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2316529</v>
+        <v>2316678</v>
       </c>
       <c r="L75" t="n">
-        <v>27.0460244615975</v>
+        <v>27.05071658642246</v>
       </c>
       <c r="M75" s="3" t="n">
         <v>0</v>
@@ -5876,7 +5876,7 @@
         <v>16.88768606224628</v>
       </c>
       <c r="Q75" t="n">
-        <v>15.6</v>
+        <v>15.7</v>
       </c>
       <c r="R75" t="n">
         <v>3</v>
@@ -5925,10 +5925,10 @@
         <v>1705000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2316529</v>
+        <v>2316678</v>
       </c>
       <c r="L76" t="n">
-        <v>26.3985039686531</v>
+        <v>26.40323773955638</v>
       </c>
       <c r="M76" s="3" t="n">
         <v>0</v>
@@ -5989,10 +5989,10 @@
         <v>1725000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2359436</v>
+        <v>2359587</v>
       </c>
       <c r="L77" t="n">
-        <v>26.8893074446605</v>
+        <v>26.89398610858596</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
@@ -6004,7 +6004,7 @@
         <v>100</v>
       </c>
       <c r="Q77" t="n">
-        <v>34.2</v>
+        <v>34.3</v>
       </c>
       <c r="R77" t="n">
         <v>3</v>
@@ -6053,22 +6053,22 @@
         <v>1780000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2445249</v>
+        <v>2445406</v>
       </c>
       <c r="L78" t="n">
-        <v>27.205777407536</v>
+        <v>27.21045094352431</v>
       </c>
       <c r="M78" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N78" t="n">
-        <v>3.260869565217391</v>
+        <v>1.657458563535912</v>
       </c>
       <c r="P78" t="n">
         <v>38.78143936249688</v>
       </c>
       <c r="Q78" t="n">
-        <v>21.1</v>
+        <v>20.6</v>
       </c>
       <c r="R78" t="n">
         <v>3</v>
@@ -6117,10 +6117,10 @@
         <v>1875000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2573969</v>
+        <v>2574134</v>
       </c>
       <c r="L79" t="n">
-        <v>27.1552998501536</v>
+        <v>27.15996913913573</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
@@ -6181,22 +6181,22 @@
         <v>1910000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2616876</v>
+        <v>2617044</v>
       </c>
       <c r="L80" t="n">
-        <v>27.01220845007559</v>
+        <v>27.01689386957193</v>
       </c>
       <c r="M80" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N80" t="n">
-        <v>2.551020408163265</v>
+        <v>1.291989664082687</v>
       </c>
       <c r="P80" t="n">
         <v>53.22486926205694</v>
       </c>
       <c r="Q80" t="n">
-        <v>23.9</v>
+        <v>23.4</v>
       </c>
       <c r="R80" t="n">
         <v>3</v>
@@ -6245,10 +6245,10 @@
         <v>2020000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2745596</v>
+        <v>2745772</v>
       </c>
       <c r="L81" t="n">
-        <v>26.42763174188774</v>
+        <v>26.43234762391051</v>
       </c>
       <c r="M81" s="3" t="n">
         <v>0</v>
@@ -6309,22 +6309,22 @@
         <v>2110000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>2874316</v>
+        <v>2874500</v>
       </c>
       <c r="L82" t="n">
-        <v>26.59123074846329</v>
+        <v>26.59592972690903</v>
       </c>
       <c r="M82" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N82" t="n">
-        <v>2.764976958525346</v>
+        <v>1.401869158878505</v>
       </c>
       <c r="P82" t="n">
         <v>79.02382335851249</v>
       </c>
       <c r="Q82" t="n">
-        <v>29.3</v>
+        <v>28.8</v>
       </c>
       <c r="R82" t="n">
         <v>3</v>
@@ -6373,10 +6373,10 @@
         <v>2210000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3003036</v>
+        <v>3003228</v>
       </c>
       <c r="L83" t="n">
-        <v>26.40780863099877</v>
+        <v>26.41251346884086</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
@@ -6437,22 +6437,22 @@
         <v>2215000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3045942</v>
+        <v>3046138</v>
       </c>
       <c r="L84" t="n">
-        <v>27.28029621049908</v>
+        <v>27.2849752703259</v>
       </c>
       <c r="M84" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N84" t="n">
-        <v>2.422907488986784</v>
+        <v>1.226309921962096</v>
       </c>
       <c r="P84" t="n">
         <v>74.28466149856153</v>
       </c>
       <c r="Q84" t="n">
-        <v>28.5</v>
+        <v>28</v>
       </c>
       <c r="R84" t="n">
         <v>3</v>
@@ -6501,10 +6501,10 @@
         <v>2315000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3174662</v>
+        <v>3174866</v>
       </c>
       <c r="L85" t="n">
-        <v>27.07885122888673</v>
+        <v>27.08353675399214</v>
       </c>
       <c r="M85" s="3" t="n">
         <v>0</v>
@@ -6565,22 +6565,22 @@
         <v>2395000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3303382</v>
+        <v>3303594</v>
       </c>
       <c r="L86" t="n">
-        <v>27.49854543010769</v>
+        <v>27.50319803220371</v>
       </c>
       <c r="M86" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N86" t="n">
-        <v>3.42741935483871</v>
+        <v>1.743589743589744</v>
       </c>
       <c r="P86" t="n">
         <v>72.76953145634144</v>
       </c>
       <c r="Q86" t="n">
-        <v>28.6</v>
+        <v>28</v>
       </c>
       <c r="R86" t="n">
         <v>3</v>
@@ -6629,22 +6629,22 @@
         <v>2410000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3303382</v>
+        <v>3303594</v>
       </c>
       <c r="L87" t="n">
-        <v>27.04446533885575</v>
+        <v>27.04914708042211</v>
       </c>
       <c r="M87" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N87" t="n">
-        <v>2.42914979757085</v>
+        <v>1.229508196721312</v>
       </c>
       <c r="P87" t="n">
         <v>88.47569242688358</v>
       </c>
       <c r="Q87" t="n">
-        <v>31.4</v>
+        <v>31</v>
       </c>
       <c r="R87" t="n">
         <v>3</v>
@@ -6693,10 +6693,10 @@
         <v>2499000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3432102</v>
+        <v>3432322</v>
       </c>
       <c r="L88" t="n">
-        <v>27.18747869381504</v>
+        <v>27.19214572525538</v>
       </c>
       <c r="M88" s="3" t="n">
         <v>0</v>
@@ -6757,10 +6757,10 @@
         <v>2510000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3432102</v>
+        <v>3432322</v>
       </c>
       <c r="L89" t="n">
-        <v>26.8669753987498</v>
+        <v>26.87166297334574</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
@@ -6821,22 +6821,22 @@
         <v>2530000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3475009</v>
+        <v>3475232</v>
       </c>
       <c r="L90" t="n">
-        <v>27.19443316549684</v>
+        <v>27.19910498061712</v>
       </c>
       <c r="M90" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N90" t="n">
-        <v>1.937984496124031</v>
+        <v>0.9784735812133072</v>
       </c>
       <c r="P90" t="n">
         <v>79.17877203176447</v>
       </c>
       <c r="Q90" t="n">
-        <v>29.3</v>
+        <v>29</v>
       </c>
       <c r="R90" t="n">
         <v>3</v>
@@ -6885,10 +6885,10 @@
         <v>2610000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>3603729</v>
+        <v>3603960</v>
       </c>
       <c r="L91" t="n">
-        <v>27.5750202082343</v>
+        <v>27.57966237139147</v>
       </c>
       <c r="M91" s="3" t="n">
         <v>0</v>
@@ -6949,22 +6949,22 @@
         <v>3015000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4161515</v>
+        <v>4161782</v>
       </c>
       <c r="L92" t="n">
-        <v>27.55042334342181</v>
+        <v>27.55507136125823</v>
       </c>
       <c r="M92" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N92" t="n">
-        <v>2.427184466019417</v>
+        <v>1.228501228501228</v>
       </c>
       <c r="P92" t="n">
         <v>100</v>
       </c>
       <c r="Q92" t="n">
-        <v>34.1</v>
+        <v>33.7</v>
       </c>
       <c r="R92" t="n">
         <v>3</v>
@@ -7013,10 +7013,10 @@
         <v>3098000</v>
       </c>
       <c r="K93" s="3" t="n">
-        <v>4290235</v>
+        <v>4290510</v>
       </c>
       <c r="L93" t="n">
-        <v>27.7895033721929</v>
+        <v>27.79413169996108</v>
       </c>
       <c r="M93" s="3" t="n">
         <v>0</v>
@@ -7312,10 +7312,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>428637</v>
+        <v>428665</v>
       </c>
       <c r="L2" t="n">
-        <v>27.67796527131349</v>
+        <v>27.6826892795073</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7379,10 +7379,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>428637</v>
+        <v>428665</v>
       </c>
       <c r="L3" t="n">
-        <v>27.67796527131349</v>
+        <v>27.6826892795073</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7446,10 +7446,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>428637</v>
+        <v>428665</v>
       </c>
       <c r="L4" t="n">
-        <v>27.6777319736747</v>
+        <v>27.6824559971073</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7513,10 +7513,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>428637</v>
+        <v>428665</v>
       </c>
       <c r="L5" t="n">
-        <v>27.6777319736747</v>
+        <v>27.6824559971073</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7580,10 +7580,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514451</v>
+        <v>514484</v>
       </c>
       <c r="L6" t="n">
-        <v>25.35732266046718</v>
+        <v>25.36211038632883</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7644,10 +7644,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>514451</v>
+        <v>514484</v>
       </c>
       <c r="L7" t="n">
-        <v>25.35732266046718</v>
+        <v>25.36211038632883</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7708,10 +7708,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>514451</v>
+        <v>514484</v>
       </c>
       <c r="L8" t="n">
-        <v>25.35732266046718</v>
+        <v>25.36211038632883</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7772,10 +7772,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>514451</v>
+        <v>514484</v>
       </c>
       <c r="L9" t="n">
-        <v>25.35732266046718</v>
+        <v>25.36211038632883</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7836,10 +7836,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>514451</v>
+        <v>514484</v>
       </c>
       <c r="L10" t="n">
-        <v>25.16294068822881</v>
+        <v>25.16774088212656</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7900,10 +7900,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>514451</v>
+        <v>514484</v>
       </c>
       <c r="L11" t="n">
-        <v>25.16294068822881</v>
+        <v>25.16774088212656</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7964,10 +7964,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>514451</v>
+        <v>514484</v>
       </c>
       <c r="L12" t="n">
-        <v>25.16294068822881</v>
+        <v>25.16774088212656</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -8028,10 +8028,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>514451</v>
+        <v>514484</v>
       </c>
       <c r="L13" t="n">
-        <v>25.16294068822881</v>
+        <v>25.16774088212656</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -8086,31 +8086,31 @@
         </is>
       </c>
       <c r="I14" s="3" t="n">
-        <v>420000</v>
+        <v>417999</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>420000</v>
+        <v>417999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>557357</v>
+        <v>557393</v>
       </c>
       <c r="L14" t="n">
-        <v>24.64434823640862</v>
+        <v>25.00820785334584</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>0</v>
+        <v>-2001</v>
       </c>
       <c r="N14" t="n">
-        <v>3.225583469086334</v>
+        <v>2.677651545578051</v>
       </c>
       <c r="O14" t="n">
         <v>100</v>
       </c>
       <c r="P14" t="n">
-        <v>3.361344537815107</v>
+        <v>1.392</v>
       </c>
       <c r="Q14" t="n">
-        <v>31.9</v>
+        <v>31.5</v>
       </c>
       <c r="R14" t="n">
         <v>4</v>
@@ -8153,31 +8153,31 @@
         </is>
       </c>
       <c r="I15" s="3" t="n">
-        <v>420000</v>
+        <v>417999</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>420000</v>
+        <v>417999</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>557357</v>
+        <v>557393</v>
       </c>
       <c r="L15" t="n">
-        <v>24.64434823640862</v>
+        <v>25.00820785334584</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>0</v>
+        <v>-2001</v>
       </c>
       <c r="N15" t="n">
-        <v>3.002085455162714</v>
+        <v>2.564222102822964</v>
       </c>
       <c r="O15" t="n">
         <v>100</v>
       </c>
       <c r="P15" t="n">
-        <v>3.361344537815107</v>
+        <v>1.392</v>
       </c>
       <c r="Q15" t="n">
-        <v>31.8</v>
+        <v>31.5</v>
       </c>
       <c r="R15" t="n">
         <v>4</v>
@@ -8220,31 +8220,31 @@
         </is>
       </c>
       <c r="I16" s="3" t="n">
-        <v>420000</v>
+        <v>417999</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>420000</v>
+        <v>417999</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>557357</v>
+        <v>557393</v>
       </c>
       <c r="L16" t="n">
-        <v>24.64434823640862</v>
+        <v>25.00820785334584</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0</v>
+        <v>-2001</v>
       </c>
       <c r="N16" t="n">
-        <v>2.325581395348837</v>
+        <v>2.222456140350877</v>
       </c>
       <c r="O16" t="n">
         <v>100</v>
       </c>
       <c r="P16" t="n">
-        <v>3.361344537815107</v>
+        <v>1.392</v>
       </c>
       <c r="Q16" t="n">
-        <v>31.6</v>
+        <v>31.4</v>
       </c>
       <c r="R16" t="n">
         <v>4</v>
@@ -8287,22 +8287,22 @@
         </is>
       </c>
       <c r="I17" s="3" t="n">
-        <v>425000</v>
+        <v>420000</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>425000</v>
+        <v>420000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>557357</v>
+        <v>557393</v>
       </c>
       <c r="L17" t="n">
-        <v>23.74725714398491</v>
+        <v>24.64921518569484</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>0</v>
+        <v>-5000</v>
       </c>
       <c r="N17" t="n">
-        <v>4.063205417607223</v>
+        <v>3.225806451612903</v>
       </c>
       <c r="O17" t="n">
         <v>0</v>
@@ -8311,7 +8311,7 @@
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>9</v>
+        <v>9.1</v>
       </c>
       <c r="R17" t="n">
         <v>4</v>
@@ -8360,10 +8360,10 @@
         <v>454000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>600264</v>
+        <v>600302</v>
       </c>
       <c r="L18" t="n">
-        <v>24.36661202404276</v>
+        <v>24.37139972880317</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -8424,10 +8424,10 @@
         <v>454000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>600264</v>
+        <v>600302</v>
       </c>
       <c r="L19" t="n">
-        <v>24.36661202404276</v>
+        <v>24.37139972880317</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -8488,10 +8488,10 @@
         <v>454000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>600264</v>
+        <v>600302</v>
       </c>
       <c r="L20" t="n">
-        <v>24.36661202404276</v>
+        <v>24.37139972880317</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -8552,10 +8552,10 @@
         <v>454000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>600264</v>
+        <v>600302</v>
       </c>
       <c r="L21" t="n">
-        <v>24.36661202404276</v>
+        <v>24.37139972880317</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -8616,10 +8616,10 @@
         <v>455000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>600264</v>
+        <v>600302</v>
       </c>
       <c r="L22" t="n">
-        <v>24.20001865845694</v>
+        <v>24.20481690882256</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -8680,10 +8680,10 @@
         <v>455000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>600264</v>
+        <v>600302</v>
       </c>
       <c r="L23" t="n">
-        <v>24.20001865845694</v>
+        <v>24.20481690882256</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -8744,10 +8744,10 @@
         <v>455000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>600264</v>
+        <v>600302</v>
       </c>
       <c r="L24" t="n">
-        <v>24.20001865845694</v>
+        <v>24.20481690882256</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -8808,10 +8808,10 @@
         <v>455000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>600264</v>
+        <v>600302</v>
       </c>
       <c r="L25" t="n">
-        <v>24.20001865845694</v>
+        <v>24.20481690882256</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -8872,10 +8872,10 @@
         <v>475000</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>686077</v>
+        <v>686121</v>
       </c>
       <c r="L26" t="n">
-        <v>30.7657886796963</v>
+        <v>30.77022857484321</v>
       </c>
       <c r="M26" s="3" t="n">
         <v>0</v>
@@ -8936,10 +8936,10 @@
         <v>475000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>686077</v>
+        <v>686121</v>
       </c>
       <c r="L27" t="n">
-        <v>30.7657886796963</v>
+        <v>30.77022857484321</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -9000,10 +9000,10 @@
         <v>475000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>686077</v>
+        <v>686121</v>
       </c>
       <c r="L28" t="n">
-        <v>30.7657886796963</v>
+        <v>30.77022857484321</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -9064,10 +9064,10 @@
         <v>475000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>686077</v>
+        <v>686121</v>
       </c>
       <c r="L29" t="n">
-        <v>30.7657886796963</v>
+        <v>30.77022857484321</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -9128,10 +9128,10 @@
         <v>477000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>643171</v>
+        <v>643212</v>
       </c>
       <c r="L30" t="n">
-        <v>25.83620841113794</v>
+        <v>25.8409358034365</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -9195,10 +9195,10 @@
         <v>477000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>643171</v>
+        <v>643212</v>
       </c>
       <c r="L31" t="n">
-        <v>25.83620841113794</v>
+        <v>25.8409358034365</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -9262,10 +9262,10 @@
         <v>477000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>643171</v>
+        <v>643212</v>
       </c>
       <c r="L32" t="n">
-        <v>25.83620841113794</v>
+        <v>25.8409358034365</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -9329,10 +9329,10 @@
         <v>479999</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>686077</v>
+        <v>686121</v>
       </c>
       <c r="L33" t="n">
-        <v>30.03715326413799</v>
+        <v>30.04163988567614</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -9341,10 +9341,10 @@
         <v>0</v>
       </c>
       <c r="P33" t="n">
-        <v>43.6979831932773</v>
+        <v>41.73965217391304</v>
       </c>
       <c r="Q33" t="n">
-        <v>22.2</v>
+        <v>21.8</v>
       </c>
       <c r="R33" t="n">
         <v>3</v>
@@ -9393,10 +9393,10 @@
         <v>479999</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>686077</v>
+        <v>686121</v>
       </c>
       <c r="L34" t="n">
-        <v>30.03715326413799</v>
+        <v>30.04163988567614</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -9405,10 +9405,10 @@
         <v>0</v>
       </c>
       <c r="P34" t="n">
-        <v>43.6979831932773</v>
+        <v>41.73965217391304</v>
       </c>
       <c r="Q34" t="n">
-        <v>22.2</v>
+        <v>21.8</v>
       </c>
       <c r="R34" t="n">
         <v>3</v>
@@ -9457,10 +9457,10 @@
         <v>479999</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>686077</v>
+        <v>686121</v>
       </c>
       <c r="L35" t="n">
-        <v>30.03715326413799</v>
+        <v>30.04163988567614</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
@@ -9469,10 +9469,10 @@
         <v>0</v>
       </c>
       <c r="P35" t="n">
-        <v>43.6979831932773</v>
+        <v>41.73965217391304</v>
       </c>
       <c r="Q35" t="n">
-        <v>22.2</v>
+        <v>21.8</v>
       </c>
       <c r="R35" t="n">
         <v>3</v>
@@ -9521,10 +9521,10 @@
         <v>479999</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>686077</v>
+        <v>686121</v>
       </c>
       <c r="L36" t="n">
-        <v>30.03715326413799</v>
+        <v>30.04163988567614</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -9533,10 +9533,10 @@
         <v>0</v>
       </c>
       <c r="P36" t="n">
-        <v>43.6979831932773</v>
+        <v>41.73965217391304</v>
       </c>
       <c r="Q36" t="n">
-        <v>22.2</v>
+        <v>21.8</v>
       </c>
       <c r="R36" t="n">
         <v>3</v>
@@ -9585,16 +9585,16 @@
         <v>479999</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>643171</v>
+        <v>643212</v>
       </c>
       <c r="L37" t="n">
-        <v>25.36992494997443</v>
+        <v>25.37468206438935</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N37" t="n">
-        <v>2.040820491470391</v>
+        <v>1.639347621613979</v>
       </c>
       <c r="O37" t="n">
         <v>0</v>
@@ -9603,7 +9603,7 @@
         <v>0</v>
       </c>
       <c r="Q37" t="n">
-        <v>9</v>
+        <v>8.9</v>
       </c>
       <c r="R37" t="n">
         <v>4</v>
@@ -9652,10 +9652,10 @@
         <v>500000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>643171</v>
+        <v>643212</v>
       </c>
       <c r="L38" t="n">
-        <v>22.26017653159113</v>
+        <v>22.2651318694303</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -9664,10 +9664,10 @@
         <v>0</v>
       </c>
       <c r="P38" t="n">
-        <v>33.61344537815125</v>
+        <v>31.30434782608695</v>
       </c>
       <c r="Q38" t="n">
-        <v>16.7</v>
+        <v>16.3</v>
       </c>
       <c r="R38" t="n">
         <v>3</v>
@@ -9716,22 +9716,22 @@
         <v>547999</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>771890</v>
+        <v>771940</v>
       </c>
       <c r="L39" t="n">
-        <v>29.00555778673127</v>
+        <v>29.01015622975879</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N39" t="n">
-        <v>0.7246389939112209</v>
+        <v>0.5444655979411941</v>
       </c>
       <c r="P39" t="n">
-        <v>64.67267226890753</v>
+        <v>63.4438956521739</v>
       </c>
       <c r="Q39" t="n">
-        <v>26.5</v>
+        <v>26.2</v>
       </c>
       <c r="R39" t="n">
         <v>3</v>
@@ -9780,22 +9780,22 @@
         <v>547999</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>771890</v>
+        <v>771940</v>
       </c>
       <c r="L40" t="n">
-        <v>29.00555778673127</v>
+        <v>29.01015622975879</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N40" t="n">
-        <v>0.7246389939112209</v>
+        <v>0.5444655979411941</v>
       </c>
       <c r="P40" t="n">
-        <v>64.67267226890753</v>
+        <v>63.4438956521739</v>
       </c>
       <c r="Q40" t="n">
-        <v>26.5</v>
+        <v>26.2</v>
       </c>
       <c r="R40" t="n">
         <v>3</v>
@@ -9844,22 +9844,22 @@
         <v>547999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>771890</v>
+        <v>771940</v>
       </c>
       <c r="L41" t="n">
-        <v>29.00555778673127</v>
+        <v>29.01015622975879</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N41" t="n">
-        <v>1.792117907021339</v>
+        <v>1.261263533808169</v>
       </c>
       <c r="P41" t="n">
-        <v>64.67267226890753</v>
+        <v>63.4438956521739</v>
       </c>
       <c r="Q41" t="n">
-        <v>26.9</v>
+        <v>26.5</v>
       </c>
       <c r="R41" t="n">
         <v>3</v>
@@ -9908,22 +9908,22 @@
         <v>547999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>771890</v>
+        <v>771940</v>
       </c>
       <c r="L42" t="n">
-        <v>29.00555778673127</v>
+        <v>29.01015622975879</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N42" t="n">
-        <v>0.7246389939112209</v>
+        <v>0.5444655979411941</v>
       </c>
       <c r="P42" t="n">
-        <v>64.67267226890753</v>
+        <v>63.4438956521739</v>
       </c>
       <c r="Q42" t="n">
-        <v>26.5</v>
+        <v>26.2</v>
       </c>
       <c r="R42" t="n">
         <v>3</v>
@@ -9972,10 +9972,10 @@
         <v>552999</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>771890</v>
+        <v>771940</v>
       </c>
       <c r="L43" t="n">
-        <v>28.35779709544106</v>
+        <v>28.36243749514211</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -10036,10 +10036,10 @@
         <v>552999</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>771890</v>
+        <v>771940</v>
       </c>
       <c r="L44" t="n">
-        <v>28.35779709544106</v>
+        <v>28.36243749514211</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -10100,10 +10100,10 @@
         <v>552999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>771890</v>
+        <v>771940</v>
       </c>
       <c r="L45" t="n">
-        <v>28.35779709544106</v>
+        <v>28.36243749514211</v>
       </c>
       <c r="M45" s="3" t="n">
         <v>0</v>
@@ -10164,10 +10164,10 @@
         <v>552999</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>771890</v>
+        <v>771940</v>
       </c>
       <c r="L46" t="n">
-        <v>28.35779709544106</v>
+        <v>28.36243749514211</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -10228,10 +10228,10 @@
         <v>585000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>728984</v>
+        <v>729031</v>
       </c>
       <c r="L47" t="n">
-        <v>19.75132513196449</v>
+        <v>19.75649869484288</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -10292,10 +10292,10 @@
         <v>595000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>728984</v>
+        <v>729031</v>
       </c>
       <c r="L48" t="n">
-        <v>18.37955291199807</v>
+        <v>18.38481491184874</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -10304,10 +10304,10 @@
         <v>0</v>
       </c>
       <c r="P48" t="n">
-        <v>45.7142857142857</v>
+        <v>43.82608695652173</v>
       </c>
       <c r="Q48" t="n">
-        <v>17.7</v>
+        <v>17.3</v>
       </c>
       <c r="R48" t="n">
         <v>3</v>
@@ -10356,10 +10356,10 @@
         <v>614999</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>857704</v>
+        <v>857759</v>
       </c>
       <c r="L49" t="n">
-        <v>28.29705819256993</v>
+        <v>28.30165582640345</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -10420,10 +10420,10 @@
         <v>614999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>857704</v>
+        <v>857759</v>
       </c>
       <c r="L50" t="n">
-        <v>28.29705819256993</v>
+        <v>28.30165582640345</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -10484,10 +10484,10 @@
         <v>614999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>857704</v>
+        <v>857759</v>
       </c>
       <c r="L51" t="n">
-        <v>28.29705819256993</v>
+        <v>28.30165582640345</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -10548,10 +10548,10 @@
         <v>614999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>857704</v>
+        <v>857759</v>
       </c>
       <c r="L52" t="n">
-        <v>28.29705819256993</v>
+        <v>28.30165582640345</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -10612,10 +10612,10 @@
         <v>650000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>814797</v>
+        <v>814849</v>
       </c>
       <c r="L53" t="n">
-        <v>20.22552856723822</v>
+        <v>20.23061941537635</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -10676,10 +10676,10 @@
         <v>672000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>857704</v>
+        <v>857759</v>
       </c>
       <c r="L54" t="n">
-        <v>21.6512922873159</v>
+        <v>21.65631605147833</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -10688,10 +10688,10 @@
         <v>0</v>
       </c>
       <c r="P54" t="n">
-        <v>59.83193277310923</v>
+        <v>58.43478260869565</v>
       </c>
       <c r="Q54" t="n">
-        <v>22.1</v>
+        <v>21.8</v>
       </c>
       <c r="R54" t="n">
         <v>3</v>
@@ -10740,10 +10740,10 @@
         <v>700000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>900610</v>
+        <v>900668</v>
       </c>
       <c r="L55" t="n">
-        <v>22.27490256603857</v>
+        <v>22.27990780176491</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -10752,10 +10752,10 @@
         <v>0</v>
       </c>
       <c r="P55" t="n">
-        <v>50.42016806722687</v>
+        <v>48.69565217391303</v>
       </c>
       <c r="Q55" t="n">
-        <v>20.4</v>
+        <v>20</v>
       </c>
       <c r="R55" t="n">
         <v>3</v>
@@ -10804,10 +10804,10 @@
         <v>715000</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>943517</v>
+        <v>943577</v>
       </c>
       <c r="L56" t="n">
-        <v>24.21970139382756</v>
+        <v>24.22452009745892</v>
       </c>
       <c r="M56" s="3" t="n">
         <v>0</v>
@@ -10868,10 +10868,10 @@
         <v>734999</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>986424</v>
+        <v>986487</v>
       </c>
       <c r="L57" t="n">
-        <v>25.48853231470443</v>
+        <v>25.49329083910888</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -10880,10 +10880,10 @@
         <v>0</v>
       </c>
       <c r="P57" t="n">
-        <v>73.94986794717886</v>
+        <v>73.04377639751551</v>
       </c>
       <c r="Q57" t="n">
-        <v>26.8</v>
+        <v>26.6</v>
       </c>
       <c r="R57" t="n">
         <v>3</v>
@@ -10932,10 +10932,10 @@
         <v>752000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>986424</v>
+        <v>986487</v>
       </c>
       <c r="L58" t="n">
-        <v>23.76503410298209</v>
+        <v>23.76990269511914</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -10996,10 +10996,10 @@
         <v>810000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1072237</v>
+        <v>1072306</v>
       </c>
       <c r="L59" t="n">
-        <v>24.45699971181744</v>
+        <v>24.46186070021058</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -11060,10 +11060,10 @@
         <v>815000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1072237</v>
+        <v>1072306</v>
       </c>
       <c r="L60" t="n">
-        <v>23.99068489522372</v>
+        <v>23.99557588971805</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -11072,10 +11072,10 @@
         <v>0</v>
       </c>
       <c r="P60" t="n">
-        <v>80.25210084033613</v>
+        <v>79.56521739130434</v>
       </c>
       <c r="Q60" t="n">
-        <v>27.5</v>
+        <v>27.3</v>
       </c>
       <c r="R60" t="n">
         <v>3</v>
@@ -11124,10 +11124,10 @@
         <v>875000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1158050</v>
+        <v>1158124</v>
       </c>
       <c r="L61" t="n">
-        <v>24.44194982945469</v>
+        <v>24.44677771982965</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -11188,10 +11188,10 @@
         <v>992000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1329677</v>
+        <v>1329762</v>
       </c>
       <c r="L62" t="n">
-        <v>25.39541557836979</v>
+        <v>25.40018439389906</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -11200,10 +11200,10 @@
         <v>0</v>
       </c>
       <c r="P62" t="n">
-        <v>85.64705882352939</v>
+        <v>85.14782608695651</v>
       </c>
       <c r="Q62" t="n">
-        <v>29.2</v>
+        <v>29.1</v>
       </c>
       <c r="R62" t="n">
         <v>3</v>
@@ -11252,10 +11252,10 @@
         <v>1050000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1415490</v>
+        <v>1415581</v>
       </c>
       <c r="L63" t="n">
-        <v>25.82074052095034</v>
+        <v>25.82550910191646</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -11264,7 +11264,7 @@
         <v>0</v>
       </c>
       <c r="P63" t="n">
-        <v>93.20091673032849</v>
+        <v>92.96442687747034</v>
       </c>
       <c r="Q63" t="n">
         <v>31</v>
@@ -11316,10 +11316,10 @@
         <v>1050000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1415490</v>
+        <v>1415581</v>
       </c>
       <c r="L64" t="n">
-        <v>25.82074052095034</v>
+        <v>25.82550910191646</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -11380,10 +11380,10 @@
         <v>1100000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1501303</v>
+        <v>1501400</v>
       </c>
       <c r="L65" t="n">
-        <v>26.73031360091867</v>
+        <v>26.73504728919675</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -11444,10 +11444,10 @@
         <v>1105000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1501303</v>
+        <v>1501400</v>
       </c>
       <c r="L66" t="n">
-        <v>26.39726957183193</v>
+        <v>26.40202477687492</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -11508,10 +11508,10 @@
         <v>1155000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1587117</v>
+        <v>1587218</v>
       </c>
       <c r="L67" t="n">
-        <v>27.22653717400797</v>
+        <v>27.23116799330653</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -11778,7 +11778,7 @@
         <v>315000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>299917</v>
+        <v>299937</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -11839,10 +11839,10 @@
         <v>380000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>385731</v>
+        <v>385755</v>
       </c>
       <c r="L3" t="n">
-        <v>1.485750432296082</v>
+        <v>1.491879560861168</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -11903,7 +11903,7 @@
         <v>415000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>385731</v>
+        <v>385755</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -11964,10 +11964,10 @@
         <v>495000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>471544</v>
+        <v>471574</v>
       </c>
       <c r="L5" t="n">
-        <v>6.689725667169978</v>
+        <v>6.695661762522954</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -12028,10 +12028,10 @@
         <v>490000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514451</v>
+        <v>514484</v>
       </c>
       <c r="L6" t="n">
-        <v>4.752833603200305</v>
+        <v>4.758942940888346</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -12092,10 +12092,10 @@
         <v>550000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>557357</v>
+        <v>557393</v>
       </c>
       <c r="L7" t="n">
-        <v>6.702526387934483</v>
+        <v>6.708552134669793</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -12156,7 +12156,7 @@
         <v>530000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>471544</v>
+        <v>471574</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -12220,10 +12220,10 @@
         <v>600000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>600264</v>
+        <v>600302</v>
       </c>
       <c r="L9" t="n">
-        <v>8.3736489278051</v>
+        <v>8.379449010664631</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -12284,10 +12284,10 @@
         <v>646000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>728984</v>
+        <v>729031</v>
       </c>
       <c r="L10" t="n">
-        <v>17.00791786925365</v>
+        <v>17.0132682972329</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -12348,7 +12348,7 @@
         <v>615000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>557357</v>
+        <v>557393</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -12412,7 +12412,7 @@
         <v>700000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>643171</v>
+        <v>643212</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -12476,7 +12476,7 @@
         <v>745000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>686077</v>
+        <v>686121</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -12540,7 +12540,7 @@
         <v>930000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>857704</v>
+        <v>857759</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -12611,7 +12611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12660,54 +12660,246 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 MDE34 10 Core CPU 10 Core GPU 24GB 1TB Space Black</t>
+          <t>Macbook Pro 14 MJLV4 M5 Pro 15 Core CPU 16 Core GPU 24GB 2TB Silver</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>643999</v>
+        <v>815000</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>644999</v>
+        <v>775000</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>1000</v>
+        <v>-40000</v>
       </c>
       <c r="F2" t="n">
-        <v>0.16</v>
+        <v>-4.91</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Macbook Pro 14 MJLW4 M5 Pro 15 Core CPU 16 Core GPU 24GB 2TB Space Black</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>790000</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>775000</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>-15000</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-1.9</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>Macbook Pro 14 M5 MJ3D4 10 Core CPU 10 Core GPU 32GB 1TB Space Black</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="n">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>780000</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>769999</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>-10001</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-1.28</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Macbook Pro 16 MGE44 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Silver</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>829999</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>822999</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>-7000</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-0.84</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Macbook Pro 14 M5 MJ3E4 10 Core CPU 10 Core GPU 32GB 1TB Silver</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
         <v>775000</v>
       </c>
-      <c r="D3" s="3" t="n">
-        <v>780000</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0.65</v>
+      <c r="D6" s="3" t="n">
+        <v>769999</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>-5001</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-0.65</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 13 MDH74 M5 10C CPU 8C GPU 16GB 512GB Silver</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>425000</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>420000</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>-5000</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-1.18</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 13 MDHE4 M5 10C CPU 8C GPU 16GB 512GB Midnight</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>420000</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>417999</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>-2001</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-0.48</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 13 MDHH4 M5 10C CPU 8C GPU 16GB 512GB Sky Blue</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>420000</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>417999</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>-2001</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-0.48</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 13 MDHA4 M5 10C CPU 8C GPU 16GB 512GB Starlight</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>420000</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>417999</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>-2001</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-0.48</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Macbook Pro 16 MGEA4 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Space Black</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>825000</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>823000</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>-2000</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-0.24</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F3"/>
-  <conditionalFormatting sqref="E2:E3">
+  <autoFilter ref="A1:F11"/>
+  <conditionalFormatting sqref="E2:E11">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
chore: price data 2026-10-05
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MacBook Pro'!$A$1:$S$93</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MacBook Air'!$A$1:$S$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20261004T095228889941+0000</t>
+          <t>20261005T103324582721+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-04T09:52:28.889941+00:00</t>
+          <t>2026-10-05T10:33:24.582721+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>276.834776</v>
+        <v>277.49233</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -624,7 +624,7 @@
         <v>1445000</v>
       </c>
       <c r="D17" t="n">
-        <v>58.5</v>
+        <v>57.9</v>
       </c>
       <c r="E17" t="n">
         <v>3</v>
@@ -675,7 +675,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 48GB 2TB Space Black</t>
+          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 24GB 4TB Silver</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -684,10 +684,10 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>1155000</v>
+        <v>1260000</v>
       </c>
       <c r="D20" t="n">
-        <v>54.1</v>
+        <v>54</v>
       </c>
       <c r="E20" t="n">
         <v>3</v>
@@ -696,7 +696,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 24GB 4TB Silver</t>
+          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 48GB 2TB Space Black</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -705,10 +705,10 @@
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>1260000</v>
+        <v>1155000</v>
       </c>
       <c r="D21" t="n">
-        <v>54</v>
+        <v>53.7</v>
       </c>
       <c r="E21" t="n">
         <v>3</v>
@@ -729,7 +729,7 @@
         <v>532000</v>
       </c>
       <c r="D22" t="n">
-        <v>51.5</v>
+        <v>51.6</v>
       </c>
       <c r="E22" t="n">
         <v>4</v>
@@ -738,7 +738,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 48GB 1TB Space Black</t>
+          <t>Apple MacBook Pro 16Inch MX2U3 14Core CPU 20Core GPU M4 Pro 48GB 512GB Silver</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -747,19 +747,19 @@
         </is>
       </c>
       <c r="C23" s="3" t="n">
-        <v>995000</v>
+        <v>810000</v>
       </c>
       <c r="D23" t="n">
-        <v>51.2</v>
+        <v>50.6</v>
       </c>
       <c r="E23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 16Inch MX2U3 14Core CPU 20Core GPU M4 Pro 48GB 512GB Silver</t>
+          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 48GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="C24" s="3" t="n">
-        <v>810000</v>
+        <v>995000</v>
       </c>
       <c r="D24" t="n">
-        <v>50.5</v>
+        <v>50.6</v>
       </c>
       <c r="E24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
@@ -792,7 +792,7 @@
         <v>1123000</v>
       </c>
       <c r="D25" t="n">
-        <v>50.4</v>
+        <v>50.5</v>
       </c>
       <c r="E25" t="n">
         <v>4</v>
@@ -834,7 +834,7 @@
         <v>847999</v>
       </c>
       <c r="D27" t="n">
-        <v>47.3</v>
+        <v>47.4</v>
       </c>
       <c r="E27" t="n">
         <v>5</v>
@@ -855,7 +855,7 @@
         <v>644999</v>
       </c>
       <c r="D28" t="n">
-        <v>44.3</v>
+        <v>44.4</v>
       </c>
       <c r="E28" t="n">
         <v>4</v>
@@ -1147,10 +1147,10 @@
         <v>470000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>686121</v>
+        <v>687751</v>
       </c>
       <c r="L2" t="n">
-        <v>35.1426351911689</v>
+        <v>35.29634998713197</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1165,7 +1165,7 @@
         <v>28.4414106939704</v>
       </c>
       <c r="Q2" t="n">
-        <v>35.3</v>
+        <v>35.4</v>
       </c>
       <c r="R2" t="n">
         <v>5</v>
@@ -1214,10 +1214,10 @@
         <v>495000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>686121</v>
+        <v>687751</v>
       </c>
       <c r="L3" t="n">
-        <v>27.85529083062609</v>
+        <v>28.02627695197826</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>771940</v>
+        <v>773773</v>
       </c>
       <c r="L4" t="n">
-        <v>35.22825608207892</v>
+        <v>35.38169463137122</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1299,7 +1299,7 @@
         <v>68.25981228668942</v>
       </c>
       <c r="Q4" t="n">
-        <v>41.7</v>
+        <v>41.8</v>
       </c>
       <c r="R4" t="n">
         <v>5</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>771940</v>
+        <v>773773</v>
       </c>
       <c r="L5" t="n">
-        <v>32.6373811436122</v>
+        <v>32.7969572471513</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>857759</v>
+        <v>859796</v>
       </c>
       <c r="L6" t="n">
-        <v>37.97791687408701</v>
+        <v>38.12485752434298</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1433,7 +1433,7 @@
         <v>100</v>
       </c>
       <c r="Q6" t="n">
-        <v>51.5</v>
+        <v>51.6</v>
       </c>
       <c r="R6" t="n">
         <v>4</v>
@@ -1606,10 +1606,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>857759</v>
+        <v>859796</v>
       </c>
       <c r="L9" t="n">
-        <v>34.1306823944721</v>
+        <v>34.28673778431163</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1673,10 +1673,10 @@
         <v>579999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>857759</v>
+        <v>859796</v>
       </c>
       <c r="L10" t="n">
-        <v>32.38205603205562</v>
+        <v>32.54225420913798</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -1740,10 +1740,10 @@
         <v>587999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>857759</v>
+        <v>859796</v>
       </c>
       <c r="L11" t="n">
-        <v>31.44939312790655</v>
+        <v>31.61180093882735</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -1758,7 +1758,7 @@
         <v>47.60029999999999</v>
       </c>
       <c r="Q11" t="n">
-        <v>18.4</v>
+        <v>18.5</v>
       </c>
       <c r="R11" t="n">
         <v>4</v>
@@ -1807,10 +1807,10 @@
         <v>600000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>857759</v>
+        <v>859796</v>
       </c>
       <c r="L12" t="n">
-        <v>30.05028218881994</v>
+        <v>30.21600472670261</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -1825,7 +1825,7 @@
         <v>45.94594594594595</v>
       </c>
       <c r="Q12" t="n">
-        <v>42</v>
+        <v>42.1</v>
       </c>
       <c r="R12" t="n">
         <v>4</v>
@@ -1874,10 +1874,10 @@
         <v>634000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>857759</v>
+        <v>859796</v>
       </c>
       <c r="L13" t="n">
-        <v>26.0864648461864</v>
+        <v>26.26157832788243</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -1941,10 +1941,10 @@
         <v>644999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>943577</v>
+        <v>945819</v>
       </c>
       <c r="L14" t="n">
-        <v>31.64320452914812</v>
+        <v>31.80523969173806</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -1959,7 +1959,7 @@
         <v>69.20023999999999</v>
       </c>
       <c r="Q14" t="n">
-        <v>44.3</v>
+        <v>44.4</v>
       </c>
       <c r="R14" t="n">
         <v>4</v>
@@ -2067,10 +2067,10 @@
         <v>650000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>943577</v>
+        <v>945819</v>
       </c>
       <c r="L16" t="n">
-        <v>31.11320008859903</v>
+        <v>31.27649159088578</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -2085,7 +2085,7 @@
         <v>68</v>
       </c>
       <c r="Q16" t="n">
-        <v>21.7</v>
+        <v>21.8</v>
       </c>
       <c r="R16" t="n">
         <v>4</v>
@@ -2134,10 +2134,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1029396</v>
+        <v>1031841</v>
       </c>
       <c r="L17" t="n">
-        <v>31.99895861262332</v>
+        <v>32.16009055658769</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2201,10 +2201,10 @@
         <v>711999</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>1072306</v>
+        <v>1074853</v>
       </c>
       <c r="L18" t="n">
-        <v>33.60113624282621</v>
+        <v>33.75847674054033</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -2330,10 +2330,10 @@
         <v>720000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>1029396</v>
+        <v>1031841</v>
       </c>
       <c r="L20" t="n">
-        <v>30.05607171584113</v>
+        <v>30.22180742963305</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -2459,10 +2459,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1072306</v>
+        <v>1074853</v>
       </c>
       <c r="L22" t="n">
-        <v>30.71007716081044</v>
+        <v>30.87426838832845</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2477,7 +2477,7 @@
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>10.2</v>
+        <v>10.3</v>
       </c>
       <c r="R22" t="n">
         <v>4</v>
@@ -2526,13 +2526,13 @@
         <v>769999</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1029396</v>
+        <v>1031841</v>
       </c>
       <c r="L23" t="n">
-        <v>25.1989516182305</v>
+        <v>25.3761965264028</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>-5001</v>
+        <v>0</v>
       </c>
       <c r="N23" t="n">
         <v>0.2591968911917099</v>
@@ -2593,13 +2593,13 @@
         <v>769999</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1029396</v>
+        <v>1031841</v>
       </c>
       <c r="L24" t="n">
-        <v>25.1989516182305</v>
+        <v>25.3761965264028</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>-10001</v>
+        <v>0</v>
       </c>
       <c r="N24" t="n">
         <v>0.2591968911917099</v>
@@ -2660,10 +2660,10 @@
         <v>772000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>1029396</v>
+        <v>1031841</v>
       </c>
       <c r="L25" t="n">
-        <v>25.00456578420744</v>
+        <v>25.182271299551</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -2678,7 +2678,7 @@
         <v>69.59999999999998</v>
       </c>
       <c r="Q25" t="n">
-        <v>19.9</v>
+        <v>20</v>
       </c>
       <c r="R25" t="n">
         <v>4</v>
@@ -2728,7 +2728,7 @@
       </c>
       <c r="K26" s="3" t="n"/>
       <c r="M26" s="3" t="n">
-        <v>-15000</v>
+        <v>0</v>
       </c>
       <c r="N26" t="n">
         <v>1.89873417721519</v>
@@ -2790,7 +2790,7 @@
       </c>
       <c r="K27" s="3" t="n"/>
       <c r="M27" s="3" t="n">
-        <v>-40000</v>
+        <v>0</v>
       </c>
       <c r="N27" t="n">
         <v>4.907975460122699</v>
@@ -2851,16 +2851,16 @@
         <v>810000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>1072306</v>
+        <v>1074853</v>
       </c>
       <c r="L28" t="n">
-        <v>24.46186070021058</v>
+        <v>24.64085786614542</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N28" t="n">
-        <v>2.702702702702703</v>
+        <v>2.409638554216868</v>
       </c>
       <c r="P28" t="n">
         <v>61.99999999999999</v>
@@ -2915,10 +2915,10 @@
         <v>810000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>1243943</v>
+        <v>1246898</v>
       </c>
       <c r="L29" t="n">
-        <v>34.88447621796175</v>
+        <v>35.03879226688952</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -2933,7 +2933,7 @@
         <v>100</v>
       </c>
       <c r="Q29" t="n">
-        <v>50.5</v>
+        <v>50.6</v>
       </c>
       <c r="R29" t="n">
         <v>4</v>
@@ -2982,13 +2982,13 @@
         <v>822999</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1286853</v>
+        <v>1289909</v>
       </c>
       <c r="L30" t="n">
-        <v>36.04560893901635</v>
+        <v>36.19712708415864</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>-7000</v>
+        <v>0</v>
       </c>
       <c r="N30" t="n">
         <v>2.023928571428571</v>
@@ -3000,7 +3000,7 @@
         <v>0.0003521901827191575</v>
       </c>
       <c r="Q30" t="n">
-        <v>34.8</v>
+        <v>34.9</v>
       </c>
       <c r="R30" t="n">
         <v>4</v>
@@ -3049,16 +3049,16 @@
         <v>823000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1286853</v>
+        <v>1289909</v>
       </c>
       <c r="L31" t="n">
-        <v>36.04553123006279</v>
+        <v>36.19704955931</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>-2000</v>
+        <v>0</v>
       </c>
       <c r="N31" t="n">
-        <v>0.5437465521127203</v>
+        <v>0.2424242424242424</v>
       </c>
       <c r="O31" t="n">
         <v>0</v>
@@ -3067,7 +3067,7 @@
         <v>0</v>
       </c>
       <c r="Q31" t="n">
-        <v>12.2</v>
+        <v>12.1</v>
       </c>
       <c r="R31" t="n">
         <v>4</v>
@@ -3116,10 +3116,10 @@
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1372671</v>
+        <v>1375932</v>
       </c>
       <c r="L32" t="n">
-        <v>38.22270595066116</v>
+        <v>38.36911998558069</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3134,7 +3134,7 @@
         <v>100</v>
       </c>
       <c r="Q32" t="n">
-        <v>47.3</v>
+        <v>47.4</v>
       </c>
       <c r="R32" t="n">
         <v>5</v>
@@ -3183,10 +3183,10 @@
         <v>930000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1372671</v>
+        <v>1375932</v>
       </c>
       <c r="L33" t="n">
-        <v>38.07700461363284</v>
+        <v>38.22376396507967</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3250,10 +3250,10 @@
         <v>860000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>1243943</v>
+        <v>1246898</v>
       </c>
       <c r="L34" t="n">
-        <v>30.86499944129273</v>
+        <v>31.02884117225306</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -3383,7 +3383,7 @@
         <v>0</v>
       </c>
       <c r="N36" t="n">
-        <v>0.84985835694051</v>
+        <v>0</v>
       </c>
       <c r="O36" t="n">
         <v>0</v>
@@ -3392,7 +3392,7 @@
         <v>0</v>
       </c>
       <c r="Q36" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="R36" t="n">
         <v>3</v>
@@ -3503,22 +3503,22 @@
         <v>880000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>1158124</v>
+        <v>1160875</v>
       </c>
       <c r="L38" t="n">
-        <v>24.01504502108583</v>
+        <v>24.19511144610746</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N38" t="n">
-        <v>0.5649717514124294</v>
+        <v>0</v>
       </c>
       <c r="P38" t="n">
         <v>73.14285714285714</v>
       </c>
       <c r="Q38" t="n">
-        <v>26.2</v>
+        <v>26</v>
       </c>
       <c r="R38" t="n">
         <v>3</v>
@@ -3567,22 +3567,22 @@
         <v>940000</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>1243943</v>
+        <v>1246898</v>
       </c>
       <c r="L39" t="n">
-        <v>24.43383659862229</v>
+        <v>24.61291942083474</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N39" t="n">
-        <v>1.052631578947368</v>
+        <v>0</v>
       </c>
       <c r="P39" t="n">
         <v>83</v>
       </c>
       <c r="Q39" t="n">
-        <v>28.6</v>
+        <v>28.3</v>
       </c>
       <c r="R39" t="n">
         <v>3</v>
@@ -3631,10 +3631,10 @@
         <v>990000</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>1501400</v>
+        <v>1504966</v>
       </c>
       <c r="L40" t="n">
-        <v>34.06154256027708</v>
+        <v>34.21778299310417</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -3646,7 +3646,7 @@
         <v>39.19647231749141</v>
       </c>
       <c r="Q40" t="n">
-        <v>24.1</v>
+        <v>24.2</v>
       </c>
       <c r="R40" t="n">
         <v>3</v>
@@ -3695,10 +3695,10 @@
         <v>990000</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>1501400</v>
+        <v>1504966</v>
       </c>
       <c r="L41" t="n">
-        <v>34.06154256027708</v>
+        <v>34.21778299310417</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
@@ -3710,7 +3710,7 @@
         <v>39.19647231749141</v>
       </c>
       <c r="Q41" t="n">
-        <v>23</v>
+        <v>23.1</v>
       </c>
       <c r="R41" t="n">
         <v>3</v>
@@ -3763,7 +3763,7 @@
         <v>0</v>
       </c>
       <c r="N42" t="n">
-        <v>1.240694789081886</v>
+        <v>0</v>
       </c>
       <c r="O42" t="n">
         <v>100</v>
@@ -3772,7 +3772,7 @@
         <v>69.23076923076923</v>
       </c>
       <c r="Q42" t="n">
-        <v>51.2</v>
+        <v>50.6</v>
       </c>
       <c r="R42" t="n">
         <v>3</v>
@@ -3821,22 +3821,22 @@
         <v>1055000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1544309</v>
+        <v>1547977</v>
       </c>
       <c r="L43" t="n">
-        <v>31.68465637382156</v>
+        <v>31.84653260352059</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>0.3777148253068933</v>
+        <v>0</v>
       </c>
       <c r="P43" t="n">
         <v>57.6271186440678</v>
       </c>
       <c r="Q43" t="n">
-        <v>26.1</v>
+        <v>26</v>
       </c>
       <c r="R43" t="n">
         <v>3</v>
@@ -3885,22 +3885,22 @@
         <v>1055000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1544309</v>
+        <v>1547977</v>
       </c>
       <c r="L44" t="n">
-        <v>31.68465637382156</v>
+        <v>31.84653260352059</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>1.17096018735363</v>
+        <v>0</v>
       </c>
       <c r="P44" t="n">
         <v>57.6271186440678</v>
       </c>
       <c r="Q44" t="n">
-        <v>26.3</v>
+        <v>26</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -3953,7 +3953,7 @@
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>1.624129930394431</v>
+        <v>0</v>
       </c>
       <c r="O45" t="n">
         <v>0</v>
@@ -3962,7 +3962,7 @@
         <v>58.11965811965813</v>
       </c>
       <c r="Q45" t="n">
-        <v>15.2</v>
+        <v>14.5</v>
       </c>
       <c r="R45" t="n">
         <v>3</v>
@@ -4011,10 +4011,10 @@
         <v>1115000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1501400</v>
+        <v>1504966</v>
       </c>
       <c r="L46" t="n">
-        <v>25.73597975223125</v>
+        <v>25.9119475124355</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -4026,7 +4026,7 @@
         <v>9.358196283135744</v>
       </c>
       <c r="Q46" t="n">
-        <v>14.1</v>
+        <v>14.2</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -4075,10 +4075,10 @@
         <v>1123000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1715947</v>
+        <v>1720022</v>
       </c>
       <c r="L47" t="n">
-        <v>34.55508823990485</v>
+        <v>34.71013742847475</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -4093,7 +4093,7 @@
         <v>100</v>
       </c>
       <c r="Q47" t="n">
-        <v>50.4</v>
+        <v>50.5</v>
       </c>
       <c r="R47" t="n">
         <v>4</v>
@@ -4142,22 +4142,22 @@
         <v>1130000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1501400</v>
+        <v>1504966</v>
       </c>
       <c r="L48" t="n">
-        <v>24.73691221526575</v>
+        <v>24.91524725475526</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N48" t="n">
-        <v>0.8771929824561403</v>
+        <v>0</v>
       </c>
       <c r="P48" t="n">
         <v>88.39999999999999</v>
       </c>
       <c r="Q48" t="n">
-        <v>29.9</v>
+        <v>29.6</v>
       </c>
       <c r="R48" t="n">
         <v>3</v>
@@ -4210,7 +4210,7 @@
         <v>0</v>
       </c>
       <c r="N49" t="n">
-        <v>1.070663811563169</v>
+        <v>0</v>
       </c>
       <c r="O49" t="n">
         <v>100</v>
@@ -4219,7 +4219,7 @@
         <v>81.36752136752136</v>
       </c>
       <c r="Q49" t="n">
-        <v>54.1</v>
+        <v>53.7</v>
       </c>
       <c r="R49" t="n">
         <v>3</v>
@@ -4268,10 +4268,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1758856</v>
+        <v>1763034</v>
       </c>
       <c r="L50" t="n">
-        <v>34.33231600540351</v>
+        <v>34.48793386854706</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4283,7 +4283,7 @@
         <v>22.53136001640632</v>
       </c>
       <c r="Q50" t="n">
-        <v>19.5</v>
+        <v>19.6</v>
       </c>
       <c r="R50" t="n">
         <v>3</v>
@@ -4332,10 +4332,10 @@
         <v>1155000</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>1758856</v>
+        <v>1763034</v>
       </c>
       <c r="L51" t="n">
-        <v>34.33231600540351</v>
+        <v>34.48793386854706</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -4347,7 +4347,7 @@
         <v>22.53136001640632</v>
       </c>
       <c r="Q51" t="n">
-        <v>19.5</v>
+        <v>19.6</v>
       </c>
       <c r="R51" t="n">
         <v>3</v>
@@ -4396,22 +4396,22 @@
         <v>1185000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1587218</v>
+        <v>1590988</v>
       </c>
       <c r="L52" t="n">
-        <v>25.34106846066514</v>
+        <v>25.5179800224766</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N52" t="n">
-        <v>1.25</v>
+        <v>0</v>
       </c>
       <c r="P52" t="n">
         <v>77.26495726495727</v>
       </c>
       <c r="Q52" t="n">
-        <v>27.9</v>
+        <v>27.5</v>
       </c>
       <c r="R52" t="n">
         <v>3</v>
@@ -4460,22 +4460,22 @@
         <v>1185000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1587218</v>
+        <v>1590988</v>
       </c>
       <c r="L53" t="n">
-        <v>25.34106846066514</v>
+        <v>25.5179800224766</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N53" t="n">
-        <v>1.04384133611691</v>
+        <v>0</v>
       </c>
       <c r="P53" t="n">
         <v>94.72727272727272</v>
       </c>
       <c r="Q53" t="n">
-        <v>31.5</v>
+        <v>31.2</v>
       </c>
       <c r="R53" t="n">
         <v>3</v>
@@ -4524,10 +4524,10 @@
         <v>1200000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1887584</v>
+        <v>1892068</v>
       </c>
       <c r="L54" t="n">
-        <v>36.42667028328276</v>
+        <v>36.57733231575187</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -4588,10 +4588,10 @@
         <v>1200000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1887584</v>
+        <v>1892068</v>
       </c>
       <c r="L55" t="n">
-        <v>36.42667028328276</v>
+        <v>36.57733231575187</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -4656,7 +4656,7 @@
         <v>0</v>
       </c>
       <c r="N56" t="n">
-        <v>1.425661914460285</v>
+        <v>0</v>
       </c>
       <c r="O56" t="n">
         <v>0</v>
@@ -4665,7 +4665,7 @@
         <v>73.84615384615385</v>
       </c>
       <c r="Q56" t="n">
-        <v>19.1</v>
+        <v>18.5</v>
       </c>
       <c r="R56" t="n">
         <v>3</v>
@@ -4714,22 +4714,22 @@
         <v>1240000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1673037</v>
+        <v>1677011</v>
       </c>
       <c r="L57" t="n">
-        <v>25.88328889319244</v>
+        <v>26.05892269042958</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N57" t="n">
-        <v>1.587301587301587</v>
+        <v>0</v>
       </c>
       <c r="P57" t="n">
         <v>100</v>
       </c>
       <c r="Q57" t="n">
-        <v>33.1</v>
+        <v>32.6</v>
       </c>
       <c r="R57" t="n">
         <v>3</v>
@@ -4840,10 +4840,10 @@
         <v>1280000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1715947</v>
+        <v>1720022</v>
       </c>
       <c r="L59" t="n">
-        <v>25.40562150229582</v>
+        <v>25.58234720253578</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -4907,10 +4907,10 @@
         <v>1298000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1758856</v>
+        <v>1763034</v>
       </c>
       <c r="L60" t="n">
-        <v>26.20203132035823</v>
+        <v>26.37691615703384</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -4922,7 +4922,7 @@
         <v>61.28109178956637</v>
       </c>
       <c r="Q60" t="n">
-        <v>25.4</v>
+        <v>25.5</v>
       </c>
       <c r="R60" t="n">
         <v>3</v>
@@ -4971,10 +4971,10 @@
         <v>1300000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1715947</v>
+        <v>1720022</v>
       </c>
       <c r="L61" t="n">
-        <v>24.24008433826919</v>
+        <v>24.4195713775754</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -4986,7 +4986,7 @@
         <v>60.92890160686771</v>
       </c>
       <c r="Q61" t="n">
-        <v>23.7</v>
+        <v>23.8</v>
       </c>
       <c r="R61" t="n">
         <v>3</v>
@@ -5039,7 +5039,7 @@
         <v>0</v>
       </c>
       <c r="N62" t="n">
-        <v>1.845018450184502</v>
+        <v>0</v>
       </c>
       <c r="O62" t="n">
         <v>0</v>
@@ -5048,7 +5048,7 @@
         <v>73.97047397047398</v>
       </c>
       <c r="Q62" t="n">
-        <v>19.3</v>
+        <v>18.5</v>
       </c>
       <c r="R62" t="n">
         <v>3</v>
@@ -5097,22 +5097,22 @@
         <v>1335000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1801765</v>
+        <v>1806045</v>
       </c>
       <c r="L63" t="n">
-        <v>25.90598662977691</v>
+        <v>26.08157604046411</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N63" t="n">
-        <v>1.293900184842884</v>
+        <v>0</v>
       </c>
       <c r="P63" t="n">
         <v>87.17948717948718</v>
       </c>
       <c r="Q63" t="n">
-        <v>30.2</v>
+        <v>29.9</v>
       </c>
       <c r="R63" t="n">
         <v>3</v>
@@ -5161,10 +5161,10 @@
         <v>1420000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1930493</v>
+        <v>1935079</v>
       </c>
       <c r="L64" t="n">
-        <v>26.44365972836991</v>
+        <v>26.61798303841859</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -5176,7 +5176,7 @@
         <v>81.47332893095606</v>
       </c>
       <c r="Q64" t="n">
-        <v>30</v>
+        <v>30.1</v>
       </c>
       <c r="R64" t="n">
         <v>3</v>
@@ -5225,10 +5225,10 @@
         <v>1430000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1930493</v>
+        <v>1935079</v>
       </c>
       <c r="L65" t="n">
-        <v>25.92565733209082</v>
+        <v>26.1012082710835</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -5289,10 +5289,10 @@
         <v>1430000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>2145040</v>
+        <v>2150135</v>
       </c>
       <c r="L66" t="n">
-        <v>33.33457651139373</v>
+        <v>33.49254814232594</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -5304,7 +5304,7 @@
         <v>0</v>
       </c>
       <c r="Q66" t="n">
-        <v>14.3</v>
+        <v>14.4</v>
       </c>
       <c r="R66" t="n">
         <v>3</v>
@@ -5353,10 +5353,10 @@
         <v>1430000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>2145040</v>
+        <v>2150135</v>
       </c>
       <c r="L67" t="n">
-        <v>33.33457651139373</v>
+        <v>33.49254814232594</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -5368,7 +5368,7 @@
         <v>0</v>
       </c>
       <c r="Q67" t="n">
-        <v>14.3</v>
+        <v>14.4</v>
       </c>
       <c r="R67" t="n">
         <v>3</v>
@@ -5421,7 +5421,7 @@
         <v>0</v>
       </c>
       <c r="N68" t="n">
-        <v>1.533219761499148</v>
+        <v>0</v>
       </c>
       <c r="O68" t="n">
         <v>100</v>
@@ -5430,7 +5430,7 @@
         <v>98.16849816849818</v>
       </c>
       <c r="Q68" t="n">
-        <v>58.5</v>
+        <v>57.9</v>
       </c>
       <c r="R68" t="n">
         <v>3</v>
@@ -5479,22 +5479,22 @@
         <v>1480000</v>
       </c>
       <c r="K69" s="3" t="n">
-        <v>2016312</v>
+        <v>2021102</v>
       </c>
       <c r="L69" t="n">
-        <v>26.59866131828804</v>
+        <v>26.77262206459644</v>
       </c>
       <c r="M69" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N69" t="n">
-        <v>1.824212271973466</v>
+        <v>0</v>
       </c>
       <c r="P69" t="n">
         <v>0</v>
       </c>
       <c r="Q69" t="n">
-        <v>12.1</v>
+        <v>11.5</v>
       </c>
       <c r="R69" t="n">
         <v>3</v>
@@ -5547,7 +5547,7 @@
         <v>0</v>
       </c>
       <c r="N70" t="n">
-        <v>1.463414634146342</v>
+        <v>0</v>
       </c>
       <c r="O70" t="n">
         <v>0</v>
@@ -5556,7 +5556,7 @@
         <v>91.33089133089133</v>
       </c>
       <c r="Q70" t="n">
-        <v>23.4</v>
+        <v>22.8</v>
       </c>
       <c r="R70" t="n">
         <v>3</v>
@@ -5605,22 +5605,22 @@
         <v>1605000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2187950</v>
+        <v>2193147</v>
       </c>
       <c r="L71" t="n">
-        <v>26.64366187527137</v>
+        <v>26.81749103001303</v>
       </c>
       <c r="M71" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N71" t="n">
-        <v>1.382488479262673</v>
+        <v>0</v>
       </c>
       <c r="P71" t="n">
         <v>36.44392794886694</v>
       </c>
       <c r="Q71" t="n">
-        <v>19.7</v>
+        <v>19.3</v>
       </c>
       <c r="R71" t="n">
         <v>3</v>
@@ -5669,22 +5669,22 @@
         <v>1610000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2187950</v>
+        <v>2193147</v>
       </c>
       <c r="L72" t="n">
-        <v>26.41513745743732</v>
+        <v>26.58950813602554</v>
       </c>
       <c r="M72" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N72" t="n">
-        <v>1.529051987767584</v>
+        <v>0</v>
       </c>
       <c r="P72" t="n">
         <v>25.72147975982957</v>
       </c>
       <c r="Q72" t="n">
-        <v>17.4</v>
+        <v>16.9</v>
       </c>
       <c r="R72" t="n">
         <v>3</v>
@@ -5733,10 +5733,10 @@
         <v>1615000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2187950</v>
+        <v>2193147</v>
       </c>
       <c r="L73" t="n">
-        <v>26.18661303960328</v>
+        <v>26.36152524203804</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
@@ -5748,7 +5748,7 @@
         <v>86.7142542687337</v>
       </c>
       <c r="Q73" t="n">
-        <v>30.8</v>
+        <v>30.9</v>
       </c>
       <c r="R73" t="n">
         <v>3</v>
@@ -5797,22 +5797,22 @@
         <v>1630000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2230859</v>
+        <v>2236158</v>
       </c>
       <c r="L74" t="n">
-        <v>26.93397476039499</v>
+        <v>27.10711854886819</v>
       </c>
       <c r="M74" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N74" t="n">
-        <v>1.510574018126888</v>
+        <v>0</v>
       </c>
       <c r="P74" t="n">
         <v>100</v>
       </c>
       <c r="Q74" t="n">
-        <v>33.5</v>
+        <v>33</v>
       </c>
       <c r="R74" t="n">
         <v>3</v>
@@ -5861,10 +5861,10 @@
         <v>1690000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2316678</v>
+        <v>2322181</v>
       </c>
       <c r="L75" t="n">
-        <v>27.05071658642246</v>
+        <v>27.22358851441813</v>
       </c>
       <c r="M75" s="3" t="n">
         <v>0</v>
@@ -5925,10 +5925,10 @@
         <v>1705000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2316678</v>
+        <v>2322181</v>
       </c>
       <c r="L76" t="n">
-        <v>26.40323773955638</v>
+        <v>26.57764403377686</v>
       </c>
       <c r="M76" s="3" t="n">
         <v>0</v>
@@ -5940,7 +5940,7 @@
         <v>1.9846639603067</v>
       </c>
       <c r="Q76" t="n">
-        <v>12.8</v>
+        <v>12.9</v>
       </c>
       <c r="R76" t="n">
         <v>3</v>
@@ -5989,10 +5989,10 @@
         <v>1725000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2359587</v>
+        <v>2365192</v>
       </c>
       <c r="L77" t="n">
-        <v>26.89398610858596</v>
+        <v>27.06723175116439</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
@@ -6053,22 +6053,22 @@
         <v>1780000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2445406</v>
+        <v>2451215</v>
       </c>
       <c r="L78" t="n">
-        <v>27.21045094352431</v>
+        <v>27.38295090393947</v>
       </c>
       <c r="M78" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N78" t="n">
-        <v>1.657458563535912</v>
+        <v>0</v>
       </c>
       <c r="P78" t="n">
         <v>38.78143936249688</v>
       </c>
       <c r="Q78" t="n">
-        <v>20.6</v>
+        <v>20</v>
       </c>
       <c r="R78" t="n">
         <v>3</v>
@@ -6117,10 +6117,10 @@
         <v>1875000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2574134</v>
+        <v>2580249</v>
       </c>
       <c r="L79" t="n">
-        <v>27.15996913913573</v>
+        <v>27.33259464493543</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
@@ -6132,7 +6132,7 @@
         <v>19.64044075004835</v>
       </c>
       <c r="Q79" t="n">
-        <v>17.1</v>
+        <v>17.2</v>
       </c>
       <c r="R79" t="n">
         <v>3</v>
@@ -6181,22 +6181,22 @@
         <v>1910000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2617044</v>
+        <v>2623260</v>
       </c>
       <c r="L80" t="n">
-        <v>27.01689386957193</v>
+        <v>27.18983249849424</v>
       </c>
       <c r="M80" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N80" t="n">
-        <v>1.291989664082687</v>
+        <v>0</v>
       </c>
       <c r="P80" t="n">
         <v>53.22486926205694</v>
       </c>
       <c r="Q80" t="n">
-        <v>23.4</v>
+        <v>23.1</v>
       </c>
       <c r="R80" t="n">
         <v>3</v>
@@ -6245,10 +6245,10 @@
         <v>2020000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2745772</v>
+        <v>2752294</v>
       </c>
       <c r="L81" t="n">
-        <v>26.43234762391051</v>
+        <v>26.60667792030938</v>
       </c>
       <c r="M81" s="3" t="n">
         <v>0</v>
@@ -6260,7 +6260,7 @@
         <v>36.26522327469554</v>
       </c>
       <c r="Q81" t="n">
-        <v>20.1</v>
+        <v>20.2</v>
       </c>
       <c r="R81" t="n">
         <v>3</v>
@@ -6309,22 +6309,22 @@
         <v>2110000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>2874500</v>
+        <v>2881328</v>
       </c>
       <c r="L82" t="n">
-        <v>26.59592972690903</v>
+        <v>26.76987833387938</v>
       </c>
       <c r="M82" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N82" t="n">
-        <v>1.401869158878505</v>
+        <v>0</v>
       </c>
       <c r="P82" t="n">
         <v>79.02382335851249</v>
       </c>
       <c r="Q82" t="n">
-        <v>28.8</v>
+        <v>28.4</v>
       </c>
       <c r="R82" t="n">
         <v>3</v>
@@ -6373,10 +6373,10 @@
         <v>2210000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3003228</v>
+        <v>3010362</v>
       </c>
       <c r="L83" t="n">
-        <v>26.41251346884086</v>
+        <v>26.58690217322701</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
@@ -6388,7 +6388,7 @@
         <v>70.36535859269283</v>
       </c>
       <c r="Q83" t="n">
-        <v>27.3</v>
+        <v>27.4</v>
       </c>
       <c r="R83" t="n">
         <v>3</v>
@@ -6437,22 +6437,22 @@
         <v>2215000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3046138</v>
+        <v>3053373</v>
       </c>
       <c r="L84" t="n">
-        <v>27.2849752703259</v>
+        <v>27.45727429960244</v>
       </c>
       <c r="M84" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N84" t="n">
-        <v>1.226309921962096</v>
+        <v>0</v>
       </c>
       <c r="P84" t="n">
         <v>74.28466149856153</v>
       </c>
       <c r="Q84" t="n">
-        <v>28</v>
+        <v>27.7</v>
       </c>
       <c r="R84" t="n">
         <v>3</v>
@@ -6501,10 +6501,10 @@
         <v>2315000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3174866</v>
+        <v>3182407</v>
       </c>
       <c r="L85" t="n">
-        <v>27.08353675399214</v>
+        <v>27.256318880646</v>
       </c>
       <c r="M85" s="3" t="n">
         <v>0</v>
@@ -6516,7 +6516,7 @@
         <v>65.11105977094954</v>
       </c>
       <c r="Q85" t="n">
-        <v>26.5</v>
+        <v>26.6</v>
       </c>
       <c r="R85" t="n">
         <v>3</v>
@@ -6565,22 +6565,22 @@
         <v>2395000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3303594</v>
+        <v>3311441</v>
       </c>
       <c r="L86" t="n">
-        <v>27.50319803220371</v>
+        <v>27.6749910386445</v>
       </c>
       <c r="M86" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N86" t="n">
-        <v>1.743589743589744</v>
+        <v>0</v>
       </c>
       <c r="P86" t="n">
         <v>72.76953145634144</v>
       </c>
       <c r="Q86" t="n">
-        <v>28</v>
+        <v>27.5</v>
       </c>
       <c r="R86" t="n">
         <v>3</v>
@@ -6629,22 +6629,22 @@
         <v>2410000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3303594</v>
+        <v>3311441</v>
       </c>
       <c r="L87" t="n">
-        <v>27.04914708042211</v>
+        <v>27.22201603471117</v>
       </c>
       <c r="M87" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N87" t="n">
-        <v>1.229508196721312</v>
+        <v>0</v>
       </c>
       <c r="P87" t="n">
         <v>88.47569242688358</v>
       </c>
       <c r="Q87" t="n">
-        <v>31</v>
+        <v>30.6</v>
       </c>
       <c r="R87" t="n">
         <v>3</v>
@@ -6693,10 +6693,10 @@
         <v>2499000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3432322</v>
+        <v>3440475</v>
       </c>
       <c r="L88" t="n">
-        <v>27.19214572525538</v>
+        <v>27.36468074902448</v>
       </c>
       <c r="M88" s="3" t="n">
         <v>0</v>
@@ -6708,7 +6708,7 @@
         <v>63.67326854471646</v>
       </c>
       <c r="Q88" t="n">
-        <v>26.4</v>
+        <v>26.5</v>
       </c>
       <c r="R88" t="n">
         <v>3</v>
@@ -6757,10 +6757,10 @@
         <v>2510000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3432322</v>
+        <v>3440475</v>
       </c>
       <c r="L89" t="n">
-        <v>26.87166297334574</v>
+        <v>27.04495745500258</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
@@ -6772,7 +6772,7 @@
         <v>83.17546233649077</v>
       </c>
       <c r="Q89" t="n">
-        <v>30.2</v>
+        <v>30.3</v>
       </c>
       <c r="R89" t="n">
         <v>3</v>
@@ -6821,22 +6821,22 @@
         <v>2530000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3475232</v>
+        <v>3483486</v>
       </c>
       <c r="L90" t="n">
-        <v>27.19910498061712</v>
+        <v>27.37160419189284</v>
       </c>
       <c r="M90" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N90" t="n">
-        <v>0.9784735812133072</v>
+        <v>0</v>
       </c>
       <c r="P90" t="n">
         <v>79.17877203176447</v>
       </c>
       <c r="Q90" t="n">
-        <v>29</v>
+        <v>28.7</v>
       </c>
       <c r="R90" t="n">
         <v>3</v>
@@ -6885,10 +6885,10 @@
         <v>2610000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>3603960</v>
+        <v>3612520</v>
       </c>
       <c r="L91" t="n">
-        <v>27.57966237139147</v>
+        <v>27.75126504489941</v>
       </c>
       <c r="M91" s="3" t="n">
         <v>0</v>
@@ -6900,7 +6900,7 @@
         <v>74.15426251691474</v>
       </c>
       <c r="Q91" t="n">
-        <v>28.4</v>
+        <v>28.5</v>
       </c>
       <c r="R91" t="n">
         <v>3</v>
@@ -6949,22 +6949,22 @@
         <v>3015000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4161782</v>
+        <v>4171667</v>
       </c>
       <c r="L92" t="n">
-        <v>27.55507136125823</v>
+        <v>27.7267337014196</v>
       </c>
       <c r="M92" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N92" t="n">
-        <v>1.228501228501228</v>
+        <v>0</v>
       </c>
       <c r="P92" t="n">
         <v>100</v>
       </c>
       <c r="Q92" t="n">
-        <v>33.7</v>
+        <v>33.3</v>
       </c>
       <c r="R92" t="n">
         <v>3</v>
@@ -7013,10 +7013,10 @@
         <v>3098000</v>
       </c>
       <c r="K93" s="3" t="n">
-        <v>4290510</v>
+        <v>4300701</v>
       </c>
       <c r="L93" t="n">
-        <v>27.79413169996108</v>
+        <v>27.96523171455072</v>
       </c>
       <c r="M93" s="3" t="n">
         <v>0</v>
@@ -7028,7 +7028,7 @@
         <v>100</v>
       </c>
       <c r="Q93" t="n">
-        <v>34.3</v>
+        <v>34.4</v>
       </c>
       <c r="R93" t="n">
         <v>3</v>
@@ -7312,10 +7312,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>428665</v>
+        <v>429683</v>
       </c>
       <c r="L2" t="n">
-        <v>27.6826892795073</v>
+        <v>27.85402261667322</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7330,7 +7330,7 @@
         <v>29.71702857142851</v>
       </c>
       <c r="Q2" t="n">
-        <v>36.4</v>
+        <v>36.5</v>
       </c>
       <c r="R2" t="n">
         <v>4</v>
@@ -7379,10 +7379,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>428665</v>
+        <v>429683</v>
       </c>
       <c r="L3" t="n">
-        <v>27.6826892795073</v>
+        <v>27.85402261667322</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7397,7 +7397,7 @@
         <v>29.71702857142851</v>
       </c>
       <c r="Q3" t="n">
-        <v>36.4</v>
+        <v>36.5</v>
       </c>
       <c r="R3" t="n">
         <v>4</v>
@@ -7446,10 +7446,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>428665</v>
+        <v>429683</v>
       </c>
       <c r="L4" t="n">
-        <v>27.6824559971073</v>
+        <v>27.85378988696318</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7513,10 +7513,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>428665</v>
+        <v>429683</v>
       </c>
       <c r="L5" t="n">
-        <v>27.6824559971073</v>
+        <v>27.85378988696318</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7580,10 +7580,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514484</v>
+        <v>515706</v>
       </c>
       <c r="L6" t="n">
-        <v>25.36211038632883</v>
+        <v>25.53896987818641</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7644,10 +7644,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>514484</v>
+        <v>515706</v>
       </c>
       <c r="L7" t="n">
-        <v>25.36211038632883</v>
+        <v>25.53896987818641</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7708,10 +7708,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>514484</v>
+        <v>515706</v>
       </c>
       <c r="L8" t="n">
-        <v>25.36211038632883</v>
+        <v>25.53896987818641</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7772,10 +7772,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>514484</v>
+        <v>515706</v>
       </c>
       <c r="L9" t="n">
-        <v>25.36211038632883</v>
+        <v>25.53896987818641</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7836,10 +7836,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>514484</v>
+        <v>515706</v>
       </c>
       <c r="L10" t="n">
-        <v>25.16774088212656</v>
+        <v>25.34506094557752</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7851,7 +7851,7 @@
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>10.8</v>
+        <v>10.9</v>
       </c>
       <c r="R10" t="n">
         <v>3</v>
@@ -7900,10 +7900,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>514484</v>
+        <v>515706</v>
       </c>
       <c r="L11" t="n">
-        <v>25.16774088212656</v>
+        <v>25.34506094557752</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7915,7 +7915,7 @@
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>10.8</v>
+        <v>10.9</v>
       </c>
       <c r="R11" t="n">
         <v>3</v>
@@ -7964,10 +7964,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>514484</v>
+        <v>515706</v>
       </c>
       <c r="L12" t="n">
-        <v>25.16774088212656</v>
+        <v>25.34506094557752</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -7979,7 +7979,7 @@
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>10.8</v>
+        <v>10.9</v>
       </c>
       <c r="R12" t="n">
         <v>3</v>
@@ -8028,10 +8028,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>514484</v>
+        <v>515706</v>
       </c>
       <c r="L13" t="n">
-        <v>25.16774088212656</v>
+        <v>25.34506094557752</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -8043,7 +8043,7 @@
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>10.8</v>
+        <v>10.9</v>
       </c>
       <c r="R13" t="n">
         <v>3</v>
@@ -8092,16 +8092,16 @@
         <v>417999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>557393</v>
+        <v>558717</v>
       </c>
       <c r="L14" t="n">
-        <v>25.00820785334584</v>
+        <v>25.18591702060256</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>-2001</v>
+        <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>2.677651545578051</v>
+        <v>1.647294117647059</v>
       </c>
       <c r="O14" t="n">
         <v>100</v>
@@ -8110,7 +8110,7 @@
         <v>1.392</v>
       </c>
       <c r="Q14" t="n">
-        <v>31.5</v>
+        <v>31.3</v>
       </c>
       <c r="R14" t="n">
         <v>4</v>
@@ -8159,16 +8159,16 @@
         <v>417999</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>557393</v>
+        <v>558717</v>
       </c>
       <c r="L15" t="n">
-        <v>25.00820785334584</v>
+        <v>25.18591702060256</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>-2001</v>
+        <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>2.564222102822964</v>
+        <v>1.647294117647059</v>
       </c>
       <c r="O15" t="n">
         <v>100</v>
@@ -8177,7 +8177,7 @@
         <v>1.392</v>
       </c>
       <c r="Q15" t="n">
-        <v>31.5</v>
+        <v>31.3</v>
       </c>
       <c r="R15" t="n">
         <v>4</v>
@@ -8226,16 +8226,16 @@
         <v>417999</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>557393</v>
+        <v>558717</v>
       </c>
       <c r="L16" t="n">
-        <v>25.00820785334584</v>
+        <v>25.18591702060256</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>-2001</v>
+        <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>2.222456140350877</v>
+        <v>1.647294117647059</v>
       </c>
       <c r="O16" t="n">
         <v>100</v>
@@ -8244,7 +8244,7 @@
         <v>1.392</v>
       </c>
       <c r="Q16" t="n">
-        <v>31.4</v>
+        <v>31.3</v>
       </c>
       <c r="R16" t="n">
         <v>4</v>
@@ -8293,16 +8293,16 @@
         <v>420000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>557393</v>
+        <v>558717</v>
       </c>
       <c r="L17" t="n">
-        <v>24.64921518569484</v>
+        <v>24.82777506322521</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>-5000</v>
+        <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>3.225806451612903</v>
+        <v>1.176470588235294</v>
       </c>
       <c r="O17" t="n">
         <v>0</v>
@@ -8311,7 +8311,7 @@
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>9.1</v>
+        <v>8.6</v>
       </c>
       <c r="R17" t="n">
         <v>4</v>
@@ -8360,10 +8360,10 @@
         <v>454000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>600302</v>
+        <v>601728</v>
       </c>
       <c r="L18" t="n">
-        <v>24.37139972880317</v>
+        <v>24.55062752605829</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -8375,7 +8375,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q18" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="R18" t="n">
         <v>3</v>
@@ -8424,10 +8424,10 @@
         <v>454000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>600302</v>
+        <v>601728</v>
       </c>
       <c r="L19" t="n">
-        <v>24.37139972880317</v>
+        <v>24.55062752605829</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -8439,7 +8439,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q19" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="R19" t="n">
         <v>3</v>
@@ -8488,10 +8488,10 @@
         <v>454000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>600302</v>
+        <v>601728</v>
       </c>
       <c r="L20" t="n">
-        <v>24.37139972880317</v>
+        <v>24.55062752605829</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -8503,7 +8503,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q20" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="R20" t="n">
         <v>3</v>
@@ -8552,10 +8552,10 @@
         <v>454000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>600302</v>
+        <v>601728</v>
       </c>
       <c r="L21" t="n">
-        <v>24.37139972880317</v>
+        <v>24.55062752605829</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -8567,7 +8567,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q21" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="R21" t="n">
         <v>3</v>
@@ -8616,10 +8616,10 @@
         <v>455000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>600302</v>
+        <v>601728</v>
       </c>
       <c r="L22" t="n">
-        <v>24.20481690882256</v>
+        <v>24.3844394809615</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -8631,7 +8631,7 @@
         <v>100</v>
       </c>
       <c r="Q22" t="n">
-        <v>31.8</v>
+        <v>31.9</v>
       </c>
       <c r="R22" t="n">
         <v>3</v>
@@ -8680,10 +8680,10 @@
         <v>455000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>600302</v>
+        <v>601728</v>
       </c>
       <c r="L23" t="n">
-        <v>24.20481690882256</v>
+        <v>24.3844394809615</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -8695,7 +8695,7 @@
         <v>100</v>
       </c>
       <c r="Q23" t="n">
-        <v>31.8</v>
+        <v>31.9</v>
       </c>
       <c r="R23" t="n">
         <v>3</v>
@@ -8744,10 +8744,10 @@
         <v>455000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>600302</v>
+        <v>601728</v>
       </c>
       <c r="L24" t="n">
-        <v>24.20481690882256</v>
+        <v>24.3844394809615</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -8759,7 +8759,7 @@
         <v>100</v>
       </c>
       <c r="Q24" t="n">
-        <v>31.8</v>
+        <v>31.9</v>
       </c>
       <c r="R24" t="n">
         <v>3</v>
@@ -8808,10 +8808,10 @@
         <v>455000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>600302</v>
+        <v>601728</v>
       </c>
       <c r="L25" t="n">
-        <v>24.20481690882256</v>
+        <v>24.3844394809615</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -8823,7 +8823,7 @@
         <v>100</v>
       </c>
       <c r="Q25" t="n">
-        <v>31.8</v>
+        <v>31.9</v>
       </c>
       <c r="R25" t="n">
         <v>3</v>
@@ -8872,10 +8872,10 @@
         <v>475000</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>686121</v>
+        <v>687751</v>
       </c>
       <c r="L26" t="n">
-        <v>30.77022857484321</v>
+        <v>30.93430616603974</v>
       </c>
       <c r="M26" s="3" t="n">
         <v>0</v>
@@ -8887,7 +8887,7 @@
         <v>100</v>
       </c>
       <c r="Q26" t="n">
-        <v>34.6</v>
+        <v>34.7</v>
       </c>
       <c r="R26" t="n">
         <v>3</v>
@@ -8936,10 +8936,10 @@
         <v>475000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>686121</v>
+        <v>687751</v>
       </c>
       <c r="L27" t="n">
-        <v>30.77022857484321</v>
+        <v>30.93430616603974</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -8951,7 +8951,7 @@
         <v>100</v>
       </c>
       <c r="Q27" t="n">
-        <v>34.6</v>
+        <v>34.7</v>
       </c>
       <c r="R27" t="n">
         <v>3</v>
@@ -9000,10 +9000,10 @@
         <v>475000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>686121</v>
+        <v>687751</v>
       </c>
       <c r="L28" t="n">
-        <v>30.77022857484321</v>
+        <v>30.93430616603974</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -9015,7 +9015,7 @@
         <v>100</v>
       </c>
       <c r="Q28" t="n">
-        <v>34.6</v>
+        <v>34.7</v>
       </c>
       <c r="R28" t="n">
         <v>3</v>
@@ -9064,10 +9064,10 @@
         <v>475000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>686121</v>
+        <v>687751</v>
       </c>
       <c r="L29" t="n">
-        <v>30.77022857484321</v>
+        <v>30.93430616603974</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -9079,7 +9079,7 @@
         <v>100</v>
       </c>
       <c r="Q29" t="n">
-        <v>34.6</v>
+        <v>34.7</v>
       </c>
       <c r="R29" t="n">
         <v>3</v>
@@ -9128,10 +9128,10 @@
         <v>477000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>643212</v>
+        <v>644740</v>
       </c>
       <c r="L30" t="n">
-        <v>25.8409358034365</v>
+        <v>26.0166888978503</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -9146,7 +9146,7 @@
         <v>1.568112774445864</v>
       </c>
       <c r="Q30" t="n">
-        <v>31.4</v>
+        <v>31.5</v>
       </c>
       <c r="R30" t="n">
         <v>4</v>
@@ -9195,10 +9195,10 @@
         <v>477000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>643212</v>
+        <v>644740</v>
       </c>
       <c r="L31" t="n">
-        <v>25.8409358034365</v>
+        <v>26.0166888978503</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -9213,7 +9213,7 @@
         <v>1.568112774445864</v>
       </c>
       <c r="Q31" t="n">
-        <v>31.4</v>
+        <v>31.5</v>
       </c>
       <c r="R31" t="n">
         <v>4</v>
@@ -9262,10 +9262,10 @@
         <v>477000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>643212</v>
+        <v>644740</v>
       </c>
       <c r="L32" t="n">
-        <v>25.8409358034365</v>
+        <v>26.0166888978503</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -9280,7 +9280,7 @@
         <v>1.568112774445864</v>
       </c>
       <c r="Q32" t="n">
-        <v>31.4</v>
+        <v>31.5</v>
       </c>
       <c r="R32" t="n">
         <v>4</v>
@@ -9329,10 +9329,10 @@
         <v>479999</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>686121</v>
+        <v>687751</v>
       </c>
       <c r="L33" t="n">
-        <v>30.04163988567614</v>
+        <v>30.20744426398508</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -9344,7 +9344,7 @@
         <v>41.73965217391304</v>
       </c>
       <c r="Q33" t="n">
-        <v>21.8</v>
+        <v>21.9</v>
       </c>
       <c r="R33" t="n">
         <v>3</v>
@@ -9393,10 +9393,10 @@
         <v>479999</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>686121</v>
+        <v>687751</v>
       </c>
       <c r="L34" t="n">
-        <v>30.04163988567614</v>
+        <v>30.20744426398508</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -9408,7 +9408,7 @@
         <v>41.73965217391304</v>
       </c>
       <c r="Q34" t="n">
-        <v>21.8</v>
+        <v>21.9</v>
       </c>
       <c r="R34" t="n">
         <v>3</v>
@@ -9457,10 +9457,10 @@
         <v>479999</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>686121</v>
+        <v>687751</v>
       </c>
       <c r="L35" t="n">
-        <v>30.04163988567614</v>
+        <v>30.20744426398508</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
@@ -9472,7 +9472,7 @@
         <v>41.73965217391304</v>
       </c>
       <c r="Q35" t="n">
-        <v>21.8</v>
+        <v>21.9</v>
       </c>
       <c r="R35" t="n">
         <v>3</v>
@@ -9521,10 +9521,10 @@
         <v>479999</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>686121</v>
+        <v>687751</v>
       </c>
       <c r="L36" t="n">
-        <v>30.04163988567614</v>
+        <v>30.20744426398508</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -9536,7 +9536,7 @@
         <v>41.73965217391304</v>
       </c>
       <c r="Q36" t="n">
-        <v>21.8</v>
+        <v>21.9</v>
       </c>
       <c r="R36" t="n">
         <v>3</v>
@@ -9585,16 +9585,16 @@
         <v>479999</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>643212</v>
+        <v>644740</v>
       </c>
       <c r="L37" t="n">
-        <v>25.37468206438935</v>
+        <v>25.55154015572169</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N37" t="n">
-        <v>1.639347621613979</v>
+        <v>1.234570441502966</v>
       </c>
       <c r="O37" t="n">
         <v>0</v>
@@ -9652,10 +9652,10 @@
         <v>500000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>643212</v>
+        <v>644740</v>
       </c>
       <c r="L38" t="n">
-        <v>22.2651318694303</v>
+        <v>22.44935943170891</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -9716,16 +9716,16 @@
         <v>547999</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>771940</v>
+        <v>773773</v>
       </c>
       <c r="L39" t="n">
-        <v>29.01015622975879</v>
+        <v>29.17832490924341</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N39" t="n">
-        <v>0.5444655979411941</v>
+        <v>0.3636370247945905</v>
       </c>
       <c r="P39" t="n">
         <v>63.4438956521739</v>
@@ -9780,16 +9780,16 @@
         <v>547999</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>771940</v>
+        <v>773773</v>
       </c>
       <c r="L40" t="n">
-        <v>29.01015622975879</v>
+        <v>29.17832490924341</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N40" t="n">
-        <v>0.5444655979411941</v>
+        <v>0.3636370247945905</v>
       </c>
       <c r="P40" t="n">
         <v>63.4438956521739</v>
@@ -9844,22 +9844,22 @@
         <v>547999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>771940</v>
+        <v>773773</v>
       </c>
       <c r="L41" t="n">
-        <v>29.01015622975879</v>
+        <v>29.17832490924341</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N41" t="n">
-        <v>1.261263533808169</v>
+        <v>0.7246389939112209</v>
       </c>
       <c r="P41" t="n">
         <v>63.4438956521739</v>
       </c>
       <c r="Q41" t="n">
-        <v>26.5</v>
+        <v>26.4</v>
       </c>
       <c r="R41" t="n">
         <v>3</v>
@@ -9908,16 +9908,16 @@
         <v>547999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>771940</v>
+        <v>773773</v>
       </c>
       <c r="L42" t="n">
-        <v>29.01015622975879</v>
+        <v>29.17832490924341</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N42" t="n">
-        <v>0.5444655979411941</v>
+        <v>0.3636370247945905</v>
       </c>
       <c r="P42" t="n">
         <v>63.4438956521739</v>
@@ -9972,10 +9972,10 @@
         <v>552999</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>771940</v>
+        <v>773773</v>
       </c>
       <c r="L43" t="n">
-        <v>28.36243749514211</v>
+        <v>28.53214056318843</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -9987,7 +9987,7 @@
         <v>34.11769473304435</v>
       </c>
       <c r="Q43" t="n">
-        <v>20.2</v>
+        <v>20.3</v>
       </c>
       <c r="R43" t="n">
         <v>3</v>
@@ -10036,10 +10036,10 @@
         <v>552999</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>771940</v>
+        <v>773773</v>
       </c>
       <c r="L44" t="n">
-        <v>28.36243749514211</v>
+        <v>28.53214056318843</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -10051,7 +10051,7 @@
         <v>34.11769473304435</v>
       </c>
       <c r="Q44" t="n">
-        <v>20.2</v>
+        <v>20.3</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -10100,10 +10100,10 @@
         <v>552999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>771940</v>
+        <v>773773</v>
       </c>
       <c r="L45" t="n">
-        <v>28.36243749514211</v>
+        <v>28.53214056318843</v>
       </c>
       <c r="M45" s="3" t="n">
         <v>0</v>
@@ -10115,7 +10115,7 @@
         <v>34.11769473304435</v>
       </c>
       <c r="Q45" t="n">
-        <v>20.2</v>
+        <v>20.3</v>
       </c>
       <c r="R45" t="n">
         <v>3</v>
@@ -10164,10 +10164,10 @@
         <v>552999</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>771940</v>
+        <v>773773</v>
       </c>
       <c r="L46" t="n">
-        <v>28.36243749514211</v>
+        <v>28.53214056318843</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -10179,7 +10179,7 @@
         <v>34.11769473304435</v>
       </c>
       <c r="Q46" t="n">
-        <v>20.2</v>
+        <v>20.3</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -10228,10 +10228,10 @@
         <v>585000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>729031</v>
+        <v>730762</v>
       </c>
       <c r="L47" t="n">
-        <v>19.75649869484288</v>
+        <v>19.94657631349194</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -10243,7 +10243,7 @@
         <v>21.56821735015607</v>
       </c>
       <c r="Q47" t="n">
-        <v>13.1</v>
+        <v>13.2</v>
       </c>
       <c r="R47" t="n">
         <v>3</v>
@@ -10292,10 +10292,10 @@
         <v>595000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>729031</v>
+        <v>730762</v>
       </c>
       <c r="L48" t="n">
-        <v>18.38481491184874</v>
+        <v>18.57814172056018</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -10307,7 +10307,7 @@
         <v>43.82608695652173</v>
       </c>
       <c r="Q48" t="n">
-        <v>17.3</v>
+        <v>17.4</v>
       </c>
       <c r="R48" t="n">
         <v>3</v>
@@ -10356,10 +10356,10 @@
         <v>614999</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>857759</v>
+        <v>859796</v>
       </c>
       <c r="L49" t="n">
-        <v>28.30165582640345</v>
+        <v>28.47152115152897</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -10420,10 +10420,10 @@
         <v>614999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>857759</v>
+        <v>859796</v>
       </c>
       <c r="L50" t="n">
-        <v>28.30165582640345</v>
+        <v>28.47152115152897</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -10484,10 +10484,10 @@
         <v>614999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>857759</v>
+        <v>859796</v>
       </c>
       <c r="L51" t="n">
-        <v>28.30165582640345</v>
+        <v>28.47152115152897</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -10548,10 +10548,10 @@
         <v>614999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>857759</v>
+        <v>859796</v>
       </c>
       <c r="L52" t="n">
-        <v>28.30165582640345</v>
+        <v>28.47152115152897</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -10612,10 +10612,10 @@
         <v>650000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>814849</v>
+        <v>816785</v>
       </c>
       <c r="L53" t="n">
-        <v>20.23061941537635</v>
+        <v>20.41969428919483</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -10676,10 +10676,10 @@
         <v>672000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>857759</v>
+        <v>859796</v>
       </c>
       <c r="L54" t="n">
-        <v>21.65631605147833</v>
+        <v>21.84192529390693</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -10691,7 +10691,7 @@
         <v>58.43478260869565</v>
       </c>
       <c r="Q54" t="n">
-        <v>21.8</v>
+        <v>21.9</v>
       </c>
       <c r="R54" t="n">
         <v>3</v>
@@ -10740,10 +10740,10 @@
         <v>700000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>900668</v>
+        <v>902807</v>
       </c>
       <c r="L55" t="n">
-        <v>22.27990780176491</v>
+        <v>22.46404824065387</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -10755,7 +10755,7 @@
         <v>48.69565217391303</v>
       </c>
       <c r="Q55" t="n">
-        <v>20</v>
+        <v>20.1</v>
       </c>
       <c r="R55" t="n">
         <v>3</v>
@@ -10804,10 +10804,10 @@
         <v>715000</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>943577</v>
+        <v>945819</v>
       </c>
       <c r="L56" t="n">
-        <v>24.22452009745892</v>
+        <v>24.40414074997436</v>
       </c>
       <c r="M56" s="3" t="n">
         <v>0</v>
@@ -10819,7 +10819,7 @@
         <v>64.05209961882153</v>
       </c>
       <c r="Q56" t="n">
-        <v>24.1</v>
+        <v>24.2</v>
       </c>
       <c r="R56" t="n">
         <v>3</v>
@@ -10868,10 +10868,10 @@
         <v>734999</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>986487</v>
+        <v>988830</v>
       </c>
       <c r="L57" t="n">
-        <v>25.49329083910888</v>
+        <v>25.66983202370478</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -10883,7 +10883,7 @@
         <v>73.04377639751551</v>
       </c>
       <c r="Q57" t="n">
-        <v>26.6</v>
+        <v>26.7</v>
       </c>
       <c r="R57" t="n">
         <v>3</v>
@@ -10932,10 +10932,10 @@
         <v>752000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>986487</v>
+        <v>988830</v>
       </c>
       <c r="L58" t="n">
-        <v>23.76990269511914</v>
+        <v>23.95052739095699</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -10947,7 +10947,7 @@
         <v>54.37884642534079</v>
       </c>
       <c r="Q58" t="n">
-        <v>21.8</v>
+        <v>21.9</v>
       </c>
       <c r="R58" t="n">
         <v>3</v>
@@ -10996,10 +10996,10 @@
         <v>810000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1072306</v>
+        <v>1074853</v>
       </c>
       <c r="L59" t="n">
-        <v>24.46186070021058</v>
+        <v>24.64085786614542</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -11060,10 +11060,10 @@
         <v>815000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1072306</v>
+        <v>1074853</v>
       </c>
       <c r="L60" t="n">
-        <v>23.99557588971805</v>
+        <v>24.17567797643026</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -11075,7 +11075,7 @@
         <v>79.56521739130434</v>
       </c>
       <c r="Q60" t="n">
-        <v>27.3</v>
+        <v>27.4</v>
       </c>
       <c r="R60" t="n">
         <v>3</v>
@@ -11124,10 +11124,10 @@
         <v>875000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1158124</v>
+        <v>1160875</v>
       </c>
       <c r="L61" t="n">
-        <v>24.44677771982965</v>
+        <v>24.62582104016367</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -11139,7 +11139,7 @@
         <v>79.41165705441597</v>
       </c>
       <c r="Q61" t="n">
-        <v>27.5</v>
+        <v>27.6</v>
       </c>
       <c r="R61" t="n">
         <v>3</v>
@@ -11188,10 +11188,10 @@
         <v>992000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1329762</v>
+        <v>1332921</v>
       </c>
       <c r="L62" t="n">
-        <v>25.40018439389906</v>
+        <v>25.57698468251306</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -11203,7 +11203,7 @@
         <v>85.14782608695651</v>
       </c>
       <c r="Q62" t="n">
-        <v>29.1</v>
+        <v>29.2</v>
       </c>
       <c r="R62" t="n">
         <v>3</v>
@@ -11252,10 +11252,10 @@
         <v>1050000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1415581</v>
+        <v>1418943</v>
       </c>
       <c r="L63" t="n">
-        <v>25.82550910191646</v>
+        <v>26.00125586440047</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -11267,7 +11267,7 @@
         <v>92.96442687747034</v>
       </c>
       <c r="Q63" t="n">
-        <v>31</v>
+        <v>31.1</v>
       </c>
       <c r="R63" t="n">
         <v>3</v>
@@ -11316,10 +11316,10 @@
         <v>1050000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1415581</v>
+        <v>1418943</v>
       </c>
       <c r="L64" t="n">
-        <v>25.82550910191646</v>
+        <v>26.00125586440047</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -11380,10 +11380,10 @@
         <v>1100000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1501400</v>
+        <v>1504966</v>
       </c>
       <c r="L65" t="n">
-        <v>26.73504728919675</v>
+        <v>26.90864777011573</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -11395,7 +11395,7 @@
         <v>94.11761630126171</v>
       </c>
       <c r="Q65" t="n">
-        <v>31.6</v>
+        <v>31.7</v>
       </c>
       <c r="R65" t="n">
         <v>3</v>
@@ -11444,10 +11444,10 @@
         <v>1105000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1501400</v>
+        <v>1504966</v>
       </c>
       <c r="L66" t="n">
-        <v>26.40202477687492</v>
+        <v>26.57641435088899</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -11459,7 +11459,7 @@
         <v>100</v>
       </c>
       <c r="Q66" t="n">
-        <v>32.7</v>
+        <v>32.8</v>
       </c>
       <c r="R66" t="n">
         <v>3</v>
@@ -11508,10 +11508,10 @@
         <v>1155000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1587218</v>
+        <v>1590988</v>
       </c>
       <c r="L67" t="n">
-        <v>27.23116799330653</v>
+        <v>27.40360078140125</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -11523,7 +11523,7 @@
         <v>100</v>
       </c>
       <c r="Q67" t="n">
-        <v>33.1</v>
+        <v>33.2</v>
       </c>
       <c r="R67" t="n">
         <v>3</v>
@@ -11778,7 +11778,7 @@
         <v>315000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>299937</v>
+        <v>300649</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -11839,10 +11839,10 @@
         <v>380000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>385755</v>
+        <v>386672</v>
       </c>
       <c r="L3" t="n">
-        <v>1.491879560861168</v>
+        <v>1.725493441469773</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -11854,7 +11854,7 @@
         <v>100</v>
       </c>
       <c r="Q3" t="n">
-        <v>22.1</v>
+        <v>22.2</v>
       </c>
       <c r="R3" t="n">
         <v>3</v>
@@ -11903,7 +11903,7 @@
         <v>415000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>385755</v>
+        <v>386672</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -11964,10 +11964,10 @@
         <v>495000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>471574</v>
+        <v>472694</v>
       </c>
       <c r="L5" t="n">
-        <v>6.695661762522954</v>
+        <v>6.916736831861627</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -11979,7 +11979,7 @@
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>3.9</v>
+        <v>4</v>
       </c>
       <c r="R5" t="n">
         <v>4</v>
@@ -12028,10 +12028,10 @@
         <v>490000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514484</v>
+        <v>515706</v>
       </c>
       <c r="L6" t="n">
-        <v>4.758942940888346</v>
+        <v>4.984623021644115</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -12043,7 +12043,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="R6" t="n">
         <v>3</v>
@@ -12092,10 +12092,10 @@
         <v>550000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>557393</v>
+        <v>558717</v>
       </c>
       <c r="L7" t="n">
-        <v>6.708552134669793</v>
+        <v>6.929626268755023</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -12107,7 +12107,7 @@
         <v>25.45360054666915</v>
       </c>
       <c r="Q7" t="n">
-        <v>8</v>
+        <v>8.1</v>
       </c>
       <c r="R7" t="n">
         <v>4</v>
@@ -12156,7 +12156,7 @@
         <v>530000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>471574</v>
+        <v>472694</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -12220,10 +12220,10 @@
         <v>600000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>600302</v>
+        <v>601728</v>
       </c>
       <c r="L9" t="n">
-        <v>8.379449010664631</v>
+        <v>8.596575196766645</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -12284,10 +12284,10 @@
         <v>646000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>729031</v>
+        <v>730762</v>
       </c>
       <c r="L10" t="n">
-        <v>17.0132682972329</v>
+        <v>17.20984397108771</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -12299,7 +12299,7 @@
         <v>100</v>
       </c>
       <c r="Q10" t="n">
-        <v>25.9</v>
+        <v>26</v>
       </c>
       <c r="R10" t="n">
         <v>4</v>
@@ -12348,7 +12348,7 @@
         <v>615000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>557393</v>
+        <v>558717</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -12412,7 +12412,7 @@
         <v>700000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>643212</v>
+        <v>644740</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -12476,7 +12476,7 @@
         <v>745000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>686121</v>
+        <v>687751</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -12540,7 +12540,7 @@
         <v>930000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>857759</v>
+        <v>859796</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -12611,7 +12611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12657,256 +12657,8 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 MJLV4 M5 Pro 15 Core CPU 16 Core GPU 24GB 2TB Silver</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>815000</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>775000</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>-40000</v>
-      </c>
-      <c r="F2" t="n">
-        <v>-4.91</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 MJLW4 M5 Pro 15 Core CPU 16 Core GPU 24GB 2TB Space Black</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>790000</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>775000</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>-15000</v>
-      </c>
-      <c r="F3" t="n">
-        <v>-1.9</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 M5 MJ3D4 10 Core CPU 10 Core GPU 32GB 1TB Space Black</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>780000</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>769999</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>-10001</v>
-      </c>
-      <c r="F4" t="n">
-        <v>-1.28</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Macbook Pro 16 MGE44 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Silver</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>829999</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>822999</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>-7000</v>
-      </c>
-      <c r="F5" t="n">
-        <v>-0.84</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 M5 MJ3E4 10 Core CPU 10 Core GPU 32GB 1TB Silver</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>775000</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>769999</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>-5001</v>
-      </c>
-      <c r="F6" t="n">
-        <v>-0.65</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDH74 M5 10C CPU 8C GPU 16GB 512GB Silver</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>425000</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>420000</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>-5000</v>
-      </c>
-      <c r="F7" t="n">
-        <v>-1.18</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDHE4 M5 10C CPU 8C GPU 16GB 512GB Midnight</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>420000</v>
-      </c>
-      <c r="D8" s="3" t="n">
-        <v>417999</v>
-      </c>
-      <c r="E8" s="3" t="n">
-        <v>-2001</v>
-      </c>
-      <c r="F8" t="n">
-        <v>-0.48</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDHH4 M5 10C CPU 8C GPU 16GB 512GB Sky Blue</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>420000</v>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>417999</v>
-      </c>
-      <c r="E9" s="3" t="n">
-        <v>-2001</v>
-      </c>
-      <c r="F9" t="n">
-        <v>-0.48</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDHA4 M5 10C CPU 8C GPU 16GB 512GB Starlight</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>420000</v>
-      </c>
-      <c r="D10" s="3" t="n">
-        <v>417999</v>
-      </c>
-      <c r="E10" s="3" t="n">
-        <v>-2001</v>
-      </c>
-      <c r="F10" t="n">
-        <v>-0.48</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Macbook Pro 16 MGEA4 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Space Black</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="n">
-        <v>825000</v>
-      </c>
-      <c r="D11" s="3" t="n">
-        <v>823000</v>
-      </c>
-      <c r="E11" s="3" t="n">
-        <v>-2000</v>
-      </c>
-      <c r="F11" t="n">
-        <v>-0.24</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:F11"/>
-  <conditionalFormatting sqref="E2:E11">
-    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
+  <autoFilter ref="A1:F1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: price data 2026-10-06
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MacBook Pro'!$A$1:$S$93</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MacBook Air'!$A$1:$S$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20261005T103324582721+0000</t>
+          <t>20261006T102505434069+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-05T10:33:24.582721+00:00</t>
+          <t>2026-10-06T10:25:05.434069+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>277.49233</v>
+        <v>277.095194</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -738,7 +738,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 16Inch MX2U3 14Core CPU 20Core GPU M4 Pro 48GB 512GB Silver</t>
+          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 48GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -747,19 +747,19 @@
         </is>
       </c>
       <c r="C23" s="3" t="n">
-        <v>810000</v>
+        <v>995000</v>
       </c>
       <c r="D23" t="n">
         <v>50.6</v>
       </c>
       <c r="E23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 48GB 1TB Space Black</t>
+          <t>Apple MacBook Pro 16Inch MX2U3 14Core CPU 20Core GPU M4 Pro 48GB 512GB Silver</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="C24" s="3" t="n">
-        <v>995000</v>
+        <v>810000</v>
       </c>
       <c r="D24" t="n">
-        <v>50.6</v>
+        <v>50.5</v>
       </c>
       <c r="E24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25">
@@ -792,7 +792,7 @@
         <v>1123000</v>
       </c>
       <c r="D25" t="n">
-        <v>50.5</v>
+        <v>50.4</v>
       </c>
       <c r="E25" t="n">
         <v>4</v>
@@ -855,7 +855,7 @@
         <v>644999</v>
       </c>
       <c r="D28" t="n">
-        <v>44.4</v>
+        <v>44.3</v>
       </c>
       <c r="E28" t="n">
         <v>4</v>
@@ -876,7 +876,7 @@
         <v>720000</v>
       </c>
       <c r="D29" t="n">
-        <v>44.2</v>
+        <v>44.1</v>
       </c>
       <c r="E29" t="n">
         <v>3</v>
@@ -897,7 +897,7 @@
         <v>725000</v>
       </c>
       <c r="D30" t="n">
-        <v>42.8</v>
+        <v>42.7</v>
       </c>
       <c r="E30" t="n">
         <v>3</v>
@@ -1147,10 +1147,10 @@
         <v>470000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>687751</v>
+        <v>686767</v>
       </c>
       <c r="L2" t="n">
-        <v>35.29634998713197</v>
+        <v>35.20364257455586</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1214,10 +1214,10 @@
         <v>495000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>687751</v>
+        <v>686767</v>
       </c>
       <c r="L3" t="n">
-        <v>28.02627695197826</v>
+        <v>27.92315297619135</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>773773</v>
+        <v>772666</v>
       </c>
       <c r="L4" t="n">
-        <v>35.38169463137122</v>
+        <v>35.28911586636399</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1299,7 +1299,7 @@
         <v>68.25981228668942</v>
       </c>
       <c r="Q4" t="n">
-        <v>41.8</v>
+        <v>41.7</v>
       </c>
       <c r="R4" t="n">
         <v>5</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>773773</v>
+        <v>772666</v>
       </c>
       <c r="L5" t="n">
-        <v>32.7969572471513</v>
+        <v>32.70067532413747</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>859796</v>
+        <v>858566</v>
       </c>
       <c r="L6" t="n">
-        <v>38.12485752434298</v>
+        <v>38.03621387289969</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1606,10 +1606,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>859796</v>
+        <v>858566</v>
       </c>
       <c r="L9" t="n">
-        <v>34.28673778431163</v>
+        <v>34.19259556050437</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1673,10 +1673,10 @@
         <v>579999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>859796</v>
+        <v>858566</v>
       </c>
       <c r="L10" t="n">
-        <v>32.54225420913798</v>
+        <v>32.44561280087961</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -1740,10 +1740,10 @@
         <v>587999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>859796</v>
+        <v>858566</v>
       </c>
       <c r="L11" t="n">
-        <v>31.61180093882735</v>
+        <v>31.51382654332923</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -1758,7 +1758,7 @@
         <v>47.60029999999999</v>
       </c>
       <c r="Q11" t="n">
-        <v>18.5</v>
+        <v>18.4</v>
       </c>
       <c r="R11" t="n">
         <v>4</v>
@@ -1807,10 +1807,10 @@
         <v>600000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>859796</v>
+        <v>858566</v>
       </c>
       <c r="L12" t="n">
-        <v>30.21600472670261</v>
+        <v>30.11603068372146</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -1874,10 +1874,10 @@
         <v>634000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>859796</v>
+        <v>858566</v>
       </c>
       <c r="L13" t="n">
-        <v>26.26157832788243</v>
+        <v>26.15593908913235</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -1941,10 +1941,10 @@
         <v>644999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>945819</v>
+        <v>944465</v>
       </c>
       <c r="L14" t="n">
-        <v>31.80523969173806</v>
+        <v>31.70747460202337</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -1959,7 +1959,7 @@
         <v>69.20023999999999</v>
       </c>
       <c r="Q14" t="n">
-        <v>44.4</v>
+        <v>44.3</v>
       </c>
       <c r="R14" t="n">
         <v>4</v>
@@ -2067,10 +2067,10 @@
         <v>650000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>945819</v>
+        <v>944465</v>
       </c>
       <c r="L16" t="n">
-        <v>31.27649159088578</v>
+        <v>31.17796847950957</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -2085,7 +2085,7 @@
         <v>68</v>
       </c>
       <c r="Q16" t="n">
-        <v>21.8</v>
+        <v>21.7</v>
       </c>
       <c r="R16" t="n">
         <v>4</v>
@@ -2134,10 +2134,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1031841</v>
+        <v>1030365</v>
       </c>
       <c r="L17" t="n">
-        <v>32.16009055658769</v>
+        <v>32.0629097455756</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2201,10 +2201,10 @@
         <v>711999</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>1074853</v>
+        <v>1073314</v>
       </c>
       <c r="L18" t="n">
-        <v>33.75847674054033</v>
+        <v>33.6634945598399</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -2272,7 +2272,7 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>0.6895181924388861</v>
+        <v>0.3459517965064336</v>
       </c>
       <c r="O19" t="n">
         <v>100</v>
@@ -2281,7 +2281,7 @@
         <v>42.39316239316239</v>
       </c>
       <c r="Q19" t="n">
-        <v>44.2</v>
+        <v>44.1</v>
       </c>
       <c r="R19" t="n">
         <v>3</v>
@@ -2330,10 +2330,10 @@
         <v>720000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>1031841</v>
+        <v>1030365</v>
       </c>
       <c r="L20" t="n">
-        <v>30.22180742963305</v>
+        <v>30.12185002402061</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -2401,7 +2401,7 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>0.684795458623916</v>
+        <v>0.3435741192949274</v>
       </c>
       <c r="O21" t="n">
         <v>96.7741935483871</v>
@@ -2410,7 +2410,7 @@
         <v>41.02564102564102</v>
       </c>
       <c r="Q21" t="n">
-        <v>42.8</v>
+        <v>42.7</v>
       </c>
       <c r="R21" t="n">
         <v>3</v>
@@ -2459,10 +2459,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1074853</v>
+        <v>1073314</v>
       </c>
       <c r="L22" t="n">
-        <v>30.87426838832845</v>
+        <v>30.77515060830288</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2526,10 +2526,10 @@
         <v>769999</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1031841</v>
+        <v>1030365</v>
       </c>
       <c r="L23" t="n">
-        <v>25.3761965264028</v>
+        <v>25.26929777311924</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -2593,10 +2593,10 @@
         <v>769999</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1031841</v>
+        <v>1030365</v>
       </c>
       <c r="L24" t="n">
-        <v>25.3761965264028</v>
+        <v>25.26929777311924</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -2660,10 +2660,10 @@
         <v>772000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>1031841</v>
+        <v>1030365</v>
       </c>
       <c r="L25" t="n">
-        <v>25.182271299551</v>
+        <v>25.07509474797766</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -2851,10 +2851,10 @@
         <v>810000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>1074853</v>
+        <v>1073314</v>
       </c>
       <c r="L28" t="n">
-        <v>24.64085786614542</v>
+        <v>24.5328021436411</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -2915,10 +2915,10 @@
         <v>810000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>1246898</v>
+        <v>1245113</v>
       </c>
       <c r="L29" t="n">
-        <v>35.03879226688952</v>
+        <v>34.94566356627872</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -2933,7 +2933,7 @@
         <v>100</v>
       </c>
       <c r="Q29" t="n">
-        <v>50.6</v>
+        <v>50.5</v>
       </c>
       <c r="R29" t="n">
         <v>4</v>
@@ -2982,10 +2982,10 @@
         <v>822999</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1289909</v>
+        <v>1288063</v>
       </c>
       <c r="L30" t="n">
-        <v>36.19712708415864</v>
+        <v>36.10568737709258</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -3000,7 +3000,7 @@
         <v>0.0003521901827191575</v>
       </c>
       <c r="Q30" t="n">
-        <v>34.9</v>
+        <v>34.8</v>
       </c>
       <c r="R30" t="n">
         <v>4</v>
@@ -3049,10 +3049,10 @@
         <v>823000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1289909</v>
+        <v>1288063</v>
       </c>
       <c r="L31" t="n">
-        <v>36.19704955931</v>
+        <v>36.10560974113844</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -3116,10 +3116,10 @@
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1375932</v>
+        <v>1373963</v>
       </c>
       <c r="L32" t="n">
-        <v>38.36911998558069</v>
+        <v>38.28079795453007</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3183,10 +3183,10 @@
         <v>930000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1375932</v>
+        <v>1373963</v>
       </c>
       <c r="L33" t="n">
-        <v>38.22376396507967</v>
+        <v>38.13523362710641</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3250,10 +3250,10 @@
         <v>860000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>1246898</v>
+        <v>1245113</v>
       </c>
       <c r="L34" t="n">
-        <v>31.02884117225306</v>
+        <v>30.92996378641939</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -3503,10 +3503,10 @@
         <v>880000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>1160875</v>
+        <v>1159214</v>
       </c>
       <c r="L38" t="n">
-        <v>24.19511144610746</v>
+        <v>24.08649308928291</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -3567,10 +3567,10 @@
         <v>940000</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>1246898</v>
+        <v>1245113</v>
       </c>
       <c r="L39" t="n">
-        <v>24.61291942083474</v>
+        <v>24.50484413864444</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -3631,10 +3631,10 @@
         <v>990000</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>1504966</v>
+        <v>1502812</v>
       </c>
       <c r="L40" t="n">
-        <v>34.21778299310417</v>
+        <v>34.12349648525564</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -3642,14 +3642,17 @@
       <c r="N40" t="n">
         <v>3.131115459882583</v>
       </c>
+      <c r="O40" t="n">
+        <v>100</v>
+      </c>
       <c r="P40" t="n">
         <v>39.19647231749141</v>
       </c>
       <c r="Q40" t="n">
-        <v>24.2</v>
+        <v>41</v>
       </c>
       <c r="R40" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S40" t="inlineStr">
         <is>
@@ -3660,28 +3663,28 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 16Inch MX303 14Core CPU 32Core GPU M4 Max 36GB 1TB Space Black</t>
+          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 48GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>M4 Max</t>
+          <t>M5 Pro</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="E41" t="n">
         <v>1024</v>
       </c>
       <c r="F41" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G41" t="n">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -3689,28 +3692,26 @@
         </is>
       </c>
       <c r="I41" s="3" t="n">
-        <v>990000</v>
+        <v>995000</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>990000</v>
-      </c>
-      <c r="K41" s="3" t="n">
-        <v>1504966</v>
-      </c>
-      <c r="L41" t="n">
-        <v>34.21778299310417</v>
-      </c>
+        <v>995000</v>
+      </c>
+      <c r="K41" s="3" t="n"/>
       <c r="M41" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N41" t="n">
         <v>0</v>
       </c>
+      <c r="O41" t="n">
+        <v>100</v>
+      </c>
       <c r="P41" t="n">
-        <v>39.19647231749141</v>
+        <v>69.23076923076923</v>
       </c>
       <c r="Q41" t="n">
-        <v>23.1</v>
+        <v>50.6</v>
       </c>
       <c r="R41" t="n">
         <v>3</v>
@@ -3724,28 +3725,28 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 48GB 1TB Space Black</t>
+          <t>Apple MacBook Pro 16Inch MX303 14Core CPU 32Core GPU M4 Max 36GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>M5 Pro</t>
+          <t>M4 Max</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="E42" t="n">
         <v>1024</v>
       </c>
       <c r="F42" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G42" t="n">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -3753,29 +3754,34 @@
         </is>
       </c>
       <c r="I42" s="3" t="n">
-        <v>995000</v>
+        <v>1000000</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>995000</v>
-      </c>
-      <c r="K42" s="3" t="n"/>
+        <v>1000000</v>
+      </c>
+      <c r="K42" s="3" t="n">
+        <v>1502812</v>
+      </c>
+      <c r="L42" t="n">
+        <v>33.45807725783398</v>
+      </c>
       <c r="M42" s="3" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="N42" t="n">
         <v>0</v>
       </c>
       <c r="O42" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="P42" t="n">
-        <v>69.23076923076923</v>
+        <v>31.35717785399315</v>
       </c>
       <c r="Q42" t="n">
-        <v>50.6</v>
+        <v>16.4</v>
       </c>
       <c r="R42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S42" t="inlineStr">
         <is>
@@ -3821,10 +3827,10 @@
         <v>1055000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1547977</v>
+        <v>1545762</v>
       </c>
       <c r="L43" t="n">
-        <v>31.84653260352059</v>
+        <v>31.74887207733144</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -3885,10 +3891,10 @@
         <v>1055000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1547977</v>
+        <v>1545762</v>
       </c>
       <c r="L44" t="n">
-        <v>31.84653260352059</v>
+        <v>31.74887207733144</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -4011,10 +4017,10 @@
         <v>1115000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1504966</v>
+        <v>1502812</v>
       </c>
       <c r="L46" t="n">
-        <v>25.9119475124355</v>
+        <v>25.80575614248489</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -4075,10 +4081,10 @@
         <v>1123000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1720022</v>
+        <v>1717561</v>
       </c>
       <c r="L47" t="n">
-        <v>34.71013742847475</v>
+        <v>34.61658712558098</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -4093,7 +4099,7 @@
         <v>100</v>
       </c>
       <c r="Q47" t="n">
-        <v>50.5</v>
+        <v>50.4</v>
       </c>
       <c r="R47" t="n">
         <v>4</v>
@@ -4142,10 +4148,10 @@
         <v>1130000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1504966</v>
+        <v>1502812</v>
       </c>
       <c r="L48" t="n">
-        <v>24.91524725475526</v>
+        <v>24.8076273013524</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -4268,10 +4274,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1763034</v>
+        <v>1760510</v>
       </c>
       <c r="L50" t="n">
-        <v>34.48793386854706</v>
+        <v>34.39401082640826</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4332,10 +4338,10 @@
         <v>1155000</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>1763034</v>
+        <v>1760510</v>
       </c>
       <c r="L51" t="n">
-        <v>34.48793386854706</v>
+        <v>34.39401082640826</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -4396,10 +4402,10 @@
         <v>1185000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1590988</v>
+        <v>1588711</v>
       </c>
       <c r="L52" t="n">
-        <v>25.5179800224766</v>
+        <v>25.41122960689515</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -4411,7 +4417,7 @@
         <v>77.26495726495727</v>
       </c>
       <c r="Q52" t="n">
-        <v>27.5</v>
+        <v>27.4</v>
       </c>
       <c r="R52" t="n">
         <v>3</v>
@@ -4460,10 +4466,10 @@
         <v>1185000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1590988</v>
+        <v>1588711</v>
       </c>
       <c r="L53" t="n">
-        <v>25.5179800224766</v>
+        <v>25.41122960689515</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -4524,22 +4530,22 @@
         <v>1200000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1892068</v>
+        <v>1889360</v>
       </c>
       <c r="L54" t="n">
-        <v>36.57733231575187</v>
+        <v>36.4864292670534</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N54" t="n">
-        <v>0.579950289975145</v>
+        <v>0.2908184461985874</v>
       </c>
       <c r="P54" t="n">
         <v>3.948101568096777</v>
       </c>
       <c r="Q54" t="n">
-        <v>16.7</v>
+        <v>16.6</v>
       </c>
       <c r="R54" t="n">
         <v>3</v>
@@ -4588,22 +4594,22 @@
         <v>1200000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1892068</v>
+        <v>1889360</v>
       </c>
       <c r="L55" t="n">
-        <v>36.57733231575187</v>
+        <v>36.4864292670534</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N55" t="n">
-        <v>0.579950289975145</v>
+        <v>0.2908184461985874</v>
       </c>
       <c r="P55" t="n">
         <v>3.948101568096777</v>
       </c>
       <c r="Q55" t="n">
-        <v>16.7</v>
+        <v>16.6</v>
       </c>
       <c r="R55" t="n">
         <v>3</v>
@@ -4714,10 +4720,10 @@
         <v>1240000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1677011</v>
+        <v>1674611</v>
       </c>
       <c r="L57" t="n">
-        <v>26.05892269042958</v>
+        <v>25.95295265587053</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -4840,10 +4846,10 @@
         <v>1280000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1720022</v>
+        <v>1717561</v>
       </c>
       <c r="L59" t="n">
-        <v>25.58234720253578</v>
+        <v>25.47571818409943</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -4907,10 +4913,10 @@
         <v>1298000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1763034</v>
+        <v>1760510</v>
       </c>
       <c r="L60" t="n">
-        <v>26.37691615703384</v>
+        <v>26.27136454777309</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -4971,10 +4977,10 @@
         <v>1300000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1720022</v>
+        <v>1717561</v>
       </c>
       <c r="L61" t="n">
-        <v>24.4195713775754</v>
+        <v>24.31127628072598</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -4986,7 +4992,7 @@
         <v>60.92890160686771</v>
       </c>
       <c r="Q61" t="n">
-        <v>23.8</v>
+        <v>23.7</v>
       </c>
       <c r="R61" t="n">
         <v>3</v>
@@ -5097,10 +5103,10 @@
         <v>1335000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1806045</v>
+        <v>1803460</v>
       </c>
       <c r="L63" t="n">
-        <v>26.08157604046411</v>
+        <v>25.97562463265057</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -5112,7 +5118,7 @@
         <v>87.17948717948718</v>
       </c>
       <c r="Q63" t="n">
-        <v>29.9</v>
+        <v>29.8</v>
       </c>
       <c r="R63" t="n">
         <v>3</v>
@@ -5161,10 +5167,10 @@
         <v>1420000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1935079</v>
+        <v>1932309</v>
       </c>
       <c r="L64" t="n">
-        <v>26.61798303841859</v>
+        <v>26.51278858609053</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -5225,10 +5231,10 @@
         <v>1430000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1935079</v>
+        <v>1932309</v>
       </c>
       <c r="L65" t="n">
-        <v>26.1012082710835</v>
+        <v>25.99527301275313</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -5289,10 +5295,10 @@
         <v>1430000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>2150135</v>
+        <v>2147058</v>
       </c>
       <c r="L66" t="n">
-        <v>33.49254814232594</v>
+        <v>33.39723472770647</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -5304,7 +5310,7 @@
         <v>0</v>
       </c>
       <c r="Q66" t="n">
-        <v>14.4</v>
+        <v>14.3</v>
       </c>
       <c r="R66" t="n">
         <v>3</v>
@@ -5353,10 +5359,10 @@
         <v>1430000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>2150135</v>
+        <v>2147058</v>
       </c>
       <c r="L67" t="n">
-        <v>33.49254814232594</v>
+        <v>33.39723472770647</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -5368,7 +5374,7 @@
         <v>0</v>
       </c>
       <c r="Q67" t="n">
-        <v>14.4</v>
+        <v>14.3</v>
       </c>
       <c r="R67" t="n">
         <v>3</v>
@@ -5479,10 +5485,10 @@
         <v>1480000</v>
       </c>
       <c r="K69" s="3" t="n">
-        <v>2021102</v>
+        <v>2018209</v>
       </c>
       <c r="L69" t="n">
-        <v>26.77262206459644</v>
+        <v>26.66765434105189</v>
       </c>
       <c r="M69" s="3" t="n">
         <v>0</v>
@@ -5494,7 +5500,7 @@
         <v>0</v>
       </c>
       <c r="Q69" t="n">
-        <v>11.5</v>
+        <v>11.4</v>
       </c>
       <c r="R69" t="n">
         <v>3</v>
@@ -5605,10 +5611,10 @@
         <v>1605000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2193147</v>
+        <v>2190008</v>
       </c>
       <c r="L71" t="n">
-        <v>26.81749103001303</v>
+        <v>26.71259648366581</v>
       </c>
       <c r="M71" s="3" t="n">
         <v>0</v>
@@ -5669,10 +5675,10 @@
         <v>1610000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2193147</v>
+        <v>2190008</v>
       </c>
       <c r="L72" t="n">
-        <v>26.58950813602554</v>
+        <v>26.48428681539063</v>
       </c>
       <c r="M72" s="3" t="n">
         <v>0</v>
@@ -5733,10 +5739,10 @@
         <v>1615000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2193147</v>
+        <v>2190008</v>
       </c>
       <c r="L73" t="n">
-        <v>26.36152524203804</v>
+        <v>26.25597714711544</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
@@ -5748,7 +5754,7 @@
         <v>86.7142542687337</v>
       </c>
       <c r="Q73" t="n">
-        <v>30.9</v>
+        <v>30.8</v>
       </c>
       <c r="R73" t="n">
         <v>3</v>
@@ -5797,10 +5803,10 @@
         <v>1630000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2236158</v>
+        <v>2232958</v>
       </c>
       <c r="L74" t="n">
-        <v>27.10711854886819</v>
+        <v>27.00265746153757</v>
       </c>
       <c r="M74" s="3" t="n">
         <v>0</v>
@@ -5861,10 +5867,10 @@
         <v>1690000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2322181</v>
+        <v>2318857</v>
       </c>
       <c r="L75" t="n">
-        <v>27.22358851441813</v>
+        <v>27.11926608669702</v>
       </c>
       <c r="M75" s="3" t="n">
         <v>0</v>
@@ -5925,10 +5931,10 @@
         <v>1705000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2322181</v>
+        <v>2318857</v>
       </c>
       <c r="L76" t="n">
-        <v>26.57764403377686</v>
+        <v>26.47239566734818</v>
       </c>
       <c r="M76" s="3" t="n">
         <v>0</v>
@@ -5940,7 +5946,7 @@
         <v>1.9846639603067</v>
       </c>
       <c r="Q76" t="n">
-        <v>12.9</v>
+        <v>12.8</v>
       </c>
       <c r="R76" t="n">
         <v>3</v>
@@ -5989,10 +5995,10 @@
         <v>1725000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2365192</v>
+        <v>2361807</v>
       </c>
       <c r="L77" t="n">
-        <v>27.06723175116439</v>
+        <v>26.96270271025532</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
@@ -6053,10 +6059,10 @@
         <v>1780000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2451215</v>
+        <v>2447707</v>
       </c>
       <c r="L78" t="n">
-        <v>27.38295090393947</v>
+        <v>27.27887774149438</v>
       </c>
       <c r="M78" s="3" t="n">
         <v>0</v>
@@ -6117,10 +6123,10 @@
         <v>1875000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2580249</v>
+        <v>2576556</v>
       </c>
       <c r="L79" t="n">
-        <v>27.33259464493543</v>
+        <v>27.22843982432363</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
@@ -6181,10 +6187,10 @@
         <v>1910000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2623260</v>
+        <v>2619506</v>
       </c>
       <c r="L80" t="n">
-        <v>27.18983249849424</v>
+        <v>27.08548863793402</v>
       </c>
       <c r="M80" s="3" t="n">
         <v>0</v>
@@ -6196,7 +6202,7 @@
         <v>53.22486926205694</v>
       </c>
       <c r="Q80" t="n">
-        <v>23.1</v>
+        <v>23</v>
       </c>
       <c r="R80" t="n">
         <v>3</v>
@@ -6245,10 +6251,10 @@
         <v>2020000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2752294</v>
+        <v>2748355</v>
       </c>
       <c r="L81" t="n">
-        <v>26.60667792030938</v>
+        <v>26.50148907255431</v>
       </c>
       <c r="M81" s="3" t="n">
         <v>0</v>
@@ -6260,7 +6266,7 @@
         <v>36.26522327469554</v>
       </c>
       <c r="Q81" t="n">
-        <v>20.2</v>
+        <v>20.1</v>
       </c>
       <c r="R81" t="n">
         <v>3</v>
@@ -6309,10 +6315,10 @@
         <v>2110000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>2881328</v>
+        <v>2877204</v>
       </c>
       <c r="L82" t="n">
-        <v>26.76987833387938</v>
+        <v>26.66491496605732</v>
       </c>
       <c r="M82" s="3" t="n">
         <v>0</v>
@@ -6373,10 +6379,10 @@
         <v>2210000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3010362</v>
+        <v>3006053</v>
       </c>
       <c r="L83" t="n">
-        <v>26.58690217322701</v>
+        <v>26.4816688195451</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
@@ -6388,7 +6394,7 @@
         <v>70.36535859269283</v>
       </c>
       <c r="Q83" t="n">
-        <v>27.4</v>
+        <v>27.3</v>
       </c>
       <c r="R83" t="n">
         <v>3</v>
@@ -6437,10 +6443,10 @@
         <v>2215000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3053373</v>
+        <v>3049003</v>
       </c>
       <c r="L84" t="n">
-        <v>27.45727429960244</v>
+        <v>27.35330204660343</v>
       </c>
       <c r="M84" s="3" t="n">
         <v>0</v>
@@ -6452,7 +6458,7 @@
         <v>74.28466149856153</v>
       </c>
       <c r="Q84" t="n">
-        <v>27.7</v>
+        <v>27.6</v>
       </c>
       <c r="R84" t="n">
         <v>3</v>
@@ -6501,10 +6507,10 @@
         <v>2315000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3182407</v>
+        <v>3177852</v>
       </c>
       <c r="L85" t="n">
-        <v>27.256318880646</v>
+        <v>27.15205113391058</v>
       </c>
       <c r="M85" s="3" t="n">
         <v>0</v>
@@ -6565,10 +6571,10 @@
         <v>2395000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3311441</v>
+        <v>3306702</v>
       </c>
       <c r="L86" t="n">
-        <v>27.6749910386445</v>
+        <v>27.57133845142381</v>
       </c>
       <c r="M86" s="3" t="n">
         <v>0</v>
@@ -6580,7 +6586,7 @@
         <v>72.76953145634144</v>
       </c>
       <c r="Q86" t="n">
-        <v>27.5</v>
+        <v>27.4</v>
       </c>
       <c r="R86" t="n">
         <v>3</v>
@@ -6629,10 +6635,10 @@
         <v>2410000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3311441</v>
+        <v>3306702</v>
       </c>
       <c r="L87" t="n">
-        <v>27.22201603471117</v>
+        <v>27.11771426635966</v>
       </c>
       <c r="M87" s="3" t="n">
         <v>0</v>
@@ -6693,10 +6699,10 @@
         <v>2499000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3440475</v>
+        <v>3435551</v>
       </c>
       <c r="L88" t="n">
-        <v>27.36468074902448</v>
+        <v>27.26057625108752</v>
       </c>
       <c r="M88" s="3" t="n">
         <v>0</v>
@@ -6757,10 +6763,10 @@
         <v>2510000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3440475</v>
+        <v>3435551</v>
       </c>
       <c r="L89" t="n">
-        <v>27.04495745500258</v>
+        <v>26.94039471397747</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
@@ -6772,7 +6778,7 @@
         <v>83.17546233649077</v>
       </c>
       <c r="Q89" t="n">
-        <v>30.3</v>
+        <v>30.2</v>
       </c>
       <c r="R89" t="n">
         <v>3</v>
@@ -6821,10 +6827,10 @@
         <v>2530000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3483486</v>
+        <v>3478501</v>
       </c>
       <c r="L90" t="n">
-        <v>27.37160419189284</v>
+        <v>27.26752126850043</v>
       </c>
       <c r="M90" s="3" t="n">
         <v>0</v>
@@ -6885,10 +6891,10 @@
         <v>2610000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>3612520</v>
+        <v>3607350</v>
       </c>
       <c r="L91" t="n">
-        <v>27.75126504489941</v>
+        <v>27.64771923988523</v>
       </c>
       <c r="M91" s="3" t="n">
         <v>0</v>
@@ -6949,10 +6955,10 @@
         <v>3015000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4171667</v>
+        <v>4165697</v>
       </c>
       <c r="L92" t="n">
-        <v>27.7267337014196</v>
+        <v>27.6231564609716</v>
       </c>
       <c r="M92" s="3" t="n">
         <v>0</v>
@@ -7013,10 +7019,10 @@
         <v>3098000</v>
       </c>
       <c r="K93" s="3" t="n">
-        <v>4300701</v>
+        <v>4294546</v>
       </c>
       <c r="L93" t="n">
-        <v>27.96523171455072</v>
+        <v>27.86199053404015</v>
       </c>
       <c r="M93" s="3" t="n">
         <v>0</v>
@@ -7312,10 +7318,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>429683</v>
+        <v>429068</v>
       </c>
       <c r="L2" t="n">
-        <v>27.85402261667322</v>
+        <v>27.75061295645446</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7330,7 +7336,7 @@
         <v>29.71702857142851</v>
       </c>
       <c r="Q2" t="n">
-        <v>36.5</v>
+        <v>36.4</v>
       </c>
       <c r="R2" t="n">
         <v>4</v>
@@ -7379,10 +7385,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>429683</v>
+        <v>429068</v>
       </c>
       <c r="L3" t="n">
-        <v>27.85402261667322</v>
+        <v>27.75061295645446</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7397,7 +7403,7 @@
         <v>29.71702857142851</v>
       </c>
       <c r="Q3" t="n">
-        <v>36.5</v>
+        <v>36.4</v>
       </c>
       <c r="R3" t="n">
         <v>4</v>
@@ -7446,10 +7452,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>429683</v>
+        <v>429068</v>
       </c>
       <c r="L4" t="n">
-        <v>27.85378988696318</v>
+        <v>27.75037989316379</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7513,10 +7519,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>429683</v>
+        <v>429068</v>
       </c>
       <c r="L5" t="n">
-        <v>27.85378988696318</v>
+        <v>27.75037989316379</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7580,10 +7586,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>515706</v>
+        <v>514968</v>
       </c>
       <c r="L6" t="n">
-        <v>25.53896987818641</v>
+        <v>25.43225986857436</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7644,10 +7650,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>515706</v>
+        <v>514968</v>
       </c>
       <c r="L7" t="n">
-        <v>25.53896987818641</v>
+        <v>25.43225986857436</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7708,10 +7714,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>515706</v>
+        <v>514968</v>
       </c>
       <c r="L8" t="n">
-        <v>25.53896987818641</v>
+        <v>25.43225986857436</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7772,10 +7778,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>515706</v>
+        <v>514968</v>
       </c>
       <c r="L9" t="n">
-        <v>25.53896987818641</v>
+        <v>25.43225986857436</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7836,10 +7842,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>515706</v>
+        <v>514968</v>
       </c>
       <c r="L10" t="n">
-        <v>25.34506094557752</v>
+        <v>25.23807304531543</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7851,7 +7857,7 @@
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>10.9</v>
+        <v>10.8</v>
       </c>
       <c r="R10" t="n">
         <v>3</v>
@@ -7900,10 +7906,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>515706</v>
+        <v>514968</v>
       </c>
       <c r="L11" t="n">
-        <v>25.34506094557752</v>
+        <v>25.23807304531543</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7915,7 +7921,7 @@
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>10.9</v>
+        <v>10.8</v>
       </c>
       <c r="R11" t="n">
         <v>3</v>
@@ -7964,10 +7970,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>515706</v>
+        <v>514968</v>
       </c>
       <c r="L12" t="n">
-        <v>25.34506094557752</v>
+        <v>25.23807304531543</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -7979,7 +7985,7 @@
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>10.9</v>
+        <v>10.8</v>
       </c>
       <c r="R12" t="n">
         <v>3</v>
@@ -8028,10 +8034,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>515706</v>
+        <v>514968</v>
       </c>
       <c r="L13" t="n">
-        <v>25.34506094557752</v>
+        <v>25.23807304531543</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -8043,7 +8049,7 @@
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>10.9</v>
+        <v>10.8</v>
       </c>
       <c r="R13" t="n">
         <v>3</v>
@@ -8092,10 +8098,10 @@
         <v>417999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>558717</v>
+        <v>557917</v>
       </c>
       <c r="L14" t="n">
-        <v>25.18591702060256</v>
+        <v>25.07864072971427</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -8159,10 +8165,10 @@
         <v>417999</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>558717</v>
+        <v>557917</v>
       </c>
       <c r="L15" t="n">
-        <v>25.18591702060256</v>
+        <v>25.07864072971427</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0</v>
@@ -8226,10 +8232,10 @@
         <v>417999</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>558717</v>
+        <v>557917</v>
       </c>
       <c r="L16" t="n">
-        <v>25.18591702060256</v>
+        <v>25.07864072971427</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -8293,10 +8299,10 @@
         <v>420000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>558717</v>
+        <v>557917</v>
       </c>
       <c r="L17" t="n">
-        <v>24.82777506322521</v>
+        <v>24.71998523077805</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -8360,10 +8366,10 @@
         <v>454000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>601728</v>
+        <v>600867</v>
       </c>
       <c r="L18" t="n">
-        <v>24.55062752605829</v>
+        <v>24.44251390074675</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -8424,10 +8430,10 @@
         <v>454000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>601728</v>
+        <v>600867</v>
       </c>
       <c r="L19" t="n">
-        <v>24.55062752605829</v>
+        <v>24.44251390074675</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -8488,10 +8494,10 @@
         <v>454000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>601728</v>
+        <v>600867</v>
       </c>
       <c r="L20" t="n">
-        <v>24.55062752605829</v>
+        <v>24.44251390074675</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -8552,10 +8558,10 @@
         <v>454000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>601728</v>
+        <v>600867</v>
       </c>
       <c r="L21" t="n">
-        <v>24.55062752605829</v>
+        <v>24.44251390074675</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -8616,10 +8622,10 @@
         <v>455000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>601728</v>
+        <v>600867</v>
       </c>
       <c r="L22" t="n">
-        <v>24.3844394809615</v>
+        <v>24.27608771991139</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -8631,7 +8637,7 @@
         <v>100</v>
       </c>
       <c r="Q22" t="n">
-        <v>31.9</v>
+        <v>31.8</v>
       </c>
       <c r="R22" t="n">
         <v>3</v>
@@ -8680,10 +8686,10 @@
         <v>455000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>601728</v>
+        <v>600867</v>
       </c>
       <c r="L23" t="n">
-        <v>24.3844394809615</v>
+        <v>24.27608771991139</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -8695,7 +8701,7 @@
         <v>100</v>
       </c>
       <c r="Q23" t="n">
-        <v>31.9</v>
+        <v>31.8</v>
       </c>
       <c r="R23" t="n">
         <v>3</v>
@@ -8744,10 +8750,10 @@
         <v>455000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>601728</v>
+        <v>600867</v>
       </c>
       <c r="L24" t="n">
-        <v>24.3844394809615</v>
+        <v>24.27608771991139</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -8759,7 +8765,7 @@
         <v>100</v>
       </c>
       <c r="Q24" t="n">
-        <v>31.9</v>
+        <v>31.8</v>
       </c>
       <c r="R24" t="n">
         <v>3</v>
@@ -8808,10 +8814,10 @@
         <v>455000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>601728</v>
+        <v>600867</v>
       </c>
       <c r="L25" t="n">
-        <v>24.3844394809615</v>
+        <v>24.27608771991139</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -8823,7 +8829,7 @@
         <v>100</v>
       </c>
       <c r="Q25" t="n">
-        <v>31.9</v>
+        <v>31.8</v>
       </c>
       <c r="R25" t="n">
         <v>3</v>
@@ -8872,10 +8878,10 @@
         <v>475000</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>687751</v>
+        <v>686767</v>
       </c>
       <c r="L26" t="n">
-        <v>30.93430616603974</v>
+        <v>30.83534881553715</v>
       </c>
       <c r="M26" s="3" t="n">
         <v>0</v>
@@ -8887,7 +8893,7 @@
         <v>100</v>
       </c>
       <c r="Q26" t="n">
-        <v>34.7</v>
+        <v>34.6</v>
       </c>
       <c r="R26" t="n">
         <v>3</v>
@@ -8936,10 +8942,10 @@
         <v>475000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>687751</v>
+        <v>686767</v>
       </c>
       <c r="L27" t="n">
-        <v>30.93430616603974</v>
+        <v>30.83534881553715</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -8951,7 +8957,7 @@
         <v>100</v>
       </c>
       <c r="Q27" t="n">
-        <v>34.7</v>
+        <v>34.6</v>
       </c>
       <c r="R27" t="n">
         <v>3</v>
@@ -9000,10 +9006,10 @@
         <v>475000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>687751</v>
+        <v>686767</v>
       </c>
       <c r="L28" t="n">
-        <v>30.93430616603974</v>
+        <v>30.83534881553715</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -9015,7 +9021,7 @@
         <v>100</v>
       </c>
       <c r="Q28" t="n">
-        <v>34.7</v>
+        <v>34.6</v>
       </c>
       <c r="R28" t="n">
         <v>3</v>
@@ -9064,10 +9070,10 @@
         <v>475000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>687751</v>
+        <v>686767</v>
       </c>
       <c r="L29" t="n">
-        <v>30.93430616603974</v>
+        <v>30.83534881553715</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -9079,7 +9085,7 @@
         <v>100</v>
       </c>
       <c r="Q29" t="n">
-        <v>34.7</v>
+        <v>34.6</v>
       </c>
       <c r="R29" t="n">
         <v>3</v>
@@ -9128,16 +9134,16 @@
         <v>477000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>644740</v>
+        <v>643817</v>
       </c>
       <c r="L30" t="n">
-        <v>26.0166888978503</v>
+        <v>25.91062367101211</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N30" t="n">
-        <v>1.242031557001153</v>
+        <v>0.9343736954801568</v>
       </c>
       <c r="O30" t="n">
         <v>100</v>
@@ -9146,7 +9152,7 @@
         <v>1.568112774445864</v>
       </c>
       <c r="Q30" t="n">
-        <v>31.5</v>
+        <v>31.4</v>
       </c>
       <c r="R30" t="n">
         <v>4</v>
@@ -9195,16 +9201,16 @@
         <v>477000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>644740</v>
+        <v>643817</v>
       </c>
       <c r="L31" t="n">
-        <v>26.0166888978503</v>
+        <v>25.91062367101211</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N31" t="n">
-        <v>1.242031557001153</v>
+        <v>0.9343736954801568</v>
       </c>
       <c r="O31" t="n">
         <v>100</v>
@@ -9213,7 +9219,7 @@
         <v>1.568112774445864</v>
       </c>
       <c r="Q31" t="n">
-        <v>31.5</v>
+        <v>31.4</v>
       </c>
       <c r="R31" t="n">
         <v>4</v>
@@ -9262,16 +9268,16 @@
         <v>477000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>644740</v>
+        <v>643817</v>
       </c>
       <c r="L32" t="n">
-        <v>26.0166888978503</v>
+        <v>25.91062367101211</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N32" t="n">
-        <v>1.242031557001153</v>
+        <v>0.9343736954801568</v>
       </c>
       <c r="O32" t="n">
         <v>100</v>
@@ -9280,7 +9286,7 @@
         <v>1.568112774445864</v>
       </c>
       <c r="Q32" t="n">
-        <v>31.5</v>
+        <v>31.4</v>
       </c>
       <c r="R32" t="n">
         <v>4</v>
@@ -9329,10 +9335,10 @@
         <v>479999</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>687751</v>
+        <v>686767</v>
       </c>
       <c r="L33" t="n">
-        <v>30.20744426398508</v>
+        <v>30.10744546549267</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -9344,7 +9350,7 @@
         <v>41.73965217391304</v>
       </c>
       <c r="Q33" t="n">
-        <v>21.9</v>
+        <v>21.8</v>
       </c>
       <c r="R33" t="n">
         <v>3</v>
@@ -9393,10 +9399,10 @@
         <v>479999</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>687751</v>
+        <v>686767</v>
       </c>
       <c r="L34" t="n">
-        <v>30.20744426398508</v>
+        <v>30.10744546549267</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -9408,7 +9414,7 @@
         <v>41.73965217391304</v>
       </c>
       <c r="Q34" t="n">
-        <v>21.9</v>
+        <v>21.8</v>
       </c>
       <c r="R34" t="n">
         <v>3</v>
@@ -9457,10 +9463,10 @@
         <v>479999</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>687751</v>
+        <v>686767</v>
       </c>
       <c r="L35" t="n">
-        <v>30.20744426398508</v>
+        <v>30.10744546549267</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
@@ -9472,7 +9478,7 @@
         <v>41.73965217391304</v>
       </c>
       <c r="Q35" t="n">
-        <v>21.9</v>
+        <v>21.8</v>
       </c>
       <c r="R35" t="n">
         <v>3</v>
@@ -9521,10 +9527,10 @@
         <v>479999</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>687751</v>
+        <v>686767</v>
       </c>
       <c r="L36" t="n">
-        <v>30.20744426398508</v>
+        <v>30.10744546549267</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -9536,7 +9542,7 @@
         <v>41.73965217391304</v>
       </c>
       <c r="Q36" t="n">
-        <v>21.9</v>
+        <v>21.8</v>
       </c>
       <c r="R36" t="n">
         <v>3</v>
@@ -9585,16 +9591,16 @@
         <v>479999</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>644740</v>
+        <v>643817</v>
       </c>
       <c r="L37" t="n">
-        <v>25.55154015572169</v>
+        <v>25.44480807434411</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N37" t="n">
-        <v>1.234570441502966</v>
+        <v>1.132855062523301</v>
       </c>
       <c r="O37" t="n">
         <v>0</v>
@@ -9603,7 +9609,7 @@
         <v>0</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="R37" t="n">
         <v>4</v>
@@ -9652,10 +9658,10 @@
         <v>500000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>644740</v>
+        <v>643817</v>
       </c>
       <c r="L38" t="n">
-        <v>22.44935943170891</v>
+        <v>22.33817994865001</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -9716,10 +9722,10 @@
         <v>547999</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>773773</v>
+        <v>772666</v>
       </c>
       <c r="L39" t="n">
-        <v>29.17832490924341</v>
+        <v>29.07685856502033</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -9780,10 +9786,10 @@
         <v>547999</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>773773</v>
+        <v>772666</v>
       </c>
       <c r="L40" t="n">
-        <v>29.17832490924341</v>
+        <v>29.07685856502033</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -9844,10 +9850,10 @@
         <v>547999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>773773</v>
+        <v>772666</v>
       </c>
       <c r="L41" t="n">
-        <v>29.17832490924341</v>
+        <v>29.07685856502033</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
@@ -9859,7 +9865,7 @@
         <v>63.4438956521739</v>
       </c>
       <c r="Q41" t="n">
-        <v>26.4</v>
+        <v>26.3</v>
       </c>
       <c r="R41" t="n">
         <v>3</v>
@@ -9908,10 +9914,10 @@
         <v>547999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>773773</v>
+        <v>772666</v>
       </c>
       <c r="L42" t="n">
-        <v>29.17832490924341</v>
+        <v>29.07685856502033</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -9972,22 +9978,22 @@
         <v>552999</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>773773</v>
+        <v>772666</v>
       </c>
       <c r="L43" t="n">
-        <v>28.53214056318843</v>
+        <v>28.4297484294637</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>2.123897564420468</v>
+        <v>1.688891891363362</v>
       </c>
       <c r="P43" t="n">
         <v>34.11769473304435</v>
       </c>
       <c r="Q43" t="n">
-        <v>20.3</v>
+        <v>20.1</v>
       </c>
       <c r="R43" t="n">
         <v>3</v>
@@ -10036,22 +10042,22 @@
         <v>552999</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>773773</v>
+        <v>772666</v>
       </c>
       <c r="L44" t="n">
-        <v>28.53214056318843</v>
+        <v>28.4297484294637</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>2.123897564420468</v>
+        <v>1.688891891363362</v>
       </c>
       <c r="P44" t="n">
         <v>34.11769473304435</v>
       </c>
       <c r="Q44" t="n">
-        <v>20.3</v>
+        <v>20.1</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -10100,22 +10106,22 @@
         <v>552999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>773773</v>
+        <v>772666</v>
       </c>
       <c r="L45" t="n">
-        <v>28.53214056318843</v>
+        <v>28.4297484294637</v>
       </c>
       <c r="M45" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>2.123897564420468</v>
+        <v>1.688891891363362</v>
       </c>
       <c r="P45" t="n">
         <v>34.11769473304435</v>
       </c>
       <c r="Q45" t="n">
-        <v>20.3</v>
+        <v>20.1</v>
       </c>
       <c r="R45" t="n">
         <v>3</v>
@@ -10164,22 +10170,22 @@
         <v>552999</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>773773</v>
+        <v>772666</v>
       </c>
       <c r="L46" t="n">
-        <v>28.53214056318843</v>
+        <v>28.4297484294637</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N46" t="n">
-        <v>2.123897564420468</v>
+        <v>1.688891891363362</v>
       </c>
       <c r="P46" t="n">
         <v>34.11769473304435</v>
       </c>
       <c r="Q46" t="n">
-        <v>20.3</v>
+        <v>20.1</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -10228,10 +10234,10 @@
         <v>585000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>730762</v>
+        <v>729716</v>
       </c>
       <c r="L47" t="n">
-        <v>19.94657631349194</v>
+        <v>19.83182498396636</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -10243,7 +10249,7 @@
         <v>21.56821735015607</v>
       </c>
       <c r="Q47" t="n">
-        <v>13.2</v>
+        <v>13.1</v>
       </c>
       <c r="R47" t="n">
         <v>3</v>
@@ -10292,10 +10298,10 @@
         <v>595000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>730762</v>
+        <v>729716</v>
       </c>
       <c r="L48" t="n">
-        <v>18.57814172056018</v>
+        <v>18.46142882984613</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -10307,7 +10313,7 @@
         <v>43.82608695652173</v>
       </c>
       <c r="Q48" t="n">
-        <v>17.4</v>
+        <v>17.3</v>
       </c>
       <c r="R48" t="n">
         <v>3</v>
@@ -10356,10 +10362,10 @@
         <v>614999</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>859796</v>
+        <v>858566</v>
       </c>
       <c r="L49" t="n">
-        <v>28.47152115152897</v>
+        <v>28.36904792409669</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -10420,10 +10426,10 @@
         <v>614999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>859796</v>
+        <v>858566</v>
       </c>
       <c r="L50" t="n">
-        <v>28.47152115152897</v>
+        <v>28.36904792409669</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -10484,10 +10490,10 @@
         <v>614999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>859796</v>
+        <v>858566</v>
       </c>
       <c r="L51" t="n">
-        <v>28.47152115152897</v>
+        <v>28.36904792409669</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -10548,10 +10554,10 @@
         <v>614999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>859796</v>
+        <v>858566</v>
       </c>
       <c r="L52" t="n">
-        <v>28.47152115152897</v>
+        <v>28.36904792409669</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -10612,10 +10618,10 @@
         <v>650000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>816785</v>
+        <v>815616</v>
       </c>
       <c r="L53" t="n">
-        <v>20.41969428919483</v>
+        <v>20.30563402385436</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -10676,10 +10682,10 @@
         <v>672000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>859796</v>
+        <v>858566</v>
       </c>
       <c r="L54" t="n">
-        <v>21.84192529390693</v>
+        <v>21.72995436576804</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -10691,7 +10697,7 @@
         <v>58.43478260869565</v>
       </c>
       <c r="Q54" t="n">
-        <v>21.9</v>
+        <v>21.8</v>
       </c>
       <c r="R54" t="n">
         <v>3</v>
@@ -10740,10 +10746,10 @@
         <v>700000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>902807</v>
+        <v>901515</v>
       </c>
       <c r="L55" t="n">
-        <v>22.46404824065387</v>
+        <v>22.35292812654254</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -10755,7 +10761,7 @@
         <v>48.69565217391303</v>
       </c>
       <c r="Q55" t="n">
-        <v>20.1</v>
+        <v>20</v>
       </c>
       <c r="R55" t="n">
         <v>3</v>
@@ -10804,10 +10810,10 @@
         <v>715000</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>945819</v>
+        <v>944465</v>
       </c>
       <c r="L56" t="n">
-        <v>24.40414074997436</v>
+        <v>24.29576532746052</v>
       </c>
       <c r="M56" s="3" t="n">
         <v>0</v>
@@ -10819,7 +10825,7 @@
         <v>64.05209961882153</v>
       </c>
       <c r="Q56" t="n">
-        <v>24.2</v>
+        <v>24.1</v>
       </c>
       <c r="R56" t="n">
         <v>3</v>
@@ -10868,10 +10874,10 @@
         <v>734999</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>988830</v>
+        <v>987415</v>
       </c>
       <c r="L57" t="n">
-        <v>25.66983202370478</v>
+        <v>25.56331431059889</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -10883,7 +10889,7 @@
         <v>73.04377639751551</v>
       </c>
       <c r="Q57" t="n">
-        <v>26.7</v>
+        <v>26.6</v>
       </c>
       <c r="R57" t="n">
         <v>3</v>
@@ -10932,10 +10938,10 @@
         <v>752000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>988830</v>
+        <v>987415</v>
       </c>
       <c r="L58" t="n">
-        <v>23.95052739095699</v>
+        <v>23.84154585457989</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -10996,10 +11002,10 @@
         <v>810000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1074853</v>
+        <v>1073314</v>
       </c>
       <c r="L59" t="n">
-        <v>24.64085786614542</v>
+        <v>24.5328021436411</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -11060,10 +11066,10 @@
         <v>815000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1074853</v>
+        <v>1073314</v>
       </c>
       <c r="L60" t="n">
-        <v>24.17567797643026</v>
+        <v>24.0669552432932</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -11124,10 +11130,10 @@
         <v>875000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1160875</v>
+        <v>1159214</v>
       </c>
       <c r="L61" t="n">
-        <v>24.62582104016367</v>
+        <v>24.5178198330938</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -11139,7 +11145,7 @@
         <v>79.41165705441597</v>
       </c>
       <c r="Q61" t="n">
-        <v>27.6</v>
+        <v>27.5</v>
       </c>
       <c r="R61" t="n">
         <v>3</v>
@@ -11188,10 +11194,10 @@
         <v>992000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1332921</v>
+        <v>1331013</v>
       </c>
       <c r="L62" t="n">
-        <v>25.57698468251306</v>
+        <v>25.47029968903384</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -11252,10 +11258,10 @@
         <v>1050000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1418943</v>
+        <v>1416912</v>
       </c>
       <c r="L63" t="n">
-        <v>26.00125586440047</v>
+        <v>25.89518615129239</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -11267,7 +11273,7 @@
         <v>92.96442687747034</v>
       </c>
       <c r="Q63" t="n">
-        <v>31.1</v>
+        <v>31</v>
       </c>
       <c r="R63" t="n">
         <v>3</v>
@@ -11316,10 +11322,10 @@
         <v>1050000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1418943</v>
+        <v>1416912</v>
       </c>
       <c r="L64" t="n">
-        <v>26.00125586440047</v>
+        <v>25.89518615129239</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -11380,10 +11386,10 @@
         <v>1100000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1504966</v>
+        <v>1502812</v>
       </c>
       <c r="L65" t="n">
-        <v>26.90864777011573</v>
+        <v>26.80388498361738</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -11444,10 +11450,10 @@
         <v>1105000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1504966</v>
+        <v>1502812</v>
       </c>
       <c r="L66" t="n">
-        <v>26.57641435088899</v>
+        <v>26.47117536990655</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -11508,10 +11514,10 @@
         <v>1155000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1590988</v>
+        <v>1588711</v>
       </c>
       <c r="L67" t="n">
-        <v>27.40360078140125</v>
+        <v>27.29955290798641</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -11523,7 +11529,7 @@
         <v>100</v>
       </c>
       <c r="Q67" t="n">
-        <v>33.2</v>
+        <v>33.1</v>
       </c>
       <c r="R67" t="n">
         <v>3</v>
@@ -11778,7 +11784,7 @@
         <v>315000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>300649</v>
+        <v>300219</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -11839,10 +11845,10 @@
         <v>380000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>386672</v>
+        <v>386118</v>
       </c>
       <c r="L3" t="n">
-        <v>1.725493441469773</v>
+        <v>1.584489715579175</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -11854,7 +11860,7 @@
         <v>100</v>
       </c>
       <c r="Q3" t="n">
-        <v>22.2</v>
+        <v>22.1</v>
       </c>
       <c r="R3" t="n">
         <v>3</v>
@@ -11903,7 +11909,7 @@
         <v>415000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>386672</v>
+        <v>386118</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -11964,10 +11970,10 @@
         <v>495000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>472694</v>
+        <v>472018</v>
       </c>
       <c r="L5" t="n">
-        <v>6.916736831861627</v>
+        <v>6.783427750636628</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -11979,7 +11985,7 @@
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="R5" t="n">
         <v>4</v>
@@ -12028,10 +12034,10 @@
         <v>490000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>515706</v>
+        <v>514968</v>
       </c>
       <c r="L6" t="n">
-        <v>4.984623021644115</v>
+        <v>4.848456603128739</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -12092,10 +12098,10 @@
         <v>550000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>558717</v>
+        <v>557917</v>
       </c>
       <c r="L7" t="n">
-        <v>6.929626268755023</v>
+        <v>6.796172190487115</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -12107,7 +12113,7 @@
         <v>25.45360054666915</v>
       </c>
       <c r="Q7" t="n">
-        <v>8.1</v>
+        <v>8</v>
       </c>
       <c r="R7" t="n">
         <v>4</v>
@@ -12156,7 +12162,7 @@
         <v>530000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>472694</v>
+        <v>472018</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -12220,10 +12226,10 @@
         <v>600000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>601728</v>
+        <v>600867</v>
       </c>
       <c r="L9" t="n">
-        <v>8.596575196766645</v>
+        <v>8.465600540552236</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -12284,10 +12290,10 @@
         <v>646000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>730762</v>
+        <v>729716</v>
       </c>
       <c r="L10" t="n">
-        <v>17.20984397108771</v>
+        <v>17.09116971534131</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -12348,7 +12354,7 @@
         <v>615000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>558717</v>
+        <v>557917</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -12412,7 +12418,7 @@
         <v>700000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>644740</v>
+        <v>643817</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -12476,7 +12482,7 @@
         <v>745000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>687751</v>
+        <v>686767</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -12540,7 +12546,7 @@
         <v>930000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>859796</v>
+        <v>858566</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -12611,7 +12617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12657,8 +12663,40 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Apple MacBook Pro 16Inch MX303 14Core CPU 32Core GPU M4 Max 36GB 1TB Space Black</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>990000</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1.01</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F1"/>
+  <autoFilter ref="A1:F2"/>
+  <conditionalFormatting sqref="E2">
+    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: price data 2026-10-07
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MacBook Pro'!$A$1:$S$93</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MacBook Air'!$A$1:$S$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20261006T102505434069+0000</t>
+          <t>20261007T102046536862+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-06T10:25:05.434069+00:00</t>
+          <t>2026-10-07T10:20:46.536862+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>277.095194</v>
+        <v>276.741533</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -729,7 +729,7 @@
         <v>532000</v>
       </c>
       <c r="D22" t="n">
-        <v>51.6</v>
+        <v>51.5</v>
       </c>
       <c r="E22" t="n">
         <v>4</v>
@@ -813,7 +813,7 @@
         <v>700000</v>
       </c>
       <c r="D26" t="n">
-        <v>49.6</v>
+        <v>49.5</v>
       </c>
       <c r="E26" t="n">
         <v>4</v>
@@ -834,7 +834,7 @@
         <v>847999</v>
       </c>
       <c r="D27" t="n">
-        <v>47.4</v>
+        <v>47.3</v>
       </c>
       <c r="E27" t="n">
         <v>5</v>
@@ -852,10 +852,10 @@
         </is>
       </c>
       <c r="C28" s="3" t="n">
-        <v>644999</v>
+        <v>642999</v>
       </c>
       <c r="D28" t="n">
-        <v>44.3</v>
+        <v>44.5</v>
       </c>
       <c r="E28" t="n">
         <v>4</v>
@@ -873,10 +873,10 @@
         </is>
       </c>
       <c r="C29" s="3" t="n">
-        <v>720000</v>
+        <v>717999</v>
       </c>
       <c r="D29" t="n">
-        <v>44.1</v>
+        <v>44.2</v>
       </c>
       <c r="E29" t="n">
         <v>3</v>
@@ -894,10 +894,10 @@
         </is>
       </c>
       <c r="C30" s="3" t="n">
-        <v>725000</v>
+        <v>723500</v>
       </c>
       <c r="D30" t="n">
-        <v>42.7</v>
+        <v>42.6</v>
       </c>
       <c r="E30" t="n">
         <v>3</v>
@@ -1147,10 +1147,10 @@
         <v>470000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>686767</v>
+        <v>685890</v>
       </c>
       <c r="L2" t="n">
-        <v>35.20364257455586</v>
+        <v>35.12079196372596</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1165,7 +1165,7 @@
         <v>28.4414106939704</v>
       </c>
       <c r="Q2" t="n">
-        <v>35.4</v>
+        <v>35.3</v>
       </c>
       <c r="R2" t="n">
         <v>5</v>
@@ -1214,10 +1214,10 @@
         <v>495000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>686767</v>
+        <v>685890</v>
       </c>
       <c r="L3" t="n">
-        <v>27.92315297619135</v>
+        <v>27.83099330796484</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>772666</v>
+        <v>771680</v>
       </c>
       <c r="L4" t="n">
-        <v>35.28911586636399</v>
+        <v>35.20643271822517</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>772666</v>
+        <v>771680</v>
       </c>
       <c r="L5" t="n">
-        <v>32.70067532413747</v>
+        <v>32.61468484345843</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>858566</v>
+        <v>857470</v>
       </c>
       <c r="L6" t="n">
-        <v>38.03621387289969</v>
+        <v>37.95701307334367</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1433,7 +1433,7 @@
         <v>100</v>
       </c>
       <c r="Q6" t="n">
-        <v>51.6</v>
+        <v>51.5</v>
       </c>
       <c r="R6" t="n">
         <v>4</v>
@@ -1606,10 +1606,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>858566</v>
+        <v>857470</v>
       </c>
       <c r="L9" t="n">
-        <v>34.19259556050437</v>
+        <v>34.10848192939694</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1667,31 +1667,31 @@
         </is>
       </c>
       <c r="I10" s="3" t="n">
-        <v>579999</v>
+        <v>578999</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>579999</v>
+        <v>578999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>858566</v>
+        <v>857470</v>
       </c>
       <c r="L10" t="n">
-        <v>32.44561280087961</v>
+        <v>32.47588836927239</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>0</v>
+        <v>-1000</v>
       </c>
       <c r="N10" t="n">
-        <v>0.5145806425053902</v>
+        <v>0.6861075233405204</v>
       </c>
       <c r="O10" t="n">
         <v>100</v>
       </c>
       <c r="P10" t="n">
-        <v>50.00029999999999</v>
+        <v>50.30029999999999</v>
       </c>
       <c r="Q10" t="n">
-        <v>41.5</v>
+        <v>41.6</v>
       </c>
       <c r="R10" t="n">
         <v>4</v>
@@ -1740,10 +1740,10 @@
         <v>587999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>858566</v>
+        <v>857470</v>
       </c>
       <c r="L11" t="n">
-        <v>31.51382654332923</v>
+        <v>31.42628896637783</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -1807,10 +1807,10 @@
         <v>600000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>858566</v>
+        <v>857470</v>
       </c>
       <c r="L12" t="n">
-        <v>30.11603068372146</v>
+        <v>30.02670647369587</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -1825,7 +1825,7 @@
         <v>45.94594594594595</v>
       </c>
       <c r="Q12" t="n">
-        <v>42.1</v>
+        <v>42</v>
       </c>
       <c r="R12" t="n">
         <v>4</v>
@@ -1874,10 +1874,10 @@
         <v>634000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>858566</v>
+        <v>857470</v>
       </c>
       <c r="L13" t="n">
-        <v>26.15593908913235</v>
+        <v>26.06155317387197</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -1935,31 +1935,31 @@
         </is>
       </c>
       <c r="I14" s="3" t="n">
-        <v>644999</v>
+        <v>642999</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>644999</v>
+        <v>642999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>944465</v>
+        <v>943260</v>
       </c>
       <c r="L14" t="n">
-        <v>31.70747460202337</v>
+        <v>31.83226257871637</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>0</v>
+        <v>-2000</v>
       </c>
       <c r="N14" t="n">
-        <v>0</v>
+        <v>0.1552797442232053</v>
       </c>
       <c r="O14" t="n">
         <v>100</v>
       </c>
       <c r="P14" t="n">
-        <v>69.20023999999999</v>
+        <v>69.68024</v>
       </c>
       <c r="Q14" t="n">
-        <v>44.3</v>
+        <v>44.5</v>
       </c>
       <c r="R14" t="n">
         <v>4</v>
@@ -2067,10 +2067,10 @@
         <v>650000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>944465</v>
+        <v>943260</v>
       </c>
       <c r="L16" t="n">
-        <v>31.17796847950957</v>
+        <v>31.09004940313381</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -2134,10 +2134,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1030365</v>
+        <v>1029050</v>
       </c>
       <c r="L17" t="n">
-        <v>32.0629097455756</v>
+        <v>31.9760944560517</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2152,7 +2152,7 @@
         <v>100</v>
       </c>
       <c r="Q17" t="n">
-        <v>49.6</v>
+        <v>49.5</v>
       </c>
       <c r="R17" t="n">
         <v>4</v>
@@ -2201,10 +2201,10 @@
         <v>711999</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>1073314</v>
+        <v>1071944</v>
       </c>
       <c r="L18" t="n">
-        <v>33.6634945598399</v>
+        <v>33.57871306710052</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -2262,26 +2262,26 @@
         </is>
       </c>
       <c r="I19" s="3" t="n">
-        <v>720000</v>
+        <v>717999</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>720000</v>
+        <v>717999</v>
       </c>
       <c r="K19" s="3" t="n"/>
       <c r="M19" s="3" t="n">
-        <v>0</v>
+        <v>-2001</v>
       </c>
       <c r="N19" t="n">
-        <v>0.3459517965064336</v>
+        <v>0.2779166666666667</v>
       </c>
       <c r="O19" t="n">
         <v>100</v>
       </c>
       <c r="P19" t="n">
-        <v>42.39316239316239</v>
+        <v>42.94044444444446</v>
       </c>
       <c r="Q19" t="n">
-        <v>44.1</v>
+        <v>44.2</v>
       </c>
       <c r="R19" t="n">
         <v>3</v>
@@ -2330,10 +2330,10 @@
         <v>720000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>1030365</v>
+        <v>1029050</v>
       </c>
       <c r="L20" t="n">
-        <v>30.12185002402061</v>
+        <v>30.03255429765317</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -2391,26 +2391,26 @@
         </is>
       </c>
       <c r="I21" s="3" t="n">
-        <v>725000</v>
+        <v>723500</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>725000</v>
+        <v>723500</v>
       </c>
       <c r="K21" s="3" t="n"/>
       <c r="M21" s="3" t="n">
-        <v>0</v>
+        <v>-1500</v>
       </c>
       <c r="N21" t="n">
-        <v>0.3435741192949274</v>
+        <v>0.2068965517241379</v>
       </c>
       <c r="O21" t="n">
-        <v>96.7741935483871</v>
+        <v>96.49620066114228</v>
       </c>
       <c r="P21" t="n">
-        <v>41.02564102564102</v>
+        <v>41.43589743589743</v>
       </c>
       <c r="Q21" t="n">
-        <v>42.7</v>
+        <v>42.6</v>
       </c>
       <c r="R21" t="n">
         <v>3</v>
@@ -2459,10 +2459,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1073314</v>
+        <v>1071944</v>
       </c>
       <c r="L22" t="n">
-        <v>30.77515060830288</v>
+        <v>30.68667766226594</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2477,7 +2477,7 @@
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>10.3</v>
+        <v>10.2</v>
       </c>
       <c r="R22" t="n">
         <v>4</v>
@@ -2526,10 +2526,10 @@
         <v>769999</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1030365</v>
+        <v>1029050</v>
       </c>
       <c r="L23" t="n">
-        <v>25.26929777311924</v>
+        <v>25.17380107866479</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -2593,10 +2593,10 @@
         <v>769999</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1030365</v>
+        <v>1029050</v>
       </c>
       <c r="L24" t="n">
-        <v>25.26929777311924</v>
+        <v>25.17380107866479</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -2660,10 +2660,10 @@
         <v>772000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>1030365</v>
+        <v>1029050</v>
       </c>
       <c r="L25" t="n">
-        <v>25.07509474797766</v>
+        <v>24.97934988581702</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -2678,7 +2678,7 @@
         <v>69.59999999999998</v>
       </c>
       <c r="Q25" t="n">
-        <v>20</v>
+        <v>19.9</v>
       </c>
       <c r="R25" t="n">
         <v>4</v>
@@ -2851,10 +2851,10 @@
         <v>810000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>1073314</v>
+        <v>1071944</v>
       </c>
       <c r="L28" t="n">
-        <v>24.5328021436411</v>
+        <v>24.43635115267215</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -2866,7 +2866,7 @@
         <v>61.99999999999999</v>
       </c>
       <c r="Q28" t="n">
-        <v>24.7</v>
+        <v>24.6</v>
       </c>
       <c r="R28" t="n">
         <v>3</v>
@@ -2915,10 +2915,10 @@
         <v>810000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>1245113</v>
+        <v>1243524</v>
       </c>
       <c r="L29" t="n">
-        <v>34.94566356627872</v>
+        <v>34.86253582560529</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -2982,10 +2982,10 @@
         <v>822999</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1288063</v>
+        <v>1286419</v>
       </c>
       <c r="L30" t="n">
-        <v>36.10568737709258</v>
+        <v>36.02403260523982</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -3049,10 +3049,10 @@
         <v>823000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1288063</v>
+        <v>1286419</v>
       </c>
       <c r="L31" t="n">
-        <v>36.10560974113844</v>
+        <v>36.02395487006955</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -3116,10 +3116,10 @@
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1373963</v>
+        <v>1372209</v>
       </c>
       <c r="L32" t="n">
-        <v>38.28079795453007</v>
+        <v>38.20190656088104</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3134,7 +3134,7 @@
         <v>100</v>
       </c>
       <c r="Q32" t="n">
-        <v>47.4</v>
+        <v>47.3</v>
       </c>
       <c r="R32" t="n">
         <v>5</v>
@@ -3183,10 +3183,10 @@
         <v>930000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1373963</v>
+        <v>1372209</v>
       </c>
       <c r="L33" t="n">
-        <v>38.13523362710641</v>
+        <v>38.05615616863029</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3250,10 +3250,10 @@
         <v>860000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>1245113</v>
+        <v>1243524</v>
       </c>
       <c r="L34" t="n">
-        <v>30.92996378641939</v>
+        <v>30.84170470372908</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -3268,7 +3268,7 @@
         <v>89.80112187659357</v>
       </c>
       <c r="Q34" t="n">
-        <v>25.3</v>
+        <v>25.2</v>
       </c>
       <c r="R34" t="n">
         <v>4</v>
@@ -3282,7 +3282,7 @@
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 MGDT4 M5 Pro 18 Core CPU 20 Core GPU 24GB 2TB Space Black</t>
+          <t>Macbook Pro 14 CTO M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -3297,7 +3297,7 @@
         <v>24</v>
       </c>
       <c r="E35" t="n">
-        <v>2048</v>
+        <v>1024</v>
       </c>
       <c r="F35" t="n">
         <v>18</v>
@@ -3311,10 +3311,10 @@
         </is>
       </c>
       <c r="I35" s="3" t="n">
-        <v>864999</v>
+        <v>875000</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>864999</v>
+        <v>875000</v>
       </c>
       <c r="K35" s="3" t="n"/>
       <c r="M35" s="3" t="n">
@@ -3324,13 +3324,13 @@
         <v>0</v>
       </c>
       <c r="O35" t="n">
-        <v>10.001</v>
+        <v>0</v>
       </c>
       <c r="P35" t="n">
-        <v>70.3298656898657</v>
+        <v>0</v>
       </c>
       <c r="Q35" t="n">
-        <v>20.9</v>
+        <v>0</v>
       </c>
       <c r="R35" t="n">
         <v>3</v>
@@ -3344,7 +3344,7 @@
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Space Black</t>
+          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 24GB 2TB Space Black</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -3352,20 +3352,20 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>M5 Pro</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="D36" t="n">
         <v>24</v>
       </c>
       <c r="E36" t="n">
-        <v>1024</v>
+        <v>2048</v>
       </c>
       <c r="F36" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="G36" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -3373,26 +3373,28 @@
         </is>
       </c>
       <c r="I36" s="3" t="n">
-        <v>875000</v>
+        <v>880000</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>875000</v>
-      </c>
-      <c r="K36" s="3" t="n"/>
+        <v>880000</v>
+      </c>
+      <c r="K36" s="3" t="n">
+        <v>1157734</v>
+      </c>
+      <c r="L36" t="n">
+        <v>23.98944835342142</v>
+      </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N36" t="n">
         <v>0</v>
       </c>
-      <c r="O36" t="n">
-        <v>0</v>
-      </c>
       <c r="P36" t="n">
-        <v>0</v>
+        <v>73.14285714285714</v>
       </c>
       <c r="Q36" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="R36" t="n">
         <v>3</v>
@@ -3406,7 +3408,7 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 MGDP4 M5 Pro 18 Core CPU 20 Core GPU 24GB 2TB Silver</t>
+          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 32GB 2TB Space Black</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -3414,47 +3416,49 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>M5 Pro</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="E37" t="n">
         <v>2048</v>
       </c>
       <c r="F37" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="G37" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I37" s="3" t="n">
-        <v>875000</v>
+        <v>940000</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>875000</v>
-      </c>
-      <c r="K37" s="3" t="n"/>
+        <v>940000</v>
+      </c>
+      <c r="K37" s="3" t="n">
+        <v>1243524</v>
+      </c>
+      <c r="L37" t="n">
+        <v>24.40837490872713</v>
+      </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N37" t="n">
         <v>0</v>
       </c>
-      <c r="O37" t="n">
-        <v>0</v>
-      </c>
       <c r="P37" t="n">
-        <v>68.37606837606837</v>
+        <v>83</v>
       </c>
       <c r="Q37" t="n">
-        <v>17.1</v>
+        <v>28.2</v>
       </c>
       <c r="R37" t="n">
         <v>3</v>
@@ -3468,7 +3472,7 @@
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 24GB 2TB Space Black</t>
+          <t>Macbook Pro 14 MGDT4 M5 Pro 18 Core CPU 20 Core GPU 24GB 2TB Space Black</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -3476,7 +3480,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M5 Pro</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -3486,10 +3490,10 @@
         <v>2048</v>
       </c>
       <c r="F38" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="G38" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -3497,28 +3501,26 @@
         </is>
       </c>
       <c r="I38" s="3" t="n">
-        <v>880000</v>
+        <v>955000</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>880000</v>
-      </c>
-      <c r="K38" s="3" t="n">
-        <v>1159214</v>
-      </c>
-      <c r="L38" t="n">
-        <v>24.08649308928291</v>
-      </c>
+        <v>955000</v>
+      </c>
+      <c r="K38" s="3" t="n"/>
       <c r="M38" s="3" t="n">
-        <v>0</v>
+        <v>90001</v>
       </c>
       <c r="N38" t="n">
         <v>0</v>
       </c>
+      <c r="O38" t="n">
+        <v>0</v>
+      </c>
       <c r="P38" t="n">
-        <v>73.14285714285714</v>
+        <v>52.74725274725276</v>
       </c>
       <c r="Q38" t="n">
-        <v>26</v>
+        <v>13.2</v>
       </c>
       <c r="R38" t="n">
         <v>3</v>
@@ -3532,7 +3534,7 @@
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 CTO 10 Core CPU 10 Core GPU 32GB 2TB Space Black</t>
+          <t>Macbook Pro 14 MGDP4 M5 Pro 18 Core CPU 20 Core GPU 24GB 2TB Silver</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -3540,49 +3542,47 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M5 Pro</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="E39" t="n">
         <v>2048</v>
       </c>
       <c r="F39" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="G39" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I39" s="3" t="n">
-        <v>940000</v>
+        <v>955000</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>940000</v>
-      </c>
-      <c r="K39" s="3" t="n">
-        <v>1245113</v>
-      </c>
-      <c r="L39" t="n">
-        <v>24.50484413864444</v>
-      </c>
+        <v>955000</v>
+      </c>
+      <c r="K39" s="3" t="n"/>
       <c r="M39" s="3" t="n">
-        <v>0</v>
+        <v>80000</v>
       </c>
       <c r="N39" t="n">
         <v>0</v>
       </c>
+      <c r="O39" t="n">
+        <v>0</v>
+      </c>
       <c r="P39" t="n">
-        <v>83</v>
+        <v>52.74725274725276</v>
       </c>
       <c r="Q39" t="n">
-        <v>28.3</v>
+        <v>13.2</v>
       </c>
       <c r="R39" t="n">
         <v>3</v>
@@ -3631,10 +3631,10 @@
         <v>990000</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>1502812</v>
+        <v>1500894</v>
       </c>
       <c r="L40" t="n">
-        <v>34.12349648525564</v>
+        <v>34.03931256970845</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -3760,13 +3760,13 @@
         <v>1000000</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>1502812</v>
+        <v>1500894</v>
       </c>
       <c r="L42" t="n">
-        <v>33.45807725783398</v>
+        <v>33.37304299970551</v>
       </c>
       <c r="M42" s="3" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="N42" t="n">
         <v>0</v>
@@ -3821,25 +3821,25 @@
         </is>
       </c>
       <c r="I43" s="3" t="n">
-        <v>1055000</v>
+        <v>1054000</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>1055000</v>
+        <v>1054000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1545762</v>
+        <v>1543789</v>
       </c>
       <c r="L43" t="n">
-        <v>31.74887207733144</v>
+        <v>31.72642116247751</v>
       </c>
       <c r="M43" s="3" t="n">
-        <v>0</v>
+        <v>-1000</v>
       </c>
       <c r="N43" t="n">
-        <v>0</v>
+        <v>0.09478672985781991</v>
       </c>
       <c r="P43" t="n">
-        <v>57.6271186440678</v>
+        <v>57.84723750825446</v>
       </c>
       <c r="Q43" t="n">
         <v>26</v>
@@ -3885,25 +3885,25 @@
         </is>
       </c>
       <c r="I44" s="3" t="n">
-        <v>1055000</v>
+        <v>1054000</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>1055000</v>
+        <v>1054000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1545762</v>
+        <v>1543789</v>
       </c>
       <c r="L44" t="n">
-        <v>31.74887207733144</v>
+        <v>31.72642116247751</v>
       </c>
       <c r="M44" s="3" t="n">
-        <v>0</v>
+        <v>-1000</v>
       </c>
       <c r="N44" t="n">
-        <v>0</v>
+        <v>0.09478672985781991</v>
       </c>
       <c r="P44" t="n">
-        <v>57.6271186440678</v>
+        <v>57.84723750825446</v>
       </c>
       <c r="Q44" t="n">
         <v>26</v>
@@ -4017,10 +4017,10 @@
         <v>1115000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1502812</v>
+        <v>1500894</v>
       </c>
       <c r="L46" t="n">
-        <v>25.80575614248489</v>
+        <v>25.71094294467164</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -4032,7 +4032,7 @@
         <v>9.358196283135744</v>
       </c>
       <c r="Q46" t="n">
-        <v>14.2</v>
+        <v>14.1</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -4081,10 +4081,10 @@
         <v>1123000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1717561</v>
+        <v>1715369</v>
       </c>
       <c r="L47" t="n">
-        <v>34.61658712558098</v>
+        <v>34.53303633212445</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -4148,10 +4148,10 @@
         <v>1130000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1502812</v>
+        <v>1500894</v>
       </c>
       <c r="L48" t="n">
-        <v>24.8076273013524</v>
+        <v>24.71153858966722</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -4163,7 +4163,7 @@
         <v>88.39999999999999</v>
       </c>
       <c r="Q48" t="n">
-        <v>29.6</v>
+        <v>29.5</v>
       </c>
       <c r="R48" t="n">
         <v>3</v>
@@ -4274,10 +4274,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1760510</v>
+        <v>1758263</v>
       </c>
       <c r="L50" t="n">
-        <v>34.39401082640826</v>
+        <v>34.31016861527542</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4289,7 +4289,7 @@
         <v>22.53136001640632</v>
       </c>
       <c r="Q50" t="n">
-        <v>19.6</v>
+        <v>19.5</v>
       </c>
       <c r="R50" t="n">
         <v>3</v>
@@ -4338,10 +4338,10 @@
         <v>1155000</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>1760510</v>
+        <v>1758263</v>
       </c>
       <c r="L51" t="n">
-        <v>34.39401082640826</v>
+        <v>34.31016861527542</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -4353,7 +4353,7 @@
         <v>22.53136001640632</v>
       </c>
       <c r="Q51" t="n">
-        <v>19.6</v>
+        <v>19.5</v>
       </c>
       <c r="R51" t="n">
         <v>3</v>
@@ -4402,10 +4402,10 @@
         <v>1185000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1588711</v>
+        <v>1586684</v>
       </c>
       <c r="L52" t="n">
-        <v>25.41122960689515</v>
+        <v>25.31594192668483</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -4466,10 +4466,10 @@
         <v>1185000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1588711</v>
+        <v>1586684</v>
       </c>
       <c r="L53" t="n">
-        <v>25.41122960689515</v>
+        <v>25.31594192668483</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -4481,7 +4481,7 @@
         <v>94.72727272727272</v>
       </c>
       <c r="Q53" t="n">
-        <v>31.2</v>
+        <v>31.1</v>
       </c>
       <c r="R53" t="n">
         <v>3</v>
@@ -4530,22 +4530,22 @@
         <v>1200000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1889360</v>
+        <v>1886948</v>
       </c>
       <c r="L54" t="n">
-        <v>36.4864292670534</v>
+        <v>36.40524275178754</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N54" t="n">
-        <v>0.2908184461985874</v>
+        <v>0</v>
       </c>
       <c r="P54" t="n">
         <v>3.948101568096777</v>
       </c>
       <c r="Q54" t="n">
-        <v>16.6</v>
+        <v>16.4</v>
       </c>
       <c r="R54" t="n">
         <v>3</v>
@@ -4594,22 +4594,22 @@
         <v>1200000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1889360</v>
+        <v>1886948</v>
       </c>
       <c r="L55" t="n">
-        <v>36.4864292670534</v>
+        <v>36.40524275178754</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N55" t="n">
-        <v>0.2908184461985874</v>
+        <v>0</v>
       </c>
       <c r="P55" t="n">
         <v>3.948101568096777</v>
       </c>
       <c r="Q55" t="n">
-        <v>16.6</v>
+        <v>16.4</v>
       </c>
       <c r="R55" t="n">
         <v>3</v>
@@ -4720,10 +4720,10 @@
         <v>1240000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1674611</v>
+        <v>1672474</v>
       </c>
       <c r="L57" t="n">
-        <v>25.95295265587053</v>
+        <v>25.85833920288148</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -4735,7 +4735,7 @@
         <v>100</v>
       </c>
       <c r="Q57" t="n">
-        <v>32.6</v>
+        <v>32.5</v>
       </c>
       <c r="R57" t="n">
         <v>3</v>
@@ -4846,10 +4846,10 @@
         <v>1280000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1717561</v>
+        <v>1715369</v>
       </c>
       <c r="L59" t="n">
-        <v>25.47571818409943</v>
+        <v>25.38048664747934</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -4913,10 +4913,10 @@
         <v>1298000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1760510</v>
+        <v>1758263</v>
       </c>
       <c r="L60" t="n">
-        <v>26.27136454777309</v>
+        <v>26.17714187240475</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -4928,7 +4928,7 @@
         <v>61.28109178956637</v>
       </c>
       <c r="Q60" t="n">
-        <v>25.5</v>
+        <v>25.4</v>
       </c>
       <c r="R60" t="n">
         <v>3</v>
@@ -4977,10 +4977,10 @@
         <v>1300000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1717561</v>
+        <v>1715369</v>
       </c>
       <c r="L61" t="n">
-        <v>24.31127628072598</v>
+        <v>24.21455675134621</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -5103,10 +5103,10 @@
         <v>1335000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1803460</v>
+        <v>1801158</v>
       </c>
       <c r="L63" t="n">
-        <v>25.97562463265057</v>
+        <v>25.88101654602206</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -5167,10 +5167,10 @@
         <v>1420000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1932309</v>
+        <v>1929843</v>
       </c>
       <c r="L64" t="n">
-        <v>26.51278858609053</v>
+        <v>26.41888485229109</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -5182,7 +5182,7 @@
         <v>81.47332893095606</v>
       </c>
       <c r="Q64" t="n">
-        <v>30.1</v>
+        <v>30</v>
       </c>
       <c r="R64" t="n">
         <v>3</v>
@@ -5231,10 +5231,10 @@
         <v>1430000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1932309</v>
+        <v>1929843</v>
       </c>
       <c r="L65" t="n">
-        <v>25.99527301275313</v>
+        <v>25.90070798505371</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -5295,10 +5295,10 @@
         <v>1430000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>2147058</v>
+        <v>2144318</v>
       </c>
       <c r="L66" t="n">
-        <v>33.39723472770647</v>
+        <v>33.31213001056746</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -5359,10 +5359,10 @@
         <v>1430000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>2147058</v>
+        <v>2144318</v>
       </c>
       <c r="L67" t="n">
-        <v>33.39723472770647</v>
+        <v>33.31213001056746</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -5485,10 +5485,10 @@
         <v>1480000</v>
       </c>
       <c r="K69" s="3" t="n">
-        <v>2018209</v>
+        <v>2015633</v>
       </c>
       <c r="L69" t="n">
-        <v>26.66765434105189</v>
+        <v>26.57393483833614</v>
       </c>
       <c r="M69" s="3" t="n">
         <v>0</v>
@@ -5611,10 +5611,10 @@
         <v>1605000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2190008</v>
+        <v>2187213</v>
       </c>
       <c r="L71" t="n">
-        <v>26.71259648366581</v>
+        <v>26.61894383400245</v>
       </c>
       <c r="M71" s="3" t="n">
         <v>0</v>
@@ -5626,7 +5626,7 @@
         <v>36.44392794886694</v>
       </c>
       <c r="Q71" t="n">
-        <v>19.3</v>
+        <v>19.2</v>
       </c>
       <c r="R71" t="n">
         <v>3</v>
@@ -5675,10 +5675,10 @@
         <v>1610000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2190008</v>
+        <v>2187213</v>
       </c>
       <c r="L72" t="n">
-        <v>26.48428681539063</v>
+        <v>26.39034241292458</v>
       </c>
       <c r="M72" s="3" t="n">
         <v>0</v>
@@ -5690,7 +5690,7 @@
         <v>25.72147975982957</v>
       </c>
       <c r="Q72" t="n">
-        <v>16.9</v>
+        <v>16.8</v>
       </c>
       <c r="R72" t="n">
         <v>3</v>
@@ -5739,10 +5739,10 @@
         <v>1615000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2190008</v>
+        <v>2187213</v>
       </c>
       <c r="L73" t="n">
-        <v>26.25597714711544</v>
+        <v>26.1617409918467</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
@@ -5803,10 +5803,10 @@
         <v>1630000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2232958</v>
+        <v>2230108</v>
       </c>
       <c r="L74" t="n">
-        <v>27.00265746153757</v>
+        <v>26.90936941170562</v>
       </c>
       <c r="M74" s="3" t="n">
         <v>0</v>
@@ -5867,10 +5867,10 @@
         <v>1690000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2318857</v>
+        <v>2315898</v>
       </c>
       <c r="L75" t="n">
-        <v>27.11926608669702</v>
+        <v>27.02614709283397</v>
       </c>
       <c r="M75" s="3" t="n">
         <v>0</v>
@@ -5882,7 +5882,7 @@
         <v>16.88768606224628</v>
       </c>
       <c r="Q75" t="n">
-        <v>15.7</v>
+        <v>15.6</v>
       </c>
       <c r="R75" t="n">
         <v>3</v>
@@ -5931,10 +5931,10 @@
         <v>1705000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2318857</v>
+        <v>2315898</v>
       </c>
       <c r="L76" t="n">
-        <v>26.47239566734818</v>
+        <v>26.3784501735396</v>
       </c>
       <c r="M76" s="3" t="n">
         <v>0</v>
@@ -5995,10 +5995,10 @@
         <v>1725000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2361807</v>
+        <v>2358793</v>
       </c>
       <c r="L77" t="n">
-        <v>26.96270271025532</v>
+        <v>26.86937768596057</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
@@ -6010,7 +6010,7 @@
         <v>100</v>
       </c>
       <c r="Q77" t="n">
-        <v>34.3</v>
+        <v>34.2</v>
       </c>
       <c r="R77" t="n">
         <v>3</v>
@@ -6059,10 +6059,10 @@
         <v>1780000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2447707</v>
+        <v>2444582</v>
       </c>
       <c r="L78" t="n">
-        <v>27.27887774149438</v>
+        <v>27.18591562892961</v>
       </c>
       <c r="M78" s="3" t="n">
         <v>0</v>
@@ -6123,10 +6123,10 @@
         <v>1875000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2576556</v>
+        <v>2573267</v>
       </c>
       <c r="L79" t="n">
-        <v>27.22843982432363</v>
+        <v>27.13542745467144</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
@@ -6138,7 +6138,7 @@
         <v>19.64044075004835</v>
       </c>
       <c r="Q79" t="n">
-        <v>17.2</v>
+        <v>17.1</v>
       </c>
       <c r="R79" t="n">
         <v>3</v>
@@ -6187,10 +6187,10 @@
         <v>1910000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2619506</v>
+        <v>2616162</v>
       </c>
       <c r="L80" t="n">
-        <v>27.08548863793402</v>
+        <v>26.99228870383409</v>
       </c>
       <c r="M80" s="3" t="n">
         <v>0</v>
@@ -6251,10 +6251,10 @@
         <v>2020000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2748355</v>
+        <v>2744847</v>
       </c>
       <c r="L81" t="n">
-        <v>26.50148907255431</v>
+        <v>26.40755568525313</v>
       </c>
       <c r="M81" s="3" t="n">
         <v>0</v>
@@ -6315,10 +6315,10 @@
         <v>2110000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>2877204</v>
+        <v>2873532</v>
       </c>
       <c r="L82" t="n">
-        <v>26.66491496605732</v>
+        <v>26.57120226954146</v>
       </c>
       <c r="M82" s="3" t="n">
         <v>0</v>
@@ -6330,7 +6330,7 @@
         <v>79.02382335851249</v>
       </c>
       <c r="Q82" t="n">
-        <v>28.4</v>
+        <v>28.3</v>
       </c>
       <c r="R82" t="n">
         <v>3</v>
@@ -6379,10 +6379,10 @@
         <v>2210000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3006053</v>
+        <v>3002217</v>
       </c>
       <c r="L83" t="n">
-        <v>26.4816688195451</v>
+        <v>26.38773279879502</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
@@ -6443,10 +6443,10 @@
         <v>2215000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3049003</v>
+        <v>3045112</v>
       </c>
       <c r="L84" t="n">
-        <v>27.35330204660343</v>
+        <v>27.26047514836893</v>
       </c>
       <c r="M84" s="3" t="n">
         <v>0</v>
@@ -6507,10 +6507,10 @@
         <v>2315000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3177852</v>
+        <v>3173796</v>
       </c>
       <c r="L85" t="n">
-        <v>27.15205113391058</v>
+        <v>27.05895400964649</v>
       </c>
       <c r="M85" s="3" t="n">
         <v>0</v>
@@ -6522,7 +6522,7 @@
         <v>65.11105977094954</v>
       </c>
       <c r="Q85" t="n">
-        <v>26.6</v>
+        <v>26.5</v>
       </c>
       <c r="R85" t="n">
         <v>3</v>
@@ -6571,10 +6571,10 @@
         <v>2395000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3306702</v>
+        <v>3302481</v>
       </c>
       <c r="L86" t="n">
-        <v>27.57133845142381</v>
+        <v>27.47876520712761</v>
       </c>
       <c r="M86" s="3" t="n">
         <v>0</v>
@@ -6635,10 +6635,10 @@
         <v>2410000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3306702</v>
+        <v>3302481</v>
       </c>
       <c r="L87" t="n">
-        <v>27.11771426635966</v>
+        <v>27.02456123138937</v>
       </c>
       <c r="M87" s="3" t="n">
         <v>0</v>
@@ -6650,7 +6650,7 @@
         <v>88.47569242688358</v>
       </c>
       <c r="Q87" t="n">
-        <v>30.6</v>
+        <v>30.5</v>
       </c>
       <c r="R87" t="n">
         <v>3</v>
@@ -6699,10 +6699,10 @@
         <v>2499000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3435551</v>
+        <v>3431166</v>
       </c>
       <c r="L88" t="n">
-        <v>27.26057625108752</v>
+        <v>27.16761590666263</v>
       </c>
       <c r="M88" s="3" t="n">
         <v>0</v>
@@ -6714,7 +6714,7 @@
         <v>63.67326854471646</v>
       </c>
       <c r="Q88" t="n">
-        <v>26.5</v>
+        <v>26.4</v>
       </c>
       <c r="R88" t="n">
         <v>3</v>
@@ -6763,10 +6763,10 @@
         <v>2510000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3435551</v>
+        <v>3431166</v>
       </c>
       <c r="L89" t="n">
-        <v>26.94039471397747</v>
+        <v>26.84702518036143</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
@@ -6827,10 +6827,10 @@
         <v>2530000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3478501</v>
+        <v>3474061</v>
       </c>
       <c r="L90" t="n">
-        <v>27.26752126850043</v>
+        <v>27.17456601942223</v>
       </c>
       <c r="M90" s="3" t="n">
         <v>0</v>
@@ -6842,7 +6842,7 @@
         <v>79.17877203176447</v>
       </c>
       <c r="Q90" t="n">
-        <v>28.7</v>
+        <v>28.6</v>
       </c>
       <c r="R90" t="n">
         <v>3</v>
@@ -6891,10 +6891,10 @@
         <v>2610000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>3607350</v>
+        <v>3602746</v>
       </c>
       <c r="L91" t="n">
-        <v>27.64771923988523</v>
+        <v>27.55525923836985</v>
       </c>
       <c r="M91" s="3" t="n">
         <v>0</v>
@@ -6906,7 +6906,7 @@
         <v>74.15426251691474</v>
       </c>
       <c r="Q91" t="n">
-        <v>28.5</v>
+        <v>28.4</v>
       </c>
       <c r="R91" t="n">
         <v>3</v>
@@ -6955,10 +6955,10 @@
         <v>3015000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4165697</v>
+        <v>4160380</v>
       </c>
       <c r="L92" t="n">
-        <v>27.6231564609716</v>
+        <v>27.53065825717843</v>
       </c>
       <c r="M92" s="3" t="n">
         <v>0</v>
@@ -6970,7 +6970,7 @@
         <v>100</v>
       </c>
       <c r="Q92" t="n">
-        <v>33.3</v>
+        <v>33.2</v>
       </c>
       <c r="R92" t="n">
         <v>3</v>
@@ -7019,10 +7019,10 @@
         <v>3098000</v>
       </c>
       <c r="K93" s="3" t="n">
-        <v>4294546</v>
+        <v>4289065</v>
       </c>
       <c r="L93" t="n">
-        <v>27.86199053404015</v>
+        <v>27.7698053072173</v>
       </c>
       <c r="M93" s="3" t="n">
         <v>0</v>
@@ -7034,7 +7034,7 @@
         <v>100</v>
       </c>
       <c r="Q93" t="n">
-        <v>34.4</v>
+        <v>34.3</v>
       </c>
       <c r="R93" t="n">
         <v>3</v>
@@ -7318,10 +7318,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>429068</v>
+        <v>428520</v>
       </c>
       <c r="L2" t="n">
-        <v>27.75061295645446</v>
+        <v>27.65821898627835</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7385,10 +7385,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>429068</v>
+        <v>428520</v>
       </c>
       <c r="L3" t="n">
-        <v>27.75061295645446</v>
+        <v>27.65821898627835</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7452,10 +7452,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>429068</v>
+        <v>428520</v>
       </c>
       <c r="L4" t="n">
-        <v>27.75037989316379</v>
+        <v>27.65798562494166</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7519,10 +7519,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>429068</v>
+        <v>428520</v>
       </c>
       <c r="L5" t="n">
-        <v>27.75037989316379</v>
+        <v>27.65798562494166</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7586,10 +7586,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514968</v>
+        <v>514310</v>
       </c>
       <c r="L6" t="n">
-        <v>25.43225986857436</v>
+        <v>25.33685909276506</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7650,10 +7650,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>514968</v>
+        <v>514310</v>
       </c>
       <c r="L7" t="n">
-        <v>25.43225986857436</v>
+        <v>25.33685909276506</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7714,10 +7714,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>514968</v>
+        <v>514310</v>
       </c>
       <c r="L8" t="n">
-        <v>25.43225986857436</v>
+        <v>25.33685909276506</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7778,10 +7778,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>514968</v>
+        <v>514310</v>
       </c>
       <c r="L9" t="n">
-        <v>25.43225986857436</v>
+        <v>25.33685909276506</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7842,10 +7842,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>514968</v>
+        <v>514310</v>
       </c>
       <c r="L10" t="n">
-        <v>25.23807304531543</v>
+        <v>25.14242382998581</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7906,10 +7906,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>514968</v>
+        <v>514310</v>
       </c>
       <c r="L11" t="n">
-        <v>25.23807304531543</v>
+        <v>25.14242382998581</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7970,10 +7970,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>514968</v>
+        <v>514310</v>
       </c>
       <c r="L12" t="n">
-        <v>25.23807304531543</v>
+        <v>25.14242382998581</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -8034,10 +8034,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>514968</v>
+        <v>514310</v>
       </c>
       <c r="L13" t="n">
-        <v>25.23807304531543</v>
+        <v>25.14242382998581</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -8092,31 +8092,31 @@
         </is>
       </c>
       <c r="I14" s="3" t="n">
-        <v>417999</v>
+        <v>415000</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>417999</v>
+        <v>415000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>557917</v>
+        <v>557205</v>
       </c>
       <c r="L14" t="n">
-        <v>25.07864072971427</v>
+        <v>25.52112777164599</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>0</v>
+        <v>-2999</v>
       </c>
       <c r="N14" t="n">
-        <v>1.647294117647059</v>
+        <v>2.352941176470588</v>
       </c>
       <c r="O14" t="n">
         <v>100</v>
       </c>
       <c r="P14" t="n">
-        <v>1.392</v>
+        <v>3.478260869565196</v>
       </c>
       <c r="Q14" t="n">
-        <v>31.3</v>
+        <v>32</v>
       </c>
       <c r="R14" t="n">
         <v>4</v>
@@ -8159,31 +8159,31 @@
         </is>
       </c>
       <c r="I15" s="3" t="n">
-        <v>417999</v>
+        <v>415000</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>417999</v>
+        <v>415000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>557917</v>
+        <v>557205</v>
       </c>
       <c r="L15" t="n">
-        <v>25.07864072971427</v>
+        <v>25.52112777164599</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>0</v>
+        <v>-2999</v>
       </c>
       <c r="N15" t="n">
-        <v>1.647294117647059</v>
+        <v>2.352941176470588</v>
       </c>
       <c r="O15" t="n">
         <v>100</v>
       </c>
       <c r="P15" t="n">
-        <v>1.392</v>
+        <v>3.478260869565196</v>
       </c>
       <c r="Q15" t="n">
-        <v>31.3</v>
+        <v>32</v>
       </c>
       <c r="R15" t="n">
         <v>4</v>
@@ -8226,31 +8226,31 @@
         </is>
       </c>
       <c r="I16" s="3" t="n">
-        <v>417999</v>
+        <v>415000</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>417999</v>
+        <v>415000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>557917</v>
+        <v>557205</v>
       </c>
       <c r="L16" t="n">
-        <v>25.07864072971427</v>
+        <v>25.52112777164599</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0</v>
+        <v>-2999</v>
       </c>
       <c r="N16" t="n">
-        <v>1.647294117647059</v>
+        <v>2.352941176470588</v>
       </c>
       <c r="O16" t="n">
         <v>100</v>
       </c>
       <c r="P16" t="n">
-        <v>1.392</v>
+        <v>3.478260869565196</v>
       </c>
       <c r="Q16" t="n">
-        <v>31.3</v>
+        <v>32</v>
       </c>
       <c r="R16" t="n">
         <v>4</v>
@@ -8299,10 +8299,10 @@
         <v>420000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>557917</v>
+        <v>557205</v>
       </c>
       <c r="L17" t="n">
-        <v>24.71998523077805</v>
+        <v>24.62379196166581</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -8317,7 +8317,7 @@
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>8.6</v>
+        <v>8.5</v>
       </c>
       <c r="R17" t="n">
         <v>4</v>
@@ -8366,10 +8366,10 @@
         <v>454000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>600867</v>
+        <v>600100</v>
       </c>
       <c r="L18" t="n">
-        <v>24.44251390074675</v>
+        <v>24.34594234294284</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -8381,7 +8381,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q18" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="R18" t="n">
         <v>3</v>
@@ -8430,10 +8430,10 @@
         <v>454000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>600867</v>
+        <v>600100</v>
       </c>
       <c r="L19" t="n">
-        <v>24.44251390074675</v>
+        <v>24.34594234294284</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -8445,7 +8445,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q19" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="R19" t="n">
         <v>3</v>
@@ -8494,10 +8494,10 @@
         <v>454000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>600867</v>
+        <v>600100</v>
       </c>
       <c r="L20" t="n">
-        <v>24.44251390074675</v>
+        <v>24.34594234294284</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -8509,7 +8509,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q20" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="R20" t="n">
         <v>3</v>
@@ -8558,10 +8558,10 @@
         <v>454000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>600867</v>
+        <v>600100</v>
       </c>
       <c r="L21" t="n">
-        <v>24.44251390074675</v>
+        <v>24.34594234294284</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -8573,7 +8573,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q21" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="R21" t="n">
         <v>3</v>
@@ -8622,10 +8622,10 @@
         <v>455000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>600867</v>
+        <v>600100</v>
       </c>
       <c r="L22" t="n">
-        <v>24.27608771991139</v>
+        <v>24.1793034494251</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -8686,10 +8686,10 @@
         <v>455000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>600867</v>
+        <v>600100</v>
       </c>
       <c r="L23" t="n">
-        <v>24.27608771991139</v>
+        <v>24.1793034494251</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -8750,10 +8750,10 @@
         <v>455000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>600867</v>
+        <v>600100</v>
       </c>
       <c r="L24" t="n">
-        <v>24.27608771991139</v>
+        <v>24.1793034494251</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -8814,10 +8814,10 @@
         <v>455000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>600867</v>
+        <v>600100</v>
       </c>
       <c r="L25" t="n">
-        <v>24.27608771991139</v>
+        <v>24.1793034494251</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -8843,22 +8843,22 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MC6L4 M4 10C CPU 10C GPU 24GB 512GB Midnight</t>
+          <t>Apple MacBook Air 13 MDHF4 M5 10C CPU 10C GPU 16GB 1TB Midnight</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E26" t="n">
-        <v>512</v>
+        <v>1024</v>
       </c>
       <c r="F26" t="n">
         <v>10</v>
@@ -8872,28 +8872,28 @@
         </is>
       </c>
       <c r="I26" s="3" t="n">
-        <v>475000</v>
+        <v>468000</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>475000</v>
+        <v>468000</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>686767</v>
+        <v>685890</v>
       </c>
       <c r="L26" t="n">
-        <v>30.83534881553715</v>
+        <v>31.76748458207584</v>
       </c>
       <c r="M26" s="3" t="n">
-        <v>0</v>
+        <v>-11999</v>
       </c>
       <c r="N26" t="n">
-        <v>0</v>
+        <v>2.499796874576822</v>
       </c>
       <c r="P26" t="n">
-        <v>100</v>
+        <v>47.99999999999999</v>
       </c>
       <c r="Q26" t="n">
-        <v>34.6</v>
+        <v>24.8</v>
       </c>
       <c r="R26" t="n">
         <v>3</v>
@@ -8907,22 +8907,22 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MC6K4 M4 10C CPU 10C GPU 24GB 512GB Starlight</t>
+          <t>Apple MacBook Air 13 MDHJ4 M5 10C CPU 10C GPU 16GB 1TB Sky Blue</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E27" t="n">
-        <v>512</v>
+        <v>1024</v>
       </c>
       <c r="F27" t="n">
         <v>10</v>
@@ -8932,32 +8932,32 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Starlight</t>
+          <t>Sky Blue</t>
         </is>
       </c>
       <c r="I27" s="3" t="n">
-        <v>475000</v>
+        <v>468000</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>475000</v>
+        <v>468000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>686767</v>
+        <v>685890</v>
       </c>
       <c r="L27" t="n">
-        <v>30.83534881553715</v>
+        <v>31.76748458207584</v>
       </c>
       <c r="M27" s="3" t="n">
-        <v>0</v>
+        <v>-11999</v>
       </c>
       <c r="N27" t="n">
-        <v>0</v>
+        <v>2.499796874576822</v>
       </c>
       <c r="P27" t="n">
-        <v>100</v>
+        <v>47.99999999999999</v>
       </c>
       <c r="Q27" t="n">
-        <v>34.6</v>
+        <v>24.8</v>
       </c>
       <c r="R27" t="n">
         <v>3</v>
@@ -8971,22 +8971,22 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MC6J4 M4 10C CPU 10C GPU 24GB 512GB Silver</t>
+          <t>Apple MacBook Air 13 MDH84 M5 10C CPU 10C GPU 16GB 1TB Silver</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E28" t="n">
-        <v>512</v>
+        <v>1024</v>
       </c>
       <c r="F28" t="n">
         <v>10</v>
@@ -9000,28 +9000,28 @@
         </is>
       </c>
       <c r="I28" s="3" t="n">
-        <v>475000</v>
+        <v>468000</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>475000</v>
+        <v>468000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>686767</v>
+        <v>685890</v>
       </c>
       <c r="L28" t="n">
-        <v>30.83534881553715</v>
+        <v>31.76748458207584</v>
       </c>
       <c r="M28" s="3" t="n">
-        <v>0</v>
+        <v>-11999</v>
       </c>
       <c r="N28" t="n">
-        <v>0</v>
+        <v>2.499796874576822</v>
       </c>
       <c r="P28" t="n">
-        <v>100</v>
+        <v>47.99999999999999</v>
       </c>
       <c r="Q28" t="n">
-        <v>34.6</v>
+        <v>24.8</v>
       </c>
       <c r="R28" t="n">
         <v>3</v>
@@ -9035,22 +9035,22 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MC7D4 M4 10C CPU 10C GPU 24GB 512GB Sky Blue</t>
+          <t>Apple MacBook Air 13 MDHC4 M5 10C CPU 10C GPU 16GB 1TB Starlight</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E29" t="n">
-        <v>512</v>
+        <v>1024</v>
       </c>
       <c r="F29" t="n">
         <v>10</v>
@@ -9060,32 +9060,32 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Sky Blue</t>
+          <t>Starlight</t>
         </is>
       </c>
       <c r="I29" s="3" t="n">
-        <v>475000</v>
+        <v>468000</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>475000</v>
+        <v>468000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>686767</v>
+        <v>685890</v>
       </c>
       <c r="L29" t="n">
-        <v>30.83534881553715</v>
+        <v>31.76748458207584</v>
       </c>
       <c r="M29" s="3" t="n">
-        <v>0</v>
+        <v>-11999</v>
       </c>
       <c r="N29" t="n">
-        <v>0</v>
+        <v>2.499796874576822</v>
       </c>
       <c r="P29" t="n">
-        <v>100</v>
+        <v>47.99999999999999</v>
       </c>
       <c r="Q29" t="n">
-        <v>34.6</v>
+        <v>24.8</v>
       </c>
       <c r="R29" t="n">
         <v>3</v>
@@ -9099,7 +9099,7 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MDVD4 M5 10C CPU 10C GPU 16GB 512GB Starlight</t>
+          <t>Apple MacBook Air 15 MC6L4 M4 10C CPU 10C GPU 24GB 512GB Midnight</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -9107,11 +9107,11 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E30" t="n">
         <v>512</v>
@@ -9124,38 +9124,35 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Starlight</t>
+          <t>Midnight</t>
         </is>
       </c>
       <c r="I30" s="3" t="n">
-        <v>477000</v>
+        <v>475000</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>477000</v>
+        <v>475000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>643817</v>
+        <v>685890</v>
       </c>
       <c r="L30" t="n">
-        <v>25.91062367101211</v>
+        <v>30.74691277026929</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N30" t="n">
-        <v>0.9343736954801568</v>
-      </c>
-      <c r="O30" t="n">
+        <v>0</v>
+      </c>
+      <c r="P30" t="n">
         <v>100</v>
       </c>
-      <c r="P30" t="n">
-        <v>1.568112774445864</v>
-      </c>
       <c r="Q30" t="n">
-        <v>31.4</v>
+        <v>34.6</v>
       </c>
       <c r="R30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S30" t="inlineStr">
         <is>
@@ -9166,7 +9163,7 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MDVQ4 M5 10C CPU 10C GPU 16GB 512GB Sky Blue</t>
+          <t>Apple MacBook Air 15 MC6K4 M4 10C CPU 10C GPU 24GB 512GB Starlight</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -9174,11 +9171,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E31" t="n">
         <v>512</v>
@@ -9191,38 +9188,35 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Sky Blue</t>
+          <t>Starlight</t>
         </is>
       </c>
       <c r="I31" s="3" t="n">
-        <v>477000</v>
+        <v>475000</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>477000</v>
+        <v>475000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>643817</v>
+        <v>685890</v>
       </c>
       <c r="L31" t="n">
-        <v>25.91062367101211</v>
+        <v>30.74691277026929</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N31" t="n">
-        <v>0.9343736954801568</v>
-      </c>
-      <c r="O31" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" t="n">
         <v>100</v>
       </c>
-      <c r="P31" t="n">
-        <v>1.568112774445864</v>
-      </c>
       <c r="Q31" t="n">
-        <v>31.4</v>
+        <v>34.6</v>
       </c>
       <c r="R31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S31" t="inlineStr">
         <is>
@@ -9233,7 +9227,7 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MDVH4 M5 10C CPU 10C GPU 16GB 512GB Midnight</t>
+          <t>Apple MacBook Air 15 MC6J4 M4 10C CPU 10C GPU 24GB 512GB Silver</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -9241,11 +9235,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E32" t="n">
         <v>512</v>
@@ -9258,38 +9252,35 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Midnight</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I32" s="3" t="n">
-        <v>477000</v>
+        <v>475000</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>477000</v>
+        <v>475000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>643817</v>
+        <v>685890</v>
       </c>
       <c r="L32" t="n">
-        <v>25.91062367101211</v>
+        <v>30.74691277026929</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N32" t="n">
-        <v>0.9343736954801568</v>
-      </c>
-      <c r="O32" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" t="n">
         <v>100</v>
       </c>
-      <c r="P32" t="n">
-        <v>1.568112774445864</v>
-      </c>
       <c r="Q32" t="n">
-        <v>31.4</v>
+        <v>34.6</v>
       </c>
       <c r="R32" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S32" t="inlineStr">
         <is>
@@ -9300,22 +9291,22 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHF4 M5 10C CPU 10C GPU 16GB 1TB Midnight</t>
+          <t>Apple MacBook Air 15 MC7D4 M4 10C CPU 10C GPU 24GB 512GB Sky Blue</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E33" t="n">
-        <v>1024</v>
+        <v>512</v>
       </c>
       <c r="F33" t="n">
         <v>10</v>
@@ -9325,20 +9316,20 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Midnight</t>
+          <t>Sky Blue</t>
         </is>
       </c>
       <c r="I33" s="3" t="n">
-        <v>479999</v>
+        <v>475000</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>479999</v>
+        <v>475000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>686767</v>
+        <v>685890</v>
       </c>
       <c r="L33" t="n">
-        <v>30.10744546549267</v>
+        <v>30.74691277026929</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -9347,10 +9338,10 @@
         <v>0</v>
       </c>
       <c r="P33" t="n">
-        <v>41.73965217391304</v>
+        <v>100</v>
       </c>
       <c r="Q33" t="n">
-        <v>21.8</v>
+        <v>34.6</v>
       </c>
       <c r="R33" t="n">
         <v>3</v>
@@ -9364,11 +9355,11 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHJ4 M5 10C CPU 10C GPU 16GB 1TB Sky Blue</t>
+          <t>Apple MacBook Air 15 MDVD4 M5 10C CPU 10C GPU 16GB 512GB Starlight</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -9379,7 +9370,7 @@
         <v>16</v>
       </c>
       <c r="E34" t="n">
-        <v>1024</v>
+        <v>512</v>
       </c>
       <c r="F34" t="n">
         <v>10</v>
@@ -9389,35 +9380,38 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Sky Blue</t>
+          <t>Starlight</t>
         </is>
       </c>
       <c r="I34" s="3" t="n">
-        <v>479999</v>
+        <v>477000</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>479999</v>
+        <v>477000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>686767</v>
+        <v>642995</v>
       </c>
       <c r="L34" t="n">
-        <v>30.10744546549267</v>
+        <v>25.815908366317</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N34" t="n">
-        <v>0</v>
+        <v>0.6247929683186839</v>
+      </c>
+      <c r="O34" t="n">
+        <v>100</v>
       </c>
       <c r="P34" t="n">
-        <v>41.73965217391304</v>
+        <v>1.568112774445864</v>
       </c>
       <c r="Q34" t="n">
-        <v>21.8</v>
+        <v>31.3</v>
       </c>
       <c r="R34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S34" t="inlineStr">
         <is>
@@ -9428,11 +9422,11 @@
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDH84 M5 10C CPU 10C GPU 16GB 1TB Silver</t>
+          <t>Apple MacBook Air 15 MDVQ4 M5 10C CPU 10C GPU 16GB 512GB Sky Blue</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -9443,7 +9437,7 @@
         <v>16</v>
       </c>
       <c r="E35" t="n">
-        <v>1024</v>
+        <v>512</v>
       </c>
       <c r="F35" t="n">
         <v>10</v>
@@ -9453,35 +9447,38 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Sky Blue</t>
         </is>
       </c>
       <c r="I35" s="3" t="n">
-        <v>479999</v>
+        <v>477000</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>479999</v>
+        <v>477000</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>686767</v>
+        <v>642995</v>
       </c>
       <c r="L35" t="n">
-        <v>30.10744546549267</v>
+        <v>25.815908366317</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N35" t="n">
-        <v>0</v>
+        <v>0.6247929683186839</v>
+      </c>
+      <c r="O35" t="n">
+        <v>100</v>
       </c>
       <c r="P35" t="n">
-        <v>41.73965217391304</v>
+        <v>1.568112774445864</v>
       </c>
       <c r="Q35" t="n">
-        <v>21.8</v>
+        <v>31.3</v>
       </c>
       <c r="R35" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S35" t="inlineStr">
         <is>
@@ -9492,11 +9489,11 @@
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHC4 M5 10C CPU 10C GPU 16GB 1TB Starlight</t>
+          <t>Apple MacBook Air 15 MDVH4 M5 10C CPU 10C GPU 16GB 512GB Midnight</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -9507,7 +9504,7 @@
         <v>16</v>
       </c>
       <c r="E36" t="n">
-        <v>1024</v>
+        <v>512</v>
       </c>
       <c r="F36" t="n">
         <v>10</v>
@@ -9517,35 +9514,38 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Starlight</t>
+          <t>Midnight</t>
         </is>
       </c>
       <c r="I36" s="3" t="n">
-        <v>479999</v>
+        <v>477000</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>479999</v>
+        <v>477000</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>686767</v>
+        <v>642995</v>
       </c>
       <c r="L36" t="n">
-        <v>30.10744546549267</v>
+        <v>25.815908366317</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N36" t="n">
-        <v>0</v>
+        <v>0.6247929683186839</v>
+      </c>
+      <c r="O36" t="n">
+        <v>100</v>
       </c>
       <c r="P36" t="n">
-        <v>41.73965217391304</v>
+        <v>1.568112774445864</v>
       </c>
       <c r="Q36" t="n">
-        <v>21.8</v>
+        <v>31.3</v>
       </c>
       <c r="R36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S36" t="inlineStr">
         <is>
@@ -9591,16 +9591,16 @@
         <v>479999</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>643817</v>
+        <v>642995</v>
       </c>
       <c r="L37" t="n">
-        <v>25.44480807434411</v>
+        <v>25.34949727447336</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N37" t="n">
-        <v>1.132855062523301</v>
+        <v>1.030929960680331</v>
       </c>
       <c r="O37" t="n">
         <v>0</v>
@@ -9609,7 +9609,7 @@
         <v>0</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.800000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="R37" t="n">
         <v>4</v>
@@ -9658,10 +9658,10 @@
         <v>500000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>643817</v>
+        <v>642995</v>
       </c>
       <c r="L38" t="n">
-        <v>22.33817994865001</v>
+        <v>22.23889765861321</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -9673,7 +9673,7 @@
         <v>31.30434782608695</v>
       </c>
       <c r="Q38" t="n">
-        <v>16.3</v>
+        <v>16.2</v>
       </c>
       <c r="R38" t="n">
         <v>3</v>
@@ -9716,28 +9716,28 @@
         </is>
       </c>
       <c r="I39" s="3" t="n">
-        <v>547999</v>
+        <v>544999</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>547999</v>
+        <v>544999</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>772666</v>
+        <v>771680</v>
       </c>
       <c r="L39" t="n">
-        <v>29.07685856502033</v>
+        <v>29.375</v>
       </c>
       <c r="M39" s="3" t="n">
-        <v>0</v>
+        <v>-3000</v>
       </c>
       <c r="N39" t="n">
-        <v>0.3636370247945905</v>
+        <v>0.9090925619864764</v>
       </c>
       <c r="P39" t="n">
-        <v>63.4438956521739</v>
+        <v>64.69606956521737</v>
       </c>
       <c r="Q39" t="n">
-        <v>26.2</v>
+        <v>26.8</v>
       </c>
       <c r="R39" t="n">
         <v>3</v>
@@ -9780,28 +9780,28 @@
         </is>
       </c>
       <c r="I40" s="3" t="n">
-        <v>547999</v>
+        <v>544999</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>547999</v>
+        <v>544999</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>772666</v>
+        <v>771680</v>
       </c>
       <c r="L40" t="n">
-        <v>29.07685856502033</v>
+        <v>29.375</v>
       </c>
       <c r="M40" s="3" t="n">
-        <v>0</v>
+        <v>-3000</v>
       </c>
       <c r="N40" t="n">
-        <v>0.3636370247945905</v>
+        <v>0.9090925619864764</v>
       </c>
       <c r="P40" t="n">
-        <v>63.4438956521739</v>
+        <v>64.69606956521737</v>
       </c>
       <c r="Q40" t="n">
-        <v>26.2</v>
+        <v>26.8</v>
       </c>
       <c r="R40" t="n">
         <v>3</v>
@@ -9844,28 +9844,28 @@
         </is>
       </c>
       <c r="I41" s="3" t="n">
-        <v>547999</v>
+        <v>544999</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>547999</v>
+        <v>544999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>772666</v>
+        <v>771680</v>
       </c>
       <c r="L41" t="n">
-        <v>29.07685856502033</v>
+        <v>29.375</v>
       </c>
       <c r="M41" s="3" t="n">
-        <v>0</v>
+        <v>-3000</v>
       </c>
       <c r="N41" t="n">
-        <v>0.7246389939112209</v>
+        <v>1.268118239344636</v>
       </c>
       <c r="P41" t="n">
-        <v>63.4438956521739</v>
+        <v>64.69606956521737</v>
       </c>
       <c r="Q41" t="n">
-        <v>26.3</v>
+        <v>26.9</v>
       </c>
       <c r="R41" t="n">
         <v>3</v>
@@ -9908,28 +9908,28 @@
         </is>
       </c>
       <c r="I42" s="3" t="n">
-        <v>547999</v>
+        <v>544999</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>547999</v>
+        <v>544999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>772666</v>
+        <v>771680</v>
       </c>
       <c r="L42" t="n">
-        <v>29.07685856502033</v>
+        <v>29.375</v>
       </c>
       <c r="M42" s="3" t="n">
-        <v>0</v>
+        <v>-3000</v>
       </c>
       <c r="N42" t="n">
-        <v>0.3636370247945905</v>
+        <v>0.9090925619864764</v>
       </c>
       <c r="P42" t="n">
-        <v>63.4438956521739</v>
+        <v>64.69606956521737</v>
       </c>
       <c r="Q42" t="n">
-        <v>26.2</v>
+        <v>26.8</v>
       </c>
       <c r="R42" t="n">
         <v>3</v>
@@ -9972,28 +9972,28 @@
         </is>
       </c>
       <c r="I43" s="3" t="n">
-        <v>552999</v>
+        <v>549999</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>552999</v>
+        <v>549999</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>772666</v>
+        <v>771680</v>
       </c>
       <c r="L43" t="n">
-        <v>28.4297484294637</v>
+        <v>28.72706303130832</v>
       </c>
       <c r="M43" s="3" t="n">
-        <v>0</v>
+        <v>-3000</v>
       </c>
       <c r="N43" t="n">
-        <v>1.688891891363362</v>
+        <v>1.78571747449549</v>
       </c>
       <c r="P43" t="n">
-        <v>34.11769473304435</v>
+        <v>35.29417147279201</v>
       </c>
       <c r="Q43" t="n">
-        <v>20.1</v>
+        <v>20.5</v>
       </c>
       <c r="R43" t="n">
         <v>3</v>
@@ -10036,28 +10036,28 @@
         </is>
       </c>
       <c r="I44" s="3" t="n">
-        <v>552999</v>
+        <v>549999</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>552999</v>
+        <v>549999</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>772666</v>
+        <v>771680</v>
       </c>
       <c r="L44" t="n">
-        <v>28.4297484294637</v>
+        <v>28.72706303130832</v>
       </c>
       <c r="M44" s="3" t="n">
-        <v>0</v>
+        <v>-3000</v>
       </c>
       <c r="N44" t="n">
-        <v>1.688891891363362</v>
+        <v>1.78571747449549</v>
       </c>
       <c r="P44" t="n">
-        <v>34.11769473304435</v>
+        <v>35.29417147279201</v>
       </c>
       <c r="Q44" t="n">
-        <v>20.1</v>
+        <v>20.5</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -10100,28 +10100,28 @@
         </is>
       </c>
       <c r="I45" s="3" t="n">
-        <v>552999</v>
+        <v>549999</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>552999</v>
+        <v>549999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>772666</v>
+        <v>771680</v>
       </c>
       <c r="L45" t="n">
-        <v>28.4297484294637</v>
+        <v>28.72706303130832</v>
       </c>
       <c r="M45" s="3" t="n">
-        <v>0</v>
+        <v>-3000</v>
       </c>
       <c r="N45" t="n">
-        <v>1.688891891363362</v>
+        <v>1.78571747449549</v>
       </c>
       <c r="P45" t="n">
-        <v>34.11769473304435</v>
+        <v>35.29417147279201</v>
       </c>
       <c r="Q45" t="n">
-        <v>20.1</v>
+        <v>20.5</v>
       </c>
       <c r="R45" t="n">
         <v>3</v>
@@ -10164,28 +10164,28 @@
         </is>
       </c>
       <c r="I46" s="3" t="n">
-        <v>552999</v>
+        <v>549999</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>552999</v>
+        <v>549999</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>772666</v>
+        <v>771680</v>
       </c>
       <c r="L46" t="n">
-        <v>28.4297484294637</v>
+        <v>28.72706303130832</v>
       </c>
       <c r="M46" s="3" t="n">
-        <v>0</v>
+        <v>-3000</v>
       </c>
       <c r="N46" t="n">
-        <v>1.688891891363362</v>
+        <v>1.78571747449549</v>
       </c>
       <c r="P46" t="n">
-        <v>34.11769473304435</v>
+        <v>35.29417147279201</v>
       </c>
       <c r="Q46" t="n">
-        <v>20.1</v>
+        <v>20.5</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -10234,10 +10234,10 @@
         <v>585000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>729716</v>
+        <v>728785</v>
       </c>
       <c r="L47" t="n">
-        <v>19.83182498396636</v>
+        <v>19.72941265256557</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -10298,10 +10298,10 @@
         <v>595000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>729716</v>
+        <v>728785</v>
       </c>
       <c r="L48" t="n">
-        <v>18.46142882984613</v>
+        <v>18.35726586030174</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -10356,28 +10356,28 @@
         </is>
       </c>
       <c r="I49" s="3" t="n">
-        <v>614999</v>
+        <v>619999</v>
       </c>
       <c r="J49" s="3" t="n">
-        <v>614999</v>
+        <v>619999</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>858566</v>
+        <v>857470</v>
       </c>
       <c r="L49" t="n">
-        <v>28.36904792409669</v>
+        <v>27.69437997830828</v>
       </c>
       <c r="M49" s="3" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="N49" t="n">
         <v>0</v>
       </c>
       <c r="P49" t="n">
-        <v>58.0393100094641</v>
+        <v>56.47067435646721</v>
       </c>
       <c r="Q49" t="n">
-        <v>24.6</v>
+        <v>24</v>
       </c>
       <c r="R49" t="n">
         <v>3</v>
@@ -10420,28 +10420,28 @@
         </is>
       </c>
       <c r="I50" s="3" t="n">
-        <v>614999</v>
+        <v>619999</v>
       </c>
       <c r="J50" s="3" t="n">
-        <v>614999</v>
+        <v>619999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>858566</v>
+        <v>857470</v>
       </c>
       <c r="L50" t="n">
-        <v>28.36904792409669</v>
+        <v>27.69437997830828</v>
       </c>
       <c r="M50" s="3" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="N50" t="n">
         <v>0</v>
       </c>
       <c r="P50" t="n">
-        <v>58.0393100094641</v>
+        <v>56.47067435646721</v>
       </c>
       <c r="Q50" t="n">
-        <v>24.6</v>
+        <v>24</v>
       </c>
       <c r="R50" t="n">
         <v>3</v>
@@ -10484,28 +10484,28 @@
         </is>
       </c>
       <c r="I51" s="3" t="n">
-        <v>614999</v>
+        <v>619999</v>
       </c>
       <c r="J51" s="3" t="n">
-        <v>614999</v>
+        <v>619999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>858566</v>
+        <v>857470</v>
       </c>
       <c r="L51" t="n">
-        <v>28.36904792409669</v>
+        <v>27.69437997830828</v>
       </c>
       <c r="M51" s="3" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="N51" t="n">
         <v>0</v>
       </c>
       <c r="P51" t="n">
-        <v>58.0393100094641</v>
+        <v>56.47067435646721</v>
       </c>
       <c r="Q51" t="n">
-        <v>24.6</v>
+        <v>24</v>
       </c>
       <c r="R51" t="n">
         <v>3</v>
@@ -10548,28 +10548,28 @@
         </is>
       </c>
       <c r="I52" s="3" t="n">
-        <v>614999</v>
+        <v>619999</v>
       </c>
       <c r="J52" s="3" t="n">
-        <v>614999</v>
+        <v>619999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>858566</v>
+        <v>857470</v>
       </c>
       <c r="L52" t="n">
-        <v>28.36904792409669</v>
+        <v>27.69437997830828</v>
       </c>
       <c r="M52" s="3" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="N52" t="n">
         <v>0</v>
       </c>
       <c r="P52" t="n">
-        <v>58.0393100094641</v>
+        <v>56.47067435646721</v>
       </c>
       <c r="Q52" t="n">
-        <v>24.6</v>
+        <v>24</v>
       </c>
       <c r="R52" t="n">
         <v>3</v>
@@ -10618,10 +10618,10 @@
         <v>650000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>815616</v>
+        <v>814575</v>
       </c>
       <c r="L53" t="n">
-        <v>20.30563402385436</v>
+        <v>20.20378725102047</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -10633,7 +10633,7 @@
         <v>47.05854671135535</v>
       </c>
       <c r="Q53" t="n">
-        <v>18.8</v>
+        <v>18.7</v>
       </c>
       <c r="R53" t="n">
         <v>3</v>
@@ -10682,10 +10682,10 @@
         <v>672000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>858566</v>
+        <v>857470</v>
       </c>
       <c r="L54" t="n">
-        <v>21.72995436576804</v>
+        <v>21.62991125053938</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -10746,10 +10746,10 @@
         <v>700000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>901515</v>
+        <v>900365</v>
       </c>
       <c r="L55" t="n">
-        <v>22.35292812654254</v>
+        <v>22.25375264476073</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -10810,10 +10810,10 @@
         <v>715000</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>944465</v>
+        <v>943260</v>
       </c>
       <c r="L56" t="n">
-        <v>24.29576532746052</v>
+        <v>24.19905434344719</v>
       </c>
       <c r="M56" s="3" t="n">
         <v>0</v>
@@ -10874,10 +10874,10 @@
         <v>734999</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>987415</v>
+        <v>986155</v>
       </c>
       <c r="L57" t="n">
-        <v>25.56331431059889</v>
+        <v>25.46820733049064</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -10938,10 +10938,10 @@
         <v>752000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>987415</v>
+        <v>986155</v>
       </c>
       <c r="L58" t="n">
-        <v>23.84154585457989</v>
+        <v>23.74423898879994</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -10953,7 +10953,7 @@
         <v>54.37884642534079</v>
       </c>
       <c r="Q58" t="n">
-        <v>21.9</v>
+        <v>21.8</v>
       </c>
       <c r="R58" t="n">
         <v>3</v>
@@ -11002,10 +11002,10 @@
         <v>810000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1073314</v>
+        <v>1071944</v>
       </c>
       <c r="L59" t="n">
-        <v>24.5328021436411</v>
+        <v>24.43635115267215</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -11066,10 +11066,10 @@
         <v>815000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1073314</v>
+        <v>1071944</v>
       </c>
       <c r="L60" t="n">
-        <v>24.0669552432932</v>
+        <v>23.9699088758368</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -11081,7 +11081,7 @@
         <v>79.56521739130434</v>
       </c>
       <c r="Q60" t="n">
-        <v>27.4</v>
+        <v>27.3</v>
       </c>
       <c r="R60" t="n">
         <v>3</v>
@@ -11130,10 +11130,10 @@
         <v>875000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1159214</v>
+        <v>1157734</v>
       </c>
       <c r="L61" t="n">
-        <v>24.5178198330938</v>
+        <v>24.42132648777698</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -11194,10 +11194,10 @@
         <v>992000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1331013</v>
+        <v>1329314</v>
       </c>
       <c r="L62" t="n">
-        <v>25.47029968903384</v>
+        <v>25.37504306732646</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -11209,7 +11209,7 @@
         <v>85.14782608695651</v>
       </c>
       <c r="Q62" t="n">
-        <v>29.2</v>
+        <v>29.1</v>
       </c>
       <c r="R62" t="n">
         <v>3</v>
@@ -11258,10 +11258,10 @@
         <v>1050000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1416912</v>
+        <v>1415104</v>
       </c>
       <c r="L63" t="n">
-        <v>25.89518615129239</v>
+        <v>25.80050653520872</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -11322,10 +11322,10 @@
         <v>1050000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1416912</v>
+        <v>1415104</v>
       </c>
       <c r="L64" t="n">
-        <v>25.89518615129239</v>
+        <v>25.80050653520872</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -11337,7 +11337,7 @@
         <v>86.27443803627732</v>
       </c>
       <c r="Q64" t="n">
-        <v>29.6</v>
+        <v>29.5</v>
       </c>
       <c r="R64" t="n">
         <v>3</v>
@@ -11386,10 +11386,10 @@
         <v>1100000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1502812</v>
+        <v>1500894</v>
       </c>
       <c r="L65" t="n">
-        <v>26.80388498361738</v>
+        <v>26.71034729967606</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -11401,7 +11401,7 @@
         <v>94.11761630126171</v>
       </c>
       <c r="Q65" t="n">
-        <v>31.7</v>
+        <v>31.6</v>
       </c>
       <c r="R65" t="n">
         <v>3</v>
@@ -11450,10 +11450,10 @@
         <v>1105000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1502812</v>
+        <v>1500894</v>
       </c>
       <c r="L66" t="n">
-        <v>26.47117536990655</v>
+        <v>26.37721251467459</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -11465,7 +11465,7 @@
         <v>100</v>
       </c>
       <c r="Q66" t="n">
-        <v>32.8</v>
+        <v>32.7</v>
       </c>
       <c r="R66" t="n">
         <v>3</v>
@@ -11514,10 +11514,10 @@
         <v>1155000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1588711</v>
+        <v>1586684</v>
       </c>
       <c r="L67" t="n">
-        <v>27.29955290798641</v>
+        <v>27.20667757411053</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -11784,7 +11784,7 @@
         <v>315000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>300219</v>
+        <v>299836</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -11845,10 +11845,10 @@
         <v>380000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>386118</v>
+        <v>385625</v>
       </c>
       <c r="L3" t="n">
-        <v>1.584489715579175</v>
+        <v>1.458670988654781</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -11909,7 +11909,7 @@
         <v>415000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>386118</v>
+        <v>385625</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -11970,10 +11970,10 @@
         <v>495000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>472018</v>
+        <v>471415</v>
       </c>
       <c r="L5" t="n">
-        <v>6.783427750636628</v>
+        <v>6.664191847947137</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -12034,10 +12034,10 @@
         <v>490000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514968</v>
+        <v>514310</v>
       </c>
       <c r="L6" t="n">
-        <v>4.848456603128739</v>
+        <v>4.726721238163754</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -12049,7 +12049,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="R6" t="n">
         <v>3</v>
@@ -12098,10 +12098,10 @@
         <v>550000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>557917</v>
+        <v>557205</v>
       </c>
       <c r="L7" t="n">
-        <v>6.796172190487115</v>
+        <v>6.677075762062437</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -12162,7 +12162,7 @@
         <v>530000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>472018</v>
+        <v>471415</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -12226,10 +12226,10 @@
         <v>600000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>600867</v>
+        <v>600100</v>
       </c>
       <c r="L9" t="n">
-        <v>8.465600540552236</v>
+        <v>8.348608565239127</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -12241,7 +12241,7 @@
         <v>30.25295873936471</v>
       </c>
       <c r="Q9" t="n">
-        <v>9.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="R9" t="n">
         <v>4</v>
@@ -12290,10 +12290,10 @@
         <v>646000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>729716</v>
+        <v>728785</v>
       </c>
       <c r="L10" t="n">
-        <v>17.09116971534131</v>
+        <v>16.98525628271713</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -12305,7 +12305,7 @@
         <v>100</v>
       </c>
       <c r="Q10" t="n">
-        <v>26</v>
+        <v>25.9</v>
       </c>
       <c r="R10" t="n">
         <v>4</v>
@@ -12354,7 +12354,7 @@
         <v>615000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>557917</v>
+        <v>557205</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -12418,7 +12418,7 @@
         <v>700000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>643817</v>
+        <v>642995</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -12482,7 +12482,7 @@
         <v>745000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>686767</v>
+        <v>685890</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -12546,7 +12546,7 @@
         <v>930000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>858566</v>
+        <v>857470</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -12617,7 +12617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12666,30 +12666,654 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 16Inch MX303 14Core CPU 32Core GPU M4 Max 36GB 1TB Space Black</t>
+          <t>Apple MacBook Air 13 MDHF4 M5 10C CPU 10C GPU 16GB 1TB Midnight</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>479999</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>468000</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>-11999</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-2.5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 13 MDHJ4 M5 10C CPU 10C GPU 16GB 1TB Sky Blue</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>479999</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>468000</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>-11999</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-2.5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 13 MDH84 M5 10C CPU 10C GPU 16GB 1TB Silver</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>479999</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>468000</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>-11999</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-2.5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 13 MDHC4 M5 10C CPU 10C GPU 16GB 1TB Starlight</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>479999</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>468000</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>-11999</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-2.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 13 MDHG4 M5 10C CPU 10C GPU 24GB 1TB Midnight</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>547999</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>544999</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>-3000</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-0.55</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 13 MDHK4 M5 10C CPU 10C GPU 24GB 1TB Sky Blue</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>547999</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>544999</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>-3000</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-0.55</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 13 MDH94 M5 10C CPU 10C GPU 24GB 1TB Silver</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>547999</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>544999</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>-3000</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-0.55</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 13 MDHD4 M5 10C CPU 10C GPU 24GB 1TB Starlight</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>547999</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>544999</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>-3000</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-0.55</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 15 MDVK4 M5 10C CPU 10C GPU 16GB 1TB Midnight</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>552999</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>549999</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>-3000</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-0.54</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 15 MDVA4 M5 10C CPU 10C GPU 16GB 1TB Silver</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>552999</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>549999</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>-3000</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-0.54</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 15 MDVE4 M5 10C CPU 10C GPU 16GB 1TB Starlight</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>552999</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>549999</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>-3000</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-0.54</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 15 MDVT4 M5 10C CPU 10C GPU 16GB 1TB Sky Blue</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>552999</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>549999</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>-3000</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-0.54</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 13 MDHE4 M5 10C CPU 8C GPU 16GB 512GB Midnight</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>417999</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>415000</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>-2999</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-0.72</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 13 MDHH4 M5 10C CPU 8C GPU 16GB 512GB Sky Blue</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>417999</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>415000</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>-2999</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-0.72</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 13 MDHA4 M5 10C CPU 8C GPU 16GB 512GB Starlight</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>417999</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>415000</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>-2999</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-0.72</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Macbook Pro 14 MGDR4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Space Black</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>720000</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>717999</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>-2001</v>
+      </c>
+      <c r="F17" t="n">
+        <v>-0.28</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Macbook Pro 14 M5 MDE34 10 Core CPU 10 Core GPU 24GB 1TB Space Black</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>644999</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>642999</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>-2000</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-0.31</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Macbook Pro 14 MGDN4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Silver</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>725000</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>723500</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>-1500</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-0.21</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Macbook Pro 14 M5 MDE14 10 Core CPU 10 Core GPU 16GB 1TB Space Black</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>579999</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>578999</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>-1000</v>
+      </c>
+      <c r="F20" t="n">
+        <v>-0.17</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Macbook Pro 16 MGEC4 M5 Pro 18 Core CPU 20 Core GPU 48GB 1TB Space Black</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>1055000</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>1054000</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>-1000</v>
+      </c>
+      <c r="F21" t="n">
+        <v>-0.09</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Macbook Pro 16 MGE64 M5 Pro 18 Core CPU 20 Core GPU 48GB 1TB Silver</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>1055000</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>1054000</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>-1000</v>
+      </c>
+      <c r="F22" t="n">
+        <v>-0.09</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 15 MDVU4 M5 10C CPU 10C GPU 24GB 1TB Sky Blue</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="C2" s="3" t="n">
-        <v>990000</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>10000</v>
-      </c>
-      <c r="F2" t="n">
-        <v>1.01</v>
+      <c r="C23" s="3" t="n">
+        <v>614999</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>619999</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 15 MDVF4 M5 10C CPU 10C GPU 24GB 1TB Starlight</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>614999</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>619999</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 15 MDVC4 M5 10C CPU 10C GPU 24GB 1TB Silver</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>614999</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>619999</v>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 15 MDVN4 M5 10C CPU 10C GPU 24GB 1TB Midnight</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>614999</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>619999</v>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Macbook Pro 14 MGDP4 M5 Pro 18 Core CPU 20 Core GPU 24GB 2TB Silver</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>875000</v>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>955000</v>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>80000</v>
+      </c>
+      <c r="F27" t="n">
+        <v>9.140000000000001</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Macbook Pro 14 MGDT4 M5 Pro 18 Core CPU 20 Core GPU 24GB 2TB Space Black</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>864999</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>955000</v>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>90001</v>
+      </c>
+      <c r="F28" t="n">
+        <v>10.4</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F2"/>
-  <conditionalFormatting sqref="E2">
+  <autoFilter ref="A1:F28"/>
+  <conditionalFormatting sqref="E2:E28">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
chore: price data 2026-10-08
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MacBook Pro'!$A$1:$S$93</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MacBook Air'!$A$1:$S$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20261007T102046536862+0000</t>
+          <t>20261008T104029385040+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-07T10:20:46.536862+00:00</t>
+          <t>2026-10-08T10:40:29.385040+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>276.741533</v>
+        <v>277.084072</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -729,7 +729,7 @@
         <v>532000</v>
       </c>
       <c r="D22" t="n">
-        <v>51.5</v>
+        <v>51.6</v>
       </c>
       <c r="E22" t="n">
         <v>4</v>
@@ -813,7 +813,7 @@
         <v>700000</v>
       </c>
       <c r="D26" t="n">
-        <v>49.5</v>
+        <v>49.6</v>
       </c>
       <c r="E26" t="n">
         <v>4</v>
@@ -834,7 +834,7 @@
         <v>847999</v>
       </c>
       <c r="D27" t="n">
-        <v>47.3</v>
+        <v>47.4</v>
       </c>
       <c r="E27" t="n">
         <v>5</v>
@@ -885,7 +885,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 MGDN4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Silver</t>
+          <t>Macbook Pro 14 M5 MJ3E4 10 Core CPU 10 Core GPU 32GB 1TB Silver</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -894,19 +894,19 @@
         </is>
       </c>
       <c r="C30" s="3" t="n">
-        <v>723500</v>
+        <v>759999</v>
       </c>
       <c r="D30" t="n">
-        <v>42.6</v>
+        <v>43.4</v>
       </c>
       <c r="E30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 MJ3E4 10 Core CPU 10 Core GPU 32GB 1TB Silver</t>
+          <t>Macbook Pro 14 M5 MJ3D4 10 Core CPU 10 Core GPU 32GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -915,10 +915,10 @@
         </is>
       </c>
       <c r="C31" s="3" t="n">
-        <v>769999</v>
+        <v>759999</v>
       </c>
       <c r="D31" t="n">
-        <v>42.4</v>
+        <v>43.4</v>
       </c>
       <c r="E31" t="n">
         <v>4</v>
@@ -1147,10 +1147,10 @@
         <v>470000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>685890</v>
+        <v>686739</v>
       </c>
       <c r="L2" t="n">
-        <v>35.12079196372596</v>
+        <v>35.20100067128851</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1165,7 +1165,7 @@
         <v>28.4414106939704</v>
       </c>
       <c r="Q2" t="n">
-        <v>35.3</v>
+        <v>35.4</v>
       </c>
       <c r="R2" t="n">
         <v>5</v>
@@ -1214,10 +1214,10 @@
         <v>495000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>685890</v>
+        <v>686739</v>
       </c>
       <c r="L3" t="n">
-        <v>27.83099330796484</v>
+        <v>27.92021422986025</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>771680</v>
+        <v>772635</v>
       </c>
       <c r="L4" t="n">
-        <v>35.20643271822517</v>
+        <v>35.28651950791771</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>771680</v>
+        <v>772635</v>
       </c>
       <c r="L5" t="n">
-        <v>32.61468484345843</v>
+        <v>32.69797511114562</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>857470</v>
+        <v>858531</v>
       </c>
       <c r="L6" t="n">
-        <v>37.95701307334367</v>
+        <v>38.03368777598013</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1433,7 +1433,7 @@
         <v>100</v>
       </c>
       <c r="Q6" t="n">
-        <v>51.5</v>
+        <v>51.6</v>
       </c>
       <c r="R6" t="n">
         <v>4</v>
@@ -1606,10 +1606,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>857470</v>
+        <v>858531</v>
       </c>
       <c r="L9" t="n">
-        <v>34.10848192939694</v>
+        <v>34.18991276960296</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1673,13 +1673,13 @@
         <v>578999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>857470</v>
+        <v>858531</v>
       </c>
       <c r="L10" t="n">
-        <v>32.47588836927239</v>
+        <v>32.55933682068557</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>-1000</v>
+        <v>0</v>
       </c>
       <c r="N10" t="n">
         <v>0.6861075233405204</v>
@@ -1734,31 +1734,31 @@
         </is>
       </c>
       <c r="I11" s="3" t="n">
-        <v>587999</v>
+        <v>584999</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>587999</v>
+        <v>584999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>857470</v>
+        <v>858531</v>
       </c>
       <c r="L11" t="n">
-        <v>31.42628896637783</v>
+        <v>31.8604686377079</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>0</v>
+        <v>-3000</v>
       </c>
       <c r="N11" t="n">
-        <v>0</v>
+        <v>0.5102049493281451</v>
       </c>
       <c r="O11" t="n">
         <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>47.60029999999999</v>
+        <v>48.50029999999999</v>
       </c>
       <c r="Q11" t="n">
-        <v>18.4</v>
+        <v>18.8</v>
       </c>
       <c r="R11" t="n">
         <v>4</v>
@@ -1807,16 +1807,16 @@
         <v>600000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>857470</v>
+        <v>858531</v>
       </c>
       <c r="L12" t="n">
-        <v>30.02670647369587</v>
+        <v>30.11318170223323</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>7.692307692307693</v>
+        <v>4</v>
       </c>
       <c r="O12" t="n">
         <v>100</v>
@@ -1825,7 +1825,7 @@
         <v>45.94594594594595</v>
       </c>
       <c r="Q12" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="R12" t="n">
         <v>4</v>
@@ -1874,16 +1874,16 @@
         <v>634000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>857470</v>
+        <v>858531</v>
       </c>
       <c r="L13" t="n">
-        <v>26.06155317387197</v>
+        <v>26.15292866535978</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>2.461538461538462</v>
+        <v>1.705426356589147</v>
       </c>
       <c r="O13" t="n">
         <v>0</v>
@@ -1892,7 +1892,7 @@
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>9.4</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="R13" t="n">
         <v>4</v>
@@ -1941,13 +1941,13 @@
         <v>642999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>943260</v>
+        <v>944427</v>
       </c>
       <c r="L14" t="n">
-        <v>31.83226257871637</v>
+        <v>31.91649539879737</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>-2000</v>
+        <v>0</v>
       </c>
       <c r="N14" t="n">
         <v>0.1552797442232053</v>
@@ -2067,10 +2067,10 @@
         <v>650000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>943260</v>
+        <v>944427</v>
       </c>
       <c r="L16" t="n">
-        <v>31.09004940313381</v>
+        <v>31.17519935368218</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -2134,10 +2134,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1029050</v>
+        <v>1030323</v>
       </c>
       <c r="L17" t="n">
-        <v>31.9760944560517</v>
+        <v>32.06014036375001</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2152,7 +2152,7 @@
         <v>100</v>
       </c>
       <c r="Q17" t="n">
-        <v>49.5</v>
+        <v>49.6</v>
       </c>
       <c r="R17" t="n">
         <v>4</v>
@@ -2201,10 +2201,10 @@
         <v>711999</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>1071944</v>
+        <v>1073271</v>
       </c>
       <c r="L18" t="n">
-        <v>33.57871306710052</v>
+        <v>33.66083682499574</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -2269,7 +2269,7 @@
       </c>
       <c r="K19" s="3" t="n"/>
       <c r="M19" s="3" t="n">
-        <v>-2001</v>
+        <v>0</v>
       </c>
       <c r="N19" t="n">
         <v>0.2779166666666667</v>
@@ -2330,10 +2330,10 @@
         <v>720000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>1029050</v>
+        <v>1030323</v>
       </c>
       <c r="L20" t="n">
-        <v>30.03255429765317</v>
+        <v>30.11900151700001</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -2398,7 +2398,7 @@
       </c>
       <c r="K21" s="3" t="n"/>
       <c r="M21" s="3" t="n">
-        <v>-1500</v>
+        <v>0</v>
       </c>
       <c r="N21" t="n">
         <v>0.2068965517241379</v>
@@ -2459,10 +2459,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1071944</v>
+        <v>1073271</v>
       </c>
       <c r="L22" t="n">
-        <v>30.68667766226594</v>
+        <v>30.77237715358004</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2477,7 +2477,7 @@
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>10.2</v>
+        <v>10.3</v>
       </c>
       <c r="R22" t="n">
         <v>4</v>
@@ -2520,31 +2520,31 @@
         </is>
       </c>
       <c r="I23" s="3" t="n">
-        <v>769999</v>
+        <v>759999</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>769999</v>
+        <v>759999</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1029050</v>
+        <v>1030323</v>
       </c>
       <c r="L23" t="n">
-        <v>25.17380107866479</v>
+        <v>26.23682088044234</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>0</v>
+        <v>-10000</v>
       </c>
       <c r="N23" t="n">
-        <v>0.2591968911917099</v>
+        <v>1.554533678756477</v>
       </c>
       <c r="O23" t="n">
         <v>100</v>
       </c>
       <c r="P23" t="n">
-        <v>70.00019999999999</v>
+        <v>72.00019999999999</v>
       </c>
       <c r="Q23" t="n">
-        <v>42.4</v>
+        <v>43.4</v>
       </c>
       <c r="R23" t="n">
         <v>4</v>
@@ -2587,31 +2587,31 @@
         </is>
       </c>
       <c r="I24" s="3" t="n">
-        <v>769999</v>
+        <v>759999</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>769999</v>
+        <v>759999</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1029050</v>
+        <v>1030323</v>
       </c>
       <c r="L24" t="n">
-        <v>25.17380107866479</v>
+        <v>26.23682088044234</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>0</v>
+        <v>-10000</v>
       </c>
       <c r="N24" t="n">
-        <v>0.2591968911917099</v>
+        <v>1.554533678756477</v>
       </c>
       <c r="O24" t="n">
         <v>100</v>
       </c>
       <c r="P24" t="n">
-        <v>70.00019999999999</v>
+        <v>72.00019999999999</v>
       </c>
       <c r="Q24" t="n">
-        <v>42.4</v>
+        <v>43.4</v>
       </c>
       <c r="R24" t="n">
         <v>4</v>
@@ -2660,10 +2660,10 @@
         <v>772000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>1029050</v>
+        <v>1030323</v>
       </c>
       <c r="L25" t="n">
-        <v>24.97934988581702</v>
+        <v>25.07204051545001</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -2678,7 +2678,7 @@
         <v>69.59999999999998</v>
       </c>
       <c r="Q25" t="n">
-        <v>19.9</v>
+        <v>20</v>
       </c>
       <c r="R25" t="n">
         <v>4</v>
@@ -2851,10 +2851,10 @@
         <v>810000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>1071944</v>
+        <v>1073271</v>
       </c>
       <c r="L28" t="n">
-        <v>24.43635115267215</v>
+        <v>24.52977859273194</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -2866,7 +2866,7 @@
         <v>61.99999999999999</v>
       </c>
       <c r="Q28" t="n">
-        <v>24.6</v>
+        <v>24.7</v>
       </c>
       <c r="R28" t="n">
         <v>3</v>
@@ -2915,10 +2915,10 @@
         <v>810000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>1243524</v>
+        <v>1245063</v>
       </c>
       <c r="L29" t="n">
-        <v>34.86253582560529</v>
+        <v>34.94305107452394</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -2982,16 +2982,16 @@
         <v>822999</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1286419</v>
+        <v>1288011</v>
       </c>
       <c r="L30" t="n">
-        <v>36.02403260523982</v>
+        <v>36.10310781507301</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N30" t="n">
-        <v>2.023928571428571</v>
+        <v>1.437186489333227</v>
       </c>
       <c r="O30" t="n">
         <v>100</v>
@@ -3000,7 +3000,7 @@
         <v>0.0003521901827191575</v>
       </c>
       <c r="Q30" t="n">
-        <v>34.8</v>
+        <v>34.7</v>
       </c>
       <c r="R30" t="n">
         <v>4</v>
@@ -3049,10 +3049,10 @@
         <v>823000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1286419</v>
+        <v>1288011</v>
       </c>
       <c r="L31" t="n">
-        <v>36.02395487006955</v>
+        <v>36.10303017598452</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -3116,10 +3116,10 @@
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1372209</v>
+        <v>1373908</v>
       </c>
       <c r="L32" t="n">
-        <v>38.20190656088104</v>
+        <v>38.27832722423918</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3134,7 +3134,7 @@
         <v>100</v>
       </c>
       <c r="Q32" t="n">
-        <v>47.3</v>
+        <v>47.4</v>
       </c>
       <c r="R32" t="n">
         <v>5</v>
@@ -3183,10 +3183,10 @@
         <v>930000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1372209</v>
+        <v>1373908</v>
       </c>
       <c r="L33" t="n">
-        <v>38.05615616863029</v>
+        <v>38.13275706961456</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3250,10 +3250,10 @@
         <v>860000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>1243524</v>
+        <v>1245063</v>
       </c>
       <c r="L34" t="n">
-        <v>30.84170470372908</v>
+        <v>30.92719002974147</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -3268,7 +3268,7 @@
         <v>89.80112187659357</v>
       </c>
       <c r="Q34" t="n">
-        <v>25.2</v>
+        <v>25.3</v>
       </c>
       <c r="R34" t="n">
         <v>4</v>
@@ -3379,10 +3379,10 @@
         <v>880000</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>1157734</v>
+        <v>1159167</v>
       </c>
       <c r="L36" t="n">
-        <v>23.98944835342142</v>
+        <v>24.0834150730654</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -3443,10 +3443,10 @@
         <v>940000</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>1243524</v>
+        <v>1245063</v>
       </c>
       <c r="L37" t="n">
-        <v>24.40837490872713</v>
+        <v>24.50181235808951</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
@@ -3458,7 +3458,7 @@
         <v>83</v>
       </c>
       <c r="Q37" t="n">
-        <v>28.2</v>
+        <v>28.3</v>
       </c>
       <c r="R37" t="n">
         <v>3</v>
@@ -3508,7 +3508,7 @@
       </c>
       <c r="K38" s="3" t="n"/>
       <c r="M38" s="3" t="n">
-        <v>90001</v>
+        <v>0</v>
       </c>
       <c r="N38" t="n">
         <v>0</v>
@@ -3570,7 +3570,7 @@
       </c>
       <c r="K39" s="3" t="n"/>
       <c r="M39" s="3" t="n">
-        <v>80000</v>
+        <v>0</v>
       </c>
       <c r="N39" t="n">
         <v>0</v>
@@ -3631,16 +3631,16 @@
         <v>990000</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>1500894</v>
+        <v>1502752</v>
       </c>
       <c r="L40" t="n">
-        <v>34.03931256970845</v>
+        <v>34.12086625071868</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N40" t="n">
-        <v>3.131115459882583</v>
+        <v>1.834407535944472</v>
       </c>
       <c r="O40" t="n">
         <v>100</v>
@@ -3649,7 +3649,7 @@
         <v>39.19647231749141</v>
       </c>
       <c r="Q40" t="n">
-        <v>41</v>
+        <v>40.6</v>
       </c>
       <c r="R40" t="n">
         <v>4</v>
@@ -3760,10 +3760,10 @@
         <v>1000000</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>1500894</v>
+        <v>1502752</v>
       </c>
       <c r="L42" t="n">
-        <v>33.37304299970551</v>
+        <v>33.45542045527139</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -3827,13 +3827,13 @@
         <v>1054000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1543789</v>
+        <v>1545700</v>
       </c>
       <c r="L43" t="n">
-        <v>31.72642116247751</v>
+        <v>31.81083004463997</v>
       </c>
       <c r="M43" s="3" t="n">
-        <v>-1000</v>
+        <v>0</v>
       </c>
       <c r="N43" t="n">
         <v>0.09478672985781991</v>
@@ -3842,7 +3842,7 @@
         <v>57.84723750825446</v>
       </c>
       <c r="Q43" t="n">
-        <v>26</v>
+        <v>26.1</v>
       </c>
       <c r="R43" t="n">
         <v>3</v>
@@ -3891,13 +3891,13 @@
         <v>1054000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1543789</v>
+        <v>1545700</v>
       </c>
       <c r="L44" t="n">
-        <v>31.72642116247751</v>
+        <v>31.81083004463997</v>
       </c>
       <c r="M44" s="3" t="n">
-        <v>-1000</v>
+        <v>0</v>
       </c>
       <c r="N44" t="n">
         <v>0.09478672985781991</v>
@@ -3906,7 +3906,7 @@
         <v>57.84723750825446</v>
       </c>
       <c r="Q44" t="n">
-        <v>26</v>
+        <v>26.1</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -4017,22 +4017,22 @@
         <v>1115000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1500894</v>
+        <v>1502752</v>
       </c>
       <c r="L46" t="n">
-        <v>25.71094294467164</v>
+        <v>25.80279380762761</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N46" t="n">
-        <v>3.043478260869565</v>
+        <v>1.545253863134658</v>
       </c>
       <c r="P46" t="n">
         <v>9.358196283135744</v>
       </c>
       <c r="Q46" t="n">
-        <v>14.1</v>
+        <v>13.6</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -4081,10 +4081,10 @@
         <v>1123000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1715369</v>
+        <v>1717492</v>
       </c>
       <c r="L47" t="n">
-        <v>34.53303633212445</v>
+        <v>34.61396035614722</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -4148,10 +4148,10 @@
         <v>1130000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1500894</v>
+        <v>1502752</v>
       </c>
       <c r="L48" t="n">
-        <v>24.71153858966722</v>
+        <v>24.80462511445668</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -4163,7 +4163,7 @@
         <v>88.39999999999999</v>
       </c>
       <c r="Q48" t="n">
-        <v>29.5</v>
+        <v>29.6</v>
       </c>
       <c r="R48" t="n">
         <v>3</v>
@@ -4274,10 +4274,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1758263</v>
+        <v>1760440</v>
       </c>
       <c r="L50" t="n">
-        <v>34.31016861527542</v>
+        <v>34.39140214946264</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4289,7 +4289,7 @@
         <v>22.53136001640632</v>
       </c>
       <c r="Q50" t="n">
-        <v>19.5</v>
+        <v>19.6</v>
       </c>
       <c r="R50" t="n">
         <v>3</v>
@@ -4338,10 +4338,10 @@
         <v>1155000</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>1758263</v>
+        <v>1760440</v>
       </c>
       <c r="L51" t="n">
-        <v>34.31016861527542</v>
+        <v>34.39140214946264</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -4353,7 +4353,7 @@
         <v>22.53136001640632</v>
       </c>
       <c r="Q51" t="n">
-        <v>19.5</v>
+        <v>19.6</v>
       </c>
       <c r="R51" t="n">
         <v>3</v>
@@ -4402,10 +4402,10 @@
         <v>1185000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1586684</v>
+        <v>1588648</v>
       </c>
       <c r="L52" t="n">
-        <v>25.31594192668483</v>
+        <v>25.40827168762369</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -4466,10 +4466,10 @@
         <v>1185000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1586684</v>
+        <v>1588648</v>
       </c>
       <c r="L53" t="n">
-        <v>25.31594192668483</v>
+        <v>25.40827168762369</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -4481,7 +4481,7 @@
         <v>94.72727272727272</v>
       </c>
       <c r="Q53" t="n">
-        <v>31.1</v>
+        <v>31.2</v>
       </c>
       <c r="R53" t="n">
         <v>3</v>
@@ -4530,10 +4530,10 @@
         <v>1200000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1886948</v>
+        <v>1889284</v>
       </c>
       <c r="L54" t="n">
-        <v>36.40524275178754</v>
+        <v>36.4838743142905</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -4545,7 +4545,7 @@
         <v>3.948101568096777</v>
       </c>
       <c r="Q54" t="n">
-        <v>16.4</v>
+        <v>16.5</v>
       </c>
       <c r="R54" t="n">
         <v>3</v>
@@ -4594,10 +4594,10 @@
         <v>1200000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1886948</v>
+        <v>1889284</v>
       </c>
       <c r="L55" t="n">
-        <v>36.40524275178754</v>
+        <v>36.4838743142905</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -4609,7 +4609,7 @@
         <v>3.948101568096777</v>
       </c>
       <c r="Q55" t="n">
-        <v>16.4</v>
+        <v>16.5</v>
       </c>
       <c r="R55" t="n">
         <v>3</v>
@@ -4720,10 +4720,10 @@
         <v>1240000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1672474</v>
+        <v>1674544</v>
       </c>
       <c r="L57" t="n">
-        <v>25.85833920288148</v>
+        <v>25.949989967418</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -4846,10 +4846,10 @@
         <v>1280000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1715369</v>
+        <v>1717492</v>
       </c>
       <c r="L59" t="n">
-        <v>25.38048664747934</v>
+        <v>25.47272418153913</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -4913,22 +4913,22 @@
         <v>1298000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1758263</v>
+        <v>1760440</v>
       </c>
       <c r="L60" t="n">
-        <v>26.17714187240475</v>
+        <v>26.26843289177706</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N60" t="n">
-        <v>2.989536621823617</v>
+        <v>1.517450682852807</v>
       </c>
       <c r="P60" t="n">
         <v>61.28109178956637</v>
       </c>
       <c r="Q60" t="n">
-        <v>25.4</v>
+        <v>24.9</v>
       </c>
       <c r="R60" t="n">
         <v>3</v>
@@ -4977,22 +4977,22 @@
         <v>1300000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1715369</v>
+        <v>1717492</v>
       </c>
       <c r="L61" t="n">
-        <v>24.21455675134621</v>
+        <v>24.30823549687568</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N61" t="n">
-        <v>0.7633587786259541</v>
+        <v>0.3831417624521072</v>
       </c>
       <c r="P61" t="n">
         <v>60.92890160686771</v>
       </c>
       <c r="Q61" t="n">
-        <v>23.7</v>
+        <v>23.6</v>
       </c>
       <c r="R61" t="n">
         <v>3</v>
@@ -5103,10 +5103,10 @@
         <v>1335000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1801158</v>
+        <v>1803388</v>
       </c>
       <c r="L63" t="n">
-        <v>25.88101654602206</v>
+        <v>25.97266922037853</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -5167,22 +5167,22 @@
         <v>1420000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1929843</v>
+        <v>1932232</v>
       </c>
       <c r="L64" t="n">
-        <v>26.41888485229109</v>
+        <v>26.50986009961537</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N64" t="n">
-        <v>3.467029231815092</v>
+        <v>1.764095468695953</v>
       </c>
       <c r="P64" t="n">
         <v>81.47332893095606</v>
       </c>
       <c r="Q64" t="n">
-        <v>30</v>
+        <v>29.4</v>
       </c>
       <c r="R64" t="n">
         <v>3</v>
@@ -5231,22 +5231,22 @@
         <v>1430000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1929843</v>
+        <v>1932232</v>
       </c>
       <c r="L65" t="n">
-        <v>25.90070798505371</v>
+        <v>25.99232390313378</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N65" t="n">
-        <v>2.787219578518015</v>
+        <v>1.413305756635643</v>
       </c>
       <c r="P65" t="n">
         <v>60.92890160686771</v>
       </c>
       <c r="Q65" t="n">
-        <v>25.2</v>
+        <v>24.7</v>
       </c>
       <c r="R65" t="n">
         <v>3</v>
@@ -5295,10 +5295,10 @@
         <v>1430000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>2144318</v>
+        <v>2146972</v>
       </c>
       <c r="L66" t="n">
-        <v>33.31213001056746</v>
+        <v>33.39456685974479</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -5359,10 +5359,10 @@
         <v>1430000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>2144318</v>
+        <v>2146972</v>
       </c>
       <c r="L67" t="n">
-        <v>33.31213001056746</v>
+        <v>33.39456685974479</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -5485,10 +5485,10 @@
         <v>1480000</v>
       </c>
       <c r="K69" s="3" t="n">
-        <v>2015633</v>
+        <v>2018128</v>
       </c>
       <c r="L69" t="n">
-        <v>26.57393483833614</v>
+        <v>26.66471105896157</v>
       </c>
       <c r="M69" s="3" t="n">
         <v>0</v>
@@ -5611,10 +5611,10 @@
         <v>1605000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2187213</v>
+        <v>2189920</v>
       </c>
       <c r="L71" t="n">
-        <v>26.61894383400245</v>
+        <v>26.70965149411851</v>
       </c>
       <c r="M71" s="3" t="n">
         <v>0</v>
@@ -5626,7 +5626,7 @@
         <v>36.44392794886694</v>
       </c>
       <c r="Q71" t="n">
-        <v>19.2</v>
+        <v>19.3</v>
       </c>
       <c r="R71" t="n">
         <v>3</v>
@@ -5675,10 +5675,10 @@
         <v>1610000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2187213</v>
+        <v>2189920</v>
       </c>
       <c r="L72" t="n">
-        <v>26.39034241292458</v>
+        <v>26.48133265142106</v>
       </c>
       <c r="M72" s="3" t="n">
         <v>0</v>
@@ -5690,7 +5690,7 @@
         <v>25.72147975982957</v>
       </c>
       <c r="Q72" t="n">
-        <v>16.8</v>
+        <v>16.9</v>
       </c>
       <c r="R72" t="n">
         <v>3</v>
@@ -5739,22 +5739,22 @@
         <v>1615000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2187213</v>
+        <v>2189920</v>
       </c>
       <c r="L73" t="n">
-        <v>26.1617409918467</v>
+        <v>26.25301380872361</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N73" t="n">
-        <v>2.769416014449127</v>
+        <v>1.404151404151404</v>
       </c>
       <c r="P73" t="n">
         <v>86.7142542687337</v>
       </c>
       <c r="Q73" t="n">
-        <v>30.8</v>
+        <v>30.3</v>
       </c>
       <c r="R73" t="n">
         <v>3</v>
@@ -5803,10 +5803,10 @@
         <v>1630000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2230108</v>
+        <v>2232868</v>
       </c>
       <c r="L74" t="n">
-        <v>26.90936941170562</v>
+        <v>26.99971516453279</v>
       </c>
       <c r="M74" s="3" t="n">
         <v>0</v>
@@ -5867,22 +5867,22 @@
         <v>1690000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2315898</v>
+        <v>2318764</v>
       </c>
       <c r="L75" t="n">
-        <v>27.02614709283397</v>
+        <v>27.11634301722815</v>
       </c>
       <c r="M75" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N75" t="n">
-        <v>1.227352425482174</v>
+        <v>0.6174654513378418</v>
       </c>
       <c r="P75" t="n">
         <v>16.88768606224628</v>
       </c>
       <c r="Q75" t="n">
-        <v>15.6</v>
+        <v>15.5</v>
       </c>
       <c r="R75" t="n">
         <v>3</v>
@@ -5931,22 +5931,22 @@
         <v>1705000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2315898</v>
+        <v>2318764</v>
       </c>
       <c r="L76" t="n">
-        <v>26.3784501735396</v>
+        <v>26.46944665347573</v>
       </c>
       <c r="M76" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N76" t="n">
-        <v>2.904328018223234</v>
+        <v>1.473562554175094</v>
       </c>
       <c r="P76" t="n">
         <v>1.9846639603067</v>
       </c>
       <c r="Q76" t="n">
-        <v>12.8</v>
+        <v>12.3</v>
       </c>
       <c r="R76" t="n">
         <v>3</v>
@@ -5995,22 +5995,22 @@
         <v>1725000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2358793</v>
+        <v>2361712</v>
       </c>
       <c r="L77" t="n">
-        <v>26.86937768596057</v>
+        <v>26.95976478080308</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N77" t="n">
-        <v>3.631284916201118</v>
+        <v>1.849217638691323</v>
       </c>
       <c r="P77" t="n">
         <v>100</v>
       </c>
       <c r="Q77" t="n">
-        <v>34.2</v>
+        <v>33.6</v>
       </c>
       <c r="R77" t="n">
         <v>3</v>
@@ -6059,10 +6059,10 @@
         <v>1780000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2444582</v>
+        <v>2447608</v>
       </c>
       <c r="L78" t="n">
-        <v>27.18591562892961</v>
+        <v>27.2759363427477</v>
       </c>
       <c r="M78" s="3" t="n">
         <v>0</v>
@@ -6123,22 +6123,22 @@
         <v>1875000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2573267</v>
+        <v>2576452</v>
       </c>
       <c r="L79" t="n">
-        <v>27.13542745467144</v>
+        <v>27.22550235750559</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N79" t="n">
-        <v>3.598971722365039</v>
+        <v>1.832460732984293</v>
       </c>
       <c r="P79" t="n">
         <v>19.64044075004835</v>
       </c>
       <c r="Q79" t="n">
-        <v>17.1</v>
+        <v>16.5</v>
       </c>
       <c r="R79" t="n">
         <v>3</v>
@@ -6187,10 +6187,10 @@
         <v>1910000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2616162</v>
+        <v>2619400</v>
       </c>
       <c r="L80" t="n">
-        <v>26.99228870383409</v>
+        <v>27.08253798579827</v>
       </c>
       <c r="M80" s="3" t="n">
         <v>0</v>
@@ -6251,22 +6251,22 @@
         <v>2020000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2744847</v>
+        <v>2748245</v>
       </c>
       <c r="L81" t="n">
-        <v>26.40755568525313</v>
+        <v>26.49854725470255</v>
       </c>
       <c r="M81" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N81" t="n">
-        <v>2.791145332050048</v>
+        <v>1.415324548560273</v>
       </c>
       <c r="P81" t="n">
         <v>36.26522327469554</v>
       </c>
       <c r="Q81" t="n">
-        <v>20.1</v>
+        <v>19.6</v>
       </c>
       <c r="R81" t="n">
         <v>3</v>
@@ -6315,10 +6315,10 @@
         <v>2110000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>2873532</v>
+        <v>2877089</v>
       </c>
       <c r="L82" t="n">
-        <v>26.57120226954146</v>
+        <v>26.66198369254479</v>
       </c>
       <c r="M82" s="3" t="n">
         <v>0</v>
@@ -6330,7 +6330,7 @@
         <v>79.02382335851249</v>
       </c>
       <c r="Q82" t="n">
-        <v>28.3</v>
+        <v>28.4</v>
       </c>
       <c r="R82" t="n">
         <v>3</v>
@@ -6379,22 +6379,22 @@
         <v>2210000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3002217</v>
+        <v>3005933</v>
       </c>
       <c r="L83" t="n">
-        <v>26.38773279879502</v>
+        <v>26.47873389060901</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N83" t="n">
-        <v>2.55731922398589</v>
+        <v>1.29522108083966</v>
       </c>
       <c r="P83" t="n">
         <v>70.36535859269283</v>
       </c>
       <c r="Q83" t="n">
-        <v>27.3</v>
+        <v>26.9</v>
       </c>
       <c r="R83" t="n">
         <v>3</v>
@@ -6443,10 +6443,10 @@
         <v>2215000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3045112</v>
+        <v>3048881</v>
       </c>
       <c r="L84" t="n">
-        <v>27.26047514836893</v>
+        <v>27.35039511217394</v>
       </c>
       <c r="M84" s="3" t="n">
         <v>0</v>
@@ -6507,22 +6507,22 @@
         <v>2315000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3173796</v>
+        <v>3177725</v>
       </c>
       <c r="L85" t="n">
-        <v>27.05895400964649</v>
+        <v>27.14913971473302</v>
       </c>
       <c r="M85" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N85" t="n">
-        <v>2.771944561108778</v>
+        <v>1.405451448040886</v>
       </c>
       <c r="P85" t="n">
         <v>65.11105977094954</v>
       </c>
       <c r="Q85" t="n">
-        <v>26.5</v>
+        <v>26.1</v>
       </c>
       <c r="R85" t="n">
         <v>3</v>
@@ -6571,10 +6571,10 @@
         <v>2395000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3302481</v>
+        <v>3306569</v>
       </c>
       <c r="L86" t="n">
-        <v>27.47876520712761</v>
+        <v>27.56842515610592</v>
       </c>
       <c r="M86" s="3" t="n">
         <v>0</v>
@@ -6635,10 +6635,10 @@
         <v>2410000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3302481</v>
+        <v>3306569</v>
       </c>
       <c r="L87" t="n">
-        <v>27.02456123138937</v>
+        <v>27.11478272493331</v>
       </c>
       <c r="M87" s="3" t="n">
         <v>0</v>
@@ -6650,7 +6650,7 @@
         <v>88.47569242688358</v>
       </c>
       <c r="Q87" t="n">
-        <v>30.5</v>
+        <v>30.6</v>
       </c>
       <c r="R87" t="n">
         <v>3</v>
@@ -6699,22 +6699,22 @@
         <v>2499000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3431166</v>
+        <v>3435413</v>
       </c>
       <c r="L88" t="n">
-        <v>27.16761590666263</v>
+        <v>27.25765431987362</v>
       </c>
       <c r="M88" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N88" t="n">
-        <v>3.17706315381635</v>
+        <v>1.614173228346457</v>
       </c>
       <c r="P88" t="n">
         <v>63.67326854471646</v>
       </c>
       <c r="Q88" t="n">
-        <v>26.4</v>
+        <v>25.9</v>
       </c>
       <c r="R88" t="n">
         <v>3</v>
@@ -6763,22 +6763,22 @@
         <v>2510000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3431166</v>
+        <v>3435413</v>
       </c>
       <c r="L89" t="n">
-        <v>26.84702518036143</v>
+        <v>26.93745992112157</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N89" t="n">
-        <v>2.372617658498639</v>
+        <v>1.200551072623499</v>
       </c>
       <c r="P89" t="n">
         <v>83.17546233649077</v>
       </c>
       <c r="Q89" t="n">
-        <v>30.2</v>
+        <v>29.8</v>
       </c>
       <c r="R89" t="n">
         <v>3</v>
@@ -6827,10 +6827,10 @@
         <v>2530000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3474061</v>
+        <v>3478361</v>
       </c>
       <c r="L90" t="n">
-        <v>27.17456601942223</v>
+        <v>27.26459387050395</v>
       </c>
       <c r="M90" s="3" t="n">
         <v>0</v>
@@ -6842,7 +6842,7 @@
         <v>79.17877203176447</v>
       </c>
       <c r="Q90" t="n">
-        <v>28.6</v>
+        <v>28.7</v>
       </c>
       <c r="R90" t="n">
         <v>3</v>
@@ -6891,22 +6891,22 @@
         <v>2610000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>3602746</v>
+        <v>3607205</v>
       </c>
       <c r="L91" t="n">
-        <v>27.55525923836985</v>
+        <v>27.64481087157508</v>
       </c>
       <c r="M91" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N91" t="n">
-        <v>2.027027027027027</v>
+        <v>1.023890784982935</v>
       </c>
       <c r="P91" t="n">
         <v>74.15426251691474</v>
       </c>
       <c r="Q91" t="n">
-        <v>28.4</v>
+        <v>28.1</v>
       </c>
       <c r="R91" t="n">
         <v>3</v>
@@ -6955,10 +6955,10 @@
         <v>3015000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4160380</v>
+        <v>4165530</v>
       </c>
       <c r="L92" t="n">
-        <v>27.53065825717843</v>
+        <v>27.62025480551094</v>
       </c>
       <c r="M92" s="3" t="n">
         <v>0</v>
@@ -6970,7 +6970,7 @@
         <v>100</v>
       </c>
       <c r="Q92" t="n">
-        <v>33.2</v>
+        <v>33.3</v>
       </c>
       <c r="R92" t="n">
         <v>3</v>
@@ -7019,22 +7019,22 @@
         <v>3098000</v>
       </c>
       <c r="K93" s="3" t="n">
-        <v>4289065</v>
+        <v>4294374</v>
       </c>
       <c r="L93" t="n">
-        <v>27.7698053072173</v>
+        <v>27.85910123338116</v>
       </c>
       <c r="M93" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N93" t="n">
-        <v>2.762084118016321</v>
+        <v>1.400381922342457</v>
       </c>
       <c r="P93" t="n">
         <v>100</v>
       </c>
       <c r="Q93" t="n">
-        <v>34.3</v>
+        <v>33.9</v>
       </c>
       <c r="R93" t="n">
         <v>3</v>
@@ -7318,10 +7318,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>428520</v>
+        <v>429051</v>
       </c>
       <c r="L2" t="n">
-        <v>27.65821898627835</v>
+        <v>27.74775026745072</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7385,10 +7385,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>428520</v>
+        <v>429051</v>
       </c>
       <c r="L3" t="n">
-        <v>27.65821898627835</v>
+        <v>27.74775026745072</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7452,10 +7452,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>428520</v>
+        <v>429051</v>
       </c>
       <c r="L4" t="n">
-        <v>27.65798562494166</v>
+        <v>27.74751719492555</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7519,10 +7519,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>428520</v>
+        <v>429051</v>
       </c>
       <c r="L5" t="n">
-        <v>27.65798562494166</v>
+        <v>27.74751719492555</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7586,10 +7586,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514310</v>
+        <v>514947</v>
       </c>
       <c r="L6" t="n">
-        <v>25.33685909276506</v>
+        <v>25.42921892932671</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7650,10 +7650,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>514310</v>
+        <v>514947</v>
       </c>
       <c r="L7" t="n">
-        <v>25.33685909276506</v>
+        <v>25.42921892932671</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7714,10 +7714,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>514310</v>
+        <v>514947</v>
       </c>
       <c r="L8" t="n">
-        <v>25.33685909276506</v>
+        <v>25.42921892932671</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7778,10 +7778,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>514310</v>
+        <v>514947</v>
       </c>
       <c r="L9" t="n">
-        <v>25.33685909276506</v>
+        <v>25.42921892932671</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7842,10 +7842,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>514310</v>
+        <v>514947</v>
       </c>
       <c r="L10" t="n">
-        <v>25.14242382998581</v>
+        <v>25.23502418695516</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7906,10 +7906,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>514310</v>
+        <v>514947</v>
       </c>
       <c r="L11" t="n">
-        <v>25.14242382998581</v>
+        <v>25.23502418695516</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7970,10 +7970,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>514310</v>
+        <v>514947</v>
       </c>
       <c r="L12" t="n">
-        <v>25.14242382998581</v>
+        <v>25.23502418695516</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -8034,10 +8034,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>514310</v>
+        <v>514947</v>
       </c>
       <c r="L13" t="n">
-        <v>25.14242382998581</v>
+        <v>25.23502418695516</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -8098,13 +8098,13 @@
         <v>415000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>557205</v>
+        <v>557895</v>
       </c>
       <c r="L14" t="n">
-        <v>25.52112777164599</v>
+        <v>25.61324263526291</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>-2999</v>
+        <v>0</v>
       </c>
       <c r="N14" t="n">
         <v>2.352941176470588</v>
@@ -8165,13 +8165,13 @@
         <v>415000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>557205</v>
+        <v>557895</v>
       </c>
       <c r="L15" t="n">
-        <v>25.52112777164599</v>
+        <v>25.61324263526291</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>-2999</v>
+        <v>0</v>
       </c>
       <c r="N15" t="n">
         <v>2.352941176470588</v>
@@ -8232,13 +8232,13 @@
         <v>415000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>557205</v>
+        <v>557895</v>
       </c>
       <c r="L16" t="n">
-        <v>25.52112777164599</v>
+        <v>25.61324263526291</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>-2999</v>
+        <v>0</v>
       </c>
       <c r="N16" t="n">
         <v>2.352941176470588</v>
@@ -8299,10 +8299,10 @@
         <v>420000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>557205</v>
+        <v>557895</v>
       </c>
       <c r="L17" t="n">
-        <v>24.62379196166581</v>
+        <v>24.71701664291668</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -8317,7 +8317,7 @@
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>8.5</v>
+        <v>8.6</v>
       </c>
       <c r="R17" t="n">
         <v>4</v>
@@ -8366,10 +8366,10 @@
         <v>454000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>600100</v>
+        <v>600843</v>
       </c>
       <c r="L18" t="n">
-        <v>24.34594234294284</v>
+        <v>24.43949584167578</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -8381,7 +8381,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q18" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="R18" t="n">
         <v>3</v>
@@ -8430,10 +8430,10 @@
         <v>454000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>600100</v>
+        <v>600843</v>
       </c>
       <c r="L19" t="n">
-        <v>24.34594234294284</v>
+        <v>24.43949584167578</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -8445,7 +8445,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q19" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="R19" t="n">
         <v>3</v>
@@ -8494,10 +8494,10 @@
         <v>454000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>600100</v>
+        <v>600843</v>
       </c>
       <c r="L20" t="n">
-        <v>24.34594234294284</v>
+        <v>24.43949584167578</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -8509,7 +8509,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q20" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="R20" t="n">
         <v>3</v>
@@ -8558,10 +8558,10 @@
         <v>454000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>600100</v>
+        <v>600843</v>
       </c>
       <c r="L21" t="n">
-        <v>24.34594234294284</v>
+        <v>24.43949584167578</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -8573,7 +8573,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q21" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="R21" t="n">
         <v>3</v>
@@ -8622,10 +8622,10 @@
         <v>455000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>600100</v>
+        <v>600843</v>
       </c>
       <c r="L22" t="n">
-        <v>24.1793034494251</v>
+        <v>24.27306301313321</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -8686,10 +8686,10 @@
         <v>455000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>600100</v>
+        <v>600843</v>
       </c>
       <c r="L23" t="n">
-        <v>24.1793034494251</v>
+        <v>24.27306301313321</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -8750,10 +8750,10 @@
         <v>455000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>600100</v>
+        <v>600843</v>
       </c>
       <c r="L24" t="n">
-        <v>24.1793034494251</v>
+        <v>24.27306301313321</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -8814,10 +8814,10 @@
         <v>455000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>600100</v>
+        <v>600843</v>
       </c>
       <c r="L25" t="n">
-        <v>24.1793034494251</v>
+        <v>24.27306301313321</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -8878,13 +8878,13 @@
         <v>468000</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>685890</v>
+        <v>686739</v>
       </c>
       <c r="L26" t="n">
-        <v>31.76748458207584</v>
+        <v>31.85183890823151</v>
       </c>
       <c r="M26" s="3" t="n">
-        <v>-11999</v>
+        <v>0</v>
       </c>
       <c r="N26" t="n">
         <v>2.499796874576822</v>
@@ -8942,13 +8942,13 @@
         <v>468000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>685890</v>
+        <v>686739</v>
       </c>
       <c r="L27" t="n">
-        <v>31.76748458207584</v>
+        <v>31.85183890823151</v>
       </c>
       <c r="M27" s="3" t="n">
-        <v>-11999</v>
+        <v>0</v>
       </c>
       <c r="N27" t="n">
         <v>2.499796874576822</v>
@@ -9006,13 +9006,13 @@
         <v>468000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>685890</v>
+        <v>686739</v>
       </c>
       <c r="L28" t="n">
-        <v>31.76748458207584</v>
+        <v>31.85183890823151</v>
       </c>
       <c r="M28" s="3" t="n">
-        <v>-11999</v>
+        <v>0</v>
       </c>
       <c r="N28" t="n">
         <v>2.499796874576822</v>
@@ -9070,13 +9070,13 @@
         <v>468000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>685890</v>
+        <v>686739</v>
       </c>
       <c r="L29" t="n">
-        <v>31.76748458207584</v>
+        <v>31.85183890823151</v>
       </c>
       <c r="M29" s="3" t="n">
-        <v>-11999</v>
+        <v>0</v>
       </c>
       <c r="N29" t="n">
         <v>2.499796874576822</v>
@@ -9134,10 +9134,10 @@
         <v>475000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>685890</v>
+        <v>686739</v>
       </c>
       <c r="L30" t="n">
-        <v>30.74691277026929</v>
+        <v>30.83252880643155</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -9198,10 +9198,10 @@
         <v>475000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>685890</v>
+        <v>686739</v>
       </c>
       <c r="L31" t="n">
-        <v>30.74691277026929</v>
+        <v>30.83252880643155</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -9262,10 +9262,10 @@
         <v>475000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>685890</v>
+        <v>686739</v>
       </c>
       <c r="L32" t="n">
-        <v>30.74691277026929</v>
+        <v>30.83252880643155</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -9326,10 +9326,10 @@
         <v>475000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>685890</v>
+        <v>686739</v>
       </c>
       <c r="L33" t="n">
-        <v>30.74691277026929</v>
+        <v>30.83252880643155</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -9390,10 +9390,10 @@
         <v>477000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>642995</v>
+        <v>643791</v>
       </c>
       <c r="L34" t="n">
-        <v>25.815908366317</v>
+        <v>25.90763151395406</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -9457,10 +9457,10 @@
         <v>477000</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>642995</v>
+        <v>643791</v>
       </c>
       <c r="L35" t="n">
-        <v>25.815908366317</v>
+        <v>25.90763151395406</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
@@ -9524,10 +9524,10 @@
         <v>477000</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>642995</v>
+        <v>643791</v>
       </c>
       <c r="L36" t="n">
-        <v>25.815908366317</v>
+        <v>25.90763151395406</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -9591,10 +9591,10 @@
         <v>479999</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>642995</v>
+        <v>643791</v>
       </c>
       <c r="L37" t="n">
-        <v>25.34949727447336</v>
+        <v>25.44179710496108</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
@@ -9609,7 +9609,7 @@
         <v>0</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.699999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="R37" t="n">
         <v>4</v>
@@ -9658,10 +9658,10 @@
         <v>500000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>642995</v>
+        <v>643791</v>
       </c>
       <c r="L38" t="n">
-        <v>22.23889765861321</v>
+        <v>22.33504351567512</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -9673,7 +9673,7 @@
         <v>31.30434782608695</v>
       </c>
       <c r="Q38" t="n">
-        <v>16.2</v>
+        <v>16.3</v>
       </c>
       <c r="R38" t="n">
         <v>3</v>
@@ -9722,13 +9722,13 @@
         <v>544999</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>771680</v>
+        <v>772635</v>
       </c>
       <c r="L39" t="n">
-        <v>29.375</v>
+        <v>29.46229461518052</v>
       </c>
       <c r="M39" s="3" t="n">
-        <v>-3000</v>
+        <v>0</v>
       </c>
       <c r="N39" t="n">
         <v>0.9090925619864764</v>
@@ -9786,13 +9786,13 @@
         <v>544999</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>771680</v>
+        <v>772635</v>
       </c>
       <c r="L40" t="n">
-        <v>29.375</v>
+        <v>29.46229461518052</v>
       </c>
       <c r="M40" s="3" t="n">
-        <v>-3000</v>
+        <v>0</v>
       </c>
       <c r="N40" t="n">
         <v>0.9090925619864764</v>
@@ -9850,13 +9850,13 @@
         <v>544999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>771680</v>
+        <v>772635</v>
       </c>
       <c r="L41" t="n">
-        <v>29.375</v>
+        <v>29.46229461518052</v>
       </c>
       <c r="M41" s="3" t="n">
-        <v>-3000</v>
+        <v>0</v>
       </c>
       <c r="N41" t="n">
         <v>1.268118239344636</v>
@@ -9914,13 +9914,13 @@
         <v>544999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>771680</v>
+        <v>772635</v>
       </c>
       <c r="L42" t="n">
-        <v>29.375</v>
+        <v>29.46229461518052</v>
       </c>
       <c r="M42" s="3" t="n">
-        <v>-3000</v>
+        <v>0</v>
       </c>
       <c r="N42" t="n">
         <v>0.9090925619864764</v>
@@ -9978,13 +9978,13 @@
         <v>549999</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>771680</v>
+        <v>772635</v>
       </c>
       <c r="L43" t="n">
-        <v>28.72706303130832</v>
+        <v>28.8151585159875</v>
       </c>
       <c r="M43" s="3" t="n">
-        <v>-3000</v>
+        <v>0</v>
       </c>
       <c r="N43" t="n">
         <v>1.78571747449549</v>
@@ -9993,7 +9993,7 @@
         <v>35.29417147279201</v>
       </c>
       <c r="Q43" t="n">
-        <v>20.5</v>
+        <v>20.6</v>
       </c>
       <c r="R43" t="n">
         <v>3</v>
@@ -10042,13 +10042,13 @@
         <v>549999</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>771680</v>
+        <v>772635</v>
       </c>
       <c r="L44" t="n">
-        <v>28.72706303130832</v>
+        <v>28.8151585159875</v>
       </c>
       <c r="M44" s="3" t="n">
-        <v>-3000</v>
+        <v>0</v>
       </c>
       <c r="N44" t="n">
         <v>1.78571747449549</v>
@@ -10057,7 +10057,7 @@
         <v>35.29417147279201</v>
       </c>
       <c r="Q44" t="n">
-        <v>20.5</v>
+        <v>20.6</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -10106,13 +10106,13 @@
         <v>549999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>771680</v>
+        <v>772635</v>
       </c>
       <c r="L45" t="n">
-        <v>28.72706303130832</v>
+        <v>28.8151585159875</v>
       </c>
       <c r="M45" s="3" t="n">
-        <v>-3000</v>
+        <v>0</v>
       </c>
       <c r="N45" t="n">
         <v>1.78571747449549</v>
@@ -10121,7 +10121,7 @@
         <v>35.29417147279201</v>
       </c>
       <c r="Q45" t="n">
-        <v>20.5</v>
+        <v>20.6</v>
       </c>
       <c r="R45" t="n">
         <v>3</v>
@@ -10170,13 +10170,13 @@
         <v>549999</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>771680</v>
+        <v>772635</v>
       </c>
       <c r="L46" t="n">
-        <v>28.72706303130832</v>
+        <v>28.8151585159875</v>
       </c>
       <c r="M46" s="3" t="n">
-        <v>-3000</v>
+        <v>0</v>
       </c>
       <c r="N46" t="n">
         <v>1.78571747449549</v>
@@ -10185,7 +10185,7 @@
         <v>35.29417147279201</v>
       </c>
       <c r="Q46" t="n">
-        <v>20.5</v>
+        <v>20.6</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -10234,10 +10234,10 @@
         <v>585000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>728785</v>
+        <v>729687</v>
       </c>
       <c r="L47" t="n">
-        <v>19.72941265256557</v>
+        <v>19.82863885474183</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -10298,10 +10298,10 @@
         <v>595000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>728785</v>
+        <v>729687</v>
       </c>
       <c r="L48" t="n">
-        <v>18.35726586030174</v>
+        <v>18.45818823687417</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -10362,13 +10362,13 @@
         <v>619999</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>857470</v>
+        <v>858531</v>
       </c>
       <c r="L49" t="n">
-        <v>27.69437997830828</v>
+        <v>27.78373757033817</v>
       </c>
       <c r="M49" s="3" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="N49" t="n">
         <v>0</v>
@@ -10426,13 +10426,13 @@
         <v>619999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>857470</v>
+        <v>858531</v>
       </c>
       <c r="L50" t="n">
-        <v>27.69437997830828</v>
+        <v>27.78373757033817</v>
       </c>
       <c r="M50" s="3" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="N50" t="n">
         <v>0</v>
@@ -10490,13 +10490,13 @@
         <v>619999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>857470</v>
+        <v>858531</v>
       </c>
       <c r="L51" t="n">
-        <v>27.69437997830828</v>
+        <v>27.78373757033817</v>
       </c>
       <c r="M51" s="3" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="N51" t="n">
         <v>0</v>
@@ -10554,13 +10554,13 @@
         <v>619999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>857470</v>
+        <v>858531</v>
       </c>
       <c r="L52" t="n">
-        <v>27.69437997830828</v>
+        <v>27.78373757033817</v>
       </c>
       <c r="M52" s="3" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="N52" t="n">
         <v>0</v>
@@ -10618,10 +10618,10 @@
         <v>650000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>814575</v>
+        <v>815583</v>
       </c>
       <c r="L53" t="n">
-        <v>20.20378725102047</v>
+        <v>20.30240944208008</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -10633,7 +10633,7 @@
         <v>47.05854671135535</v>
       </c>
       <c r="Q53" t="n">
-        <v>18.7</v>
+        <v>18.8</v>
       </c>
       <c r="R53" t="n">
         <v>3</v>
@@ -10682,10 +10682,10 @@
         <v>672000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>857470</v>
+        <v>858531</v>
       </c>
       <c r="L54" t="n">
-        <v>21.62991125053938</v>
+        <v>21.72676350650122</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -10746,10 +10746,10 @@
         <v>700000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>900365</v>
+        <v>901479</v>
       </c>
       <c r="L55" t="n">
-        <v>22.25375264476073</v>
+        <v>22.34982733929465</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -10810,10 +10810,10 @@
         <v>715000</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>943260</v>
+        <v>944427</v>
       </c>
       <c r="L56" t="n">
-        <v>24.19905434344719</v>
+        <v>24.2927192890504</v>
       </c>
       <c r="M56" s="3" t="n">
         <v>0</v>
@@ -10874,10 +10874,10 @@
         <v>734999</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>986155</v>
+        <v>987375</v>
       </c>
       <c r="L57" t="n">
-        <v>25.46820733049064</v>
+        <v>25.56029877199645</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -10938,10 +10938,10 @@
         <v>752000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>986155</v>
+        <v>987375</v>
       </c>
       <c r="L58" t="n">
-        <v>23.74423898879994</v>
+        <v>23.83846056462843</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -10953,7 +10953,7 @@
         <v>54.37884642534079</v>
       </c>
       <c r="Q58" t="n">
-        <v>21.8</v>
+        <v>21.9</v>
       </c>
       <c r="R58" t="n">
         <v>3</v>
@@ -11002,10 +11002,10 @@
         <v>810000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1071944</v>
+        <v>1073271</v>
       </c>
       <c r="L59" t="n">
-        <v>24.43635115267215</v>
+        <v>24.52977859273194</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -11066,10 +11066,10 @@
         <v>815000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1071944</v>
+        <v>1073271</v>
       </c>
       <c r="L60" t="n">
-        <v>23.9699088758368</v>
+        <v>24.06391302848954</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -11081,7 +11081,7 @@
         <v>79.56521739130434</v>
       </c>
       <c r="Q60" t="n">
-        <v>27.3</v>
+        <v>27.4</v>
       </c>
       <c r="R60" t="n">
         <v>3</v>
@@ -11130,10 +11130,10 @@
         <v>875000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1157734</v>
+        <v>1159167</v>
       </c>
       <c r="L61" t="n">
-        <v>24.42132648777698</v>
+        <v>24.5147593056048</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -11194,10 +11194,10 @@
         <v>992000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1329314</v>
+        <v>1330959</v>
       </c>
       <c r="L62" t="n">
-        <v>25.37504306732646</v>
+        <v>25.46727585147251</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -11209,7 +11209,7 @@
         <v>85.14782608695651</v>
       </c>
       <c r="Q62" t="n">
-        <v>29.1</v>
+        <v>29.2</v>
       </c>
       <c r="R62" t="n">
         <v>3</v>
@@ -11258,10 +11258,10 @@
         <v>1050000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1415104</v>
+        <v>1416856</v>
       </c>
       <c r="L63" t="n">
-        <v>25.80050653520872</v>
+        <v>25.89225722303467</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -11322,10 +11322,10 @@
         <v>1050000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1415104</v>
+        <v>1416856</v>
       </c>
       <c r="L64" t="n">
-        <v>25.80050653520872</v>
+        <v>25.89225722303467</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -11337,7 +11337,7 @@
         <v>86.27443803627732</v>
       </c>
       <c r="Q64" t="n">
-        <v>29.5</v>
+        <v>29.6</v>
       </c>
       <c r="R64" t="n">
         <v>3</v>
@@ -11386,10 +11386,10 @@
         <v>1100000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1500894</v>
+        <v>1502752</v>
       </c>
       <c r="L65" t="n">
-        <v>26.71034729967606</v>
+        <v>26.80096250079854</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -11401,7 +11401,7 @@
         <v>94.11761630126171</v>
       </c>
       <c r="Q65" t="n">
-        <v>31.6</v>
+        <v>31.7</v>
       </c>
       <c r="R65" t="n">
         <v>3</v>
@@ -11450,10 +11450,10 @@
         <v>1105000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1500894</v>
+        <v>1502752</v>
       </c>
       <c r="L66" t="n">
-        <v>26.37721251467459</v>
+        <v>26.4682396030749</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -11465,7 +11465,7 @@
         <v>100</v>
       </c>
       <c r="Q66" t="n">
-        <v>32.7</v>
+        <v>32.8</v>
       </c>
       <c r="R66" t="n">
         <v>3</v>
@@ -11514,10 +11514,10 @@
         <v>1155000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1586684</v>
+        <v>1588648</v>
       </c>
       <c r="L67" t="n">
-        <v>27.20667757411053</v>
+        <v>27.29666987274714</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -11784,7 +11784,7 @@
         <v>315000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>299836</v>
+        <v>300207</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -11845,10 +11845,10 @@
         <v>380000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>385625</v>
+        <v>386103</v>
       </c>
       <c r="L3" t="n">
-        <v>1.458670988654781</v>
+        <v>1.580666298889156</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -11909,7 +11909,7 @@
         <v>415000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>385625</v>
+        <v>386103</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -11970,10 +11970,10 @@
         <v>495000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>471415</v>
+        <v>471999</v>
       </c>
       <c r="L5" t="n">
-        <v>6.664191847947137</v>
+        <v>6.779675380668179</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -12034,10 +12034,10 @@
         <v>490000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514310</v>
+        <v>514947</v>
       </c>
       <c r="L6" t="n">
-        <v>4.726721238163754</v>
+        <v>4.844576237942934</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -12049,7 +12049,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="R6" t="n">
         <v>3</v>
@@ -12098,10 +12098,10 @@
         <v>550000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>557205</v>
+        <v>557895</v>
       </c>
       <c r="L7" t="n">
-        <v>6.677075762062437</v>
+        <v>6.792496795992077</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -12162,7 +12162,7 @@
         <v>530000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>471415</v>
+        <v>471999</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -12226,10 +12226,10 @@
         <v>600000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>600100</v>
+        <v>600843</v>
       </c>
       <c r="L9" t="n">
-        <v>8.348608565239127</v>
+        <v>8.4619443015896</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -12241,7 +12241,7 @@
         <v>30.25295873936471</v>
       </c>
       <c r="Q9" t="n">
-        <v>9.800000000000001</v>
+        <v>9.9</v>
       </c>
       <c r="R9" t="n">
         <v>4</v>
@@ -12290,10 +12290,10 @@
         <v>646000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>728785</v>
+        <v>729687</v>
       </c>
       <c r="L10" t="n">
-        <v>16.98525628271713</v>
+        <v>17.08787466406829</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -12305,7 +12305,7 @@
         <v>100</v>
       </c>
       <c r="Q10" t="n">
-        <v>25.9</v>
+        <v>26</v>
       </c>
       <c r="R10" t="n">
         <v>4</v>
@@ -12354,7 +12354,7 @@
         <v>615000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>557205</v>
+        <v>557895</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -12418,7 +12418,7 @@
         <v>700000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>642995</v>
+        <v>643791</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -12482,7 +12482,7 @@
         <v>745000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>685890</v>
+        <v>686739</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -12546,7 +12546,7 @@
         <v>930000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>857470</v>
+        <v>858531</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -12617,7 +12617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12666,7 +12666,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHF4 M5 10C CPU 10C GPU 16GB 1TB Midnight</t>
+          <t>Macbook Pro 14 M5 MJ3E4 10 Core CPU 10 Core GPU 32GB 1TB Silver</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -12675,22 +12675,22 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>479999</v>
+        <v>769999</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>468000</v>
+        <v>759999</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-11999</v>
+        <v>-10000</v>
       </c>
       <c r="F2" t="n">
-        <v>-2.5</v>
+        <v>-1.3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHJ4 M5 10C CPU 10C GPU 16GB 1TB Sky Blue</t>
+          <t>Macbook Pro 14 M5 MJ3D4 10 Core CPU 10 Core GPU 32GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -12699,22 +12699,22 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>479999</v>
+        <v>769999</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>468000</v>
+        <v>759999</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>-11999</v>
+        <v>-10000</v>
       </c>
       <c r="F3" t="n">
-        <v>-2.5</v>
+        <v>-1.3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDH84 M5 10C CPU 10C GPU 16GB 1TB Silver</t>
+          <t>Macbook Pro 14 M5 MDE54 10 Core CPU 10 Core GPU 16GB 1TB Silver</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -12723,597 +12723,21 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>479999</v>
+        <v>587999</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>468000</v>
+        <v>584999</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>-11999</v>
+        <v>-3000</v>
       </c>
       <c r="F4" t="n">
-        <v>-2.5</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDHC4 M5 10C CPU 10C GPU 16GB 1TB Starlight</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>479999</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>468000</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>-11999</v>
-      </c>
-      <c r="F5" t="n">
-        <v>-2.5</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDHG4 M5 10C CPU 10C GPU 24GB 1TB Midnight</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>547999</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>544999</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>-3000</v>
-      </c>
-      <c r="F6" t="n">
-        <v>-0.55</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDHK4 M5 10C CPU 10C GPU 24GB 1TB Sky Blue</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>547999</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>544999</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>-3000</v>
-      </c>
-      <c r="F7" t="n">
-        <v>-0.55</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDH94 M5 10C CPU 10C GPU 24GB 1TB Silver</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>547999</v>
-      </c>
-      <c r="D8" s="3" t="n">
-        <v>544999</v>
-      </c>
-      <c r="E8" s="3" t="n">
-        <v>-3000</v>
-      </c>
-      <c r="F8" t="n">
-        <v>-0.55</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDHD4 M5 10C CPU 10C GPU 24GB 1TB Starlight</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>547999</v>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>544999</v>
-      </c>
-      <c r="E9" s="3" t="n">
-        <v>-3000</v>
-      </c>
-      <c r="F9" t="n">
-        <v>-0.55</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDVK4 M5 10C CPU 10C GPU 16GB 1TB Midnight</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>552999</v>
-      </c>
-      <c r="D10" s="3" t="n">
-        <v>549999</v>
-      </c>
-      <c r="E10" s="3" t="n">
-        <v>-3000</v>
-      </c>
-      <c r="F10" t="n">
-        <v>-0.54</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDVA4 M5 10C CPU 10C GPU 16GB 1TB Silver</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="n">
-        <v>552999</v>
-      </c>
-      <c r="D11" s="3" t="n">
-        <v>549999</v>
-      </c>
-      <c r="E11" s="3" t="n">
-        <v>-3000</v>
-      </c>
-      <c r="F11" t="n">
-        <v>-0.54</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDVE4 M5 10C CPU 10C GPU 16GB 1TB Starlight</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="n">
-        <v>552999</v>
-      </c>
-      <c r="D12" s="3" t="n">
-        <v>549999</v>
-      </c>
-      <c r="E12" s="3" t="n">
-        <v>-3000</v>
-      </c>
-      <c r="F12" t="n">
-        <v>-0.54</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDVT4 M5 10C CPU 10C GPU 16GB 1TB Sky Blue</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="n">
-        <v>552999</v>
-      </c>
-      <c r="D13" s="3" t="n">
-        <v>549999</v>
-      </c>
-      <c r="E13" s="3" t="n">
-        <v>-3000</v>
-      </c>
-      <c r="F13" t="n">
-        <v>-0.54</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDHE4 M5 10C CPU 8C GPU 16GB 512GB Midnight</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="n">
-        <v>417999</v>
-      </c>
-      <c r="D14" s="3" t="n">
-        <v>415000</v>
-      </c>
-      <c r="E14" s="3" t="n">
-        <v>-2999</v>
-      </c>
-      <c r="F14" t="n">
-        <v>-0.72</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDHH4 M5 10C CPU 8C GPU 16GB 512GB Sky Blue</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="n">
-        <v>417999</v>
-      </c>
-      <c r="D15" s="3" t="n">
-        <v>415000</v>
-      </c>
-      <c r="E15" s="3" t="n">
-        <v>-2999</v>
-      </c>
-      <c r="F15" t="n">
-        <v>-0.72</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 13 MDHA4 M5 10C CPU 8C GPU 16GB 512GB Starlight</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="n">
-        <v>417999</v>
-      </c>
-      <c r="D16" s="3" t="n">
-        <v>415000</v>
-      </c>
-      <c r="E16" s="3" t="n">
-        <v>-2999</v>
-      </c>
-      <c r="F16" t="n">
-        <v>-0.72</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 MGDR4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Space Black</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="n">
-        <v>720000</v>
-      </c>
-      <c r="D17" s="3" t="n">
-        <v>717999</v>
-      </c>
-      <c r="E17" s="3" t="n">
-        <v>-2001</v>
-      </c>
-      <c r="F17" t="n">
-        <v>-0.28</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 M5 MDE34 10 Core CPU 10 Core GPU 24GB 1TB Space Black</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="n">
-        <v>644999</v>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>642999</v>
-      </c>
-      <c r="E18" s="3" t="n">
-        <v>-2000</v>
-      </c>
-      <c r="F18" t="n">
-        <v>-0.31</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 MGDN4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Silver</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="n">
-        <v>725000</v>
-      </c>
-      <c r="D19" s="3" t="n">
-        <v>723500</v>
-      </c>
-      <c r="E19" s="3" t="n">
-        <v>-1500</v>
-      </c>
-      <c r="F19" t="n">
-        <v>-0.21</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 M5 MDE14 10 Core CPU 10 Core GPU 16GB 1TB Space Black</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="n">
-        <v>579999</v>
-      </c>
-      <c r="D20" s="3" t="n">
-        <v>578999</v>
-      </c>
-      <c r="E20" s="3" t="n">
-        <v>-1000</v>
-      </c>
-      <c r="F20" t="n">
-        <v>-0.17</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Macbook Pro 16 MGEC4 M5 Pro 18 Core CPU 20 Core GPU 48GB 1TB Space Black</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="n">
-        <v>1055000</v>
-      </c>
-      <c r="D21" s="3" t="n">
-        <v>1054000</v>
-      </c>
-      <c r="E21" s="3" t="n">
-        <v>-1000</v>
-      </c>
-      <c r="F21" t="n">
-        <v>-0.09</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Macbook Pro 16 MGE64 M5 Pro 18 Core CPU 20 Core GPU 48GB 1TB Silver</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="n">
-        <v>1055000</v>
-      </c>
-      <c r="D22" s="3" t="n">
-        <v>1054000</v>
-      </c>
-      <c r="E22" s="3" t="n">
-        <v>-1000</v>
-      </c>
-      <c r="F22" t="n">
-        <v>-0.09</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDVU4 M5 10C CPU 10C GPU 24GB 1TB Sky Blue</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="n">
-        <v>614999</v>
-      </c>
-      <c r="D23" s="3" t="n">
-        <v>619999</v>
-      </c>
-      <c r="E23" s="3" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F23" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDVF4 M5 10C CPU 10C GPU 24GB 1TB Starlight</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="n">
-        <v>614999</v>
-      </c>
-      <c r="D24" s="3" t="n">
-        <v>619999</v>
-      </c>
-      <c r="E24" s="3" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F24" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDVC4 M5 10C CPU 10C GPU 24GB 1TB Silver</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="n">
-        <v>614999</v>
-      </c>
-      <c r="D25" s="3" t="n">
-        <v>619999</v>
-      </c>
-      <c r="E25" s="3" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F25" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDVN4 M5 10C CPU 10C GPU 24GB 1TB Midnight</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="n">
-        <v>614999</v>
-      </c>
-      <c r="D26" s="3" t="n">
-        <v>619999</v>
-      </c>
-      <c r="E26" s="3" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F26" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 MGDP4 M5 Pro 18 Core CPU 20 Core GPU 24GB 2TB Silver</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="n">
-        <v>875000</v>
-      </c>
-      <c r="D27" s="3" t="n">
-        <v>955000</v>
-      </c>
-      <c r="E27" s="3" t="n">
-        <v>80000</v>
-      </c>
-      <c r="F27" t="n">
-        <v>9.140000000000001</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 MGDT4 M5 Pro 18 Core CPU 20 Core GPU 24GB 2TB Space Black</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="n">
-        <v>864999</v>
-      </c>
-      <c r="D28" s="3" t="n">
-        <v>955000</v>
-      </c>
-      <c r="E28" s="3" t="n">
-        <v>90001</v>
-      </c>
-      <c r="F28" t="n">
-        <v>10.4</v>
+        <v>-0.51</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F28"/>
-  <conditionalFormatting sqref="E2:E28">
+  <autoFilter ref="A1:F4"/>
+  <conditionalFormatting sqref="E2:E4">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
chore: price data 2026-10-09
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MacBook Pro'!$A$1:$S$93</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MacBook Air'!$A$1:$S$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20261008T104029385040+0000</t>
+          <t>20261009T103947329100+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-08T10:40:29.385040+00:00</t>
+          <t>2026-10-09T10:39:47.329100+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>277.084072</v>
+        <v>277.018</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -1147,10 +1147,10 @@
         <v>470000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>686739</v>
+        <v>686575</v>
       </c>
       <c r="L2" t="n">
-        <v>35.20100067128851</v>
+        <v>35.18552233914722</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1214,10 +1214,10 @@
         <v>495000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>686739</v>
+        <v>686575</v>
       </c>
       <c r="L3" t="n">
-        <v>27.92021422986025</v>
+        <v>27.90299675927612</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>772635</v>
+        <v>772451</v>
       </c>
       <c r="L4" t="n">
-        <v>35.28651950791771</v>
+        <v>35.27110457491802</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>772635</v>
+        <v>772451</v>
       </c>
       <c r="L5" t="n">
-        <v>32.69797511114562</v>
+        <v>32.68194357959275</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>858531</v>
+        <v>858326</v>
       </c>
       <c r="L6" t="n">
-        <v>38.03368777598013</v>
+        <v>38.01888792836288</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1606,10 +1606,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>858531</v>
+        <v>858326</v>
       </c>
       <c r="L9" t="n">
-        <v>34.18991276960296</v>
+        <v>34.17419488632525</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1673,10 +1673,10 @@
         <v>578999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>858531</v>
+        <v>858326</v>
       </c>
       <c r="L10" t="n">
-        <v>32.55933682068557</v>
+        <v>32.54322949555297</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -1740,13 +1740,13 @@
         <v>584999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>858531</v>
+        <v>858326</v>
       </c>
       <c r="L11" t="n">
-        <v>31.8604686377079</v>
+        <v>31.84419439700067</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>-3000</v>
+        <v>0</v>
       </c>
       <c r="N11" t="n">
         <v>0.5102049493281451</v>
@@ -1772,7 +1772,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 14Inch MX2H3 M4 Pro 12Core CPU 16Core GPU 24GB 512GB Space Black</t>
+          <t>Apple MacBook Pro 14Inch MX2E3 M4 Pro 12Core CPU 16Core GPU 24GB 512GB Silver</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -1797,38 +1797,35 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I12" s="3" t="n">
-        <v>600000</v>
+        <v>634000</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>600000</v>
+        <v>634000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>858531</v>
+        <v>858326</v>
       </c>
       <c r="L12" t="n">
-        <v>30.11318170223323</v>
+        <v>26.13529125297381</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>4</v>
-      </c>
-      <c r="O12" t="n">
-        <v>100</v>
+        <v>0.9375</v>
       </c>
       <c r="P12" t="n">
-        <v>45.94594594594595</v>
+        <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>41</v>
+        <v>11.5</v>
       </c>
       <c r="R12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -1839,7 +1836,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 14Inch MX2E3 M4 Pro 12Core CPU 16Core GPU 24GB 512GB Silver</t>
+          <t>Apple MacBook Pro 14Inch MX2H3 M4 Pro 12Core CPU 16Core GPU 24GB 512GB Space Black</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1864,7 +1861,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I13" s="3" t="n">
@@ -1874,28 +1871,25 @@
         <v>634000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>858531</v>
+        <v>858326</v>
       </c>
       <c r="L13" t="n">
-        <v>26.15292866535978</v>
+        <v>26.13529125297381</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>0</v>
+        <v>34000</v>
       </c>
       <c r="N13" t="n">
-        <v>1.705426356589147</v>
-      </c>
-      <c r="O13" t="n">
         <v>0</v>
       </c>
       <c r="P13" t="n">
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>9.199999999999999</v>
+        <v>11.2</v>
       </c>
       <c r="R13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
@@ -1941,10 +1935,10 @@
         <v>642999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>944427</v>
+        <v>944202</v>
       </c>
       <c r="L14" t="n">
-        <v>31.91649539879737</v>
+        <v>31.90027134024287</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -2067,10 +2061,10 @@
         <v>650000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>944427</v>
+        <v>944202</v>
       </c>
       <c r="L16" t="n">
-        <v>31.17519935368218</v>
+        <v>31.15879864689971</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -2134,10 +2128,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1030323</v>
+        <v>1030078</v>
       </c>
       <c r="L17" t="n">
-        <v>32.06014036375001</v>
+        <v>32.04398113540916</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2201,10 +2195,10 @@
         <v>711999</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>1073271</v>
+        <v>1073015</v>
       </c>
       <c r="L18" t="n">
-        <v>33.66083682499574</v>
+        <v>33.64500962241907</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -2330,10 +2324,10 @@
         <v>720000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>1030323</v>
+        <v>1030078</v>
       </c>
       <c r="L20" t="n">
-        <v>30.11900151700001</v>
+        <v>30.10238059642085</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -2459,10 +2453,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1073271</v>
+        <v>1073015</v>
       </c>
       <c r="L22" t="n">
-        <v>30.77237715358004</v>
+        <v>30.75586082207612</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2526,13 +2520,13 @@
         <v>759999</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1030323</v>
+        <v>1030078</v>
       </c>
       <c r="L23" t="n">
-        <v>26.23682088044234</v>
+        <v>26.21927659847119</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>-10000</v>
+        <v>0</v>
       </c>
       <c r="N23" t="n">
         <v>1.554533678756477</v>
@@ -2593,13 +2587,13 @@
         <v>759999</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1030323</v>
+        <v>1030078</v>
       </c>
       <c r="L24" t="n">
-        <v>26.23682088044234</v>
+        <v>26.21927659847119</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>-10000</v>
+        <v>0</v>
       </c>
       <c r="N24" t="n">
         <v>1.554533678756477</v>
@@ -2660,10 +2654,10 @@
         <v>772000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>1030323</v>
+        <v>1030078</v>
       </c>
       <c r="L25" t="n">
-        <v>25.07204051545001</v>
+        <v>25.05421919505125</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -2851,10 +2845,10 @@
         <v>810000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>1073271</v>
+        <v>1073015</v>
       </c>
       <c r="L28" t="n">
-        <v>24.52977859273194</v>
+        <v>24.51177290159038</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -2915,10 +2909,10 @@
         <v>810000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>1245063</v>
+        <v>1244767</v>
       </c>
       <c r="L29" t="n">
-        <v>34.94305107452394</v>
+        <v>34.92758082436311</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -2982,16 +2976,16 @@
         <v>822999</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1288011</v>
+        <v>1287704</v>
       </c>
       <c r="L30" t="n">
-        <v>36.10310781507301</v>
+        <v>36.08787423196635</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N30" t="n">
-        <v>1.437186489333227</v>
+        <v>0.8433745100897712</v>
       </c>
       <c r="O30" t="n">
         <v>100</v>
@@ -3000,7 +2994,7 @@
         <v>0.0003521901827191575</v>
       </c>
       <c r="Q30" t="n">
-        <v>34.7</v>
+        <v>34.5</v>
       </c>
       <c r="R30" t="n">
         <v>4</v>
@@ -3049,10 +3043,10 @@
         <v>823000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1288011</v>
+        <v>1287704</v>
       </c>
       <c r="L31" t="n">
-        <v>36.10303017598452</v>
+        <v>36.08779657436803</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -3116,10 +3110,10 @@
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1373908</v>
+        <v>1373580</v>
       </c>
       <c r="L32" t="n">
-        <v>38.27832722423918</v>
+        <v>38.26358857875042</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3183,10 +3177,10 @@
         <v>930000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1373908</v>
+        <v>1373580</v>
       </c>
       <c r="L33" t="n">
-        <v>38.13275706961456</v>
+        <v>38.11798366312847</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3250,10 +3244,10 @@
         <v>860000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>1245063</v>
+        <v>1244767</v>
       </c>
       <c r="L34" t="n">
-        <v>30.92719002974147</v>
+        <v>30.91076482586701</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -3379,10 +3373,10 @@
         <v>880000</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>1159167</v>
+        <v>1158891</v>
       </c>
       <c r="L36" t="n">
-        <v>24.0834150730654</v>
+        <v>24.06533487618767</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -3443,10 +3437,10 @@
         <v>940000</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>1245063</v>
+        <v>1244767</v>
       </c>
       <c r="L37" t="n">
-        <v>24.50181235808951</v>
+        <v>24.48385922827324</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
@@ -3631,16 +3625,16 @@
         <v>990000</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>1502752</v>
+        <v>1502393</v>
       </c>
       <c r="L40" t="n">
-        <v>34.12086625071868</v>
+        <v>34.10512429171328</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N40" t="n">
-        <v>1.834407535944472</v>
+        <v>0.5025125628140703</v>
       </c>
       <c r="O40" t="n">
         <v>100</v>
@@ -3649,7 +3643,7 @@
         <v>39.19647231749141</v>
       </c>
       <c r="Q40" t="n">
-        <v>40.6</v>
+        <v>40.3</v>
       </c>
       <c r="R40" t="n">
         <v>4</v>
@@ -3760,10 +3754,10 @@
         <v>1000000</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>1502752</v>
+        <v>1502393</v>
       </c>
       <c r="L42" t="n">
-        <v>33.45542045527139</v>
+        <v>33.43951948657908</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -3827,10 +3821,10 @@
         <v>1054000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1545700</v>
+        <v>1545331</v>
       </c>
       <c r="L43" t="n">
-        <v>31.81083004463997</v>
+        <v>31.79454757589151</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -3891,10 +3885,10 @@
         <v>1054000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1545700</v>
+        <v>1545331</v>
       </c>
       <c r="L44" t="n">
-        <v>31.81083004463997</v>
+        <v>31.79454757589151</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -4017,22 +4011,22 @@
         <v>1115000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1502752</v>
+        <v>1502393</v>
       </c>
       <c r="L46" t="n">
-        <v>25.80279380762761</v>
+        <v>25.78506422753567</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N46" t="n">
-        <v>1.545253863134658</v>
+        <v>0</v>
       </c>
       <c r="P46" t="n">
         <v>9.358196283135744</v>
       </c>
       <c r="Q46" t="n">
-        <v>13.6</v>
+        <v>13.1</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -4081,10 +4075,10 @@
         <v>1123000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1717492</v>
+        <v>1717082</v>
       </c>
       <c r="L47" t="n">
-        <v>34.61396035614722</v>
+        <v>34.59834766190549</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -4148,10 +4142,10 @@
         <v>1130000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1502752</v>
+        <v>1502393</v>
       </c>
       <c r="L48" t="n">
-        <v>24.80462511445668</v>
+        <v>24.78665701983436</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -4274,10 +4268,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1760440</v>
+        <v>1760020</v>
       </c>
       <c r="L50" t="n">
-        <v>34.39140214946264</v>
+        <v>34.37574573016215</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4338,10 +4332,10 @@
         <v>1155000</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>1760440</v>
+        <v>1760020</v>
       </c>
       <c r="L51" t="n">
-        <v>34.39140214946264</v>
+        <v>34.37574573016215</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -4402,10 +4396,10 @@
         <v>1185000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1588648</v>
+        <v>1588269</v>
       </c>
       <c r="L52" t="n">
-        <v>25.40827168762369</v>
+        <v>25.39047226886629</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -4466,10 +4460,10 @@
         <v>1185000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1588648</v>
+        <v>1588269</v>
       </c>
       <c r="L53" t="n">
-        <v>25.40827168762369</v>
+        <v>25.39047226886629</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -4530,10 +4524,10 @@
         <v>1200000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1889284</v>
+        <v>1888833</v>
       </c>
       <c r="L54" t="n">
-        <v>36.4838743142905</v>
+        <v>36.46870845649139</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -4594,10 +4588,10 @@
         <v>1200000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1889284</v>
+        <v>1888833</v>
       </c>
       <c r="L55" t="n">
-        <v>36.4838743142905</v>
+        <v>36.46870845649139</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -4720,10 +4714,10 @@
         <v>1240000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1674544</v>
+        <v>1674144</v>
       </c>
       <c r="L57" t="n">
-        <v>25.949989967418</v>
+        <v>25.9322973412084</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -4846,10 +4840,10 @@
         <v>1280000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1717492</v>
+        <v>1717082</v>
       </c>
       <c r="L59" t="n">
-        <v>25.47272418153913</v>
+        <v>25.45492876869014</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -4913,22 +4907,22 @@
         <v>1298000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1760440</v>
+        <v>1760020</v>
       </c>
       <c r="L60" t="n">
-        <v>26.26843289177706</v>
+        <v>26.25083805865843</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N60" t="n">
-        <v>1.517450682852807</v>
+        <v>0</v>
       </c>
       <c r="P60" t="n">
         <v>61.28109178956637</v>
       </c>
       <c r="Q60" t="n">
-        <v>24.9</v>
+        <v>24.4</v>
       </c>
       <c r="R60" t="n">
         <v>3</v>
@@ -4977,22 +4971,22 @@
         <v>1300000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1717492</v>
+        <v>1717082</v>
       </c>
       <c r="L61" t="n">
-        <v>24.30823549687568</v>
+        <v>24.29016203070092</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N61" t="n">
-        <v>0.3831417624521072</v>
+        <v>0</v>
       </c>
       <c r="P61" t="n">
         <v>60.92890160686771</v>
       </c>
       <c r="Q61" t="n">
-        <v>23.6</v>
+        <v>23.5</v>
       </c>
       <c r="R61" t="n">
         <v>3</v>
@@ -5103,10 +5097,10 @@
         <v>1335000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1803388</v>
+        <v>1802958</v>
       </c>
       <c r="L63" t="n">
-        <v>25.97266922037853</v>
+        <v>25.95501392711311</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -5167,22 +5161,22 @@
         <v>1420000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1932232</v>
+        <v>1931771</v>
       </c>
       <c r="L64" t="n">
-        <v>26.50986009961537</v>
+        <v>26.49232233013126</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N64" t="n">
-        <v>1.764095468695953</v>
+        <v>0</v>
       </c>
       <c r="P64" t="n">
         <v>81.47332893095606</v>
       </c>
       <c r="Q64" t="n">
-        <v>29.4</v>
+        <v>28.8</v>
       </c>
       <c r="R64" t="n">
         <v>3</v>
@@ -5231,22 +5225,22 @@
         <v>1430000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1932232</v>
+        <v>1931771</v>
       </c>
       <c r="L65" t="n">
-        <v>25.99232390313378</v>
+        <v>25.97466262823078</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N65" t="n">
-        <v>1.413305756635643</v>
+        <v>0</v>
       </c>
       <c r="P65" t="n">
         <v>60.92890160686771</v>
       </c>
       <c r="Q65" t="n">
-        <v>24.7</v>
+        <v>24.2</v>
       </c>
       <c r="R65" t="n">
         <v>3</v>
@@ -5295,10 +5289,10 @@
         <v>1430000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>2146972</v>
+        <v>2146460</v>
       </c>
       <c r="L66" t="n">
-        <v>33.39456685974479</v>
+        <v>33.37867931384699</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -5359,10 +5353,10 @@
         <v>1430000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>2146972</v>
+        <v>2146460</v>
       </c>
       <c r="L67" t="n">
-        <v>33.39456685974479</v>
+        <v>33.37867931384699</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -5485,10 +5479,10 @@
         <v>1480000</v>
       </c>
       <c r="K69" s="3" t="n">
-        <v>2018128</v>
+        <v>2017647</v>
       </c>
       <c r="L69" t="n">
-        <v>26.66471105896157</v>
+        <v>26.64722818213493</v>
       </c>
       <c r="M69" s="3" t="n">
         <v>0</v>
@@ -5611,10 +5605,10 @@
         <v>1605000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2189920</v>
+        <v>2189398</v>
       </c>
       <c r="L71" t="n">
-        <v>26.70965149411851</v>
+        <v>26.69217748440439</v>
       </c>
       <c r="M71" s="3" t="n">
         <v>0</v>
@@ -5626,7 +5620,7 @@
         <v>36.44392794886694</v>
       </c>
       <c r="Q71" t="n">
-        <v>19.3</v>
+        <v>19.2</v>
       </c>
       <c r="R71" t="n">
         <v>3</v>
@@ -5675,10 +5669,10 @@
         <v>1610000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2189920</v>
+        <v>2189398</v>
       </c>
       <c r="L72" t="n">
-        <v>26.48133265142106</v>
+        <v>26.4638042055396</v>
       </c>
       <c r="M72" s="3" t="n">
         <v>0</v>
@@ -5739,22 +5733,22 @@
         <v>1615000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2189920</v>
+        <v>2189398</v>
       </c>
       <c r="L73" t="n">
-        <v>26.25301380872361</v>
+        <v>26.23543092667482</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N73" t="n">
-        <v>1.404151404151404</v>
+        <v>0</v>
       </c>
       <c r="P73" t="n">
         <v>86.7142542687337</v>
       </c>
       <c r="Q73" t="n">
-        <v>30.3</v>
+        <v>29.8</v>
       </c>
       <c r="R73" t="n">
         <v>3</v>
@@ -5803,10 +5797,10 @@
         <v>1630000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2232868</v>
+        <v>2232336</v>
       </c>
       <c r="L74" t="n">
-        <v>26.99971516453279</v>
+        <v>26.98231807398169</v>
       </c>
       <c r="M74" s="3" t="n">
         <v>0</v>
@@ -5867,22 +5861,22 @@
         <v>1690000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2318764</v>
+        <v>2318211</v>
       </c>
       <c r="L75" t="n">
-        <v>27.11634301722815</v>
+        <v>27.09895691116986</v>
       </c>
       <c r="M75" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N75" t="n">
-        <v>0.6174654513378418</v>
+        <v>0</v>
       </c>
       <c r="P75" t="n">
         <v>16.88768606224628</v>
       </c>
       <c r="Q75" t="n">
-        <v>15.5</v>
+        <v>15.2</v>
       </c>
       <c r="R75" t="n">
         <v>3</v>
@@ -5931,22 +5925,22 @@
         <v>1705000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2318764</v>
+        <v>2318211</v>
       </c>
       <c r="L76" t="n">
-        <v>26.46944665347573</v>
+        <v>26.45190623286664</v>
       </c>
       <c r="M76" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N76" t="n">
-        <v>1.473562554175094</v>
+        <v>0</v>
       </c>
       <c r="P76" t="n">
         <v>1.9846639603067</v>
       </c>
       <c r="Q76" t="n">
-        <v>12.3</v>
+        <v>11.8</v>
       </c>
       <c r="R76" t="n">
         <v>3</v>
@@ -5995,22 +5989,22 @@
         <v>1725000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2361712</v>
+        <v>2361149</v>
       </c>
       <c r="L77" t="n">
-        <v>26.95976478080308</v>
+        <v>26.94234883101405</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N77" t="n">
-        <v>1.849217638691323</v>
+        <v>0</v>
       </c>
       <c r="P77" t="n">
         <v>100</v>
       </c>
       <c r="Q77" t="n">
-        <v>33.6</v>
+        <v>33</v>
       </c>
       <c r="R77" t="n">
         <v>3</v>
@@ -6059,10 +6053,10 @@
         <v>1780000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2447608</v>
+        <v>2447025</v>
       </c>
       <c r="L78" t="n">
-        <v>27.2759363427477</v>
+        <v>27.2586099447288</v>
       </c>
       <c r="M78" s="3" t="n">
         <v>0</v>
@@ -6123,22 +6117,22 @@
         <v>1875000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2576452</v>
+        <v>2575838</v>
       </c>
       <c r="L79" t="n">
-        <v>27.22550235750559</v>
+        <v>27.20815517124912</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N79" t="n">
-        <v>1.832460732984293</v>
+        <v>0</v>
       </c>
       <c r="P79" t="n">
         <v>19.64044075004835</v>
       </c>
       <c r="Q79" t="n">
-        <v>16.5</v>
+        <v>15.9</v>
       </c>
       <c r="R79" t="n">
         <v>3</v>
@@ -6187,10 +6181,10 @@
         <v>1910000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2619400</v>
+        <v>2618776</v>
       </c>
       <c r="L80" t="n">
-        <v>27.08253798579827</v>
+        <v>27.0651632671141</v>
       </c>
       <c r="M80" s="3" t="n">
         <v>0</v>
@@ -6251,22 +6245,22 @@
         <v>2020000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2748245</v>
+        <v>2747589</v>
       </c>
       <c r="L81" t="n">
-        <v>26.49854725470255</v>
+        <v>26.48099843171595</v>
       </c>
       <c r="M81" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N81" t="n">
-        <v>1.415324548560273</v>
+        <v>0</v>
       </c>
       <c r="P81" t="n">
         <v>36.26522327469554</v>
       </c>
       <c r="Q81" t="n">
-        <v>19.6</v>
+        <v>19.1</v>
       </c>
       <c r="R81" t="n">
         <v>3</v>
@@ -6315,10 +6309,10 @@
         <v>2110000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>2877089</v>
+        <v>2876403</v>
       </c>
       <c r="L82" t="n">
-        <v>26.66198369254479</v>
+        <v>26.64449313952182</v>
       </c>
       <c r="M82" s="3" t="n">
         <v>0</v>
@@ -6379,22 +6373,22 @@
         <v>2210000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3005933</v>
+        <v>3005216</v>
       </c>
       <c r="L83" t="n">
-        <v>26.47873389060901</v>
+        <v>26.46119280610778</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N83" t="n">
-        <v>1.29522108083966</v>
+        <v>0</v>
       </c>
       <c r="P83" t="n">
         <v>70.36535859269283</v>
       </c>
       <c r="Q83" t="n">
-        <v>26.9</v>
+        <v>26.4</v>
       </c>
       <c r="R83" t="n">
         <v>3</v>
@@ -6443,10 +6437,10 @@
         <v>2215000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3048881</v>
+        <v>3048154</v>
       </c>
       <c r="L84" t="n">
-        <v>27.35039511217394</v>
+        <v>27.33306781743967</v>
       </c>
       <c r="M84" s="3" t="n">
         <v>0</v>
@@ -6507,22 +6501,22 @@
         <v>2315000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3177725</v>
+        <v>3176967</v>
       </c>
       <c r="L85" t="n">
-        <v>27.14913971473302</v>
+        <v>27.13175805729175</v>
       </c>
       <c r="M85" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N85" t="n">
-        <v>1.405451448040886</v>
+        <v>0</v>
       </c>
       <c r="P85" t="n">
         <v>65.11105977094954</v>
       </c>
       <c r="Q85" t="n">
-        <v>26.1</v>
+        <v>25.6</v>
       </c>
       <c r="R85" t="n">
         <v>3</v>
@@ -6571,10 +6565,10 @@
         <v>2395000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3306569</v>
+        <v>3305780</v>
       </c>
       <c r="L86" t="n">
-        <v>27.56842515610592</v>
+        <v>27.55113770426344</v>
       </c>
       <c r="M86" s="3" t="n">
         <v>0</v>
@@ -6635,10 +6629,10 @@
         <v>2410000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3306569</v>
+        <v>3305780</v>
       </c>
       <c r="L87" t="n">
-        <v>27.11478272493331</v>
+        <v>27.09738700094985</v>
       </c>
       <c r="M87" s="3" t="n">
         <v>0</v>
@@ -6699,22 +6693,22 @@
         <v>2499000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3435413</v>
+        <v>3434594</v>
       </c>
       <c r="L88" t="n">
-        <v>27.25765431987362</v>
+        <v>27.24030846149501</v>
       </c>
       <c r="M88" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N88" t="n">
-        <v>1.614173228346457</v>
+        <v>0</v>
       </c>
       <c r="P88" t="n">
         <v>63.67326854471646</v>
       </c>
       <c r="Q88" t="n">
-        <v>25.9</v>
+        <v>25.3</v>
       </c>
       <c r="R88" t="n">
         <v>3</v>
@@ -6763,22 +6757,22 @@
         <v>2510000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3435413</v>
+        <v>3434594</v>
       </c>
       <c r="L89" t="n">
-        <v>26.93745992112157</v>
+        <v>26.92003771042516</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N89" t="n">
-        <v>1.200551072623499</v>
+        <v>0</v>
       </c>
       <c r="P89" t="n">
         <v>83.17546233649077</v>
       </c>
       <c r="Q89" t="n">
-        <v>29.8</v>
+        <v>29.4</v>
       </c>
       <c r="R89" t="n">
         <v>3</v>
@@ -6827,10 +6821,10 @@
         <v>2530000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3478361</v>
+        <v>3477532</v>
       </c>
       <c r="L90" t="n">
-        <v>27.26459387050395</v>
+        <v>27.24725466221447</v>
       </c>
       <c r="M90" s="3" t="n">
         <v>0</v>
@@ -6842,7 +6836,7 @@
         <v>79.17877203176447</v>
       </c>
       <c r="Q90" t="n">
-        <v>28.7</v>
+        <v>28.6</v>
       </c>
       <c r="R90" t="n">
         <v>3</v>
@@ -6891,22 +6885,22 @@
         <v>2610000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>3607205</v>
+        <v>3606345</v>
       </c>
       <c r="L91" t="n">
-        <v>27.64481087157508</v>
+        <v>27.62755643178897</v>
       </c>
       <c r="M91" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N91" t="n">
-        <v>1.023890784982935</v>
+        <v>0</v>
       </c>
       <c r="P91" t="n">
         <v>74.15426251691474</v>
       </c>
       <c r="Q91" t="n">
-        <v>28.1</v>
+        <v>27.7</v>
       </c>
       <c r="R91" t="n">
         <v>3</v>
@@ -6955,10 +6949,10 @@
         <v>3015000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4165530</v>
+        <v>4164536</v>
       </c>
       <c r="L92" t="n">
-        <v>27.62025480551094</v>
+        <v>27.6029790593718</v>
       </c>
       <c r="M92" s="3" t="n">
         <v>0</v>
@@ -7019,22 +7013,22 @@
         <v>3098000</v>
       </c>
       <c r="K93" s="3" t="n">
-        <v>4294374</v>
+        <v>4293350</v>
       </c>
       <c r="L93" t="n">
-        <v>27.85910123338116</v>
+        <v>27.84189502369944</v>
       </c>
       <c r="M93" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N93" t="n">
-        <v>1.400381922342457</v>
+        <v>0</v>
       </c>
       <c r="P93" t="n">
         <v>100</v>
       </c>
       <c r="Q93" t="n">
-        <v>33.9</v>
+        <v>33.4</v>
       </c>
       <c r="R93" t="n">
         <v>3</v>
@@ -7318,10 +7312,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>429051</v>
+        <v>428949</v>
       </c>
       <c r="L2" t="n">
-        <v>27.74775026745072</v>
+        <v>27.73056936838645</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7385,10 +7379,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>429051</v>
+        <v>428949</v>
       </c>
       <c r="L3" t="n">
-        <v>27.74775026745072</v>
+        <v>27.73056936838645</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7452,10 +7446,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>429051</v>
+        <v>428949</v>
       </c>
       <c r="L4" t="n">
-        <v>27.74751719492555</v>
+        <v>27.73033624043884</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7519,10 +7513,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>429051</v>
+        <v>428949</v>
       </c>
       <c r="L5" t="n">
-        <v>27.74751719492555</v>
+        <v>27.73033624043884</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7586,10 +7580,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514947</v>
+        <v>514824</v>
       </c>
       <c r="L6" t="n">
-        <v>25.42921892932671</v>
+        <v>25.41140273180737</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7650,10 +7644,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>514947</v>
+        <v>514824</v>
       </c>
       <c r="L7" t="n">
-        <v>25.42921892932671</v>
+        <v>25.41140273180737</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7714,10 +7708,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>514947</v>
+        <v>514824</v>
       </c>
       <c r="L8" t="n">
-        <v>25.42921892932671</v>
+        <v>25.41140273180737</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7778,10 +7772,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>514947</v>
+        <v>514824</v>
       </c>
       <c r="L9" t="n">
-        <v>25.42921892932671</v>
+        <v>25.41140273180737</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7842,10 +7836,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>514947</v>
+        <v>514824</v>
       </c>
       <c r="L10" t="n">
-        <v>25.23502418695516</v>
+        <v>25.21716159308812</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7906,10 +7900,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>514947</v>
+        <v>514824</v>
       </c>
       <c r="L11" t="n">
-        <v>25.23502418695516</v>
+        <v>25.21716159308812</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7970,10 +7964,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>514947</v>
+        <v>514824</v>
       </c>
       <c r="L12" t="n">
-        <v>25.23502418695516</v>
+        <v>25.21716159308812</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -8034,10 +8028,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>514947</v>
+        <v>514824</v>
       </c>
       <c r="L13" t="n">
-        <v>25.23502418695516</v>
+        <v>25.21716159308812</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -8098,10 +8092,10 @@
         <v>415000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>557895</v>
+        <v>557762</v>
       </c>
       <c r="L14" t="n">
-        <v>25.61324263526291</v>
+        <v>25.59550489276788</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -8165,10 +8159,10 @@
         <v>415000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>557895</v>
+        <v>557762</v>
       </c>
       <c r="L15" t="n">
-        <v>25.61324263526291</v>
+        <v>25.59550489276788</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0</v>
@@ -8232,10 +8226,10 @@
         <v>415000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>557895</v>
+        <v>557762</v>
       </c>
       <c r="L16" t="n">
-        <v>25.61324263526291</v>
+        <v>25.59550489276788</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -8299,10 +8293,10 @@
         <v>420000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>557895</v>
+        <v>557762</v>
       </c>
       <c r="L17" t="n">
-        <v>24.71701664291668</v>
+        <v>24.69906519268075</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -8366,10 +8360,10 @@
         <v>454000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>600843</v>
+        <v>600700</v>
       </c>
       <c r="L18" t="n">
-        <v>24.43949584167578</v>
+        <v>24.42150824038622</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -8430,10 +8424,10 @@
         <v>454000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>600843</v>
+        <v>600700</v>
       </c>
       <c r="L19" t="n">
-        <v>24.43949584167578</v>
+        <v>24.42150824038622</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -8494,10 +8488,10 @@
         <v>454000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>600843</v>
+        <v>600700</v>
       </c>
       <c r="L20" t="n">
-        <v>24.43949584167578</v>
+        <v>24.42150824038622</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -8558,10 +8552,10 @@
         <v>454000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>600843</v>
+        <v>600700</v>
       </c>
       <c r="L21" t="n">
-        <v>24.43949584167578</v>
+        <v>24.42150824038622</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -8622,10 +8616,10 @@
         <v>455000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>600843</v>
+        <v>600700</v>
       </c>
       <c r="L22" t="n">
-        <v>24.27306301313321</v>
+        <v>24.25503579157649</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -8686,10 +8680,10 @@
         <v>455000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>600843</v>
+        <v>600700</v>
       </c>
       <c r="L23" t="n">
-        <v>24.27306301313321</v>
+        <v>24.25503579157649</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -8750,10 +8744,10 @@
         <v>455000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>600843</v>
+        <v>600700</v>
       </c>
       <c r="L24" t="n">
-        <v>24.27306301313321</v>
+        <v>24.25503579157649</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -8814,10 +8808,10 @@
         <v>455000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>600843</v>
+        <v>600700</v>
       </c>
       <c r="L25" t="n">
-        <v>24.27306301313321</v>
+        <v>24.25503579157649</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -8878,10 +8872,10 @@
         <v>468000</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>686739</v>
+        <v>686575</v>
       </c>
       <c r="L26" t="n">
-        <v>31.85183890823151</v>
+        <v>31.83556057240651</v>
       </c>
       <c r="M26" s="3" t="n">
         <v>0</v>
@@ -8942,10 +8936,10 @@
         <v>468000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>686739</v>
+        <v>686575</v>
       </c>
       <c r="L27" t="n">
-        <v>31.85183890823151</v>
+        <v>31.83556057240651</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -9006,10 +9000,10 @@
         <v>468000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>686739</v>
+        <v>686575</v>
       </c>
       <c r="L28" t="n">
-        <v>31.85183890823151</v>
+        <v>31.83556057240651</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -9070,10 +9064,10 @@
         <v>468000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>686739</v>
+        <v>686575</v>
       </c>
       <c r="L29" t="n">
-        <v>31.85183890823151</v>
+        <v>31.83556057240651</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -9134,10 +9128,10 @@
         <v>475000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>686739</v>
+        <v>686575</v>
       </c>
       <c r="L30" t="n">
-        <v>30.83252880643155</v>
+        <v>30.81600699122456</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -9198,10 +9192,10 @@
         <v>475000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>686739</v>
+        <v>686575</v>
       </c>
       <c r="L31" t="n">
-        <v>30.83252880643155</v>
+        <v>30.81600699122456</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -9262,10 +9256,10 @@
         <v>475000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>686739</v>
+        <v>686575</v>
       </c>
       <c r="L32" t="n">
-        <v>30.83252880643155</v>
+        <v>30.81600699122456</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -9326,10 +9320,10 @@
         <v>475000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>686739</v>
+        <v>686575</v>
       </c>
       <c r="L33" t="n">
-        <v>30.83252880643155</v>
+        <v>30.81600699122456</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -9390,10 +9384,10 @@
         <v>477000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>643791</v>
+        <v>643637</v>
       </c>
       <c r="L34" t="n">
-        <v>25.90763151395406</v>
+        <v>25.88990378116858</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -9457,10 +9451,10 @@
         <v>477000</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>643791</v>
+        <v>643637</v>
       </c>
       <c r="L35" t="n">
-        <v>25.90763151395406</v>
+        <v>25.88990378116858</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
@@ -9524,10 +9518,10 @@
         <v>477000</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>643791</v>
+        <v>643637</v>
       </c>
       <c r="L36" t="n">
-        <v>25.90763151395406</v>
+        <v>25.88990378116858</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -9591,10 +9585,10 @@
         <v>479999</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>643791</v>
+        <v>643637</v>
       </c>
       <c r="L37" t="n">
-        <v>25.44179710496108</v>
+        <v>25.42395791416591</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
@@ -9658,10 +9652,10 @@
         <v>500000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>643791</v>
+        <v>643637</v>
       </c>
       <c r="L38" t="n">
-        <v>22.33504351567512</v>
+        <v>22.31646098654987</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -9722,10 +9716,10 @@
         <v>544999</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>772635</v>
+        <v>772451</v>
       </c>
       <c r="L39" t="n">
-        <v>29.46229461518052</v>
+        <v>29.44549233543616</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -9786,10 +9780,10 @@
         <v>544999</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>772635</v>
+        <v>772451</v>
       </c>
       <c r="L40" t="n">
-        <v>29.46229461518052</v>
+        <v>29.44549233543616</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -9850,10 +9844,10 @@
         <v>544999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>772635</v>
+        <v>772451</v>
       </c>
       <c r="L41" t="n">
-        <v>29.46229461518052</v>
+        <v>29.44549233543616</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
@@ -9914,10 +9908,10 @@
         <v>544999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>772635</v>
+        <v>772451</v>
       </c>
       <c r="L42" t="n">
-        <v>29.46229461518052</v>
+        <v>29.44549233543616</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -9978,10 +9972,10 @@
         <v>549999</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>772635</v>
+        <v>772451</v>
       </c>
       <c r="L43" t="n">
-        <v>28.8151585159875</v>
+        <v>28.79820208660485</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -9993,7 +9987,7 @@
         <v>35.29417147279201</v>
       </c>
       <c r="Q43" t="n">
-        <v>20.6</v>
+        <v>20.5</v>
       </c>
       <c r="R43" t="n">
         <v>3</v>
@@ -10042,10 +10036,10 @@
         <v>549999</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>772635</v>
+        <v>772451</v>
       </c>
       <c r="L44" t="n">
-        <v>28.8151585159875</v>
+        <v>28.79820208660485</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -10057,7 +10051,7 @@
         <v>35.29417147279201</v>
       </c>
       <c r="Q44" t="n">
-        <v>20.6</v>
+        <v>20.5</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -10106,10 +10100,10 @@
         <v>549999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>772635</v>
+        <v>772451</v>
       </c>
       <c r="L45" t="n">
-        <v>28.8151585159875</v>
+        <v>28.79820208660485</v>
       </c>
       <c r="M45" s="3" t="n">
         <v>0</v>
@@ -10121,7 +10115,7 @@
         <v>35.29417147279201</v>
       </c>
       <c r="Q45" t="n">
-        <v>20.6</v>
+        <v>20.5</v>
       </c>
       <c r="R45" t="n">
         <v>3</v>
@@ -10170,10 +10164,10 @@
         <v>549999</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>772635</v>
+        <v>772451</v>
       </c>
       <c r="L46" t="n">
-        <v>28.8151585159875</v>
+        <v>28.79820208660485</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -10185,7 +10179,7 @@
         <v>35.29417147279201</v>
       </c>
       <c r="Q46" t="n">
-        <v>20.6</v>
+        <v>20.5</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -10234,10 +10228,10 @@
         <v>585000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>729687</v>
+        <v>729513</v>
       </c>
       <c r="L47" t="n">
-        <v>19.82863885474183</v>
+        <v>19.809516759811</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -10298,10 +10292,10 @@
         <v>595000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>729687</v>
+        <v>729513</v>
       </c>
       <c r="L48" t="n">
-        <v>18.45818823687417</v>
+        <v>18.43873926852572</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -10362,10 +10356,10 @@
         <v>619999</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>858531</v>
+        <v>858326</v>
       </c>
       <c r="L49" t="n">
-        <v>27.78373757033817</v>
+        <v>27.7664896554456</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -10426,10 +10420,10 @@
         <v>619999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>858531</v>
+        <v>858326</v>
       </c>
       <c r="L50" t="n">
-        <v>27.78373757033817</v>
+        <v>27.7664896554456</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -10490,10 +10484,10 @@
         <v>619999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>858531</v>
+        <v>858326</v>
       </c>
       <c r="L51" t="n">
-        <v>27.78373757033817</v>
+        <v>27.7664896554456</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -10554,10 +10548,10 @@
         <v>619999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>858531</v>
+        <v>858326</v>
       </c>
       <c r="L52" t="n">
-        <v>27.78373757033817</v>
+        <v>27.7664896554456</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -10618,10 +10612,10 @@
         <v>650000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>815583</v>
+        <v>815389</v>
       </c>
       <c r="L53" t="n">
-        <v>20.30240944208008</v>
+        <v>20.28344753240478</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -10682,10 +10676,10 @@
         <v>672000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>858531</v>
+        <v>858326</v>
       </c>
       <c r="L54" t="n">
-        <v>21.72676350650122</v>
+        <v>21.70806896214259</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -10746,10 +10740,10 @@
         <v>700000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>901479</v>
+        <v>901264</v>
       </c>
       <c r="L55" t="n">
-        <v>22.34982733929465</v>
+        <v>22.33130359140052</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -10810,10 +10804,10 @@
         <v>715000</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>944427</v>
+        <v>944202</v>
       </c>
       <c r="L56" t="n">
-        <v>24.2927192890504</v>
+        <v>24.27467851158968</v>
       </c>
       <c r="M56" s="3" t="n">
         <v>0</v>
@@ -10874,10 +10868,10 @@
         <v>734999</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>987375</v>
+        <v>987140</v>
       </c>
       <c r="L57" t="n">
-        <v>25.56029877199645</v>
+        <v>25.54257754725773</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -10938,10 +10932,10 @@
         <v>752000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>987375</v>
+        <v>987140</v>
       </c>
       <c r="L58" t="n">
-        <v>23.83846056462843</v>
+        <v>23.82032943655409</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -11002,10 +10996,10 @@
         <v>810000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1073271</v>
+        <v>1073015</v>
       </c>
       <c r="L59" t="n">
-        <v>24.52977859273194</v>
+        <v>24.51177290159038</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -11066,10 +11060,10 @@
         <v>815000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1073271</v>
+        <v>1073015</v>
       </c>
       <c r="L60" t="n">
-        <v>24.06391302848954</v>
+        <v>24.04579619110637</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -11130,10 +11124,10 @@
         <v>875000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1159167</v>
+        <v>1158891</v>
       </c>
       <c r="L61" t="n">
-        <v>24.5147593056048</v>
+        <v>24.49678183711842</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -11194,10 +11188,10 @@
         <v>992000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1330959</v>
+        <v>1330642</v>
       </c>
       <c r="L62" t="n">
-        <v>25.46727585147251</v>
+        <v>25.44951985582899</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -11258,10 +11252,10 @@
         <v>1050000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1416856</v>
+        <v>1416518</v>
       </c>
       <c r="L63" t="n">
-        <v>25.89225722303467</v>
+        <v>25.87457413177948</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -11322,10 +11316,10 @@
         <v>1050000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1416856</v>
+        <v>1416518</v>
       </c>
       <c r="L64" t="n">
-        <v>25.89225722303467</v>
+        <v>25.87457413177948</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -11386,10 +11380,10 @@
         <v>1100000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1502752</v>
+        <v>1502393</v>
       </c>
       <c r="L65" t="n">
-        <v>26.80096250079854</v>
+        <v>26.78347143523698</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -11401,7 +11395,7 @@
         <v>94.11761630126171</v>
       </c>
       <c r="Q65" t="n">
-        <v>31.7</v>
+        <v>31.6</v>
       </c>
       <c r="R65" t="n">
         <v>3</v>
@@ -11450,10 +11444,10 @@
         <v>1105000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1502752</v>
+        <v>1502393</v>
       </c>
       <c r="L66" t="n">
-        <v>26.4682396030749</v>
+        <v>26.45066903266988</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -11514,10 +11508,10 @@
         <v>1155000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1588648</v>
+        <v>1588269</v>
       </c>
       <c r="L67" t="n">
-        <v>27.29666987274714</v>
+        <v>27.27932107218614</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -11784,7 +11778,7 @@
         <v>315000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>300207</v>
+        <v>300135</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -11845,10 +11839,10 @@
         <v>380000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>386103</v>
+        <v>386011</v>
       </c>
       <c r="L3" t="n">
-        <v>1.580666298889156</v>
+        <v>1.557209509573561</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -11909,7 +11903,7 @@
         <v>415000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>386103</v>
+        <v>386011</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -11970,10 +11964,10 @@
         <v>495000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>471999</v>
+        <v>471886</v>
       </c>
       <c r="L5" t="n">
-        <v>6.779675380668179</v>
+        <v>6.757352411387496</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -12034,10 +12028,10 @@
         <v>490000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514947</v>
+        <v>514824</v>
       </c>
       <c r="L6" t="n">
-        <v>4.844576237942934</v>
+        <v>4.821842027566702</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -12098,10 +12092,10 @@
         <v>550000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>557895</v>
+        <v>557762</v>
       </c>
       <c r="L7" t="n">
-        <v>6.792496795992077</v>
+        <v>6.770271190938071</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -12162,7 +12156,7 @@
         <v>530000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>471999</v>
+        <v>471886</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -12226,10 +12220,10 @@
         <v>600000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>600843</v>
+        <v>600700</v>
       </c>
       <c r="L9" t="n">
-        <v>8.4619443015896</v>
+        <v>8.440153154652904</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -12290,10 +12284,10 @@
         <v>646000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>729687</v>
+        <v>729513</v>
       </c>
       <c r="L10" t="n">
-        <v>17.08787466406829</v>
+        <v>17.06809885498956</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -12305,7 +12299,7 @@
         <v>100</v>
       </c>
       <c r="Q10" t="n">
-        <v>26</v>
+        <v>25.9</v>
       </c>
       <c r="R10" t="n">
         <v>4</v>
@@ -12354,7 +12348,7 @@
         <v>615000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>557895</v>
+        <v>557762</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -12418,7 +12412,7 @@
         <v>700000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>643791</v>
+        <v>643637</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -12482,7 +12476,7 @@
         <v>745000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>686739</v>
+        <v>686575</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -12546,7 +12540,7 @@
         <v>930000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>858531</v>
+        <v>858326</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -12617,7 +12611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12666,78 +12660,30 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 MJ3E4 10 Core CPU 10 Core GPU 32GB 1TB Silver</t>
+          <t>Apple MacBook Pro 14Inch MX2H3 M4 Pro 12Core CPU 16Core GPU 24GB 512GB Space Black</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>769999</v>
+        <v>600000</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>759999</v>
+        <v>634000</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-10000</v>
+        <v>34000</v>
       </c>
       <c r="F2" t="n">
-        <v>-1.3</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 M5 MJ3D4 10 Core CPU 10 Core GPU 32GB 1TB Space Black</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>769999</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>759999</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>-10000</v>
-      </c>
-      <c r="F3" t="n">
-        <v>-1.3</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Macbook Pro 14 M5 MDE54 10 Core CPU 10 Core GPU 16GB 1TB Silver</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>587999</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>584999</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>-3000</v>
-      </c>
-      <c r="F4" t="n">
-        <v>-0.51</v>
+        <v>5.67</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F4"/>
-  <conditionalFormatting sqref="E2:E4">
+  <autoFilter ref="A1:F2"/>
+  <conditionalFormatting sqref="E2">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
chore: price data 2026-10-10
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MacBook Pro'!$A$1:$S$93</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MacBook Air'!$A$1:$S$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20261009T103947329100+0000</t>
+          <t>20261010T095542822990+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-09T10:39:47.329100+00:00</t>
+          <t>2026-10-10T09:55:42.822990+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>277.018</v>
+        <v>276.883168</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -1147,10 +1147,10 @@
         <v>470000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>686575</v>
+        <v>686241</v>
       </c>
       <c r="L2" t="n">
-        <v>35.18552233914722</v>
+        <v>35.15397651845343</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1165,7 +1165,7 @@
         <v>28.4414106939704</v>
       </c>
       <c r="Q2" t="n">
-        <v>35.4</v>
+        <v>35.3</v>
       </c>
       <c r="R2" t="n">
         <v>5</v>
@@ -1214,10 +1214,10 @@
         <v>495000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>686575</v>
+        <v>686241</v>
       </c>
       <c r="L3" t="n">
-        <v>27.90299675927612</v>
+        <v>27.86790646434708</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>772451</v>
+        <v>772075</v>
       </c>
       <c r="L4" t="n">
-        <v>35.27110457491802</v>
+        <v>35.23958164686074</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>772451</v>
+        <v>772075</v>
       </c>
       <c r="L5" t="n">
-        <v>32.68194357959275</v>
+        <v>32.64915973189133</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>858326</v>
+        <v>857909</v>
       </c>
       <c r="L6" t="n">
-        <v>38.01888792836288</v>
+        <v>37.98876104575194</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1606,10 +1606,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>858326</v>
+        <v>857909</v>
       </c>
       <c r="L9" t="n">
-        <v>34.17419488632525</v>
+        <v>34.14219923092076</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1673,10 +1673,10 @@
         <v>578999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>858326</v>
+        <v>857909</v>
       </c>
       <c r="L10" t="n">
-        <v>32.54322949555297</v>
+        <v>32.51044108407768</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -1740,10 +1740,10 @@
         <v>584999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>858326</v>
+        <v>857909</v>
       </c>
       <c r="L11" t="n">
-        <v>31.84419439700067</v>
+        <v>31.81106620865383</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -1807,10 +1807,10 @@
         <v>634000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>858326</v>
+        <v>857909</v>
       </c>
       <c r="L12" t="n">
-        <v>26.13529125297381</v>
+        <v>26.09938816354648</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -1871,13 +1871,13 @@
         <v>634000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>858326</v>
+        <v>857909</v>
       </c>
       <c r="L13" t="n">
-        <v>26.13529125297381</v>
+        <v>26.09938816354648</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>34000</v>
+        <v>0</v>
       </c>
       <c r="N13" t="n">
         <v>0</v>
@@ -1935,10 +1935,10 @@
         <v>642999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>944202</v>
+        <v>943742</v>
       </c>
       <c r="L14" t="n">
-        <v>31.90027134024287</v>
+        <v>31.86707807854265</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -2061,10 +2061,10 @@
         <v>650000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>944202</v>
+        <v>943742</v>
       </c>
       <c r="L16" t="n">
-        <v>31.15879864689971</v>
+        <v>31.12524397557807</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -2128,10 +2128,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1030078</v>
+        <v>1029576</v>
       </c>
       <c r="L17" t="n">
-        <v>32.04398113540916</v>
+        <v>32.01084718369503</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2195,10 +2195,10 @@
         <v>711999</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>1073015</v>
+        <v>1072493</v>
       </c>
       <c r="L18" t="n">
-        <v>33.64500962241907</v>
+        <v>33.61271355617239</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -2324,10 +2324,10 @@
         <v>720000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>1030078</v>
+        <v>1029576</v>
       </c>
       <c r="L20" t="n">
-        <v>30.10238059642085</v>
+        <v>30.06829996037204</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -2453,10 +2453,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1073015</v>
+        <v>1072493</v>
       </c>
       <c r="L22" t="n">
-        <v>30.75586082207612</v>
+        <v>30.72215855954304</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2471,7 +2471,7 @@
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>10.3</v>
+        <v>10.2</v>
       </c>
       <c r="R22" t="n">
         <v>4</v>
@@ -2520,10 +2520,10 @@
         <v>759999</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1030078</v>
+        <v>1029576</v>
       </c>
       <c r="L23" t="n">
-        <v>26.21927659847119</v>
+        <v>26.1833026410872</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -2587,10 +2587,10 @@
         <v>759999</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1030078</v>
+        <v>1029576</v>
       </c>
       <c r="L24" t="n">
-        <v>26.21927659847119</v>
+        <v>26.1833026410872</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -2654,10 +2654,10 @@
         <v>772000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>1030078</v>
+        <v>1029576</v>
       </c>
       <c r="L25" t="n">
-        <v>25.05421919505125</v>
+        <v>25.01767717973224</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -2672,7 +2672,7 @@
         <v>69.59999999999998</v>
       </c>
       <c r="Q25" t="n">
-        <v>20</v>
+        <v>19.9</v>
       </c>
       <c r="R25" t="n">
         <v>4</v>
@@ -2845,10 +2845,10 @@
         <v>810000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>1073015</v>
+        <v>1072493</v>
       </c>
       <c r="L28" t="n">
-        <v>24.51177290159038</v>
+        <v>24.47503153866738</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -2860,7 +2860,7 @@
         <v>61.99999999999999</v>
       </c>
       <c r="Q28" t="n">
-        <v>24.7</v>
+        <v>24.6</v>
       </c>
       <c r="R28" t="n">
         <v>3</v>
@@ -2909,10 +2909,10 @@
         <v>810000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>1244767</v>
+        <v>1244161</v>
       </c>
       <c r="L29" t="n">
-        <v>34.92758082436311</v>
+        <v>34.89588566110013</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -2941,7 +2941,7 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 MGE44 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Silver</t>
+          <t>Macbook Pro 16 MGEA4 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -2966,38 +2966,35 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I30" s="3" t="n">
-        <v>822999</v>
+        <v>820000</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>822999</v>
+        <v>820000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1287704</v>
+        <v>1287078</v>
       </c>
       <c r="L30" t="n">
-        <v>36.08787423196635</v>
+        <v>36.2897975103296</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>0</v>
+        <v>-3000</v>
       </c>
       <c r="N30" t="n">
-        <v>0.8433745100897712</v>
-      </c>
-      <c r="O30" t="n">
-        <v>100</v>
+        <v>0.6060606060606061</v>
       </c>
       <c r="P30" t="n">
-        <v>0.0003521901827191575</v>
+        <v>0</v>
       </c>
       <c r="Q30" t="n">
-        <v>34.5</v>
+        <v>15.8</v>
       </c>
       <c r="R30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S30" t="inlineStr">
         <is>
@@ -3008,7 +3005,7 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 MGEA4 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Space Black</t>
+          <t>Macbook Pro 16 MGE44 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Silver</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -3033,38 +3030,35 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I31" s="3" t="n">
-        <v>823000</v>
+        <v>820000</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>823000</v>
+        <v>820000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1287704</v>
+        <v>1287078</v>
       </c>
       <c r="L31" t="n">
-        <v>36.08779657436803</v>
+        <v>36.2897975103296</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>0</v>
+        <v>-2999</v>
       </c>
       <c r="N31" t="n">
-        <v>0.2424242424242424</v>
-      </c>
-      <c r="O31" t="n">
-        <v>0</v>
+        <v>1.204700246626803</v>
       </c>
       <c r="P31" t="n">
         <v>0</v>
       </c>
       <c r="Q31" t="n">
-        <v>12.1</v>
+        <v>16</v>
       </c>
       <c r="R31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S31" t="inlineStr">
         <is>
@@ -3110,10 +3104,10 @@
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1373580</v>
+        <v>1372911</v>
       </c>
       <c r="L32" t="n">
-        <v>38.26358857875042</v>
+        <v>38.23350530369412</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3177,10 +3171,10 @@
         <v>930000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1373580</v>
+        <v>1372911</v>
       </c>
       <c r="L33" t="n">
-        <v>38.11798366312847</v>
+        <v>38.08782943686808</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3244,10 +3238,10 @@
         <v>860000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>1244767</v>
+        <v>1244161</v>
       </c>
       <c r="L34" t="n">
-        <v>30.91076482586701</v>
+        <v>30.87711317104458</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -3373,10 +3367,10 @@
         <v>880000</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>1158891</v>
+        <v>1158327</v>
       </c>
       <c r="L36" t="n">
-        <v>24.06533487618767</v>
+        <v>24.02836159391951</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -3437,10 +3431,10 @@
         <v>940000</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>1244767</v>
+        <v>1244161</v>
       </c>
       <c r="L37" t="n">
-        <v>24.48385922827324</v>
+        <v>24.44707718695571</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
@@ -3625,10 +3619,10 @@
         <v>990000</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>1502393</v>
+        <v>1501662</v>
       </c>
       <c r="L40" t="n">
-        <v>34.10512429171328</v>
+        <v>34.07304706385325</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -3754,10 +3748,10 @@
         <v>1000000</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>1502393</v>
+        <v>1501662</v>
       </c>
       <c r="L42" t="n">
-        <v>33.43951948657908</v>
+        <v>33.40711824631641</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -3821,10 +3815,10 @@
         <v>1054000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1545331</v>
+        <v>1544579</v>
       </c>
       <c r="L43" t="n">
-        <v>31.79454757589151</v>
+        <v>31.76134079253958</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -3833,10 +3827,10 @@
         <v>0.09478672985781991</v>
       </c>
       <c r="P43" t="n">
-        <v>57.84723750825446</v>
+        <v>57.39710789766407</v>
       </c>
       <c r="Q43" t="n">
-        <v>26.1</v>
+        <v>25.9</v>
       </c>
       <c r="R43" t="n">
         <v>3</v>
@@ -3885,10 +3879,10 @@
         <v>1054000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1545331</v>
+        <v>1544579</v>
       </c>
       <c r="L44" t="n">
-        <v>31.79454757589151</v>
+        <v>31.76134079253958</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -3897,10 +3891,10 @@
         <v>0.09478672985781991</v>
       </c>
       <c r="P44" t="n">
-        <v>57.84723750825446</v>
+        <v>57.39710789766407</v>
       </c>
       <c r="Q44" t="n">
-        <v>26.1</v>
+        <v>25.9</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -4011,10 +4005,10 @@
         <v>1115000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1502393</v>
+        <v>1501662</v>
       </c>
       <c r="L46" t="n">
-        <v>25.78506422753567</v>
+        <v>25.7489368446428</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -4023,10 +4017,10 @@
         <v>0</v>
       </c>
       <c r="P46" t="n">
-        <v>9.358196283135744</v>
+        <v>8.390274908628628</v>
       </c>
       <c r="Q46" t="n">
-        <v>13.1</v>
+        <v>12.8</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -4075,10 +4069,10 @@
         <v>1123000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1717082</v>
+        <v>1716246</v>
       </c>
       <c r="L47" t="n">
-        <v>34.59834766190549</v>
+        <v>34.56648988548262</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -4142,10 +4136,10 @@
         <v>1130000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1502393</v>
+        <v>1501662</v>
       </c>
       <c r="L48" t="n">
-        <v>24.78665701983436</v>
+        <v>24.75004361833755</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -4268,10 +4262,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1760020</v>
+        <v>1759163</v>
       </c>
       <c r="L50" t="n">
-        <v>34.37574573016215</v>
+        <v>34.343775988922</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4283,7 +4277,7 @@
         <v>22.53136001640632</v>
       </c>
       <c r="Q50" t="n">
-        <v>19.6</v>
+        <v>19.5</v>
       </c>
       <c r="R50" t="n">
         <v>3</v>
@@ -4332,10 +4326,10 @@
         <v>1155000</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>1760020</v>
+        <v>1759163</v>
       </c>
       <c r="L51" t="n">
-        <v>34.37574573016215</v>
+        <v>34.343775988922</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -4347,7 +4341,7 @@
         <v>22.53136001640632</v>
       </c>
       <c r="Q51" t="n">
-        <v>19.6</v>
+        <v>19.5</v>
       </c>
       <c r="R51" t="n">
         <v>3</v>
@@ -4396,10 +4390,10 @@
         <v>1185000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1588269</v>
+        <v>1587496</v>
       </c>
       <c r="L52" t="n">
-        <v>25.39047226886629</v>
+        <v>25.35414262461134</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -4460,10 +4454,10 @@
         <v>1185000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1588269</v>
+        <v>1587496</v>
       </c>
       <c r="L53" t="n">
-        <v>25.39047226886629</v>
+        <v>25.35414262461134</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -4524,10 +4518,10 @@
         <v>1200000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1888833</v>
+        <v>1887914</v>
       </c>
       <c r="L54" t="n">
-        <v>36.46870845649139</v>
+        <v>36.43778265323526</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -4588,10 +4582,10 @@
         <v>1200000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1888833</v>
+        <v>1887914</v>
       </c>
       <c r="L55" t="n">
-        <v>36.46870845649139</v>
+        <v>36.43778265323526</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -4714,10 +4708,10 @@
         <v>1240000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1674144</v>
+        <v>1673330</v>
       </c>
       <c r="L57" t="n">
-        <v>25.9322973412084</v>
+        <v>25.89626672563093</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -4840,10 +4834,10 @@
         <v>1280000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1717082</v>
+        <v>1716246</v>
       </c>
       <c r="L59" t="n">
-        <v>25.45492876869014</v>
+        <v>25.41861714462845</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -4907,10 +4901,10 @@
         <v>1298000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1760020</v>
+        <v>1759163</v>
       </c>
       <c r="L60" t="n">
-        <v>26.25083805865843</v>
+        <v>26.21491015897902</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -4919,10 +4913,10 @@
         <v>0</v>
       </c>
       <c r="P60" t="n">
-        <v>61.28109178956637</v>
+        <v>60.86763070077864</v>
       </c>
       <c r="Q60" t="n">
-        <v>24.4</v>
+        <v>24.3</v>
       </c>
       <c r="R60" t="n">
         <v>3</v>
@@ -4971,10 +4965,10 @@
         <v>1300000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1717082</v>
+        <v>1716246</v>
       </c>
       <c r="L61" t="n">
-        <v>24.29016203070092</v>
+        <v>24.25328303751327</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -4983,10 +4977,10 @@
         <v>0</v>
       </c>
       <c r="P61" t="n">
-        <v>60.92890160686771</v>
+        <v>60.51167964404895</v>
       </c>
       <c r="Q61" t="n">
-        <v>23.5</v>
+        <v>23.4</v>
       </c>
       <c r="R61" t="n">
         <v>3</v>
@@ -5097,10 +5091,10 @@
         <v>1335000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1802958</v>
+        <v>1802080</v>
       </c>
       <c r="L63" t="n">
-        <v>25.95501392711311</v>
+        <v>25.9189381159549</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -5161,10 +5155,10 @@
         <v>1420000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1931771</v>
+        <v>1930831</v>
       </c>
       <c r="L64" t="n">
-        <v>26.49232233013126</v>
+        <v>26.45653607177428</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -5173,7 +5167,7 @@
         <v>0</v>
       </c>
       <c r="P64" t="n">
-        <v>81.47332893095606</v>
+        <v>81.27549128661477</v>
       </c>
       <c r="Q64" t="n">
         <v>28.8</v>
@@ -5225,10 +5219,10 @@
         <v>1430000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1931771</v>
+        <v>1930831</v>
       </c>
       <c r="L65" t="n">
-        <v>25.97466262823078</v>
+        <v>25.93862435396987</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -5237,10 +5231,10 @@
         <v>0</v>
       </c>
       <c r="P65" t="n">
-        <v>60.92890160686771</v>
+        <v>60.51167964404895</v>
       </c>
       <c r="Q65" t="n">
-        <v>24.2</v>
+        <v>24.1</v>
       </c>
       <c r="R65" t="n">
         <v>3</v>
@@ -5289,10 +5283,10 @@
         <v>1430000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>2146460</v>
+        <v>2145415</v>
       </c>
       <c r="L66" t="n">
-        <v>33.37867931384699</v>
+        <v>33.34622905125582</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -5353,10 +5347,10 @@
         <v>1430000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>2146460</v>
+        <v>2145415</v>
       </c>
       <c r="L67" t="n">
-        <v>33.37867931384699</v>
+        <v>33.34622905125582</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -5479,10 +5473,10 @@
         <v>1480000</v>
       </c>
       <c r="K69" s="3" t="n">
-        <v>2017647</v>
+        <v>2016665</v>
       </c>
       <c r="L69" t="n">
-        <v>26.64722818213493</v>
+        <v>26.61150959628892</v>
       </c>
       <c r="M69" s="3" t="n">
         <v>0</v>
@@ -5605,10 +5599,10 @@
         <v>1605000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2189398</v>
+        <v>2188332</v>
       </c>
       <c r="L71" t="n">
-        <v>26.69217748440439</v>
+        <v>26.65646711742094</v>
       </c>
       <c r="M71" s="3" t="n">
         <v>0</v>
@@ -5669,10 +5663,10 @@
         <v>1610000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2189398</v>
+        <v>2188332</v>
       </c>
       <c r="L72" t="n">
-        <v>26.4638042055396</v>
+        <v>26.42798259130699</v>
       </c>
       <c r="M72" s="3" t="n">
         <v>0</v>
@@ -5684,7 +5678,7 @@
         <v>25.72147975982957</v>
       </c>
       <c r="Q72" t="n">
-        <v>16.9</v>
+        <v>16.8</v>
       </c>
       <c r="R72" t="n">
         <v>3</v>
@@ -5733,10 +5727,10 @@
         <v>1615000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2189398</v>
+        <v>2188332</v>
       </c>
       <c r="L73" t="n">
-        <v>26.23543092667482</v>
+        <v>26.19949806519303</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
@@ -5745,7 +5739,7 @@
         <v>0</v>
       </c>
       <c r="P73" t="n">
-        <v>86.7142542687337</v>
+        <v>86.5723820117591</v>
       </c>
       <c r="Q73" t="n">
         <v>29.8</v>
@@ -5797,10 +5791,10 @@
         <v>1630000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2232336</v>
+        <v>2231249</v>
       </c>
       <c r="L74" t="n">
-        <v>26.98231807398169</v>
+        <v>26.9467459705304</v>
       </c>
       <c r="M74" s="3" t="n">
         <v>0</v>
@@ -5861,10 +5855,10 @@
         <v>1690000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2318211</v>
+        <v>2317083</v>
       </c>
       <c r="L75" t="n">
-        <v>27.09895691116986</v>
+        <v>27.06346729918609</v>
       </c>
       <c r="M75" s="3" t="n">
         <v>0</v>
@@ -5925,10 +5919,10 @@
         <v>1705000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2318211</v>
+        <v>2317083</v>
       </c>
       <c r="L76" t="n">
-        <v>26.45190623286664</v>
+        <v>26.41610162432679</v>
       </c>
       <c r="M76" s="3" t="n">
         <v>0</v>
@@ -5940,7 +5934,7 @@
         <v>1.9846639603067</v>
       </c>
       <c r="Q76" t="n">
-        <v>11.8</v>
+        <v>11.7</v>
       </c>
       <c r="R76" t="n">
         <v>3</v>
@@ -5989,10 +5983,10 @@
         <v>1725000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2361149</v>
+        <v>2360000</v>
       </c>
       <c r="L77" t="n">
-        <v>26.94234883101405</v>
+        <v>26.90677966101695</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
@@ -6053,10 +6047,10 @@
         <v>1780000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2447025</v>
+        <v>2445834</v>
       </c>
       <c r="L78" t="n">
-        <v>27.2586099447288</v>
+        <v>27.22318849112409</v>
       </c>
       <c r="M78" s="3" t="n">
         <v>0</v>
@@ -6117,10 +6111,10 @@
         <v>1875000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2575838</v>
+        <v>2574584</v>
       </c>
       <c r="L79" t="n">
-        <v>27.20815517124912</v>
+        <v>27.17270052171535</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
@@ -6181,10 +6175,10 @@
         <v>1910000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2618776</v>
+        <v>2617501</v>
       </c>
       <c r="L80" t="n">
-        <v>27.0651632671141</v>
+        <v>27.02963628285147</v>
       </c>
       <c r="M80" s="3" t="n">
         <v>0</v>
@@ -6245,10 +6239,10 @@
         <v>2020000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2747589</v>
+        <v>2746252</v>
       </c>
       <c r="L81" t="n">
-        <v>26.48099843171595</v>
+        <v>26.44520604809755</v>
       </c>
       <c r="M81" s="3" t="n">
         <v>0</v>
@@ -6309,10 +6303,10 @@
         <v>2110000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>2876403</v>
+        <v>2875003</v>
       </c>
       <c r="L82" t="n">
-        <v>26.64449313952182</v>
+        <v>26.60877223432462</v>
       </c>
       <c r="M82" s="3" t="n">
         <v>0</v>
@@ -6324,7 +6318,7 @@
         <v>79.02382335851249</v>
       </c>
       <c r="Q82" t="n">
-        <v>28.4</v>
+        <v>28.3</v>
       </c>
       <c r="R82" t="n">
         <v>3</v>
@@ -6373,10 +6367,10 @@
         <v>2210000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3005216</v>
+        <v>3003753</v>
       </c>
       <c r="L83" t="n">
-        <v>26.46119280610778</v>
+        <v>26.42537518897193</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
@@ -6437,10 +6431,10 @@
         <v>2215000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3048154</v>
+        <v>3046670</v>
       </c>
       <c r="L84" t="n">
-        <v>27.33306781743967</v>
+        <v>27.29767254083967</v>
       </c>
       <c r="M84" s="3" t="n">
         <v>0</v>
@@ -6501,10 +6495,10 @@
         <v>2315000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3176967</v>
+        <v>3175421</v>
       </c>
       <c r="L85" t="n">
-        <v>27.13175805729175</v>
+        <v>27.0962810915466</v>
       </c>
       <c r="M85" s="3" t="n">
         <v>0</v>
@@ -6565,10 +6559,10 @@
         <v>2395000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3305780</v>
+        <v>3304171</v>
       </c>
       <c r="L86" t="n">
-        <v>27.55113770426344</v>
+        <v>27.51585798676884</v>
       </c>
       <c r="M86" s="3" t="n">
         <v>0</v>
@@ -6629,10 +6623,10 @@
         <v>2410000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3305780</v>
+        <v>3304171</v>
       </c>
       <c r="L87" t="n">
-        <v>27.09738700094985</v>
+        <v>27.06188632489057</v>
       </c>
       <c r="M87" s="3" t="n">
         <v>0</v>
@@ -6693,10 +6687,10 @@
         <v>2499000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3434594</v>
+        <v>3432922</v>
       </c>
       <c r="L88" t="n">
-        <v>27.24030846149501</v>
+        <v>27.20487095250052</v>
       </c>
       <c r="M88" s="3" t="n">
         <v>0</v>
@@ -6757,10 +6751,10 @@
         <v>2510000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3434594</v>
+        <v>3432922</v>
       </c>
       <c r="L89" t="n">
-        <v>26.92003771042516</v>
+        <v>26.88444421399612</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
@@ -6772,7 +6766,7 @@
         <v>83.17546233649077</v>
       </c>
       <c r="Q89" t="n">
-        <v>29.4</v>
+        <v>29.3</v>
       </c>
       <c r="R89" t="n">
         <v>3</v>
@@ -6821,10 +6815,10 @@
         <v>2530000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3477532</v>
+        <v>3475839</v>
       </c>
       <c r="L90" t="n">
-        <v>27.24725466221447</v>
+        <v>27.21181849907317</v>
       </c>
       <c r="M90" s="3" t="n">
         <v>0</v>
@@ -6885,10 +6879,10 @@
         <v>2610000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>3606345</v>
+        <v>3604590</v>
       </c>
       <c r="L91" t="n">
-        <v>27.62755643178897</v>
+        <v>27.59231979226486</v>
       </c>
       <c r="M91" s="3" t="n">
         <v>0</v>
@@ -6949,10 +6943,10 @@
         <v>3015000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4164536</v>
+        <v>4162509</v>
       </c>
       <c r="L92" t="n">
-        <v>27.6029790593718</v>
+        <v>27.56772417789367</v>
       </c>
       <c r="M92" s="3" t="n">
         <v>0</v>
@@ -6964,7 +6958,7 @@
         <v>100</v>
       </c>
       <c r="Q92" t="n">
-        <v>33.3</v>
+        <v>33.2</v>
       </c>
       <c r="R92" t="n">
         <v>3</v>
@@ -7013,10 +7007,10 @@
         <v>3098000</v>
       </c>
       <c r="K93" s="3" t="n">
-        <v>4293350</v>
+        <v>4291260</v>
       </c>
       <c r="L93" t="n">
-        <v>27.84189502369944</v>
+        <v>27.80675139702558</v>
       </c>
       <c r="M93" s="3" t="n">
         <v>0</v>
@@ -7028,7 +7022,7 @@
         <v>100</v>
       </c>
       <c r="Q93" t="n">
-        <v>33.4</v>
+        <v>33.3</v>
       </c>
       <c r="R93" t="n">
         <v>3</v>
@@ -7312,10 +7306,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>428949</v>
+        <v>428740</v>
       </c>
       <c r="L2" t="n">
-        <v>27.73056936838645</v>
+        <v>27.69533983299902</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7379,10 +7373,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>428949</v>
+        <v>428740</v>
       </c>
       <c r="L3" t="n">
-        <v>27.73056936838645</v>
+        <v>27.69533983299902</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7446,10 +7440,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>428949</v>
+        <v>428740</v>
       </c>
       <c r="L4" t="n">
-        <v>27.73033624043884</v>
+        <v>27.69510659140738</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7513,10 +7507,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>428949</v>
+        <v>428740</v>
       </c>
       <c r="L5" t="n">
-        <v>27.73033624043884</v>
+        <v>27.69510659140738</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7580,10 +7574,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514824</v>
+        <v>514574</v>
       </c>
       <c r="L6" t="n">
-        <v>25.41140273180737</v>
+        <v>25.37516469934353</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7644,10 +7638,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>514824</v>
+        <v>514574</v>
       </c>
       <c r="L7" t="n">
-        <v>25.41140273180737</v>
+        <v>25.37516469934353</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7708,10 +7702,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>514824</v>
+        <v>514574</v>
       </c>
       <c r="L8" t="n">
-        <v>25.41140273180737</v>
+        <v>25.37516469934353</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7772,10 +7766,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>514824</v>
+        <v>514574</v>
       </c>
       <c r="L9" t="n">
-        <v>25.41140273180737</v>
+        <v>25.37516469934353</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7836,10 +7830,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>514824</v>
+        <v>514574</v>
       </c>
       <c r="L10" t="n">
-        <v>25.21716159308812</v>
+        <v>25.18082919074808</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7900,10 +7894,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>514824</v>
+        <v>514574</v>
       </c>
       <c r="L11" t="n">
-        <v>25.21716159308812</v>
+        <v>25.18082919074808</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7964,10 +7958,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>514824</v>
+        <v>514574</v>
       </c>
       <c r="L12" t="n">
-        <v>25.21716159308812</v>
+        <v>25.18082919074808</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -8028,10 +8022,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>514824</v>
+        <v>514574</v>
       </c>
       <c r="L13" t="n">
-        <v>25.21716159308812</v>
+        <v>25.18082919074808</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -8092,16 +8086,16 @@
         <v>415000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>557762</v>
+        <v>557490</v>
       </c>
       <c r="L14" t="n">
-        <v>25.59550489276788</v>
+        <v>25.5592028556566</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>2.352941176470588</v>
+        <v>2.007083825265644</v>
       </c>
       <c r="O14" t="n">
         <v>100</v>
@@ -8110,7 +8104,7 @@
         <v>3.478260869565196</v>
       </c>
       <c r="Q14" t="n">
-        <v>32</v>
+        <v>31.9</v>
       </c>
       <c r="R14" t="n">
         <v>4</v>
@@ -8159,16 +8153,16 @@
         <v>415000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>557762</v>
+        <v>557490</v>
       </c>
       <c r="L15" t="n">
-        <v>25.59550489276788</v>
+        <v>25.5592028556566</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>2.352941176470588</v>
+        <v>2.007083825265644</v>
       </c>
       <c r="O15" t="n">
         <v>100</v>
@@ -8177,7 +8171,7 @@
         <v>3.478260869565196</v>
       </c>
       <c r="Q15" t="n">
-        <v>32</v>
+        <v>31.9</v>
       </c>
       <c r="R15" t="n">
         <v>4</v>
@@ -8226,16 +8220,16 @@
         <v>415000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>557762</v>
+        <v>557490</v>
       </c>
       <c r="L16" t="n">
-        <v>25.59550489276788</v>
+        <v>25.5592028556566</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>2.352941176470588</v>
+        <v>2.007083825265644</v>
       </c>
       <c r="O16" t="n">
         <v>100</v>
@@ -8244,7 +8238,7 @@
         <v>3.478260869565196</v>
       </c>
       <c r="Q16" t="n">
-        <v>32</v>
+        <v>31.9</v>
       </c>
       <c r="R16" t="n">
         <v>4</v>
@@ -8293,10 +8287,10 @@
         <v>420000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>557762</v>
+        <v>557490</v>
       </c>
       <c r="L17" t="n">
-        <v>24.69906519268075</v>
+        <v>24.66232578162837</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -8311,7 +8305,7 @@
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>8.6</v>
+        <v>8.5</v>
       </c>
       <c r="R17" t="n">
         <v>4</v>
@@ -8360,10 +8354,10 @@
         <v>454000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>600700</v>
+        <v>600407</v>
       </c>
       <c r="L18" t="n">
-        <v>24.42150824038622</v>
+        <v>24.38462576219131</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -8375,7 +8369,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q18" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="R18" t="n">
         <v>3</v>
@@ -8424,10 +8418,10 @@
         <v>454000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>600700</v>
+        <v>600407</v>
       </c>
       <c r="L19" t="n">
-        <v>24.42150824038622</v>
+        <v>24.38462576219131</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -8439,7 +8433,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q19" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="R19" t="n">
         <v>3</v>
@@ -8488,10 +8482,10 @@
         <v>454000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>600700</v>
+        <v>600407</v>
       </c>
       <c r="L20" t="n">
-        <v>24.42150824038622</v>
+        <v>24.38462576219131</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -8503,7 +8497,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q20" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="R20" t="n">
         <v>3</v>
@@ -8552,10 +8546,10 @@
         <v>454000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>600700</v>
+        <v>600407</v>
       </c>
       <c r="L21" t="n">
-        <v>24.42150824038622</v>
+        <v>24.38462576219131</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -8567,7 +8561,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q21" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="R21" t="n">
         <v>3</v>
@@ -8616,10 +8610,10 @@
         <v>455000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>600700</v>
+        <v>600407</v>
       </c>
       <c r="L22" t="n">
-        <v>24.25503579157649</v>
+        <v>24.21807207444284</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -8680,10 +8674,10 @@
         <v>455000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>600700</v>
+        <v>600407</v>
       </c>
       <c r="L23" t="n">
-        <v>24.25503579157649</v>
+        <v>24.21807207444284</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -8744,10 +8738,10 @@
         <v>455000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>600700</v>
+        <v>600407</v>
       </c>
       <c r="L24" t="n">
-        <v>24.25503579157649</v>
+        <v>24.21807207444284</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -8808,10 +8802,10 @@
         <v>455000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>600700</v>
+        <v>600407</v>
       </c>
       <c r="L25" t="n">
-        <v>24.25503579157649</v>
+        <v>24.21807207444284</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -8872,10 +8866,10 @@
         <v>468000</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>686575</v>
+        <v>686241</v>
       </c>
       <c r="L26" t="n">
-        <v>31.83556057240651</v>
+        <v>31.80238429356451</v>
       </c>
       <c r="M26" s="3" t="n">
         <v>0</v>
@@ -8936,10 +8930,10 @@
         <v>468000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>686575</v>
+        <v>686241</v>
       </c>
       <c r="L27" t="n">
-        <v>31.83556057240651</v>
+        <v>31.80238429356451</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -9000,10 +8994,10 @@
         <v>468000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>686575</v>
+        <v>686241</v>
       </c>
       <c r="L28" t="n">
-        <v>31.83556057240651</v>
+        <v>31.80238429356451</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -9064,10 +9058,10 @@
         <v>468000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>686575</v>
+        <v>686241</v>
       </c>
       <c r="L29" t="n">
-        <v>31.83556057240651</v>
+        <v>31.80238429356451</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -9093,7 +9087,7 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MC6L4 M4 10C CPU 10C GPU 24GB 512GB Midnight</t>
+          <t>Apple MacBook Air 15 MDV94 M5 10C CPU 10C GPU 16GB 512GB Silver</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -9101,11 +9095,11 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E30" t="n">
         <v>512</v>
@@ -9118,35 +9112,38 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Midnight</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I30" s="3" t="n">
-        <v>475000</v>
+        <v>474999</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>475000</v>
+        <v>474999</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>686575</v>
+        <v>643324</v>
       </c>
       <c r="L30" t="n">
-        <v>30.81600699122456</v>
+        <v>26.16488736624159</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>0</v>
+        <v>-5000</v>
       </c>
       <c r="N30" t="n">
-        <v>0</v>
+        <v>2.061859921360663</v>
+      </c>
+      <c r="O30" t="n">
+        <v>100</v>
       </c>
       <c r="P30" t="n">
-        <v>100</v>
+        <v>0.0005369127516934785</v>
       </c>
       <c r="Q30" t="n">
-        <v>34.6</v>
+        <v>31.5</v>
       </c>
       <c r="R30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S30" t="inlineStr">
         <is>
@@ -9157,7 +9154,7 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MC6K4 M4 10C CPU 10C GPU 24GB 512GB Starlight</t>
+          <t>Apple MacBook Air 15 MDVD4 M5 10C CPU 10C GPU 16GB 512GB Starlight</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -9165,11 +9162,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E31" t="n">
         <v>512</v>
@@ -9192,25 +9189,28 @@
         <v>475000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>686575</v>
+        <v>643324</v>
       </c>
       <c r="L31" t="n">
-        <v>30.81600699122456</v>
+        <v>26.16473192357195</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>0</v>
+        <v>-2000</v>
       </c>
       <c r="N31" t="n">
+        <v>1.041460503042715</v>
+      </c>
+      <c r="O31" t="n">
         <v>0</v>
       </c>
       <c r="P31" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="Q31" t="n">
-        <v>34.6</v>
+        <v>9</v>
       </c>
       <c r="R31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S31" t="inlineStr">
         <is>
@@ -9221,7 +9221,7 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MC6J4 M4 10C CPU 10C GPU 24GB 512GB Silver</t>
+          <t>Apple MacBook Air 15 MDVQ4 M5 10C CPU 10C GPU 16GB 512GB Sky Blue</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -9229,11 +9229,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E32" t="n">
         <v>512</v>
@@ -9246,7 +9246,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Sky Blue</t>
         </is>
       </c>
       <c r="I32" s="3" t="n">
@@ -9256,25 +9256,28 @@
         <v>475000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>686575</v>
+        <v>643324</v>
       </c>
       <c r="L32" t="n">
-        <v>30.81600699122456</v>
+        <v>26.16473192357195</v>
       </c>
       <c r="M32" s="3" t="n">
-        <v>0</v>
+        <v>-2000</v>
       </c>
       <c r="N32" t="n">
+        <v>1.041460503042715</v>
+      </c>
+      <c r="O32" t="n">
         <v>0</v>
       </c>
       <c r="P32" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="Q32" t="n">
-        <v>34.6</v>
+        <v>9</v>
       </c>
       <c r="R32" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S32" t="inlineStr">
         <is>
@@ -9285,7 +9288,7 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MC7D4 M4 10C CPU 10C GPU 24GB 512GB Sky Blue</t>
+          <t>Apple MacBook Air 15 MDVH4 M5 10C CPU 10C GPU 16GB 512GB Midnight</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -9293,11 +9296,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E33" t="n">
         <v>512</v>
@@ -9310,7 +9313,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Sky Blue</t>
+          <t>Midnight</t>
         </is>
       </c>
       <c r="I33" s="3" t="n">
@@ -9320,25 +9323,28 @@
         <v>475000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>686575</v>
+        <v>643324</v>
       </c>
       <c r="L33" t="n">
-        <v>30.81600699122456</v>
+        <v>26.16473192357195</v>
       </c>
       <c r="M33" s="3" t="n">
-        <v>0</v>
+        <v>-2000</v>
       </c>
       <c r="N33" t="n">
+        <v>1.041460503042715</v>
+      </c>
+      <c r="O33" t="n">
         <v>0</v>
       </c>
       <c r="P33" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="Q33" t="n">
-        <v>34.6</v>
+        <v>9</v>
       </c>
       <c r="R33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S33" t="inlineStr">
         <is>
@@ -9349,7 +9355,7 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MDVD4 M5 10C CPU 10C GPU 16GB 512GB Starlight</t>
+          <t>Apple MacBook Air 15 MC6L4 M4 10C CPU 10C GPU 24GB 512GB Midnight</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -9357,11 +9363,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E34" t="n">
         <v>512</v>
@@ -9374,38 +9380,35 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Starlight</t>
+          <t>Midnight</t>
         </is>
       </c>
       <c r="I34" s="3" t="n">
-        <v>477000</v>
+        <v>475000</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>477000</v>
+        <v>475000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>643637</v>
+        <v>686241</v>
       </c>
       <c r="L34" t="n">
-        <v>25.88990378116858</v>
+        <v>30.78233448598962</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N34" t="n">
-        <v>0.6247929683186839</v>
-      </c>
-      <c r="O34" t="n">
+        <v>0</v>
+      </c>
+      <c r="P34" t="n">
         <v>100</v>
       </c>
-      <c r="P34" t="n">
-        <v>1.568112774445864</v>
-      </c>
       <c r="Q34" t="n">
-        <v>31.3</v>
+        <v>34.6</v>
       </c>
       <c r="R34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S34" t="inlineStr">
         <is>
@@ -9416,7 +9419,7 @@
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MDVQ4 M5 10C CPU 10C GPU 16GB 512GB Sky Blue</t>
+          <t>Apple MacBook Air 15 MC6K4 M4 10C CPU 10C GPU 24GB 512GB Starlight</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -9424,11 +9427,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E35" t="n">
         <v>512</v>
@@ -9441,38 +9444,35 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Sky Blue</t>
+          <t>Starlight</t>
         </is>
       </c>
       <c r="I35" s="3" t="n">
-        <v>477000</v>
+        <v>475000</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>477000</v>
+        <v>475000</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>643637</v>
+        <v>686241</v>
       </c>
       <c r="L35" t="n">
-        <v>25.88990378116858</v>
+        <v>30.78233448598962</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N35" t="n">
-        <v>0.6247929683186839</v>
-      </c>
-      <c r="O35" t="n">
+        <v>0</v>
+      </c>
+      <c r="P35" t="n">
         <v>100</v>
       </c>
-      <c r="P35" t="n">
-        <v>1.568112774445864</v>
-      </c>
       <c r="Q35" t="n">
-        <v>31.3</v>
+        <v>34.6</v>
       </c>
       <c r="R35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S35" t="inlineStr">
         <is>
@@ -9483,7 +9483,7 @@
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MDVH4 M5 10C CPU 10C GPU 16GB 512GB Midnight</t>
+          <t>Apple MacBook Air 15 MC6J4 M4 10C CPU 10C GPU 24GB 512GB Silver</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -9491,11 +9491,11 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E36" t="n">
         <v>512</v>
@@ -9508,38 +9508,35 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Midnight</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I36" s="3" t="n">
-        <v>477000</v>
+        <v>475000</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>477000</v>
+        <v>475000</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>643637</v>
+        <v>686241</v>
       </c>
       <c r="L36" t="n">
-        <v>25.88990378116858</v>
+        <v>30.78233448598962</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N36" t="n">
-        <v>0.6247929683186839</v>
-      </c>
-      <c r="O36" t="n">
+        <v>0</v>
+      </c>
+      <c r="P36" t="n">
         <v>100</v>
       </c>
-      <c r="P36" t="n">
-        <v>1.568112774445864</v>
-      </c>
       <c r="Q36" t="n">
-        <v>31.3</v>
+        <v>34.6</v>
       </c>
       <c r="R36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S36" t="inlineStr">
         <is>
@@ -9550,7 +9547,7 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MDV94 M5 10C CPU 10C GPU 16GB 512GB Silver</t>
+          <t>Apple MacBook Air 15 MC7D4 M4 10C CPU 10C GPU 24GB 512GB Sky Blue</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -9558,11 +9555,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E37" t="n">
         <v>512</v>
@@ -9575,38 +9572,35 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Sky Blue</t>
         </is>
       </c>
       <c r="I37" s="3" t="n">
-        <v>479999</v>
+        <v>475000</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>479999</v>
+        <v>475000</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>643637</v>
+        <v>686241</v>
       </c>
       <c r="L37" t="n">
-        <v>25.42395791416591</v>
+        <v>30.78233448598962</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N37" t="n">
-        <v>1.030929960680331</v>
-      </c>
-      <c r="O37" t="n">
         <v>0</v>
       </c>
       <c r="P37" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.800000000000001</v>
+        <v>34.6</v>
       </c>
       <c r="R37" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S37" t="inlineStr">
         <is>
@@ -9652,10 +9646,10 @@
         <v>500000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>643637</v>
+        <v>643324</v>
       </c>
       <c r="L38" t="n">
-        <v>22.31646098654987</v>
+        <v>22.27866518270731</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -9716,22 +9710,22 @@
         <v>544999</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>772451</v>
+        <v>772075</v>
       </c>
       <c r="L39" t="n">
-        <v>29.44549233543616</v>
+        <v>29.41113233817958</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N39" t="n">
-        <v>0.9090925619864764</v>
+        <v>0.7285987770469528</v>
       </c>
       <c r="P39" t="n">
         <v>64.69606956521737</v>
       </c>
       <c r="Q39" t="n">
-        <v>26.8</v>
+        <v>26.7</v>
       </c>
       <c r="R39" t="n">
         <v>3</v>
@@ -9780,22 +9774,22 @@
         <v>544999</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>772451</v>
+        <v>772075</v>
       </c>
       <c r="L40" t="n">
-        <v>29.44549233543616</v>
+        <v>29.41113233817958</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N40" t="n">
-        <v>0.9090925619864764</v>
+        <v>0.7285987770469528</v>
       </c>
       <c r="P40" t="n">
         <v>64.69606956521737</v>
       </c>
       <c r="Q40" t="n">
-        <v>26.8</v>
+        <v>26.7</v>
       </c>
       <c r="R40" t="n">
         <v>3</v>
@@ -9844,22 +9838,22 @@
         <v>544999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>772451</v>
+        <v>772075</v>
       </c>
       <c r="L41" t="n">
-        <v>29.44549233543616</v>
+        <v>29.41113233817958</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N41" t="n">
-        <v>1.268118239344636</v>
+        <v>0.9090925619864764</v>
       </c>
       <c r="P41" t="n">
         <v>64.69606956521737</v>
       </c>
       <c r="Q41" t="n">
-        <v>26.9</v>
+        <v>26.8</v>
       </c>
       <c r="R41" t="n">
         <v>3</v>
@@ -9908,22 +9902,22 @@
         <v>544999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>772451</v>
+        <v>772075</v>
       </c>
       <c r="L42" t="n">
-        <v>29.44549233543616</v>
+        <v>29.41113233817958</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N42" t="n">
-        <v>0.9090925619864764</v>
+        <v>0.7285987770469528</v>
       </c>
       <c r="P42" t="n">
         <v>64.69606956521737</v>
       </c>
       <c r="Q42" t="n">
-        <v>26.8</v>
+        <v>26.7</v>
       </c>
       <c r="R42" t="n">
         <v>3</v>
@@ -9972,22 +9966,22 @@
         <v>549999</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>772451</v>
+        <v>772075</v>
       </c>
       <c r="L43" t="n">
-        <v>28.79820208660485</v>
+        <v>28.76352685943723</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>1.78571747449549</v>
+        <v>1.168016474423135</v>
       </c>
       <c r="P43" t="n">
-        <v>35.29417147279201</v>
+        <v>33.55744966442954</v>
       </c>
       <c r="Q43" t="n">
-        <v>20.5</v>
+        <v>19.9</v>
       </c>
       <c r="R43" t="n">
         <v>3</v>
@@ -10036,22 +10030,22 @@
         <v>549999</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>772451</v>
+        <v>772075</v>
       </c>
       <c r="L44" t="n">
-        <v>28.79820208660485</v>
+        <v>28.76352685943723</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>1.78571747449549</v>
+        <v>1.168016474423135</v>
       </c>
       <c r="P44" t="n">
-        <v>35.29417147279201</v>
+        <v>33.55744966442954</v>
       </c>
       <c r="Q44" t="n">
-        <v>20.5</v>
+        <v>19.9</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -10100,22 +10094,22 @@
         <v>549999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>772451</v>
+        <v>772075</v>
       </c>
       <c r="L45" t="n">
-        <v>28.79820208660485</v>
+        <v>28.76352685943723</v>
       </c>
       <c r="M45" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>1.78571747449549</v>
+        <v>1.168016474423135</v>
       </c>
       <c r="P45" t="n">
-        <v>35.29417147279201</v>
+        <v>33.55744966442954</v>
       </c>
       <c r="Q45" t="n">
-        <v>20.5</v>
+        <v>19.9</v>
       </c>
       <c r="R45" t="n">
         <v>3</v>
@@ -10164,22 +10158,22 @@
         <v>549999</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>772451</v>
+        <v>772075</v>
       </c>
       <c r="L46" t="n">
-        <v>28.79820208660485</v>
+        <v>28.76352685943723</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N46" t="n">
-        <v>1.78571747449549</v>
+        <v>1.168016474423135</v>
       </c>
       <c r="P46" t="n">
-        <v>35.29417147279201</v>
+        <v>33.55744966442954</v>
       </c>
       <c r="Q46" t="n">
-        <v>20.5</v>
+        <v>19.9</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -10228,10 +10222,10 @@
         <v>585000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>729513</v>
+        <v>729158</v>
       </c>
       <c r="L47" t="n">
-        <v>19.809516759811</v>
+        <v>19.77047498621698</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -10240,10 +10234,10 @@
         <v>0</v>
       </c>
       <c r="P47" t="n">
-        <v>21.56821735015607</v>
+        <v>19.46308724832216</v>
       </c>
       <c r="Q47" t="n">
-        <v>13.1</v>
+        <v>12.6</v>
       </c>
       <c r="R47" t="n">
         <v>3</v>
@@ -10292,10 +10286,10 @@
         <v>595000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>729513</v>
+        <v>729158</v>
       </c>
       <c r="L48" t="n">
-        <v>18.43873926852572</v>
+        <v>18.3990301141865</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -10356,10 +10350,10 @@
         <v>619999</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>858326</v>
+        <v>857909</v>
       </c>
       <c r="L49" t="n">
-        <v>27.7664896554456</v>
+        <v>27.73137943534804</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -10368,10 +10362,10 @@
         <v>0</v>
       </c>
       <c r="P49" t="n">
-        <v>56.47067435646721</v>
+        <v>55.30233557046979</v>
       </c>
       <c r="Q49" t="n">
-        <v>24</v>
+        <v>23.7</v>
       </c>
       <c r="R49" t="n">
         <v>3</v>
@@ -10420,10 +10414,10 @@
         <v>619999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>858326</v>
+        <v>857909</v>
       </c>
       <c r="L50" t="n">
-        <v>27.7664896554456</v>
+        <v>27.73137943534804</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -10432,10 +10426,10 @@
         <v>0</v>
       </c>
       <c r="P50" t="n">
-        <v>56.47067435646721</v>
+        <v>55.30233557046979</v>
       </c>
       <c r="Q50" t="n">
-        <v>24</v>
+        <v>23.7</v>
       </c>
       <c r="R50" t="n">
         <v>3</v>
@@ -10484,10 +10478,10 @@
         <v>619999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>858326</v>
+        <v>857909</v>
       </c>
       <c r="L51" t="n">
-        <v>27.7664896554456</v>
+        <v>27.73137943534804</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -10496,10 +10490,10 @@
         <v>0</v>
       </c>
       <c r="P51" t="n">
-        <v>56.47067435646721</v>
+        <v>55.30233557046979</v>
       </c>
       <c r="Q51" t="n">
-        <v>24</v>
+        <v>23.7</v>
       </c>
       <c r="R51" t="n">
         <v>3</v>
@@ -10548,10 +10542,10 @@
         <v>619999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>858326</v>
+        <v>857909</v>
       </c>
       <c r="L52" t="n">
-        <v>27.7664896554456</v>
+        <v>27.73137943534804</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -10560,10 +10554,10 @@
         <v>0</v>
       </c>
       <c r="P52" t="n">
-        <v>56.47067435646721</v>
+        <v>55.30233557046979</v>
       </c>
       <c r="Q52" t="n">
-        <v>24</v>
+        <v>23.7</v>
       </c>
       <c r="R52" t="n">
         <v>3</v>
@@ -10612,10 +10606,10 @@
         <v>650000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>815389</v>
+        <v>814992</v>
       </c>
       <c r="L53" t="n">
-        <v>20.28344753240478</v>
+        <v>20.24461589807017</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -10624,10 +10618,10 @@
         <v>0</v>
       </c>
       <c r="P53" t="n">
-        <v>47.05854671135535</v>
+        <v>45.63758389261746</v>
       </c>
       <c r="Q53" t="n">
-        <v>18.8</v>
+        <v>18.5</v>
       </c>
       <c r="R53" t="n">
         <v>3</v>
@@ -10676,10 +10670,10 @@
         <v>672000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>858326</v>
+        <v>857909</v>
       </c>
       <c r="L54" t="n">
-        <v>21.70806896214259</v>
+        <v>21.67001395252877</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -10740,10 +10734,10 @@
         <v>700000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>901264</v>
+        <v>900826</v>
       </c>
       <c r="L55" t="n">
-        <v>22.33130359140052</v>
+        <v>22.29353948487277</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -10804,10 +10798,10 @@
         <v>715000</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>944202</v>
+        <v>943742</v>
       </c>
       <c r="L56" t="n">
-        <v>24.27467851158968</v>
+        <v>24.23776837313588</v>
       </c>
       <c r="M56" s="3" t="n">
         <v>0</v>
@@ -10816,10 +10810,10 @@
         <v>0</v>
       </c>
       <c r="P56" t="n">
-        <v>64.05209961882153</v>
+        <v>63.08724832214765</v>
       </c>
       <c r="Q56" t="n">
-        <v>24.1</v>
+        <v>23.9</v>
       </c>
       <c r="R56" t="n">
         <v>3</v>
@@ -10868,10 +10862,10 @@
         <v>734999</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>987140</v>
+        <v>986659</v>
       </c>
       <c r="L57" t="n">
-        <v>25.54257754725773</v>
+        <v>25.50627927176461</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -10932,10 +10926,10 @@
         <v>752000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>987140</v>
+        <v>986659</v>
       </c>
       <c r="L58" t="n">
-        <v>23.82032943655409</v>
+        <v>23.78319155858306</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -10944,10 +10938,10 @@
         <v>0</v>
       </c>
       <c r="P58" t="n">
-        <v>54.37884642534079</v>
+        <v>53.15436241610739</v>
       </c>
       <c r="Q58" t="n">
-        <v>21.9</v>
+        <v>21.6</v>
       </c>
       <c r="R58" t="n">
         <v>3</v>
@@ -10996,10 +10990,10 @@
         <v>810000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1073015</v>
+        <v>1072493</v>
       </c>
       <c r="L59" t="n">
-        <v>24.51177290159038</v>
+        <v>24.47503153866738</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -11008,10 +11002,10 @@
         <v>0</v>
       </c>
       <c r="P59" t="n">
-        <v>69.46762746845361</v>
+        <v>68.64813039309685</v>
       </c>
       <c r="Q59" t="n">
-        <v>25.4</v>
+        <v>25.2</v>
       </c>
       <c r="R59" t="n">
         <v>3</v>
@@ -11060,10 +11054,10 @@
         <v>815000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1073015</v>
+        <v>1072493</v>
       </c>
       <c r="L60" t="n">
-        <v>24.04579619110637</v>
+        <v>24.00882802964681</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -11075,7 +11069,7 @@
         <v>79.56521739130434</v>
       </c>
       <c r="Q60" t="n">
-        <v>27.4</v>
+        <v>27.3</v>
       </c>
       <c r="R60" t="n">
         <v>3</v>
@@ -11124,10 +11118,10 @@
         <v>875000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1158891</v>
+        <v>1158327</v>
       </c>
       <c r="L61" t="n">
-        <v>24.49678183711842</v>
+        <v>24.46001863031769</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -11136,10 +11130,10 @@
         <v>0</v>
       </c>
       <c r="P61" t="n">
-        <v>79.41165705441597</v>
+        <v>78.85906040268456</v>
       </c>
       <c r="Q61" t="n">
-        <v>27.5</v>
+        <v>27.4</v>
       </c>
       <c r="R61" t="n">
         <v>3</v>
@@ -11188,10 +11182,10 @@
         <v>992000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1330642</v>
+        <v>1329994</v>
       </c>
       <c r="L62" t="n">
-        <v>25.44951985582899</v>
+        <v>25.41319735277001</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -11203,7 +11197,7 @@
         <v>85.14782608695651</v>
       </c>
       <c r="Q62" t="n">
-        <v>29.2</v>
+        <v>29.1</v>
       </c>
       <c r="R62" t="n">
         <v>3</v>
@@ -11252,10 +11246,10 @@
         <v>1050000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1416518</v>
+        <v>1415828</v>
       </c>
       <c r="L63" t="n">
-        <v>25.87457413177948</v>
+        <v>25.83844930316395</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -11316,10 +11310,10 @@
         <v>1050000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1416518</v>
+        <v>1415828</v>
       </c>
       <c r="L64" t="n">
-        <v>25.87457413177948</v>
+        <v>25.83844930316395</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -11328,10 +11322,10 @@
         <v>0</v>
       </c>
       <c r="P64" t="n">
-        <v>86.27443803627732</v>
+        <v>85.90604026845638</v>
       </c>
       <c r="Q64" t="n">
-        <v>29.6</v>
+        <v>29.5</v>
       </c>
       <c r="R64" t="n">
         <v>3</v>
@@ -11380,10 +11374,10 @@
         <v>1100000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1502393</v>
+        <v>1501662</v>
       </c>
       <c r="L65" t="n">
-        <v>26.78347143523698</v>
+        <v>26.74783007094806</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -11392,7 +11386,7 @@
         <v>0</v>
       </c>
       <c r="P65" t="n">
-        <v>94.11761630126171</v>
+        <v>93.95973154362416</v>
       </c>
       <c r="Q65" t="n">
         <v>31.6</v>
@@ -11444,10 +11438,10 @@
         <v>1105000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1502393</v>
+        <v>1501662</v>
       </c>
       <c r="L66" t="n">
-        <v>26.45066903266988</v>
+        <v>26.41486566217964</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -11459,7 +11453,7 @@
         <v>100</v>
       </c>
       <c r="Q66" t="n">
-        <v>32.8</v>
+        <v>32.7</v>
       </c>
       <c r="R66" t="n">
         <v>3</v>
@@ -11508,10 +11502,10 @@
         <v>1155000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1588269</v>
+        <v>1587496</v>
       </c>
       <c r="L67" t="n">
-        <v>27.27932107218614</v>
+        <v>27.24391116576042</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -11778,7 +11772,7 @@
         <v>315000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>300135</v>
+        <v>299989</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -11839,10 +11833,10 @@
         <v>380000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>386011</v>
+        <v>385823</v>
       </c>
       <c r="L3" t="n">
-        <v>1.557209509573561</v>
+        <v>1.509241284215819</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -11903,7 +11897,7 @@
         <v>415000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>386011</v>
+        <v>385823</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -11964,10 +11958,10 @@
         <v>495000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>471886</v>
+        <v>471657</v>
       </c>
       <c r="L5" t="n">
-        <v>6.757352411387496</v>
+        <v>6.712081024982138</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -12028,10 +12022,10 @@
         <v>490000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514824</v>
+        <v>514574</v>
       </c>
       <c r="L6" t="n">
-        <v>4.821842027566702</v>
+        <v>4.775600788224823</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -12043,7 +12037,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="R6" t="n">
         <v>3</v>
@@ -12092,10 +12086,10 @@
         <v>550000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>557762</v>
+        <v>557490</v>
       </c>
       <c r="L7" t="n">
-        <v>6.770271190938071</v>
+        <v>6.724784301063696</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -12156,7 +12150,7 @@
         <v>530000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>471886</v>
+        <v>471657</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -12220,10 +12214,10 @@
         <v>600000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>600700</v>
+        <v>600407</v>
       </c>
       <c r="L9" t="n">
-        <v>8.440153154652904</v>
+        <v>8.395471738337495</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -12284,10 +12278,10 @@
         <v>646000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>729513</v>
+        <v>729158</v>
       </c>
       <c r="L10" t="n">
-        <v>17.06809885498956</v>
+        <v>17.02772238664322</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -12348,7 +12342,7 @@
         <v>615000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>557762</v>
+        <v>557490</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -12412,7 +12406,7 @@
         <v>700000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>643637</v>
+        <v>643324</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -12476,7 +12470,7 @@
         <v>745000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>686575</v>
+        <v>686241</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -12540,7 +12534,7 @@
         <v>930000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>858326</v>
+        <v>857909</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -12611,7 +12605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12660,30 +12654,150 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 14Inch MX2H3 M4 Pro 12Core CPU 16Core GPU 24GB 512GB Space Black</t>
+          <t>Apple MacBook Air 15 MDV94 M5 10C CPU 10C GPU 16GB 512GB Silver</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>600000</v>
+        <v>479999</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>634000</v>
+        <v>474999</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>34000</v>
+        <v>-5000</v>
       </c>
       <c r="F2" t="n">
-        <v>5.67</v>
+        <v>-1.04</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Macbook Pro 16 MGEA4 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Space Black</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>823000</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>820000</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>-3000</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-0.36</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Macbook Pro 16 MGE44 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Silver</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>822999</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>820000</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>-2999</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-0.36</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 15 MDVD4 M5 10C CPU 10C GPU 16GB 512GB Starlight</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>477000</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>475000</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>-2000</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-0.42</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 15 MDVQ4 M5 10C CPU 10C GPU 16GB 512GB Sky Blue</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>477000</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>475000</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>-2000</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-0.42</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 15 MDVH4 M5 10C CPU 10C GPU 16GB 512GB Midnight</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>477000</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>475000</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>-2000</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-0.42</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F2"/>
-  <conditionalFormatting sqref="E2">
+  <autoFilter ref="A1:F7"/>
+  <conditionalFormatting sqref="E2:E7">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
chore: price data 2026-10-11
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -16,8 +16,8 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MacBook Pro'!$A$1:$S$93</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MacBook Air'!$A$1:$S$67</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20261010T095542822990+0000</t>
+          <t>20261011T100509295831+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-10T09:55:42.822990+00:00</t>
+          <t>2026-10-11T10:05:09.295831+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>276.883168</v>
+        <v>276.868026</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -528,7 +528,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="8">
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12">
@@ -1112,7 +1112,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 14Inch MW2W3 M4 10Core CPU 10Core GPU 16GB 512GB Silver</t>
+          <t>Apple MacBook Pro 14Inch MW2U3 M4 10Core CPU 10Core GPU 16GB 512GB Space Black</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -1137,20 +1137,20 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I2" s="3" t="n">
-        <v>445000</v>
+        <v>495000</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>470000</v>
+        <v>495000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>686241</v>
+        <v>686204</v>
       </c>
       <c r="L2" t="n">
-        <v>35.15397651845343</v>
+        <v>27.8640171144441</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1162,13 +1162,13 @@
         <v>100</v>
       </c>
       <c r="P2" t="n">
-        <v>28.4414106939704</v>
+        <v>1.677852348993289</v>
       </c>
       <c r="Q2" t="n">
-        <v>35.3</v>
+        <v>31.8</v>
       </c>
       <c r="R2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -1179,7 +1179,7 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 14Inch MW2U3 M4 10Core CPU 10Core GPU 16GB 512GB Space Black</t>
+          <t>Apple MacBook Pro 14Inch MW2W3 M4 10Core CPU 10Core GPU 16GB 512GB Silver</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -1204,23 +1204,23 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I3" s="3" t="n">
-        <v>495000</v>
+        <v>498000</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>495000</v>
+        <v>498000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>686241</v>
+        <v>686204</v>
       </c>
       <c r="L3" t="n">
-        <v>27.86790646434708</v>
+        <v>27.42682933938013</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>0</v>
+        <v>53000</v>
       </c>
       <c r="N3" t="n">
         <v>0</v>
@@ -1232,7 +1232,7 @@
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>9.300000000000001</v>
+        <v>9.1</v>
       </c>
       <c r="R3" t="n">
         <v>4</v>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>772075</v>
+        <v>772033</v>
       </c>
       <c r="L4" t="n">
-        <v>35.23958164686074</v>
+        <v>35.23605856226353</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1296,10 +1296,10 @@
         <v>100</v>
       </c>
       <c r="P4" t="n">
-        <v>68.25981228668942</v>
+        <v>68.79236577181209</v>
       </c>
       <c r="Q4" t="n">
-        <v>41.7</v>
+        <v>41.8</v>
       </c>
       <c r="R4" t="n">
         <v>5</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>772075</v>
+        <v>772033</v>
       </c>
       <c r="L5" t="n">
-        <v>32.64915973189133</v>
+        <v>32.64549572362839</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1363,10 +1363,10 @@
         <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>59.72738907849829</v>
+        <v>60.40310402684563</v>
       </c>
       <c r="Q5" t="n">
-        <v>19.3</v>
+        <v>19.4</v>
       </c>
       <c r="R5" t="n">
         <v>5</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>857909</v>
+        <v>857862</v>
       </c>
       <c r="L6" t="n">
-        <v>37.98876104575194</v>
+        <v>37.98536361326181</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1606,10 +1606,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>857909</v>
+        <v>857862</v>
       </c>
       <c r="L9" t="n">
-        <v>34.14219923092076</v>
+        <v>34.13859105543782</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1621,7 +1621,7 @@
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>88.73720136518772</v>
+        <v>88.92617449664429</v>
       </c>
       <c r="Q9" t="n">
         <v>26.2</v>
@@ -1673,10 +1673,10 @@
         <v>578999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>857909</v>
+        <v>857862</v>
       </c>
       <c r="L10" t="n">
-        <v>32.51044108407768</v>
+        <v>32.50674350886273</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -1740,10 +1740,10 @@
         <v>584999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>857909</v>
+        <v>857862</v>
       </c>
       <c r="L11" t="n">
-        <v>31.81106620865383</v>
+        <v>31.8073303165311</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -1807,10 +1807,10 @@
         <v>634000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>857909</v>
+        <v>857862</v>
       </c>
       <c r="L12" t="n">
-        <v>26.09938816354648</v>
+        <v>26.09533934362404</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -1871,10 +1871,10 @@
         <v>634000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>857909</v>
+        <v>857862</v>
       </c>
       <c r="L13" t="n">
-        <v>26.09938816354648</v>
+        <v>26.09533934362404</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -1935,10 +1935,10 @@
         <v>642999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>943742</v>
+        <v>943691</v>
       </c>
       <c r="L14" t="n">
-        <v>31.86707807854265</v>
+        <v>31.86339596329731</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -2061,10 +2061,10 @@
         <v>650000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>943742</v>
+        <v>943691</v>
       </c>
       <c r="L16" t="n">
-        <v>31.12524397557807</v>
+        <v>31.12152176930796</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -2128,10 +2128,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1029576</v>
+        <v>1029520</v>
       </c>
       <c r="L17" t="n">
-        <v>32.01084718369503</v>
+        <v>32.00714896262336</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2195,10 +2195,10 @@
         <v>711999</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>1072493</v>
+        <v>1072434</v>
       </c>
       <c r="L18" t="n">
-        <v>33.61271355617239</v>
+        <v>33.60906125691651</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -2324,10 +2324,10 @@
         <v>720000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>1029576</v>
+        <v>1029520</v>
       </c>
       <c r="L20" t="n">
-        <v>30.06829996037204</v>
+        <v>30.06449607584117</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -2453,10 +2453,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1072493</v>
+        <v>1072434</v>
       </c>
       <c r="L22" t="n">
-        <v>30.72215855954304</v>
+        <v>30.7183472362868</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2520,10 +2520,10 @@
         <v>759999</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1029576</v>
+        <v>1029520</v>
       </c>
       <c r="L23" t="n">
-        <v>26.1833026410872</v>
+        <v>26.17928743492113</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -2587,10 +2587,10 @@
         <v>759999</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1029576</v>
+        <v>1029520</v>
       </c>
       <c r="L24" t="n">
-        <v>26.1833026410872</v>
+        <v>26.17928743492113</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -2654,10 +2654,10 @@
         <v>772000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>1029576</v>
+        <v>1029520</v>
       </c>
       <c r="L25" t="n">
-        <v>25.01767717973224</v>
+        <v>25.01359857020747</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -2845,10 +2845,10 @@
         <v>810000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>1072493</v>
+        <v>1072434</v>
       </c>
       <c r="L28" t="n">
-        <v>24.47503153866738</v>
+        <v>24.47087652946475</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -2909,10 +2909,10 @@
         <v>810000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>1244161</v>
+        <v>1244093</v>
       </c>
       <c r="L29" t="n">
-        <v>34.89588566110013</v>
+        <v>34.89232718132808</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -2976,13 +2976,13 @@
         <v>820000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1287078</v>
+        <v>1287007</v>
       </c>
       <c r="L30" t="n">
-        <v>36.2897975103296</v>
+        <v>36.28628282519054</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>-3000</v>
+        <v>0</v>
       </c>
       <c r="N30" t="n">
         <v>0.6060606060606061</v>
@@ -3040,13 +3040,13 @@
         <v>820000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1287078</v>
+        <v>1287007</v>
       </c>
       <c r="L31" t="n">
-        <v>36.2897975103296</v>
+        <v>36.28628282519054</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>-2999</v>
+        <v>0</v>
       </c>
       <c r="N31" t="n">
         <v>1.204700246626803</v>
@@ -3104,10 +3104,10 @@
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1372911</v>
+        <v>1372836</v>
       </c>
       <c r="L32" t="n">
-        <v>38.23350530369412</v>
+        <v>38.23013091148542</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3171,10 +3171,10 @@
         <v>930000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1372911</v>
+        <v>1372836</v>
       </c>
       <c r="L33" t="n">
-        <v>38.08782943686808</v>
+        <v>38.08444708617781</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3238,10 +3238,10 @@
         <v>860000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>1244161</v>
+        <v>1244093</v>
       </c>
       <c r="L34" t="n">
-        <v>30.87711317104458</v>
+        <v>30.87333503202735</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -3367,10 +3367,10 @@
         <v>880000</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>1158327</v>
+        <v>1158264</v>
       </c>
       <c r="L36" t="n">
-        <v>24.02836159391951</v>
+        <v>24.02422936394466</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -3431,10 +3431,10 @@
         <v>940000</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>1244161</v>
+        <v>1244093</v>
       </c>
       <c r="L37" t="n">
-        <v>24.44707718695571</v>
+        <v>24.44294759314617</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
@@ -3619,10 +3619,10 @@
         <v>990000</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>1501662</v>
+        <v>1501580</v>
       </c>
       <c r="L40" t="n">
-        <v>34.07304706385325</v>
+        <v>34.06944684931872</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -3748,10 +3748,10 @@
         <v>1000000</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>1501662</v>
+        <v>1501580</v>
       </c>
       <c r="L42" t="n">
-        <v>33.40711824631641</v>
+        <v>33.4034816659785</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -3815,10 +3815,10 @@
         <v>1054000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1544579</v>
+        <v>1544494</v>
       </c>
       <c r="L43" t="n">
-        <v>31.76134079253958</v>
+        <v>31.75758533215409</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -3879,10 +3879,10 @@
         <v>1054000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1544579</v>
+        <v>1544494</v>
       </c>
       <c r="L44" t="n">
-        <v>31.76134079253958</v>
+        <v>31.75758533215409</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -4005,10 +4005,10 @@
         <v>1115000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1501662</v>
+        <v>1501580</v>
       </c>
       <c r="L46" t="n">
-        <v>25.7489368446428</v>
+        <v>25.74488205756603</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -4069,10 +4069,10 @@
         <v>1123000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1716246</v>
+        <v>1716153</v>
       </c>
       <c r="L47" t="n">
-        <v>34.56648988548262</v>
+        <v>34.56294397993652</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -4136,10 +4136,10 @@
         <v>1130000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1501662</v>
+        <v>1501580</v>
       </c>
       <c r="L48" t="n">
-        <v>24.75004361833755</v>
+        <v>24.74593428255571</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -4151,7 +4151,7 @@
         <v>88.39999999999999</v>
       </c>
       <c r="Q48" t="n">
-        <v>29.6</v>
+        <v>29.5</v>
       </c>
       <c r="R48" t="n">
         <v>3</v>
@@ -4262,10 +4262,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1759163</v>
+        <v>1759067</v>
       </c>
       <c r="L50" t="n">
-        <v>34.343775988922</v>
+        <v>34.34019284086393</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4326,10 +4326,10 @@
         <v>1155000</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>1759163</v>
+        <v>1759067</v>
       </c>
       <c r="L51" t="n">
-        <v>34.343775988922</v>
+        <v>34.34019284086393</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -4390,10 +4390,10 @@
         <v>1185000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1587496</v>
+        <v>1587409</v>
       </c>
       <c r="L52" t="n">
-        <v>25.35414262461134</v>
+        <v>25.3500515620108</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -4454,10 +4454,10 @@
         <v>1185000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1587496</v>
+        <v>1587409</v>
       </c>
       <c r="L53" t="n">
-        <v>25.35414262461134</v>
+        <v>25.3500515620108</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -4518,10 +4518,10 @@
         <v>1200000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1887914</v>
+        <v>1887811</v>
       </c>
       <c r="L54" t="n">
-        <v>36.43778265323526</v>
+        <v>36.43431466391498</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -4582,10 +4582,10 @@
         <v>1200000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1887914</v>
+        <v>1887811</v>
       </c>
       <c r="L55" t="n">
-        <v>36.43778265323526</v>
+        <v>36.43431466391498</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -4708,10 +4708,10 @@
         <v>1240000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1673330</v>
+        <v>1673238</v>
       </c>
       <c r="L57" t="n">
-        <v>25.89626672563093</v>
+        <v>25.89219226434016</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -4737,11 +4737,11 @@
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 24GB 4TB Silver</t>
+          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 64GB 1TB Silver</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -4749,16 +4749,16 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>24</v>
+        <v>64</v>
       </c>
       <c r="E58" t="n">
-        <v>4096</v>
+        <v>1024</v>
       </c>
       <c r="F58" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G58" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
@@ -4766,79 +4766,76 @@
         </is>
       </c>
       <c r="I58" s="3" t="n">
-        <v>1260000</v>
+        <v>1255000</v>
       </c>
       <c r="J58" s="3" t="n">
-        <v>1260000</v>
-      </c>
-      <c r="K58" s="3" t="n"/>
+        <v>1255000</v>
+      </c>
+      <c r="K58" s="3" t="n">
+        <v>1716153</v>
+      </c>
+      <c r="L58" t="n">
+        <v>26.87132207909201</v>
+      </c>
       <c r="M58" s="3" t="n">
-        <v>0</v>
+        <v>-45000</v>
       </c>
       <c r="N58" t="n">
-        <v>0</v>
-      </c>
-      <c r="O58" t="n">
-        <v>100</v>
+        <v>3.461538461538462</v>
       </c>
       <c r="P58" t="n">
-        <v>82.67288267288268</v>
+        <v>68.52057842046719</v>
       </c>
       <c r="Q58" t="n">
-        <v>54</v>
+        <v>27.4</v>
       </c>
       <c r="R58" t="n">
         <v>3</v>
       </c>
       <c r="S58" t="inlineStr">
         <is>
-          <t>2026-09-26T08:39:40.619332+00:00</t>
+          <t>2026-09-16T00:22:18.878661+00:00</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 16Inch MX313 16Core CPU 40 Core GPU M4 Max 48GB 1TB Space Black</t>
+          <t>Macbook Pro 14 CTO M5 Pro 15 Core CPU 16 Core GPU 24GB 4TB Silver</t>
         </is>
       </c>
       <c r="B59" t="n">
+        <v>14</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>M5 Pro</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>24</v>
+      </c>
+      <c r="E59" t="n">
+        <v>4096</v>
+      </c>
+      <c r="F59" t="n">
+        <v>15</v>
+      </c>
+      <c r="G59" t="n">
         <v>16</v>
       </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>M4 Max</t>
-        </is>
-      </c>
-      <c r="D59" t="n">
-        <v>48</v>
-      </c>
-      <c r="E59" t="n">
-        <v>1024</v>
-      </c>
-      <c r="F59" t="n">
-        <v>16</v>
-      </c>
-      <c r="G59" t="n">
-        <v>40</v>
-      </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Space Black</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I59" s="3" t="n">
-        <v>1280000</v>
+        <v>1260000</v>
       </c>
       <c r="J59" s="3" t="n">
-        <v>1280000</v>
-      </c>
-      <c r="K59" s="3" t="n">
-        <v>1716246</v>
-      </c>
-      <c r="L59" t="n">
-        <v>25.41861714462845</v>
-      </c>
+        <v>1260000</v>
+      </c>
+      <c r="K59" s="3" t="n"/>
       <c r="M59" s="3" t="n">
         <v>0</v>
       </c>
@@ -4846,27 +4843,27 @@
         <v>0</v>
       </c>
       <c r="O59" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="P59" t="n">
-        <v>0</v>
+        <v>82.67288267288268</v>
       </c>
       <c r="Q59" t="n">
-        <v>8.5</v>
+        <v>54</v>
       </c>
       <c r="R59" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>2026-09-16T00:22:18.878661+00:00</t>
+          <t>2026-09-26T08:39:40.619332+00:00</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 48GB 2TB Silver</t>
+          <t>Apple MacBook Pro 16Inch MX313 16Core CPU 40 Core GPU M4 Max 48GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -4874,37 +4871,37 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>M5 Pro</t>
+          <t>M4 Max</t>
         </is>
       </c>
       <c r="D60" t="n">
         <v>48</v>
       </c>
       <c r="E60" t="n">
-        <v>2048</v>
+        <v>1024</v>
       </c>
       <c r="F60" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G60" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Space Black</t>
         </is>
       </c>
       <c r="I60" s="3" t="n">
-        <v>1298000</v>
+        <v>1280000</v>
       </c>
       <c r="J60" s="3" t="n">
-        <v>1298000</v>
+        <v>1280000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1759163</v>
+        <v>1716153</v>
       </c>
       <c r="L60" t="n">
-        <v>26.21491015897902</v>
+        <v>25.41457550696237</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -4912,14 +4909,17 @@
       <c r="N60" t="n">
         <v>0</v>
       </c>
+      <c r="O60" t="n">
+        <v>0</v>
+      </c>
       <c r="P60" t="n">
-        <v>60.86763070077864</v>
+        <v>0</v>
       </c>
       <c r="Q60" t="n">
-        <v>24.3</v>
+        <v>8.5</v>
       </c>
       <c r="R60" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S60" t="inlineStr">
         <is>
@@ -4930,7 +4930,7 @@
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 64GB 1TB Silver</t>
+          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 48GB 2TB Silver</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -4942,10 +4942,10 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="E61" t="n">
-        <v>1024</v>
+        <v>2048</v>
       </c>
       <c r="F61" t="n">
         <v>18</v>
@@ -4959,16 +4959,16 @@
         </is>
       </c>
       <c r="I61" s="3" t="n">
-        <v>1300000</v>
+        <v>1298000</v>
       </c>
       <c r="J61" s="3" t="n">
-        <v>1300000</v>
+        <v>1298000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1716246</v>
+        <v>1759067</v>
       </c>
       <c r="L61" t="n">
-        <v>24.25328303751327</v>
+        <v>26.21088338306614</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -4977,10 +4977,10 @@
         <v>0</v>
       </c>
       <c r="P61" t="n">
-        <v>60.51167964404895</v>
+        <v>60.86763070077864</v>
       </c>
       <c r="Q61" t="n">
-        <v>23.4</v>
+        <v>24.3</v>
       </c>
       <c r="R61" t="n">
         <v>3</v>
@@ -5091,10 +5091,10 @@
         <v>1335000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1802080</v>
+        <v>1801982</v>
       </c>
       <c r="L63" t="n">
-        <v>25.9189381159549</v>
+        <v>25.91490924992592</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -5155,10 +5155,10 @@
         <v>1420000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1930831</v>
+        <v>1930725</v>
       </c>
       <c r="L64" t="n">
-        <v>26.45653607177428</v>
+        <v>26.45249841380829</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -5219,10 +5219,10 @@
         <v>1430000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1930831</v>
+        <v>1930725</v>
       </c>
       <c r="L65" t="n">
-        <v>25.93862435396987</v>
+        <v>25.93455826179285</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -5283,10 +5283,10 @@
         <v>1430000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>2145415</v>
+        <v>2145298</v>
       </c>
       <c r="L66" t="n">
-        <v>33.34622905125582</v>
+        <v>33.34259389604614</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -5347,10 +5347,10 @@
         <v>1430000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>2145415</v>
+        <v>2145298</v>
       </c>
       <c r="L67" t="n">
-        <v>33.34622905125582</v>
+        <v>33.34259389604614</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -5473,10 +5473,10 @@
         <v>1480000</v>
       </c>
       <c r="K69" s="3" t="n">
-        <v>2016665</v>
+        <v>2016554</v>
       </c>
       <c r="L69" t="n">
-        <v>26.61150959628892</v>
+        <v>26.60746997104962</v>
       </c>
       <c r="M69" s="3" t="n">
         <v>0</v>
@@ -5599,10 +5599,10 @@
         <v>1605000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2188332</v>
+        <v>2188213</v>
       </c>
       <c r="L71" t="n">
-        <v>26.65646711742094</v>
+        <v>26.65247852928394</v>
       </c>
       <c r="M71" s="3" t="n">
         <v>0</v>
@@ -5663,10 +5663,10 @@
         <v>1610000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2188332</v>
+        <v>2188213</v>
       </c>
       <c r="L72" t="n">
-        <v>26.42798259130699</v>
+        <v>26.42398157766177</v>
       </c>
       <c r="M72" s="3" t="n">
         <v>0</v>
@@ -5727,10 +5727,10 @@
         <v>1615000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2188332</v>
+        <v>2188213</v>
       </c>
       <c r="L73" t="n">
-        <v>26.19949806519303</v>
+        <v>26.1954846260396</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
@@ -5791,10 +5791,10 @@
         <v>1630000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2231249</v>
+        <v>2231127</v>
       </c>
       <c r="L74" t="n">
-        <v>26.9467459705304</v>
+        <v>26.94275135391217</v>
       </c>
       <c r="M74" s="3" t="n">
         <v>0</v>
@@ -5855,10 +5855,10 @@
         <v>1690000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2317083</v>
+        <v>2316956</v>
       </c>
       <c r="L75" t="n">
-        <v>27.06346729918609</v>
+        <v>27.05946940727403</v>
       </c>
       <c r="M75" s="3" t="n">
         <v>0</v>
@@ -5919,10 +5919,10 @@
         <v>1705000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2317083</v>
+        <v>2316956</v>
       </c>
       <c r="L76" t="n">
-        <v>26.41610162432679</v>
+        <v>26.41206824816699</v>
       </c>
       <c r="M76" s="3" t="n">
         <v>0</v>
@@ -5983,10 +5983,10 @@
         <v>1725000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2360000</v>
+        <v>2359871</v>
       </c>
       <c r="L77" t="n">
-        <v>26.90677966101695</v>
+        <v>26.90278409285931</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
@@ -6047,10 +6047,10 @@
         <v>1780000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2445834</v>
+        <v>2445700</v>
       </c>
       <c r="L78" t="n">
-        <v>27.22318849112409</v>
+        <v>27.21920104673509</v>
       </c>
       <c r="M78" s="3" t="n">
         <v>0</v>
@@ -6111,10 +6111,10 @@
         <v>1875000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2574584</v>
+        <v>2574443</v>
       </c>
       <c r="L79" t="n">
-        <v>27.17270052171535</v>
+        <v>27.16871183397729</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
@@ -6175,10 +6175,10 @@
         <v>1910000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2617501</v>
+        <v>2617358</v>
       </c>
       <c r="L80" t="n">
-        <v>27.02963628285147</v>
+        <v>27.02564952902889</v>
       </c>
       <c r="M80" s="3" t="n">
         <v>0</v>
@@ -6239,10 +6239,10 @@
         <v>2020000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2746252</v>
+        <v>2746102</v>
       </c>
       <c r="L81" t="n">
-        <v>26.44520604809755</v>
+        <v>26.44118827341446</v>
       </c>
       <c r="M81" s="3" t="n">
         <v>0</v>
@@ -6303,10 +6303,10 @@
         <v>2110000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>2875003</v>
+        <v>2874845</v>
       </c>
       <c r="L82" t="n">
-        <v>26.60877223432462</v>
+        <v>26.60473869025982</v>
       </c>
       <c r="M82" s="3" t="n">
         <v>0</v>
@@ -6367,10 +6367,10 @@
         <v>2210000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3003753</v>
+        <v>3003589</v>
       </c>
       <c r="L83" t="n">
-        <v>26.42537518897193</v>
+        <v>26.42135791548045</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
@@ -6431,10 +6431,10 @@
         <v>2215000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3046670</v>
+        <v>3046503</v>
       </c>
       <c r="L84" t="n">
-        <v>27.29767254083967</v>
+        <v>27.29368722105312</v>
       </c>
       <c r="M84" s="3" t="n">
         <v>0</v>
@@ -6495,10 +6495,10 @@
         <v>2315000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3175421</v>
+        <v>3175247</v>
       </c>
       <c r="L85" t="n">
-        <v>27.0962810915466</v>
+        <v>27.09228604892785</v>
       </c>
       <c r="M85" s="3" t="n">
         <v>0</v>
@@ -6559,10 +6559,10 @@
         <v>2395000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3304171</v>
+        <v>3303991</v>
       </c>
       <c r="L86" t="n">
-        <v>27.51585798676884</v>
+        <v>27.5119090820768</v>
       </c>
       <c r="M86" s="3" t="n">
         <v>0</v>
@@ -6623,10 +6623,10 @@
         <v>2410000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3304171</v>
+        <v>3303991</v>
       </c>
       <c r="L87" t="n">
-        <v>27.06188632489057</v>
+        <v>27.05791268801882</v>
       </c>
       <c r="M87" s="3" t="n">
         <v>0</v>
@@ -6687,10 +6687,10 @@
         <v>2499000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3432922</v>
+        <v>3432734</v>
       </c>
       <c r="L88" t="n">
-        <v>27.20487095250052</v>
+        <v>27.20088419318246</v>
       </c>
       <c r="M88" s="3" t="n">
         <v>0</v>
@@ -6751,10 +6751,10 @@
         <v>2510000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3432922</v>
+        <v>3432734</v>
       </c>
       <c r="L89" t="n">
-        <v>26.88444421399612</v>
+        <v>26.88043990591756</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
@@ -6815,10 +6815,10 @@
         <v>2530000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3475839</v>
+        <v>3475649</v>
       </c>
       <c r="L90" t="n">
-        <v>27.21181849907317</v>
+        <v>27.20783945674606</v>
       </c>
       <c r="M90" s="3" t="n">
         <v>0</v>
@@ -6879,10 +6879,10 @@
         <v>2610000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>3604590</v>
+        <v>3604393</v>
       </c>
       <c r="L91" t="n">
-        <v>27.59231979226486</v>
+        <v>27.58836231232277</v>
       </c>
       <c r="M91" s="3" t="n">
         <v>0</v>
@@ -6943,10 +6943,10 @@
         <v>3015000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4162509</v>
+        <v>4162282</v>
       </c>
       <c r="L92" t="n">
-        <v>27.56772417789367</v>
+        <v>27.56377391056156</v>
       </c>
       <c r="M92" s="3" t="n">
         <v>0</v>
@@ -7007,10 +7007,10 @@
         <v>3098000</v>
       </c>
       <c r="K93" s="3" t="n">
-        <v>4291260</v>
+        <v>4291025</v>
       </c>
       <c r="L93" t="n">
-        <v>27.80675139702558</v>
+        <v>27.80279769985027</v>
       </c>
       <c r="M93" s="3" t="n">
         <v>0</v>
@@ -7306,10 +7306,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>428740</v>
+        <v>428716</v>
       </c>
       <c r="L2" t="n">
-        <v>27.69533983299902</v>
+        <v>27.6912921374523</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7373,10 +7373,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>428740</v>
+        <v>428716</v>
       </c>
       <c r="L3" t="n">
-        <v>27.69533983299902</v>
+        <v>27.6912921374523</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7440,10 +7440,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>428740</v>
+        <v>428716</v>
       </c>
       <c r="L4" t="n">
-        <v>27.69510659140738</v>
+        <v>27.69105888280353</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7507,10 +7507,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>428740</v>
+        <v>428716</v>
       </c>
       <c r="L5" t="n">
-        <v>27.69510659140738</v>
+        <v>27.69105888280353</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7574,10 +7574,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514574</v>
+        <v>514545</v>
       </c>
       <c r="L6" t="n">
-        <v>25.37516469934353</v>
+        <v>25.3709588082675</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7638,10 +7638,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>514574</v>
+        <v>514545</v>
       </c>
       <c r="L7" t="n">
-        <v>25.37516469934353</v>
+        <v>25.3709588082675</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7702,10 +7702,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>514574</v>
+        <v>514545</v>
       </c>
       <c r="L8" t="n">
-        <v>25.37516469934353</v>
+        <v>25.3709588082675</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7766,10 +7766,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>514574</v>
+        <v>514545</v>
       </c>
       <c r="L9" t="n">
-        <v>25.37516469934353</v>
+        <v>25.3709588082675</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7830,10 +7830,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>514574</v>
+        <v>514545</v>
       </c>
       <c r="L10" t="n">
-        <v>25.18082919074808</v>
+        <v>25.17661234683069</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7894,10 +7894,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>514574</v>
+        <v>514545</v>
       </c>
       <c r="L11" t="n">
-        <v>25.18082919074808</v>
+        <v>25.17661234683069</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7958,10 +7958,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>514574</v>
+        <v>514545</v>
       </c>
       <c r="L12" t="n">
-        <v>25.18082919074808</v>
+        <v>25.17661234683069</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -8022,10 +8022,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>514574</v>
+        <v>514545</v>
       </c>
       <c r="L13" t="n">
-        <v>25.18082919074808</v>
+        <v>25.17661234683069</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -8086,16 +8086,16 @@
         <v>415000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>557490</v>
+        <v>557460</v>
       </c>
       <c r="L14" t="n">
-        <v>25.5592028556566</v>
+        <v>25.55519678541958</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>2.007083825265644</v>
+        <v>1.658767772511848</v>
       </c>
       <c r="O14" t="n">
         <v>100</v>
@@ -8104,7 +8104,7 @@
         <v>3.478260869565196</v>
       </c>
       <c r="Q14" t="n">
-        <v>31.9</v>
+        <v>31.8</v>
       </c>
       <c r="R14" t="n">
         <v>4</v>
@@ -8153,16 +8153,16 @@
         <v>415000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>557490</v>
+        <v>557460</v>
       </c>
       <c r="L15" t="n">
-        <v>25.5592028556566</v>
+        <v>25.55519678541958</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>2.007083825265644</v>
+        <v>1.658767772511848</v>
       </c>
       <c r="O15" t="n">
         <v>100</v>
@@ -8171,7 +8171,7 @@
         <v>3.478260869565196</v>
       </c>
       <c r="Q15" t="n">
-        <v>31.9</v>
+        <v>31.8</v>
       </c>
       <c r="R15" t="n">
         <v>4</v>
@@ -8220,16 +8220,16 @@
         <v>415000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>557490</v>
+        <v>557460</v>
       </c>
       <c r="L16" t="n">
-        <v>25.5592028556566</v>
+        <v>25.55519678541958</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>2.007083825265644</v>
+        <v>1.658767772511848</v>
       </c>
       <c r="O16" t="n">
         <v>100</v>
@@ -8238,7 +8238,7 @@
         <v>3.478260869565196</v>
       </c>
       <c r="Q16" t="n">
-        <v>31.9</v>
+        <v>31.8</v>
       </c>
       <c r="R16" t="n">
         <v>4</v>
@@ -8287,10 +8287,10 @@
         <v>420000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>557490</v>
+        <v>557460</v>
       </c>
       <c r="L17" t="n">
-        <v>24.66232578162837</v>
+        <v>24.65827144548488</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -8354,10 +8354,10 @@
         <v>454000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>600407</v>
+        <v>600374</v>
       </c>
       <c r="L18" t="n">
-        <v>24.38462576219131</v>
+        <v>24.38046950734043</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -8418,10 +8418,10 @@
         <v>454000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>600407</v>
+        <v>600374</v>
       </c>
       <c r="L19" t="n">
-        <v>24.38462576219131</v>
+        <v>24.38046950734043</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -8482,10 +8482,10 @@
         <v>454000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>600407</v>
+        <v>600374</v>
       </c>
       <c r="L20" t="n">
-        <v>24.38462576219131</v>
+        <v>24.38046950734043</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -8546,10 +8546,10 @@
         <v>454000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>600407</v>
+        <v>600374</v>
       </c>
       <c r="L21" t="n">
-        <v>24.38462576219131</v>
+        <v>24.38046950734043</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -8610,10 +8610,10 @@
         <v>455000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>600407</v>
+        <v>600374</v>
       </c>
       <c r="L22" t="n">
-        <v>24.21807207444284</v>
+        <v>24.21390666484558</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -8674,10 +8674,10 @@
         <v>455000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>600407</v>
+        <v>600374</v>
       </c>
       <c r="L23" t="n">
-        <v>24.21807207444284</v>
+        <v>24.21390666484558</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -8738,10 +8738,10 @@
         <v>455000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>600407</v>
+        <v>600374</v>
       </c>
       <c r="L24" t="n">
-        <v>24.21807207444284</v>
+        <v>24.21390666484558</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -8802,10 +8802,10 @@
         <v>455000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>600407</v>
+        <v>600374</v>
       </c>
       <c r="L25" t="n">
-        <v>24.21807207444284</v>
+        <v>24.21390666484558</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -8866,10 +8866,10 @@
         <v>468000</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>686241</v>
+        <v>686204</v>
       </c>
       <c r="L26" t="n">
-        <v>31.80238429356451</v>
+        <v>31.79870709001988</v>
       </c>
       <c r="M26" s="3" t="n">
         <v>0</v>
@@ -8930,10 +8930,10 @@
         <v>468000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>686241</v>
+        <v>686204</v>
       </c>
       <c r="L27" t="n">
-        <v>31.80238429356451</v>
+        <v>31.79870709001988</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -8994,10 +8994,10 @@
         <v>468000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>686241</v>
+        <v>686204</v>
       </c>
       <c r="L28" t="n">
-        <v>31.80238429356451</v>
+        <v>31.79870709001988</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -9058,10 +9058,10 @@
         <v>468000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>686241</v>
+        <v>686204</v>
       </c>
       <c r="L29" t="n">
-        <v>31.80238429356451</v>
+        <v>31.79870709001988</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -9122,13 +9122,13 @@
         <v>474999</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>643324</v>
+        <v>643289</v>
       </c>
       <c r="L30" t="n">
-        <v>26.16488736624159</v>
+        <v>26.16087015322818</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>-5000</v>
+        <v>0</v>
       </c>
       <c r="N30" t="n">
         <v>2.061859921360663</v>
@@ -9189,13 +9189,13 @@
         <v>475000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>643324</v>
+        <v>643289</v>
       </c>
       <c r="L31" t="n">
-        <v>26.16473192357195</v>
+        <v>26.16071470210123</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>-2000</v>
+        <v>0</v>
       </c>
       <c r="N31" t="n">
         <v>1.041460503042715</v>
@@ -9256,13 +9256,13 @@
         <v>475000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>643324</v>
+        <v>643289</v>
       </c>
       <c r="L32" t="n">
-        <v>26.16473192357195</v>
+        <v>26.16071470210123</v>
       </c>
       <c r="M32" s="3" t="n">
-        <v>-2000</v>
+        <v>0</v>
       </c>
       <c r="N32" t="n">
         <v>1.041460503042715</v>
@@ -9323,13 +9323,13 @@
         <v>475000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>643324</v>
+        <v>643289</v>
       </c>
       <c r="L33" t="n">
-        <v>26.16473192357195</v>
+        <v>26.16071470210123</v>
       </c>
       <c r="M33" s="3" t="n">
-        <v>-2000</v>
+        <v>0</v>
       </c>
       <c r="N33" t="n">
         <v>1.041460503042715</v>
@@ -9390,10 +9390,10 @@
         <v>475000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>686241</v>
+        <v>686204</v>
       </c>
       <c r="L34" t="n">
-        <v>30.78233448598962</v>
+        <v>30.77860228153727</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -9454,10 +9454,10 @@
         <v>475000</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>686241</v>
+        <v>686204</v>
       </c>
       <c r="L35" t="n">
-        <v>30.78233448598962</v>
+        <v>30.77860228153727</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
@@ -9518,10 +9518,10 @@
         <v>475000</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>686241</v>
+        <v>686204</v>
       </c>
       <c r="L36" t="n">
-        <v>30.78233448598962</v>
+        <v>30.77860228153727</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -9582,10 +9582,10 @@
         <v>475000</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>686241</v>
+        <v>686204</v>
       </c>
       <c r="L37" t="n">
-        <v>30.78233448598962</v>
+        <v>30.77860228153727</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
@@ -9646,10 +9646,10 @@
         <v>500000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>643324</v>
+        <v>643289</v>
       </c>
       <c r="L38" t="n">
-        <v>22.27866518270731</v>
+        <v>22.27443652852761</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -9710,16 +9710,16 @@
         <v>544999</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>772075</v>
+        <v>772033</v>
       </c>
       <c r="L39" t="n">
-        <v>29.41113233817958</v>
+        <v>29.40729217533448</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N39" t="n">
-        <v>0.7285987770469528</v>
+        <v>0.547446254463968</v>
       </c>
       <c r="P39" t="n">
         <v>64.69606956521737</v>
@@ -9774,16 +9774,16 @@
         <v>544999</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>772075</v>
+        <v>772033</v>
       </c>
       <c r="L40" t="n">
-        <v>29.41113233817958</v>
+        <v>29.40729217533448</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N40" t="n">
-        <v>0.7285987770469528</v>
+        <v>0.547446254463968</v>
       </c>
       <c r="P40" t="n">
         <v>64.69606956521737</v>
@@ -9838,22 +9838,22 @@
         <v>544999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>772075</v>
+        <v>772033</v>
       </c>
       <c r="L41" t="n">
-        <v>29.41113233817958</v>
+        <v>29.40729217533448</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N41" t="n">
-        <v>0.9090925619864764</v>
+        <v>0.547446254463968</v>
       </c>
       <c r="P41" t="n">
         <v>64.69606956521737</v>
       </c>
       <c r="Q41" t="n">
-        <v>26.8</v>
+        <v>26.7</v>
       </c>
       <c r="R41" t="n">
         <v>3</v>
@@ -9902,16 +9902,16 @@
         <v>544999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>772075</v>
+        <v>772033</v>
       </c>
       <c r="L42" t="n">
-        <v>29.41113233817958</v>
+        <v>29.40729217533448</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N42" t="n">
-        <v>0.7285987770469528</v>
+        <v>0.547446254463968</v>
       </c>
       <c r="P42" t="n">
         <v>64.69606956521737</v>
@@ -9966,22 +9966,22 @@
         <v>549999</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>772075</v>
+        <v>772033</v>
       </c>
       <c r="L43" t="n">
-        <v>28.76352685943723</v>
+        <v>28.75965146567569</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>1.168016474423135</v>
+        <v>0.5424964602105971</v>
       </c>
       <c r="P43" t="n">
         <v>33.55744966442954</v>
       </c>
       <c r="Q43" t="n">
-        <v>19.9</v>
+        <v>19.7</v>
       </c>
       <c r="R43" t="n">
         <v>3</v>
@@ -10030,22 +10030,22 @@
         <v>549999</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>772075</v>
+        <v>772033</v>
       </c>
       <c r="L44" t="n">
-        <v>28.76352685943723</v>
+        <v>28.75965146567569</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>1.168016474423135</v>
+        <v>0.5424964602105971</v>
       </c>
       <c r="P44" t="n">
         <v>33.55744966442954</v>
       </c>
       <c r="Q44" t="n">
-        <v>19.9</v>
+        <v>19.7</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -10094,22 +10094,22 @@
         <v>549999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>772075</v>
+        <v>772033</v>
       </c>
       <c r="L45" t="n">
-        <v>28.76352685943723</v>
+        <v>28.75965146567569</v>
       </c>
       <c r="M45" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>1.168016474423135</v>
+        <v>0.5424964602105971</v>
       </c>
       <c r="P45" t="n">
         <v>33.55744966442954</v>
       </c>
       <c r="Q45" t="n">
-        <v>19.9</v>
+        <v>19.7</v>
       </c>
       <c r="R45" t="n">
         <v>3</v>
@@ -10158,22 +10158,22 @@
         <v>549999</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>772075</v>
+        <v>772033</v>
       </c>
       <c r="L46" t="n">
-        <v>28.76352685943723</v>
+        <v>28.75965146567569</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N46" t="n">
-        <v>1.168016474423135</v>
+        <v>0.5424964602105971</v>
       </c>
       <c r="P46" t="n">
         <v>33.55744966442954</v>
       </c>
       <c r="Q46" t="n">
-        <v>19.9</v>
+        <v>19.7</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -10222,10 +10222,10 @@
         <v>585000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>729158</v>
+        <v>729118</v>
       </c>
       <c r="L47" t="n">
-        <v>19.77047498621698</v>
+        <v>19.76607352993617</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -10286,10 +10286,10 @@
         <v>595000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>729158</v>
+        <v>729118</v>
       </c>
       <c r="L48" t="n">
-        <v>18.3990301141865</v>
+        <v>18.39455341933679</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -10350,10 +10350,10 @@
         <v>619999</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>857909</v>
+        <v>857862</v>
       </c>
       <c r="L49" t="n">
-        <v>27.73137943534804</v>
+        <v>27.7274200279299</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -10414,10 +10414,10 @@
         <v>619999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>857909</v>
+        <v>857862</v>
       </c>
       <c r="L50" t="n">
-        <v>27.73137943534804</v>
+        <v>27.7274200279299</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -10478,10 +10478,10 @@
         <v>619999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>857909</v>
+        <v>857862</v>
       </c>
       <c r="L51" t="n">
-        <v>27.73137943534804</v>
+        <v>27.7274200279299</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -10542,10 +10542,10 @@
         <v>619999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>857909</v>
+        <v>857862</v>
       </c>
       <c r="L52" t="n">
-        <v>27.73137943534804</v>
+        <v>27.7274200279299</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -10606,10 +10606,10 @@
         <v>650000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>814992</v>
+        <v>814947</v>
       </c>
       <c r="L53" t="n">
-        <v>20.24461589807017</v>
+        <v>20.24021194016298</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -10670,10 +10670,10 @@
         <v>672000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>857909</v>
+        <v>857862</v>
       </c>
       <c r="L54" t="n">
-        <v>21.67001395252877</v>
+        <v>21.66572245885702</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -10734,10 +10734,10 @@
         <v>700000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>900826</v>
+        <v>900776</v>
       </c>
       <c r="L55" t="n">
-        <v>22.29353948487277</v>
+        <v>22.28922617831736</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -10798,10 +10798,10 @@
         <v>715000</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>943742</v>
+        <v>943691</v>
       </c>
       <c r="L56" t="n">
-        <v>24.23776837313588</v>
+        <v>24.23367394623876</v>
       </c>
       <c r="M56" s="3" t="n">
         <v>0</v>
@@ -10862,10 +10862,10 @@
         <v>734999</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>986659</v>
+        <v>986605</v>
       </c>
       <c r="L57" t="n">
-        <v>25.50627927176461</v>
+        <v>25.50220199573284</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -10926,10 +10926,10 @@
         <v>752000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>986659</v>
+        <v>986605</v>
       </c>
       <c r="L58" t="n">
-        <v>23.78319155858306</v>
+        <v>23.77901997253207</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -10990,10 +10990,10 @@
         <v>810000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1072493</v>
+        <v>1072434</v>
       </c>
       <c r="L59" t="n">
-        <v>24.47503153866738</v>
+        <v>24.47087652946475</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -11054,10 +11054,10 @@
         <v>815000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1072493</v>
+        <v>1072434</v>
       </c>
       <c r="L60" t="n">
-        <v>24.00882802964681</v>
+        <v>24.00464737223922</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -11118,10 +11118,10 @@
         <v>875000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1158327</v>
+        <v>1158264</v>
       </c>
       <c r="L61" t="n">
-        <v>24.46001863031769</v>
+        <v>24.45590987892225</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -11182,10 +11182,10 @@
         <v>992000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1329994</v>
+        <v>1329922</v>
       </c>
       <c r="L62" t="n">
-        <v>25.41319735277001</v>
+        <v>25.40915933415644</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -11246,10 +11246,10 @@
         <v>1050000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1415828</v>
+        <v>1415751</v>
       </c>
       <c r="L63" t="n">
-        <v>25.83844930316395</v>
+        <v>25.83441579769324</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -11310,10 +11310,10 @@
         <v>1050000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1415828</v>
+        <v>1415751</v>
       </c>
       <c r="L64" t="n">
-        <v>25.83844930316395</v>
+        <v>25.83441579769324</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -11374,10 +11374,10 @@
         <v>1100000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1501662</v>
+        <v>1501580</v>
       </c>
       <c r="L65" t="n">
-        <v>26.74783007094806</v>
+        <v>26.74382983257636</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -11438,10 +11438,10 @@
         <v>1105000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1501662</v>
+        <v>1501580</v>
       </c>
       <c r="L66" t="n">
-        <v>26.41486566217964</v>
+        <v>26.41084724090624</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -11502,10 +11502,10 @@
         <v>1155000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1587496</v>
+        <v>1587409</v>
       </c>
       <c r="L67" t="n">
-        <v>27.24391116576042</v>
+        <v>27.23992367436496</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -11626,7 +11626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S14"/>
+  <dimension ref="A1:S17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -11772,7 +11772,7 @@
         <v>315000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>299989</v>
+        <v>299973</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -11833,10 +11833,10 @@
         <v>380000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>385823</v>
+        <v>385802</v>
       </c>
       <c r="L3" t="n">
-        <v>1.509241284215819</v>
+        <v>1.503880228718358</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -11897,7 +11897,7 @@
         <v>415000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>385823</v>
+        <v>385802</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -11958,10 +11958,10 @@
         <v>495000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>471657</v>
+        <v>471631</v>
       </c>
       <c r="L5" t="n">
-        <v>6.712081024982138</v>
+        <v>6.706938263176085</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -12022,10 +12022,10 @@
         <v>490000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514574</v>
+        <v>514545</v>
       </c>
       <c r="L6" t="n">
-        <v>4.775600788224823</v>
+        <v>4.77023389596634</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -12086,10 +12086,10 @@
         <v>550000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>557490</v>
+        <v>557460</v>
       </c>
       <c r="L7" t="n">
-        <v>6.724784301063696</v>
+        <v>6.719764646790802</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -12150,7 +12150,7 @@
         <v>530000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>471657</v>
+        <v>471631</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -12214,10 +12214,10 @@
         <v>600000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>600407</v>
+        <v>600374</v>
       </c>
       <c r="L9" t="n">
-        <v>8.395471738337495</v>
+        <v>8.390436627835316</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -12243,86 +12243,78 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Apple Iphone Air 1TB</t>
+          <t>Apple iPhone 18 Pro 256GB Burgundy</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>6.5</v>
+        <v>6.3</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Apple A19 Pro</t>
+          <t>A20 Pro chip</t>
         </is>
       </c>
       <c r="D10" t="n">
         <v>12</v>
       </c>
       <c r="E10" t="n">
-        <v>1024</v>
+        <v>256</v>
       </c>
       <c r="F10" t="n">
         <v>6</v>
       </c>
       <c r="G10" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Space Black, Cloud White, Light Gold, Sky Blue</t>
+          <t>Black, Silver, Glacier, Burgundy</t>
         </is>
       </c>
       <c r="I10" s="3" t="n">
-        <v>604999</v>
+        <v>590000</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>646000</v>
+        <v>590000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>729158</v>
+        <v>514545</v>
       </c>
       <c r="L10" t="n">
-        <v>17.02772238664322</v>
-      </c>
-      <c r="M10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" t="n">
-        <v>100</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M10" s="3" t="n"/>
       <c r="Q10" t="n">
-        <v>25.9</v>
+        <v>0</v>
       </c>
       <c r="R10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>2026-09-16T00:22:18.878661+00:00</t>
+          <t>2026-10-11T10:05:09.295831+00:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Apple Iphone 17 Pro 512GB</t>
+          <t>Apple Iphone Air 1TB</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>6.3</v>
+        <v>6.5</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>A19 Pro</t>
+          <t>Apple A19 Pro</t>
         </is>
       </c>
       <c r="D11" t="n">
         <v>12</v>
       </c>
       <c r="E11" t="n">
-        <v>512</v>
+        <v>1024</v>
       </c>
       <c r="F11" t="n">
         <v>6</v>
@@ -12332,20 +12324,20 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Silver, Cosmic Orange, Deep Blue</t>
+          <t>Space Black, Cloud White, Light Gold, Sky Blue</t>
         </is>
       </c>
       <c r="I11" s="3" t="n">
-        <v>608500</v>
+        <v>604999</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>615000</v>
+        <v>646000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>557490</v>
+        <v>729118</v>
       </c>
       <c r="L11" t="n">
-        <v>0</v>
+        <v>17.02317046074847</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -12354,10 +12346,10 @@
         <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>29.68767123287672</v>
+        <v>100</v>
       </c>
       <c r="Q11" t="n">
-        <v>5.7</v>
+        <v>25.9</v>
       </c>
       <c r="R11" t="n">
         <v>4</v>
@@ -12371,7 +12363,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Apple Iphone 17 Pro 1TB</t>
+          <t>Apple Iphone 17 Pro 512GB</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -12386,7 +12378,7 @@
         <v>12</v>
       </c>
       <c r="E12" t="n">
-        <v>1024</v>
+        <v>512</v>
       </c>
       <c r="F12" t="n">
         <v>6</v>
@@ -12400,13 +12392,13 @@
         </is>
       </c>
       <c r="I12" s="3" t="n">
-        <v>691500</v>
+        <v>608500</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>700000</v>
+        <v>615000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>643324</v>
+        <v>557460</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -12418,10 +12410,10 @@
         <v>0</v>
       </c>
       <c r="P12" t="n">
-        <v>100</v>
+        <v>29.68767123287672</v>
       </c>
       <c r="Q12" t="n">
-        <v>18.9</v>
+        <v>5.7</v>
       </c>
       <c r="R12" t="n">
         <v>4</v>
@@ -12435,7 +12427,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Apple iphone 17 Pro Max 1TB</t>
+          <t>Apple iPhone 18 Pro Max 256GB Burgundy</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -12443,67 +12435,62 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>A19 Pro</t>
+          <t>A20 Pro chip</t>
         </is>
       </c>
       <c r="D13" t="n">
         <v>12</v>
       </c>
       <c r="E13" t="n">
-        <v>1024</v>
+        <v>256</v>
       </c>
       <c r="F13" t="n">
         <v>6</v>
       </c>
       <c r="G13" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Silver, Cosmic Orange, Deep Blue</t>
+          <t>Black, Silver, Glacier, Burgundy</t>
         </is>
       </c>
       <c r="I13" s="3" t="n">
-        <v>740000</v>
+        <v>655000</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>745000</v>
+        <v>655000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>686241</v>
+        <v>557460</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
       </c>
-      <c r="M13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" t="n">
-        <v>0</v>
-      </c>
+      <c r="M13" s="3" t="n"/>
       <c r="P13" t="n">
-        <v>40.62540173571834</v>
+        <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>7.7</v>
+        <v>0</v>
       </c>
       <c r="R13" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>2026-09-16T00:22:18.878661+00:00</t>
+          <t>2026-10-11T10:05:09.295831+00:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Apple iphone 17 Pro Max 2TB</t>
+          <t>Apple Iphone 17 Pro 1TB</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>6.9</v>
+        <v>6.3</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -12514,7 +12501,7 @@
         <v>12</v>
       </c>
       <c r="E14" t="n">
-        <v>2048</v>
+        <v>1024</v>
       </c>
       <c r="F14" t="n">
         <v>6</v>
@@ -12528,13 +12515,13 @@
         </is>
       </c>
       <c r="I14" s="3" t="n">
-        <v>892999</v>
+        <v>691500</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>930000</v>
+        <v>700000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>857909</v>
+        <v>643289</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -12549,7 +12536,7 @@
         <v>100</v>
       </c>
       <c r="Q14" t="n">
-        <v>19.2</v>
+        <v>18.9</v>
       </c>
       <c r="R14" t="n">
         <v>4</v>
@@ -12560,9 +12547,196 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Apple iphone 17 Pro Max 1TB</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>A19 Pro</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>12</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1024</v>
+      </c>
+      <c r="F15" t="n">
+        <v>6</v>
+      </c>
+      <c r="G15" t="n">
+        <v>5</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Silver, Cosmic Orange, Deep Blue</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>740000</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>745000</v>
+      </c>
+      <c r="K15" s="3" t="n">
+        <v>686204</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="n">
+        <v>40.62540173571834</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="R15" t="n">
+        <v>4</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>2026-09-16T00:22:18.878661+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Apple iPhone 18 Pro Max 512GB Glacier</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>A20 Pro chip</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>12</v>
+      </c>
+      <c r="E16" t="n">
+        <v>512</v>
+      </c>
+      <c r="F16" t="n">
+        <v>6</v>
+      </c>
+      <c r="G16" t="n">
+        <v>7</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Black, Silver, Glacier, Burgundy</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>755000</v>
+      </c>
+      <c r="J16" s="3" t="n">
+        <v>755000</v>
+      </c>
+      <c r="K16" s="3" t="n">
+        <v>643289</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="3" t="n"/>
+      <c r="P16" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="R16" t="n">
+        <v>2</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>2026-10-11T10:05:09.295831+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Apple iphone 17 Pro Max 2TB</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>A19 Pro</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>12</v>
+      </c>
+      <c r="E17" t="n">
+        <v>2048</v>
+      </c>
+      <c r="F17" t="n">
+        <v>6</v>
+      </c>
+      <c r="G17" t="n">
+        <v>5</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Silver, Cosmic Orange, Deep Blue</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="n">
+        <v>892999</v>
+      </c>
+      <c r="J17" s="3" t="n">
+        <v>930000</v>
+      </c>
+      <c r="K17" s="3" t="n">
+        <v>857862</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="R17" t="n">
+        <v>4</v>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>2026-09-16T00:22:18.878661+00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S14"/>
-  <conditionalFormatting sqref="Q2:Q14">
+  <autoFilter ref="A1:S17"/>
+  <conditionalFormatting sqref="Q2:Q17">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -12572,7 +12746,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M2:M14">
+  <conditionalFormatting sqref="M2:M17">
     <cfRule type="cellIs" priority="2" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -12594,6 +12768,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12605,7 +12782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12654,7 +12831,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MDV94 M5 10C CPU 10C GPU 16GB 512GB Silver</t>
+          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 64GB 1TB Silver</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -12663,141 +12840,45 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>479999</v>
+        <v>1300000</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>474999</v>
+        <v>1255000</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-5000</v>
+        <v>-45000</v>
       </c>
       <c r="F2" t="n">
-        <v>-1.04</v>
+        <v>-3.46</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 MGEA4 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Space Black</t>
+          <t>Apple MacBook Pro 14Inch MW2W3 M4 10Core CPU 10Core GPU 16GB 512GB Silver</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>823000</v>
+        <v>445000</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>820000</v>
+        <v>498000</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>-3000</v>
+        <v>53000</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.36</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Macbook Pro 16 MGE44 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Silver</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>822999</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>820000</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>-2999</v>
-      </c>
-      <c r="F4" t="n">
-        <v>-0.36</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDVD4 M5 10C CPU 10C GPU 16GB 512GB Starlight</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>477000</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>475000</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>-2000</v>
-      </c>
-      <c r="F5" t="n">
-        <v>-0.42</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDVQ4 M5 10C CPU 10C GPU 16GB 512GB Sky Blue</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>477000</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>475000</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>-2000</v>
-      </c>
-      <c r="F6" t="n">
-        <v>-0.42</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Apple MacBook Air 15 MDVH4 M5 10C CPU 10C GPU 16GB 512GB Midnight</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>477000</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>475000</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>-2000</v>
-      </c>
-      <c r="F7" t="n">
-        <v>-0.42</v>
+        <v>11.91</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F7"/>
-  <conditionalFormatting sqref="E2:E7">
+  <autoFilter ref="A1:F3"/>
+  <conditionalFormatting sqref="E2:E3">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
chore: price data 2026-10-12
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MacBook Pro'!$A$1:$S$93</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MacBook Air'!$A$1:$S$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20261011T100509295831+0000</t>
+          <t>20261012T105752620082+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-11T10:05:09.295831+00:00</t>
+          <t>2026-10-12T10:57:52.620082+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>276.868026</v>
+        <v>277.205784</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -1147,10 +1147,10 @@
         <v>495000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>686204</v>
+        <v>687041</v>
       </c>
       <c r="L2" t="n">
-        <v>27.8640171144441</v>
+        <v>27.95189806721869</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1214,13 +1214,13 @@
         <v>498000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>686204</v>
+        <v>687041</v>
       </c>
       <c r="L3" t="n">
-        <v>27.42682933938013</v>
+        <v>27.51524290398972</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>53000</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
         <v>0</v>
@@ -1232,7 +1232,7 @@
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>9.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="R3" t="n">
         <v>4</v>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>772033</v>
+        <v>772974</v>
       </c>
       <c r="L4" t="n">
-        <v>35.23605856226353</v>
+        <v>35.31490063055161</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>772033</v>
+        <v>772974</v>
       </c>
       <c r="L5" t="n">
-        <v>32.64549572362839</v>
+        <v>32.72749148095537</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>857862</v>
+        <v>858908</v>
       </c>
       <c r="L6" t="n">
-        <v>37.98536361326181</v>
+        <v>38.0608866141659</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1606,10 +1606,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>857862</v>
+        <v>858908</v>
       </c>
       <c r="L9" t="n">
-        <v>34.13859105543782</v>
+        <v>34.21879875376641</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1673,10 +1673,10 @@
         <v>578999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>857862</v>
+        <v>858908</v>
       </c>
       <c r="L10" t="n">
-        <v>32.50674350886273</v>
+        <v>32.588938512623</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -1691,7 +1691,7 @@
         <v>50.30029999999999</v>
       </c>
       <c r="Q10" t="n">
-        <v>41.6</v>
+        <v>41.7</v>
       </c>
       <c r="R10" t="n">
         <v>4</v>
@@ -1740,10 +1740,10 @@
         <v>584999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>857862</v>
+        <v>858908</v>
       </c>
       <c r="L11" t="n">
-        <v>31.8073303165311</v>
+        <v>31.89037708345947</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -1758,7 +1758,7 @@
         <v>48.50029999999999</v>
       </c>
       <c r="Q11" t="n">
-        <v>18.8</v>
+        <v>18.9</v>
       </c>
       <c r="R11" t="n">
         <v>4</v>
@@ -1807,22 +1807,22 @@
         <v>634000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>857862</v>
+        <v>858908</v>
       </c>
       <c r="L12" t="n">
-        <v>26.09533934362404</v>
+        <v>26.18534231838567</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>0.9375</v>
+        <v>0.4709576138147566</v>
       </c>
       <c r="P12" t="n">
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>11.5</v>
+        <v>11.4</v>
       </c>
       <c r="R12" t="n">
         <v>3</v>
@@ -1871,10 +1871,10 @@
         <v>634000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>857862</v>
+        <v>858908</v>
       </c>
       <c r="L13" t="n">
-        <v>26.09533934362404</v>
+        <v>26.18534231838567</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -1935,10 +1935,10 @@
         <v>642999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>943691</v>
+        <v>944842</v>
       </c>
       <c r="L14" t="n">
-        <v>31.86339596329731</v>
+        <v>31.94639950383239</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -2061,10 +2061,10 @@
         <v>650000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>943691</v>
+        <v>944842</v>
       </c>
       <c r="L16" t="n">
-        <v>31.12152176930796</v>
+        <v>31.20542905586331</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -2128,10 +2128,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1029520</v>
+        <v>1030776</v>
       </c>
       <c r="L17" t="n">
-        <v>32.00714896262336</v>
+        <v>32.08999821493709</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2195,10 +2195,10 @@
         <v>711999</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>1072434</v>
+        <v>1073743</v>
       </c>
       <c r="L18" t="n">
-        <v>33.60906125691651</v>
+        <v>33.689998444693</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -2324,10 +2324,10 @@
         <v>720000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>1029520</v>
+        <v>1030776</v>
       </c>
       <c r="L20" t="n">
-        <v>30.06449607584117</v>
+        <v>30.14971244964958</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -2453,10 +2453,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1072434</v>
+        <v>1073743</v>
       </c>
       <c r="L22" t="n">
-        <v>30.7183472362868</v>
+        <v>30.80280849328005</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2471,7 +2471,7 @@
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>10.2</v>
+        <v>10.3</v>
       </c>
       <c r="R22" t="n">
         <v>4</v>
@@ -2520,16 +2520,16 @@
         <v>759999</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1029520</v>
+        <v>1030776</v>
       </c>
       <c r="L23" t="n">
-        <v>26.17928743492113</v>
+        <v>26.26923793336283</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>1.554533678756477</v>
+        <v>1.426784323465839</v>
       </c>
       <c r="O23" t="n">
         <v>100</v>
@@ -2587,16 +2587,16 @@
         <v>759999</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1029520</v>
+        <v>1030776</v>
       </c>
       <c r="L24" t="n">
-        <v>26.17928743492113</v>
+        <v>26.26923793336283</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>1.554533678756477</v>
+        <v>1.426784323465839</v>
       </c>
       <c r="O24" t="n">
         <v>100</v>
@@ -2654,10 +2654,10 @@
         <v>772000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>1029520</v>
+        <v>1030776</v>
       </c>
       <c r="L25" t="n">
-        <v>25.01359857020747</v>
+        <v>25.10496945990205</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -2672,7 +2672,7 @@
         <v>69.59999999999998</v>
       </c>
       <c r="Q25" t="n">
-        <v>19.9</v>
+        <v>20</v>
       </c>
       <c r="R25" t="n">
         <v>4</v>
@@ -2845,22 +2845,22 @@
         <v>810000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>1072434</v>
+        <v>1073743</v>
       </c>
       <c r="L28" t="n">
-        <v>24.47087652946475</v>
+        <v>24.56295407746547</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N28" t="n">
-        <v>2.409638554216868</v>
+        <v>1.219512195121951</v>
       </c>
       <c r="P28" t="n">
         <v>61.99999999999999</v>
       </c>
       <c r="Q28" t="n">
-        <v>24.6</v>
+        <v>24.2</v>
       </c>
       <c r="R28" t="n">
         <v>3</v>
@@ -2909,10 +2909,10 @@
         <v>810000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>1244093</v>
+        <v>1245610</v>
       </c>
       <c r="L29" t="n">
-        <v>34.89232718132808</v>
+        <v>34.97162033060107</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -2976,10 +2976,10 @@
         <v>820000</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1287007</v>
+        <v>1288577</v>
       </c>
       <c r="L30" t="n">
-        <v>36.28628282519054</v>
+        <v>36.3639115085866</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -3040,10 +3040,10 @@
         <v>820000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1287007</v>
+        <v>1288577</v>
       </c>
       <c r="L31" t="n">
-        <v>36.28628282519054</v>
+        <v>36.3639115085866</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -3104,10 +3104,10 @@
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1372836</v>
+        <v>1374511</v>
       </c>
       <c r="L32" t="n">
-        <v>38.23013091148542</v>
+        <v>38.305404612986</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3171,10 +3171,10 @@
         <v>930000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1372836</v>
+        <v>1374511</v>
       </c>
       <c r="L33" t="n">
-        <v>38.08444708617781</v>
+        <v>38.1598983202026</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3238,10 +3238,10 @@
         <v>860000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>1244093</v>
+        <v>1245610</v>
       </c>
       <c r="L34" t="n">
-        <v>30.87333503202735</v>
+        <v>30.95752282014434</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -3367,10 +3367,10 @@
         <v>880000</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>1158264</v>
+        <v>1159677</v>
       </c>
       <c r="L36" t="n">
-        <v>24.02422936394466</v>
+        <v>24.11680148869038</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -3431,10 +3431,10 @@
         <v>940000</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>1244093</v>
+        <v>1245610</v>
       </c>
       <c r="L37" t="n">
-        <v>24.44294759314617</v>
+        <v>24.53496680341359</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
@@ -3619,10 +3619,10 @@
         <v>990000</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>1501580</v>
+        <v>1503412</v>
       </c>
       <c r="L40" t="n">
-        <v>34.06944684931872</v>
+        <v>34.14978728385832</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -3748,10 +3748,10 @@
         <v>1000000</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>1501580</v>
+        <v>1503412</v>
       </c>
       <c r="L42" t="n">
-        <v>33.4034816659785</v>
+        <v>33.48463362005891</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -3815,10 +3815,10 @@
         <v>1054000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1544494</v>
+        <v>1546379</v>
       </c>
       <c r="L43" t="n">
-        <v>31.75758533215409</v>
+        <v>31.84077124689355</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -3830,7 +3830,7 @@
         <v>57.39710789766407</v>
       </c>
       <c r="Q43" t="n">
-        <v>25.9</v>
+        <v>26</v>
       </c>
       <c r="R43" t="n">
         <v>3</v>
@@ -3879,10 +3879,10 @@
         <v>1054000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1544494</v>
+        <v>1546379</v>
       </c>
       <c r="L44" t="n">
-        <v>31.75758533215409</v>
+        <v>31.84077124689355</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -3894,7 +3894,7 @@
         <v>57.39710789766407</v>
       </c>
       <c r="Q44" t="n">
-        <v>25.9</v>
+        <v>26</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -4005,10 +4005,10 @@
         <v>1115000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1501580</v>
+        <v>1503412</v>
       </c>
       <c r="L46" t="n">
-        <v>25.74488205756603</v>
+        <v>25.83536648636568</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -4020,7 +4020,7 @@
         <v>8.390274908628628</v>
       </c>
       <c r="Q46" t="n">
-        <v>12.8</v>
+        <v>12.9</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -4069,10 +4069,10 @@
         <v>1123000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1716153</v>
+        <v>1718246</v>
       </c>
       <c r="L47" t="n">
-        <v>34.56294397993652</v>
+        <v>34.64265303105608</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -4136,10 +4136,10 @@
         <v>1130000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1501580</v>
+        <v>1503412</v>
       </c>
       <c r="L48" t="n">
-        <v>24.74593428255571</v>
+        <v>24.83763599066657</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -4151,7 +4151,7 @@
         <v>88.39999999999999</v>
       </c>
       <c r="Q48" t="n">
-        <v>29.5</v>
+        <v>29.6</v>
       </c>
       <c r="R48" t="n">
         <v>3</v>
@@ -4262,10 +4262,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1759067</v>
+        <v>1761213</v>
       </c>
       <c r="L50" t="n">
-        <v>34.34019284086393</v>
+        <v>34.42019789769892</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4277,7 +4277,7 @@
         <v>22.53136001640632</v>
       </c>
       <c r="Q50" t="n">
-        <v>19.5</v>
+        <v>19.6</v>
       </c>
       <c r="R50" t="n">
         <v>3</v>
@@ -4326,10 +4326,10 @@
         <v>1155000</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>1759067</v>
+        <v>1761213</v>
       </c>
       <c r="L51" t="n">
-        <v>34.34019284086393</v>
+        <v>34.42019789769892</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -4341,7 +4341,7 @@
         <v>22.53136001640632</v>
       </c>
       <c r="Q51" t="n">
-        <v>19.5</v>
+        <v>19.6</v>
       </c>
       <c r="R51" t="n">
         <v>3</v>
@@ -4390,10 +4390,10 @@
         <v>1185000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1587409</v>
+        <v>1589346</v>
       </c>
       <c r="L52" t="n">
-        <v>25.3500515620108</v>
+        <v>25.44103046158608</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -4405,7 +4405,7 @@
         <v>77.26495726495727</v>
       </c>
       <c r="Q52" t="n">
-        <v>27.4</v>
+        <v>27.5</v>
       </c>
       <c r="R52" t="n">
         <v>3</v>
@@ -4454,10 +4454,10 @@
         <v>1185000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1587409</v>
+        <v>1589346</v>
       </c>
       <c r="L53" t="n">
-        <v>25.3500515620108</v>
+        <v>25.44103046158608</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -4518,10 +4518,10 @@
         <v>1200000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1887811</v>
+        <v>1890114</v>
       </c>
       <c r="L54" t="n">
-        <v>36.43431466391498</v>
+        <v>36.51176595697402</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -4582,10 +4582,10 @@
         <v>1200000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1887811</v>
+        <v>1890114</v>
       </c>
       <c r="L55" t="n">
-        <v>36.43431466391498</v>
+        <v>36.51176595697402</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -4708,10 +4708,10 @@
         <v>1240000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1673238</v>
+        <v>1675279</v>
       </c>
       <c r="L57" t="n">
-        <v>25.89219226434016</v>
+        <v>25.98247814244672</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -4723,7 +4723,7 @@
         <v>100</v>
       </c>
       <c r="Q57" t="n">
-        <v>32.5</v>
+        <v>32.6</v>
       </c>
       <c r="R57" t="n">
         <v>3</v>
@@ -4772,13 +4772,13 @@
         <v>1255000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>1716153</v>
+        <v>1718246</v>
       </c>
       <c r="L58" t="n">
-        <v>26.87132207909201</v>
+        <v>26.96040031520516</v>
       </c>
       <c r="M58" s="3" t="n">
-        <v>-45000</v>
+        <v>0</v>
       </c>
       <c r="N58" t="n">
         <v>3.461538461538462</v>
@@ -4787,7 +4787,7 @@
         <v>68.52057842046719</v>
       </c>
       <c r="Q58" t="n">
-        <v>27.4</v>
+        <v>27.5</v>
       </c>
       <c r="R58" t="n">
         <v>3</v>
@@ -4898,10 +4898,10 @@
         <v>1280000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1716153</v>
+        <v>1718246</v>
       </c>
       <c r="L60" t="n">
-        <v>25.41457550696237</v>
+        <v>25.50542820993036</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -4965,10 +4965,10 @@
         <v>1298000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1759067</v>
+        <v>1761213</v>
       </c>
       <c r="L61" t="n">
-        <v>26.21088338306614</v>
+        <v>26.30079382789021</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -5091,10 +5091,10 @@
         <v>1335000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1801982</v>
+        <v>1804180</v>
       </c>
       <c r="L63" t="n">
-        <v>25.91490924992592</v>
+        <v>26.00516578168475</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -5155,10 +5155,10 @@
         <v>1420000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1930725</v>
+        <v>1933081</v>
       </c>
       <c r="L64" t="n">
-        <v>26.45249841380829</v>
+        <v>26.54213662024509</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -5219,10 +5219,10 @@
         <v>1430000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1930725</v>
+        <v>1933081</v>
       </c>
       <c r="L65" t="n">
-        <v>25.93455826179285</v>
+        <v>26.02482772320456</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -5283,10 +5283,10 @@
         <v>1430000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>2145298</v>
+        <v>2147915</v>
       </c>
       <c r="L66" t="n">
-        <v>33.34259389604614</v>
+        <v>33.42380867026861</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -5347,10 +5347,10 @@
         <v>1430000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>2145298</v>
+        <v>2147915</v>
       </c>
       <c r="L67" t="n">
-        <v>33.34259389604614</v>
+        <v>33.42380867026861</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -5473,10 +5473,10 @@
         <v>1480000</v>
       </c>
       <c r="K69" s="3" t="n">
-        <v>2016554</v>
+        <v>2019014</v>
       </c>
       <c r="L69" t="n">
-        <v>26.60746997104962</v>
+        <v>26.69689264165578</v>
       </c>
       <c r="M69" s="3" t="n">
         <v>0</v>
@@ -5599,10 +5599,10 @@
         <v>1605000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2188213</v>
+        <v>2190882</v>
       </c>
       <c r="L71" t="n">
-        <v>26.65247852928394</v>
+        <v>26.74183274133431</v>
       </c>
       <c r="M71" s="3" t="n">
         <v>0</v>
@@ -5614,7 +5614,7 @@
         <v>36.44392794886694</v>
       </c>
       <c r="Q71" t="n">
-        <v>19.2</v>
+        <v>19.3</v>
       </c>
       <c r="R71" t="n">
         <v>3</v>
@@ -5663,10 +5663,10 @@
         <v>1610000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2188213</v>
+        <v>2190882</v>
       </c>
       <c r="L72" t="n">
-        <v>26.42398157766177</v>
+        <v>26.51361415174345</v>
       </c>
       <c r="M72" s="3" t="n">
         <v>0</v>
@@ -5678,7 +5678,7 @@
         <v>25.72147975982957</v>
       </c>
       <c r="Q72" t="n">
-        <v>16.8</v>
+        <v>16.9</v>
       </c>
       <c r="R72" t="n">
         <v>3</v>
@@ -5727,10 +5727,10 @@
         <v>1615000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2188213</v>
+        <v>2190882</v>
       </c>
       <c r="L73" t="n">
-        <v>26.1954846260396</v>
+        <v>26.2853955621526</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
@@ -5791,10 +5791,10 @@
         <v>1630000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2231127</v>
+        <v>2233849</v>
       </c>
       <c r="L74" t="n">
-        <v>26.94275135391217</v>
+        <v>27.03177340993057</v>
       </c>
       <c r="M74" s="3" t="n">
         <v>0</v>
@@ -5855,10 +5855,10 @@
         <v>1690000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2316956</v>
+        <v>2319783</v>
       </c>
       <c r="L75" t="n">
-        <v>27.05946940727403</v>
+        <v>27.14835827316607</v>
       </c>
       <c r="M75" s="3" t="n">
         <v>0</v>
@@ -5870,7 +5870,7 @@
         <v>16.88768606224628</v>
       </c>
       <c r="Q75" t="n">
-        <v>15.2</v>
+        <v>15.3</v>
       </c>
       <c r="R75" t="n">
         <v>3</v>
@@ -5919,10 +5919,10 @@
         <v>1705000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2316956</v>
+        <v>2319783</v>
       </c>
       <c r="L76" t="n">
-        <v>26.41206824816699</v>
+        <v>26.50174606849003</v>
       </c>
       <c r="M76" s="3" t="n">
         <v>0</v>
@@ -5934,7 +5934,7 @@
         <v>1.9846639603067</v>
       </c>
       <c r="Q76" t="n">
-        <v>11.7</v>
+        <v>11.8</v>
       </c>
       <c r="R76" t="n">
         <v>3</v>
@@ -5983,10 +5983,10 @@
         <v>1725000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2359871</v>
+        <v>2362750</v>
       </c>
       <c r="L77" t="n">
-        <v>26.90278409285931</v>
+        <v>26.99185271399852</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
@@ -6047,10 +6047,10 @@
         <v>1780000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2445700</v>
+        <v>2448683</v>
       </c>
       <c r="L78" t="n">
-        <v>27.21920104673509</v>
+        <v>27.30786304311338</v>
       </c>
       <c r="M78" s="3" t="n">
         <v>0</v>
@@ -6111,10 +6111,10 @@
         <v>1875000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2574443</v>
+        <v>2577584</v>
       </c>
       <c r="L79" t="n">
-        <v>27.16871183397729</v>
+        <v>27.25746280237618</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
@@ -6175,10 +6175,10 @@
         <v>1910000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2617358</v>
+        <v>2620551</v>
       </c>
       <c r="L80" t="n">
-        <v>27.02564952902889</v>
+        <v>27.11456483770016</v>
       </c>
       <c r="M80" s="3" t="n">
         <v>0</v>
@@ -6239,10 +6239,10 @@
         <v>2020000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2746102</v>
+        <v>2749452</v>
       </c>
       <c r="L81" t="n">
-        <v>26.44118827341446</v>
+        <v>26.5308141404178</v>
       </c>
       <c r="M81" s="3" t="n">
         <v>0</v>
@@ -6303,10 +6303,10 @@
         <v>2110000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>2874845</v>
+        <v>2878352</v>
       </c>
       <c r="L82" t="n">
-        <v>26.60473869025982</v>
+        <v>26.6941638826662</v>
       </c>
       <c r="M82" s="3" t="n">
         <v>0</v>
@@ -6318,7 +6318,7 @@
         <v>79.02382335851249</v>
       </c>
       <c r="Q82" t="n">
-        <v>28.3</v>
+        <v>28.4</v>
       </c>
       <c r="R82" t="n">
         <v>3</v>
@@ -6367,10 +6367,10 @@
         <v>2210000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3003589</v>
+        <v>3007253</v>
       </c>
       <c r="L83" t="n">
-        <v>26.42135791548045</v>
+        <v>26.51100522636439</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
@@ -6431,10 +6431,10 @@
         <v>2215000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3046503</v>
+        <v>3050220</v>
       </c>
       <c r="L84" t="n">
-        <v>27.29368722105312</v>
+        <v>27.38228717928543</v>
       </c>
       <c r="M84" s="3" t="n">
         <v>0</v>
@@ -6446,7 +6446,7 @@
         <v>74.28466149856153</v>
       </c>
       <c r="Q84" t="n">
-        <v>27.6</v>
+        <v>27.7</v>
       </c>
       <c r="R84" t="n">
         <v>3</v>
@@ -6495,10 +6495,10 @@
         <v>2315000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3175247</v>
+        <v>3179121</v>
       </c>
       <c r="L85" t="n">
-        <v>27.09228604892785</v>
+        <v>27.18112962671128</v>
       </c>
       <c r="M85" s="3" t="n">
         <v>0</v>
@@ -6559,10 +6559,10 @@
         <v>2395000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3303991</v>
+        <v>3308021</v>
       </c>
       <c r="L86" t="n">
-        <v>27.5119090820768</v>
+        <v>27.60021777370821</v>
       </c>
       <c r="M86" s="3" t="n">
         <v>0</v>
@@ -6623,10 +6623,10 @@
         <v>2410000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3303991</v>
+        <v>3308021</v>
       </c>
       <c r="L87" t="n">
-        <v>27.05791268801882</v>
+        <v>27.14677446122622</v>
       </c>
       <c r="M87" s="3" t="n">
         <v>0</v>
@@ -6687,10 +6687,10 @@
         <v>2499000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3432734</v>
+        <v>3436922</v>
       </c>
       <c r="L88" t="n">
-        <v>27.20088419318246</v>
+        <v>27.28959225725809</v>
       </c>
       <c r="M88" s="3" t="n">
         <v>0</v>
@@ -6751,10 +6751,10 @@
         <v>2510000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3432734</v>
+        <v>3436922</v>
       </c>
       <c r="L89" t="n">
-        <v>26.88043990591756</v>
+        <v>26.96953844166379</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
@@ -6766,7 +6766,7 @@
         <v>83.17546233649077</v>
       </c>
       <c r="Q89" t="n">
-        <v>29.3</v>
+        <v>29.4</v>
       </c>
       <c r="R89" t="n">
         <v>3</v>
@@ -6815,10 +6815,10 @@
         <v>2530000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3475649</v>
+        <v>3479889</v>
       </c>
       <c r="L90" t="n">
-        <v>27.20783945674606</v>
+        <v>27.29653158477181</v>
       </c>
       <c r="M90" s="3" t="n">
         <v>0</v>
@@ -6830,7 +6830,7 @@
         <v>79.17877203176447</v>
       </c>
       <c r="Q90" t="n">
-        <v>28.6</v>
+        <v>28.7</v>
       </c>
       <c r="R90" t="n">
         <v>3</v>
@@ -6879,10 +6879,10 @@
         <v>2610000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>3604393</v>
+        <v>3608790</v>
       </c>
       <c r="L91" t="n">
-        <v>27.58836231232277</v>
+        <v>27.67658966024623</v>
       </c>
       <c r="M91" s="3" t="n">
         <v>0</v>
@@ -6894,7 +6894,7 @@
         <v>74.15426251691474</v>
       </c>
       <c r="Q91" t="n">
-        <v>27.7</v>
+        <v>27.8</v>
       </c>
       <c r="R91" t="n">
         <v>3</v>
@@ -6943,10 +6943,10 @@
         <v>3015000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4162282</v>
+        <v>4167359</v>
       </c>
       <c r="L92" t="n">
-        <v>27.56377391056156</v>
+        <v>27.65202134013413</v>
       </c>
       <c r="M92" s="3" t="n">
         <v>0</v>
@@ -6958,7 +6958,7 @@
         <v>100</v>
       </c>
       <c r="Q92" t="n">
-        <v>33.2</v>
+        <v>33.3</v>
       </c>
       <c r="R92" t="n">
         <v>3</v>
@@ -7007,10 +7007,10 @@
         <v>3098000</v>
       </c>
       <c r="K93" s="3" t="n">
-        <v>4291025</v>
+        <v>4296260</v>
       </c>
       <c r="L93" t="n">
-        <v>27.80279769985027</v>
+        <v>27.89077011167853</v>
       </c>
       <c r="M93" s="3" t="n">
         <v>0</v>
@@ -7022,7 +7022,7 @@
         <v>100</v>
       </c>
       <c r="Q93" t="n">
-        <v>33.3</v>
+        <v>33.4</v>
       </c>
       <c r="R93" t="n">
         <v>3</v>
@@ -7306,10 +7306,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>428716</v>
+        <v>429239</v>
       </c>
       <c r="L2" t="n">
-        <v>27.6912921374523</v>
+        <v>27.77939562807666</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7373,10 +7373,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>428716</v>
+        <v>429239</v>
       </c>
       <c r="L3" t="n">
-        <v>27.6912921374523</v>
+        <v>27.77939562807666</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7440,10 +7440,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>428716</v>
+        <v>429239</v>
       </c>
       <c r="L4" t="n">
-        <v>27.69105888280353</v>
+        <v>27.77916265763363</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7507,10 +7507,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>428716</v>
+        <v>429239</v>
       </c>
       <c r="L5" t="n">
-        <v>27.69105888280353</v>
+        <v>27.77916265763363</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7574,10 +7574,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514545</v>
+        <v>515173</v>
       </c>
       <c r="L6" t="n">
-        <v>25.3709588082675</v>
+        <v>25.46193220529803</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7638,10 +7638,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>514545</v>
+        <v>515173</v>
       </c>
       <c r="L7" t="n">
-        <v>25.3709588082675</v>
+        <v>25.46193220529803</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7702,10 +7702,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>514545</v>
+        <v>515173</v>
       </c>
       <c r="L8" t="n">
-        <v>25.3709588082675</v>
+        <v>25.46193220529803</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7766,10 +7766,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>514545</v>
+        <v>515173</v>
       </c>
       <c r="L9" t="n">
-        <v>25.3709588082675</v>
+        <v>25.46193220529803</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7830,10 +7830,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>514545</v>
+        <v>515173</v>
       </c>
       <c r="L10" t="n">
-        <v>25.17661234683069</v>
+        <v>25.26782265374932</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7894,10 +7894,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>514545</v>
+        <v>515173</v>
       </c>
       <c r="L11" t="n">
-        <v>25.17661234683069</v>
+        <v>25.26782265374932</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7958,10 +7958,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>514545</v>
+        <v>515173</v>
       </c>
       <c r="L12" t="n">
-        <v>25.17661234683069</v>
+        <v>25.26782265374932</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -8022,10 +8022,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>514545</v>
+        <v>515173</v>
       </c>
       <c r="L13" t="n">
-        <v>25.17661234683069</v>
+        <v>25.26782265374932</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -8086,10 +8086,10 @@
         <v>415000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>557460</v>
+        <v>558140</v>
       </c>
       <c r="L14" t="n">
-        <v>25.55519678541958</v>
+        <v>25.64589529508726</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -8153,10 +8153,10 @@
         <v>415000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>557460</v>
+        <v>558140</v>
       </c>
       <c r="L15" t="n">
-        <v>25.55519678541958</v>
+        <v>25.64589529508726</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0</v>
@@ -8220,10 +8220,10 @@
         <v>415000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>557460</v>
+        <v>558140</v>
       </c>
       <c r="L16" t="n">
-        <v>25.55519678541958</v>
+        <v>25.64589529508726</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -8287,10 +8287,10 @@
         <v>420000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>557460</v>
+        <v>558140</v>
       </c>
       <c r="L17" t="n">
-        <v>24.65827144548488</v>
+        <v>24.75006270828107</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>8.5</v>
+        <v>8.6</v>
       </c>
       <c r="R17" t="n">
         <v>4</v>
@@ -8354,10 +8354,10 @@
         <v>454000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>600374</v>
+        <v>601107</v>
       </c>
       <c r="L18" t="n">
-        <v>24.38046950734043</v>
+        <v>24.47268123645208</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -8369,7 +8369,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q18" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="R18" t="n">
         <v>3</v>
@@ -8418,10 +8418,10 @@
         <v>454000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>600374</v>
+        <v>601107</v>
       </c>
       <c r="L19" t="n">
-        <v>24.38046950734043</v>
+        <v>24.47268123645208</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -8433,7 +8433,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q19" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="R19" t="n">
         <v>3</v>
@@ -8482,10 +8482,10 @@
         <v>454000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>600374</v>
+        <v>601107</v>
       </c>
       <c r="L20" t="n">
-        <v>24.38046950734043</v>
+        <v>24.47268123645208</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -8497,7 +8497,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q20" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="R20" t="n">
         <v>3</v>
@@ -8546,10 +8546,10 @@
         <v>454000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>600374</v>
+        <v>601107</v>
       </c>
       <c r="L21" t="n">
-        <v>24.38046950734043</v>
+        <v>24.47268123645208</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -8561,7 +8561,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q21" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="R21" t="n">
         <v>3</v>
@@ -8610,10 +8610,10 @@
         <v>455000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>600374</v>
+        <v>601107</v>
       </c>
       <c r="L22" t="n">
-        <v>24.21390666484558</v>
+        <v>24.30632150349272</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -8674,10 +8674,10 @@
         <v>455000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>600374</v>
+        <v>601107</v>
       </c>
       <c r="L23" t="n">
-        <v>24.21390666484558</v>
+        <v>24.30632150349272</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -8738,10 +8738,10 @@
         <v>455000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>600374</v>
+        <v>601107</v>
       </c>
       <c r="L24" t="n">
-        <v>24.21390666484558</v>
+        <v>24.30632150349272</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -8802,10 +8802,10 @@
         <v>455000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>600374</v>
+        <v>601107</v>
       </c>
       <c r="L25" t="n">
-        <v>24.21390666484558</v>
+        <v>24.30632150349272</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -8866,10 +8866,10 @@
         <v>468000</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>686204</v>
+        <v>687041</v>
       </c>
       <c r="L26" t="n">
-        <v>31.79870709001988</v>
+        <v>31.8817945362795</v>
       </c>
       <c r="M26" s="3" t="n">
         <v>0</v>
@@ -8930,10 +8930,10 @@
         <v>468000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>686204</v>
+        <v>687041</v>
       </c>
       <c r="L27" t="n">
-        <v>31.79870709001988</v>
+        <v>31.8817945362795</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -8994,10 +8994,10 @@
         <v>468000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>686204</v>
+        <v>687041</v>
       </c>
       <c r="L28" t="n">
-        <v>31.79870709001988</v>
+        <v>31.8817945362795</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -9058,10 +9058,10 @@
         <v>468000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>686204</v>
+        <v>687041</v>
       </c>
       <c r="L29" t="n">
-        <v>31.79870709001988</v>
+        <v>31.8817945362795</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -9122,10 +9122,10 @@
         <v>474999</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>643289</v>
+        <v>644074</v>
       </c>
       <c r="L30" t="n">
-        <v>26.16087015322818</v>
+        <v>26.25086558376832</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -9189,10 +9189,10 @@
         <v>475000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>643289</v>
+        <v>644074</v>
       </c>
       <c r="L31" t="n">
-        <v>26.16071470210123</v>
+        <v>26.25071032210585</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -9256,10 +9256,10 @@
         <v>475000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>643289</v>
+        <v>644074</v>
       </c>
       <c r="L32" t="n">
-        <v>26.16071470210123</v>
+        <v>26.25071032210585</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -9323,10 +9323,10 @@
         <v>475000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>643289</v>
+        <v>644074</v>
       </c>
       <c r="L33" t="n">
-        <v>26.16071470210123</v>
+        <v>26.25071032210585</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -9390,10 +9390,10 @@
         <v>475000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>686204</v>
+        <v>687041</v>
       </c>
       <c r="L34" t="n">
-        <v>30.77860228153727</v>
+        <v>30.86293248874522</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -9405,7 +9405,7 @@
         <v>100</v>
       </c>
       <c r="Q34" t="n">
-        <v>34.6</v>
+        <v>34.7</v>
       </c>
       <c r="R34" t="n">
         <v>3</v>
@@ -9454,10 +9454,10 @@
         <v>475000</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>686204</v>
+        <v>687041</v>
       </c>
       <c r="L35" t="n">
-        <v>30.77860228153727</v>
+        <v>30.86293248874522</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
@@ -9469,7 +9469,7 @@
         <v>100</v>
       </c>
       <c r="Q35" t="n">
-        <v>34.6</v>
+        <v>34.7</v>
       </c>
       <c r="R35" t="n">
         <v>3</v>
@@ -9518,10 +9518,10 @@
         <v>475000</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>686204</v>
+        <v>687041</v>
       </c>
       <c r="L36" t="n">
-        <v>30.77860228153727</v>
+        <v>30.86293248874522</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -9533,7 +9533,7 @@
         <v>100</v>
       </c>
       <c r="Q36" t="n">
-        <v>34.6</v>
+        <v>34.7</v>
       </c>
       <c r="R36" t="n">
         <v>3</v>
@@ -9582,10 +9582,10 @@
         <v>475000</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>686204</v>
+        <v>687041</v>
       </c>
       <c r="L37" t="n">
-        <v>30.77860228153727</v>
+        <v>30.86293248874522</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
@@ -9597,7 +9597,7 @@
         <v>100</v>
       </c>
       <c r="Q37" t="n">
-        <v>34.6</v>
+        <v>34.7</v>
       </c>
       <c r="R37" t="n">
         <v>3</v>
@@ -9646,10 +9646,10 @@
         <v>500000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>643289</v>
+        <v>644074</v>
       </c>
       <c r="L38" t="n">
-        <v>22.27443652852761</v>
+        <v>22.36916876011142</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -9710,10 +9710,10 @@
         <v>544999</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>772033</v>
+        <v>772974</v>
       </c>
       <c r="L39" t="n">
-        <v>29.40729217533448</v>
+        <v>29.49323004396008</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -9774,10 +9774,10 @@
         <v>544999</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>772033</v>
+        <v>772974</v>
       </c>
       <c r="L40" t="n">
-        <v>29.40729217533448</v>
+        <v>29.49323004396008</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -9838,10 +9838,10 @@
         <v>544999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>772033</v>
+        <v>772974</v>
       </c>
       <c r="L41" t="n">
-        <v>29.40729217533448</v>
+        <v>29.49323004396008</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
@@ -9902,10 +9902,10 @@
         <v>544999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>772033</v>
+        <v>772974</v>
       </c>
       <c r="L42" t="n">
-        <v>29.40729217533448</v>
+        <v>29.49323004396008</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -9966,10 +9966,10 @@
         <v>549999</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>772033</v>
+        <v>772974</v>
       </c>
       <c r="L43" t="n">
-        <v>28.75965146567569</v>
+        <v>28.84637775656102</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -10030,10 +10030,10 @@
         <v>549999</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>772033</v>
+        <v>772974</v>
       </c>
       <c r="L44" t="n">
-        <v>28.75965146567569</v>
+        <v>28.84637775656102</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -10094,10 +10094,10 @@
         <v>549999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>772033</v>
+        <v>772974</v>
       </c>
       <c r="L45" t="n">
-        <v>28.75965146567569</v>
+        <v>28.84637775656102</v>
       </c>
       <c r="M45" s="3" t="n">
         <v>0</v>
@@ -10158,10 +10158,10 @@
         <v>549999</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>772033</v>
+        <v>772974</v>
       </c>
       <c r="L46" t="n">
-        <v>28.75965146567569</v>
+        <v>28.84637775656102</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -10222,10 +10222,10 @@
         <v>585000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>729118</v>
+        <v>730008</v>
       </c>
       <c r="L47" t="n">
-        <v>19.76607352993617</v>
+        <v>19.86389190255449</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -10237,7 +10237,7 @@
         <v>19.46308724832216</v>
       </c>
       <c r="Q47" t="n">
-        <v>12.6</v>
+        <v>12.7</v>
       </c>
       <c r="R47" t="n">
         <v>3</v>
@@ -10286,10 +10286,10 @@
         <v>595000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>729118</v>
+        <v>730008</v>
       </c>
       <c r="L48" t="n">
-        <v>18.39455341933679</v>
+        <v>18.49404390088876</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -10350,10 +10350,10 @@
         <v>619999</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>857862</v>
+        <v>858908</v>
       </c>
       <c r="L49" t="n">
-        <v>27.7274200279299</v>
+        <v>27.8154354133388</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -10365,7 +10365,7 @@
         <v>55.30233557046979</v>
       </c>
       <c r="Q49" t="n">
-        <v>23.7</v>
+        <v>23.8</v>
       </c>
       <c r="R49" t="n">
         <v>3</v>
@@ -10414,10 +10414,10 @@
         <v>619999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>857862</v>
+        <v>858908</v>
       </c>
       <c r="L50" t="n">
-        <v>27.7274200279299</v>
+        <v>27.8154354133388</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -10429,7 +10429,7 @@
         <v>55.30233557046979</v>
       </c>
       <c r="Q50" t="n">
-        <v>23.7</v>
+        <v>23.8</v>
       </c>
       <c r="R50" t="n">
         <v>3</v>
@@ -10478,10 +10478,10 @@
         <v>619999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>857862</v>
+        <v>858908</v>
       </c>
       <c r="L51" t="n">
-        <v>27.7274200279299</v>
+        <v>27.8154354133388</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -10493,7 +10493,7 @@
         <v>55.30233557046979</v>
       </c>
       <c r="Q51" t="n">
-        <v>23.7</v>
+        <v>23.8</v>
       </c>
       <c r="R51" t="n">
         <v>3</v>
@@ -10542,10 +10542,10 @@
         <v>619999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>857862</v>
+        <v>858908</v>
       </c>
       <c r="L52" t="n">
-        <v>27.7274200279299</v>
+        <v>27.8154354133388</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -10557,7 +10557,7 @@
         <v>55.30233557046979</v>
       </c>
       <c r="Q52" t="n">
-        <v>23.7</v>
+        <v>23.8</v>
       </c>
       <c r="R52" t="n">
         <v>3</v>
@@ -10606,10 +10606,10 @@
         <v>650000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>814947</v>
+        <v>815941</v>
       </c>
       <c r="L53" t="n">
-        <v>20.24021194016298</v>
+        <v>20.33737733488083</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -10670,10 +10670,10 @@
         <v>672000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>857862</v>
+        <v>858908</v>
       </c>
       <c r="L54" t="n">
-        <v>21.66572245885702</v>
+        <v>21.76111993368323</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -10734,10 +10734,10 @@
         <v>700000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>900776</v>
+        <v>901875</v>
       </c>
       <c r="L55" t="n">
-        <v>22.28922617831736</v>
+        <v>22.38392238392238</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -10798,10 +10798,10 @@
         <v>715000</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>943691</v>
+        <v>944842</v>
       </c>
       <c r="L56" t="n">
-        <v>24.23367394623876</v>
+        <v>24.32597196144964</v>
       </c>
       <c r="M56" s="3" t="n">
         <v>0</v>
@@ -10862,10 +10862,10 @@
         <v>734999</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>986605</v>
+        <v>987809</v>
       </c>
       <c r="L57" t="n">
-        <v>25.50220199573284</v>
+        <v>25.59300431561162</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -10926,10 +10926,10 @@
         <v>752000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>986605</v>
+        <v>987809</v>
       </c>
       <c r="L58" t="n">
-        <v>23.77901997253207</v>
+        <v>23.87192260852047</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -10990,10 +10990,10 @@
         <v>810000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1072434</v>
+        <v>1073743</v>
       </c>
       <c r="L59" t="n">
-        <v>24.47087652946475</v>
+        <v>24.56295407746547</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -11054,10 +11054,10 @@
         <v>815000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1072434</v>
+        <v>1073743</v>
       </c>
       <c r="L60" t="n">
-        <v>24.00464737223922</v>
+        <v>24.09729330016587</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -11069,7 +11069,7 @@
         <v>79.56521739130434</v>
       </c>
       <c r="Q60" t="n">
-        <v>27.3</v>
+        <v>27.4</v>
       </c>
       <c r="R60" t="n">
         <v>3</v>
@@ -11118,10 +11118,10 @@
         <v>875000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1158264</v>
+        <v>1159677</v>
       </c>
       <c r="L61" t="n">
-        <v>24.45590987892225</v>
+        <v>24.54795602568646</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -11182,10 +11182,10 @@
         <v>992000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1329922</v>
+        <v>1331544</v>
       </c>
       <c r="L62" t="n">
-        <v>25.40915933415644</v>
+        <v>25.50002102821987</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -11197,7 +11197,7 @@
         <v>85.14782608695651</v>
       </c>
       <c r="Q62" t="n">
-        <v>29.1</v>
+        <v>29.2</v>
       </c>
       <c r="R62" t="n">
         <v>3</v>
@@ -11246,10 +11246,10 @@
         <v>1050000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1415751</v>
+        <v>1417478</v>
       </c>
       <c r="L63" t="n">
-        <v>25.83441579769324</v>
+        <v>25.92477625755038</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -11310,10 +11310,10 @@
         <v>1050000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1415751</v>
+        <v>1417478</v>
       </c>
       <c r="L64" t="n">
-        <v>25.83441579769324</v>
+        <v>25.92477625755038</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -11374,10 +11374,10 @@
         <v>1100000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1501580</v>
+        <v>1503412</v>
       </c>
       <c r="L65" t="n">
-        <v>26.74382983257636</v>
+        <v>26.8330969820648</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -11438,10 +11438,10 @@
         <v>1105000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1501580</v>
+        <v>1503412</v>
       </c>
       <c r="L66" t="n">
-        <v>26.41084724090624</v>
+        <v>26.50052015016509</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -11453,7 +11453,7 @@
         <v>100</v>
       </c>
       <c r="Q66" t="n">
-        <v>32.7</v>
+        <v>32.8</v>
       </c>
       <c r="R66" t="n">
         <v>3</v>
@@ -11502,10 +11502,10 @@
         <v>1155000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1587409</v>
+        <v>1589346</v>
       </c>
       <c r="L67" t="n">
-        <v>27.23992367436496</v>
+        <v>27.32859931065986</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -11772,7 +11772,7 @@
         <v>315000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>299973</v>
+        <v>300339</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -11833,10 +11833,10 @@
         <v>380000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>385802</v>
+        <v>386272</v>
       </c>
       <c r="L3" t="n">
-        <v>1.503880228718358</v>
+        <v>1.623726286140336</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -11897,7 +11897,7 @@
         <v>415000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>385802</v>
+        <v>386272</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -11958,10 +11958,10 @@
         <v>495000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>471631</v>
+        <v>472206</v>
       </c>
       <c r="L5" t="n">
-        <v>6.706938263176085</v>
+        <v>6.82054018796881</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -12022,10 +12022,10 @@
         <v>490000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514545</v>
+        <v>515173</v>
       </c>
       <c r="L6" t="n">
-        <v>4.77023389596634</v>
+        <v>4.886319741135503</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -12037,7 +12037,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="R6" t="n">
         <v>3</v>
@@ -12086,10 +12086,10 @@
         <v>550000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>557460</v>
+        <v>558140</v>
       </c>
       <c r="L7" t="n">
-        <v>6.719764646790802</v>
+        <v>6.833410972157523</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -12150,7 +12150,7 @@
         <v>530000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>471631</v>
+        <v>472206</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -12214,10 +12214,10 @@
         <v>600000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>600374</v>
+        <v>601107</v>
       </c>
       <c r="L9" t="n">
-        <v>8.390436627835316</v>
+        <v>8.50214687235384</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -12278,17 +12278,22 @@
         <v>590000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>514545</v>
+        <v>515173</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
       </c>
-      <c r="M10" s="3" t="n"/>
+      <c r="M10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
       <c r="Q10" t="n">
         <v>0</v>
       </c>
       <c r="R10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
@@ -12334,10 +12339,10 @@
         <v>646000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>729118</v>
+        <v>730008</v>
       </c>
       <c r="L11" t="n">
-        <v>17.02317046074847</v>
+        <v>17.12433288402319</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -12349,7 +12354,7 @@
         <v>100</v>
       </c>
       <c r="Q11" t="n">
-        <v>25.9</v>
+        <v>26</v>
       </c>
       <c r="R11" t="n">
         <v>4</v>
@@ -12398,7 +12403,7 @@
         <v>615000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>557460</v>
+        <v>558140</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -12462,12 +12467,17 @@
         <v>655000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>557460</v>
+        <v>558140</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
       </c>
-      <c r="M13" s="3" t="n"/>
+      <c r="M13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0</v>
+      </c>
       <c r="P13" t="n">
         <v>0</v>
       </c>
@@ -12475,7 +12485,7 @@
         <v>0</v>
       </c>
       <c r="R13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
@@ -12521,7 +12531,7 @@
         <v>700000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>643289</v>
+        <v>644074</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -12585,7 +12595,7 @@
         <v>745000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>686204</v>
+        <v>687041</v>
       </c>
       <c r="L15" t="n">
         <v>0</v>
@@ -12649,20 +12659,25 @@
         <v>755000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>643289</v>
+        <v>644074</v>
       </c>
       <c r="L16" t="n">
         <v>0</v>
       </c>
-      <c r="M16" s="3" t="n"/>
+      <c r="M16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
       <c r="P16" t="n">
         <v>100</v>
       </c>
       <c r="Q16" t="n">
-        <v>33.3</v>
+        <v>21.4</v>
       </c>
       <c r="R16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>
@@ -12708,7 +12723,7 @@
         <v>930000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>857862</v>
+        <v>858908</v>
       </c>
       <c r="L17" t="n">
         <v>0</v>
@@ -12782,7 +12797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12828,64 +12843,8 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Macbook Pro 16 CTO M5 Pro 18 Core CPU 20 Core GPU 64GB 1TB Silver</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>1300000</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>1255000</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>-45000</v>
-      </c>
-      <c r="F2" t="n">
-        <v>-3.46</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Apple MacBook Pro 14Inch MW2W3 M4 10Core CPU 10Core GPU 16GB 512GB Silver</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>445000</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>498000</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>53000</v>
-      </c>
-      <c r="F3" t="n">
-        <v>11.91</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:F3"/>
-  <conditionalFormatting sqref="E2:E3">
-    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
+  <autoFilter ref="A1:F1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: price data 2026-10-13
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MacBook Pro'!$A$1:$S$93</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MacBook Air'!$A$1:$S$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20261012T105752620082+0000</t>
+          <t>20261013T104158222929+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-12T10:57:52.620082+00:00</t>
+          <t>2026-10-13T10:41:58.222929+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>277.205784</v>
+        <v>276.919098</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -897,7 +897,7 @@
         <v>759999</v>
       </c>
       <c r="D30" t="n">
-        <v>43.4</v>
+        <v>43.3</v>
       </c>
       <c r="E30" t="n">
         <v>4</v>
@@ -918,7 +918,7 @@
         <v>759999</v>
       </c>
       <c r="D31" t="n">
-        <v>43.4</v>
+        <v>43.3</v>
       </c>
       <c r="E31" t="n">
         <v>4</v>
@@ -1147,10 +1147,10 @@
         <v>495000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>687041</v>
+        <v>686330</v>
       </c>
       <c r="L2" t="n">
-        <v>27.95189806721869</v>
+        <v>27.87726021010301</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1214,10 +1214,10 @@
         <v>498000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>687041</v>
+        <v>686330</v>
       </c>
       <c r="L3" t="n">
-        <v>27.51524290398972</v>
+        <v>27.44015269622485</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -1232,7 +1232,7 @@
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>9.199999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="R3" t="n">
         <v>4</v>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>772974</v>
+        <v>772175</v>
       </c>
       <c r="L4" t="n">
-        <v>35.31490063055161</v>
+        <v>35.24796840094538</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>772974</v>
+        <v>772175</v>
       </c>
       <c r="L5" t="n">
-        <v>32.72749148095537</v>
+        <v>32.65788195681031</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>858908</v>
+        <v>858020</v>
       </c>
       <c r="L6" t="n">
-        <v>38.0608866141659</v>
+        <v>37.99678329176476</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1606,10 +1606,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>858908</v>
+        <v>858020</v>
       </c>
       <c r="L9" t="n">
-        <v>34.21879875376641</v>
+        <v>34.15071909745694</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1673,10 +1673,10 @@
         <v>578999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>858908</v>
+        <v>858020</v>
       </c>
       <c r="L10" t="n">
-        <v>32.588938512623</v>
+        <v>32.51917204727162</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -1691,7 +1691,7 @@
         <v>50.30029999999999</v>
       </c>
       <c r="Q10" t="n">
-        <v>41.7</v>
+        <v>41.6</v>
       </c>
       <c r="R10" t="n">
         <v>4</v>
@@ -1740,10 +1740,10 @@
         <v>584999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>858908</v>
+        <v>858020</v>
       </c>
       <c r="L11" t="n">
-        <v>31.89037708345947</v>
+        <v>31.81988764830657</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -1758,7 +1758,7 @@
         <v>48.50029999999999</v>
       </c>
       <c r="Q11" t="n">
-        <v>18.9</v>
+        <v>18.8</v>
       </c>
       <c r="R11" t="n">
         <v>4</v>
@@ -1807,22 +1807,22 @@
         <v>634000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>858908</v>
+        <v>858020</v>
       </c>
       <c r="L12" t="n">
-        <v>26.18534231838567</v>
+        <v>26.10894850935875</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>0.4709576138147566</v>
+        <v>0</v>
       </c>
       <c r="P12" t="n">
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>11.4</v>
+        <v>11.2</v>
       </c>
       <c r="R12" t="n">
         <v>3</v>
@@ -1871,10 +1871,10 @@
         <v>634000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>858908</v>
+        <v>858020</v>
       </c>
       <c r="L13" t="n">
-        <v>26.18534231838567</v>
+        <v>26.10894850935875</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -1935,10 +1935,10 @@
         <v>642999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>944842</v>
+        <v>943865</v>
       </c>
       <c r="L14" t="n">
-        <v>31.94639950383239</v>
+        <v>31.87595683704767</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -2061,10 +2061,10 @@
         <v>650000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>944842</v>
+        <v>943865</v>
       </c>
       <c r="L16" t="n">
-        <v>31.20542905586331</v>
+        <v>31.13421940637697</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -2128,10 +2128,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1030776</v>
+        <v>1029710</v>
       </c>
       <c r="L17" t="n">
-        <v>32.08999821493709</v>
+        <v>32.01969486554466</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2160,28 +2160,28 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 16Inch MX2X3 14Core CPU 20Core GPU M4 Pro 24GB 512GB Space Black</t>
+          <t>Macbook Pro 14 MGDR4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>M4 Pro</t>
+          <t>M5 Pro</t>
         </is>
       </c>
       <c r="D18" t="n">
         <v>24</v>
       </c>
       <c r="E18" t="n">
-        <v>512</v>
+        <v>1024</v>
       </c>
       <c r="F18" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G18" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -2189,34 +2189,29 @@
         </is>
       </c>
       <c r="I18" s="3" t="n">
-        <v>711999</v>
+        <v>717999</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>711999</v>
-      </c>
-      <c r="K18" s="3" t="n">
-        <v>1073743</v>
-      </c>
-      <c r="L18" t="n">
-        <v>33.689998444693</v>
-      </c>
+        <v>717999</v>
+      </c>
+      <c r="K18" s="3" t="n"/>
       <c r="M18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>0</v>
+        <v>0.2779166666666667</v>
       </c>
       <c r="O18" t="n">
         <v>100</v>
       </c>
       <c r="P18" t="n">
-        <v>11.06613972463029</v>
+        <v>42.94044444444446</v>
       </c>
       <c r="Q18" t="n">
-        <v>35.3</v>
+        <v>44.2</v>
       </c>
       <c r="R18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S18" t="inlineStr">
         <is>
@@ -2227,28 +2222,28 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 MGDR4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Space Black</t>
+          <t>Apple MacBook Pro 16Inch MX2X3 14Core CPU 20Core GPU M4 Pro 24GB 512GB Space Black</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>M5 Pro</t>
+          <t>M4 Pro</t>
         </is>
       </c>
       <c r="D19" t="n">
         <v>24</v>
       </c>
       <c r="E19" t="n">
-        <v>1024</v>
+        <v>512</v>
       </c>
       <c r="F19" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G19" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -2256,29 +2251,34 @@
         </is>
       </c>
       <c r="I19" s="3" t="n">
-        <v>717999</v>
+        <v>719999</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>717999</v>
-      </c>
-      <c r="K19" s="3" t="n"/>
+        <v>719999</v>
+      </c>
+      <c r="K19" s="3" t="n">
+        <v>1072632</v>
+      </c>
+      <c r="L19" t="n">
+        <v>32.8754875856771</v>
+      </c>
       <c r="M19" s="3" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="N19" t="n">
-        <v>0.2779166666666667</v>
+        <v>0</v>
       </c>
       <c r="O19" t="n">
         <v>100</v>
       </c>
       <c r="P19" t="n">
-        <v>42.94044444444446</v>
+        <v>8.21045385007649</v>
       </c>
       <c r="Q19" t="n">
-        <v>44.2</v>
+        <v>34.5</v>
       </c>
       <c r="R19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S19" t="inlineStr">
         <is>
@@ -2324,10 +2324,10 @@
         <v>720000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>1030776</v>
+        <v>1029710</v>
       </c>
       <c r="L20" t="n">
-        <v>30.14971244964958</v>
+        <v>30.07740043313166</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -2453,10 +2453,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1073743</v>
+        <v>1072632</v>
       </c>
       <c r="L22" t="n">
-        <v>30.80280849328005</v>
+        <v>30.73113612124195</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2471,7 +2471,7 @@
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>10.3</v>
+        <v>10.2</v>
       </c>
       <c r="R22" t="n">
         <v>4</v>
@@ -2520,16 +2520,16 @@
         <v>759999</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1030776</v>
+        <v>1029710</v>
       </c>
       <c r="L23" t="n">
-        <v>26.26923793336283</v>
+        <v>26.19290868302726</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>1.426784323465839</v>
+        <v>1.298702985328553</v>
       </c>
       <c r="O23" t="n">
         <v>100</v>
@@ -2538,7 +2538,7 @@
         <v>72.00019999999999</v>
       </c>
       <c r="Q23" t="n">
-        <v>43.4</v>
+        <v>43.3</v>
       </c>
       <c r="R23" t="n">
         <v>4</v>
@@ -2587,16 +2587,16 @@
         <v>759999</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1030776</v>
+        <v>1029710</v>
       </c>
       <c r="L24" t="n">
-        <v>26.26923793336283</v>
+        <v>26.19290868302726</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>1.426784323465839</v>
+        <v>1.298702985328553</v>
       </c>
       <c r="O24" t="n">
         <v>100</v>
@@ -2605,7 +2605,7 @@
         <v>72.00019999999999</v>
       </c>
       <c r="Q24" t="n">
-        <v>43.4</v>
+        <v>43.3</v>
       </c>
       <c r="R24" t="n">
         <v>4</v>
@@ -2654,10 +2654,10 @@
         <v>772000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>1030776</v>
+        <v>1029710</v>
       </c>
       <c r="L25" t="n">
-        <v>25.10496945990205</v>
+        <v>25.02743490885783</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -2672,7 +2672,7 @@
         <v>69.59999999999998</v>
       </c>
       <c r="Q25" t="n">
-        <v>20</v>
+        <v>19.9</v>
       </c>
       <c r="R25" t="n">
         <v>4</v>
@@ -2845,22 +2845,22 @@
         <v>810000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>1073743</v>
+        <v>1072632</v>
       </c>
       <c r="L28" t="n">
-        <v>24.56295407746547</v>
+        <v>24.48481865169042</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N28" t="n">
-        <v>1.219512195121951</v>
+        <v>0</v>
       </c>
       <c r="P28" t="n">
         <v>61.99999999999999</v>
       </c>
       <c r="Q28" t="n">
-        <v>24.2</v>
+        <v>23.8</v>
       </c>
       <c r="R28" t="n">
         <v>3</v>
@@ -2909,10 +2909,10 @@
         <v>810000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>1245610</v>
+        <v>1244322</v>
       </c>
       <c r="L29" t="n">
-        <v>34.97162033060107</v>
+        <v>34.90430933472204</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -2970,31 +2970,34 @@
         </is>
       </c>
       <c r="I30" s="3" t="n">
-        <v>820000</v>
+        <v>815999</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>820000</v>
+        <v>815999</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1288577</v>
+        <v>1287245</v>
       </c>
       <c r="L30" t="n">
-        <v>36.3639115085866</v>
+        <v>36.60888175910569</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>0</v>
+        <v>-4001</v>
       </c>
       <c r="N30" t="n">
-        <v>0.6060606060606061</v>
+        <v>1.091030303030303</v>
+      </c>
+      <c r="O30" t="n">
+        <v>100</v>
       </c>
       <c r="P30" t="n">
-        <v>0</v>
+        <v>1.424160177975549</v>
       </c>
       <c r="Q30" t="n">
-        <v>15.8</v>
+        <v>35</v>
       </c>
       <c r="R30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S30" t="inlineStr">
         <is>
@@ -3040,10 +3043,10 @@
         <v>820000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1288577</v>
+        <v>1287245</v>
       </c>
       <c r="L31" t="n">
-        <v>36.3639115085866</v>
+        <v>36.29806291731566</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -3051,14 +3054,17 @@
       <c r="N31" t="n">
         <v>1.204700246626803</v>
       </c>
+      <c r="O31" t="n">
+        <v>0</v>
+      </c>
       <c r="P31" t="n">
         <v>0</v>
       </c>
       <c r="Q31" t="n">
-        <v>16</v>
+        <v>12.4</v>
       </c>
       <c r="R31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S31" t="inlineStr">
         <is>
@@ -3104,10 +3110,10 @@
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1374511</v>
+        <v>1373090</v>
       </c>
       <c r="L32" t="n">
-        <v>38.305404612986</v>
+        <v>38.24155736331923</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3171,10 +3177,10 @@
         <v>930000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1374511</v>
+        <v>1373090</v>
       </c>
       <c r="L33" t="n">
-        <v>38.1598983202026</v>
+        <v>38.09590048722225</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3238,10 +3244,10 @@
         <v>860000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>1245610</v>
+        <v>1244322</v>
       </c>
       <c r="L34" t="n">
-        <v>30.95752282014434</v>
+        <v>30.8860568245197</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -3367,10 +3373,10 @@
         <v>880000</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>1159677</v>
+        <v>1158477</v>
       </c>
       <c r="L36" t="n">
-        <v>24.11680148869038</v>
+        <v>24.03819842776335</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -3431,10 +3437,10 @@
         <v>940000</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>1245610</v>
+        <v>1244322</v>
       </c>
       <c r="L37" t="n">
-        <v>24.53496680341359</v>
+        <v>24.45685280819595</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
@@ -3619,10 +3625,10 @@
         <v>990000</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>1503412</v>
+        <v>1501857</v>
       </c>
       <c r="L40" t="n">
-        <v>34.14978728385832</v>
+        <v>34.08160697057043</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -3748,10 +3754,10 @@
         <v>1000000</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>1503412</v>
+        <v>1501857</v>
       </c>
       <c r="L42" t="n">
-        <v>33.48463362005891</v>
+        <v>33.41576461673782</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -3815,10 +3821,10 @@
         <v>1054000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1546379</v>
+        <v>1544779</v>
       </c>
       <c r="L43" t="n">
-        <v>31.84077124689355</v>
+        <v>31.77017553967266</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -3830,7 +3836,7 @@
         <v>57.39710789766407</v>
       </c>
       <c r="Q43" t="n">
-        <v>26</v>
+        <v>25.9</v>
       </c>
       <c r="R43" t="n">
         <v>3</v>
@@ -3879,10 +3885,10 @@
         <v>1054000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1546379</v>
+        <v>1544779</v>
       </c>
       <c r="L44" t="n">
-        <v>31.84077124689355</v>
+        <v>31.77017553967266</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -3894,7 +3900,7 @@
         <v>57.39710789766407</v>
       </c>
       <c r="Q44" t="n">
-        <v>26</v>
+        <v>25.9</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -4005,10 +4011,10 @@
         <v>1115000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1503412</v>
+        <v>1501857</v>
       </c>
       <c r="L46" t="n">
-        <v>25.83536648636568</v>
+        <v>25.75857754766266</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -4020,7 +4026,7 @@
         <v>8.390274908628628</v>
       </c>
       <c r="Q46" t="n">
-        <v>12.9</v>
+        <v>12.8</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -4069,10 +4075,10 @@
         <v>1123000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1718246</v>
+        <v>1716469</v>
       </c>
       <c r="L47" t="n">
-        <v>34.64265303105608</v>
+        <v>34.57499086788052</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -4136,10 +4142,10 @@
         <v>1130000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1503412</v>
+        <v>1501857</v>
       </c>
       <c r="L48" t="n">
-        <v>24.83763599066657</v>
+        <v>24.75981401691373</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -4262,10 +4268,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1761213</v>
+        <v>1759392</v>
       </c>
       <c r="L50" t="n">
-        <v>34.42019789769892</v>
+        <v>34.35232171113658</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4326,10 +4332,10 @@
         <v>1155000</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>1761213</v>
+        <v>1759392</v>
       </c>
       <c r="L51" t="n">
-        <v>34.42019789769892</v>
+        <v>34.35232171113658</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -4390,10 +4396,10 @@
         <v>1185000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1589346</v>
+        <v>1587702</v>
       </c>
       <c r="L52" t="n">
-        <v>25.44103046158608</v>
+        <v>25.36382772081915</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -4405,7 +4411,7 @@
         <v>77.26495726495727</v>
       </c>
       <c r="Q52" t="n">
-        <v>27.5</v>
+        <v>27.4</v>
       </c>
       <c r="R52" t="n">
         <v>3</v>
@@ -4454,10 +4460,10 @@
         <v>1185000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1589346</v>
+        <v>1587702</v>
       </c>
       <c r="L53" t="n">
-        <v>25.44103046158608</v>
+        <v>25.36382772081915</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -4518,10 +4524,10 @@
         <v>1200000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1890114</v>
+        <v>1888159</v>
       </c>
       <c r="L54" t="n">
-        <v>36.51176595697402</v>
+        <v>36.44603023368266</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -4582,10 +4588,10 @@
         <v>1200000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1890114</v>
+        <v>1888159</v>
       </c>
       <c r="L55" t="n">
-        <v>36.51176595697402</v>
+        <v>36.44603023368266</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -4708,10 +4714,10 @@
         <v>1240000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1675279</v>
+        <v>1673547</v>
       </c>
       <c r="L57" t="n">
-        <v>25.98247814244672</v>
+        <v>25.9058753653169</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -4723,7 +4729,7 @@
         <v>100</v>
       </c>
       <c r="Q57" t="n">
-        <v>32.6</v>
+        <v>32.5</v>
       </c>
       <c r="R57" t="n">
         <v>3</v>
@@ -4772,10 +4778,10 @@
         <v>1255000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>1718246</v>
+        <v>1716469</v>
       </c>
       <c r="L58" t="n">
-        <v>26.96040031520516</v>
+        <v>26.88478498592168</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -4787,7 +4793,7 @@
         <v>68.52057842046719</v>
       </c>
       <c r="Q58" t="n">
-        <v>27.5</v>
+        <v>27.4</v>
       </c>
       <c r="R58" t="n">
         <v>3</v>
@@ -4898,10 +4904,10 @@
         <v>1280000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1718246</v>
+        <v>1716469</v>
       </c>
       <c r="L60" t="n">
-        <v>25.50542820993036</v>
+        <v>25.42830659918705</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -4965,10 +4971,10 @@
         <v>1298000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1761213</v>
+        <v>1759392</v>
       </c>
       <c r="L61" t="n">
-        <v>26.30079382789021</v>
+        <v>26.22451392299158</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -5091,10 +5097,10 @@
         <v>1335000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1804180</v>
+        <v>1802314</v>
       </c>
       <c r="L63" t="n">
-        <v>26.00516578168475</v>
+        <v>25.92855628930364</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -5155,10 +5161,10 @@
         <v>1420000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1933081</v>
+        <v>1931081</v>
       </c>
       <c r="L64" t="n">
-        <v>26.54213662024509</v>
+        <v>26.46605709444606</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -5219,10 +5225,10 @@
         <v>1430000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1933081</v>
+        <v>1931081</v>
       </c>
       <c r="L65" t="n">
-        <v>26.02482772320456</v>
+        <v>25.94821242609709</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -5283,10 +5289,10 @@
         <v>1430000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>2147915</v>
+        <v>2145694</v>
       </c>
       <c r="L66" t="n">
-        <v>33.42380867026861</v>
+        <v>33.35489589848319</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -5347,10 +5353,10 @@
         <v>1430000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>2147915</v>
+        <v>2145694</v>
       </c>
       <c r="L67" t="n">
-        <v>33.42380867026861</v>
+        <v>33.35489589848319</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -5473,10 +5479,10 @@
         <v>1480000</v>
       </c>
       <c r="K69" s="3" t="n">
-        <v>2019014</v>
+        <v>2016926</v>
       </c>
       <c r="L69" t="n">
-        <v>26.69689264165578</v>
+        <v>26.62100642264516</v>
       </c>
       <c r="M69" s="3" t="n">
         <v>0</v>
@@ -5599,10 +5605,10 @@
         <v>1605000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2190882</v>
+        <v>2188616</v>
       </c>
       <c r="L71" t="n">
-        <v>26.74183274133431</v>
+        <v>26.66598434809944</v>
       </c>
       <c r="M71" s="3" t="n">
         <v>0</v>
@@ -5614,7 +5620,7 @@
         <v>36.44392794886694</v>
       </c>
       <c r="Q71" t="n">
-        <v>19.3</v>
+        <v>19.2</v>
       </c>
       <c r="R71" t="n">
         <v>3</v>
@@ -5663,10 +5669,10 @@
         <v>1610000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2190882</v>
+        <v>2188616</v>
       </c>
       <c r="L72" t="n">
-        <v>26.51361415174345</v>
+        <v>26.43752947067919</v>
       </c>
       <c r="M72" s="3" t="n">
         <v>0</v>
@@ -5678,7 +5684,7 @@
         <v>25.72147975982957</v>
       </c>
       <c r="Q72" t="n">
-        <v>16.9</v>
+        <v>16.8</v>
       </c>
       <c r="R72" t="n">
         <v>3</v>
@@ -5727,10 +5733,10 @@
         <v>1615000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2190882</v>
+        <v>2188616</v>
       </c>
       <c r="L73" t="n">
-        <v>26.2853955621526</v>
+        <v>26.20907459325894</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
@@ -5791,10 +5797,10 @@
         <v>1630000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2233849</v>
+        <v>2231539</v>
       </c>
       <c r="L74" t="n">
-        <v>27.03177340993057</v>
+        <v>26.95623961759127</v>
       </c>
       <c r="M74" s="3" t="n">
         <v>0</v>
@@ -5855,10 +5861,10 @@
         <v>1690000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2319783</v>
+        <v>2317384</v>
       </c>
       <c r="L75" t="n">
-        <v>27.14835827316607</v>
+        <v>27.07294086780611</v>
       </c>
       <c r="M75" s="3" t="n">
         <v>0</v>
@@ -5870,7 +5876,7 @@
         <v>16.88768606224628</v>
       </c>
       <c r="Q75" t="n">
-        <v>15.3</v>
+        <v>15.2</v>
       </c>
       <c r="R75" t="n">
         <v>3</v>
@@ -5919,10 +5925,10 @@
         <v>1705000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2319783</v>
+        <v>2317384</v>
       </c>
       <c r="L76" t="n">
-        <v>26.50174606849003</v>
+        <v>26.4256592778754</v>
       </c>
       <c r="M76" s="3" t="n">
         <v>0</v>
@@ -5983,10 +5989,10 @@
         <v>1725000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2362750</v>
+        <v>2360306</v>
       </c>
       <c r="L77" t="n">
-        <v>26.99185271399852</v>
+        <v>26.9162557736158</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
@@ -6047,10 +6053,10 @@
         <v>1780000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2448683</v>
+        <v>2446151</v>
       </c>
       <c r="L78" t="n">
-        <v>27.30786304311338</v>
+        <v>27.23261973606699</v>
       </c>
       <c r="M78" s="3" t="n">
         <v>0</v>
@@ -6111,10 +6117,10 @@
         <v>1875000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2577584</v>
+        <v>2574918</v>
       </c>
       <c r="L79" t="n">
-        <v>27.25746280237618</v>
+        <v>27.1821471596377</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
@@ -6175,10 +6181,10 @@
         <v>1910000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2620551</v>
+        <v>2617841</v>
       </c>
       <c r="L80" t="n">
-        <v>27.11456483770016</v>
+        <v>27.03911352904932</v>
       </c>
       <c r="M80" s="3" t="n">
         <v>0</v>
@@ -6239,10 +6245,10 @@
         <v>2020000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2749452</v>
+        <v>2746608</v>
       </c>
       <c r="L81" t="n">
-        <v>26.5308141404178</v>
+        <v>26.45473980997652</v>
       </c>
       <c r="M81" s="3" t="n">
         <v>0</v>
@@ -6303,10 +6309,10 @@
         <v>2110000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>2878352</v>
+        <v>2875376</v>
       </c>
       <c r="L82" t="n">
-        <v>26.6941638826662</v>
+        <v>26.61829270328472</v>
       </c>
       <c r="M82" s="3" t="n">
         <v>0</v>
@@ -6318,7 +6324,7 @@
         <v>79.02382335851249</v>
       </c>
       <c r="Q82" t="n">
-        <v>28.4</v>
+        <v>28.3</v>
       </c>
       <c r="R82" t="n">
         <v>3</v>
@@ -6367,10 +6373,10 @@
         <v>2210000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3007253</v>
+        <v>3004143</v>
       </c>
       <c r="L83" t="n">
-        <v>26.51100522636439</v>
+        <v>26.43492669956124</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
@@ -6431,10 +6437,10 @@
         <v>2215000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3050220</v>
+        <v>3047065</v>
       </c>
       <c r="L84" t="n">
-        <v>27.38228717928543</v>
+        <v>27.30709715742854</v>
       </c>
       <c r="M84" s="3" t="n">
         <v>0</v>
@@ -6446,7 +6452,7 @@
         <v>74.28466149856153</v>
       </c>
       <c r="Q84" t="n">
-        <v>27.7</v>
+        <v>27.6</v>
       </c>
       <c r="R84" t="n">
         <v>3</v>
@@ -6495,10 +6501,10 @@
         <v>2315000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3179121</v>
+        <v>3175833</v>
       </c>
       <c r="L85" t="n">
-        <v>27.18112962671128</v>
+        <v>27.10573887228957</v>
       </c>
       <c r="M85" s="3" t="n">
         <v>0</v>
@@ -6559,10 +6565,10 @@
         <v>2395000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3308021</v>
+        <v>3304600</v>
       </c>
       <c r="L86" t="n">
-        <v>27.60021777370821</v>
+        <v>27.52526780850935</v>
       </c>
       <c r="M86" s="3" t="n">
         <v>0</v>
@@ -6623,10 +6629,10 @@
         <v>2410000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3308021</v>
+        <v>3304600</v>
       </c>
       <c r="L87" t="n">
-        <v>27.14677446122622</v>
+        <v>27.07135508079647</v>
       </c>
       <c r="M87" s="3" t="n">
         <v>0</v>
@@ -6687,10 +6693,10 @@
         <v>2499000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3436922</v>
+        <v>3433368</v>
       </c>
       <c r="L88" t="n">
-        <v>27.28959225725809</v>
+        <v>27.21432715630833</v>
       </c>
       <c r="M88" s="3" t="n">
         <v>0</v>
@@ -6751,10 +6757,10 @@
         <v>2510000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3436922</v>
+        <v>3433368</v>
       </c>
       <c r="L89" t="n">
-        <v>26.96953844166379</v>
+        <v>26.89394204175026</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
@@ -6766,7 +6772,7 @@
         <v>83.17546233649077</v>
       </c>
       <c r="Q89" t="n">
-        <v>29.4</v>
+        <v>29.3</v>
       </c>
       <c r="R89" t="n">
         <v>3</v>
@@ -6815,10 +6821,10 @@
         <v>2530000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3479889</v>
+        <v>3476290</v>
       </c>
       <c r="L90" t="n">
-        <v>27.29653158477181</v>
+        <v>27.22126174743764</v>
       </c>
       <c r="M90" s="3" t="n">
         <v>0</v>
@@ -6830,7 +6836,7 @@
         <v>79.17877203176447</v>
       </c>
       <c r="Q90" t="n">
-        <v>28.7</v>
+        <v>28.6</v>
       </c>
       <c r="R90" t="n">
         <v>3</v>
@@ -6879,10 +6885,10 @@
         <v>2610000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>3608790</v>
+        <v>3605057</v>
       </c>
       <c r="L91" t="n">
-        <v>27.67658966024623</v>
+        <v>27.60169950156128</v>
       </c>
       <c r="M91" s="3" t="n">
         <v>0</v>
@@ -6894,7 +6900,7 @@
         <v>74.15426251691474</v>
       </c>
       <c r="Q91" t="n">
-        <v>27.8</v>
+        <v>27.7</v>
       </c>
       <c r="R91" t="n">
         <v>3</v>
@@ -6943,10 +6949,10 @@
         <v>3015000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4167359</v>
+        <v>4163049</v>
       </c>
       <c r="L92" t="n">
-        <v>27.65202134013413</v>
+        <v>27.57711955828529</v>
       </c>
       <c r="M92" s="3" t="n">
         <v>0</v>
@@ -6958,7 +6964,7 @@
         <v>100</v>
       </c>
       <c r="Q92" t="n">
-        <v>33.3</v>
+        <v>33.2</v>
       </c>
       <c r="R92" t="n">
         <v>3</v>
@@ -7007,10 +7013,10 @@
         <v>3098000</v>
       </c>
       <c r="K93" s="3" t="n">
-        <v>4296260</v>
+        <v>4291817</v>
       </c>
       <c r="L93" t="n">
-        <v>27.89077011167853</v>
+        <v>27.8161207712258</v>
       </c>
       <c r="M93" s="3" t="n">
         <v>0</v>
@@ -7022,7 +7028,7 @@
         <v>100</v>
       </c>
       <c r="Q93" t="n">
-        <v>33.4</v>
+        <v>33.3</v>
       </c>
       <c r="R93" t="n">
         <v>3</v>
@@ -7306,10 +7312,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>429239</v>
+        <v>428795</v>
       </c>
       <c r="L2" t="n">
-        <v>27.77939562807666</v>
+        <v>27.70461409298149</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7373,10 +7379,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>429239</v>
+        <v>428795</v>
       </c>
       <c r="L3" t="n">
-        <v>27.77939562807666</v>
+        <v>27.70461409298149</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7440,10 +7446,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>429239</v>
+        <v>428795</v>
       </c>
       <c r="L4" t="n">
-        <v>27.77916265763363</v>
+        <v>27.70438088130692</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7507,10 +7513,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>429239</v>
+        <v>428795</v>
       </c>
       <c r="L5" t="n">
-        <v>27.77916265763363</v>
+        <v>27.70438088130692</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7574,10 +7580,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>515173</v>
+        <v>514640</v>
       </c>
       <c r="L6" t="n">
-        <v>25.46193220529803</v>
+        <v>25.38473496036064</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7638,10 +7644,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>515173</v>
+        <v>514640</v>
       </c>
       <c r="L7" t="n">
-        <v>25.46193220529803</v>
+        <v>25.38473496036064</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7702,10 +7708,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>515173</v>
+        <v>514640</v>
       </c>
       <c r="L8" t="n">
-        <v>25.46193220529803</v>
+        <v>25.38473496036064</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7766,10 +7772,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>515173</v>
+        <v>514640</v>
       </c>
       <c r="L9" t="n">
-        <v>25.46193220529803</v>
+        <v>25.38473496036064</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7830,10 +7836,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>515173</v>
+        <v>514640</v>
       </c>
       <c r="L10" t="n">
-        <v>25.26782265374932</v>
+        <v>25.19042437431991</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7894,10 +7900,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>515173</v>
+        <v>514640</v>
       </c>
       <c r="L11" t="n">
-        <v>25.26782265374932</v>
+        <v>25.19042437431991</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7958,10 +7964,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>515173</v>
+        <v>514640</v>
       </c>
       <c r="L12" t="n">
-        <v>25.26782265374932</v>
+        <v>25.19042437431991</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -8022,10 +8028,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>515173</v>
+        <v>514640</v>
       </c>
       <c r="L13" t="n">
-        <v>25.26782265374932</v>
+        <v>25.19042437431991</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -8086,10 +8092,10 @@
         <v>415000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>558140</v>
+        <v>557563</v>
       </c>
       <c r="L14" t="n">
-        <v>25.64589529508726</v>
+        <v>25.56894915910848</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -8153,10 +8159,10 @@
         <v>415000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>558140</v>
+        <v>557563</v>
       </c>
       <c r="L15" t="n">
-        <v>25.64589529508726</v>
+        <v>25.56894915910848</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0</v>
@@ -8220,10 +8226,10 @@
         <v>415000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>558140</v>
+        <v>557563</v>
       </c>
       <c r="L16" t="n">
-        <v>25.64589529508726</v>
+        <v>25.56894915910848</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -8287,10 +8293,10 @@
         <v>420000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>558140</v>
+        <v>557563</v>
       </c>
       <c r="L17" t="n">
-        <v>24.75006270828107</v>
+        <v>24.67218951042304</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -8354,10 +8360,10 @@
         <v>454000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>601107</v>
+        <v>600485</v>
       </c>
       <c r="L18" t="n">
-        <v>24.47268123645208</v>
+        <v>24.39444782134441</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -8369,7 +8375,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q18" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="R18" t="n">
         <v>3</v>
@@ -8418,10 +8424,10 @@
         <v>454000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>601107</v>
+        <v>600485</v>
       </c>
       <c r="L19" t="n">
-        <v>24.47268123645208</v>
+        <v>24.39444782134441</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -8433,7 +8439,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q19" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="R19" t="n">
         <v>3</v>
@@ -8482,10 +8488,10 @@
         <v>454000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>601107</v>
+        <v>600485</v>
       </c>
       <c r="L20" t="n">
-        <v>24.47268123645208</v>
+        <v>24.39444782134441</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -8497,7 +8503,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q20" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="R20" t="n">
         <v>3</v>
@@ -8546,10 +8552,10 @@
         <v>454000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>601107</v>
+        <v>600485</v>
       </c>
       <c r="L21" t="n">
-        <v>24.47268123645208</v>
+        <v>24.39444782134441</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -8561,7 +8567,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q21" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="R21" t="n">
         <v>3</v>
@@ -8610,10 +8616,10 @@
         <v>455000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>601107</v>
+        <v>600485</v>
       </c>
       <c r="L22" t="n">
-        <v>24.30632150349272</v>
+        <v>24.22791576808746</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -8674,10 +8680,10 @@
         <v>455000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>601107</v>
+        <v>600485</v>
       </c>
       <c r="L23" t="n">
-        <v>24.30632150349272</v>
+        <v>24.22791576808746</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -8738,10 +8744,10 @@
         <v>455000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>601107</v>
+        <v>600485</v>
       </c>
       <c r="L24" t="n">
-        <v>24.30632150349272</v>
+        <v>24.22791576808746</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -8802,10 +8808,10 @@
         <v>455000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>601107</v>
+        <v>600485</v>
       </c>
       <c r="L25" t="n">
-        <v>24.30632150349272</v>
+        <v>24.22791576808746</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -8866,10 +8872,10 @@
         <v>468000</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>687041</v>
+        <v>686330</v>
       </c>
       <c r="L26" t="n">
-        <v>31.8817945362795</v>
+        <v>31.81122783500648</v>
       </c>
       <c r="M26" s="3" t="n">
         <v>0</v>
@@ -8930,10 +8936,10 @@
         <v>468000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>687041</v>
+        <v>686330</v>
       </c>
       <c r="L27" t="n">
-        <v>31.8817945362795</v>
+        <v>31.81122783500648</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -8994,10 +9000,10 @@
         <v>468000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>687041</v>
+        <v>686330</v>
       </c>
       <c r="L28" t="n">
-        <v>31.8817945362795</v>
+        <v>31.81122783500648</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -9058,10 +9064,10 @@
         <v>468000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>687041</v>
+        <v>686330</v>
       </c>
       <c r="L29" t="n">
-        <v>31.8817945362795</v>
+        <v>31.81122783500648</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -9122,10 +9128,10 @@
         <v>474999</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>644074</v>
+        <v>643408</v>
       </c>
       <c r="L30" t="n">
-        <v>26.25086558376832</v>
+        <v>26.17452689428792</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -9189,10 +9195,10 @@
         <v>475000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>644074</v>
+        <v>643408</v>
       </c>
       <c r="L31" t="n">
-        <v>26.25071032210585</v>
+        <v>26.17437147191207</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -9256,10 +9262,10 @@
         <v>475000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>644074</v>
+        <v>643408</v>
       </c>
       <c r="L32" t="n">
-        <v>26.25071032210585</v>
+        <v>26.17437147191207</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -9323,10 +9329,10 @@
         <v>475000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>644074</v>
+        <v>643408</v>
       </c>
       <c r="L33" t="n">
-        <v>26.25071032210585</v>
+        <v>26.17437147191207</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -9390,10 +9396,10 @@
         <v>475000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>687041</v>
+        <v>686330</v>
       </c>
       <c r="L34" t="n">
-        <v>30.86293248874522</v>
+        <v>30.7913103026241</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -9405,7 +9411,7 @@
         <v>100</v>
       </c>
       <c r="Q34" t="n">
-        <v>34.7</v>
+        <v>34.6</v>
       </c>
       <c r="R34" t="n">
         <v>3</v>
@@ -9454,10 +9460,10 @@
         <v>475000</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>687041</v>
+        <v>686330</v>
       </c>
       <c r="L35" t="n">
-        <v>30.86293248874522</v>
+        <v>30.7913103026241</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
@@ -9469,7 +9475,7 @@
         <v>100</v>
       </c>
       <c r="Q35" t="n">
-        <v>34.7</v>
+        <v>34.6</v>
       </c>
       <c r="R35" t="n">
         <v>3</v>
@@ -9518,10 +9524,10 @@
         <v>475000</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>687041</v>
+        <v>686330</v>
       </c>
       <c r="L36" t="n">
-        <v>30.86293248874522</v>
+        <v>30.7913103026241</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -9533,7 +9539,7 @@
         <v>100</v>
       </c>
       <c r="Q36" t="n">
-        <v>34.7</v>
+        <v>34.6</v>
       </c>
       <c r="R36" t="n">
         <v>3</v>
@@ -9582,10 +9588,10 @@
         <v>475000</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>687041</v>
+        <v>686330</v>
       </c>
       <c r="L37" t="n">
-        <v>30.86293248874522</v>
+        <v>30.7913103026241</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
@@ -9597,7 +9603,7 @@
         <v>100</v>
       </c>
       <c r="Q37" t="n">
-        <v>34.7</v>
+        <v>34.6</v>
       </c>
       <c r="R37" t="n">
         <v>3</v>
@@ -9646,10 +9652,10 @@
         <v>500000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>644074</v>
+        <v>643408</v>
       </c>
       <c r="L38" t="n">
-        <v>22.36916876011142</v>
+        <v>22.28881207569691</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -9710,10 +9716,10 @@
         <v>544999</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>772974</v>
+        <v>772175</v>
       </c>
       <c r="L39" t="n">
-        <v>29.49323004396008</v>
+        <v>29.42027390164147</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -9774,10 +9780,10 @@
         <v>544999</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>772974</v>
+        <v>772175</v>
       </c>
       <c r="L40" t="n">
-        <v>29.49323004396008</v>
+        <v>29.42027390164147</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -9838,10 +9844,10 @@
         <v>544999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>772974</v>
+        <v>772175</v>
       </c>
       <c r="L41" t="n">
-        <v>29.49323004396008</v>
+        <v>29.42027390164147</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>0</v>
@@ -9902,10 +9908,10 @@
         <v>544999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>772974</v>
+        <v>772175</v>
       </c>
       <c r="L42" t="n">
-        <v>29.49323004396008</v>
+        <v>29.42027390164147</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -9966,10 +9972,10 @@
         <v>549999</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>772974</v>
+        <v>772175</v>
       </c>
       <c r="L43" t="n">
-        <v>28.84637775656102</v>
+        <v>28.7727522906077</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
@@ -10030,10 +10036,10 @@
         <v>549999</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>772974</v>
+        <v>772175</v>
       </c>
       <c r="L44" t="n">
-        <v>28.84637775656102</v>
+        <v>28.7727522906077</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -10094,10 +10100,10 @@
         <v>549999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>772974</v>
+        <v>772175</v>
       </c>
       <c r="L45" t="n">
-        <v>28.84637775656102</v>
+        <v>28.7727522906077</v>
       </c>
       <c r="M45" s="3" t="n">
         <v>0</v>
@@ -10158,10 +10164,10 @@
         <v>549999</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>772974</v>
+        <v>772175</v>
       </c>
       <c r="L46" t="n">
-        <v>28.84637775656102</v>
+        <v>28.7727522906077</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -10222,10 +10228,10 @@
         <v>585000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>730008</v>
+        <v>729253</v>
       </c>
       <c r="L47" t="n">
-        <v>19.86389190255449</v>
+        <v>19.78092650972982</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -10237,7 +10243,7 @@
         <v>19.46308724832216</v>
       </c>
       <c r="Q47" t="n">
-        <v>12.7</v>
+        <v>12.6</v>
       </c>
       <c r="R47" t="n">
         <v>3</v>
@@ -10286,10 +10292,10 @@
         <v>595000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>730008</v>
+        <v>729253</v>
       </c>
       <c r="L48" t="n">
-        <v>18.49404390088876</v>
+        <v>18.40966029622093</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -10350,10 +10356,10 @@
         <v>619999</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>858908</v>
+        <v>858020</v>
       </c>
       <c r="L49" t="n">
-        <v>27.8154354133388</v>
+        <v>27.74072865434372</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -10365,7 +10371,7 @@
         <v>55.30233557046979</v>
       </c>
       <c r="Q49" t="n">
-        <v>23.8</v>
+        <v>23.7</v>
       </c>
       <c r="R49" t="n">
         <v>3</v>
@@ -10414,10 +10420,10 @@
         <v>619999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>858908</v>
+        <v>858020</v>
       </c>
       <c r="L50" t="n">
-        <v>27.8154354133388</v>
+        <v>27.74072865434372</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -10429,7 +10435,7 @@
         <v>55.30233557046979</v>
       </c>
       <c r="Q50" t="n">
-        <v>23.8</v>
+        <v>23.7</v>
       </c>
       <c r="R50" t="n">
         <v>3</v>
@@ -10478,10 +10484,10 @@
         <v>619999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>858908</v>
+        <v>858020</v>
       </c>
       <c r="L51" t="n">
-        <v>27.8154354133388</v>
+        <v>27.74072865434372</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -10493,7 +10499,7 @@
         <v>55.30233557046979</v>
       </c>
       <c r="Q51" t="n">
-        <v>23.8</v>
+        <v>23.7</v>
       </c>
       <c r="R51" t="n">
         <v>3</v>
@@ -10542,10 +10548,10 @@
         <v>619999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>858908</v>
+        <v>858020</v>
       </c>
       <c r="L52" t="n">
-        <v>27.8154354133388</v>
+        <v>27.74072865434372</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -10557,7 +10563,7 @@
         <v>55.30233557046979</v>
       </c>
       <c r="Q52" t="n">
-        <v>23.8</v>
+        <v>23.7</v>
       </c>
       <c r="R52" t="n">
         <v>3</v>
@@ -10606,10 +10612,10 @@
         <v>650000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>815941</v>
+        <v>815098</v>
       </c>
       <c r="L53" t="n">
-        <v>20.33737733488083</v>
+        <v>20.25498774380504</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -10670,10 +10676,10 @@
         <v>672000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>858908</v>
+        <v>858020</v>
       </c>
       <c r="L54" t="n">
-        <v>21.76111993368323</v>
+        <v>21.68014731591338</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -10734,10 +10740,10 @@
         <v>700000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>901875</v>
+        <v>900942</v>
       </c>
       <c r="L55" t="n">
-        <v>22.38392238392238</v>
+        <v>22.30354451229935</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -10798,10 +10804,10 @@
         <v>715000</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>944842</v>
+        <v>943865</v>
       </c>
       <c r="L56" t="n">
-        <v>24.32597196144964</v>
+        <v>24.24764134701467</v>
       </c>
       <c r="M56" s="3" t="n">
         <v>0</v>
@@ -10862,10 +10868,10 @@
         <v>734999</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>987809</v>
+        <v>986787</v>
       </c>
       <c r="L57" t="n">
-        <v>25.59300431561162</v>
+        <v>25.51594214354263</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -10926,10 +10932,10 @@
         <v>752000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>987809</v>
+        <v>986787</v>
       </c>
       <c r="L58" t="n">
-        <v>23.87192260852047</v>
+        <v>23.79307793880544</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -10990,10 +10996,10 @@
         <v>810000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1073743</v>
+        <v>1072632</v>
       </c>
       <c r="L59" t="n">
-        <v>24.56295407746547</v>
+        <v>24.48481865169042</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -11054,10 +11060,10 @@
         <v>815000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1073743</v>
+        <v>1072632</v>
       </c>
       <c r="L60" t="n">
-        <v>24.09729330016587</v>
+        <v>24.01867555694777</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -11069,7 +11075,7 @@
         <v>79.56521739130434</v>
       </c>
       <c r="Q60" t="n">
-        <v>27.4</v>
+        <v>27.3</v>
       </c>
       <c r="R60" t="n">
         <v>3</v>
@@ -11118,10 +11124,10 @@
         <v>875000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1159677</v>
+        <v>1158477</v>
       </c>
       <c r="L61" t="n">
-        <v>24.54795602568646</v>
+        <v>24.46979957306015</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -11182,10 +11188,10 @@
         <v>992000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1331544</v>
+        <v>1330167</v>
       </c>
       <c r="L62" t="n">
-        <v>25.50002102821987</v>
+        <v>25.42289802708983</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -11197,7 +11203,7 @@
         <v>85.14782608695651</v>
       </c>
       <c r="Q62" t="n">
-        <v>29.2</v>
+        <v>29.1</v>
       </c>
       <c r="R62" t="n">
         <v>3</v>
@@ -11246,10 +11252,10 @@
         <v>1050000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1417478</v>
+        <v>1416012</v>
       </c>
       <c r="L63" t="n">
-        <v>25.92477625755038</v>
+        <v>25.84808603316921</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -11310,10 +11316,10 @@
         <v>1050000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1417478</v>
+        <v>1416012</v>
       </c>
       <c r="L64" t="n">
-        <v>25.92477625755038</v>
+        <v>25.84808603316921</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -11374,10 +11380,10 @@
         <v>1100000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1503412</v>
+        <v>1501857</v>
       </c>
       <c r="L65" t="n">
-        <v>26.8330969820648</v>
+        <v>26.7573410784116</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -11438,10 +11444,10 @@
         <v>1105000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1503412</v>
+        <v>1501857</v>
       </c>
       <c r="L66" t="n">
-        <v>26.50052015016509</v>
+        <v>26.42441990149528</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -11502,10 +11508,10 @@
         <v>1155000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1589346</v>
+        <v>1587702</v>
       </c>
       <c r="L67" t="n">
-        <v>27.32859931065986</v>
+        <v>27.25335106965916</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -11772,7 +11778,7 @@
         <v>315000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>300339</v>
+        <v>300028</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -11833,10 +11839,10 @@
         <v>380000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>386272</v>
+        <v>385873</v>
       </c>
       <c r="L3" t="n">
-        <v>1.623726286140336</v>
+        <v>1.522003353434938</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -11897,7 +11903,7 @@
         <v>415000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>386272</v>
+        <v>385873</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -11958,10 +11964,10 @@
         <v>495000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>472206</v>
+        <v>471718</v>
       </c>
       <c r="L5" t="n">
-        <v>6.82054018796881</v>
+        <v>6.724144510067455</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -12022,10 +12028,10 @@
         <v>490000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>515173</v>
+        <v>514640</v>
       </c>
       <c r="L6" t="n">
-        <v>4.886319741135503</v>
+        <v>4.787812840043525</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -12086,10 +12092,10 @@
         <v>550000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>558140</v>
+        <v>557563</v>
       </c>
       <c r="L7" t="n">
-        <v>6.833410972157523</v>
+        <v>6.736996536714236</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -12150,7 +12156,7 @@
         <v>530000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>472206</v>
+        <v>471718</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -12214,10 +12220,10 @@
         <v>600000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>601107</v>
+        <v>600485</v>
       </c>
       <c r="L9" t="n">
-        <v>8.50214687235384</v>
+        <v>8.407370708677153</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -12278,7 +12284,7 @@
         <v>590000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>515173</v>
+        <v>514640</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
@@ -12339,10 +12345,10 @@
         <v>646000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>730008</v>
+        <v>729253</v>
       </c>
       <c r="L11" t="n">
-        <v>17.12433288402319</v>
+        <v>17.03853120933339</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -12354,7 +12360,7 @@
         <v>100</v>
       </c>
       <c r="Q11" t="n">
-        <v>26</v>
+        <v>25.9</v>
       </c>
       <c r="R11" t="n">
         <v>4</v>
@@ -12403,7 +12409,7 @@
         <v>615000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>558140</v>
+        <v>557563</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -12467,7 +12473,7 @@
         <v>655000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>558140</v>
+        <v>557563</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -12531,7 +12537,7 @@
         <v>700000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>644074</v>
+        <v>643408</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -12595,7 +12601,7 @@
         <v>745000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>687041</v>
+        <v>686330</v>
       </c>
       <c r="L15" t="n">
         <v>0</v>
@@ -12659,7 +12665,7 @@
         <v>755000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>644074</v>
+        <v>643408</v>
       </c>
       <c r="L16" t="n">
         <v>0</v>
@@ -12723,7 +12729,7 @@
         <v>930000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>858908</v>
+        <v>858020</v>
       </c>
       <c r="L17" t="n">
         <v>0</v>
@@ -12797,7 +12803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12843,8 +12849,64 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Macbook Pro 16 MGEA4 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Space Black</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>820000</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>815999</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>-4001</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-0.49</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Apple MacBook Pro 16Inch MX2X3 14Core CPU 20Core GPU M4 Pro 24GB 512GB Space Black</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>711999</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>719999</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1.12</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F1"/>
+  <autoFilter ref="A1:F3"/>
+  <conditionalFormatting sqref="E2:E3">
+    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: price data 2026-10-14
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MacBook Pro'!$A$1:$S$93</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MacBook Air'!$A$1:$S$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20261013T104158222929+0000</t>
+          <t>20261014T084743581810+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-13T10:41:58.222929+00:00</t>
+          <t>2026-10-14T08:47:43.581810+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>276.919098</v>
+        <v>277.05126</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -843,7 +843,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 M5 MDE34 10 Core CPU 10 Core GPU 24GB 1TB Space Black</t>
+          <t>Macbook Pro 14 MGDR4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -852,19 +852,19 @@
         </is>
       </c>
       <c r="C28" s="3" t="n">
-        <v>642999</v>
+        <v>714999</v>
       </c>
       <c r="D28" t="n">
-        <v>44.5</v>
+        <v>44.6</v>
       </c>
       <c r="E28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Macbook Pro 14 MGDR4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Space Black</t>
+          <t>Macbook Pro 14 M5 MDE34 10 Core CPU 10 Core GPU 24GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -873,13 +873,13 @@
         </is>
       </c>
       <c r="C29" s="3" t="n">
-        <v>717999</v>
+        <v>642999</v>
       </c>
       <c r="D29" t="n">
-        <v>44.2</v>
+        <v>44.5</v>
       </c>
       <c r="E29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30">
@@ -1147,10 +1147,10 @@
         <v>495000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>686330</v>
+        <v>686658</v>
       </c>
       <c r="L2" t="n">
-        <v>27.87726021010301</v>
+        <v>27.91171150703844</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1214,10 +1214,10 @@
         <v>498000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>686330</v>
+        <v>686658</v>
       </c>
       <c r="L3" t="n">
-        <v>27.44015269622485</v>
+        <v>27.47481278889928</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -1232,7 +1232,7 @@
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>9.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="R3" t="n">
         <v>4</v>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>772175</v>
+        <v>772544</v>
       </c>
       <c r="L4" t="n">
-        <v>35.24796840094538</v>
+        <v>35.27889673597879</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>772175</v>
+        <v>772544</v>
       </c>
       <c r="L5" t="n">
-        <v>32.65788195681031</v>
+        <v>32.69004742771933</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>858020</v>
+        <v>858429</v>
       </c>
       <c r="L6" t="n">
-        <v>37.99678329176476</v>
+        <v>38.02632483292153</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1606,10 +1606,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>858020</v>
+        <v>858429</v>
       </c>
       <c r="L9" t="n">
-        <v>34.15071909745694</v>
+        <v>34.18209310263283</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1667,31 +1667,31 @@
         </is>
       </c>
       <c r="I10" s="3" t="n">
-        <v>578999</v>
+        <v>574999</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>578999</v>
+        <v>574999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>858020</v>
+        <v>858429</v>
       </c>
       <c r="L10" t="n">
-        <v>32.51917204727162</v>
+        <v>33.01729088835535</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>0</v>
+        <v>-4000</v>
       </c>
       <c r="N10" t="n">
-        <v>0.6861075233405204</v>
+        <v>1.372215046681041</v>
       </c>
       <c r="O10" t="n">
         <v>100</v>
       </c>
       <c r="P10" t="n">
-        <v>50.30029999999999</v>
+        <v>51.50029999999999</v>
       </c>
       <c r="Q10" t="n">
-        <v>41.6</v>
+        <v>42.2</v>
       </c>
       <c r="R10" t="n">
         <v>4</v>
@@ -1734,31 +1734,31 @@
         </is>
       </c>
       <c r="I11" s="3" t="n">
-        <v>584999</v>
+        <v>582999</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>584999</v>
+        <v>582999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>858020</v>
+        <v>858429</v>
       </c>
       <c r="L11" t="n">
-        <v>31.81988764830657</v>
+        <v>32.08535592343688</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>0</v>
+        <v>-2000</v>
       </c>
       <c r="N11" t="n">
-        <v>0.5102049493281451</v>
+        <v>0.8503415822135753</v>
       </c>
       <c r="O11" t="n">
         <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>48.50029999999999</v>
+        <v>49.10029999999999</v>
       </c>
       <c r="Q11" t="n">
-        <v>18.8</v>
+        <v>19.1</v>
       </c>
       <c r="R11" t="n">
         <v>4</v>
@@ -1807,10 +1807,10 @@
         <v>634000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>858020</v>
+        <v>858429</v>
       </c>
       <c r="L12" t="n">
-        <v>26.10894850935875</v>
+        <v>26.144154030211</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -1871,10 +1871,10 @@
         <v>634000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>858020</v>
+        <v>858429</v>
       </c>
       <c r="L13" t="n">
-        <v>26.10894850935875</v>
+        <v>26.144154030211</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -1935,10 +1935,10 @@
         <v>642999</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>943865</v>
+        <v>944315</v>
       </c>
       <c r="L14" t="n">
-        <v>31.87595683704767</v>
+        <v>31.90842038938278</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
@@ -2061,10 +2061,10 @@
         <v>650000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>943865</v>
+        <v>944315</v>
       </c>
       <c r="L16" t="n">
-        <v>31.13421940637697</v>
+        <v>31.16703642322742</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
@@ -2128,10 +2128,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1029710</v>
+        <v>1030201</v>
       </c>
       <c r="L17" t="n">
-        <v>32.01969486554466</v>
+        <v>32.05209468831811</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2189,26 +2189,26 @@
         </is>
       </c>
       <c r="I18" s="3" t="n">
-        <v>717999</v>
+        <v>714999</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>717999</v>
+        <v>714999</v>
       </c>
       <c r="K18" s="3" t="n"/>
       <c r="M18" s="3" t="n">
-        <v>0</v>
+        <v>-3000</v>
       </c>
       <c r="N18" t="n">
-        <v>0.2779166666666667</v>
+        <v>0.6945833333333333</v>
       </c>
       <c r="O18" t="n">
         <v>100</v>
       </c>
       <c r="P18" t="n">
-        <v>42.94044444444446</v>
+        <v>43.76095726495728</v>
       </c>
       <c r="Q18" t="n">
-        <v>44.2</v>
+        <v>44.6</v>
       </c>
       <c r="R18" t="n">
         <v>3</v>
@@ -2257,13 +2257,13 @@
         <v>719999</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>1072632</v>
+        <v>1073144</v>
       </c>
       <c r="L19" t="n">
-        <v>32.8754875856771</v>
+        <v>32.90751287804805</v>
       </c>
       <c r="M19" s="3" t="n">
-        <v>8000</v>
+        <v>0</v>
       </c>
       <c r="N19" t="n">
         <v>0</v>
@@ -2275,7 +2275,7 @@
         <v>8.21045385007649</v>
       </c>
       <c r="Q19" t="n">
-        <v>34.5</v>
+        <v>34.6</v>
       </c>
       <c r="R19" t="n">
         <v>4</v>
@@ -2324,10 +2324,10 @@
         <v>720000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>1029710</v>
+        <v>1030201</v>
       </c>
       <c r="L20" t="n">
-        <v>30.07740043313166</v>
+        <v>30.11072596512719</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -2398,13 +2398,13 @@
         <v>0.2068965517241379</v>
       </c>
       <c r="O21" t="n">
-        <v>96.49620066114228</v>
+        <v>94.6869082068237</v>
       </c>
       <c r="P21" t="n">
         <v>41.43589743589743</v>
       </c>
       <c r="Q21" t="n">
-        <v>42.6</v>
+        <v>42</v>
       </c>
       <c r="R21" t="n">
         <v>3</v>
@@ -2453,10 +2453,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1072632</v>
+        <v>1073144</v>
       </c>
       <c r="L22" t="n">
-        <v>30.73113612124195</v>
+        <v>30.76418448968638</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2471,7 +2471,7 @@
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>10.2</v>
+        <v>10.3</v>
       </c>
       <c r="R22" t="n">
         <v>4</v>
@@ -2520,10 +2520,10 @@
         <v>759999</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1029710</v>
+        <v>1030201</v>
       </c>
       <c r="L23" t="n">
-        <v>26.19290868302726</v>
+        <v>26.22808558718153</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -2587,10 +2587,10 @@
         <v>759999</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1029710</v>
+        <v>1030201</v>
       </c>
       <c r="L24" t="n">
-        <v>26.19290868302726</v>
+        <v>26.22808558718153</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -2654,10 +2654,10 @@
         <v>772000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>1029710</v>
+        <v>1030201</v>
       </c>
       <c r="L25" t="n">
-        <v>25.02743490885783</v>
+        <v>25.06316728483082</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -2672,7 +2672,7 @@
         <v>69.59999999999998</v>
       </c>
       <c r="Q25" t="n">
-        <v>19.9</v>
+        <v>20</v>
       </c>
       <c r="R25" t="n">
         <v>4</v>
@@ -2845,10 +2845,10 @@
         <v>810000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>1072632</v>
+        <v>1073144</v>
       </c>
       <c r="L28" t="n">
-        <v>24.48481865169042</v>
+        <v>24.52084715564733</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -2909,10 +2909,10 @@
         <v>810000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>1244322</v>
+        <v>1244916</v>
       </c>
       <c r="L29" t="n">
-        <v>34.90430933472204</v>
+        <v>34.93536913333912</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -2976,13 +2976,13 @@
         <v>815999</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1287245</v>
+        <v>1287859</v>
       </c>
       <c r="L30" t="n">
-        <v>36.60888175910569</v>
+        <v>36.63910412552927</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>-4001</v>
+        <v>0</v>
       </c>
       <c r="N30" t="n">
         <v>1.091030303030303</v>
@@ -3043,10 +3043,10 @@
         <v>820000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1287245</v>
+        <v>1287859</v>
       </c>
       <c r="L31" t="n">
-        <v>36.29806291731566</v>
+        <v>36.32843346981308</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -3110,10 +3110,10 @@
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1373090</v>
+        <v>1373745</v>
       </c>
       <c r="L32" t="n">
-        <v>38.24155736331923</v>
+        <v>38.27100371611908</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3177,10 +3177,10 @@
         <v>930000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1373090</v>
+        <v>1373745</v>
       </c>
       <c r="L33" t="n">
-        <v>38.09590048722225</v>
+        <v>38.12541628904928</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3244,10 +3244,10 @@
         <v>860000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>1244322</v>
+        <v>1244916</v>
       </c>
       <c r="L34" t="n">
-        <v>30.8860568245197</v>
+        <v>30.91903389465634</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -3373,10 +3373,10 @@
         <v>880000</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>1158477</v>
+        <v>1159030</v>
       </c>
       <c r="L36" t="n">
-        <v>24.03819842776335</v>
+        <v>24.07444155888976</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -3437,10 +3437,10 @@
         <v>940000</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>1244322</v>
+        <v>1244916</v>
       </c>
       <c r="L37" t="n">
-        <v>24.45685280819595</v>
+        <v>24.49289751276391</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
@@ -3625,16 +3625,16 @@
         <v>990000</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>1501857</v>
+        <v>1502574</v>
       </c>
       <c r="L40" t="n">
-        <v>34.08160697057043</v>
+        <v>34.11306198563265</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N40" t="n">
-        <v>0.5025125628140703</v>
+        <v>0.2518891687657431</v>
       </c>
       <c r="O40" t="n">
         <v>100</v>
@@ -3643,7 +3643,7 @@
         <v>39.19647231749141</v>
       </c>
       <c r="Q40" t="n">
-        <v>40.3</v>
+        <v>40.2</v>
       </c>
       <c r="R40" t="n">
         <v>4</v>
@@ -3754,10 +3754,10 @@
         <v>1000000</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>1501857</v>
+        <v>1502574</v>
       </c>
       <c r="L42" t="n">
-        <v>33.41576461673782</v>
+        <v>33.4475373592249</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -3815,31 +3815,34 @@
         </is>
       </c>
       <c r="I43" s="3" t="n">
-        <v>1054000</v>
+        <v>1044000</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>1054000</v>
+        <v>1044000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1544779</v>
+        <v>1545517</v>
       </c>
       <c r="L43" t="n">
-        <v>31.77017553967266</v>
+        <v>32.44978864677645</v>
       </c>
       <c r="M43" s="3" t="n">
-        <v>0</v>
+        <v>-10000</v>
       </c>
       <c r="N43" t="n">
-        <v>0.09478672985781991</v>
+        <v>1.042654028436019</v>
+      </c>
+      <c r="O43" t="n">
+        <v>100</v>
       </c>
       <c r="P43" t="n">
-        <v>57.39710789766407</v>
+        <v>59.62180200222469</v>
       </c>
       <c r="Q43" t="n">
-        <v>25.9</v>
+        <v>43.3</v>
       </c>
       <c r="R43" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S43" t="inlineStr">
         <is>
@@ -3885,10 +3888,10 @@
         <v>1054000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1544779</v>
+        <v>1545517</v>
       </c>
       <c r="L44" t="n">
-        <v>31.77017553967266</v>
+        <v>31.80275597097929</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -3896,14 +3899,17 @@
       <c r="N44" t="n">
         <v>0.09478672985781991</v>
       </c>
+      <c r="O44" t="n">
+        <v>0</v>
+      </c>
       <c r="P44" t="n">
         <v>57.39710789766407</v>
       </c>
       <c r="Q44" t="n">
-        <v>25.9</v>
+        <v>20.2</v>
       </c>
       <c r="R44" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S44" t="inlineStr">
         <is>
@@ -4011,10 +4017,10 @@
         <v>1115000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1501857</v>
+        <v>1502574</v>
       </c>
       <c r="L46" t="n">
-        <v>25.75857754766266</v>
+        <v>25.79400415553577</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -4026,7 +4032,7 @@
         <v>8.390274908628628</v>
       </c>
       <c r="Q46" t="n">
-        <v>12.8</v>
+        <v>12.9</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -4075,10 +4081,10 @@
         <v>1123000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1716469</v>
+        <v>1717288</v>
       </c>
       <c r="L47" t="n">
-        <v>34.57499086788052</v>
+        <v>34.60619302062322</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -4142,10 +4148,10 @@
         <v>1130000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1501857</v>
+        <v>1502574</v>
       </c>
       <c r="L48" t="n">
-        <v>24.75981401691373</v>
+        <v>24.79571721592414</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -4268,10 +4274,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1759392</v>
+        <v>1760231</v>
       </c>
       <c r="L50" t="n">
-        <v>34.35232171113658</v>
+        <v>34.38361215090519</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4332,10 +4338,10 @@
         <v>1155000</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>1759392</v>
+        <v>1760231</v>
       </c>
       <c r="L51" t="n">
-        <v>34.35232171113658</v>
+        <v>34.38361215090519</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -4396,10 +4402,10 @@
         <v>1185000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1587702</v>
+        <v>1588460</v>
       </c>
       <c r="L52" t="n">
-        <v>25.36382772081915</v>
+        <v>25.39944348614381</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -4460,10 +4466,10 @@
         <v>1185000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1587702</v>
+        <v>1588460</v>
       </c>
       <c r="L53" t="n">
-        <v>25.36382772081915</v>
+        <v>25.39944348614381</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -4524,10 +4530,10 @@
         <v>1200000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1888159</v>
+        <v>1889060</v>
       </c>
       <c r="L54" t="n">
-        <v>36.44603023368266</v>
+        <v>36.47634273130551</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -4588,10 +4594,10 @@
         <v>1200000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1888159</v>
+        <v>1889060</v>
       </c>
       <c r="L55" t="n">
-        <v>36.44603023368266</v>
+        <v>36.47634273130551</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -4714,10 +4720,10 @@
         <v>1240000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1673547</v>
+        <v>1674345</v>
       </c>
       <c r="L57" t="n">
-        <v>25.9058753653169</v>
+        <v>25.94118894254171</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -4778,10 +4784,10 @@
         <v>1255000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>1716469</v>
+        <v>1717288</v>
       </c>
       <c r="L58" t="n">
-        <v>26.88478498592168</v>
+        <v>26.91965471138214</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -4793,7 +4799,7 @@
         <v>68.52057842046719</v>
       </c>
       <c r="Q58" t="n">
-        <v>27.4</v>
+        <v>27.5</v>
       </c>
       <c r="R58" t="n">
         <v>3</v>
@@ -4904,10 +4910,10 @@
         <v>1280000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1716469</v>
+        <v>1717288</v>
       </c>
       <c r="L60" t="n">
-        <v>25.42830659918705</v>
+        <v>25.46387094069253</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -4971,10 +4977,10 @@
         <v>1298000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1759392</v>
+        <v>1760231</v>
       </c>
       <c r="L61" t="n">
-        <v>26.22451392299158</v>
+        <v>26.25967841720774</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -5097,10 +5103,10 @@
         <v>1335000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1802314</v>
+        <v>1803174</v>
       </c>
       <c r="L63" t="n">
-        <v>25.92855628930364</v>
+        <v>25.96388368510193</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -5161,10 +5167,10 @@
         <v>1420000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1931081</v>
+        <v>1932003</v>
       </c>
       <c r="L64" t="n">
-        <v>26.46605709444606</v>
+        <v>26.50114932533749</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -5225,10 +5231,10 @@
         <v>1430000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1931081</v>
+        <v>1932003</v>
       </c>
       <c r="L65" t="n">
-        <v>25.94821242609709</v>
+        <v>25.98355178537507</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -5289,10 +5295,10 @@
         <v>1430000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>2145694</v>
+        <v>2146718</v>
       </c>
       <c r="L66" t="n">
-        <v>33.35489589848319</v>
+        <v>33.38668609477351</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -5353,10 +5359,10 @@
         <v>1430000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>2145694</v>
+        <v>2146718</v>
       </c>
       <c r="L67" t="n">
-        <v>33.35489589848319</v>
+        <v>33.38668609477351</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -5479,10 +5485,10 @@
         <v>1480000</v>
       </c>
       <c r="K69" s="3" t="n">
-        <v>2016926</v>
+        <v>2017889</v>
       </c>
       <c r="L69" t="n">
-        <v>26.62100642264516</v>
+        <v>26.65602518275287</v>
       </c>
       <c r="M69" s="3" t="n">
         <v>0</v>
@@ -5605,10 +5611,10 @@
         <v>1605000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2188616</v>
+        <v>2189661</v>
       </c>
       <c r="L71" t="n">
-        <v>26.66598434809944</v>
+        <v>26.70098248084978</v>
       </c>
       <c r="M71" s="3" t="n">
         <v>0</v>
@@ -5620,7 +5626,7 @@
         <v>36.44392794886694</v>
       </c>
       <c r="Q71" t="n">
-        <v>19.2</v>
+        <v>19.3</v>
       </c>
       <c r="R71" t="n">
         <v>3</v>
@@ -5669,10 +5675,10 @@
         <v>1610000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2188616</v>
+        <v>2189661</v>
       </c>
       <c r="L72" t="n">
-        <v>26.43752947067919</v>
+        <v>26.47263663188046</v>
       </c>
       <c r="M72" s="3" t="n">
         <v>0</v>
@@ -5684,7 +5690,7 @@
         <v>25.72147975982957</v>
       </c>
       <c r="Q72" t="n">
-        <v>16.8</v>
+        <v>16.9</v>
       </c>
       <c r="R72" t="n">
         <v>3</v>
@@ -5733,10 +5739,10 @@
         <v>1615000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2188616</v>
+        <v>2189661</v>
       </c>
       <c r="L73" t="n">
-        <v>26.20907459325894</v>
+        <v>26.24429078291114</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
@@ -5797,10 +5803,10 @@
         <v>1630000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2231539</v>
+        <v>2232604</v>
       </c>
       <c r="L74" t="n">
-        <v>26.95623961759127</v>
+        <v>26.99108305816885</v>
       </c>
       <c r="M74" s="3" t="n">
         <v>0</v>
@@ -5861,10 +5867,10 @@
         <v>1690000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2317384</v>
+        <v>2318490</v>
       </c>
       <c r="L75" t="n">
-        <v>27.07294086780611</v>
+        <v>27.10772959986888</v>
       </c>
       <c r="M75" s="3" t="n">
         <v>0</v>
@@ -5925,10 +5931,10 @@
         <v>1705000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2317384</v>
+        <v>2318490</v>
       </c>
       <c r="L76" t="n">
-        <v>26.4256592778754</v>
+        <v>26.46075678566653</v>
       </c>
       <c r="M76" s="3" t="n">
         <v>0</v>
@@ -5989,10 +5995,10 @@
         <v>1725000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2360306</v>
+        <v>2361433</v>
       </c>
       <c r="L77" t="n">
-        <v>26.9162557736158</v>
+        <v>26.95113517935932</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
@@ -6053,10 +6059,10 @@
         <v>1780000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2446151</v>
+        <v>2447318</v>
       </c>
       <c r="L78" t="n">
-        <v>27.23261973606699</v>
+        <v>27.26731875465305</v>
       </c>
       <c r="M78" s="3" t="n">
         <v>0</v>
@@ -6117,10 +6123,10 @@
         <v>1875000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2574918</v>
+        <v>2576147</v>
       </c>
       <c r="L79" t="n">
-        <v>27.1821471596377</v>
+        <v>27.21688630346017</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
@@ -6181,10 +6187,10 @@
         <v>1910000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2617841</v>
+        <v>2619090</v>
       </c>
       <c r="L80" t="n">
-        <v>27.03911352904932</v>
+        <v>27.07390734949925</v>
       </c>
       <c r="M80" s="3" t="n">
         <v>0</v>
@@ -6245,10 +6251,10 @@
         <v>2020000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2746608</v>
+        <v>2747919</v>
       </c>
       <c r="L81" t="n">
-        <v>26.45473980997652</v>
+        <v>26.48982739301995</v>
       </c>
       <c r="M81" s="3" t="n">
         <v>0</v>
@@ -6309,10 +6315,10 @@
         <v>2110000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>2875376</v>
+        <v>2876748</v>
       </c>
       <c r="L82" t="n">
-        <v>26.61829270328472</v>
+        <v>26.65329045157935</v>
       </c>
       <c r="M82" s="3" t="n">
         <v>0</v>
@@ -6324,7 +6330,7 @@
         <v>79.02382335851249</v>
       </c>
       <c r="Q82" t="n">
-        <v>28.3</v>
+        <v>28.4</v>
       </c>
       <c r="R82" t="n">
         <v>3</v>
@@ -6373,10 +6379,10 @@
         <v>2210000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3004143</v>
+        <v>3005577</v>
       </c>
       <c r="L83" t="n">
-        <v>26.43492669956124</v>
+        <v>26.47002555582506</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
@@ -6437,10 +6443,10 @@
         <v>2215000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3047065</v>
+        <v>3048520</v>
       </c>
       <c r="L84" t="n">
-        <v>27.30709715742854</v>
+        <v>27.34179208271555</v>
       </c>
       <c r="M84" s="3" t="n">
         <v>0</v>
@@ -6501,10 +6507,10 @@
         <v>2315000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3175833</v>
+        <v>3177349</v>
       </c>
       <c r="L85" t="n">
-        <v>27.10573887228957</v>
+        <v>27.14051871544486</v>
       </c>
       <c r="M85" s="3" t="n">
         <v>0</v>
@@ -6565,10 +6571,10 @@
         <v>2395000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3304600</v>
+        <v>3306177</v>
       </c>
       <c r="L86" t="n">
-        <v>27.52526780850935</v>
+        <v>27.55983723799422</v>
       </c>
       <c r="M86" s="3" t="n">
         <v>0</v>
@@ -6629,10 +6635,10 @@
         <v>2410000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3304600</v>
+        <v>3306177</v>
       </c>
       <c r="L87" t="n">
-        <v>27.07135508079647</v>
+        <v>27.1061410202781</v>
       </c>
       <c r="M87" s="3" t="n">
         <v>0</v>
@@ -6693,10 +6699,10 @@
         <v>2499000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3433368</v>
+        <v>3435006</v>
       </c>
       <c r="L88" t="n">
-        <v>27.21432715630833</v>
+        <v>27.24903537286398</v>
       </c>
       <c r="M88" s="3" t="n">
         <v>0</v>
@@ -6757,10 +6763,10 @@
         <v>2510000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3433368</v>
+        <v>3435006</v>
       </c>
       <c r="L89" t="n">
-        <v>26.89394204175026</v>
+        <v>26.92880303556966</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
@@ -6772,7 +6778,7 @@
         <v>83.17546233649077</v>
       </c>
       <c r="Q89" t="n">
-        <v>29.3</v>
+        <v>29.4</v>
       </c>
       <c r="R89" t="n">
         <v>3</v>
@@ -6821,10 +6827,10 @@
         <v>2530000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3476290</v>
+        <v>3477949</v>
       </c>
       <c r="L90" t="n">
-        <v>27.22126174743764</v>
+        <v>27.25597758909058</v>
       </c>
       <c r="M90" s="3" t="n">
         <v>0</v>
@@ -6885,10 +6891,10 @@
         <v>2610000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>3605057</v>
+        <v>3606778</v>
       </c>
       <c r="L91" t="n">
-        <v>27.60169950156128</v>
+        <v>27.63624487007518</v>
       </c>
       <c r="M91" s="3" t="n">
         <v>0</v>
@@ -6949,10 +6955,10 @@
         <v>3015000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4163049</v>
+        <v>4165036</v>
       </c>
       <c r="L92" t="n">
-        <v>27.57711955828529</v>
+        <v>27.61167010321159</v>
       </c>
       <c r="M92" s="3" t="n">
         <v>0</v>
@@ -6964,7 +6970,7 @@
         <v>100</v>
       </c>
       <c r="Q92" t="n">
-        <v>33.2</v>
+        <v>33.3</v>
       </c>
       <c r="R92" t="n">
         <v>3</v>
@@ -7013,10 +7019,10 @@
         <v>3098000</v>
       </c>
       <c r="K93" s="3" t="n">
-        <v>4291817</v>
+        <v>4293865</v>
       </c>
       <c r="L93" t="n">
-        <v>27.8161207712258</v>
+        <v>27.85054956315581</v>
       </c>
       <c r="M93" s="3" t="n">
         <v>0</v>
@@ -7028,7 +7034,7 @@
         <v>100</v>
       </c>
       <c r="Q93" t="n">
-        <v>33.3</v>
+        <v>33.4</v>
       </c>
       <c r="R93" t="n">
         <v>3</v>
@@ -7312,10 +7318,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>428795</v>
+        <v>429000</v>
       </c>
       <c r="L2" t="n">
-        <v>27.70461409298149</v>
+        <v>27.73916083916084</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7379,10 +7385,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>428795</v>
+        <v>429000</v>
       </c>
       <c r="L3" t="n">
-        <v>27.70461409298149</v>
+        <v>27.73916083916084</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7446,10 +7452,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>428795</v>
+        <v>429000</v>
       </c>
       <c r="L4" t="n">
-        <v>27.70438088130692</v>
+        <v>27.73892773892774</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7513,10 +7519,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>428795</v>
+        <v>429000</v>
       </c>
       <c r="L5" t="n">
-        <v>27.70438088130692</v>
+        <v>27.73892773892774</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7580,10 +7586,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514640</v>
+        <v>514886</v>
       </c>
       <c r="L6" t="n">
-        <v>25.38473496036064</v>
+        <v>25.42038431808206</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7644,10 +7650,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>514640</v>
+        <v>514886</v>
       </c>
       <c r="L7" t="n">
-        <v>25.38473496036064</v>
+        <v>25.42038431808206</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7708,10 +7714,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>514640</v>
+        <v>514886</v>
       </c>
       <c r="L8" t="n">
-        <v>25.38473496036064</v>
+        <v>25.42038431808206</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7772,10 +7778,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>514640</v>
+        <v>514886</v>
       </c>
       <c r="L9" t="n">
-        <v>25.38473496036064</v>
+        <v>25.42038431808206</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7836,10 +7842,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>514640</v>
+        <v>514886</v>
       </c>
       <c r="L10" t="n">
-        <v>25.19042437431991</v>
+        <v>25.2261665689104</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7900,10 +7906,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>514640</v>
+        <v>514886</v>
       </c>
       <c r="L11" t="n">
-        <v>25.19042437431991</v>
+        <v>25.2261665689104</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7964,10 +7970,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>514640</v>
+        <v>514886</v>
       </c>
       <c r="L12" t="n">
-        <v>25.19042437431991</v>
+        <v>25.2261665689104</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -8028,10 +8034,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>514640</v>
+        <v>514886</v>
       </c>
       <c r="L13" t="n">
-        <v>25.19042437431991</v>
+        <v>25.2261665689104</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -8092,16 +8098,16 @@
         <v>415000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>557563</v>
+        <v>557829</v>
       </c>
       <c r="L14" t="n">
-        <v>25.56894915910848</v>
+        <v>25.60444150447538</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>1.658767772511848</v>
+        <v>1.425178147268409</v>
       </c>
       <c r="O14" t="n">
         <v>100</v>
@@ -8110,7 +8116,7 @@
         <v>3.478260869565196</v>
       </c>
       <c r="Q14" t="n">
-        <v>31.8</v>
+        <v>31.7</v>
       </c>
       <c r="R14" t="n">
         <v>4</v>
@@ -8159,16 +8165,16 @@
         <v>415000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>557563</v>
+        <v>557829</v>
       </c>
       <c r="L15" t="n">
-        <v>25.56894915910848</v>
+        <v>25.60444150447538</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>1.658767772511848</v>
+        <v>1.425178147268409</v>
       </c>
       <c r="O15" t="n">
         <v>100</v>
@@ -8177,7 +8183,7 @@
         <v>3.478260869565196</v>
       </c>
       <c r="Q15" t="n">
-        <v>31.8</v>
+        <v>31.7</v>
       </c>
       <c r="R15" t="n">
         <v>4</v>
@@ -8226,16 +8232,16 @@
         <v>415000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>557563</v>
+        <v>557829</v>
       </c>
       <c r="L16" t="n">
-        <v>25.56894915910848</v>
+        <v>25.60444150447538</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>1.658767772511848</v>
+        <v>1.425178147268409</v>
       </c>
       <c r="O16" t="n">
         <v>100</v>
@@ -8244,7 +8250,7 @@
         <v>3.478260869565196</v>
       </c>
       <c r="Q16" t="n">
-        <v>31.8</v>
+        <v>31.7</v>
       </c>
       <c r="R16" t="n">
         <v>4</v>
@@ -8293,10 +8299,10 @@
         <v>420000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>557563</v>
+        <v>557829</v>
       </c>
       <c r="L17" t="n">
-        <v>24.67218951042304</v>
+        <v>24.70810947440882</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -8360,10 +8366,10 @@
         <v>454000</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>600485</v>
+        <v>600772</v>
       </c>
       <c r="L18" t="n">
-        <v>24.39444782134441</v>
+        <v>24.43056600507347</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
@@ -8375,7 +8381,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q18" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="R18" t="n">
         <v>3</v>
@@ -8424,10 +8430,10 @@
         <v>454000</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>600485</v>
+        <v>600772</v>
       </c>
       <c r="L19" t="n">
-        <v>24.39444782134441</v>
+        <v>24.43056600507347</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0</v>
@@ -8439,7 +8445,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q19" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="R19" t="n">
         <v>3</v>
@@ -8488,10 +8494,10 @@
         <v>454000</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>600485</v>
+        <v>600772</v>
       </c>
       <c r="L20" t="n">
-        <v>24.39444782134441</v>
+        <v>24.43056600507347</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -8503,7 +8509,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q20" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="R20" t="n">
         <v>3</v>
@@ -8552,10 +8558,10 @@
         <v>454000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>600485</v>
+        <v>600772</v>
       </c>
       <c r="L21" t="n">
-        <v>24.39444782134441</v>
+        <v>24.43056600507347</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -8567,7 +8573,7 @@
         <v>6.504065040650378</v>
       </c>
       <c r="Q21" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="R21" t="n">
         <v>3</v>
@@ -8616,10 +8622,10 @@
         <v>455000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>600485</v>
+        <v>600772</v>
       </c>
       <c r="L22" t="n">
-        <v>24.22791576808746</v>
+        <v>24.26411350728729</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -8680,10 +8686,10 @@
         <v>455000</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>600485</v>
+        <v>600772</v>
       </c>
       <c r="L23" t="n">
-        <v>24.22791576808746</v>
+        <v>24.26411350728729</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -8744,10 +8750,10 @@
         <v>455000</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>600485</v>
+        <v>600772</v>
       </c>
       <c r="L24" t="n">
-        <v>24.22791576808746</v>
+        <v>24.26411350728729</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -8808,10 +8814,10 @@
         <v>455000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>600485</v>
+        <v>600772</v>
       </c>
       <c r="L25" t="n">
-        <v>24.22791576808746</v>
+        <v>24.26411350728729</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>0</v>
@@ -8872,10 +8878,10 @@
         <v>468000</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>686330</v>
+        <v>686658</v>
       </c>
       <c r="L26" t="n">
-        <v>31.81122783500648</v>
+        <v>31.84379997029089</v>
       </c>
       <c r="M26" s="3" t="n">
         <v>0</v>
@@ -8936,10 +8942,10 @@
         <v>468000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>686330</v>
+        <v>686658</v>
       </c>
       <c r="L27" t="n">
-        <v>31.81122783500648</v>
+        <v>31.84379997029089</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -9000,10 +9006,10 @@
         <v>468000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>686330</v>
+        <v>686658</v>
       </c>
       <c r="L28" t="n">
-        <v>31.81122783500648</v>
+        <v>31.84379997029089</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -9064,10 +9070,10 @@
         <v>468000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>686330</v>
+        <v>686658</v>
       </c>
       <c r="L29" t="n">
-        <v>31.81122783500648</v>
+        <v>31.84379997029089</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -9128,10 +9134,10 @@
         <v>474999</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>643408</v>
+        <v>643715</v>
       </c>
       <c r="L30" t="n">
-        <v>26.17452689428792</v>
+        <v>26.20973567494932</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -9195,10 +9201,10 @@
         <v>475000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>643408</v>
+        <v>643715</v>
       </c>
       <c r="L31" t="n">
-        <v>26.17437147191207</v>
+        <v>26.20958032669737</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -9262,10 +9268,10 @@
         <v>475000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>643408</v>
+        <v>643715</v>
       </c>
       <c r="L32" t="n">
-        <v>26.17437147191207</v>
+        <v>26.20958032669737</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -9329,10 +9335,10 @@
         <v>475000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>643408</v>
+        <v>643715</v>
       </c>
       <c r="L33" t="n">
-        <v>26.17437147191207</v>
+        <v>26.20958032669737</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -9396,10 +9402,10 @@
         <v>475000</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>686330</v>
+        <v>686658</v>
       </c>
       <c r="L34" t="n">
-        <v>30.7913103026241</v>
+        <v>30.82436962796618</v>
       </c>
       <c r="M34" s="3" t="n">
         <v>0</v>
@@ -9460,10 +9466,10 @@
         <v>475000</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>686330</v>
+        <v>686658</v>
       </c>
       <c r="L35" t="n">
-        <v>30.7913103026241</v>
+        <v>30.82436962796618</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0</v>
@@ -9524,10 +9530,10 @@
         <v>475000</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>686330</v>
+        <v>686658</v>
       </c>
       <c r="L36" t="n">
-        <v>30.7913103026241</v>
+        <v>30.82436962796618</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -9588,10 +9594,10 @@
         <v>475000</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>686330</v>
+        <v>686658</v>
       </c>
       <c r="L37" t="n">
-        <v>30.7913103026241</v>
+        <v>30.82436962796618</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0</v>
@@ -9652,10 +9658,10 @@
         <v>500000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>643408</v>
+        <v>643715</v>
       </c>
       <c r="L38" t="n">
-        <v>22.28881207569691</v>
+        <v>22.3258740281025</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -9681,11 +9687,11 @@
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHG4 M5 10C CPU 10C GPU 24GB 1TB Midnight</t>
+          <t>Apple MacBook Air 15 MDVK4 M5 10C CPU 10C GPU 16GB 1TB Midnight</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -9693,7 +9699,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E39" t="n">
         <v>1024</v>
@@ -9710,28 +9716,28 @@
         </is>
       </c>
       <c r="I39" s="3" t="n">
-        <v>544999</v>
+        <v>539999</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>544999</v>
+        <v>539999</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>772175</v>
+        <v>772544</v>
       </c>
       <c r="L39" t="n">
-        <v>29.42027390164147</v>
+        <v>30.10119811945986</v>
       </c>
       <c r="M39" s="3" t="n">
-        <v>0</v>
+        <v>-10000</v>
       </c>
       <c r="N39" t="n">
-        <v>0.547446254463968</v>
+        <v>2.350817994245921</v>
       </c>
       <c r="P39" t="n">
-        <v>64.69606956521737</v>
+        <v>37.58429530201343</v>
       </c>
       <c r="Q39" t="n">
-        <v>26.7</v>
+        <v>21.8</v>
       </c>
       <c r="R39" t="n">
         <v>3</v>
@@ -9745,11 +9751,11 @@
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHK4 M5 10C CPU 10C GPU 24GB 1TB Sky Blue</t>
+          <t>Apple MacBook Air 15 MDVA4 M5 10C CPU 10C GPU 16GB 1TB Silver</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -9757,7 +9763,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E40" t="n">
         <v>1024</v>
@@ -9770,32 +9776,32 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Sky Blue</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I40" s="3" t="n">
-        <v>544999</v>
+        <v>539999</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>544999</v>
+        <v>539999</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>772175</v>
+        <v>772544</v>
       </c>
       <c r="L40" t="n">
-        <v>29.42027390164147</v>
+        <v>30.10119811945986</v>
       </c>
       <c r="M40" s="3" t="n">
-        <v>0</v>
+        <v>-10000</v>
       </c>
       <c r="N40" t="n">
-        <v>0.547446254463968</v>
+        <v>2.350817994245921</v>
       </c>
       <c r="P40" t="n">
-        <v>64.69606956521737</v>
+        <v>37.58429530201343</v>
       </c>
       <c r="Q40" t="n">
-        <v>26.7</v>
+        <v>21.8</v>
       </c>
       <c r="R40" t="n">
         <v>3</v>
@@ -9809,11 +9815,11 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDH94 M5 10C CPU 10C GPU 24GB 1TB Silver</t>
+          <t>Apple MacBook Air 15 MDVE4 M5 10C CPU 10C GPU 16GB 1TB Starlight</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -9821,7 +9827,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E41" t="n">
         <v>1024</v>
@@ -9834,32 +9840,32 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Starlight</t>
         </is>
       </c>
       <c r="I41" s="3" t="n">
-        <v>544999</v>
+        <v>539999</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>544999</v>
+        <v>539999</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>772175</v>
+        <v>772544</v>
       </c>
       <c r="L41" t="n">
-        <v>29.42027390164147</v>
+        <v>30.10119811945986</v>
       </c>
       <c r="M41" s="3" t="n">
-        <v>0</v>
+        <v>-10000</v>
       </c>
       <c r="N41" t="n">
-        <v>0.547446254463968</v>
+        <v>2.350817994245921</v>
       </c>
       <c r="P41" t="n">
-        <v>64.69606956521737</v>
+        <v>37.58429530201343</v>
       </c>
       <c r="Q41" t="n">
-        <v>26.7</v>
+        <v>21.8</v>
       </c>
       <c r="R41" t="n">
         <v>3</v>
@@ -9873,11 +9879,11 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHD4 M5 10C CPU 10C GPU 24GB 1TB Starlight</t>
+          <t>Apple MacBook Air 15 MDVT4 M5 10C CPU 10C GPU 16GB 1TB Sky Blue</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -9885,7 +9891,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E42" t="n">
         <v>1024</v>
@@ -9898,32 +9904,32 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Starlight</t>
+          <t>Sky Blue</t>
         </is>
       </c>
       <c r="I42" s="3" t="n">
-        <v>544999</v>
+        <v>539999</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>544999</v>
+        <v>539999</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>772175</v>
+        <v>772544</v>
       </c>
       <c r="L42" t="n">
-        <v>29.42027390164147</v>
+        <v>30.10119811945986</v>
       </c>
       <c r="M42" s="3" t="n">
-        <v>0</v>
+        <v>-10000</v>
       </c>
       <c r="N42" t="n">
-        <v>0.547446254463968</v>
+        <v>2.350817994245921</v>
       </c>
       <c r="P42" t="n">
-        <v>64.69606956521737</v>
+        <v>37.58429530201343</v>
       </c>
       <c r="Q42" t="n">
-        <v>26.7</v>
+        <v>21.8</v>
       </c>
       <c r="R42" t="n">
         <v>3</v>
@@ -9937,11 +9943,11 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MDVK4 M5 10C CPU 10C GPU 16GB 1TB Midnight</t>
+          <t>Apple MacBook Air 13 MDHG4 M5 10C CPU 10C GPU 24GB 1TB Midnight</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -9949,7 +9955,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E43" t="n">
         <v>1024</v>
@@ -9966,28 +9972,28 @@
         </is>
       </c>
       <c r="I43" s="3" t="n">
-        <v>549999</v>
+        <v>544999</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>549999</v>
+        <v>544999</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>772175</v>
+        <v>772544</v>
       </c>
       <c r="L43" t="n">
-        <v>28.7727522906077</v>
+        <v>29.453985792395</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>0.5424964602105971</v>
+        <v>0.547446254463968</v>
       </c>
       <c r="P43" t="n">
-        <v>33.55744966442954</v>
+        <v>64.69606956521737</v>
       </c>
       <c r="Q43" t="n">
-        <v>19.7</v>
+        <v>26.7</v>
       </c>
       <c r="R43" t="n">
         <v>3</v>
@@ -10001,11 +10007,11 @@
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MDVA4 M5 10C CPU 10C GPU 16GB 1TB Silver</t>
+          <t>Apple MacBook Air 13 MDHK4 M5 10C CPU 10C GPU 24GB 1TB Sky Blue</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -10013,7 +10019,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E44" t="n">
         <v>1024</v>
@@ -10026,32 +10032,32 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Sky Blue</t>
         </is>
       </c>
       <c r="I44" s="3" t="n">
-        <v>549999</v>
+        <v>544999</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>549999</v>
+        <v>544999</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>772175</v>
+        <v>772544</v>
       </c>
       <c r="L44" t="n">
-        <v>28.7727522906077</v>
+        <v>29.453985792395</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>0.5424964602105971</v>
+        <v>0.547446254463968</v>
       </c>
       <c r="P44" t="n">
-        <v>33.55744966442954</v>
+        <v>64.69606956521737</v>
       </c>
       <c r="Q44" t="n">
-        <v>19.7</v>
+        <v>26.7</v>
       </c>
       <c r="R44" t="n">
         <v>3</v>
@@ -10065,11 +10071,11 @@
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MDVE4 M5 10C CPU 10C GPU 16GB 1TB Starlight</t>
+          <t>Apple MacBook Air 13 MDH94 M5 10C CPU 10C GPU 24GB 1TB Silver</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -10077,7 +10083,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E45" t="n">
         <v>1024</v>
@@ -10090,32 +10096,32 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Starlight</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="I45" s="3" t="n">
-        <v>549999</v>
+        <v>544999</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>549999</v>
+        <v>544999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>772175</v>
+        <v>772544</v>
       </c>
       <c r="L45" t="n">
-        <v>28.7727522906077</v>
+        <v>29.453985792395</v>
       </c>
       <c r="M45" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>0.5424964602105971</v>
+        <v>0.547446254463968</v>
       </c>
       <c r="P45" t="n">
-        <v>33.55744966442954</v>
+        <v>64.69606956521737</v>
       </c>
       <c r="Q45" t="n">
-        <v>19.7</v>
+        <v>26.7</v>
       </c>
       <c r="R45" t="n">
         <v>3</v>
@@ -10129,11 +10135,11 @@
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 15 MDVT4 M5 10C CPU 10C GPU 16GB 1TB Sky Blue</t>
+          <t>Apple MacBook Air 13 MDHD4 M5 10C CPU 10C GPU 24GB 1TB Starlight</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -10141,7 +10147,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E46" t="n">
         <v>1024</v>
@@ -10154,32 +10160,32 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Sky Blue</t>
+          <t>Starlight</t>
         </is>
       </c>
       <c r="I46" s="3" t="n">
-        <v>549999</v>
+        <v>544999</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>549999</v>
+        <v>544999</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>772175</v>
+        <v>772544</v>
       </c>
       <c r="L46" t="n">
-        <v>28.7727522906077</v>
+        <v>29.453985792395</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N46" t="n">
-        <v>0.5424964602105971</v>
+        <v>0.547446254463968</v>
       </c>
       <c r="P46" t="n">
-        <v>33.55744966442954</v>
+        <v>64.69606956521737</v>
       </c>
       <c r="Q46" t="n">
-        <v>19.7</v>
+        <v>26.7</v>
       </c>
       <c r="R46" t="n">
         <v>3</v>
@@ -10228,10 +10234,10 @@
         <v>585000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>729253</v>
+        <v>729601</v>
       </c>
       <c r="L47" t="n">
-        <v>19.78092650972982</v>
+        <v>19.81918884431353</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -10243,7 +10249,7 @@
         <v>19.46308724832216</v>
       </c>
       <c r="Q47" t="n">
-        <v>12.6</v>
+        <v>12.7</v>
       </c>
       <c r="R47" t="n">
         <v>3</v>
@@ -10292,10 +10298,10 @@
         <v>595000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>729253</v>
+        <v>729601</v>
       </c>
       <c r="L48" t="n">
-        <v>18.40966029622093</v>
+        <v>18.44857668780607</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -10356,10 +10362,10 @@
         <v>619999</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>858020</v>
+        <v>858429</v>
       </c>
       <c r="L49" t="n">
-        <v>27.74072865434372</v>
+        <v>27.77515671068894</v>
       </c>
       <c r="M49" s="3" t="n">
         <v>0</v>
@@ -10371,7 +10377,7 @@
         <v>55.30233557046979</v>
       </c>
       <c r="Q49" t="n">
-        <v>23.7</v>
+        <v>23.8</v>
       </c>
       <c r="R49" t="n">
         <v>3</v>
@@ -10420,10 +10426,10 @@
         <v>619999</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>858020</v>
+        <v>858429</v>
       </c>
       <c r="L50" t="n">
-        <v>27.74072865434372</v>
+        <v>27.77515671068894</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -10435,7 +10441,7 @@
         <v>55.30233557046979</v>
       </c>
       <c r="Q50" t="n">
-        <v>23.7</v>
+        <v>23.8</v>
       </c>
       <c r="R50" t="n">
         <v>3</v>
@@ -10484,10 +10490,10 @@
         <v>619999</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>858020</v>
+        <v>858429</v>
       </c>
       <c r="L51" t="n">
-        <v>27.74072865434372</v>
+        <v>27.77515671068894</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -10499,7 +10505,7 @@
         <v>55.30233557046979</v>
       </c>
       <c r="Q51" t="n">
-        <v>23.7</v>
+        <v>23.8</v>
       </c>
       <c r="R51" t="n">
         <v>3</v>
@@ -10548,10 +10554,10 @@
         <v>619999</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>858020</v>
+        <v>858429</v>
       </c>
       <c r="L52" t="n">
-        <v>27.74072865434372</v>
+        <v>27.77515671068894</v>
       </c>
       <c r="M52" s="3" t="n">
         <v>0</v>
@@ -10563,7 +10569,7 @@
         <v>55.30233557046979</v>
       </c>
       <c r="Q52" t="n">
-        <v>23.7</v>
+        <v>23.8</v>
       </c>
       <c r="R52" t="n">
         <v>3</v>
@@ -10612,10 +10618,10 @@
         <v>650000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>815098</v>
+        <v>815487</v>
       </c>
       <c r="L53" t="n">
-        <v>20.25498774380504</v>
+        <v>20.29302735665927</v>
       </c>
       <c r="M53" s="3" t="n">
         <v>0</v>
@@ -10676,10 +10682,10 @@
         <v>672000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>858020</v>
+        <v>858429</v>
       </c>
       <c r="L54" t="n">
-        <v>21.68014731591338</v>
+        <v>21.71746294684825</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -10740,10 +10746,10 @@
         <v>700000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>900942</v>
+        <v>901372</v>
       </c>
       <c r="L55" t="n">
-        <v>22.30354451229935</v>
+        <v>22.34060964840266</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -10804,10 +10810,10 @@
         <v>715000</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>943865</v>
+        <v>944315</v>
       </c>
       <c r="L56" t="n">
-        <v>24.24764134701467</v>
+        <v>24.28374006555016</v>
       </c>
       <c r="M56" s="3" t="n">
         <v>0</v>
@@ -10868,10 +10874,10 @@
         <v>734999</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>986787</v>
+        <v>987258</v>
       </c>
       <c r="L57" t="n">
-        <v>25.51594214354263</v>
+        <v>25.55147691890063</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -10932,10 +10938,10 @@
         <v>752000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>986787</v>
+        <v>987258</v>
       </c>
       <c r="L58" t="n">
-        <v>23.79307793880544</v>
+        <v>23.82943465639174</v>
       </c>
       <c r="M58" s="3" t="n">
         <v>0</v>
@@ -10996,10 +11002,10 @@
         <v>810000</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1072632</v>
+        <v>1073144</v>
       </c>
       <c r="L59" t="n">
-        <v>24.48481865169042</v>
+        <v>24.52084715564733</v>
       </c>
       <c r="M59" s="3" t="n">
         <v>0</v>
@@ -11060,10 +11066,10 @@
         <v>815000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1072632</v>
+        <v>1073144</v>
       </c>
       <c r="L60" t="n">
-        <v>24.01867555694777</v>
+        <v>24.05492645907725</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -11075,7 +11081,7 @@
         <v>79.56521739130434</v>
       </c>
       <c r="Q60" t="n">
-        <v>27.3</v>
+        <v>27.4</v>
       </c>
       <c r="R60" t="n">
         <v>3</v>
@@ -11124,10 +11130,10 @@
         <v>875000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1158477</v>
+        <v>1159030</v>
       </c>
       <c r="L61" t="n">
-        <v>24.46979957306015</v>
+        <v>24.50583677730516</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -11188,10 +11194,10 @@
         <v>992000</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>1330167</v>
+        <v>1330802</v>
       </c>
       <c r="L62" t="n">
-        <v>25.42289802708983</v>
+        <v>25.45848292984231</v>
       </c>
       <c r="M62" s="3" t="n">
         <v>0</v>
@@ -11203,7 +11209,7 @@
         <v>85.14782608695651</v>
       </c>
       <c r="Q62" t="n">
-        <v>29.1</v>
+        <v>29.2</v>
       </c>
       <c r="R62" t="n">
         <v>3</v>
@@ -11252,10 +11258,10 @@
         <v>1050000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1416012</v>
+        <v>1416688</v>
       </c>
       <c r="L63" t="n">
-        <v>25.84808603316921</v>
+        <v>25.88346904893667</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -11316,10 +11322,10 @@
         <v>1050000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1416012</v>
+        <v>1416688</v>
       </c>
       <c r="L64" t="n">
-        <v>25.84808603316921</v>
+        <v>25.88346904893667</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -11380,10 +11386,10 @@
         <v>1100000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1501857</v>
+        <v>1502574</v>
       </c>
       <c r="L65" t="n">
-        <v>26.7573410784116</v>
+        <v>26.79229109514739</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -11444,10 +11450,10 @@
         <v>1105000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1501857</v>
+        <v>1502574</v>
       </c>
       <c r="L66" t="n">
-        <v>26.42441990149528</v>
+        <v>26.45952878194352</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -11508,10 +11514,10 @@
         <v>1155000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>1587702</v>
+        <v>1588460</v>
       </c>
       <c r="L67" t="n">
-        <v>27.25335106965916</v>
+        <v>27.28806517003891</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -11778,7 +11784,7 @@
         <v>315000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>300028</v>
+        <v>300171</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -11839,10 +11845,10 @@
         <v>380000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>385873</v>
+        <v>386057</v>
       </c>
       <c r="L3" t="n">
-        <v>1.522003353434938</v>
+        <v>1.568939301709333</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -11903,7 +11909,7 @@
         <v>415000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>385873</v>
+        <v>386057</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -11964,10 +11970,10 @@
         <v>495000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>471718</v>
+        <v>471943</v>
       </c>
       <c r="L5" t="n">
-        <v>6.724144510067455</v>
+        <v>6.768614006352462</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -12028,10 +12034,10 @@
         <v>490000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514640</v>
+        <v>514886</v>
       </c>
       <c r="L6" t="n">
-        <v>4.787812840043525</v>
+        <v>4.833302905885963</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -12092,10 +12098,10 @@
         <v>550000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>557563</v>
+        <v>557829</v>
       </c>
       <c r="L7" t="n">
-        <v>6.736996536714236</v>
+        <v>6.781468873077593</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -12156,7 +12162,7 @@
         <v>530000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>471718</v>
+        <v>471943</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -12220,10 +12226,10 @@
         <v>600000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>600485</v>
+        <v>600772</v>
       </c>
       <c r="L9" t="n">
-        <v>8.407370708677153</v>
+        <v>8.451126217600022</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -12284,7 +12290,7 @@
         <v>590000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>514640</v>
+        <v>514886</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
@@ -12345,10 +12351,10 @@
         <v>646000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>729253</v>
+        <v>729601</v>
       </c>
       <c r="L11" t="n">
-        <v>17.03853120933339</v>
+        <v>17.07810159251427</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -12409,7 +12415,7 @@
         <v>615000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>557563</v>
+        <v>557829</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -12473,7 +12479,7 @@
         <v>655000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>557563</v>
+        <v>557829</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -12537,7 +12543,7 @@
         <v>700000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>643408</v>
+        <v>643715</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -12601,7 +12607,7 @@
         <v>745000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>686330</v>
+        <v>686658</v>
       </c>
       <c r="L15" t="n">
         <v>0</v>
@@ -12665,7 +12671,7 @@
         <v>755000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>643408</v>
+        <v>643715</v>
       </c>
       <c r="L16" t="n">
         <v>0</v>
@@ -12729,7 +12735,7 @@
         <v>930000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>858020</v>
+        <v>858429</v>
       </c>
       <c r="L17" t="n">
         <v>0</v>
@@ -12803,7 +12809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12852,7 +12858,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Macbook Pro 16 MGEA4 M5 Pro 18 Core CPU 20 Core GPU 24GB 1TB Space Black</t>
+          <t>Macbook Pro 16 MGEC4 M5 Pro 18 Core CPU 20 Core GPU 48GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -12861,45 +12867,189 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>820000</v>
+        <v>1054000</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>815999</v>
+        <v>1044000</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-4001</v>
+        <v>-10000</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.49</v>
+        <v>-0.95</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Apple MacBook Pro 16Inch MX2X3 14Core CPU 20Core GPU M4 Pro 24GB 512GB Space Black</t>
+          <t>Apple MacBook Air 15 MDVK4 M5 10C CPU 10C GPU 16GB 1TB Midnight</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>711999</v>
+        <v>549999</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>719999</v>
+        <v>539999</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>8000</v>
+        <v>-10000</v>
       </c>
       <c r="F3" t="n">
-        <v>1.12</v>
+        <v>-1.82</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 15 MDVA4 M5 10C CPU 10C GPU 16GB 1TB Silver</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>549999</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>539999</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>-10000</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-1.82</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 15 MDVE4 M5 10C CPU 10C GPU 16GB 1TB Starlight</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>549999</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>539999</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>-10000</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-1.82</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 15 MDVT4 M5 10C CPU 10C GPU 16GB 1TB Sky Blue</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>549999</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>539999</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>-10000</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-1.82</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Macbook Pro 14 M5 MDE14 10 Core CPU 10 Core GPU 16GB 1TB Space Black</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>578999</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>574999</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>-4000</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-0.6899999999999999</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Macbook Pro 14 MGDR4 M5 Pro 15 Core CPU 16 Core GPU 24GB 1TB Space Black</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>717999</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>714999</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>-3000</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-0.42</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Macbook Pro 14 M5 MDE54 10 Core CPU 10 Core GPU 16GB 1TB Silver</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>584999</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>582999</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>-2000</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-0.34</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F3"/>
-  <conditionalFormatting sqref="E2:E3">
+  <autoFilter ref="A1:F9"/>
+  <conditionalFormatting sqref="E2:E9">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
chore: price data 2026-10-16
</commit_message>
<xml_diff>
--- a/web/downloads/applemac-prices.xlsx
+++ b/web/downloads/applemac-prices.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MacBook Pro'!$A$1:$S$93</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MacBook Air'!$A$1:$S$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'iPhone'!$A$1:$S$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Price Changes'!$A$1:$F$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20261015T082307180226+0000</t>
+          <t>20261016T081534274858+0000</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-15T08:23:07.180226+00:00</t>
+          <t>2026-10-16T08:15:34.274858+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>276.883421</v>
+        <v>276.982736</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -864,19 +864,19 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHK4 M5 10C CPU 10C GPU 24GB 1TB Sky Blue</t>
+          <t>Macbook Pro 14 M5 MDE34 10 Core CPU 10 Core GPU 24GB 1TB Space Black</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>macbook_air</t>
+          <t>macbook_pro</t>
         </is>
       </c>
       <c r="C29" s="3" t="n">
-        <v>527000</v>
+        <v>640000</v>
       </c>
       <c r="D29" t="n">
-        <v>44.8</v>
+        <v>44.9</v>
       </c>
       <c r="E29" t="n">
         <v>4</v>
@@ -885,7 +885,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDH94 M5 10C CPU 10C GPU 24GB 1TB Silver</t>
+          <t>Apple MacBook Air 13 MDHK4 M5 10C CPU 10C GPU 24GB 1TB Sky Blue</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -906,7 +906,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Apple MacBook Air 13 MDHD4 M5 10C CPU 10C GPU 24GB 1TB Starlight</t>
+          <t>Apple MacBook Air 13 MDH94 M5 10C CPU 10C GPU 24GB 1TB Silver</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1147,10 +1147,10 @@
         <v>495000</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>686242</v>
+        <v>686488</v>
       </c>
       <c r="L2" t="n">
-        <v>27.86801157609123</v>
+        <v>27.89385976156903</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -1214,10 +1214,10 @@
         <v>498000</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>686242</v>
+        <v>686488</v>
       </c>
       <c r="L3" t="n">
-        <v>27.43084800988573</v>
+        <v>27.45685285103309</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -1232,7 +1232,7 @@
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>9.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="R3" t="n">
         <v>4</v>
@@ -1281,10 +1281,10 @@
         <v>550000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>772076</v>
+        <v>772353</v>
       </c>
       <c r="L4" t="n">
-        <v>35.23966552515556</v>
+        <v>35.26289144989402</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -1348,10 +1348,10 @@
         <v>550000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>772076</v>
+        <v>772353</v>
       </c>
       <c r="L5" t="n">
-        <v>32.64924696532466</v>
+        <v>32.67340192891074</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -1415,10 +1415,10 @@
         <v>532000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>857909</v>
+        <v>858217</v>
       </c>
       <c r="L6" t="n">
-        <v>37.98876104575194</v>
+        <v>38.01101586195566</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -1606,10 +1606,10 @@
         <v>565000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>857909</v>
+        <v>858217</v>
       </c>
       <c r="L9" t="n">
-        <v>34.14219923092076</v>
+        <v>34.1658345150469</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -1667,31 +1667,31 @@
         </is>
       </c>
       <c r="I10" s="3" t="n">
-        <v>574999</v>
+        <v>578999</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>574999</v>
+        <v>578999</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>857909</v>
+        <v>858217</v>
       </c>
       <c r="L10" t="n">
-        <v>32.97669100102691</v>
+        <v>32.53466197942944</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="N10" t="n">
-        <v>1.372215046681041</v>
+        <v>0.6861075233405204</v>
       </c>
       <c r="O10" t="n">
         <v>100</v>
       </c>
       <c r="P10" t="n">
-        <v>51.50029999999999</v>
+        <v>50.30029999999999</v>
       </c>
       <c r="Q10" t="n">
-        <v>42.2</v>
+        <v>41.6</v>
       </c>
       <c r="R10" t="n">
         <v>4</v>
@@ -1740,10 +1740,10 @@
         <v>582999</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>857909</v>
+        <v>858217</v>
       </c>
       <c r="L11" t="n">
-        <v>32.04419116712845</v>
+        <v>32.06857939192535</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -1807,10 +1807,10 @@
         <v>634000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>857909</v>
+        <v>858217</v>
       </c>
       <c r="L12" t="n">
-        <v>26.09938816354648</v>
+        <v>26.1259098806013</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -1871,10 +1871,10 @@
         <v>634000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>857909</v>
+        <v>858217</v>
       </c>
       <c r="L13" t="n">
-        <v>26.09938816354648</v>
+        <v>26.1259098806013</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -1929,31 +1929,31 @@
         </is>
       </c>
       <c r="I14" s="3" t="n">
-        <v>642999</v>
+        <v>640000</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>642999</v>
+        <v>640000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>943743</v>
+        <v>944082</v>
       </c>
       <c r="L14" t="n">
-        <v>31.86715027290269</v>
+        <v>32.2092784313227</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>0</v>
+        <v>-2999</v>
       </c>
       <c r="N14" t="n">
-        <v>0.1552797442232053</v>
+        <v>0.620963697148598</v>
       </c>
       <c r="O14" t="n">
         <v>100</v>
       </c>
       <c r="P14" t="n">
-        <v>69.68024</v>
+        <v>70.39999999999999</v>
       </c>
       <c r="Q14" t="n">
-        <v>44.5</v>
+        <v>44.9</v>
       </c>
       <c r="R14" t="n">
         <v>4</v>
@@ -1996,31 +1996,31 @@
         </is>
       </c>
       <c r="I15" s="3" t="n">
-        <v>645000</v>
+        <v>642999</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>645000</v>
+        <v>642999</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>943743</v>
+        <v>944082</v>
       </c>
       <c r="L15" t="n">
-        <v>31.65512221017798</v>
+        <v>31.89161534697198</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>-5000</v>
+        <v>-2001</v>
       </c>
       <c r="N15" t="n">
-        <v>0.7692307692307693</v>
+        <v>1.077076923076923</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
       </c>
       <c r="P15" t="n">
-        <v>69.19999999999999</v>
+        <v>69.68024</v>
       </c>
       <c r="Q15" t="n">
-        <v>22.3</v>
+        <v>22.5</v>
       </c>
       <c r="R15" t="n">
         <v>4</v>
@@ -2128,10 +2128,10 @@
         <v>700000</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1029577</v>
+        <v>1029946</v>
       </c>
       <c r="L17" t="n">
-        <v>32.0109132197009</v>
+        <v>32.03527175211128</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>0</v>
@@ -2196,7 +2196,7 @@
       </c>
       <c r="K18" s="3" t="n"/>
       <c r="M18" s="3" t="n">
-        <v>-4999</v>
+        <v>0</v>
       </c>
       <c r="N18" t="n">
         <v>1.388888888888889</v>
@@ -2258,7 +2258,7 @@
       </c>
       <c r="K19" s="3" t="n"/>
       <c r="M19" s="3" t="n">
-        <v>-4501</v>
+        <v>0</v>
       </c>
       <c r="N19" t="n">
         <v>0.8277241379310345</v>
@@ -2319,10 +2319,10 @@
         <v>719999</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>1072494</v>
+        <v>1072879</v>
       </c>
       <c r="L20" t="n">
-        <v>32.86685053715918</v>
+        <v>32.89094110333038</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
@@ -2337,7 +2337,7 @@
         <v>8.21045385007649</v>
       </c>
       <c r="Q20" t="n">
-        <v>34.5</v>
+        <v>34.6</v>
       </c>
       <c r="R20" t="n">
         <v>4</v>
@@ -2386,10 +2386,10 @@
         <v>720000</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>1029577</v>
+        <v>1029946</v>
       </c>
       <c r="L21" t="n">
-        <v>30.06836788312093</v>
+        <v>30.09342237360017</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0</v>
@@ -2453,10 +2453,10 @@
         <v>743000</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>1072494</v>
+        <v>1072879</v>
       </c>
       <c r="L22" t="n">
-        <v>30.72222315462837</v>
+        <v>30.74708331508026</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0</v>
@@ -2520,10 +2520,10 @@
         <v>759999</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>1029577</v>
+        <v>1029946</v>
       </c>
       <c r="L23" t="n">
-        <v>26.18337433722781</v>
+        <v>26.20982070904688</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>0</v>
@@ -2587,10 +2587,10 @@
         <v>759999</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>1029577</v>
+        <v>1029946</v>
       </c>
       <c r="L24" t="n">
-        <v>26.18337433722781</v>
+        <v>26.20982070904688</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0</v>
@@ -2655,7 +2655,7 @@
       </c>
       <c r="K25" s="3" t="n"/>
       <c r="M25" s="3" t="n">
-        <v>-5000</v>
+        <v>0</v>
       </c>
       <c r="N25" t="n">
         <v>2.531645569620253</v>
@@ -2717,7 +2717,7 @@
       </c>
       <c r="K26" s="3" t="n"/>
       <c r="M26" s="3" t="n">
-        <v>-5000</v>
+        <v>0</v>
       </c>
       <c r="N26" t="n">
         <v>5.521472392638037</v>
@@ -2778,10 +2778,10 @@
         <v>772000</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>1029577</v>
+        <v>1029946</v>
       </c>
       <c r="L27" t="n">
-        <v>25.017750008013</v>
+        <v>25.04461398947129</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>0</v>
@@ -2845,10 +2845,10 @@
         <v>810000</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>1072494</v>
+        <v>1072879</v>
       </c>
       <c r="L28" t="n">
-        <v>24.47510195861236</v>
+        <v>24.50220388319652</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>0</v>
@@ -2909,10 +2909,10 @@
         <v>810000</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>1244162</v>
+        <v>1244608</v>
       </c>
       <c r="L29" t="n">
-        <v>34.89593798878281</v>
+        <v>34.91926775338099</v>
       </c>
       <c r="M29" s="3" t="n">
         <v>0</v>
@@ -2976,10 +2976,10 @@
         <v>815999</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1287079</v>
+        <v>1287540</v>
       </c>
       <c r="L30" t="n">
-        <v>36.60070593957325</v>
+        <v>36.62340587476894</v>
       </c>
       <c r="M30" s="3" t="n">
         <v>0</v>
@@ -3043,10 +3043,10 @@
         <v>820000</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>1287079</v>
+        <v>1287540</v>
       </c>
       <c r="L31" t="n">
-        <v>36.28984701016799</v>
+        <v>36.31265824751076</v>
       </c>
       <c r="M31" s="3" t="n">
         <v>0</v>
@@ -3110,10 +3110,10 @@
         <v>930000</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1372913</v>
+        <v>1373405</v>
       </c>
       <c r="L32" t="n">
-        <v>38.2335952824396</v>
+        <v>38.25572209217237</v>
       </c>
       <c r="M32" s="3" t="n">
         <v>0</v>
@@ -3177,10 +3177,10 @@
         <v>930000</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1372913</v>
+        <v>1373405</v>
       </c>
       <c r="L33" t="n">
-        <v>38.08791962782784</v>
+        <v>38.11009862349416</v>
       </c>
       <c r="M33" s="3" t="n">
         <v>0</v>
@@ -3245,7 +3245,7 @@
       </c>
       <c r="K34" s="3" t="n"/>
       <c r="M34" s="3" t="n">
-        <v>-100000</v>
+        <v>0</v>
       </c>
       <c r="N34" t="n">
         <v>1.155955093589704</v>
@@ -3307,7 +3307,7 @@
       </c>
       <c r="K35" s="3" t="n"/>
       <c r="M35" s="3" t="n">
-        <v>-100000</v>
+        <v>0</v>
       </c>
       <c r="N35" t="n">
         <v>2.285714285714286</v>
@@ -3368,10 +3368,10 @@
         <v>860000</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>1244162</v>
+        <v>1244608</v>
       </c>
       <c r="L36" t="n">
-        <v>30.87716872883113</v>
+        <v>30.90193860235512</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>0</v>
@@ -3497,10 +3497,10 @@
         <v>880000</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>1158328</v>
+        <v>1158743</v>
       </c>
       <c r="L38" t="n">
-        <v>24.02842718124745</v>
+        <v>24.0556361505528</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0</v>
@@ -3561,10 +3561,10 @@
         <v>940000</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>1244162</v>
+        <v>1244608</v>
       </c>
       <c r="L39" t="n">
-        <v>24.44713791290845</v>
+        <v>24.47421196071373</v>
       </c>
       <c r="M39" s="3" t="n">
         <v>0</v>
@@ -3625,10 +3625,10 @@
         <v>990000</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>1501663</v>
+        <v>1502202</v>
       </c>
       <c r="L40" t="n">
-        <v>34.07309096648183</v>
+        <v>34.0967459769059</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0</v>
@@ -3754,10 +3754,10 @@
         <v>1000000</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>1501663</v>
+        <v>1502202</v>
       </c>
       <c r="L42" t="n">
-        <v>33.40716259240589</v>
+        <v>33.43105654232919</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0</v>
@@ -3821,13 +3821,13 @@
         <v>1043000</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>1544580</v>
+        <v>1545134</v>
       </c>
       <c r="L43" t="n">
-        <v>32.47355268098771</v>
+        <v>32.49776394798121</v>
       </c>
       <c r="M43" s="3" t="n">
-        <v>-1000</v>
+        <v>0</v>
       </c>
       <c r="N43" t="n">
         <v>1.137440758293839</v>
@@ -3888,10 +3888,10 @@
         <v>1054000</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>1544580</v>
+        <v>1545134</v>
       </c>
       <c r="L44" t="n">
-        <v>31.76138497196649</v>
+        <v>31.78585158309894</v>
       </c>
       <c r="M44" s="3" t="n">
         <v>0</v>
@@ -4017,10 +4017,10 @@
         <v>1115000</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>1501663</v>
+        <v>1502202</v>
       </c>
       <c r="L46" t="n">
-        <v>25.74898629053256</v>
+        <v>25.77562804469705</v>
       </c>
       <c r="M46" s="3" t="n">
         <v>0</v>
@@ -4081,10 +4081,10 @@
         <v>1123000</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>1716248</v>
+        <v>1716864</v>
       </c>
       <c r="L47" t="n">
-        <v>34.56656613729484</v>
+        <v>34.59004324163125</v>
       </c>
       <c r="M47" s="3" t="n">
         <v>0</v>
@@ -4148,10 +4148,10 @@
         <v>1130000</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>1501663</v>
+        <v>1502202</v>
       </c>
       <c r="L48" t="n">
-        <v>24.75009372941865</v>
+        <v>24.77709389283199</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -4274,10 +4274,10 @@
         <v>1155000</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>1759165</v>
+        <v>1759796</v>
       </c>
       <c r="L50" t="n">
-        <v>34.34385063368132</v>
+        <v>34.36739258414043</v>
       </c>
       <c r="M50" s="3" t="n">
         <v>0</v>
@@ -4289,7 +4289,7 @@
         <v>22.53136001640632</v>
       </c>
       <c r="Q50" t="n">
-        <v>19.5</v>
+        <v>19.6</v>
       </c>
       <c r="R50" t="n">
         <v>3</v>
@@ -4338,10 +4338,10 @@
         <v>1155000</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>1759165</v>
+        <v>1759796</v>
       </c>
       <c r="L51" t="n">
-        <v>34.34385063368132</v>
+        <v>34.36739258414043</v>
       </c>
       <c r="M51" s="3" t="n">
         <v>0</v>
@@ -4353,7 +4353,7 @@
         <v>22.53136001640632</v>
       </c>
       <c r="Q51" t="n">
-        <v>19.5</v>
+        <v>19.6</v>
       </c>
       <c r="R51" t="n">
         <v>3</v>
@@ -4402,13 +4402,13 @@
         <v>1175000</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>1887916</v>
+        <v>1888593</v>
       </c>
       <c r="L52" t="n">
-        <v>37.76206144764915</v>
+        <v>37.7843717518809</v>
       </c>
       <c r="M52" s="3" t="n">
-        <v>-25000</v>
+        <v>0</v>
       </c>
       <c r="N52" t="n">
         <v>2.083333333333333</v>
@@ -4466,13 +4466,13 @@
         <v>1175000</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1887916</v>
+        <v>1888593</v>
       </c>
       <c r="L53" t="n">
-        <v>37.76206144764915</v>
+        <v>37.7843717518809</v>
       </c>
       <c r="M53" s="3" t="n">
-        <v>-25000</v>
+        <v>0</v>
       </c>
       <c r="N53" t="n">
         <v>2.083333333333333</v>
@@ -4530,10 +4530,10 @@
         <v>1185000</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>1587497</v>
+        <v>1588067</v>
       </c>
       <c r="L54" t="n">
-        <v>25.35418964571272</v>
+        <v>25.38098203665211</v>
       </c>
       <c r="M54" s="3" t="n">
         <v>0</v>
@@ -4594,10 +4594,10 @@
         <v>1185000</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>1587497</v>
+        <v>1588067</v>
       </c>
       <c r="L55" t="n">
-        <v>25.35418964571272</v>
+        <v>25.38098203665211</v>
       </c>
       <c r="M55" s="3" t="n">
         <v>0</v>
@@ -4720,10 +4720,10 @@
         <v>1240000</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>1673331</v>
+        <v>1673931</v>
       </c>
       <c r="L57" t="n">
-        <v>25.89631101079225</v>
+        <v>25.92287256762674</v>
       </c>
       <c r="M57" s="3" t="n">
         <v>0</v>
@@ -4784,13 +4784,13 @@
         <v>1250000</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>1716248</v>
+        <v>1716864</v>
       </c>
       <c r="L58" t="n">
-        <v>27.16670318042614</v>
+        <v>27.19283530902856</v>
       </c>
       <c r="M58" s="3" t="n">
-        <v>-5000</v>
+        <v>0</v>
       </c>
       <c r="N58" t="n">
         <v>3.846153846153846</v>
@@ -4910,10 +4910,10 @@
         <v>1280000</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>1716248</v>
+        <v>1716864</v>
       </c>
       <c r="L60" t="n">
-        <v>25.41870405675636</v>
+        <v>25.44546335644524</v>
       </c>
       <c r="M60" s="3" t="n">
         <v>0</v>
@@ -4977,10 +4977,10 @@
         <v>1298000</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>1759165</v>
+        <v>1759796</v>
       </c>
       <c r="L61" t="n">
-        <v>26.21499404547044</v>
+        <v>26.24145071360544</v>
       </c>
       <c r="M61" s="3" t="n">
         <v>0</v>
@@ -5103,10 +5103,10 @@
         <v>1335000</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>1802082</v>
+        <v>1802728</v>
       </c>
       <c r="L63" t="n">
-        <v>25.91902033314799</v>
+        <v>25.94556694076977</v>
       </c>
       <c r="M63" s="3" t="n">
         <v>0</v>
@@ -5167,10 +5167,10 @@
         <v>1420000</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>1930833</v>
+        <v>1931525</v>
       </c>
       <c r="L64" t="n">
-        <v>26.45661224973884</v>
+        <v>26.48296035515979</v>
       </c>
       <c r="M64" s="3" t="n">
         <v>0</v>
@@ -5231,10 +5231,10 @@
         <v>1430000</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1930833</v>
+        <v>1931525</v>
       </c>
       <c r="L65" t="n">
-        <v>25.93870106839898</v>
+        <v>25.96523472385809</v>
       </c>
       <c r="M65" s="3" t="n">
         <v>0</v>
@@ -5295,10 +5295,10 @@
         <v>1430000</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>2145417</v>
+        <v>2146187</v>
       </c>
       <c r="L66" t="n">
-        <v>33.34629118721442</v>
+        <v>33.37020492622497</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>0</v>
@@ -5359,10 +5359,10 @@
         <v>1430000</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>2145417</v>
+        <v>2146187</v>
       </c>
       <c r="L67" t="n">
-        <v>33.34629118721442</v>
+        <v>33.37020492622497</v>
       </c>
       <c r="M67" s="3" t="n">
         <v>0</v>
@@ -5485,10 +5485,10 @@
         <v>1480000</v>
       </c>
       <c r="K69" s="3" t="n">
-        <v>2016667</v>
+        <v>2017390</v>
       </c>
       <c r="L69" t="n">
-        <v>26.61158237825085</v>
+        <v>26.63788360207991</v>
       </c>
       <c r="M69" s="3" t="n">
         <v>0</v>
@@ -5611,10 +5611,10 @@
         <v>1605000</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>2188334</v>
+        <v>2189119</v>
       </c>
       <c r="L71" t="n">
-        <v>26.6565341488091</v>
+        <v>26.68283451013856</v>
       </c>
       <c r="M71" s="3" t="n">
         <v>0</v>
@@ -5675,10 +5675,10 @@
         <v>1610000</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>2188334</v>
+        <v>2189119</v>
       </c>
       <c r="L72" t="n">
-        <v>26.42804983151566</v>
+        <v>26.45443212543493</v>
       </c>
       <c r="M72" s="3" t="n">
         <v>0</v>
@@ -5739,10 +5739,10 @@
         <v>1615000</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>2188334</v>
+        <v>2189119</v>
       </c>
       <c r="L73" t="n">
-        <v>26.19956551422223</v>
+        <v>26.22602974073132</v>
       </c>
       <c r="M73" s="3" t="n">
         <v>0</v>
@@ -5803,10 +5803,10 @@
         <v>1630000</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2231251</v>
+        <v>2232052</v>
       </c>
       <c r="L74" t="n">
-        <v>26.94681145240943</v>
+        <v>26.97302751011177</v>
       </c>
       <c r="M74" s="3" t="n">
         <v>0</v>
@@ -5867,10 +5867,10 @@
         <v>1690000</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>2317085</v>
+        <v>2317916</v>
       </c>
       <c r="L75" t="n">
-        <v>27.0635302546087</v>
+        <v>27.08967883219237</v>
       </c>
       <c r="M75" s="3" t="n">
         <v>0</v>
@@ -5931,10 +5931,10 @@
         <v>1705000</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>2317085</v>
+        <v>2317916</v>
       </c>
       <c r="L76" t="n">
-        <v>26.41616513852534</v>
+        <v>26.44254580407573</v>
       </c>
       <c r="M76" s="3" t="n">
         <v>0</v>
@@ -5946,7 +5946,7 @@
         <v>1.9846639603067</v>
       </c>
       <c r="Q76" t="n">
-        <v>11.7</v>
+        <v>11.8</v>
       </c>
       <c r="R76" t="n">
         <v>3</v>
@@ -5995,10 +5995,10 @@
         <v>1725000</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>2360002</v>
+        <v>2360849</v>
       </c>
       <c r="L77" t="n">
-        <v>26.90684160437152</v>
+        <v>26.93306518121235</v>
       </c>
       <c r="M77" s="3" t="n">
         <v>0</v>
@@ -6059,10 +6059,10 @@
         <v>1780000</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>2445836</v>
+        <v>2446713</v>
       </c>
       <c r="L78" t="n">
-        <v>27.22324800191018</v>
+        <v>27.24933410661569</v>
       </c>
       <c r="M78" s="3" t="n">
         <v>0</v>
@@ -6123,10 +6123,10 @@
         <v>1875000</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>2574587</v>
+        <v>2575510</v>
       </c>
       <c r="L79" t="n">
-        <v>27.17278538266526</v>
+        <v>27.19888488105269</v>
       </c>
       <c r="M79" s="3" t="n">
         <v>0</v>
@@ -6187,10 +6187,10 @@
         <v>1910000</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2617504</v>
+        <v>2618442</v>
       </c>
       <c r="L80" t="n">
-        <v>27.02971991637835</v>
+        <v>27.05585993503007</v>
       </c>
       <c r="M80" s="3" t="n">
         <v>0</v>
@@ -6251,10 +6251,10 @@
         <v>2020000</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>2746254</v>
+        <v>2747239</v>
       </c>
       <c r="L81" t="n">
-        <v>26.44525961546164</v>
+        <v>26.47163206404685</v>
       </c>
       <c r="M81" s="3" t="n">
         <v>0</v>
@@ -6315,10 +6315,10 @@
         <v>2110000</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>2875005</v>
+        <v>2876036</v>
       </c>
       <c r="L82" t="n">
-        <v>26.60882328900297</v>
+        <v>26.63513252268052</v>
       </c>
       <c r="M82" s="3" t="n">
         <v>0</v>
@@ -6379,10 +6379,10 @@
         <v>2210000</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>3003756</v>
+        <v>3004833</v>
       </c>
       <c r="L83" t="n">
-        <v>26.4254486715965</v>
+        <v>26.45181945219585</v>
       </c>
       <c r="M83" s="3" t="n">
         <v>0</v>
@@ -6443,10 +6443,10 @@
         <v>2215000</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3046673</v>
+        <v>3047766</v>
       </c>
       <c r="L84" t="n">
-        <v>27.29774412941592</v>
+        <v>27.32381685470603</v>
       </c>
       <c r="M84" s="3" t="n">
         <v>0</v>
@@ -6507,10 +6507,10 @@
         <v>2315000</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3175424</v>
+        <v>3176563</v>
       </c>
       <c r="L85" t="n">
-        <v>27.09634996775234</v>
+        <v>27.1224905660615</v>
       </c>
       <c r="M85" s="3" t="n">
         <v>0</v>
@@ -6571,10 +6571,10 @@
         <v>2395000</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>3304174</v>
+        <v>3305360</v>
       </c>
       <c r="L86" t="n">
-        <v>27.51592379820191</v>
+        <v>27.54193189244137</v>
       </c>
       <c r="M86" s="3" t="n">
         <v>0</v>
@@ -6635,10 +6635,10 @@
         <v>2410000</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3304174</v>
+        <v>3305360</v>
       </c>
       <c r="L87" t="n">
-        <v>27.0619525485038</v>
+        <v>27.0881235326863</v>
       </c>
       <c r="M87" s="3" t="n">
         <v>0</v>
@@ -6699,10 +6699,10 @@
         <v>2499000</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>3432925</v>
+        <v>3434157</v>
       </c>
       <c r="L88" t="n">
-        <v>27.20493456746069</v>
+        <v>27.23104971613121</v>
       </c>
       <c r="M88" s="3" t="n">
         <v>0</v>
@@ -6763,10 +6763,10 @@
         <v>2510000</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>3432925</v>
+        <v>3434157</v>
       </c>
       <c r="L89" t="n">
-        <v>26.88450810897412</v>
+        <v>26.91073821027985</v>
       </c>
       <c r="M89" s="3" t="n">
         <v>0</v>
@@ -6778,7 +6778,7 @@
         <v>83.17546233649077</v>
       </c>
       <c r="Q89" t="n">
-        <v>29.3</v>
+        <v>29.4</v>
       </c>
       <c r="R89" t="n">
         <v>3</v>
@@ -6827,10 +6827,10 @@
         <v>2530000</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>3475842</v>
+        <v>3477089</v>
       </c>
       <c r="L90" t="n">
-        <v>27.21188132256875</v>
+        <v>27.23798556781262</v>
       </c>
       <c r="M90" s="3" t="n">
         <v>0</v>
@@ -6891,10 +6891,10 @@
         <v>2610000</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>3604593</v>
+        <v>3605886</v>
       </c>
       <c r="L91" t="n">
-        <v>27.59238005511302</v>
+        <v>27.61834400754766</v>
       </c>
       <c r="M91" s="3" t="n">
         <v>0</v>
@@ -6955,10 +6955,10 @@
         <v>3015000</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>4162513</v>
+        <v>4164006</v>
       </c>
       <c r="L92" t="n">
-        <v>27.56779378226566</v>
+        <v>27.59376427411488</v>
       </c>
       <c r="M92" s="3" t="n">
         <v>0</v>
@@ -6970,7 +6970,7 @@
         <v>100</v>
       </c>
       <c r="Q92" t="n">
-        <v>33.2</v>
+        <v>33.3</v>
       </c>
       <c r="R92" t="n">
         <v>3</v>
@@ -7019,10 +7019,10 @@
         <v>3098000</v>
       </c>
       <c r="K93" s="3" t="n">
-        <v>4291264</v>
+        <v>4292803</v>
       </c>
       <c r="L93" t="n">
-        <v>27.80681869025071</v>
+        <v>27.83270045236178</v>
       </c>
       <c r="M93" s="3" t="n">
         <v>0</v>
@@ -7034,7 +7034,7 @@
         <v>100</v>
       </c>
       <c r="Q93" t="n">
-        <v>33.3</v>
+        <v>33.4</v>
       </c>
       <c r="R93" t="n">
         <v>3</v>
@@ -7318,10 +7318,10 @@
         <v>309999</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>428740</v>
+        <v>428894</v>
       </c>
       <c r="L2" t="n">
-        <v>27.69533983299902</v>
+        <v>27.72130176687014</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>0</v>
@@ -7385,10 +7385,10 @@
         <v>309999</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>428740</v>
+        <v>428894</v>
       </c>
       <c r="L3" t="n">
-        <v>27.69533983299902</v>
+        <v>27.72130176687014</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0</v>
@@ -7452,10 +7452,10 @@
         <v>310000</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>428740</v>
+        <v>428894</v>
       </c>
       <c r="L4" t="n">
-        <v>27.69510659140738</v>
+        <v>27.72106860902694</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0</v>
@@ -7519,10 +7519,10 @@
         <v>310000</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>428740</v>
+        <v>428894</v>
       </c>
       <c r="L5" t="n">
-        <v>27.69510659140738</v>
+        <v>27.72106860902694</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>0</v>
@@ -7586,10 +7586,10 @@
         <v>384000</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>514574</v>
+        <v>514759</v>
       </c>
       <c r="L6" t="n">
-        <v>25.37516469934353</v>
+        <v>25.40198422951323</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
@@ -7650,10 +7650,10 @@
         <v>384000</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>514574</v>
+        <v>514759</v>
       </c>
       <c r="L7" t="n">
-        <v>25.37516469934353</v>
+        <v>25.40198422951323</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>0</v>
@@ -7714,10 +7714,10 @@
         <v>384000</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>514574</v>
+        <v>514759</v>
       </c>
       <c r="L8" t="n">
-        <v>25.37516469934353</v>
+        <v>25.40198422951323</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
@@ -7778,10 +7778,10 @@
         <v>384000</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>514574</v>
+        <v>514759</v>
       </c>
       <c r="L9" t="n">
-        <v>25.37516469934353</v>
+        <v>25.40198422951323</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>0</v>
@@ -7842,10 +7842,10 @@
         <v>385000</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>514574</v>
+        <v>514759</v>
       </c>
       <c r="L10" t="n">
-        <v>25.18082919074808</v>
+        <v>25.20771856344425</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
@@ -7906,10 +7906,10 @@
         <v>385000</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>514574</v>
+        <v>514759</v>
       </c>
       <c r="L11" t="n">
-        <v>25.18082919074808</v>
+        <v>25.20771856344425</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0</v>
@@ -7970,10 +7970,10 @@
         <v>385000</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>514574</v>
+        <v>514759</v>
       </c>
       <c r="L12" t="n">
-        <v>25.18082919074808</v>
+        <v>25.20771856344425</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
@@ -8034,10 +8034,10 @@
         <v>385000</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>514574</v>
+        <v>514759</v>
       </c>
       <c r="L13" t="n">
-        <v>25.18082919074808</v>
+        <v>25.20771856344425</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0</v>
@@ -8098,13 +8098,13 @@
         <v>388000</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>557491</v>
+        <v>557691</v>
       </c>
       <c r="L14" t="n">
-        <v>30.40246389627815</v>
+        <v>30.42742307119893</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>-27000</v>
+        <v>0</v>
       </c>
       <c r="N14" t="n">
         <v>7.61904761904762</v>
@@ -8165,13 +8165,13 @@
         <v>388000</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>557491</v>
+        <v>557691</v>
       </c>
       <c r="L15" t="n">
-        <v>30.40246389627815</v>
+        <v>30.42742307119893</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>-32000</v>
+        <v>0</v>
       </c>
       <c r="N15" t="n">
         <v>8.705882352941176</v>
@@ -8232,13 +8232,13 @@
         <v>388000</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>557491</v>
+        <v>557691</v>
       </c>
       <c r="L16" t="n">
-        <v>30.40246389627815</v>
+        <v>30.42742307119893</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>-27000</v>
+        <v>0</v>
       </c>
       <c r="N16" t="n">
         <